<commit_message>
Daily workbook: 2026-09-14 23:11 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 14 Sep 2026, 09:00 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 14 Sep 2026, 11:11 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 14 Sep 2026, 09:00 PM · Yahoo Finance data</t>
+          <t>Built 14 Sep 2026, 11:11 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -5140,10 +5140,10 @@
         <v>182.0800018310547</v>
       </c>
       <c r="W15" s="73" t="n">
-        <v>8457430</v>
+        <v>8458066</v>
       </c>
       <c r="X15" s="74" t="n">
-        <v>1.321151097275251</v>
+        <v>1.321243884706015</v>
       </c>
       <c r="Y15" s="28" t="n">
         <v>48.76874867168439</v>
@@ -5816,12 +5816,12 @@
       </c>
       <c r="AY19" s="79" t="inlineStr">
         <is>
+          <t>S&amp;P 500, Nasdaq, Dow Drop On Chipmaker Weakness, Treasury Yield Pressure — MSFT, NFLX, ORCL, CRWD, RBLX In ...</t>
+        </is>
+      </c>
+      <c r="AZ19" s="79" t="inlineStr">
+        <is>
           <t>Texas Instruments Is Up 55% in 2026: This Is the Secret Tech Stock You’re Missing Out On</t>
-        </is>
-      </c>
-      <c r="AZ19" s="79" t="inlineStr">
-        <is>
-          <t>CHWY Is Still Down 34% This Year: Did CHWY Stock Just Find a Bottom?</t>
         </is>
       </c>
     </row>
@@ -5908,7 +5908,7 @@
         <v>-5.70001220703125</v>
       </c>
       <c r="T20" s="83" t="n">
-        <v>703.3250122070312</v>
+        <v>703.2899780273438</v>
       </c>
       <c r="U20" s="83" t="n">
         <v>712.9500122070312</v>
@@ -5999,12 +5999,12 @@
       </c>
       <c r="AX20" s="90" t="inlineStr">
         <is>
+          <t>Forget JEPI: QQQ’s Sponsor Sells an Equal-Weight S&amp;P Income Fund That Charges Less and Is Beating It by 8 P...</t>
+        </is>
+      </c>
+      <c r="AY20" s="90" t="inlineStr">
+        <is>
           <t>Exchange-Traded Funds Mixed as US Equities Fall After Midday</t>
-        </is>
-      </c>
-      <c r="AY20" s="90" t="inlineStr">
-        <is>
-          <t>Exchange-Traded Funds, US Equities Rise After Midday</t>
         </is>
       </c>
       <c r="AZ20" s="90" t="inlineStr">
@@ -6493,7 +6493,7 @@
         <v>0.80999755859375</v>
       </c>
       <c r="T24" s="72" t="n">
-        <v>334.7900085449219</v>
+        <v>334.8299865722656</v>
       </c>
       <c r="U24" s="72" t="n">
         <v>335.5</v>
@@ -6681,7 +6681,7 @@
         <v>-22.72000122070312</v>
       </c>
       <c r="T25" s="83" t="n">
-        <v>486.2799987792969</v>
+        <v>486.1300048828125</v>
       </c>
       <c r="U25" s="83" t="n">
         <v>498.3900146484375</v>
@@ -6772,7 +6772,7 @@
       </c>
       <c r="AX25" s="90" t="inlineStr">
         <is>
-          <t>Chip stocks fall as oil prices gain, Treasury yields stay elevated: AlphaCheck</t>
+          <t>AI-linked stocks slide after tech bosses call for slowdown in ‘reckless’ development</t>
         </is>
       </c>
       <c r="AY25" s="90" t="inlineStr">
@@ -6782,7 +6782,7 @@
       </c>
       <c r="AZ25" s="90" t="inlineStr">
         <is>
-          <t>AI-linked stocks slide after tech bosses call for slowdown in ‘reckless’ development</t>
+          <t>Musk Biographer Says AI Giants May Face Liability After Admitting Risks as Nvidia, AMD Slide</t>
         </is>
       </c>
     </row>
@@ -6869,7 +6869,7 @@
         <v>-3.240005493164062</v>
       </c>
       <c r="T26" s="72" t="n">
-        <v>253.1499938964844</v>
+        <v>253.375</v>
       </c>
       <c r="U26" s="72" t="n">
         <v>255.9499969482422</v>
@@ -6960,17 +6960,17 @@
       </c>
       <c r="AX26" s="79" t="inlineStr">
         <is>
-          <t>Sector Update: Tech Stocks Fall Late Afternoon</t>
+          <t>AMAZON TEAMSTERS RALLY FOR DELIVERY PROTECTION ACT</t>
         </is>
       </c>
       <c r="AY26" s="79" t="inlineStr">
         <is>
-          <t>Sector Update: Consumer Stocks Mixed Late Afternoon</t>
+          <t>FREEHILL Expands Amazon Winter Apparel Collection With Three Heated Products</t>
         </is>
       </c>
       <c r="AZ26" s="79" t="inlineStr">
         <is>
-          <t>Amazon Falls as Its Advertising Reach Extends Into ChatGPT</t>
+          <t>Amazon Faces Tough Questions After Major Crash</t>
         </is>
       </c>
     </row>
@@ -7433,7 +7433,7 @@
         <v>0.1399993896484375</v>
       </c>
       <c r="T29" s="83" t="n">
-        <v>57.43000030517578</v>
+        <v>57.41999816894531</v>
       </c>
       <c r="U29" s="83" t="n">
         <v>61.08990097045898</v>
@@ -7621,7 +7621,7 @@
         <v>-17.26998901367188</v>
       </c>
       <c r="T30" s="72" t="n">
-        <v>349.6300048828125</v>
+        <v>349.4599914550781</v>
       </c>
       <c r="U30" s="72" t="n">
         <v>350.25</v>
@@ -7712,17 +7712,17 @@
       </c>
       <c r="AX30" s="79" t="inlineStr">
         <is>
+          <t>Broadcom Drops Over 4% as $21.7 Billion AI Forecast Meets Slowdown Fears</t>
+        </is>
+      </c>
+      <c r="AY30" s="79" t="inlineStr">
+        <is>
           <t>Broadcom buys its Irvine office building</t>
         </is>
       </c>
-      <c r="AY30" s="79" t="inlineStr">
+      <c r="AZ30" s="79" t="inlineStr">
         <is>
           <t>Is Broadcom Stock in Trouble?</t>
-        </is>
-      </c>
-      <c r="AZ30" s="79" t="inlineStr">
-        <is>
-          <t>Vertiv vs. Broadcom: Which AI Infrastructure Stock Has More Upside?</t>
         </is>
       </c>
     </row>
@@ -7997,7 +7997,7 @@
         <v>-6.009994506835938</v>
       </c>
       <c r="T32" s="72" t="n">
-        <v>82.65000152587891</v>
+        <v>82.47250366210938</v>
       </c>
       <c r="U32" s="72" t="n">
         <v>85.93000030517578</v>
@@ -8098,7 +8098,7 @@
       </c>
       <c r="AZ32" s="79" t="inlineStr">
         <is>
-          <t>Nvidia Stock Could Get a Boost From CoreWeave's Latest Announcement</t>
+          <t>CoreWeave stock drops as analyst flags a major AI demand risk</t>
         </is>
       </c>
     </row>
@@ -8464,17 +8464,17 @@
       </c>
       <c r="AX34" s="79" t="inlineStr">
         <is>
+          <t>Big Tech Issued About $220 Billion of Bonds. Alphabet and Meta Show How AI Is Warping the Credit Market</t>
+        </is>
+      </c>
+      <c r="AY34" s="79" t="inlineStr">
+        <is>
+          <t>Maryland Seeks To Reinstate Digital Ad Tax</t>
+        </is>
+      </c>
+      <c r="AZ34" s="79" t="inlineStr">
+        <is>
           <t>Why Google and Meta Stocks Are the Big Winners From the Latest AI Concerns</t>
-        </is>
-      </c>
-      <c r="AY34" s="79" t="inlineStr">
-        <is>
-          <t>Google, OpenAI, Anthropic Weigh High-Stakes AI Pact</t>
-        </is>
-      </c>
-      <c r="AZ34" s="79" t="inlineStr">
-        <is>
-          <t>Alphabet Gains as AI Slowdown Fears Split the Computing Trade</t>
         </is>
       </c>
     </row>
@@ -8561,7 +8561,7 @@
         <v>-0.660003662109375</v>
       </c>
       <c r="T35" s="83" t="n">
-        <v>41.97000122070312</v>
+        <v>41.95000076293945</v>
       </c>
       <c r="U35" s="83" t="n">
         <v>44.35499954223633</v>
@@ -8749,7 +8749,7 @@
         <v>-5.75</v>
       </c>
       <c r="T36" s="72" t="n">
-        <v>95.81999969482422</v>
+        <v>95.72000122070312</v>
       </c>
       <c r="U36" s="72" t="n">
         <v>98.86000061035156</v>
@@ -8840,17 +8840,17 @@
       </c>
       <c r="AX36" s="79" t="inlineStr">
         <is>
+          <t>Stocks pop when the Trump administration invests, but the gains often fade fast</t>
+        </is>
+      </c>
+      <c r="AY36" s="79" t="inlineStr">
+        <is>
           <t>Oracle, Corning, Alphabet, GE Vernova, CrowdStrike, SpaceX, and More Stocks That Explain Today’s Market</t>
         </is>
       </c>
-      <c r="AY36" s="79" t="inlineStr">
+      <c r="AZ36" s="79" t="inlineStr">
         <is>
           <t>AI Warning Sends Nvidia, AMD, Micron and Intel Shares Tumbling</t>
-        </is>
-      </c>
-      <c r="AZ36" s="79" t="inlineStr">
-        <is>
-          <t>Nvidia’s Training Trade Hit a Speed Bump. Intel Could Win From What Comes Next</t>
         </is>
       </c>
     </row>
@@ -8937,7 +8937,7 @@
         <v>9.779998779296875</v>
       </c>
       <c r="T37" s="83" t="n">
-        <v>497.0599975585938</v>
+        <v>497.5</v>
       </c>
       <c r="U37" s="83" t="n">
         <v>509.9299926757812</v>
@@ -9028,17 +9028,17 @@
       </c>
       <c r="AX37" s="90" t="inlineStr">
         <is>
+          <t>Microsoft Just Made a Move That Could Put More Pressure on Its Azure Business. Here's Why It Could Turn Out...</t>
+        </is>
+      </c>
+      <c r="AY37" s="90" t="inlineStr">
+        <is>
+          <t>Why the Market Dipped But Microsoft (MSFT) Gained Today</t>
+        </is>
+      </c>
+      <c r="AZ37" s="90" t="inlineStr">
+        <is>
           <t>MSFT Stock Gains 2% — Microsoft Unveils ‘Humanist AI’ Code Of Conduct To Curb Autonomous AI Risks</t>
-        </is>
-      </c>
-      <c r="AY37" s="90" t="inlineStr">
-        <is>
-          <t>Sector Update: Tech Stocks Fall Late Afternoon</t>
-        </is>
-      </c>
-      <c r="AZ37" s="90" t="inlineStr">
-        <is>
-          <t>Michael Burry Spots Troubling Signal for AI Stocks</t>
         </is>
       </c>
     </row>
@@ -9125,7 +9125,7 @@
         <v>5.970001220703125</v>
       </c>
       <c r="T38" s="72" t="n">
-        <v>130.8999938964844</v>
+        <v>130.8800048828125</v>
       </c>
       <c r="U38" s="72" t="n">
         <v>137.5099945068359</v>
@@ -9313,7 +9313,7 @@
         <v>-51.22998046875</v>
       </c>
       <c r="T39" s="83" t="n">
-        <v>906.030029296875</v>
+        <v>906.75</v>
       </c>
       <c r="U39" s="83" t="n">
         <v>932.2100219726562</v>
@@ -9404,17 +9404,17 @@
       </c>
       <c r="AX39" s="90" t="inlineStr">
         <is>
+          <t>Dow Jones Futures: Nvidia, Micron, Sandisk Dive On AI Fears; Fed Rate Hike Looms</t>
+        </is>
+      </c>
+      <c r="AY39" s="90" t="inlineStr">
+        <is>
+          <t>Micron (MU) Falls More Steeply Than Broader Market: What Investors Need to Know</t>
+        </is>
+      </c>
+      <c r="AZ39" s="90" t="inlineStr">
+        <is>
           <t>AI Warning Sends Nvidia, AMD, Micron and Intel Shares Tumbling</t>
-        </is>
-      </c>
-      <c r="AY39" s="90" t="inlineStr">
-        <is>
-          <t>Micron Stock Sends Urgent Signal as Shares Slide</t>
-        </is>
-      </c>
-      <c r="AZ39" s="90" t="inlineStr">
-        <is>
-          <t>Micron Stock Sinks Again. What AI Safety Fears Mean for Memory Chips.</t>
         </is>
       </c>
     </row>
@@ -9780,17 +9780,17 @@
       </c>
       <c r="AX41" s="90" t="inlineStr">
         <is>
+          <t>Why Netflix Stock Rallied Today</t>
+        </is>
+      </c>
+      <c r="AY41" s="90" t="inlineStr">
+        <is>
+          <t>Netflix stock jumps as Wall Street sees a new growth engine</t>
+        </is>
+      </c>
+      <c r="AZ41" s="90" t="inlineStr">
+        <is>
           <t>Netflix Stock Rose 4% While the AI Trade Sold Off on Monday. Its Capital Goes Into Shows, Not Silicon.</t>
-        </is>
-      </c>
-      <c r="AY41" s="90" t="inlineStr">
-        <is>
-          <t>Netflix Shares Jump After Evercore Raises Price Target To $110</t>
-        </is>
-      </c>
-      <c r="AZ41" s="90" t="inlineStr">
-        <is>
-          <t>Netflix Climbs 4%, Alphabet Ticks Up, Amazon Barely Budges as New Streaming Policy Alliance Launches</t>
         </is>
       </c>
     </row>
@@ -10065,7 +10065,7 @@
         <v>-7.329986572265625</v>
       </c>
       <c r="T43" s="83" t="n">
-        <v>211.2400054931641</v>
+        <v>211.0800018310547</v>
       </c>
       <c r="U43" s="83" t="n">
         <v>212.7700042724609</v>
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
-          <t>Coda Octopus Group, Inc. Q3 2026 Earnings Call Summary</t>
+          <t>Dow Jones Futures: Nvidia, Micron, Sandisk Dive On AI Fears; Fed Rate Hike Looms</t>
         </is>
       </c>
       <c r="AY43" s="90" t="inlineStr">
         <is>
-          <t>The Hain Celestial Group, Inc. Q1 2027 Earnings Call Summary</t>
+          <t>New Fed Chair Warsh Vowed a Policy Overhaul to Crush Inflation When He Took Office. Has He Followed Through?</t>
         </is>
       </c>
       <c r="AZ43" s="90" t="inlineStr">
         <is>
-          <t>5 Top AI Stocks to Buy on the Dip as Slowdown Fears Hit Markets</t>
+          <t>Why Did GE Vernova Stock Fall Today?</t>
         </is>
       </c>
     </row>
@@ -10253,7 +10253,7 @@
         <v>6.080001831054688</v>
       </c>
       <c r="T44" s="72" t="n">
-        <v>169.6950073242188</v>
+        <v>169.6999969482422</v>
       </c>
       <c r="U44" s="72" t="n">
         <v>174.3598937988281</v>
@@ -10629,7 +10629,7 @@
         <v>-0.4000015258789062</v>
       </c>
       <c r="T46" s="72" t="n">
-        <v>60.54999923706055</v>
+        <v>60.56999969482422</v>
       </c>
       <c r="U46" s="72" t="n">
         <v>63.375</v>
@@ -10913,12 +10913,12 @@
       </c>
       <c r="AY47" s="90" t="inlineStr">
         <is>
+          <t>Dow Jones Futures: Nvidia, Micron, Sandisk Dive On AI Fears; Fed Rate Hike Looms</t>
+        </is>
+      </c>
+      <c r="AZ47" s="90" t="inlineStr">
+        <is>
           <t>Should You Buy SanDisk Stock Because It Has Started Retiring Its Own Shares?</t>
-        </is>
-      </c>
-      <c r="AZ47" s="90" t="inlineStr">
-        <is>
-          <t>SanDisk Falls 4.6% With Prices Driving Two-Thirds of Its Quarterly Sales Jump</t>
         </is>
       </c>
     </row>
@@ -11005,7 +11005,7 @@
         <v>-6.470001220703125</v>
       </c>
       <c r="T48" s="72" t="n">
-        <v>359.7799987792969</v>
+        <v>359.9500122070312</v>
       </c>
       <c r="U48" s="72" t="n">
         <v>367.7300109863281</v>
@@ -11096,17 +11096,17 @@
       </c>
       <c r="AX48" s="79" t="inlineStr">
         <is>
-          <t>Elon Musk: I've been 'sounding the alarm' on AI for a while</t>
+          <t>Musk offers radical fix to welfare state bankruptcy</t>
         </is>
       </c>
       <c r="AY48" s="79" t="inlineStr">
         <is>
-          <t>Elon Musk Says Optimus Will Ship to Customers in 2027. Here's How Much Revenue That Could Actually Generate.</t>
+          <t>If You'd Invested $1,000 in Tesla Stock 1 Year Ago, Here's How Much You'd Have Today</t>
         </is>
       </c>
       <c r="AZ48" s="79" t="inlineStr">
         <is>
-          <t>VFS Stock Pressured As Tesla Gains A Legal Foothold In VinFast’s Home Market</t>
+          <t>Tesla Roadster Reveal Could Be Musk's Biggest Test Yet</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 14 Sep 2026, 09:00 PM · Yahoo Finance data</t>
+          <t>Built 14 Sep 2026, 11:11 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 14 Sep 2026, 09:00 PM · Yahoo Finance data</t>
+          <t>Built 14 Sep 2026, 11:11 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 14 Sep 2026, 09:00 PM · Yahoo Finance data</t>
+          <t>Built 14 Sep 2026, 11:11 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 14 Sep 2026, 09:00 PM · Yahoo Finance data</t>
+          <t>Built 14 Sep 2026, 11:11 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -44416,7 +44416,7 @@
       </c>
       <c r="D23" s="105" t="inlineStr">
         <is>
-          <t>Gapped down 4.2% at the open</t>
+          <t>Gapped down 4.3% at the open</t>
         </is>
       </c>
       <c r="E23" s="33" t="n">
@@ -44584,7 +44584,7 @@
       </c>
       <c r="D29" s="105" t="inlineStr">
         <is>
-          <t>Gapped down 6.9% at the open</t>
+          <t>Gapped down 7.0% at the open</t>
         </is>
       </c>
       <c r="E29" s="33" t="n">
@@ -45480,7 +45480,7 @@
       </c>
       <c r="D61" s="105" t="inlineStr">
         <is>
-          <t>Gapped down 3.2% at the open</t>
+          <t>Gapped down 3.3% at the open</t>
         </is>
       </c>
       <c r="E61" s="33" t="n">
@@ -45592,7 +45592,7 @@
       </c>
       <c r="D65" s="105" t="inlineStr">
         <is>
-          <t>Gapped down 7.1% at the open</t>
+          <t>Gapped down 7.0% at the open</t>
         </is>
       </c>
       <c r="E65" s="33" t="n">
@@ -46152,7 +46152,7 @@
       </c>
       <c r="D85" s="105" t="inlineStr">
         <is>
-          <t>Gapped down 3.4% at the open</t>
+          <t>Gapped down 3.5% at the open</t>
         </is>
       </c>
       <c r="E85" s="33" t="n">
@@ -46292,7 +46292,7 @@
       </c>
       <c r="D90" s="106" t="inlineStr">
         <is>
-          <t>Gapped down 7.1% at the open</t>
+          <t>Gapped down 7.3% at the open</t>
         </is>
       </c>
       <c r="E90" s="26" t="n">

</xml_diff>

<commit_message>
Daily workbook: 2026-09-14 23:51 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 14 Sep 2026, 11:11 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 14 Sep 2026, 11:51 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 14 Sep 2026, 11:11 PM · Yahoo Finance data</t>
+          <t>Built 14 Sep 2026, 11:51 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -7712,17 +7712,17 @@
       </c>
       <c r="AX30" s="79" t="inlineStr">
         <is>
+          <t>3 Stocks That Offer AI Exposure and Dividends</t>
+        </is>
+      </c>
+      <c r="AY30" s="79" t="inlineStr">
+        <is>
           <t>Broadcom Drops Over 4% as $21.7 Billion AI Forecast Meets Slowdown Fears</t>
         </is>
       </c>
-      <c r="AY30" s="79" t="inlineStr">
+      <c r="AZ30" s="79" t="inlineStr">
         <is>
           <t>Broadcom buys its Irvine office building</t>
-        </is>
-      </c>
-      <c r="AZ30" s="79" t="inlineStr">
-        <is>
-          <t>Is Broadcom Stock in Trouble?</t>
         </is>
       </c>
     </row>
@@ -8652,17 +8652,17 @@
       </c>
       <c r="AX35" s="90" t="inlineStr">
         <is>
+          <t>IREN Stock Slips, But A Top Wall Street Bank Is Bullish With Double-Upgrade And 50% Upside</t>
+        </is>
+      </c>
+      <c r="AY35" s="90" t="inlineStr">
+        <is>
           <t>AI Leaders Say Slow Down. IREN Says Compute Demand May Never Be Satisfied. Nvidia Sits in the Middle</t>
         </is>
       </c>
-      <c r="AY35" s="90" t="inlineStr">
+      <c r="AZ35" s="90" t="inlineStr">
         <is>
           <t>Why Iren Stock Just Got a Double Upgrade to Buy</t>
-        </is>
-      </c>
-      <c r="AZ35" s="90" t="inlineStr">
-        <is>
-          <t>IREN falls 5% despite CEO's bullish AI supply warning</t>
         </is>
       </c>
     </row>
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
+          <t>Prediction: Interactive Brokers Ends 2026 With More Than 6 Million Customer Accounts</t>
+        </is>
+      </c>
+      <c r="AY43" s="90" t="inlineStr">
+        <is>
           <t>Dow Jones Futures: Nvidia, Micron, Sandisk Dive On AI Fears; Fed Rate Hike Looms</t>
         </is>
       </c>
-      <c r="AY43" s="90" t="inlineStr">
+      <c r="AZ43" s="90" t="inlineStr">
         <is>
           <t>New Fed Chair Warsh Vowed a Policy Overhaul to Crush Inflation When He Took Office. Has He Followed Through?</t>
-        </is>
-      </c>
-      <c r="AZ43" s="90" t="inlineStr">
-        <is>
-          <t>Why Did GE Vernova Stock Fall Today?</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 14 Sep 2026, 11:11 PM · Yahoo Finance data</t>
+          <t>Built 14 Sep 2026, 11:51 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 14 Sep 2026, 11:11 PM · Yahoo Finance data</t>
+          <t>Built 14 Sep 2026, 11:51 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 14 Sep 2026, 11:11 PM · Yahoo Finance data</t>
+          <t>Built 14 Sep 2026, 11:51 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 14 Sep 2026, 11:11 PM · Yahoo Finance data</t>
+          <t>Built 14 Sep 2026, 11:51 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-09-15 22:55 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 15 Sep 2026, 08:21 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 15 Sep 2026, 10:55 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -2321,7 +2321,7 @@
         </is>
       </c>
       <c r="I38" s="33" t="n">
-        <v>-0.009586362858249764</v>
+        <v>-0.009621023856200339</v>
       </c>
       <c r="J38" s="34" t="n">
         <v>1</v>
@@ -2332,7 +2332,7 @@
         </is>
       </c>
       <c r="L38" s="35" t="n">
-        <v>33.94947524439775</v>
+        <v>33.93817844669225</v>
       </c>
     </row>
     <row r="41" ht="22" customHeight="1">
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 15 Sep 2026, 08:21 PM · Yahoo Finance data</t>
+          <t>Built 15 Sep 2026, 10:55 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -3620,10 +3620,10 @@
         <v>168.4199981689453</v>
       </c>
       <c r="W7" s="73" t="n">
-        <v>8841535</v>
+        <v>8841594</v>
       </c>
       <c r="X7" s="74" t="n">
-        <v>1.242360641681684</v>
+        <v>1.242368417033189</v>
       </c>
       <c r="Y7" s="28" t="n">
         <v>30.53889453483444</v>
@@ -3810,10 +3810,10 @@
         <v>166.1782989501953</v>
       </c>
       <c r="W8" s="84" t="n">
-        <v>7188241</v>
+        <v>7188476</v>
       </c>
       <c r="X8" s="85" t="n">
-        <v>0.9099595525273283</v>
+        <v>0.9099879476355602</v>
       </c>
       <c r="Y8" s="35" t="n">
         <v>47.65071236962449</v>
@@ -4000,10 +4000,10 @@
         <v>56.45999908447266</v>
       </c>
       <c r="W9" s="73" t="n">
-        <v>30074678</v>
+        <v>30083475</v>
       </c>
       <c r="X9" s="74" t="n">
-        <v>1.02388282387244</v>
+        <v>1.024166978489999</v>
       </c>
       <c r="Y9" s="28" t="n">
         <v>44.64960658538779</v>
@@ -4190,10 +4190,10 @@
         <v>64.81500244140625</v>
       </c>
       <c r="W10" s="84" t="n">
-        <v>34139670</v>
+        <v>34174929</v>
       </c>
       <c r="X10" s="85" t="n">
-        <v>1.196303470643423</v>
+        <v>1.197465022074775</v>
       </c>
       <c r="Y10" s="35" t="n">
         <v>67.26827292365583</v>
@@ -4380,10 +4380,10 @@
         <v>83.56500244140625</v>
       </c>
       <c r="W11" s="73" t="n">
-        <v>14142441</v>
+        <v>14142799</v>
       </c>
       <c r="X11" s="74" t="n">
-        <v>1.414560671605502</v>
+        <v>1.414593946929188</v>
       </c>
       <c r="Y11" s="28" t="n">
         <v>43.7557145451249</v>
@@ -4570,10 +4570,10 @@
         <v>110.5599975585938</v>
       </c>
       <c r="W12" s="84" t="n">
-        <v>12647267</v>
+        <v>12671661</v>
       </c>
       <c r="X12" s="85" t="n">
-        <v>2.181502318579946</v>
+        <v>2.185250250915156</v>
       </c>
       <c r="Y12" s="35" t="n">
         <v>35.31020243702154</v>
@@ -4760,10 +4760,10 @@
         <v>113.8249969482422</v>
       </c>
       <c r="W13" s="73" t="n">
-        <v>5497266</v>
+        <v>5497565</v>
       </c>
       <c r="X13" s="74" t="n">
-        <v>1.314690896496646</v>
+        <v>1.314757702706007</v>
       </c>
       <c r="Y13" s="28" t="n">
         <v>57.15102292992972</v>
@@ -4950,10 +4950,10 @@
         <v>50.2599983215332</v>
       </c>
       <c r="W14" s="84" t="n">
-        <v>9772767</v>
+        <v>9773383</v>
       </c>
       <c r="X14" s="85" t="n">
-        <v>0.8786679005113653</v>
+        <v>0.8787208515977358</v>
       </c>
       <c r="Y14" s="35" t="n">
         <v>38.76369503995539</v>
@@ -5140,10 +5140,10 @@
         <v>183.4649963378906</v>
       </c>
       <c r="W15" s="73" t="n">
-        <v>6077830</v>
+        <v>6129392</v>
       </c>
       <c r="X15" s="74" t="n">
-        <v>0.9490349451529745</v>
+        <v>0.9567010649123473</v>
       </c>
       <c r="Y15" s="28" t="n">
         <v>47.82556828665138</v>
@@ -5330,10 +5330,10 @@
         <v>42.70500183105469</v>
       </c>
       <c r="W16" s="84" t="n">
-        <v>4538615</v>
+        <v>4538847</v>
       </c>
       <c r="X16" s="85" t="n">
-        <v>0.9164243113728384</v>
+        <v>0.9164690095673887</v>
       </c>
       <c r="Y16" s="35" t="n">
         <v>34.71971041574344</v>
@@ -5520,10 +5520,10 @@
         <v>41.29000091552734</v>
       </c>
       <c r="W17" s="73" t="n">
-        <v>24067061</v>
+        <v>24130795</v>
       </c>
       <c r="X17" s="74" t="n">
-        <v>1.172991453582146</v>
+        <v>1.175915113421329</v>
       </c>
       <c r="Y17" s="28" t="n">
         <v>29.98237596156805</v>
@@ -5645,7 +5645,7 @@
         </is>
       </c>
       <c r="C19" s="26" t="n">
-        <v>-0.00452108403339635</v>
+        <v>-0.004586781374170235</v>
       </c>
       <c r="D19" s="27" t="n">
         <v>2</v>
@@ -5714,10 +5714,10 @@
         </is>
       </c>
       <c r="R19" s="70" t="n">
-        <v>757.4400024414062</v>
+        <v>757.3900146484375</v>
       </c>
       <c r="S19" s="71" t="n">
-        <v>-3.44000244140625</v>
+        <v>-3.489990234375</v>
       </c>
       <c r="T19" s="72" t="n">
         <v>760.1170043945312</v>
@@ -5729,61 +5729,61 @@
         <v>756.1500244140625</v>
       </c>
       <c r="W19" s="73" t="n">
-        <v>44101770</v>
+        <v>44728394</v>
       </c>
       <c r="X19" s="74" t="n">
-        <v>1.14574310454329</v>
+        <v>1.161077417500923</v>
       </c>
       <c r="Y19" s="28" t="n">
-        <v>44.44806392657969</v>
+        <v>44.40892774135338</v>
       </c>
       <c r="Z19" s="28" t="n">
-        <v>6.736190570289367</v>
+        <v>6.475157209652179</v>
       </c>
       <c r="AA19" s="28" t="n">
         <v>11.45692164683003</v>
       </c>
       <c r="AB19" s="75" t="n">
-        <v>0.01674445058256424</v>
+        <v>0.01275682037419301</v>
       </c>
       <c r="AC19" s="75" t="n">
-        <v>1.690704846873231</v>
+        <v>1.689907320831557</v>
       </c>
       <c r="AD19" s="75" t="n">
-        <v>-1.673960396290667</v>
+        <v>-1.677150500457364</v>
       </c>
       <c r="AE19" s="72" t="n">
-        <v>762.3333564934067</v>
+        <v>762.3222480949692</v>
       </c>
       <c r="AF19" s="72" t="n">
-        <v>763.8894575165893</v>
+        <v>763.884913171774</v>
       </c>
       <c r="AG19" s="72" t="n">
-        <v>759.0616003417969</v>
+        <v>759.0606005859376</v>
       </c>
       <c r="AH19" s="72" t="n">
-        <v>748.644301147461</v>
+        <v>748.6438012695312</v>
       </c>
       <c r="AI19" s="72" t="n">
-        <v>715.1068002319336</v>
+        <v>715.1065502929688</v>
       </c>
       <c r="AJ19" s="72" t="n">
-        <v>773.4545103432985</v>
+        <v>773.4617785432248</v>
       </c>
       <c r="AK19" s="72" t="n">
-        <v>765.3444946289062</v>
+        <v>765.3419952392578</v>
       </c>
       <c r="AL19" s="72" t="n">
-        <v>757.2344789145139</v>
+        <v>757.2222119352908</v>
       </c>
       <c r="AM19" s="76" t="n">
-        <v>0.01267096970771457</v>
+        <v>0.01033295513346331</v>
       </c>
       <c r="AN19" s="29" t="n">
-        <v>2.119311178510424</v>
+        <v>2.121870576676931</v>
       </c>
       <c r="AO19" s="77" t="n">
-        <v>0.8077308601216064</v>
+        <v>0.8077841704138328</v>
       </c>
       <c r="AP19" s="72" t="n">
         <v>779.3699951171875</v>
@@ -5792,22 +5792,22 @@
         <v>629.280029296875</v>
       </c>
       <c r="AR19" s="29" t="n">
-        <v>-2.813810233031078</v>
+        <v>-2.820224104912461</v>
       </c>
       <c r="AS19" s="78" t="n">
-        <v>85.3887682924548</v>
+        <v>85.35546307268508</v>
       </c>
       <c r="AT19" s="26" t="n">
-        <v>-0.01112332143563777</v>
+        <v>-0.01118858305704717</v>
       </c>
       <c r="AU19" s="26" t="n">
-        <v>-0.02434503408334643</v>
+        <v>-0.02440942312840344</v>
       </c>
       <c r="AV19" s="26" t="n">
-        <v>0.003457712720043915</v>
+        <v>0.003391488812889865</v>
       </c>
       <c r="AW19" s="26" t="n">
-        <v>0.110746159995138</v>
+        <v>0.1106728555104162</v>
       </c>
       <c r="AX19" s="79" t="inlineStr">
         <is>
@@ -5816,12 +5816,12 @@
       </c>
       <c r="AY19" s="79" t="inlineStr">
         <is>
-          <t>Norwegian Falls 3% as Wells Fargo Trims Carnival Target on Caribbean Pricing Pressure; Carnival Slips, Roya...</t>
+          <t>S&amp;P 500, Nasdaq, Dow End Lower As Investors Price In Rate Hike Ahead Of Fed Meeting — AMZN, META, MU, TSLA,...</t>
         </is>
       </c>
       <c r="AZ19" s="79" t="inlineStr">
         <is>
-          <t>Offshore Oil Stocks Rally While the Broad Market Slips: Transocean Climbs 6%, Valaris Rises 6%, W&amp;T Offshor...</t>
+          <t>Wells Fargo's new S&amp;P 500 call signals trouble ahead</t>
         </is>
       </c>
     </row>
@@ -5908,7 +5908,7 @@
         <v>-4.6400146484375</v>
       </c>
       <c r="T20" s="83" t="n">
-        <v>708.7999877929688</v>
+        <v>708.760009765625</v>
       </c>
       <c r="U20" s="83" t="n">
         <v>709.5299072265625</v>
@@ -5917,10 +5917,10 @@
         <v>703.635009765625</v>
       </c>
       <c r="W20" s="84" t="n">
-        <v>25950029</v>
+        <v>26166846</v>
       </c>
       <c r="X20" s="85" t="n">
-        <v>0.8320831618446323</v>
+        <v>0.8387438054934007</v>
       </c>
       <c r="Y20" s="35" t="n">
         <v>43.97758397350066</v>
@@ -6021,7 +6021,7 @@
         </is>
       </c>
       <c r="C21" s="26" t="n">
-        <v>-0.009586362858249764</v>
+        <v>-0.009621023856200339</v>
       </c>
       <c r="D21" s="27" t="n">
         <v>4</v>
@@ -6090,10 +6090,10 @@
         </is>
       </c>
       <c r="R21" s="70" t="n">
-        <v>285.1499938964844</v>
+        <v>285.1400146484375</v>
       </c>
       <c r="S21" s="71" t="n">
-        <v>-2.760009765625</v>
+        <v>-2.769989013671875</v>
       </c>
       <c r="T21" s="72" t="n">
         <v>286.6199951171875</v>
@@ -6105,61 +6105,61 @@
         <v>284.0799865722656</v>
       </c>
       <c r="W21" s="73" t="n">
-        <v>24594139</v>
+        <v>24844188</v>
       </c>
       <c r="X21" s="74" t="n">
-        <v>1.274930523768115</v>
+        <v>1.287058604509135</v>
       </c>
       <c r="Y21" s="28" t="n">
-        <v>33.94947524439775</v>
+        <v>33.93817844669225</v>
       </c>
       <c r="Z21" s="28" t="n">
-        <v>6.560426010436957</v>
+        <v>6.499241271819282</v>
       </c>
       <c r="AA21" s="28" t="n">
         <v>27.0957038405081</v>
       </c>
       <c r="AB21" s="75" t="n">
-        <v>-2.66474726090172</v>
+        <v>-2.665543326272996</v>
       </c>
       <c r="AC21" s="75" t="n">
-        <v>-1.439835242773871</v>
+        <v>-1.439994455848126</v>
       </c>
       <c r="AD21" s="75" t="n">
-        <v>-1.224912018127849</v>
+        <v>-1.22554887042487</v>
       </c>
       <c r="AE21" s="72" t="n">
-        <v>289.7711615700357</v>
+        <v>289.7689439593586</v>
       </c>
       <c r="AF21" s="72" t="n">
-        <v>293.4189204086947</v>
+        <v>293.4180132043268</v>
       </c>
       <c r="AG21" s="72" t="n">
-        <v>295.8122021484375</v>
+        <v>295.8120025634765</v>
       </c>
       <c r="AH21" s="72" t="n">
-        <v>291.420901184082</v>
+        <v>291.4208013916016</v>
       </c>
       <c r="AI21" s="72" t="n">
-        <v>274.272350692749</v>
+        <v>274.2723007965088</v>
       </c>
       <c r="AJ21" s="72" t="n">
-        <v>304.2744718946124</v>
+        <v>304.2760052661416</v>
       </c>
       <c r="AK21" s="72" t="n">
-        <v>294.797004699707</v>
+        <v>294.7965057373047</v>
       </c>
       <c r="AL21" s="72" t="n">
-        <v>285.3195375048016</v>
+        <v>285.3170062084678</v>
       </c>
       <c r="AM21" s="76" t="n">
-        <v>-0.008944563185004091</v>
+        <v>-0.009335490734079264</v>
       </c>
       <c r="AN21" s="29" t="n">
-        <v>6.429825977750042</v>
+        <v>6.43121566527937</v>
       </c>
       <c r="AO21" s="77" t="n">
-        <v>1.165110131182611</v>
+        <v>1.165150907371163</v>
       </c>
       <c r="AP21" s="72" t="n">
         <v>305.1799926757812</v>
@@ -6168,22 +6168,22 @@
         <v>228.8999938964844</v>
       </c>
       <c r="AR21" s="29" t="n">
-        <v>-6.563339425915926</v>
+        <v>-6.566609380790545</v>
       </c>
       <c r="AS21" s="78" t="n">
-        <v>73.74147994253349</v>
+        <v>73.72839755107233</v>
       </c>
       <c r="AT21" s="26" t="n">
-        <v>-0.03230739164976049</v>
+        <v>-0.03234125749152295</v>
       </c>
       <c r="AU21" s="26" t="n">
-        <v>-0.06535777206972881</v>
+        <v>-0.06539048126428337</v>
       </c>
       <c r="AV21" s="26" t="n">
-        <v>-0.03220886600646067</v>
+        <v>-0.03224273529627442</v>
       </c>
       <c r="AW21" s="26" t="n">
-        <v>0.1583928731488584</v>
+        <v>0.158352333467763</v>
       </c>
       <c r="AX21" s="79" t="inlineStr">
         <is>
@@ -6293,10 +6293,10 @@
         <v>100.961799621582</v>
       </c>
       <c r="W22" s="84" t="n">
-        <v>55970069</v>
+        <v>56370700</v>
       </c>
       <c r="X22" s="85" t="n">
-        <v>0.9668000469932991</v>
+        <v>0.9733835485027614</v>
       </c>
       <c r="Y22" s="35" t="n">
         <v>40.19585585346517</v>
@@ -6493,7 +6493,7 @@
         <v>-1.739990234375</v>
       </c>
       <c r="T24" s="72" t="n">
-        <v>330.135009765625</v>
+        <v>330.260009765625</v>
       </c>
       <c r="U24" s="72" t="n">
         <v>331.760009765625</v>
@@ -6502,10 +6502,10 @@
         <v>328.3500061035156</v>
       </c>
       <c r="W24" s="73" t="n">
-        <v>31387302</v>
+        <v>31420574</v>
       </c>
       <c r="X24" s="74" t="n">
-        <v>0.7342710756796513</v>
+        <v>0.7350208315765693</v>
       </c>
       <c r="Y24" s="28" t="n">
         <v>61.30857194712112</v>
@@ -6584,17 +6584,17 @@
       </c>
       <c r="AX24" s="79" t="inlineStr">
         <is>
+          <t>Dow Jones Tech Titan Apple, Nvidia Chipmaker TSMC, AMD, Bloom Energy In Or Near Buy Zones</t>
+        </is>
+      </c>
+      <c r="AY24" s="79" t="inlineStr">
+        <is>
+          <t>Jim Cramer Believes Apple (AAPL) Could See “Off The Charts” Demand For Its New Foldable</t>
+        </is>
+      </c>
+      <c r="AZ24" s="79" t="inlineStr">
+        <is>
           <t>Apple Falls as Siri AI Arrives Behind a Beta Label</t>
-        </is>
-      </c>
-      <c r="AY24" s="79" t="inlineStr">
-        <is>
-          <t>Apple Stock: New CEO, Foldable iPhone-Time to Buy the Dip?</t>
-        </is>
-      </c>
-      <c r="AZ24" s="79" t="inlineStr">
-        <is>
-          <t>Skyworks gains 12% on Apple component hopes and Qorvo merger progress</t>
         </is>
       </c>
     </row>
@@ -6681,7 +6681,7 @@
         <v>10.79000854492188</v>
       </c>
       <c r="T25" s="83" t="n">
-        <v>501.7000122070312</v>
+        <v>501.125</v>
       </c>
       <c r="U25" s="83" t="n">
         <v>513.6649780273438</v>
@@ -6690,10 +6690,10 @@
         <v>497.510986328125</v>
       </c>
       <c r="W25" s="84" t="n">
-        <v>16821679</v>
+        <v>16963710</v>
       </c>
       <c r="X25" s="85" t="n">
-        <v>0.944073178639971</v>
+        <v>0.9516650088633875</v>
       </c>
       <c r="Y25" s="35" t="n">
         <v>54.13058387754214</v>
@@ -6772,17 +6772,17 @@
       </c>
       <c r="AX25" s="90" t="inlineStr">
         <is>
+          <t>Dow Jones Tech Titan Apple, Nvidia Chipmaker TSMC, AMD, Bloom Energy In Or Near Buy Zones</t>
+        </is>
+      </c>
+      <c r="AY25" s="90" t="inlineStr">
+        <is>
           <t>Bank of America says investors get AMD stock wrong</t>
         </is>
       </c>
-      <c r="AY25" s="90" t="inlineStr">
+      <c r="AZ25" s="90" t="inlineStr">
         <is>
           <t>AMD Rebounds 3% as Its 58% AI Engine Faces a Pause</t>
-        </is>
-      </c>
-      <c r="AZ25" s="90" t="inlineStr">
-        <is>
-          <t>Nvidia Will Still Beat AMD Through 2028. Here's the Data Behind My Conviction.</t>
         </is>
       </c>
     </row>
@@ -6869,7 +6869,7 @@
         <v>-5.1199951171875</v>
       </c>
       <c r="T26" s="72" t="n">
-        <v>252.2400054931641</v>
+        <v>252.375</v>
       </c>
       <c r="U26" s="72" t="n">
         <v>253.2700042724609</v>
@@ -6878,10 +6878,10 @@
         <v>247.2200012207031</v>
       </c>
       <c r="W26" s="73" t="n">
-        <v>35500070</v>
+        <v>35783529</v>
       </c>
       <c r="X26" s="74" t="n">
-        <v>1.113527565720463</v>
+        <v>1.121920036532986</v>
       </c>
       <c r="Y26" s="28" t="n">
         <v>41.41705451283769</v>
@@ -6960,17 +6960,17 @@
       </c>
       <c r="AX26" s="79" t="inlineStr">
         <is>
-          <t>Sector Update: Tech Stocks Mixed Late Afternoon</t>
+          <t>Amazon (AMZN) Dips More Than Broader Market: What You Should Know</t>
         </is>
       </c>
       <c r="AY26" s="79" t="inlineStr">
         <is>
-          <t>California Investor Scoops Up Amazon Warehouse: The Chicago Deal Sheet</t>
+          <t>Amazon sells luxury solar-powered watches from brands like Seiko and Citizen starting at $210</t>
         </is>
       </c>
       <c r="AZ26" s="79" t="inlineStr">
         <is>
-          <t>AI Slowdown Fears Rise: Buy NVIDIA, HPE That Connect AI and Quantum</t>
+          <t>AMZN Stock Slips 2%: Amazon Unable To Recover Data Lost From Middle East Centers Affected By Iran War</t>
         </is>
       </c>
     </row>
@@ -7066,10 +7066,10 @@
         <v>82.91999816894531</v>
       </c>
       <c r="W27" s="84" t="n">
-        <v>3860165</v>
+        <v>3860834</v>
       </c>
       <c r="X27" s="85" t="n">
-        <v>0.7949386402074619</v>
+        <v>0.7950709331171207</v>
       </c>
       <c r="Y27" s="35" t="n">
         <v>51.07859672472348</v>
@@ -7245,7 +7245,7 @@
         <v>2.82000732421875</v>
       </c>
       <c r="T28" s="72" t="n">
-        <v>241.625</v>
+        <v>242</v>
       </c>
       <c r="U28" s="72" t="n">
         <v>253.1549987792969</v>
@@ -7254,10 +7254,10 @@
         <v>240.6799926757812</v>
       </c>
       <c r="W28" s="73" t="n">
-        <v>3741240</v>
+        <v>3760370</v>
       </c>
       <c r="X28" s="74" t="n">
-        <v>0.9455916544568227</v>
+        <v>0.9501970138195842</v>
       </c>
       <c r="Y28" s="28" t="n">
         <v>44.21546767091107</v>
@@ -7370,7 +7370,7 @@
       </c>
       <c r="F29" s="30" t="inlineStr">
         <is>
-          <t>Same</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G29" s="30" t="inlineStr">
@@ -7433,7 +7433,7 @@
         <v>-1.229999542236328</v>
       </c>
       <c r="T29" s="83" t="n">
-        <v>59.70999908447266</v>
+        <v>59.47999954223633</v>
       </c>
       <c r="U29" s="83" t="n">
         <v>60.7599983215332</v>
@@ -7442,10 +7442,10 @@
         <v>57.81050109863281</v>
       </c>
       <c r="W29" s="84" t="n">
-        <v>6911602</v>
+        <v>7136907</v>
       </c>
       <c r="X29" s="85" t="n">
-        <v>0.7475776338153681</v>
+        <v>0.7710077766335546</v>
       </c>
       <c r="Y29" s="35" t="n">
         <v>42.86787724041201</v>
@@ -7524,17 +7524,17 @@
       </c>
       <c r="AX29" s="90" t="inlineStr">
         <is>
+          <t>AST SpaceMobile, Inc. (ASTS) Declines More Than Market: Some Information for Investors</t>
+        </is>
+      </c>
+      <c r="AY29" s="90" t="inlineStr">
+        <is>
+          <t>AST SpaceMobile vs. Redwire: Which Space Infrastructure Stock Is a Better Buy in 2026?</t>
+        </is>
+      </c>
+      <c r="AZ29" s="90" t="inlineStr">
+        <is>
           <t>Aviat Plunges 16% in a Year: Should Investors Avoid the Stock Now?</t>
-        </is>
-      </c>
-      <c r="AY29" s="90" t="inlineStr">
-        <is>
-          <t>AST SpaceMobile (ASTS) Stock May Be Expensive Despite Its Huge 3 Year Run</t>
-        </is>
-      </c>
-      <c r="AZ29" s="90" t="inlineStr">
-        <is>
-          <t>Can AST SpaceMobile's Expanding MNO Base Boost Its Revenue Prospects?</t>
         </is>
       </c>
     </row>
@@ -7621,7 +7621,7 @@
         <v>-5.45001220703125</v>
       </c>
       <c r="T30" s="72" t="n">
-        <v>346.0400085449219</v>
+        <v>346.0199890136719</v>
       </c>
       <c r="U30" s="72" t="n">
         <v>347.2598876953125</v>
@@ -7630,10 +7630,10 @@
         <v>337.9150085449219</v>
       </c>
       <c r="W30" s="73" t="n">
-        <v>23179868</v>
+        <v>23370886</v>
       </c>
       <c r="X30" s="74" t="n">
-        <v>0.8894886418100324</v>
+        <v>0.8964900744454805</v>
       </c>
       <c r="Y30" s="28" t="n">
         <v>32.26759683478718</v>
@@ -7712,17 +7712,17 @@
       </c>
       <c r="AX30" s="79" t="inlineStr">
         <is>
+          <t>Why Rule Breakers Dig Stocks With Multiple Futures</t>
+        </is>
+      </c>
+      <c r="AY30" s="79" t="inlineStr">
+        <is>
           <t>Broadcom CEO Doubles Down on Massive AI Growth Target</t>
         </is>
       </c>
-      <c r="AY30" s="79" t="inlineStr">
+      <c r="AZ30" s="79" t="inlineStr">
         <is>
           <t>Broadcom (AVGO) Could Be 47% Below Fair Value On Buybacks And Revenue Guidance</t>
-        </is>
-      </c>
-      <c r="AZ30" s="79" t="inlineStr">
-        <is>
-          <t>Broadcom Slips Again as AI Approaches 62% of Quarterly Sales</t>
         </is>
       </c>
     </row>
@@ -7818,10 +7818,10 @@
         <v>91.02999877929688</v>
       </c>
       <c r="W31" s="84" t="n">
-        <v>2228679</v>
+        <v>2253991</v>
       </c>
       <c r="X31" s="85" t="n">
-        <v>0.8348772889828893</v>
+        <v>0.8439592021603196</v>
       </c>
       <c r="Y31" s="35" t="n">
         <v>37.9552633333654</v>
@@ -7900,17 +7900,17 @@
       </c>
       <c r="AX31" s="90" t="inlineStr">
         <is>
+          <t>Cameco vs. USA Rare Earth: Which Renewable Energy Stock Is a Better Buy in 2026?</t>
+        </is>
+      </c>
+      <c r="AY31" s="90" t="inlineStr">
+        <is>
+          <t>Jim Cramer Favors BWX Technologies (BWXT) Over Cameco (CCJ)</t>
+        </is>
+      </c>
+      <c r="AZ31" s="90" t="inlineStr">
+        <is>
           <t>Cameco Controls the Uranium Refinery That Puts Canada in the Driver's Seat</t>
-        </is>
-      </c>
-      <c r="AY31" s="90" t="inlineStr">
-        <is>
-          <t>Cameco (CCJ) Registers a Bigger Fall Than the Market: Important Facts to Note</t>
-        </is>
-      </c>
-      <c r="AZ31" s="90" t="inlineStr">
-        <is>
-          <t>Cameco vs. MP Materials: Which Crucial Renewable Energy Supplier Stock Is a Better Buy in 2026?</t>
         </is>
       </c>
     </row>
@@ -7997,7 +7997,7 @@
         <v>-2.060005187988281</v>
       </c>
       <c r="T32" s="72" t="n">
-        <v>82.62000274658203</v>
+        <v>82.38999938964844</v>
       </c>
       <c r="U32" s="72" t="n">
         <v>83.86000061035156</v>
@@ -8006,10 +8006,10 @@
         <v>80.51999664306641</v>
       </c>
       <c r="W32" s="73" t="n">
-        <v>15519291</v>
+        <v>15555201</v>
       </c>
       <c r="X32" s="74" t="n">
-        <v>0.7140043404107623</v>
+        <v>0.7155973580155705</v>
       </c>
       <c r="Y32" s="28" t="n">
         <v>42.81522285543067</v>
@@ -8122,7 +8122,7 @@
       </c>
       <c r="F33" s="30" t="inlineStr">
         <is>
-          <t>Same</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G33" s="30" t="inlineStr">
@@ -8194,10 +8194,10 @@
         <v>539</v>
       </c>
       <c r="W33" s="84" t="n">
-        <v>9238523</v>
+        <v>9584257</v>
       </c>
       <c r="X33" s="85" t="n">
-        <v>0.9945733099765736</v>
+        <v>1.029876707646598</v>
       </c>
       <c r="Y33" s="35" t="n">
         <v>60.57000111295811</v>
@@ -8373,7 +8373,7 @@
         <v>-4.279998779296875</v>
       </c>
       <c r="T34" s="72" t="n">
-        <v>343.3399963378906</v>
+        <v>343.1549987792969</v>
       </c>
       <c r="U34" s="72" t="n">
         <v>344.3599853515625</v>
@@ -8382,10 +8382,10 @@
         <v>339.1799926757812</v>
       </c>
       <c r="W34" s="73" t="n">
-        <v>12397214</v>
+        <v>12407733</v>
       </c>
       <c r="X34" s="74" t="n">
-        <v>0.7790353095225032</v>
+        <v>0.7796705502453861</v>
       </c>
       <c r="Y34" s="28" t="n">
         <v>51.06975329421959</v>
@@ -8570,10 +8570,10 @@
         <v>40.97000122070312</v>
       </c>
       <c r="W35" s="84" t="n">
-        <v>27923189</v>
+        <v>28474918</v>
       </c>
       <c r="X35" s="85" t="n">
-        <v>0.6716771143847666</v>
+        <v>0.6844944404095682</v>
       </c>
       <c r="Y35" s="35" t="n">
         <v>49.40387539153045</v>
@@ -8749,7 +8749,7 @@
         <v>-0.0500030517578125</v>
       </c>
       <c r="T36" s="72" t="n">
-        <v>98.83000183105469</v>
+        <v>98.83999633789062</v>
       </c>
       <c r="U36" s="72" t="n">
         <v>100.4800033569336</v>
@@ -8758,10 +8758,10 @@
         <v>96.52050018310547</v>
       </c>
       <c r="W36" s="73" t="n">
-        <v>79153928</v>
+        <v>83570756</v>
       </c>
       <c r="X36" s="74" t="n">
-        <v>0.8670882319680225</v>
+        <v>0.9132628174779696</v>
       </c>
       <c r="Y36" s="28" t="n">
         <v>50.27464804382544</v>
@@ -8937,7 +8937,7 @@
         <v>-8.290008544921875</v>
       </c>
       <c r="T37" s="83" t="n">
-        <v>500.0599975585938</v>
+        <v>500.0020141601562</v>
       </c>
       <c r="U37" s="83" t="n">
         <v>505.8999938964844</v>
@@ -8946,10 +8946,10 @@
         <v>495.5400085449219</v>
       </c>
       <c r="W37" s="84" t="n">
-        <v>17364843</v>
+        <v>17700788</v>
       </c>
       <c r="X37" s="85" t="n">
-        <v>0.8458618239995616</v>
+        <v>0.8615211896499759</v>
       </c>
       <c r="Y37" s="35" t="n">
         <v>55.85050839719622</v>
@@ -9028,17 +9028,17 @@
       </c>
       <c r="AX37" s="90" t="inlineStr">
         <is>
-          <t>Magnificent Seven Stocks Eye Breakout After Sideways 2026</t>
+          <t>Microsoft announces quarterly dividend increase</t>
         </is>
       </c>
       <c r="AY37" s="90" t="inlineStr">
         <is>
-          <t>Sunrise Technologies Achieves the 2026-2027 Microsoft AI Business Solutions Inner Circle Award</t>
+          <t>Microsoft Pays Out More in Dividends Than It Spends Buying Back Stock. Here's What That Does for Investors.</t>
         </is>
       </c>
       <c r="AZ37" s="90" t="inlineStr">
         <is>
-          <t>ORCL vs. MSFT: Which Stock Should Value Investors Buy Now?</t>
+          <t>Microsoft At Key Level After Earnings Surge; Is Microsoft A Buy Now?</t>
         </is>
       </c>
     </row>
@@ -9125,7 +9125,7 @@
         <v>-7.339996337890625</v>
       </c>
       <c r="T38" s="72" t="n">
-        <v>131.6799926757812</v>
+        <v>131.6499938964844</v>
       </c>
       <c r="U38" s="72" t="n">
         <v>133.9998931884766</v>
@@ -9134,10 +9134,10 @@
         <v>125.4400024414062</v>
       </c>
       <c r="W38" s="73" t="n">
-        <v>22578278</v>
+        <v>22689051</v>
       </c>
       <c r="X38" s="74" t="n">
-        <v>0.7897948097561538</v>
+        <v>0.7935159432580614</v>
       </c>
       <c r="Y38" s="28" t="n">
         <v>54.74082353591855</v>
@@ -9216,17 +9216,17 @@
       </c>
       <c r="AX38" s="79" t="inlineStr">
         <is>
+          <t>The Price of Bitcoin May Be Soaring, But a New Risk Has Emerged for Strategy. Here's What MSTR Investors Ne...</t>
+        </is>
+      </c>
+      <c r="AY38" s="79" t="inlineStr">
+        <is>
           <t>Morning Minute: Clarity Act Odds Slump After Democrat Pushback</t>
         </is>
       </c>
-      <c r="AY38" s="79" t="inlineStr">
+      <c r="AZ38" s="79" t="inlineStr">
         <is>
           <t>Coinbase Drops 6%, Strategy Slides 5%, MARA Holdings Slips 1% as Clarity Act Anxiety Builds</t>
-        </is>
-      </c>
-      <c r="AZ38" s="79" t="inlineStr">
-        <is>
-          <t>Crypto Stocks MSTR, COIN, CRCL, HOOD Tumble 3-5% Ahead of CLARITY Act Senate Vote</t>
         </is>
       </c>
     </row>
@@ -9313,7 +9313,7 @@
         <v>3.5699462890625</v>
       </c>
       <c r="T39" s="83" t="n">
-        <v>937.5</v>
+        <v>937.8079833984375</v>
       </c>
       <c r="U39" s="83" t="n">
         <v>944.8900146484375</v>
@@ -9322,10 +9322,10 @@
         <v>920.1300048828125</v>
       </c>
       <c r="W39" s="84" t="n">
-        <v>20260215</v>
+        <v>20305657</v>
       </c>
       <c r="X39" s="85" t="n">
-        <v>0.797870990887266</v>
+        <v>0.7995890044668565</v>
       </c>
       <c r="Y39" s="35" t="n">
         <v>46.90861914833569</v>
@@ -9404,17 +9404,17 @@
       </c>
       <c r="AX39" s="90" t="inlineStr">
         <is>
+          <t>Micron Technology (MU), What Is Behind The Fresh Attention?</t>
+        </is>
+      </c>
+      <c r="AY39" s="90" t="inlineStr">
+        <is>
+          <t>Micron Investors Get New Reason to Watch Closely</t>
+        </is>
+      </c>
+      <c r="AZ39" s="90" t="inlineStr">
+        <is>
           <t>Micron's AI boom just ran into an unexpected labor problem</t>
-        </is>
-      </c>
-      <c r="AY39" s="90" t="inlineStr">
-        <is>
-          <t>Micron Appoints Deirdre Hanford to Lead Micron Research Labs</t>
-        </is>
-      </c>
-      <c r="AZ39" s="90" t="inlineStr">
-        <is>
-          <t>Nvidia vs. Micron: Which Is the Better Artificial Intelligence (AI) Semiconductor Stock to Own for the Next...</t>
         </is>
       </c>
     </row>
@@ -9501,7 +9501,7 @@
         <v>-4.82000732421875</v>
       </c>
       <c r="T40" s="72" t="n">
-        <v>211.0299987792969</v>
+        <v>211.1699981689453</v>
       </c>
       <c r="U40" s="72" t="n">
         <v>216.5594940185547</v>
@@ -9510,10 +9510,10 @@
         <v>206.8473052978516</v>
       </c>
       <c r="W40" s="73" t="n">
-        <v>10309780</v>
+        <v>10407318</v>
       </c>
       <c r="X40" s="74" t="n">
-        <v>0.6127604651587129</v>
+        <v>0.6183783819241668</v>
       </c>
       <c r="Y40" s="28" t="n">
         <v>45.66170890066309</v>
@@ -9689,7 +9689,7 @@
         <v>-2.419998168945312</v>
       </c>
       <c r="T41" s="83" t="n">
-        <v>79.375</v>
+        <v>79.31999969482422</v>
       </c>
       <c r="U41" s="83" t="n">
         <v>79.48079681396484</v>
@@ -9698,10 +9698,10 @@
         <v>77.45999908447266</v>
       </c>
       <c r="W41" s="84" t="n">
-        <v>27471174</v>
+        <v>27529569</v>
       </c>
       <c r="X41" s="85" t="n">
-        <v>1.010484767828535</v>
+        <v>1.012523994284178</v>
       </c>
       <c r="Y41" s="35" t="n">
         <v>49.24669293517496</v>
@@ -9780,17 +9780,17 @@
       </c>
       <c r="AX41" s="90" t="inlineStr">
         <is>
+          <t>Netflix (NFLX) Suffers a Larger Drop Than the General Market: Key Insights</t>
+        </is>
+      </c>
+      <c r="AY41" s="90" t="inlineStr">
+        <is>
           <t>22 Prominent Investors Hold Netflix Stock, With 14 Increasing Their Stakes Recently -- Including Bill Ackma...</t>
         </is>
       </c>
-      <c r="AY41" s="90" t="inlineStr">
+      <c r="AZ41" s="90" t="inlineStr">
         <is>
           <t>Why Netflix Stock Rallied Today</t>
-        </is>
-      </c>
-      <c r="AZ41" s="90" t="inlineStr">
-        <is>
-          <t>Netflix stock jumps as Wall Street sees a new growth engine</t>
         </is>
       </c>
     </row>
@@ -9886,10 +9886,10 @@
         <v>9.800100326538086</v>
       </c>
       <c r="W42" s="73" t="n">
-        <v>83456584</v>
+        <v>83579001</v>
       </c>
       <c r="X42" s="74" t="n">
-        <v>1.165017866250927</v>
+        <v>1.166627072920558</v>
       </c>
       <c r="Y42" s="28" t="n">
         <v>45.12036315526083</v>
@@ -10065,7 +10065,7 @@
         <v>1.209991455078125</v>
       </c>
       <c r="T43" s="83" t="n">
-        <v>213.375</v>
+        <v>213.0899963378906</v>
       </c>
       <c r="U43" s="83" t="n">
         <v>213.9400024414062</v>
@@ -10074,10 +10074,10 @@
         <v>211.1600036621094</v>
       </c>
       <c r="W43" s="84" t="n">
-        <v>86373669</v>
+        <v>85131691</v>
       </c>
       <c r="X43" s="85" t="n">
-        <v>0.6634783626168946</v>
+        <v>0.6542502078404915</v>
       </c>
       <c r="Y43" s="35" t="n">
         <v>45.06651576393133</v>
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
-          <t>Magnificent Seven Stocks Eye Breakout After Sideways 2026</t>
+          <t>Pinterest, Nvidia Partner To Boost AI Shopping, Search Offerings</t>
         </is>
       </c>
       <c r="AY43" s="90" t="inlineStr">
         <is>
-          <t>3 Resilient Artificial Intelligence (AI) Stocks That Did Well the Last Time the Fed Raised Interest Rates</t>
+          <t>Nvidia (NVDA) Is Discussing Up To $10 Billion For An AI IPO</t>
         </is>
       </c>
       <c r="AZ43" s="90" t="inlineStr">
         <is>
-          <t>Imagine You Invested $10,000 in Nvidia 10 Years Ago. Here's What Your Stake Would Be Worth Today.</t>
+          <t>Nvidia May Have Won the AI Training Race, but the Bigger Opportunity Is Likely Still Ahead</t>
         </is>
       </c>
     </row>
@@ -10253,7 +10253,7 @@
         <v>-0.75</v>
       </c>
       <c r="T44" s="72" t="n">
-        <v>170.5</v>
+        <v>170.2350006103516</v>
       </c>
       <c r="U44" s="72" t="n">
         <v>176.5899963378906</v>
@@ -10262,10 +10262,10 @@
         <v>169.4499969482422</v>
       </c>
       <c r="W44" s="73" t="n">
-        <v>31070295</v>
+        <v>31164073</v>
       </c>
       <c r="X44" s="74" t="n">
-        <v>1.06394116998808</v>
+        <v>1.066981096444209</v>
       </c>
       <c r="Y44" s="28" t="n">
         <v>53.08228958642693</v>
@@ -10344,17 +10344,17 @@
       </c>
       <c r="AX44" s="79" t="inlineStr">
         <is>
+          <t>Can Palantir Technologies (PLTR) Justify Its Price On Cash Flow?</t>
+        </is>
+      </c>
+      <c r="AY44" s="79" t="inlineStr">
+        <is>
           <t>Palantir Looks Cheap Among AI Software Stocks, UBS Says — Why PLTR Could Have More Room To Run</t>
         </is>
       </c>
-      <c r="AY44" s="79" t="inlineStr">
+      <c r="AZ44" s="79" t="inlineStr">
         <is>
           <t>Palantir wins higher UBS target as customer demand outpaces capacity</t>
-        </is>
-      </c>
-      <c r="AZ44" s="79" t="inlineStr">
-        <is>
-          <t>Palantir Sees Strong AI Demand, Wider Enterprise Use Cases, UBS Says</t>
         </is>
       </c>
     </row>
@@ -10441,7 +10441,7 @@
         <v>7.650009155273438</v>
       </c>
       <c r="T45" s="83" t="n">
-        <v>180.5350036621094</v>
+        <v>181.0800018310547</v>
       </c>
       <c r="U45" s="83" t="n">
         <v>190.0599975585938</v>
@@ -10450,10 +10450,10 @@
         <v>180.9949951171875</v>
       </c>
       <c r="W45" s="84" t="n">
-        <v>13624241</v>
+        <v>13701105</v>
       </c>
       <c r="X45" s="85" t="n">
-        <v>1.176542497845436</v>
+        <v>1.18278765789832</v>
       </c>
       <c r="Y45" s="35" t="n">
         <v>69.49348609970977</v>
@@ -10638,10 +10638,10 @@
         <v>62.02000045776367</v>
       </c>
       <c r="W46" s="73" t="n">
-        <v>20214615</v>
+        <v>20269701</v>
       </c>
       <c r="X46" s="74" t="n">
-        <v>1.218027762794834</v>
+        <v>1.221144298307168</v>
       </c>
       <c r="Y46" s="28" t="n">
         <v>39.79143610199673</v>
@@ -10720,17 +10720,17 @@
       </c>
       <c r="AX46" s="79" t="inlineStr">
         <is>
+          <t>Rocket Lab Corporation (RKLB) Advances While Market Declines: Some Information for Investors</t>
+        </is>
+      </c>
+      <c r="AY46" s="79" t="inlineStr">
+        <is>
+          <t>Rocket Lab Makes Bold Move to Broaden Space Business</t>
+        </is>
+      </c>
+      <c r="AZ46" s="79" t="inlineStr">
+        <is>
           <t>Rocket Lab Raises Funds To Prepare For Closing Of Iridium Acquisition</t>
-        </is>
-      </c>
-      <c r="AY46" s="79" t="inlineStr">
-        <is>
-          <t>Rocket Lab Stock Jumps After $1.94 Billion Financing for Iridium Deal</t>
-        </is>
-      </c>
-      <c r="AZ46" s="79" t="inlineStr">
-        <is>
-          <t>Boeing vs. Rocket Lab: Which Aerospace Stock Is a Better Buy in 2026?</t>
         </is>
       </c>
     </row>
@@ -10826,10 +10826,10 @@
         <v>1509.14013671875</v>
       </c>
       <c r="W47" s="84" t="n">
-        <v>6817861</v>
+        <v>6830792</v>
       </c>
       <c r="X47" s="85" t="n">
-        <v>0.5991675961694692</v>
+        <v>0.6002698915296589</v>
       </c>
       <c r="Y47" s="35" t="n">
         <v>47.66082157617929</v>
@@ -11005,7 +11005,7 @@
         <v>-2.3900146484375</v>
       </c>
       <c r="T48" s="72" t="n">
-        <v>358.75</v>
+        <v>358.7250061035156</v>
       </c>
       <c r="U48" s="72" t="n">
         <v>362.3900146484375</v>
@@ -11014,10 +11014,10 @@
         <v>354.0499877929688</v>
       </c>
       <c r="W48" s="73" t="n">
-        <v>30163254</v>
+        <v>30215079</v>
       </c>
       <c r="X48" s="74" t="n">
-        <v>0.7714289017860761</v>
+        <v>0.7727031242630257</v>
       </c>
       <c r="Y48" s="28" t="n">
         <v>50.41800696093863</v>
@@ -11096,17 +11096,17 @@
       </c>
       <c r="AX48" s="79" t="inlineStr">
         <is>
-          <t>Magnificent Seven Stocks Eye Breakout After Sideways 2026</t>
+          <t>Where Tesla's Robotaxi Rollout Stands Today and What Investors Should Know</t>
         </is>
       </c>
       <c r="AY48" s="79" t="inlineStr">
         <is>
-          <t>Tesla Launches the Cybercab: 2 Key Takeaways for Investors</t>
+          <t>TSLA Edges Lower After Regulator Asks If Wheel-Less Cybercab Can Be Driven By A Human</t>
         </is>
       </c>
       <c r="AZ48" s="79" t="inlineStr">
         <is>
-          <t>Nine Years Later: Can Tesla Finally Deliver on Its $250,000 Roadster Promise?</t>
+          <t>The Tesla Roadster Will ‘Blow People’s Minds’</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 15 Sep 2026, 08:21 PM · Yahoo Finance data</t>
+          <t>Built 15 Sep 2026, 10:55 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 15 Sep 2026, 08:21 PM · Yahoo Finance data</t>
+          <t>Built 15 Sep 2026, 10:55 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 15 Sep 2026, 08:21 PM · Yahoo Finance data</t>
+          <t>Built 15 Sep 2026, 10:55 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 15 Sep 2026, 08:21 PM · Yahoo Finance data</t>
+          <t>Built 15 Sep 2026, 10:55 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -43996,7 +43996,7 @@
       </c>
       <c r="D8" s="106" t="inlineStr">
         <is>
-          <t>Gapped up 1.7% at the open</t>
+          <t>Gapped up 1.6% at the open</t>
         </is>
       </c>
       <c r="E8" s="26" t="n">
@@ -44080,7 +44080,7 @@
       </c>
       <c r="D11" s="105" t="inlineStr">
         <is>
-          <t>Gapped down 1.6% at the open</t>
+          <t>Gapped down 1.8% at the open</t>
         </is>
       </c>
       <c r="E11" s="33" t="n">
@@ -44192,7 +44192,7 @@
       </c>
       <c r="D15" s="105" t="inlineStr">
         <is>
-          <t>Gapped down 3.8% at the open</t>
+          <t>Gapped down 3.9% at the open</t>
         </is>
       </c>
       <c r="E15" s="33" t="n">
@@ -44700,7 +44700,7 @@
         </is>
       </c>
       <c r="E33" s="33" t="n">
-        <v>-0.00452108403339635</v>
+        <v>-0.004586781374170235</v>
       </c>
       <c r="F33" s="34" t="n">
         <v>2</v>
@@ -44728,7 +44728,7 @@
         </is>
       </c>
       <c r="E34" s="26" t="n">
-        <v>-0.00452108403339635</v>
+        <v>-0.004586781374170235</v>
       </c>
       <c r="F34" s="27" t="n">
         <v>2</v>
@@ -44868,7 +44868,7 @@
         </is>
       </c>
       <c r="E39" s="33" t="n">
-        <v>-0.009586362858249764</v>
+        <v>-0.009621023856200339</v>
       </c>
       <c r="F39" s="34" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
Daily workbook: 2026-09-15 23:31 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 15 Sep 2026, 10:55 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 15 Sep 2026, 11:31 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 15 Sep 2026, 10:55 PM · Yahoo Finance data</t>
+          <t>Built 15 Sep 2026, 11:31 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -8276,17 +8276,17 @@
       </c>
       <c r="AX33" s="90" t="inlineStr">
         <is>
+          <t>What Could Dell Technologies (DELL) Europa AI Push Mean For Enterprise Infrastructure?</t>
+        </is>
+      </c>
+      <c r="AY33" s="90" t="inlineStr">
+        <is>
           <t>Dell Technologies (DELL) Rallies on Bullish RBC Outlook: Is the Stock a Buy?</t>
         </is>
       </c>
-      <c r="AY33" s="90" t="inlineStr">
+      <c r="AZ33" s="90" t="inlineStr">
         <is>
           <t>Dell Jumps 5.8% as Europe's AI Chip Challenger Enters Its Servers</t>
-        </is>
-      </c>
-      <c r="AZ33" s="90" t="inlineStr">
-        <is>
-          <t>Hewlett Packard Enterprise Rises 4% a Day After Evercore ISI Downgrade; Dell Climbs 4%, Super Micro Holds S...</t>
         </is>
       </c>
     </row>
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
+          <t>Calls for Slower AI Development Have Created a Compelling Dip for AI Stocks</t>
+        </is>
+      </c>
+      <c r="AY43" s="90" t="inlineStr">
+        <is>
           <t>Pinterest, Nvidia Partner To Boost AI Shopping, Search Offerings</t>
         </is>
       </c>
-      <c r="AY43" s="90" t="inlineStr">
+      <c r="AZ43" s="90" t="inlineStr">
         <is>
           <t>Nvidia (NVDA) Is Discussing Up To $10 Billion For An AI IPO</t>
-        </is>
-      </c>
-      <c r="AZ43" s="90" t="inlineStr">
-        <is>
-          <t>Nvidia May Have Won the AI Training Race, but the Bigger Opportunity Is Likely Still Ahead</t>
         </is>
       </c>
     </row>
@@ -10908,17 +10908,17 @@
       </c>
       <c r="AX47" s="90" t="inlineStr">
         <is>
+          <t>Sandisk (SNDK) Refinances Credit Line As Valuation Debate Sharpens</t>
+        </is>
+      </c>
+      <c r="AY47" s="90" t="inlineStr">
+        <is>
           <t>Western Digital Falls 4% Despite Its AI Storage Pitch; Seagate Drops 5%, Micron Holds Steady</t>
         </is>
       </c>
-      <c r="AY47" s="90" t="inlineStr">
+      <c r="AZ47" s="90" t="inlineStr">
         <is>
           <t>Sandisk $1,500 Stock Price Ignites Fresh Split Frenzy</t>
-        </is>
-      </c>
-      <c r="AZ47" s="90" t="inlineStr">
-        <is>
-          <t>SNDK Stock Rewarded Dip Buyers Before, But Is It Still The Same Company?</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 15 Sep 2026, 10:55 PM · Yahoo Finance data</t>
+          <t>Built 15 Sep 2026, 11:31 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 15 Sep 2026, 10:55 PM · Yahoo Finance data</t>
+          <t>Built 15 Sep 2026, 11:31 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 15 Sep 2026, 10:55 PM · Yahoo Finance data</t>
+          <t>Built 15 Sep 2026, 11:31 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 15 Sep 2026, 10:55 PM · Yahoo Finance data</t>
+          <t>Built 15 Sep 2026, 11:31 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-09-16 23:38 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1299,7 +1299,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 16 Sep 2026, 10:59 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 16 Sep 2026, 11:38 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3104,7 +3104,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 16 Sep 2026, 10:59 PM · Yahoo Finance data</t>
+          <t>Built 16 Sep 2026, 11:38 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -6957,17 +6957,17 @@
       </c>
       <c r="AX26" s="79" t="inlineStr">
         <is>
+          <t>The Next Short? Economist Compares Hyperscaler AI Debt Stress to 2008 Housing Collapse</t>
+        </is>
+      </c>
+      <c r="AY26" s="79" t="inlineStr">
+        <is>
           <t>Generac Stock Soars on Amazon Generator Deal</t>
         </is>
       </c>
-      <c r="AY26" s="79" t="inlineStr">
+      <c r="AZ26" s="79" t="inlineStr">
         <is>
           <t>The E-Commerce Stocks to Buy Before the Holiday Quarter</t>
-        </is>
-      </c>
-      <c r="AZ26" s="79" t="inlineStr">
-        <is>
-          <t>Generac stock surges 18% on $8B Amazon supply deal</t>
         </is>
       </c>
     </row>
@@ -8461,17 +8461,17 @@
       </c>
       <c r="AX34" s="79" t="inlineStr">
         <is>
+          <t>Waymo Expands Robotaxi Battle to Las Vegas — Alphabet-Backed Service Plans Unsupervised Tokyo Launch in 202...</t>
+        </is>
+      </c>
+      <c r="AY34" s="79" t="inlineStr">
+        <is>
           <t>Anthropic IPO Underwriter Says AI Spending Won't Slow: Can He Be Neutral?</t>
         </is>
       </c>
-      <c r="AY34" s="79" t="inlineStr">
+      <c r="AZ34" s="79" t="inlineStr">
         <is>
           <t>GOOGL, BX Stock In Focus — Banking Consortium Reportedly Lines Up $22B AI Chip Financing For Blackstone-Alp...</t>
-        </is>
-      </c>
-      <c r="AZ34" s="79" t="inlineStr">
-        <is>
-          <t>Greg Abel Grew Berkshire Hathaway's Alphabet Stake by 83% Last Quarter, One of His Boldest Equity Bets Yet ...</t>
         </is>
       </c>
     </row>
@@ -11640,7 +11640,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 16 Sep 2026, 10:59 PM · Yahoo Finance data</t>
+          <t>Built 16 Sep 2026, 11:38 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19576,7 +19576,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 16 Sep 2026, 10:59 PM · Yahoo Finance data</t>
+          <t>Built 16 Sep 2026, 11:38 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27512,7 +27512,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 16 Sep 2026, 10:59 PM · Yahoo Finance data</t>
+          <t>Built 16 Sep 2026, 11:38 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35448,7 +35448,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 16 Sep 2026, 10:59 PM · Yahoo Finance data</t>
+          <t>Built 16 Sep 2026, 11:38 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-09-17 22:52 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1299,7 +1299,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 17 Sep 2026, 08:28 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 17 Sep 2026, 10:52 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -1387,7 +1387,7 @@
       <c r="J8" s="6" t="n"/>
       <c r="K8" s="15" t="inlineStr">
         <is>
-          <t>5.3</t>
+          <t>5.4</t>
         </is>
       </c>
       <c r="L8" s="10" t="n"/>
@@ -1610,31 +1610,31 @@
       </c>
       <c r="C17" s="31" t="inlineStr">
         <is>
-          <t>XLB</t>
+          <t>XLE</t>
         </is>
       </c>
       <c r="D17" s="32" t="inlineStr">
         <is>
-          <t>State Street Materials Select Sector SPDR ETF</t>
+          <t>State Street Energy Select Sector SPDR ETF</t>
         </is>
       </c>
       <c r="E17" s="33" t="n">
-        <v>0.006949929902287488</v>
+        <v>0.007028027271839044</v>
       </c>
       <c r="F17" s="34" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G17" s="35" t="n">
-        <v>40.17082520459962</v>
+        <v>56.62949827527311</v>
       </c>
       <c r="H17" s="36" t="n">
-        <v>-2.0550870727015</v>
+        <v>5.727802201530707</v>
       </c>
       <c r="I17" s="33" t="n">
-        <v>-0.00098501258301531</v>
+        <v>-0.006930493548855221</v>
       </c>
       <c r="J17" s="33" t="n">
-        <v>-0.0206643437630214</v>
+        <v>0.01256286193347878</v>
       </c>
     </row>
     <row r="18">
@@ -1643,31 +1643,31 @@
       </c>
       <c r="C18" s="24" t="inlineStr">
         <is>
-          <t>XLE</t>
+          <t>XLB</t>
         </is>
       </c>
       <c r="D18" s="25" t="inlineStr">
         <is>
-          <t>State Street Energy Select Sector SPDR ETF</t>
+          <t>State Street Materials Select Sector SPDR ETF</t>
         </is>
       </c>
       <c r="E18" s="26" t="n">
-        <v>0.006871817113770051</v>
+        <v>0.006949929902287488</v>
       </c>
       <c r="F18" s="27" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G18" s="28" t="n">
-        <v>56.58505618877323</v>
+        <v>40.17082520459962</v>
       </c>
       <c r="H18" s="29" t="n">
-        <v>5.711748452922993</v>
+        <v>-2.0550870727015</v>
       </c>
       <c r="I18" s="26" t="n">
-        <v>-0.007084538461583634</v>
+        <v>-0.00098501258301531</v>
       </c>
       <c r="J18" s="26" t="n">
-        <v>0.0124057932120194</v>
+        <v>-0.0206643437630214</v>
       </c>
     </row>
     <row r="19">
@@ -2702,7 +2702,7 @@
         </is>
       </c>
       <c r="I50" s="33" t="n">
-        <v>0.00514226326440248</v>
+        <v>0.005318326206797064</v>
       </c>
       <c r="J50" s="34" t="n">
         <v>2</v>
@@ -2713,7 +2713,7 @@
         </is>
       </c>
       <c r="L50" s="35" t="n">
-        <v>35.97682353421516</v>
+        <v>36.08911153912589</v>
       </c>
     </row>
     <row r="51">
@@ -2778,22 +2778,22 @@
       </c>
       <c r="H52" s="31" t="inlineStr">
         <is>
-          <t>XLE</t>
+          <t>XLB</t>
         </is>
       </c>
       <c r="I52" s="33" t="n">
-        <v>0.006871817113770051</v>
+        <v>0.006949929902287488</v>
       </c>
       <c r="J52" s="34" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="K52" s="30" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="L52" s="35" t="n">
-        <v>56.58505618877323</v>
+        <v>40.17082520459962</v>
       </c>
     </row>
   </sheetData>
@@ -3104,7 +3104,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 17 Sep 2026, 08:28 PM · Yahoo Finance data</t>
+          <t>Built 17 Sep 2026, 10:52 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -3139,7 +3139,7 @@
       </c>
       <c r="AC3" s="46" t="inlineStr">
         <is>
-          <t>5.3 / 9</t>
+          <t>5.4 / 9</t>
         </is>
       </c>
       <c r="AE3" s="47" t="inlineStr">
@@ -3617,10 +3617,10 @@
         <v>168.6600036621094</v>
       </c>
       <c r="W7" s="73" t="n">
-        <v>5785044</v>
+        <v>5840674</v>
       </c>
       <c r="X7" s="74" t="n">
-        <v>0.8028163220739698</v>
+        <v>0.8102235977109219</v>
       </c>
       <c r="Y7" s="28" t="n">
         <v>31.46829525388786</v>
@@ -3807,10 +3807,10 @@
         <v>167.7700042724609</v>
       </c>
       <c r="W8" s="84" t="n">
-        <v>5336683</v>
+        <v>5347489</v>
       </c>
       <c r="X8" s="85" t="n">
-        <v>0.7277656418341811</v>
+        <v>0.7291855334010648</v>
       </c>
       <c r="Y8" s="35" t="n">
         <v>51.05041102212405</v>
@@ -3997,10 +3997,10 @@
         <v>55.56000137329102</v>
       </c>
       <c r="W9" s="73" t="n">
-        <v>28273546</v>
+        <v>28849911</v>
       </c>
       <c r="X9" s="74" t="n">
-        <v>0.9302668271113718</v>
+        <v>0.9483314074668173</v>
       </c>
       <c r="Y9" s="28" t="n">
         <v>37.08635589509742</v>
@@ -4103,10 +4103,10 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>0.006871817113770051</v>
+        <v>0.007028027271839044</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E10" s="30" t="inlineStr">
         <is>
@@ -4172,10 +4172,10 @@
         </is>
       </c>
       <c r="R10" s="81" t="n">
-        <v>64.47000122070312</v>
+        <v>64.48000335693359</v>
       </c>
       <c r="S10" s="82" t="n">
-        <v>0.44000244140625</v>
+        <v>0.4500045776367188</v>
       </c>
       <c r="T10" s="83" t="n">
         <v>63.5</v>
@@ -4187,61 +4187,61 @@
         <v>63.45999908447266</v>
       </c>
       <c r="W10" s="84" t="n">
-        <v>33933579</v>
+        <v>34003831</v>
       </c>
       <c r="X10" s="85" t="n">
-        <v>1.129409037776444</v>
+        <v>1.131614933704711</v>
       </c>
       <c r="Y10" s="35" t="n">
-        <v>56.58505618877323</v>
+        <v>56.62949827527311</v>
       </c>
       <c r="Z10" s="35" t="n">
-        <v>58.02475880276882</v>
+        <v>58.2717251759706</v>
       </c>
       <c r="AA10" s="35" t="n">
         <v>22.6930018858906</v>
       </c>
       <c r="AB10" s="86" t="n">
-        <v>1.114020572176585</v>
+        <v>1.114818463385852</v>
       </c>
       <c r="AC10" s="86" t="n">
-        <v>1.3038987540682</v>
+        <v>1.304058332310053</v>
       </c>
       <c r="AD10" s="86" t="n">
-        <v>-0.1898781818916147</v>
+        <v>-0.1892398689242012</v>
       </c>
       <c r="AE10" s="83" t="n">
-        <v>64.66033111502684</v>
+        <v>64.66255381196694</v>
       </c>
       <c r="AF10" s="83" t="n">
-        <v>63.78585116616682</v>
+        <v>63.78676045127868</v>
       </c>
       <c r="AG10" s="83" t="n">
-        <v>60.98660003662109</v>
+        <v>60.98680007934571</v>
       </c>
       <c r="AH10" s="83" t="n">
-        <v>58.91570003509521</v>
+        <v>58.91580005645752</v>
       </c>
       <c r="AI10" s="83" t="n">
-        <v>55.63457490921021</v>
+        <v>55.63462491989136</v>
       </c>
       <c r="AJ10" s="83" t="n">
-        <v>66.20728304726941</v>
+        <v>66.20815509951672</v>
       </c>
       <c r="AK10" s="83" t="n">
-        <v>64.07899951934814</v>
+        <v>64.07949962615967</v>
       </c>
       <c r="AL10" s="83" t="n">
-        <v>61.95071599142688</v>
+        <v>61.95084415280264</v>
       </c>
       <c r="AM10" s="87" t="n">
-        <v>0.5918584615783966</v>
+        <v>0.5940743431209875</v>
       </c>
       <c r="AN10" s="36" t="n">
-        <v>6.642686508482863</v>
+        <v>6.643795553260036</v>
       </c>
       <c r="AO10" s="88" t="n">
-        <v>2.055370726587314</v>
+        <v>2.05505189754046</v>
       </c>
       <c r="AP10" s="83" t="n">
         <v>66.16999816894531</v>
@@ -4250,22 +4250,22 @@
         <v>42.34999847412109</v>
       </c>
       <c r="AR10" s="36" t="n">
-        <v>-2.569135552795021</v>
+        <v>-2.554019735193014</v>
       </c>
       <c r="AS10" s="89" t="n">
-        <v>92.86315293861412</v>
+        <v>92.90514343550167</v>
       </c>
       <c r="AT10" s="33" t="n">
-        <v>-0.007084538461583634</v>
+        <v>-0.006930493548855221</v>
       </c>
       <c r="AU10" s="33" t="n">
-        <v>0.0124057932120194</v>
+        <v>0.01256286193347878</v>
       </c>
       <c r="AV10" s="33" t="n">
-        <v>0.1792574241812321</v>
+        <v>0.1794403789382373</v>
       </c>
       <c r="AW10" s="33" t="n">
-        <v>0.4419593500527028</v>
+        <v>0.4421830614469162</v>
       </c>
       <c r="AX10" s="90" t="inlineStr">
         <is>
@@ -4377,10 +4377,10 @@
         <v>83.00499725341797</v>
       </c>
       <c r="W11" s="73" t="n">
-        <v>7566089</v>
+        <v>7592533</v>
       </c>
       <c r="X11" s="74" t="n">
-        <v>0.7740304325318853</v>
+        <v>0.7766306714448535</v>
       </c>
       <c r="Y11" s="28" t="n">
         <v>42.86077646368995</v>
@@ -4567,10 +4567,10 @@
         <v>111.1725997924805</v>
       </c>
       <c r="W12" s="84" t="n">
-        <v>4350432</v>
+        <v>4378930</v>
       </c>
       <c r="X12" s="85" t="n">
-        <v>0.7474613835363083</v>
+        <v>0.752173569874718</v>
       </c>
       <c r="Y12" s="35" t="n">
         <v>38.99198318866176</v>
@@ -4757,10 +4757,10 @@
         <v>112.2099990844727</v>
       </c>
       <c r="W13" s="73" t="n">
-        <v>4247196</v>
+        <v>4247206</v>
       </c>
       <c r="X13" s="74" t="n">
-        <v>1.000086229026649</v>
+        <v>1.000088465978968</v>
       </c>
       <c r="Y13" s="28" t="n">
         <v>51.02913306530867</v>
@@ -4866,7 +4866,7 @@
         <v>0.006949929902287488</v>
       </c>
       <c r="D14" s="34" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E14" s="30" t="inlineStr">
         <is>
@@ -4947,10 +4947,10 @@
         <v>50.52000045776367</v>
       </c>
       <c r="W14" s="84" t="n">
-        <v>8916958</v>
+        <v>8946107</v>
       </c>
       <c r="X14" s="85" t="n">
-        <v>0.8020161289198295</v>
+        <v>0.804532407620723</v>
       </c>
       <c r="Y14" s="35" t="n">
         <v>40.17082520459962</v>
@@ -5137,10 +5137,10 @@
         <v>186.7299957275391</v>
       </c>
       <c r="W15" s="73" t="n">
-        <v>7382339</v>
+        <v>7382684</v>
       </c>
       <c r="X15" s="74" t="n">
-        <v>1.154830803273164</v>
+        <v>1.154881655777287</v>
       </c>
       <c r="Y15" s="28" t="n">
         <v>55.74220115860763</v>
@@ -5327,10 +5327,10 @@
         <v>42.84500122070312</v>
       </c>
       <c r="W16" s="84" t="n">
-        <v>4346693</v>
+        <v>4347175</v>
       </c>
       <c r="X16" s="85" t="n">
-        <v>0.8867409532799864</v>
+        <v>0.8868349228959492</v>
       </c>
       <c r="Y16" s="35" t="n">
         <v>34.74774022483162</v>
@@ -5517,10 +5517,10 @@
         <v>41.31999969482422</v>
       </c>
       <c r="W17" s="73" t="n">
-        <v>20462393</v>
+        <v>20468772</v>
       </c>
       <c r="X17" s="74" t="n">
-        <v>0.9761295238989158</v>
+        <v>0.9764189688019287</v>
       </c>
       <c r="Y17" s="28" t="n">
         <v>35.70541017702637</v>
@@ -5726,10 +5726,10 @@
         <v>759.9600219726562</v>
       </c>
       <c r="W19" s="73" t="n">
-        <v>45077681</v>
+        <v>49288087</v>
       </c>
       <c r="X19" s="74" t="n">
-        <v>1.138327173552452</v>
+        <v>1.238068939547282</v>
       </c>
       <c r="Y19" s="28" t="n">
         <v>49.97910149000068</v>
@@ -5881,11 +5881,11 @@
         </is>
       </c>
       <c r="N20" s="80" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="O20" s="30" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Very Strong</t>
         </is>
       </c>
       <c r="P20" s="32" t="inlineStr">
@@ -5914,10 +5914,10 @@
         <v>713.3200073242188</v>
       </c>
       <c r="W20" s="84" t="n">
-        <v>35340138</v>
+        <v>36358508</v>
       </c>
       <c r="X20" s="85" t="n">
-        <v>1.157464736217355</v>
+        <v>1.188835912311762</v>
       </c>
       <c r="Y20" s="35" t="n">
         <v>53.04527642962599</v>
@@ -5996,17 +5996,17 @@
       </c>
       <c r="AX20" s="90" t="inlineStr">
         <is>
+          <t>$500,000 Split Between VOO and QQQ Owns the Same Seven Stocks Twice, and Nobody Adds Up the Overlap</t>
+        </is>
+      </c>
+      <c r="AY20" s="90" t="inlineStr">
+        <is>
           <t>If QQQ Repeats Its Last Decade, $100,000 at 40 Could Hit $1 Million by 52</t>
         </is>
       </c>
-      <c r="AY20" s="90" t="inlineStr">
+      <c r="AZ20" s="90" t="inlineStr">
         <is>
           <t>Exchange-Traded Funds Higher as US Equities Advance After Midday</t>
-        </is>
-      </c>
-      <c r="AZ20" s="90" t="inlineStr">
-        <is>
-          <t>Exchange-Traded Funds, Equity Futures Higher Pre-Bell Thursday Amid Economic Data, Fed Rate Hike</t>
         </is>
       </c>
     </row>
@@ -6018,7 +6018,7 @@
         </is>
       </c>
       <c r="C21" s="26" t="n">
-        <v>0.00514226326440248</v>
+        <v>0.005318326206797064</v>
       </c>
       <c r="D21" s="27" t="n">
         <v>4</v>
@@ -6087,10 +6087,10 @@
         </is>
       </c>
       <c r="R21" s="70" t="n">
-        <v>285.3800048828125</v>
+        <v>285.4299926757812</v>
       </c>
       <c r="S21" s="71" t="n">
-        <v>1.459991455078125</v>
+        <v>1.509979248046875</v>
       </c>
       <c r="T21" s="72" t="n">
         <v>287.9500122070312</v>
@@ -6102,61 +6102,61 @@
         <v>285.2799987792969</v>
       </c>
       <c r="W21" s="73" t="n">
-        <v>21694200</v>
+        <v>22064017</v>
       </c>
       <c r="X21" s="74" t="n">
-        <v>1.077833422762773</v>
+        <v>1.095200908418419</v>
       </c>
       <c r="Y21" s="28" t="n">
-        <v>35.97682353421516</v>
+        <v>36.08911153912589</v>
       </c>
       <c r="Z21" s="28" t="n">
-        <v>22.46902137332141</v>
+        <v>22.7272225716398</v>
       </c>
       <c r="AA21" s="28" t="n">
         <v>30.29687863664913</v>
       </c>
       <c r="AB21" s="75" t="n">
-        <v>-3.21735161466313</v>
+        <v>-3.213363984454816</v>
       </c>
       <c r="AC21" s="75" t="n">
-        <v>-2.054634515437876</v>
+        <v>-2.053836989396213</v>
       </c>
       <c r="AD21" s="75" t="n">
-        <v>-1.162717099225254</v>
+        <v>-1.159526995058602</v>
       </c>
       <c r="AE21" s="72" t="n">
-        <v>287.7826978998454</v>
+        <v>287.7938062982829</v>
       </c>
       <c r="AF21" s="72" t="n">
-        <v>291.9023265158758</v>
+        <v>291.9068708606911</v>
       </c>
       <c r="AG21" s="72" t="n">
-        <v>295.4046026611328</v>
+        <v>295.4056024169922</v>
       </c>
       <c r="AH21" s="72" t="n">
-        <v>291.5921017456055</v>
+        <v>291.5926016235351</v>
       </c>
       <c r="AI21" s="72" t="n">
-        <v>274.6385508728027</v>
+        <v>274.6388008117676</v>
       </c>
       <c r="AJ21" s="72" t="n">
-        <v>303.4159742029564</v>
+        <v>303.4109031165285</v>
       </c>
       <c r="AK21" s="72" t="n">
-        <v>293.1640060424805</v>
+        <v>293.1665054321289</v>
       </c>
       <c r="AL21" s="72" t="n">
-        <v>282.9120378820046</v>
+        <v>282.9221077477294</v>
       </c>
       <c r="AM21" s="76" t="n">
-        <v>0.1203655221210394</v>
+        <v>0.1224027514995309</v>
       </c>
       <c r="AN21" s="29" t="n">
-        <v>6.994015601622211</v>
+        <v>6.988791348656448</v>
       </c>
       <c r="AO21" s="77" t="n">
-        <v>1.252609388648028</v>
+        <v>1.252390017242089</v>
       </c>
       <c r="AP21" s="72" t="n">
         <v>305.1799926757812</v>
@@ -6165,22 +6165,22 @@
         <v>228.8999938964844</v>
       </c>
       <c r="AR21" s="29" t="n">
-        <v>-6.487970466007564</v>
+        <v>-6.471590692048446</v>
       </c>
       <c r="AS21" s="78" t="n">
-        <v>74.04301506315355</v>
+        <v>74.10854704239935</v>
       </c>
       <c r="AT21" s="26" t="n">
-        <v>-0.00806398062489222</v>
+        <v>-0.007890230917392049</v>
       </c>
       <c r="AU21" s="26" t="n">
-        <v>-0.04946209759220865</v>
+        <v>-0.04929559927045679</v>
       </c>
       <c r="AV21" s="26" t="n">
-        <v>-0.01552366470332844</v>
+        <v>-0.01535122165059377</v>
       </c>
       <c r="AW21" s="26" t="n">
-        <v>0.1593272694070087</v>
+        <v>0.1595303397361647</v>
       </c>
       <c r="AX21" s="79" t="inlineStr">
         <is>
@@ -6290,10 +6290,10 @@
         <v>112.0101013183594</v>
       </c>
       <c r="W22" s="84" t="n">
-        <v>55527137</v>
+        <v>55751188</v>
       </c>
       <c r="X22" s="85" t="n">
-        <v>0.9880274041332086</v>
+        <v>0.9918163745853109</v>
       </c>
       <c r="Y22" s="35" t="n">
         <v>47.29178331537246</v>
@@ -6490,7 +6490,7 @@
         <v>4.589996337890625</v>
       </c>
       <c r="T24" s="72" t="n">
-        <v>334.7699890136719</v>
+        <v>334.7550048828125</v>
       </c>
       <c r="U24" s="72" t="n">
         <v>338.3399963378906</v>
@@ -6499,10 +6499,10 @@
         <v>330.1936950683594</v>
       </c>
       <c r="W24" s="73" t="n">
-        <v>36188003</v>
+        <v>36423997</v>
       </c>
       <c r="X24" s="74" t="n">
-        <v>0.8788573802939148</v>
+        <v>0.8843352810121078</v>
       </c>
       <c r="Y24" s="28" t="n">
         <v>65.39135406375546</v>
@@ -6581,17 +6581,17 @@
       </c>
       <c r="AX24" s="79" t="inlineStr">
         <is>
+          <t>Apple (AAPL) Outperforms Broader Market: What You Need to Know</t>
+        </is>
+      </c>
+      <c r="AY24" s="79" t="inlineStr">
+        <is>
           <t>Apple iPhone 18 Pro Sales Helped By Carrier Promotions</t>
         </is>
       </c>
-      <c r="AY24" s="79" t="inlineStr">
+      <c r="AZ24" s="79" t="inlineStr">
         <is>
           <t>Apple's iPhone 18 lineup keeps Bank of America bullish</t>
-        </is>
-      </c>
-      <c r="AZ24" s="79" t="inlineStr">
-        <is>
-          <t>Bank of America flags surprising iPhone 18 pre-order trend</t>
         </is>
       </c>
     </row>
@@ -6678,7 +6678,7 @@
         <v>32.59002685546875</v>
       </c>
       <c r="T25" s="83" t="n">
-        <v>533.5999755859375</v>
+        <v>533.9000244140625</v>
       </c>
       <c r="U25" s="83" t="n">
         <v>551.4199829101562</v>
@@ -6687,10 +6687,10 @@
         <v>527.6500244140625</v>
       </c>
       <c r="W25" s="84" t="n">
-        <v>28150974</v>
+        <v>28330537</v>
       </c>
       <c r="X25" s="85" t="n">
-        <v>1.545843856491194</v>
+        <v>1.554937526409733</v>
       </c>
       <c r="Y25" s="35" t="n">
         <v>62.78140838923331</v>
@@ -6769,17 +6769,17 @@
       </c>
       <c r="AX25" s="90" t="inlineStr">
         <is>
+          <t>Dow Jones Futures: S&amp;P 500, Nasdaq Rebound Above Key Level; Moderna, AMD, SpaceX Flash Buy Signals</t>
+        </is>
+      </c>
+      <c r="AY25" s="90" t="inlineStr">
+        <is>
+          <t>AMD Leads Chip Stocks Higher Amid Sector Rebound</t>
+        </is>
+      </c>
+      <c r="AZ25" s="90" t="inlineStr">
+        <is>
           <t>AMD Jumps 7% as Semiconductor Rebound Reaches a Third Session; Broadcom Rises 3%, NVIDIA Edges Higher</t>
-        </is>
-      </c>
-      <c r="AY25" s="90" t="inlineStr">
-        <is>
-          <t>AMD Leads Chip Stocks Higher Amid Sector Rebound</t>
-        </is>
-      </c>
-      <c r="AZ25" s="90" t="inlineStr">
-        <is>
-          <t>Forget the AI Doom Headlines. Watch This AMD Number Instead.</t>
         </is>
       </c>
     </row>
@@ -6866,7 +6866,7 @@
         <v>5.229995727539062</v>
       </c>
       <c r="T26" s="72" t="n">
-        <v>251.0650024414062</v>
+        <v>251.1300048828125</v>
       </c>
       <c r="U26" s="72" t="n">
         <v>252.7299957275391</v>
@@ -6875,10 +6875,10 @@
         <v>249.2400054931641</v>
       </c>
       <c r="W26" s="73" t="n">
-        <v>29611821</v>
+        <v>29639613</v>
       </c>
       <c r="X26" s="74" t="n">
-        <v>0.9362585007640764</v>
+        <v>0.9370960484124431</v>
       </c>
       <c r="Y26" s="28" t="n">
         <v>45.39446648532397</v>
@@ -6957,17 +6957,17 @@
       </c>
       <c r="AX26" s="79" t="inlineStr">
         <is>
+          <t>AI Power Stocks Rally After Generac's Deal For Amazon Data Centers</t>
+        </is>
+      </c>
+      <c r="AY26" s="79" t="inlineStr">
+        <is>
+          <t>Amazon, Walmart Face FTC Probe Call Over AI Chatbots And ‘Made In USA’ Claims — AMZN, WMT Stocks In Focus</t>
+        </is>
+      </c>
+      <c r="AZ26" s="79" t="inlineStr">
+        <is>
           <t>Qualcomm Gains 2% as Amazon's Warrant Prices AI Commitment</t>
-        </is>
-      </c>
-      <c r="AY26" s="79" t="inlineStr">
-        <is>
-          <t>Amazon Jumps 2.5% While $2.4 Billion Buys Backup Power--and Equity</t>
-        </is>
-      </c>
-      <c r="AZ26" s="79" t="inlineStr">
-        <is>
-          <t>Hour Loop Falls 22% in Three Months: Should You Buy the Dip or Wait?</t>
         </is>
       </c>
     </row>
@@ -7063,10 +7063,10 @@
         <v>85.04000091552734</v>
       </c>
       <c r="W27" s="84" t="n">
-        <v>6757012</v>
+        <v>6757192</v>
       </c>
       <c r="X27" s="85" t="n">
-        <v>1.442506617329911</v>
+        <v>1.442542272631419</v>
       </c>
       <c r="Y27" s="35" t="n">
         <v>58.76148109917678</v>
@@ -7242,7 +7242,7 @@
         <v>20.91999816894531</v>
       </c>
       <c r="T28" s="72" t="n">
-        <v>262</v>
+        <v>261.3949890136719</v>
       </c>
       <c r="U28" s="72" t="n">
         <v>267</v>
@@ -7251,10 +7251,10 @@
         <v>256</v>
       </c>
       <c r="W28" s="73" t="n">
-        <v>5695481</v>
+        <v>6082058</v>
       </c>
       <c r="X28" s="74" t="n">
-        <v>1.481129205438949</v>
+        <v>1.573749365699924</v>
       </c>
       <c r="Y28" s="28" t="n">
         <v>53.99511353441969</v>
@@ -7430,7 +7430,7 @@
         <v>3.439998626708984</v>
       </c>
       <c r="T29" s="83" t="n">
-        <v>61.84999847412109</v>
+        <v>61.63059997558594</v>
       </c>
       <c r="U29" s="83" t="n">
         <v>63.70000076293945</v>
@@ -7439,10 +7439,10 @@
         <v>61.15000152587891</v>
       </c>
       <c r="W29" s="84" t="n">
-        <v>9121593</v>
+        <v>9141060</v>
       </c>
       <c r="X29" s="85" t="n">
-        <v>0.9869851459195024</v>
+        <v>0.988987377050883</v>
       </c>
       <c r="Y29" s="35" t="n">
         <v>49.89077054284351</v>
@@ -7618,7 +7618,7 @@
         <v>7.78997802734375</v>
       </c>
       <c r="T30" s="72" t="n">
-        <v>346.614990234375</v>
+        <v>346.0700073242188</v>
       </c>
       <c r="U30" s="72" t="n">
         <v>350.9400024414062</v>
@@ -7627,10 +7627,10 @@
         <v>345.3099975585938</v>
       </c>
       <c r="W30" s="73" t="n">
-        <v>22732113</v>
+        <v>22973542</v>
       </c>
       <c r="X30" s="74" t="n">
-        <v>0.8902083991116969</v>
+        <v>0.899237864081413</v>
       </c>
       <c r="Y30" s="28" t="n">
         <v>38.54302565021518</v>
@@ -7709,17 +7709,17 @@
       </c>
       <c r="AX30" s="79" t="inlineStr">
         <is>
+          <t>Jim Cramer on Broadcom (AVGO): “The Stock May Be Too Cheap to Ignore”</t>
+        </is>
+      </c>
+      <c r="AY30" s="79" t="inlineStr">
+        <is>
           <t>AMD Jumps 7% as Semiconductor Rebound Reaches a Third Session; Broadcom Rises 3%, NVIDIA Edges Higher</t>
         </is>
       </c>
-      <c r="AY30" s="79" t="inlineStr">
-        <is>
-          <t>Looking for a Good Deal on an AI Stock? This Leading Chipmaker Is Cheaper Than Broadcom and AMD.</t>
-        </is>
-      </c>
       <c r="AZ30" s="79" t="inlineStr">
         <is>
-          <t>Investors Want to Know When Broadcom’s Custom Hyperscaler Chips Will Move Share Prices</t>
+          <t>Broadcom CEO Hock Tan Says He Isn’t Worried – ‘No, Not in the Least’ – About AVGO as AI Extinction Fears Ra...</t>
         </is>
       </c>
     </row>
@@ -7815,10 +7815,10 @@
         <v>91.59999847412109</v>
       </c>
       <c r="W31" s="84" t="n">
-        <v>2073516</v>
+        <v>2097025</v>
       </c>
       <c r="X31" s="85" t="n">
-        <v>0.7809997834988129</v>
+        <v>0.7895050169396127</v>
       </c>
       <c r="Y31" s="35" t="n">
         <v>41.86387168601646</v>
@@ -7897,17 +7897,17 @@
       </c>
       <c r="AX31" s="90" t="inlineStr">
         <is>
+          <t>Cameco (CCJ) Beats Stock Market Upswing: What Investors Need to Know</t>
+        </is>
+      </c>
+      <c r="AY31" s="90" t="inlineStr">
+        <is>
           <t>Cameco vs. USA Rare Earth: Which Renewable Energy Stock Is a Better Buy in 2026?</t>
         </is>
       </c>
-      <c r="AY31" s="90" t="inlineStr">
+      <c r="AZ31" s="90" t="inlineStr">
         <is>
           <t>Jim Cramer Favors BWX Technologies (BWXT) Over Cameco (CCJ)</t>
-        </is>
-      </c>
-      <c r="AZ31" s="90" t="inlineStr">
-        <is>
-          <t>Cameco Controls the Uranium Refinery That Puts Canada in the Driver's Seat</t>
         </is>
       </c>
     </row>
@@ -8003,10 +8003,10 @@
         <v>78.26999664306641</v>
       </c>
       <c r="W32" s="73" t="n">
-        <v>78946643</v>
+        <v>79167396</v>
       </c>
       <c r="X32" s="74" t="n">
-        <v>3.374715177904115</v>
+        <v>3.382555687811552</v>
       </c>
       <c r="Y32" s="28" t="n">
         <v>42.43570914735687</v>
@@ -8090,12 +8090,12 @@
       </c>
       <c r="AY32" s="79" t="inlineStr">
         <is>
-          <t>Bernstein Flags CoreWeave as Most Exposed to an AI Training Slowdown</t>
+          <t>Stock Market Today, Sept. 17: CoreWeave Falls on Convertible Debt and Share Sale Announcement</t>
         </is>
       </c>
       <c r="AZ32" s="79" t="inlineStr">
         <is>
-          <t>CoreWeave Shares Sink on $3 Billion Convertible Notes</t>
+          <t>Nvidia cloud partner crosses major compute threshold</t>
         </is>
       </c>
     </row>
@@ -8191,10 +8191,10 @@
         <v>565.5</v>
       </c>
       <c r="W33" s="84" t="n">
-        <v>9047492</v>
+        <v>9164982</v>
       </c>
       <c r="X33" s="85" t="n">
-        <v>0.9236461127669434</v>
+        <v>0.9350797208296411</v>
       </c>
       <c r="Y33" s="35" t="n">
         <v>66.4322074343258</v>
@@ -8370,7 +8370,7 @@
         <v>4.32000732421875</v>
       </c>
       <c r="T34" s="72" t="n">
-        <v>345</v>
+        <v>344.9100036621094</v>
       </c>
       <c r="U34" s="72" t="n">
         <v>345.9649963378906</v>
@@ -8379,10 +8379,10 @@
         <v>340.5</v>
       </c>
       <c r="W34" s="73" t="n">
-        <v>13959247</v>
+        <v>14669379</v>
       </c>
       <c r="X34" s="74" t="n">
-        <v>0.876702624707572</v>
+        <v>0.9192521574020952</v>
       </c>
       <c r="Y34" s="28" t="n">
         <v>52.9140455982907</v>
@@ -8461,17 +8461,17 @@
       </c>
       <c r="AX34" s="79" t="inlineStr">
         <is>
-          <t>Nearly 90% of the Fortune 100 Now Use Sundar Pichai's Gemini Enterprise Tool. Here's Why That Adoption Rate...</t>
+          <t>Alphabet (GOOGL) Rises Higher Than Market: Key Facts</t>
         </is>
       </c>
       <c r="AY34" s="79" t="inlineStr">
         <is>
-          <t>Alphabet Gains 1.5% as $20 Opens Google Home to Rival Agents</t>
+          <t>Why Alphabet Inc. (GOOG) Outpaced the Stock Market Today</t>
         </is>
       </c>
       <c r="AZ34" s="79" t="inlineStr">
         <is>
-          <t>Google Faces 6 Years Of Global Oversight</t>
+          <t>PubMatic (PUBM) Stock Trades Up, Here Is Why</t>
         </is>
       </c>
     </row>
@@ -8567,10 +8567,10 @@
         <v>42.3400993347168</v>
       </c>
       <c r="W35" s="84" t="n">
-        <v>45998227</v>
+        <v>46263384</v>
       </c>
       <c r="X35" s="85" t="n">
-        <v>1.115318447080283</v>
+        <v>1.121387221195862</v>
       </c>
       <c r="Y35" s="35" t="n">
         <v>53.28211459267038</v>
@@ -8755,10 +8755,10 @@
         <v>104.6999969482422</v>
       </c>
       <c r="W36" s="73" t="n">
-        <v>147245737</v>
+        <v>147854414</v>
       </c>
       <c r="X36" s="74" t="n">
-        <v>1.577758860469852</v>
+        <v>1.583764450121718</v>
       </c>
       <c r="Y36" s="28" t="n">
         <v>62.01205099819376</v>
@@ -8837,12 +8837,12 @@
       </c>
       <c r="AX36" s="79" t="inlineStr">
         <is>
+          <t>Stock Market Today, Sept. 17: Intel Surges 8% on Rumored SK Hynix Talks</t>
+        </is>
+      </c>
+      <c r="AY36" s="79" t="inlineStr">
+        <is>
           <t>Intel Soars 9% On A Memory Deal That Doesn’t Exist Yet</t>
-        </is>
-      </c>
-      <c r="AY36" s="79" t="inlineStr">
-        <is>
-          <t>Why Intel Stock Popped Today</t>
         </is>
       </c>
       <c r="AZ36" s="79" t="inlineStr">
@@ -8943,10 +8943,10 @@
         <v>493.2749938964844</v>
       </c>
       <c r="W37" s="84" t="n">
-        <v>17638517</v>
+        <v>17779010</v>
       </c>
       <c r="X37" s="85" t="n">
-        <v>0.8791290832409536</v>
+        <v>0.8858213140625413</v>
       </c>
       <c r="Y37" s="35" t="n">
         <v>55.58408669054174</v>
@@ -9035,7 +9035,7 @@
       </c>
       <c r="AZ37" s="90" t="inlineStr">
         <is>
-          <t>Mintlify's 2026 State of Knowledge Report Finds AI Agents Have Overtaken Humans as the Primary Readers of C...</t>
+          <t>Generac, Nebius, CoreWeave, Nokia, Lucid, Paramount, and More Stocks That Explain Today’s Market</t>
         </is>
       </c>
     </row>
@@ -9131,10 +9131,10 @@
         <v>127.8199996948242</v>
       </c>
       <c r="W38" s="73" t="n">
-        <v>18250549</v>
+        <v>18294084</v>
       </c>
       <c r="X38" s="74" t="n">
-        <v>0.6676628518674707</v>
+        <v>0.669202209789635</v>
       </c>
       <c r="Y38" s="28" t="n">
         <v>56.02279627077972</v>
@@ -9319,10 +9319,10 @@
         <v>953.5</v>
       </c>
       <c r="W39" s="84" t="n">
-        <v>21670977</v>
+        <v>21883599</v>
       </c>
       <c r="X39" s="85" t="n">
-        <v>0.8923468559245589</v>
+        <v>0.9007077107958854</v>
       </c>
       <c r="Y39" s="35" t="n">
         <v>53.81015608594149</v>
@@ -9401,17 +9401,17 @@
       </c>
       <c r="AX39" s="90" t="inlineStr">
         <is>
+          <t>Prediction: A $5,000 Investment Split Between Micron and Sandisk Will Triple Before 2028</t>
+        </is>
+      </c>
+      <c r="AY39" s="90" t="inlineStr">
+        <is>
+          <t>Micron, Qualcomm, Nova, Lattice Semiconductor, and Workday Shares Are Soaring, What You Need To Know</t>
+        </is>
+      </c>
+      <c r="AZ39" s="90" t="inlineStr">
+        <is>
           <t>Micron Jumps 5.5% as Labor Claims AI's Margin Windfall</t>
-        </is>
-      </c>
-      <c r="AY39" s="90" t="inlineStr">
-        <is>
-          <t>The Memory Shortage Is Not Over: More Upside for Micron and Sandisk?</t>
-        </is>
-      </c>
-      <c r="AZ39" s="90" t="inlineStr">
-        <is>
-          <t>Micron Stock Soars as India Facility Bets Big on AI Memory Demand</t>
         </is>
       </c>
     </row>
@@ -9507,10 +9507,10 @@
         <v>209.6499938964844</v>
       </c>
       <c r="W40" s="73" t="n">
-        <v>30332699</v>
+        <v>30594337</v>
       </c>
       <c r="X40" s="74" t="n">
-        <v>1.971769676360077</v>
+        <v>1.987087599633421</v>
       </c>
       <c r="Y40" s="28" t="n">
         <v>49.86367030792658</v>
@@ -9594,12 +9594,12 @@
       </c>
       <c r="AY40" s="79" t="inlineStr">
         <is>
+          <t>Generac, Nebius, CoreWeave, Nokia, Lucid, Paramount, and More Stocks That Explain Today’s Market</t>
+        </is>
+      </c>
+      <c r="AZ40" s="79" t="inlineStr">
+        <is>
           <t>Why Nvidia-Backed Nebius Group Stock Skyrocketed Thursday Morning</t>
-        </is>
-      </c>
-      <c r="AZ40" s="79" t="inlineStr">
-        <is>
-          <t>Nebius Stock and IREN Gain. AI Neoclouds Are Flexing Their Pricing Power.</t>
         </is>
       </c>
     </row>
@@ -9695,10 +9695,10 @@
         <v>75.30000305175781</v>
       </c>
       <c r="W41" s="84" t="n">
-        <v>27702245</v>
+        <v>27803406</v>
       </c>
       <c r="X41" s="85" t="n">
-        <v>1.045872231066478</v>
+        <v>1.049491056738339</v>
       </c>
       <c r="Y41" s="35" t="n">
         <v>43.14417828904085</v>
@@ -9811,7 +9811,7 @@
       </c>
       <c r="F42" s="23" t="inlineStr">
         <is>
-          <t>Same</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G42" s="23" t="inlineStr">
@@ -9883,10 +9883,10 @@
         <v>10.4601001739502</v>
       </c>
       <c r="W42" s="73" t="n">
-        <v>131161318</v>
+        <v>136551436</v>
       </c>
       <c r="X42" s="74" t="n">
-        <v>1.755894156893716</v>
+        <v>1.821481392690107</v>
       </c>
       <c r="Y42" s="28" t="n">
         <v>53.38839167234221</v>
@@ -10071,10 +10071,10 @@
         <v>217.1450042724609</v>
       </c>
       <c r="W43" s="84" t="n">
-        <v>92249429</v>
+        <v>92845751</v>
       </c>
       <c r="X43" s="85" t="n">
-        <v>0.7111877697208117</v>
+        <v>0.7156205591065099</v>
       </c>
       <c r="Y43" s="35" t="n">
         <v>51.71826192266046</v>
@@ -10153,17 +10153,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
-          <t>Intel Soars 9% On A Memory Deal That Doesn’t Exist Yet</t>
+          <t>Trump-Xi Dinner Next Week Brings AI Titans To The Table — OpenAI, NVDA, and QCOM CEOs To Attend, Says Report</t>
         </is>
       </c>
       <c r="AY43" s="90" t="inlineStr">
         <is>
-          <t>Nvidia Stock Rises. Jensen Huang Sees Chip Sales Doubling in 2027</t>
+          <t>S&amp;P 500, Nasdaq, Dow End Higher As Drop In Oil Prices Allays Inflationary Concerns — NVDA, MCD, CRWV, LMT, ...</t>
         </is>
       </c>
       <c r="AZ43" s="90" t="inlineStr">
         <is>
-          <t>3 Stocks to Buy if You Believe the AI Power Crunch Is Just Getting Started</t>
+          <t>Michael Burry returns to a difficult corner of Wall Street</t>
         </is>
       </c>
     </row>
@@ -10259,10 +10259,10 @@
         <v>172.6069946289062</v>
       </c>
       <c r="W44" s="73" t="n">
-        <v>22629390</v>
+        <v>22869993</v>
       </c>
       <c r="X44" s="74" t="n">
-        <v>0.8029917091088913</v>
+        <v>0.8111830963124707</v>
       </c>
       <c r="Y44" s="28" t="n">
         <v>55.93108877372765</v>
@@ -10341,17 +10341,17 @@
       </c>
       <c r="AX44" s="79" t="inlineStr">
         <is>
+          <t>Palantir, Rocket Lab among biggest climbers in power ranking</t>
+        </is>
+      </c>
+      <c r="AY44" s="79" t="inlineStr">
+        <is>
+          <t>'You’re Liable For Your Own Actions': Palantir CEO Alex Karp Opens a Third Front In The AI Safety Fight</t>
+        </is>
+      </c>
+      <c r="AZ44" s="79" t="inlineStr">
+        <is>
           <t>Palantir Gains as Europe Builds a Sovereign AI Counterweight</t>
-        </is>
-      </c>
-      <c r="AY44" s="79" t="inlineStr">
-        <is>
-          <t>Palantir CEO Karp Says the Quiet Part Out Loud in the AI Risk Debate</t>
-        </is>
-      </c>
-      <c r="AZ44" s="79" t="inlineStr">
-        <is>
-          <t>Mad Money Jim Cramer Sees 40% Upside for Palantir Stock. Does Wall Street Agree?</t>
         </is>
       </c>
     </row>
@@ -10447,10 +10447,10 @@
         <v>187.7601013183594</v>
       </c>
       <c r="W45" s="84" t="n">
-        <v>12056736</v>
+        <v>12213121</v>
       </c>
       <c r="X45" s="85" t="n">
-        <v>1.028588528092138</v>
+        <v>1.041235514598102</v>
       </c>
       <c r="Y45" s="35" t="n">
         <v>67.90284307896547</v>
@@ -10529,17 +10529,17 @@
       </c>
       <c r="AX45" s="90" t="inlineStr">
         <is>
+          <t>Trump-Xi Dinner Next Week Brings AI Titans To The Table — OpenAI, NVDA, and QCOM CEOs To Attend, Says Report</t>
+        </is>
+      </c>
+      <c r="AY45" s="90" t="inlineStr">
+        <is>
+          <t>Qualcomm (QCOM) Outpaces Stock Market Gains: What You Should Know</t>
+        </is>
+      </c>
+      <c r="AZ45" s="90" t="inlineStr">
+        <is>
           <t>Qualcomm Just Rallied 18% in a Month: Take Profits, or Buy More?</t>
-        </is>
-      </c>
-      <c r="AY45" s="90" t="inlineStr">
-        <is>
-          <t>Qualcomm Gains 2% as Amazon's Warrant Prices AI Commitment</t>
-        </is>
-      </c>
-      <c r="AZ45" s="90" t="inlineStr">
-        <is>
-          <t>Qualcomm Faces Margin Pressure From Rising Costs: Can it Recover?</t>
         </is>
       </c>
     </row>
@@ -10626,7 +10626,7 @@
         <v>4.119998931884766</v>
       </c>
       <c r="T46" s="72" t="n">
-        <v>65.55000305175781</v>
+        <v>65.48000335693359</v>
       </c>
       <c r="U46" s="72" t="n">
         <v>68.33070373535156</v>
@@ -10635,10 +10635,10 @@
         <v>65.26000213623047</v>
       </c>
       <c r="W46" s="73" t="n">
-        <v>21066097</v>
+        <v>21810895</v>
       </c>
       <c r="X46" s="74" t="n">
-        <v>1.242339923201914</v>
+        <v>1.283444557933647</v>
       </c>
       <c r="Y46" s="28" t="n">
         <v>50.12651944486846</v>
@@ -10717,17 +10717,17 @@
       </c>
       <c r="AX46" s="79" t="inlineStr">
         <is>
+          <t>Palantir, Rocket Lab among biggest climbers in power ranking</t>
+        </is>
+      </c>
+      <c r="AY46" s="79" t="inlineStr">
+        <is>
           <t>Rocket Lab Is Playing a Much Bigger Game Than Rocket Launches, Eyes 90% Upside</t>
         </is>
       </c>
-      <c r="AY46" s="79" t="inlineStr">
+      <c r="AZ46" s="79" t="inlineStr">
         <is>
           <t>Rocket Lab Jumps 6% as FCC Clears First Hurdle on Iridium Deal; Iridium Communications Barely Budges</t>
-        </is>
-      </c>
-      <c r="AZ46" s="79" t="inlineStr">
-        <is>
-          <t>RKLB Stock Eyes Ending 5-Week Slide: Iridium Deal Clears First FCC Hurdle, VC Backer Hails Solar Breakthrough</t>
         </is>
       </c>
     </row>
@@ -10814,7 +10814,7 @@
         <v>94.4200439453125</v>
       </c>
       <c r="T47" s="83" t="n">
-        <v>1564.530029296875</v>
+        <v>1564.501953125</v>
       </c>
       <c r="U47" s="83" t="n">
         <v>1625.35498046875</v>
@@ -10823,10 +10823,10 @@
         <v>1564.500122070312</v>
       </c>
       <c r="W47" s="84" t="n">
-        <v>8378922</v>
+        <v>8402626</v>
       </c>
       <c r="X47" s="85" t="n">
-        <v>0.8037295855557006</v>
+        <v>0.8059117171553075</v>
       </c>
       <c r="Y47" s="35" t="n">
         <v>52.84955340505821</v>
@@ -10905,17 +10905,17 @@
       </c>
       <c r="AX47" s="90" t="inlineStr">
         <is>
+          <t>Prediction: A $5,000 Investment Split Between Micron and Sandisk Will Triple Before 2028</t>
+        </is>
+      </c>
+      <c r="AY47" s="90" t="inlineStr">
+        <is>
           <t>Sandisk Is Up More Than 1,700% in a Year and Still 33% Off Its Peak. History Says This is What Happens Next.</t>
         </is>
       </c>
-      <c r="AY47" s="90" t="inlineStr">
+      <c r="AZ47" s="90" t="inlineStr">
         <is>
           <t>The Memory Shortage Is Not Over: More Upside for Micron and Sandisk?</t>
-        </is>
-      </c>
-      <c r="AZ47" s="90" t="inlineStr">
-        <is>
-          <t>Sandisk Stock Has Dropped 35% Since June. Here’s Where the Stock Could Go in 2026</t>
         </is>
       </c>
     </row>
@@ -11002,7 +11002,7 @@
         <v>8.120025634765625</v>
       </c>
       <c r="T48" s="72" t="n">
-        <v>367.4800109863281</v>
+        <v>367.5899963378906</v>
       </c>
       <c r="U48" s="72" t="n">
         <v>374.1199951171875</v>
@@ -11011,10 +11011,10 @@
         <v>363.2200012207031</v>
       </c>
       <c r="W48" s="73" t="n">
-        <v>37852555</v>
+        <v>38770658</v>
       </c>
       <c r="X48" s="74" t="n">
-        <v>0.9613781234100275</v>
+        <v>0.9835493595483629</v>
       </c>
       <c r="Y48" s="28" t="n">
         <v>54.8147739891341</v>
@@ -11093,17 +11093,17 @@
       </c>
       <c r="AX48" s="79" t="inlineStr">
         <is>
+          <t>Tesla (TSLA) Exceeds Market Returns: Some Facts to Consider</t>
+        </is>
+      </c>
+      <c r="AY48" s="79" t="inlineStr">
+        <is>
+          <t>Rivian Reports Q3 Deliveries for the R2 SUV in October. Here's How Investors Should Prepare.</t>
+        </is>
+      </c>
+      <c r="AZ48" s="79" t="inlineStr">
+        <is>
           <t>Tesla Jumps 2% as 30 Megawatts Build a Semi Beachhead</t>
-        </is>
-      </c>
-      <c r="AY48" s="79" t="inlineStr">
-        <is>
-          <t>Elon Musk warns one AI milestone dwarfs nuclear weapons</t>
-        </is>
-      </c>
-      <c r="AZ48" s="79" t="inlineStr">
-        <is>
-          <t>Elon Musk sends strong message to SpaceX and Tesla investors</t>
         </is>
       </c>
     </row>
@@ -11640,7 +11640,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 17 Sep 2026, 08:28 PM · Yahoo Finance data</t>
+          <t>Built 17 Sep 2026, 10:52 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19576,7 +19576,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 17 Sep 2026, 08:28 PM · Yahoo Finance data</t>
+          <t>Built 17 Sep 2026, 10:52 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27512,7 +27512,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 17 Sep 2026, 08:28 PM · Yahoo Finance data</t>
+          <t>Built 17 Sep 2026, 10:52 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35448,7 +35448,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 17 Sep 2026, 08:28 PM · Yahoo Finance data</t>
+          <t>Built 17 Sep 2026, 10:52 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -43428,22 +43428,22 @@
         </is>
       </c>
       <c r="D8" s="26" t="n">
-        <v>0.006871817113770051</v>
+        <v>0.007028027271839044</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>-0.007084538461583634</v>
+        <v>-0.006930493548855221</v>
       </c>
       <c r="F8" s="26" t="n">
-        <v>0.0124057932120194</v>
+        <v>0.01256286193347878</v>
       </c>
       <c r="G8" s="26" t="n">
-        <v>0.1792574241812321</v>
+        <v>0.1794403789382373</v>
       </c>
       <c r="H8" s="26" t="n">
-        <v>0.103371570836571</v>
+        <v>0.1035427523559656</v>
       </c>
       <c r="I8" s="26" t="n">
-        <v>0.4419593500527028</v>
+        <v>0.4421830614469162</v>
       </c>
       <c r="J8" s="27" t="n">
         <v>6</v>
@@ -43993,7 +43993,7 @@
       </c>
       <c r="D8" s="104" t="inlineStr">
         <is>
-          <t>Gapped up 7.4% at the open</t>
+          <t>Gapped up 7.1% at the open</t>
         </is>
       </c>
       <c r="E8" s="26" t="n">
@@ -44133,7 +44133,7 @@
       </c>
       <c r="D13" s="105" t="inlineStr">
         <is>
-          <t>Gapped up 4.1% at the open</t>
+          <t>Gapped up 4.2% at the open</t>
         </is>
       </c>
       <c r="E13" s="33" t="n">
@@ -44581,7 +44581,7 @@
       </c>
       <c r="D29" s="105" t="inlineStr">
         <is>
-          <t>Gapped up 2.6% at the open</t>
+          <t>Gapped up 2.7% at the open</t>
         </is>
       </c>
       <c r="E29" s="33" t="n">
@@ -44683,21 +44683,21 @@
     <row r="33">
       <c r="B33" s="31" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="C33" s="102" t="inlineStr">
         <is>
-          <t>Microsoft Corporation</t>
+          <t>Invesco QQQ Trust</t>
         </is>
       </c>
       <c r="D33" s="105" t="inlineStr">
         <is>
-          <t>Gapped up 1.5% at the open</t>
+          <t>RSI crossed back above 50</t>
         </is>
       </c>
       <c r="E33" s="33" t="n">
-        <v>0.01519480398228579</v>
+        <v>0.0173118582049816</v>
       </c>
       <c r="F33" s="34" t="n">
         <v>8</v>
@@ -44711,21 +44711,21 @@
     <row r="34">
       <c r="B34" s="24" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="C34" s="101" t="inlineStr">
         <is>
-          <t>Microsoft Corporation</t>
+          <t>Invesco QQQ Trust</t>
         </is>
       </c>
       <c r="D34" s="104" t="inlineStr">
         <is>
-          <t>Bands squeezing — a big move often follows</t>
+          <t>Reclaimed the 50 DMA</t>
         </is>
       </c>
       <c r="E34" s="26" t="n">
-        <v>0.01519480398228579</v>
+        <v>0.0173118582049816</v>
       </c>
       <c r="F34" s="27" t="n">
         <v>8</v>
@@ -44739,21 +44739,21 @@
     <row r="35">
       <c r="B35" s="31" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="C35" s="102" t="inlineStr">
         <is>
-          <t>Alphabet Inc.</t>
+          <t>Invesco QQQ Trust</t>
         </is>
       </c>
       <c r="D35" s="105" t="inlineStr">
         <is>
-          <t>RSI crossed back above 50</t>
+          <t>Gapped up 1.6% at the open</t>
         </is>
       </c>
       <c r="E35" s="33" t="n">
-        <v>0.01272986654494157</v>
+        <v>0.0173118582049816</v>
       </c>
       <c r="F35" s="34" t="n">
         <v>8</v>
@@ -44767,21 +44767,21 @@
     <row r="36">
       <c r="B36" s="24" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="C36" s="101" t="inlineStr">
         <is>
-          <t>Alphabet Inc.</t>
+          <t>Invesco QQQ Trust</t>
         </is>
       </c>
       <c r="D36" s="104" t="inlineStr">
         <is>
-          <t>Gapped up 1.7% at the open</t>
+          <t>Bands squeezing — a big move often follows</t>
         </is>
       </c>
       <c r="E36" s="26" t="n">
-        <v>0.01272986654494157</v>
+        <v>0.0173118582049816</v>
       </c>
       <c r="F36" s="27" t="n">
         <v>8</v>
@@ -44795,21 +44795,21 @@
     <row r="37">
       <c r="B37" s="31" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="C37" s="102" t="inlineStr">
         <is>
-          <t>Alphabet Inc.</t>
+          <t>Microsoft Corporation</t>
         </is>
       </c>
       <c r="D37" s="105" t="inlineStr">
         <is>
-          <t>Bands squeezing — a big move often follows</t>
+          <t>Gapped up 1.5% at the open</t>
         </is>
       </c>
       <c r="E37" s="33" t="n">
-        <v>0.01272986654494157</v>
+        <v>0.01519480398228579</v>
       </c>
       <c r="F37" s="34" t="n">
         <v>8</v>
@@ -44823,133 +44823,133 @@
     <row r="38">
       <c r="B38" s="24" t="inlineStr">
         <is>
-          <t>RKLB</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="C38" s="101" t="inlineStr">
         <is>
-          <t>Rocket Lab Corporation</t>
+          <t>Microsoft Corporation</t>
         </is>
       </c>
       <c r="D38" s="104" t="inlineStr">
         <is>
-          <t>RSI crossed back above 50</t>
+          <t>Bands squeezing — a big move often follows</t>
         </is>
       </c>
       <c r="E38" s="26" t="n">
-        <v>0.06467816142133831</v>
+        <v>0.01519480398228579</v>
       </c>
       <c r="F38" s="27" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G38" s="23" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Very Strong</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="31" t="inlineStr">
         <is>
-          <t>RKLB</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="C39" s="102" t="inlineStr">
         <is>
-          <t>Rocket Lab Corporation</t>
+          <t>Alphabet Inc.</t>
         </is>
       </c>
       <c r="D39" s="105" t="inlineStr">
         <is>
-          <t>Gapped up 2.9% at the open</t>
+          <t>RSI crossed back above 50</t>
         </is>
       </c>
       <c r="E39" s="33" t="n">
-        <v>0.06467816142133831</v>
+        <v>0.01272986654494157</v>
       </c>
       <c r="F39" s="34" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G39" s="30" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Very Strong</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="B40" s="24" t="inlineStr">
         <is>
-          <t>RKLB</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="C40" s="101" t="inlineStr">
         <is>
-          <t>Rocket Lab Corporation</t>
+          <t>Alphabet Inc.</t>
         </is>
       </c>
       <c r="D40" s="104" t="inlineStr">
         <is>
-          <t>Bands squeezing — a big move often follows</t>
+          <t>Gapped up 1.6% at the open</t>
         </is>
       </c>
       <c r="E40" s="26" t="n">
-        <v>0.06467816142133831</v>
+        <v>0.01272986654494157</v>
       </c>
       <c r="F40" s="27" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G40" s="23" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Very Strong</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="31" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="C41" s="102" t="inlineStr">
         <is>
-          <t>NVIDIA Corporation</t>
+          <t>Alphabet Inc.</t>
         </is>
       </c>
       <c r="D41" s="105" t="inlineStr">
         <is>
-          <t>RSI crossed back above 50</t>
+          <t>Bands squeezing — a big move often follows</t>
         </is>
       </c>
       <c r="E41" s="33" t="n">
-        <v>0.0254324572072635</v>
+        <v>0.01272986654494157</v>
       </c>
       <c r="F41" s="34" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G41" s="30" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Very Strong</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="B42" s="24" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>RKLB</t>
         </is>
       </c>
       <c r="C42" s="101" t="inlineStr">
         <is>
-          <t>NVIDIA Corporation</t>
+          <t>Rocket Lab Corporation</t>
         </is>
       </c>
       <c r="D42" s="104" t="inlineStr">
         <is>
-          <t>Gapped up 2.1% at the open</t>
+          <t>RSI crossed back above 50</t>
         </is>
       </c>
       <c r="E42" s="26" t="n">
-        <v>0.0254324572072635</v>
+        <v>0.06467816142133831</v>
       </c>
       <c r="F42" s="27" t="n">
         <v>7</v>
@@ -44963,21 +44963,21 @@
     <row r="43">
       <c r="B43" s="31" t="inlineStr">
         <is>
-          <t>XLK</t>
+          <t>RKLB</t>
         </is>
       </c>
       <c r="C43" s="102" t="inlineStr">
         <is>
-          <t>State Street Technology Select Sector SPDR ETF</t>
+          <t>Rocket Lab Corporation</t>
         </is>
       </c>
       <c r="D43" s="105" t="inlineStr">
         <is>
-          <t>RSI crossed back above 50</t>
+          <t>Gapped up 2.8% at the open</t>
         </is>
       </c>
       <c r="E43" s="33" t="n">
-        <v>0.02245422197179425</v>
+        <v>0.06467816142133831</v>
       </c>
       <c r="F43" s="34" t="n">
         <v>7</v>
@@ -44991,21 +44991,21 @@
     <row r="44">
       <c r="B44" s="24" t="inlineStr">
         <is>
-          <t>XLK</t>
+          <t>RKLB</t>
         </is>
       </c>
       <c r="C44" s="101" t="inlineStr">
         <is>
-          <t>State Street Technology Select Sector SPDR ETF</t>
+          <t>Rocket Lab Corporation</t>
         </is>
       </c>
       <c r="D44" s="104" t="inlineStr">
         <is>
-          <t>Gapped up 1.8% at the open</t>
+          <t>Bands squeezing — a big move often follows</t>
         </is>
       </c>
       <c r="E44" s="26" t="n">
-        <v>0.02245422197179425</v>
+        <v>0.06467816142133831</v>
       </c>
       <c r="F44" s="27" t="n">
         <v>7</v>
@@ -45019,21 +45019,21 @@
     <row r="45">
       <c r="B45" s="31" t="inlineStr">
         <is>
-          <t>XLK</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="C45" s="102" t="inlineStr">
         <is>
-          <t>State Street Technology Select Sector SPDR ETF</t>
+          <t>NVIDIA Corporation</t>
         </is>
       </c>
       <c r="D45" s="105" t="inlineStr">
         <is>
-          <t>Bands squeezing — a big move often follows</t>
+          <t>RSI crossed back above 50</t>
         </is>
       </c>
       <c r="E45" s="33" t="n">
-        <v>0.02245422197179425</v>
+        <v>0.0254324572072635</v>
       </c>
       <c r="F45" s="34" t="n">
         <v>7</v>
@@ -45047,21 +45047,21 @@
     <row r="46">
       <c r="B46" s="24" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="C46" s="101" t="inlineStr">
         <is>
-          <t>Invesco QQQ Trust</t>
+          <t>NVIDIA Corporation</t>
         </is>
       </c>
       <c r="D46" s="104" t="inlineStr">
         <is>
-          <t>RSI crossed back above 50</t>
+          <t>Gapped up 2.1% at the open</t>
         </is>
       </c>
       <c r="E46" s="26" t="n">
-        <v>0.0173118582049816</v>
+        <v>0.0254324572072635</v>
       </c>
       <c r="F46" s="27" t="n">
         <v>7</v>
@@ -45075,21 +45075,21 @@
     <row r="47">
       <c r="B47" s="31" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>XLK</t>
         </is>
       </c>
       <c r="C47" s="102" t="inlineStr">
         <is>
-          <t>Invesco QQQ Trust</t>
+          <t>State Street Technology Select Sector SPDR ETF</t>
         </is>
       </c>
       <c r="D47" s="105" t="inlineStr">
         <is>
-          <t>Reclaimed the 50 DMA</t>
+          <t>RSI crossed back above 50</t>
         </is>
       </c>
       <c r="E47" s="33" t="n">
-        <v>0.0173118582049816</v>
+        <v>0.02245422197179425</v>
       </c>
       <c r="F47" s="34" t="n">
         <v>7</v>
@@ -45103,21 +45103,21 @@
     <row r="48">
       <c r="B48" s="24" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>XLK</t>
         </is>
       </c>
       <c r="C48" s="101" t="inlineStr">
         <is>
-          <t>Invesco QQQ Trust</t>
+          <t>State Street Technology Select Sector SPDR ETF</t>
         </is>
       </c>
       <c r="D48" s="104" t="inlineStr">
         <is>
-          <t>Gapped up 1.6% at the open</t>
+          <t>Gapped up 1.8% at the open</t>
         </is>
       </c>
       <c r="E48" s="26" t="n">
-        <v>0.0173118582049816</v>
+        <v>0.02245422197179425</v>
       </c>
       <c r="F48" s="27" t="n">
         <v>7</v>
@@ -45131,12 +45131,12 @@
     <row r="49">
       <c r="B49" s="31" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>XLK</t>
         </is>
       </c>
       <c r="C49" s="102" t="inlineStr">
         <is>
-          <t>Invesco QQQ Trust</t>
+          <t>State Street Technology Select Sector SPDR ETF</t>
         </is>
       </c>
       <c r="D49" s="105" t="inlineStr">
@@ -45145,7 +45145,7 @@
         </is>
       </c>
       <c r="E49" s="33" t="n">
-        <v>0.0173118582049816</v>
+        <v>0.02245422197179425</v>
       </c>
       <c r="F49" s="34" t="n">
         <v>7</v>
@@ -45197,7 +45197,7 @@
       </c>
       <c r="D51" s="105" t="inlineStr">
         <is>
-          <t>Gapped up 4.4% at the open</t>
+          <t>Gapped up 4.0% at the open</t>
         </is>
       </c>
       <c r="E51" s="33" t="n">
@@ -45397,7 +45397,7 @@
         </is>
       </c>
       <c r="E58" s="26" t="n">
-        <v>0.006871817113770051</v>
+        <v>0.007028027271839044</v>
       </c>
       <c r="F58" s="27" t="n">
         <v>6</v>
@@ -45617,7 +45617,7 @@
       </c>
       <c r="D66" s="104" t="inlineStr">
         <is>
-          <t>Gapped up 2.1% at the open</t>
+          <t>Gapped up 1.9% at the open</t>
         </is>
       </c>
       <c r="E66" s="26" t="n">

</xml_diff>

<commit_message>
Daily workbook: 2026-09-17 23:33 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -28,7 +28,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'09-14'!$5:$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'09-11'!$A$6:$AZ$48</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'09-11'!$5:$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Signals'!$B$5:$G$74</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Signals'!$B$5:$G$71</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1299,7 +1299,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 17 Sep 2026, 10:52 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 17 Sep 2026, 11:32 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -1373,21 +1373,21 @@
       <c r="D8" s="6" t="n"/>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F8" s="8" t="n"/>
       <c r="G8" s="8" t="n"/>
       <c r="H8" s="13" t="inlineStr">
         <is>
-          <t>90%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="I8" s="6" t="n"/>
       <c r="J8" s="6" t="n"/>
       <c r="K8" s="15" t="inlineStr">
         <is>
-          <t>5.4</t>
+          <t>5.5</t>
         </is>
       </c>
       <c r="L8" s="10" t="n"/>
@@ -1401,7 +1401,7 @@
       <c r="P8" s="10" t="n"/>
       <c r="Q8" s="16" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>66</t>
         </is>
       </c>
       <c r="R8" s="12" t="n"/>
@@ -1410,14 +1410,14 @@
     <row r="9" ht="15" customHeight="1">
       <c r="B9" s="17" t="inlineStr">
         <is>
-          <t>of 40 names</t>
+          <t>of 39 names</t>
         </is>
       </c>
       <c r="C9" s="6" t="n"/>
       <c r="D9" s="6" t="n"/>
       <c r="E9" s="18" t="inlineStr">
         <is>
-          <t>of 40 names</t>
+          <t>of 39 names</t>
         </is>
       </c>
       <c r="F9" s="8" t="n"/>
@@ -1438,7 +1438,7 @@
       <c r="M9" s="10" t="n"/>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>of 40 names</t>
+          <t>of 39 names</t>
         </is>
       </c>
       <c r="O9" s="10" t="n"/>
@@ -1954,11 +1954,11 @@
       </c>
       <c r="H29" s="24" t="inlineStr">
         <is>
-          <t>CRWV</t>
+          <t>NFLX</t>
         </is>
       </c>
       <c r="I29" s="26" t="n">
-        <v>-0.04163168907292192</v>
+        <v>-0.01439610065168861</v>
       </c>
       <c r="J29" s="27" t="n">
         <v>1</v>
@@ -1969,7 +1969,7 @@
         </is>
       </c>
       <c r="L29" s="28" t="n">
-        <v>42.43570914735687</v>
+        <v>43.14417828904085</v>
       </c>
     </row>
     <row r="30">
@@ -1994,11 +1994,11 @@
       </c>
       <c r="H30" s="31" t="inlineStr">
         <is>
-          <t>NFLX</t>
+          <t>XLF</t>
         </is>
       </c>
       <c r="I30" s="33" t="n">
-        <v>-0.01439610065168861</v>
+        <v>-0.0008939609652732772</v>
       </c>
       <c r="J30" s="34" t="n">
         <v>1</v>
@@ -2009,7 +2009,7 @@
         </is>
       </c>
       <c r="L30" s="35" t="n">
-        <v>43.14417828904085</v>
+        <v>37.08635589509742</v>
       </c>
     </row>
     <row r="31">
@@ -2034,11 +2034,11 @@
       </c>
       <c r="H31" s="24" t="inlineStr">
         <is>
-          <t>XLF</t>
+          <t>XLI</t>
         </is>
       </c>
       <c r="I31" s="26" t="n">
-        <v>-0.0008939609652732772</v>
+        <v>0.001778126850990658</v>
       </c>
       <c r="J31" s="27" t="n">
         <v>1</v>
@@ -2049,7 +2049,7 @@
         </is>
       </c>
       <c r="L31" s="28" t="n">
-        <v>37.08635589509742</v>
+        <v>31.46829525388786</v>
       </c>
     </row>
     <row r="32">
@@ -2074,11 +2074,11 @@
       </c>
       <c r="H32" s="31" t="inlineStr">
         <is>
-          <t>XLI</t>
+          <t>XLP</t>
         </is>
       </c>
       <c r="I32" s="33" t="n">
-        <v>0.001778126850990658</v>
+        <v>0.00192002915155598</v>
       </c>
       <c r="J32" s="34" t="n">
         <v>1</v>
@@ -2089,7 +2089,7 @@
         </is>
       </c>
       <c r="L32" s="35" t="n">
-        <v>31.46829525388786</v>
+        <v>42.86077646368995</v>
       </c>
     </row>
     <row r="33">
@@ -2114,11 +2114,11 @@
       </c>
       <c r="H33" s="24" t="inlineStr">
         <is>
-          <t>XLP</t>
+          <t>XLRE</t>
         </is>
       </c>
       <c r="I33" s="26" t="n">
-        <v>0.00192002915155598</v>
+        <v>0.003036609419477143</v>
       </c>
       <c r="J33" s="27" t="n">
         <v>1</v>
@@ -2129,7 +2129,7 @@
         </is>
       </c>
       <c r="L33" s="28" t="n">
-        <v>42.86077646368995</v>
+        <v>34.74774022483162</v>
       </c>
     </row>
     <row r="34">
@@ -2154,11 +2154,11 @@
       </c>
       <c r="H34" s="31" t="inlineStr">
         <is>
-          <t>XLRE</t>
+          <t>XLU</t>
         </is>
       </c>
       <c r="I34" s="33" t="n">
-        <v>0.003036609419477143</v>
+        <v>0.008954475668379924</v>
       </c>
       <c r="J34" s="34" t="n">
         <v>1</v>
@@ -2169,7 +2169,7 @@
         </is>
       </c>
       <c r="L34" s="35" t="n">
-        <v>34.74774022483162</v>
+        <v>35.70541017702637</v>
       </c>
     </row>
     <row r="35">
@@ -2194,11 +2194,11 @@
       </c>
       <c r="H35" s="24" t="inlineStr">
         <is>
-          <t>XLU</t>
+          <t>XLY</t>
         </is>
       </c>
       <c r="I35" s="26" t="n">
-        <v>0.008954475668379924</v>
+        <v>0.01098202106662916</v>
       </c>
       <c r="J35" s="27" t="n">
         <v>1</v>
@@ -2209,7 +2209,7 @@
         </is>
       </c>
       <c r="L35" s="28" t="n">
-        <v>35.70541017702637</v>
+        <v>38.99198318866176</v>
       </c>
     </row>
     <row r="36">
@@ -2234,11 +2234,11 @@
       </c>
       <c r="H36" s="31" t="inlineStr">
         <is>
-          <t>XLY</t>
+          <t>CCJ</t>
         </is>
       </c>
       <c r="I36" s="33" t="n">
-        <v>0.01098202106662916</v>
+        <v>0.02090210664449743</v>
       </c>
       <c r="J36" s="34" t="n">
         <v>1</v>
@@ -2249,7 +2249,7 @@
         </is>
       </c>
       <c r="L36" s="35" t="n">
-        <v>38.99198318866176</v>
+        <v>41.86387168601646</v>
       </c>
     </row>
     <row r="37">
@@ -2274,11 +2274,11 @@
       </c>
       <c r="H37" s="24" t="inlineStr">
         <is>
-          <t>CCJ</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="I37" s="26" t="n">
-        <v>0.02090210664449743</v>
+        <v>0.02294476687954328</v>
       </c>
       <c r="J37" s="27" t="n">
         <v>1</v>
@@ -2289,7 +2289,7 @@
         </is>
       </c>
       <c r="L37" s="28" t="n">
-        <v>41.86387168601646</v>
+        <v>38.54302565021518</v>
       </c>
     </row>
     <row r="38">
@@ -2314,22 +2314,22 @@
       </c>
       <c r="H38" s="31" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>IWM</t>
         </is>
       </c>
       <c r="I38" s="33" t="n">
-        <v>0.02294476687954328</v>
+        <v>0.005318326206797064</v>
       </c>
       <c r="J38" s="34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K38" s="30" t="inlineStr">
         <is>
-          <t>Very Weak</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="L38" s="35" t="n">
-        <v>38.54302565021518</v>
+        <v>36.08911153912589</v>
       </c>
     </row>
     <row r="41" ht="22" customHeight="1">
@@ -2418,11 +2418,11 @@
       </c>
       <c r="H43" s="24" t="inlineStr">
         <is>
-          <t>CRWV</t>
+          <t>NFLX</t>
         </is>
       </c>
       <c r="I43" s="26" t="n">
-        <v>-0.04163168907292192</v>
+        <v>-0.01439610065168861</v>
       </c>
       <c r="J43" s="27" t="n">
         <v>1</v>
@@ -2433,7 +2433,7 @@
         </is>
       </c>
       <c r="L43" s="28" t="n">
-        <v>42.43570914735687</v>
+        <v>43.14417828904085</v>
       </c>
     </row>
     <row r="44">
@@ -2458,22 +2458,22 @@
       </c>
       <c r="H44" s="31" t="inlineStr">
         <is>
-          <t>NFLX</t>
+          <t>XLC</t>
         </is>
       </c>
       <c r="I44" s="33" t="n">
-        <v>-0.01439610065168861</v>
+        <v>-0.00575222589273372</v>
       </c>
       <c r="J44" s="34" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K44" s="30" t="inlineStr">
         <is>
-          <t>Very Weak</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="L44" s="35" t="n">
-        <v>43.14417828904085</v>
+        <v>51.02913306530867</v>
       </c>
     </row>
     <row r="45">
@@ -2498,22 +2498,22 @@
       </c>
       <c r="H45" s="24" t="inlineStr">
         <is>
-          <t>XLC</t>
+          <t>XLF</t>
         </is>
       </c>
       <c r="I45" s="26" t="n">
-        <v>-0.00575222589273372</v>
+        <v>-0.0008939609652732772</v>
       </c>
       <c r="J45" s="27" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K45" s="23" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Very Weak</t>
         </is>
       </c>
       <c r="L45" s="28" t="n">
-        <v>51.02913306530867</v>
+        <v>37.08635589509742</v>
       </c>
     </row>
     <row r="46">
@@ -2538,11 +2538,11 @@
       </c>
       <c r="H46" s="31" t="inlineStr">
         <is>
-          <t>XLF</t>
+          <t>XLI</t>
         </is>
       </c>
       <c r="I46" s="33" t="n">
-        <v>-0.0008939609652732772</v>
+        <v>0.001778126850990658</v>
       </c>
       <c r="J46" s="34" t="n">
         <v>1</v>
@@ -2553,7 +2553,7 @@
         </is>
       </c>
       <c r="L46" s="35" t="n">
-        <v>37.08635589509742</v>
+        <v>31.46829525388786</v>
       </c>
     </row>
     <row r="47">
@@ -2578,11 +2578,11 @@
       </c>
       <c r="H47" s="24" t="inlineStr">
         <is>
-          <t>XLI</t>
+          <t>XLP</t>
         </is>
       </c>
       <c r="I47" s="26" t="n">
-        <v>0.001778126850990658</v>
+        <v>0.00192002915155598</v>
       </c>
       <c r="J47" s="27" t="n">
         <v>1</v>
@@ -2593,7 +2593,7 @@
         </is>
       </c>
       <c r="L47" s="28" t="n">
-        <v>31.46829525388786</v>
+        <v>42.86077646368995</v>
       </c>
     </row>
     <row r="48">
@@ -2618,11 +2618,11 @@
       </c>
       <c r="H48" s="31" t="inlineStr">
         <is>
-          <t>XLP</t>
+          <t>XLRE</t>
         </is>
       </c>
       <c r="I48" s="33" t="n">
-        <v>0.00192002915155598</v>
+        <v>0.003036609419477143</v>
       </c>
       <c r="J48" s="34" t="n">
         <v>1</v>
@@ -2633,7 +2633,7 @@
         </is>
       </c>
       <c r="L48" s="35" t="n">
-        <v>42.86077646368995</v>
+        <v>34.74774022483162</v>
       </c>
     </row>
     <row r="49">
@@ -2658,22 +2658,22 @@
       </c>
       <c r="H49" s="24" t="inlineStr">
         <is>
-          <t>XLRE</t>
+          <t>IWM</t>
         </is>
       </c>
       <c r="I49" s="26" t="n">
-        <v>0.003036609419477143</v>
+        <v>0.005318326206797064</v>
       </c>
       <c r="J49" s="27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K49" s="23" t="inlineStr">
         <is>
-          <t>Very Weak</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="L49" s="28" t="n">
-        <v>34.74774022483162</v>
+        <v>36.08911153912589</v>
       </c>
     </row>
     <row r="50">
@@ -2698,22 +2698,22 @@
       </c>
       <c r="H50" s="31" t="inlineStr">
         <is>
-          <t>IWM</t>
+          <t>XLV</t>
         </is>
       </c>
       <c r="I50" s="33" t="n">
-        <v>0.005318326206797064</v>
+        <v>0.006198922689683251</v>
       </c>
       <c r="J50" s="34" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="K50" s="30" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Strong</t>
         </is>
       </c>
       <c r="L50" s="35" t="n">
-        <v>36.08911153912589</v>
+        <v>51.05041102212405</v>
       </c>
     </row>
     <row r="51">
@@ -2738,22 +2738,22 @@
       </c>
       <c r="H51" s="24" t="inlineStr">
         <is>
-          <t>XLV</t>
+          <t>XLB</t>
         </is>
       </c>
       <c r="I51" s="26" t="n">
-        <v>0.006198922689683251</v>
+        <v>0.006949929902287488</v>
       </c>
       <c r="J51" s="27" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="K51" s="23" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="L51" s="28" t="n">
-        <v>51.05041102212405</v>
+        <v>40.17082520459962</v>
       </c>
     </row>
     <row r="52">
@@ -2778,22 +2778,22 @@
       </c>
       <c r="H52" s="31" t="inlineStr">
         <is>
-          <t>XLB</t>
+          <t>XLE</t>
         </is>
       </c>
       <c r="I52" s="33" t="n">
-        <v>0.006949929902287488</v>
+        <v>0.007028027271839044</v>
       </c>
       <c r="J52" s="34" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="K52" s="30" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Strong</t>
         </is>
       </c>
       <c r="L52" s="35" t="n">
-        <v>40.17082520459962</v>
+        <v>56.62949827527311</v>
       </c>
     </row>
   </sheetData>
@@ -3104,7 +3104,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 17 Sep 2026, 10:52 PM · Yahoo Finance data</t>
+          <t>Built 17 Sep 2026, 11:32 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -3129,22 +3129,22 @@
       </c>
       <c r="Y3" s="44" t="inlineStr">
         <is>
-          <t>36 of 40</t>
+          <t>36 of 39</t>
         </is>
       </c>
       <c r="AA3" s="45" t="inlineStr">
         <is>
-          <t>4 of 40</t>
+          <t>3 of 39</t>
         </is>
       </c>
       <c r="AC3" s="46" t="inlineStr">
         <is>
-          <t>5.4 / 9</t>
+          <t>5.5 / 9</t>
         </is>
       </c>
       <c r="AE3" s="47" t="inlineStr">
         <is>
-          <t>24 of 40</t>
+          <t>24 of 39</t>
         </is>
       </c>
     </row>
@@ -6769,7 +6769,7 @@
       </c>
       <c r="AX25" s="90" t="inlineStr">
         <is>
-          <t>Dow Jones Futures: S&amp;P 500, Nasdaq Rebound Above Key Level; Moderna, AMD, SpaceX Flash Buy Signals</t>
+          <t>Dow Jones Futures Fall After S&amp;P 500, Nasdaq Rebound Above Key Level; Moderna, AMD, SpaceX Flash Buy Signals</t>
         </is>
       </c>
       <c r="AY25" s="90" t="inlineStr">
@@ -6957,17 +6957,17 @@
       </c>
       <c r="AX26" s="79" t="inlineStr">
         <is>
+          <t>Amazon Can Absorb the 21 Air Suspension. Replacing Its Fleet Is a Different Story.</t>
+        </is>
+      </c>
+      <c r="AY26" s="79" t="inlineStr">
+        <is>
           <t>AI Power Stocks Rally After Generac's Deal For Amazon Data Centers</t>
         </is>
       </c>
-      <c r="AY26" s="79" t="inlineStr">
+      <c r="AZ26" s="79" t="inlineStr">
         <is>
           <t>Amazon, Walmart Face FTC Probe Call Over AI Chatbots And ‘Made In USA’ Claims — AMZN, WMT Stocks In Focus</t>
-        </is>
-      </c>
-      <c r="AZ26" s="79" t="inlineStr">
-        <is>
-          <t>Qualcomm Gains 2% as Amazon's Warrant Prices AI Commitment</t>
         </is>
       </c>
     </row>
@@ -7918,171 +7918,57 @@
           <t>CRWV</t>
         </is>
       </c>
-      <c r="C32" s="26" t="n">
-        <v>-0.04163168907292192</v>
-      </c>
-      <c r="D32" s="27" t="n">
-        <v>25</v>
-      </c>
-      <c r="E32" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F32" s="23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G32" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H32" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I32" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J32" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K32" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L32" s="23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M32" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N32" s="69" t="n">
-        <v>1</v>
-      </c>
-      <c r="O32" s="23" t="inlineStr">
-        <is>
-          <t>Very Weak</t>
-        </is>
-      </c>
-      <c r="P32" s="25" t="inlineStr">
-        <is>
-          <t>Below every average</t>
-        </is>
-      </c>
+      <c r="C32" s="26" t="n"/>
+      <c r="D32" s="27" t="n"/>
+      <c r="E32" s="23" t="n"/>
+      <c r="F32" s="23" t="n"/>
+      <c r="G32" s="23" t="n"/>
+      <c r="H32" s="23" t="n"/>
+      <c r="I32" s="23" t="n"/>
+      <c r="J32" s="23" t="n"/>
+      <c r="K32" s="23" t="n"/>
+      <c r="L32" s="23" t="n"/>
+      <c r="M32" s="23" t="n"/>
+      <c r="N32" s="69" t="n"/>
+      <c r="O32" s="23" t="n"/>
+      <c r="P32" s="25" t="n"/>
       <c r="Q32" s="25" t="inlineStr">
         <is>
           <t>CoreWeave, Inc.</t>
         </is>
       </c>
-      <c r="R32" s="70" t="n">
-        <v>79.87999725341797</v>
-      </c>
-      <c r="S32" s="71" t="n">
-        <v>-3.470001220703125</v>
-      </c>
-      <c r="T32" s="72" t="n">
-        <v>81.44999694824219</v>
-      </c>
-      <c r="U32" s="72" t="n">
-        <v>82.43000030517578</v>
-      </c>
-      <c r="V32" s="72" t="n">
-        <v>78.26999664306641</v>
-      </c>
-      <c r="W32" s="73" t="n">
-        <v>79167396</v>
-      </c>
-      <c r="X32" s="74" t="n">
-        <v>3.382555687811552</v>
-      </c>
-      <c r="Y32" s="28" t="n">
-        <v>42.43570914735687</v>
-      </c>
-      <c r="Z32" s="28" t="n">
-        <v>6.117023666486464</v>
-      </c>
-      <c r="AA32" s="28" t="n">
-        <v>11.18271937790753</v>
-      </c>
-      <c r="AB32" s="75" t="n">
-        <v>-1.401287641096843</v>
-      </c>
-      <c r="AC32" s="75" t="n">
-        <v>-0.4341544543350912</v>
-      </c>
-      <c r="AD32" s="75" t="n">
-        <v>-0.9671331867617519</v>
-      </c>
-      <c r="AE32" s="72" t="n">
-        <v>84.58512701199008</v>
-      </c>
-      <c r="AF32" s="72" t="n">
-        <v>86.74166549208448</v>
-      </c>
-      <c r="AG32" s="72" t="n">
-        <v>85.23660034179687</v>
-      </c>
-      <c r="AH32" s="72" t="n">
-        <v>96.07024986267089</v>
-      </c>
-      <c r="AI32" s="72" t="n">
-        <v>92.05597499847413</v>
-      </c>
-      <c r="AJ32" s="72" t="n">
-        <v>96.09830641724119</v>
-      </c>
-      <c r="AK32" s="72" t="n">
-        <v>86.62700042724609</v>
-      </c>
-      <c r="AL32" s="72" t="n">
-        <v>77.15569443725099</v>
-      </c>
-      <c r="AM32" s="76" t="n">
-        <v>0.1438187520836496</v>
-      </c>
-      <c r="AN32" s="29" t="n">
-        <v>21.86686816646642</v>
-      </c>
-      <c r="AO32" s="77" t="n">
-        <v>7.561065908090909</v>
-      </c>
-      <c r="AP32" s="72" t="n">
-        <v>153.1999969482422</v>
-      </c>
-      <c r="AQ32" s="72" t="n">
-        <v>60.54999923706055</v>
-      </c>
-      <c r="AR32" s="29" t="n">
-        <v>-47.85900858705303</v>
-      </c>
-      <c r="AS32" s="78" t="n">
-        <v>20.86346302631861</v>
-      </c>
-      <c r="AT32" s="26" t="n">
-        <v>-0.1036804893222295</v>
-      </c>
-      <c r="AU32" s="26" t="n">
-        <v>-0.1426424941152039</v>
-      </c>
-      <c r="AV32" s="26" t="n">
-        <v>-0.3066574265411678</v>
-      </c>
-      <c r="AW32" s="26" t="n">
-        <v>0.1154866160114365</v>
-      </c>
+      <c r="R32" s="70" t="n"/>
+      <c r="S32" s="71" t="n"/>
+      <c r="T32" s="72" t="n"/>
+      <c r="U32" s="72" t="n"/>
+      <c r="V32" s="72" t="n"/>
+      <c r="W32" s="73" t="n"/>
+      <c r="X32" s="74" t="n"/>
+      <c r="Y32" s="28" t="n"/>
+      <c r="Z32" s="28" t="n"/>
+      <c r="AA32" s="28" t="n"/>
+      <c r="AB32" s="75" t="n"/>
+      <c r="AC32" s="75" t="n"/>
+      <c r="AD32" s="75" t="n"/>
+      <c r="AE32" s="72" t="n"/>
+      <c r="AF32" s="72" t="n"/>
+      <c r="AG32" s="72" t="n"/>
+      <c r="AH32" s="72" t="n"/>
+      <c r="AI32" s="72" t="n"/>
+      <c r="AJ32" s="72" t="n"/>
+      <c r="AK32" s="72" t="n"/>
+      <c r="AL32" s="72" t="n"/>
+      <c r="AM32" s="76" t="n"/>
+      <c r="AN32" s="29" t="n"/>
+      <c r="AO32" s="77" t="n"/>
+      <c r="AP32" s="72" t="n"/>
+      <c r="AQ32" s="72" t="n"/>
+      <c r="AR32" s="29" t="n"/>
+      <c r="AS32" s="78" t="n"/>
+      <c r="AT32" s="26" t="n"/>
+      <c r="AU32" s="26" t="n"/>
+      <c r="AV32" s="26" t="n"/>
+      <c r="AW32" s="26" t="n"/>
       <c r="AX32" s="79" t="inlineStr">
         <is>
           <t>10-year Treasury yield eases, oil falls to $100: AlphaCheck</t>
@@ -9401,17 +9287,17 @@
       </c>
       <c r="AX39" s="90" t="inlineStr">
         <is>
+          <t>Why Was Micron Technology Stock Up Today?</t>
+        </is>
+      </c>
+      <c r="AY39" s="90" t="inlineStr">
+        <is>
           <t>Prediction: A $5,000 Investment Split Between Micron and Sandisk Will Triple Before 2028</t>
         </is>
       </c>
-      <c r="AY39" s="90" t="inlineStr">
+      <c r="AZ39" s="90" t="inlineStr">
         <is>
           <t>Micron, Qualcomm, Nova, Lattice Semiconductor, and Workday Shares Are Soaring, What You Need To Know</t>
-        </is>
-      </c>
-      <c r="AZ39" s="90" t="inlineStr">
-        <is>
-          <t>Micron Jumps 5.5% as Labor Claims AI's Margin Windfall</t>
         </is>
       </c>
     </row>
@@ -10153,17 +10039,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
+          <t>China's Homegrown AI Chip Push Just Got Faster. Is This a Real Threat to Nvidia?</t>
+        </is>
+      </c>
+      <c r="AY43" s="90" t="inlineStr">
+        <is>
           <t>Trump-Xi Dinner Next Week Brings AI Titans To The Table — OpenAI, NVDA, and QCOM CEOs To Attend, Says Report</t>
         </is>
       </c>
-      <c r="AY43" s="90" t="inlineStr">
+      <c r="AZ43" s="90" t="inlineStr">
         <is>
           <t>S&amp;P 500, Nasdaq, Dow End Higher As Drop In Oil Prices Allays Inflationary Concerns — NVDA, MCD, CRWV, LMT, ...</t>
-        </is>
-      </c>
-      <c r="AZ43" s="90" t="inlineStr">
-        <is>
-          <t>Michael Burry returns to a difficult corner of Wall Street</t>
         </is>
       </c>
     </row>
@@ -11093,17 +10979,17 @@
       </c>
       <c r="AX48" s="79" t="inlineStr">
         <is>
+          <t>Tesla Posted Negative $1.1 Billion in Free Cash Flow Last Quarter as Elon Musk Ramps Up Spending on Robotax...</t>
+        </is>
+      </c>
+      <c r="AY48" s="79" t="inlineStr">
+        <is>
           <t>Tesla (TSLA) Exceeds Market Returns: Some Facts to Consider</t>
         </is>
       </c>
-      <c r="AY48" s="79" t="inlineStr">
+      <c r="AZ48" s="79" t="inlineStr">
         <is>
           <t>Rivian Reports Q3 Deliveries for the R2 SUV in October. Here's How Investors Should Prepare.</t>
-        </is>
-      </c>
-      <c r="AZ48" s="79" t="inlineStr">
-        <is>
-          <t>Tesla Jumps 2% as 30 Megawatts Build a Semi Beachhead</t>
         </is>
       </c>
     </row>
@@ -11640,7 +11526,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 17 Sep 2026, 10:52 PM · Yahoo Finance data</t>
+          <t>Built 17 Sep 2026, 11:32 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -11665,12 +11551,12 @@
       </c>
       <c r="Y3" s="44" t="inlineStr">
         <is>
-          <t>19 of 40</t>
+          <t>18 of 39</t>
         </is>
       </c>
       <c r="AA3" s="45" t="inlineStr">
         <is>
-          <t>20 of 40</t>
+          <t>20 of 39</t>
         </is>
       </c>
       <c r="AC3" s="46" t="inlineStr">
@@ -11680,7 +11566,7 @@
       </c>
       <c r="AE3" s="47" t="inlineStr">
         <is>
-          <t>9 of 40</t>
+          <t>9 of 39</t>
         </is>
       </c>
     </row>
@@ -14774,7 +14660,7 @@
         <v>0.003229333421998382</v>
       </c>
       <c r="D24" s="27" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E24" s="23" t="inlineStr">
         <is>
@@ -14950,7 +14836,7 @@
         <v>0.01646169692983013</v>
       </c>
       <c r="D25" s="34" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E25" s="30" t="inlineStr">
         <is>
@@ -15126,7 +15012,7 @@
         <v>-0.009902550008897171</v>
       </c>
       <c r="D26" s="27" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E26" s="23" t="inlineStr">
         <is>
@@ -15302,7 +15188,7 @@
         <v>-0.00371299037639905</v>
       </c>
       <c r="D27" s="34" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E27" s="30" t="inlineStr">
         <is>
@@ -15478,7 +15364,7 @@
         <v>0.008890517637205164</v>
       </c>
       <c r="D28" s="27" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E28" s="23" t="inlineStr">
         <is>
@@ -15654,7 +15540,7 @@
         <v>0.008507741978993844</v>
       </c>
       <c r="D29" s="34" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E29" s="30" t="inlineStr">
         <is>
@@ -15830,7 +15716,7 @@
         <v>0.000707462374290424</v>
       </c>
       <c r="D30" s="27" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E30" s="23" t="inlineStr">
         <is>
@@ -16006,7 +15892,7 @@
         <v>-0.003398723404290926</v>
       </c>
       <c r="D31" s="34" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E31" s="30" t="inlineStr">
         <is>
@@ -16178,171 +16064,57 @@
           <t>CRWV</t>
         </is>
       </c>
-      <c r="C32" s="26" t="n">
-        <v>0.03002966337322954</v>
-      </c>
-      <c r="D32" s="27" t="n">
-        <v>4</v>
-      </c>
-      <c r="E32" s="23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F32" s="23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G32" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H32" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I32" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J32" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K32" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L32" s="23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M32" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N32" s="69" t="n">
-        <v>2</v>
-      </c>
-      <c r="O32" s="23" t="inlineStr">
-        <is>
-          <t>Weak</t>
-        </is>
-      </c>
-      <c r="P32" s="25" t="inlineStr">
-        <is>
-          <t>Below every average</t>
-        </is>
-      </c>
+      <c r="C32" s="26" t="n"/>
+      <c r="D32" s="27" t="n"/>
+      <c r="E32" s="23" t="n"/>
+      <c r="F32" s="23" t="n"/>
+      <c r="G32" s="23" t="n"/>
+      <c r="H32" s="23" t="n"/>
+      <c r="I32" s="23" t="n"/>
+      <c r="J32" s="23" t="n"/>
+      <c r="K32" s="23" t="n"/>
+      <c r="L32" s="23" t="n"/>
+      <c r="M32" s="23" t="n"/>
+      <c r="N32" s="69" t="n"/>
+      <c r="O32" s="23" t="n"/>
+      <c r="P32" s="25" t="n"/>
       <c r="Q32" s="25" t="inlineStr">
         <is>
           <t>CoreWeave, Inc.</t>
         </is>
       </c>
-      <c r="R32" s="70" t="n">
-        <v>83.34999847412109</v>
-      </c>
-      <c r="S32" s="71" t="n">
-        <v>2.430000305175781</v>
-      </c>
-      <c r="T32" s="72" t="n">
-        <v>83.75</v>
-      </c>
-      <c r="U32" s="72" t="n">
-        <v>85.25800323486328</v>
-      </c>
-      <c r="V32" s="72" t="n">
-        <v>81.15699768066406</v>
-      </c>
-      <c r="W32" s="73" t="n">
-        <v>18787600</v>
-      </c>
-      <c r="X32" s="74" t="n">
-        <v>0.9040634397728533</v>
-      </c>
-      <c r="Y32" s="28" t="n">
-        <v>45.50313450220389</v>
-      </c>
-      <c r="Z32" s="28" t="n">
-        <v>16.90140887111217</v>
-      </c>
-      <c r="AA32" s="28" t="n">
-        <v>11.78247741933556</v>
-      </c>
-      <c r="AB32" s="75" t="n">
-        <v>-0.9256043807190508</v>
-      </c>
-      <c r="AC32" s="75" t="n">
-        <v>-0.1923711576446532</v>
-      </c>
-      <c r="AD32" s="75" t="n">
-        <v>-0.7332332230743976</v>
-      </c>
-      <c r="AE32" s="72" t="n">
-        <v>85.92944980015353</v>
-      </c>
-      <c r="AF32" s="72" t="n">
-        <v>87.42783231595114</v>
-      </c>
-      <c r="AG32" s="72" t="n">
-        <v>85.43900039672852</v>
-      </c>
-      <c r="AH32" s="72" t="n">
-        <v>96.3728498840332</v>
-      </c>
-      <c r="AI32" s="72" t="n">
-        <v>92.02217502593994</v>
-      </c>
-      <c r="AJ32" s="72" t="n">
-        <v>96.28660708545257</v>
-      </c>
-      <c r="AK32" s="72" t="n">
-        <v>87.1765007019043</v>
-      </c>
-      <c r="AL32" s="72" t="n">
-        <v>78.06639431835603</v>
-      </c>
-      <c r="AM32" s="76" t="n">
-        <v>0.2899858647812609</v>
-      </c>
-      <c r="AN32" s="29" t="n">
-        <v>20.90037179789959</v>
-      </c>
-      <c r="AO32" s="77" t="n">
-        <v>7.334863087064737</v>
-      </c>
-      <c r="AP32" s="72" t="n">
-        <v>153.1999969482422</v>
-      </c>
-      <c r="AQ32" s="72" t="n">
-        <v>60.54999923706055</v>
-      </c>
-      <c r="AR32" s="29" t="n">
-        <v>-45.59399469029987</v>
-      </c>
-      <c r="AS32" s="78" t="n">
-        <v>24.60874236406903</v>
-      </c>
-      <c r="AT32" s="26" t="n">
-        <v>-0.1220771399751976</v>
-      </c>
-      <c r="AU32" s="26" t="n">
-        <v>-0.2136792596781029</v>
-      </c>
-      <c r="AV32" s="26" t="n">
-        <v>-0.2877894613046337</v>
-      </c>
-      <c r="AW32" s="26" t="n">
-        <v>0.1639435520696317</v>
-      </c>
+      <c r="R32" s="70" t="n"/>
+      <c r="S32" s="71" t="n"/>
+      <c r="T32" s="72" t="n"/>
+      <c r="U32" s="72" t="n"/>
+      <c r="V32" s="72" t="n"/>
+      <c r="W32" s="73" t="n"/>
+      <c r="X32" s="74" t="n"/>
+      <c r="Y32" s="28" t="n"/>
+      <c r="Z32" s="28" t="n"/>
+      <c r="AA32" s="28" t="n"/>
+      <c r="AB32" s="75" t="n"/>
+      <c r="AC32" s="75" t="n"/>
+      <c r="AD32" s="75" t="n"/>
+      <c r="AE32" s="72" t="n"/>
+      <c r="AF32" s="72" t="n"/>
+      <c r="AG32" s="72" t="n"/>
+      <c r="AH32" s="72" t="n"/>
+      <c r="AI32" s="72" t="n"/>
+      <c r="AJ32" s="72" t="n"/>
+      <c r="AK32" s="72" t="n"/>
+      <c r="AL32" s="72" t="n"/>
+      <c r="AM32" s="76" t="n"/>
+      <c r="AN32" s="29" t="n"/>
+      <c r="AO32" s="77" t="n"/>
+      <c r="AP32" s="72" t="n"/>
+      <c r="AQ32" s="72" t="n"/>
+      <c r="AR32" s="29" t="n"/>
+      <c r="AS32" s="78" t="n"/>
+      <c r="AT32" s="26" t="n"/>
+      <c r="AU32" s="26" t="n"/>
+      <c r="AV32" s="26" t="n"/>
+      <c r="AW32" s="26" t="n"/>
       <c r="AX32" s="25" t="n"/>
       <c r="AY32" s="25" t="n"/>
       <c r="AZ32" s="25" t="n"/>
@@ -16534,7 +16306,7 @@
         <v>-0.00606275772083209</v>
       </c>
       <c r="D34" s="27" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E34" s="23" t="inlineStr">
         <is>
@@ -16710,7 +16482,7 @@
         <v>0.02501195418546942</v>
       </c>
       <c r="D35" s="34" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E35" s="30" t="inlineStr">
         <is>
@@ -17062,7 +16834,7 @@
         <v>-0.01371903643226224</v>
       </c>
       <c r="D37" s="34" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E37" s="30" t="inlineStr">
         <is>
@@ -17238,7 +17010,7 @@
         <v>-0.02638893238637796</v>
       </c>
       <c r="D38" s="27" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E38" s="23" t="inlineStr">
         <is>
@@ -17414,7 +17186,7 @@
         <v>-0.00113194029819319</v>
       </c>
       <c r="D39" s="34" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E39" s="30" t="inlineStr">
         <is>
@@ -17590,7 +17362,7 @@
         <v>0.009644596841841935</v>
       </c>
       <c r="D40" s="27" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E40" s="23" t="inlineStr">
         <is>
@@ -17766,7 +17538,7 @@
         <v>-0.01912705821032035</v>
       </c>
       <c r="D41" s="34" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E41" s="30" t="inlineStr">
         <is>
@@ -18118,7 +17890,7 @@
         <v>0.008153818836165172</v>
       </c>
       <c r="D43" s="34" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E43" s="30" t="inlineStr">
         <is>
@@ -18294,7 +18066,7 @@
         <v>0.0103152457376019</v>
       </c>
       <c r="D44" s="27" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E44" s="23" t="inlineStr">
         <is>
@@ -18470,7 +18242,7 @@
         <v>-0.01576148384327447</v>
       </c>
       <c r="D45" s="34" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E45" s="30" t="inlineStr">
         <is>
@@ -18646,7 +18418,7 @@
         <v>0.002360370223127184</v>
       </c>
       <c r="D46" s="27" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E46" s="23" t="inlineStr">
         <is>
@@ -18822,7 +18594,7 @@
         <v>-0.007136380149352251</v>
       </c>
       <c r="D47" s="34" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E47" s="30" t="inlineStr">
         <is>
@@ -18998,7 +18770,7 @@
         <v>0.004206629806734918</v>
       </c>
       <c r="D48" s="27" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E48" s="23" t="inlineStr">
         <is>
@@ -19576,7 +19348,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 17 Sep 2026, 10:52 PM · Yahoo Finance data</t>
+          <t>Built 17 Sep 2026, 11:32 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19601,22 +19373,22 @@
       </c>
       <c r="Y3" s="44" t="inlineStr">
         <is>
-          <t>11 of 40</t>
+          <t>11 of 39</t>
         </is>
       </c>
       <c r="AA3" s="45" t="inlineStr">
         <is>
-          <t>29 of 40</t>
+          <t>28 of 39</t>
         </is>
       </c>
       <c r="AC3" s="46" t="inlineStr">
         <is>
-          <t>3.1 / 9</t>
+          <t>3.2 / 9</t>
         </is>
       </c>
       <c r="AE3" s="47" t="inlineStr">
         <is>
-          <t>8 of 40</t>
+          <t>8 of 39</t>
         </is>
       </c>
     </row>
@@ -24114,171 +23886,57 @@
           <t>CRWV</t>
         </is>
       </c>
-      <c r="C32" s="26" t="n">
-        <v>-0.02482532061522447</v>
-      </c>
-      <c r="D32" s="27" t="n">
-        <v>22</v>
-      </c>
-      <c r="E32" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F32" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G32" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H32" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I32" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J32" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K32" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L32" s="23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M32" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N32" s="69" t="n">
-        <v>0</v>
-      </c>
-      <c r="O32" s="23" t="inlineStr">
-        <is>
-          <t>Very Weak</t>
-        </is>
-      </c>
-      <c r="P32" s="25" t="inlineStr">
-        <is>
-          <t>Below every average</t>
-        </is>
-      </c>
+      <c r="C32" s="26" t="n"/>
+      <c r="D32" s="27" t="n"/>
+      <c r="E32" s="23" t="n"/>
+      <c r="F32" s="23" t="n"/>
+      <c r="G32" s="23" t="n"/>
+      <c r="H32" s="23" t="n"/>
+      <c r="I32" s="23" t="n"/>
+      <c r="J32" s="23" t="n"/>
+      <c r="K32" s="23" t="n"/>
+      <c r="L32" s="23" t="n"/>
+      <c r="M32" s="23" t="n"/>
+      <c r="N32" s="69" t="n"/>
+      <c r="O32" s="23" t="n"/>
+      <c r="P32" s="25" t="n"/>
       <c r="Q32" s="25" t="inlineStr">
         <is>
           <t>CoreWeave, Inc.</t>
         </is>
       </c>
-      <c r="R32" s="70" t="n">
-        <v>80.91999816894531</v>
-      </c>
-      <c r="S32" s="71" t="n">
-        <v>-2.060005187988281</v>
-      </c>
-      <c r="T32" s="72" t="n">
-        <v>82.62000274658203</v>
-      </c>
-      <c r="U32" s="72" t="n">
-        <v>83.86000061035156</v>
-      </c>
-      <c r="V32" s="72" t="n">
-        <v>80.51999664306641</v>
-      </c>
-      <c r="W32" s="73" t="n">
-        <v>15675200</v>
-      </c>
-      <c r="X32" s="74" t="n">
-        <v>0.7209187722323569</v>
-      </c>
-      <c r="Y32" s="28" t="n">
-        <v>42.81522285543067</v>
-      </c>
-      <c r="Z32" s="28" t="n">
-        <v>7.39436451555131</v>
-      </c>
-      <c r="AA32" s="28" t="n">
-        <v>12.48624130820947</v>
-      </c>
-      <c r="AB32" s="75" t="n">
-        <v>-0.65830544349798</v>
-      </c>
-      <c r="AC32" s="75" t="n">
-        <v>-0.009062851876053837</v>
-      </c>
-      <c r="AD32" s="75" t="n">
-        <v>-0.6492425916219262</v>
-      </c>
-      <c r="AE32" s="72" t="n">
-        <v>86.66643589330566</v>
-      </c>
-      <c r="AF32" s="72" t="n">
-        <v>87.83561570013414</v>
-      </c>
-      <c r="AG32" s="72" t="n">
-        <v>85.44260040283203</v>
-      </c>
-      <c r="AH32" s="72" t="n">
-        <v>96.71354988098145</v>
-      </c>
-      <c r="AI32" s="72" t="n">
-        <v>91.97687503814697</v>
-      </c>
-      <c r="AJ32" s="72" t="n">
-        <v>96.95650993936681</v>
-      </c>
-      <c r="AK32" s="72" t="n">
-        <v>87.66750068664551</v>
-      </c>
-      <c r="AL32" s="72" t="n">
-        <v>78.37849143392421</v>
-      </c>
-      <c r="AM32" s="76" t="n">
-        <v>0.1368018195415482</v>
-      </c>
-      <c r="AN32" s="29" t="n">
-        <v>21.19145448419589</v>
-      </c>
-      <c r="AO32" s="77" t="n">
-        <v>7.723916552789404</v>
-      </c>
-      <c r="AP32" s="72" t="n">
-        <v>153.1999969482422</v>
-      </c>
-      <c r="AQ32" s="72" t="n">
-        <v>60.54999923706055</v>
-      </c>
-      <c r="AR32" s="29" t="n">
-        <v>-47.18015680099281</v>
-      </c>
-      <c r="AS32" s="78" t="n">
-        <v>21.98596808969632</v>
-      </c>
-      <c r="AT32" s="26" t="n">
-        <v>-0.1894220506387583</v>
-      </c>
-      <c r="AU32" s="26" t="n">
-        <v>-0.2312369701055452</v>
-      </c>
-      <c r="AV32" s="26" t="n">
-        <v>-0.2416830769074577</v>
-      </c>
-      <c r="AW32" s="26" t="n">
-        <v>0.1300097399698659</v>
-      </c>
+      <c r="R32" s="70" t="n"/>
+      <c r="S32" s="71" t="n"/>
+      <c r="T32" s="72" t="n"/>
+      <c r="U32" s="72" t="n"/>
+      <c r="V32" s="72" t="n"/>
+      <c r="W32" s="73" t="n"/>
+      <c r="X32" s="74" t="n"/>
+      <c r="Y32" s="28" t="n"/>
+      <c r="Z32" s="28" t="n"/>
+      <c r="AA32" s="28" t="n"/>
+      <c r="AB32" s="75" t="n"/>
+      <c r="AC32" s="75" t="n"/>
+      <c r="AD32" s="75" t="n"/>
+      <c r="AE32" s="72" t="n"/>
+      <c r="AF32" s="72" t="n"/>
+      <c r="AG32" s="72" t="n"/>
+      <c r="AH32" s="72" t="n"/>
+      <c r="AI32" s="72" t="n"/>
+      <c r="AJ32" s="72" t="n"/>
+      <c r="AK32" s="72" t="n"/>
+      <c r="AL32" s="72" t="n"/>
+      <c r="AM32" s="76" t="n"/>
+      <c r="AN32" s="29" t="n"/>
+      <c r="AO32" s="77" t="n"/>
+      <c r="AP32" s="72" t="n"/>
+      <c r="AQ32" s="72" t="n"/>
+      <c r="AR32" s="29" t="n"/>
+      <c r="AS32" s="78" t="n"/>
+      <c r="AT32" s="26" t="n"/>
+      <c r="AU32" s="26" t="n"/>
+      <c r="AV32" s="26" t="n"/>
+      <c r="AW32" s="26" t="n"/>
       <c r="AX32" s="25" t="n"/>
       <c r="AY32" s="25" t="n"/>
       <c r="AZ32" s="25" t="n"/>
@@ -24646,7 +24304,7 @@
         <v>-0.03683104946329141</v>
       </c>
       <c r="D35" s="34" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E35" s="30" t="inlineStr">
         <is>
@@ -25174,7 +24832,7 @@
         <v>-0.05360008914145631</v>
       </c>
       <c r="D38" s="27" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E38" s="23" t="inlineStr">
         <is>
@@ -25702,7 +25360,7 @@
         <v>-0.03012945938919442</v>
       </c>
       <c r="D41" s="34" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E41" s="30" t="inlineStr">
         <is>
@@ -27512,7 +27170,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 17 Sep 2026, 10:52 PM · Yahoo Finance data</t>
+          <t>Built 17 Sep 2026, 11:32 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27537,22 +27195,22 @@
       </c>
       <c r="Y3" s="44" t="inlineStr">
         <is>
-          <t>11 of 40</t>
+          <t>11 of 39</t>
         </is>
       </c>
       <c r="AA3" s="45" t="inlineStr">
         <is>
-          <t>29 of 40</t>
+          <t>28 of 39</t>
         </is>
       </c>
       <c r="AC3" s="46" t="inlineStr">
         <is>
-          <t>3.9 / 9</t>
+          <t>4.0 / 9</t>
         </is>
       </c>
       <c r="AE3" s="47" t="inlineStr">
         <is>
-          <t>15 of 40</t>
+          <t>15 of 39</t>
         </is>
       </c>
     </row>
@@ -31350,7 +31008,7 @@
         <v>-0.09736022208599437</v>
       </c>
       <c r="D28" s="27" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E28" s="23" t="inlineStr">
         <is>
@@ -32050,171 +31708,57 @@
           <t>CRWV</t>
         </is>
       </c>
-      <c r="C32" s="26" t="n">
-        <v>-0.06753561805941777</v>
-      </c>
-      <c r="D32" s="27" t="n">
-        <v>23</v>
-      </c>
-      <c r="E32" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F32" s="23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G32" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H32" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I32" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J32" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K32" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L32" s="23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M32" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N32" s="69" t="n">
-        <v>1</v>
-      </c>
-      <c r="O32" s="23" t="inlineStr">
-        <is>
-          <t>Very Weak</t>
-        </is>
-      </c>
-      <c r="P32" s="25" t="inlineStr">
-        <is>
-          <t>Below every average</t>
-        </is>
-      </c>
+      <c r="C32" s="26" t="n"/>
+      <c r="D32" s="27" t="n"/>
+      <c r="E32" s="23" t="n"/>
+      <c r="F32" s="23" t="n"/>
+      <c r="G32" s="23" t="n"/>
+      <c r="H32" s="23" t="n"/>
+      <c r="I32" s="23" t="n"/>
+      <c r="J32" s="23" t="n"/>
+      <c r="K32" s="23" t="n"/>
+      <c r="L32" s="23" t="n"/>
+      <c r="M32" s="23" t="n"/>
+      <c r="N32" s="69" t="n"/>
+      <c r="O32" s="23" t="n"/>
+      <c r="P32" s="25" t="n"/>
       <c r="Q32" s="25" t="inlineStr">
         <is>
           <t>CoreWeave, Inc.</t>
         </is>
       </c>
-      <c r="R32" s="70" t="n">
-        <v>82.98000335693359</v>
-      </c>
-      <c r="S32" s="71" t="n">
-        <v>-6.009994506835938</v>
-      </c>
-      <c r="T32" s="72" t="n">
-        <v>82.65000152587891</v>
-      </c>
-      <c r="U32" s="72" t="n">
-        <v>85.93000030517578</v>
-      </c>
-      <c r="V32" s="72" t="n">
-        <v>82.08000183105469</v>
-      </c>
-      <c r="W32" s="73" t="n">
-        <v>26522600</v>
-      </c>
-      <c r="X32" s="74" t="n">
-        <v>1.174630295670459</v>
-      </c>
-      <c r="Y32" s="28" t="n">
-        <v>44.54470820082564</v>
-      </c>
-      <c r="Z32" s="28" t="n">
-        <v>15.4538535012835</v>
-      </c>
-      <c r="AA32" s="28" t="n">
-        <v>13.433430018822</v>
-      </c>
-      <c r="AB32" s="75" t="n">
-        <v>-0.06014123519430825</v>
-      </c>
-      <c r="AC32" s="75" t="n">
-        <v>0.1532477960294277</v>
-      </c>
-      <c r="AD32" s="75" t="n">
-        <v>-0.213389031223736</v>
-      </c>
-      <c r="AE32" s="72" t="n">
-        <v>88.30827524312289</v>
-      </c>
-      <c r="AF32" s="72" t="n">
-        <v>88.52717745325302</v>
-      </c>
-      <c r="AG32" s="72" t="n">
-        <v>85.55340042114258</v>
-      </c>
-      <c r="AH32" s="72" t="n">
-        <v>97.12974990844727</v>
-      </c>
-      <c r="AI32" s="72" t="n">
-        <v>91.92872505187988</v>
-      </c>
-      <c r="AJ32" s="72" t="n">
-        <v>100.6733506814363</v>
-      </c>
-      <c r="AK32" s="72" t="n">
-        <v>88.92150077819824</v>
-      </c>
-      <c r="AL32" s="72" t="n">
-        <v>77.16965087496015</v>
-      </c>
-      <c r="AM32" s="76" t="n">
-        <v>0.2472101213772508</v>
-      </c>
-      <c r="AN32" s="29" t="n">
-        <v>26.43196482378623</v>
-      </c>
-      <c r="AO32" s="77" t="n">
-        <v>7.801944536326479</v>
-      </c>
-      <c r="AP32" s="72" t="n">
-        <v>153.1999969482422</v>
-      </c>
-      <c r="AQ32" s="72" t="n">
-        <v>60.54999923706055</v>
-      </c>
-      <c r="AR32" s="29" t="n">
-        <v>-45.83550586820968</v>
-      </c>
-      <c r="AS32" s="78" t="n">
-        <v>24.20939522286253</v>
-      </c>
-      <c r="AT32" s="26" t="n">
-        <v>-0.07139656680663564</v>
-      </c>
-      <c r="AU32" s="26" t="n">
-        <v>-0.2193056483000605</v>
-      </c>
-      <c r="AV32" s="26" t="n">
-        <v>-0.1747389275143046</v>
-      </c>
-      <c r="AW32" s="26" t="n">
-        <v>0.1587767441652339</v>
-      </c>
+      <c r="R32" s="70" t="n"/>
+      <c r="S32" s="71" t="n"/>
+      <c r="T32" s="72" t="n"/>
+      <c r="U32" s="72" t="n"/>
+      <c r="V32" s="72" t="n"/>
+      <c r="W32" s="73" t="n"/>
+      <c r="X32" s="74" t="n"/>
+      <c r="Y32" s="28" t="n"/>
+      <c r="Z32" s="28" t="n"/>
+      <c r="AA32" s="28" t="n"/>
+      <c r="AB32" s="75" t="n"/>
+      <c r="AC32" s="75" t="n"/>
+      <c r="AD32" s="75" t="n"/>
+      <c r="AE32" s="72" t="n"/>
+      <c r="AF32" s="72" t="n"/>
+      <c r="AG32" s="72" t="n"/>
+      <c r="AH32" s="72" t="n"/>
+      <c r="AI32" s="72" t="n"/>
+      <c r="AJ32" s="72" t="n"/>
+      <c r="AK32" s="72" t="n"/>
+      <c r="AL32" s="72" t="n"/>
+      <c r="AM32" s="76" t="n"/>
+      <c r="AN32" s="29" t="n"/>
+      <c r="AO32" s="77" t="n"/>
+      <c r="AP32" s="72" t="n"/>
+      <c r="AQ32" s="72" t="n"/>
+      <c r="AR32" s="29" t="n"/>
+      <c r="AS32" s="78" t="n"/>
+      <c r="AT32" s="26" t="n"/>
+      <c r="AU32" s="26" t="n"/>
+      <c r="AV32" s="26" t="n"/>
+      <c r="AW32" s="26" t="n"/>
       <c r="AX32" s="25" t="n"/>
       <c r="AY32" s="25" t="n"/>
       <c r="AZ32" s="25" t="n"/>
@@ -33814,7 +33358,7 @@
         <v>-0.132973987483646</v>
       </c>
       <c r="D42" s="27" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E42" s="23" t="inlineStr">
         <is>
@@ -35448,7 +34992,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 17 Sep 2026, 10:52 PM · Yahoo Finance data</t>
+          <t>Built 17 Sep 2026, 11:32 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35473,12 +35017,12 @@
       </c>
       <c r="Y3" s="44" t="inlineStr">
         <is>
-          <t>31 of 40</t>
+          <t>31 of 39</t>
         </is>
       </c>
       <c r="AA3" s="45" t="inlineStr">
         <is>
-          <t>9 of 40</t>
+          <t>8 of 39</t>
         </is>
       </c>
       <c r="AC3" s="46" t="inlineStr">
@@ -35488,7 +35032,7 @@
       </c>
       <c r="AE3" s="47" t="inlineStr">
         <is>
-          <t>18 of 40</t>
+          <t>18 of 39</t>
         </is>
       </c>
     </row>
@@ -39814,7 +39358,7 @@
         <v>-0.007595954400309357</v>
       </c>
       <c r="D31" s="34" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E31" s="30" t="inlineStr">
         <is>
@@ -39986,171 +39530,57 @@
           <t>CRWV</t>
         </is>
       </c>
-      <c r="C32" s="26" t="n">
-        <v>-0.001458762105092992</v>
-      </c>
-      <c r="D32" s="27" t="n">
-        <v>21</v>
-      </c>
-      <c r="E32" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F32" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G32" s="23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H32" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I32" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J32" s="23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K32" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L32" s="23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M32" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N32" s="69" t="n">
-        <v>3</v>
-      </c>
-      <c r="O32" s="23" t="inlineStr">
-        <is>
-          <t>Weak</t>
-        </is>
-      </c>
-      <c r="P32" s="25" t="inlineStr">
-        <is>
-          <t>Long-term down, short-term mixed</t>
-        </is>
-      </c>
+      <c r="C32" s="26" t="n"/>
+      <c r="D32" s="27" t="n"/>
+      <c r="E32" s="23" t="n"/>
+      <c r="F32" s="23" t="n"/>
+      <c r="G32" s="23" t="n"/>
+      <c r="H32" s="23" t="n"/>
+      <c r="I32" s="23" t="n"/>
+      <c r="J32" s="23" t="n"/>
+      <c r="K32" s="23" t="n"/>
+      <c r="L32" s="23" t="n"/>
+      <c r="M32" s="23" t="n"/>
+      <c r="N32" s="69" t="n"/>
+      <c r="O32" s="23" t="n"/>
+      <c r="P32" s="25" t="n"/>
       <c r="Q32" s="25" t="inlineStr">
         <is>
           <t>CoreWeave, Inc.</t>
         </is>
       </c>
-      <c r="R32" s="70" t="n">
-        <v>88.98999786376953</v>
-      </c>
-      <c r="S32" s="71" t="n">
-        <v>-0.1300048828125</v>
-      </c>
-      <c r="T32" s="72" t="n">
-        <v>91.08000183105469</v>
-      </c>
-      <c r="U32" s="72" t="n">
-        <v>91.98999786376953</v>
-      </c>
-      <c r="V32" s="72" t="n">
-        <v>88.62000274658203</v>
-      </c>
-      <c r="W32" s="73" t="n">
-        <v>17682400</v>
-      </c>
-      <c r="X32" s="74" t="n">
-        <v>0.7714734910698139</v>
-      </c>
-      <c r="Y32" s="28" t="n">
-        <v>50.01824729755901</v>
-      </c>
-      <c r="Z32" s="28" t="n">
-        <v>38.96713629037072</v>
-      </c>
-      <c r="AA32" s="28" t="n">
-        <v>14.24366789464034</v>
-      </c>
-      <c r="AB32" s="75" t="n">
-        <v>0.494462607684568</v>
-      </c>
-      <c r="AC32" s="75" t="n">
-        <v>0.2065950538353617</v>
-      </c>
-      <c r="AD32" s="75" t="n">
-        <v>0.2878675538492063</v>
-      </c>
-      <c r="AE32" s="72" t="n">
-        <v>89.83063863917697</v>
-      </c>
-      <c r="AF32" s="72" t="n">
-        <v>89.08189486288497</v>
-      </c>
-      <c r="AG32" s="72" t="n">
-        <v>85.52870040893555</v>
-      </c>
-      <c r="AH32" s="72" t="n">
-        <v>97.45154991149903</v>
-      </c>
-      <c r="AI32" s="72" t="n">
-        <v>91.88182502746582</v>
-      </c>
-      <c r="AJ32" s="72" t="n">
-        <v>103.4321808915975</v>
-      </c>
-      <c r="AK32" s="72" t="n">
-        <v>90.03550071716309</v>
-      </c>
-      <c r="AL32" s="72" t="n">
-        <v>76.63882054272864</v>
-      </c>
-      <c r="AM32" s="76" t="n">
-        <v>0.4609790321266032</v>
-      </c>
-      <c r="AN32" s="29" t="n">
-        <v>29.75866201159627</v>
-      </c>
-      <c r="AO32" s="77" t="n">
-        <v>7.23735248656006</v>
-      </c>
-      <c r="AP32" s="72" t="n">
-        <v>153.1999969482422</v>
-      </c>
-      <c r="AQ32" s="72" t="n">
-        <v>60.54999923706055</v>
-      </c>
-      <c r="AR32" s="29" t="n">
-        <v>-41.91253287437444</v>
-      </c>
-      <c r="AS32" s="78" t="n">
-        <v>30.69616765168754</v>
-      </c>
-      <c r="AT32" s="26" t="n">
-        <v>0.05238884145078315</v>
-      </c>
-      <c r="AU32" s="26" t="n">
-        <v>-0.1739534475931857</v>
-      </c>
-      <c r="AV32" s="26" t="n">
-        <v>-0.07050344840831013</v>
-      </c>
-      <c r="AW32" s="26" t="n">
-        <v>0.2427034926027583</v>
-      </c>
+      <c r="R32" s="70" t="n"/>
+      <c r="S32" s="71" t="n"/>
+      <c r="T32" s="72" t="n"/>
+      <c r="U32" s="72" t="n"/>
+      <c r="V32" s="72" t="n"/>
+      <c r="W32" s="73" t="n"/>
+      <c r="X32" s="74" t="n"/>
+      <c r="Y32" s="28" t="n"/>
+      <c r="Z32" s="28" t="n"/>
+      <c r="AA32" s="28" t="n"/>
+      <c r="AB32" s="75" t="n"/>
+      <c r="AC32" s="75" t="n"/>
+      <c r="AD32" s="75" t="n"/>
+      <c r="AE32" s="72" t="n"/>
+      <c r="AF32" s="72" t="n"/>
+      <c r="AG32" s="72" t="n"/>
+      <c r="AH32" s="72" t="n"/>
+      <c r="AI32" s="72" t="n"/>
+      <c r="AJ32" s="72" t="n"/>
+      <c r="AK32" s="72" t="n"/>
+      <c r="AL32" s="72" t="n"/>
+      <c r="AM32" s="76" t="n"/>
+      <c r="AN32" s="29" t="n"/>
+      <c r="AO32" s="77" t="n"/>
+      <c r="AP32" s="72" t="n"/>
+      <c r="AQ32" s="72" t="n"/>
+      <c r="AR32" s="29" t="n"/>
+      <c r="AS32" s="78" t="n"/>
+      <c r="AT32" s="26" t="n"/>
+      <c r="AU32" s="26" t="n"/>
+      <c r="AV32" s="26" t="n"/>
+      <c r="AW32" s="26" t="n"/>
       <c r="AX32" s="25" t="n"/>
       <c r="AY32" s="25" t="n"/>
       <c r="AZ32" s="25" t="n"/>
@@ -41222,7 +40652,7 @@
         <v>-0.002199653613098929</v>
       </c>
       <c r="D39" s="34" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E39" s="30" t="inlineStr">
         <is>
@@ -41398,7 +40828,7 @@
         <v>-0.01560649488873045</v>
       </c>
       <c r="D40" s="27" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E40" s="23" t="inlineStr">
         <is>
@@ -42630,7 +42060,7 @@
         <v>-0.0349996109102918</v>
       </c>
       <c r="D47" s="34" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E47" s="30" t="inlineStr">
         <is>
@@ -43861,7 +43291,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:G74"/>
+  <dimension ref="B2:G71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -45772,96 +45202,12 @@
         </is>
       </c>
     </row>
-    <row r="72">
-      <c r="B72" s="24" t="inlineStr">
-        <is>
-          <t>CRWV</t>
-        </is>
-      </c>
-      <c r="C72" s="101" t="inlineStr">
-        <is>
-          <t>CoreWeave, Inc.</t>
-        </is>
-      </c>
-      <c r="D72" s="104" t="inlineStr">
-        <is>
-          <t>Volume 3.4x its 20-day average</t>
-        </is>
-      </c>
-      <c r="E72" s="26" t="n">
-        <v>-0.04163168907292192</v>
-      </c>
-      <c r="F72" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="G72" s="23" t="inlineStr">
-        <is>
-          <t>Very Weak</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="B73" s="31" t="inlineStr">
-        <is>
-          <t>CRWV</t>
-        </is>
-      </c>
-      <c r="C73" s="102" t="inlineStr">
-        <is>
-          <t>CoreWeave, Inc.</t>
-        </is>
-      </c>
-      <c r="D73" s="105" t="inlineStr">
-        <is>
-          <t>Gapped down 2.3% at the open</t>
-        </is>
-      </c>
-      <c r="E73" s="33" t="n">
-        <v>-0.04163168907292192</v>
-      </c>
-      <c r="F73" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="G73" s="30" t="inlineStr">
-        <is>
-          <t>Very Weak</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="B74" s="24" t="inlineStr">
-        <is>
-          <t>CRWV</t>
-        </is>
-      </c>
-      <c r="C74" s="101" t="inlineStr">
-        <is>
-          <t>CoreWeave, Inc.</t>
-        </is>
-      </c>
-      <c r="D74" s="104" t="inlineStr">
-        <is>
-          <t>Bands squeezing — a big move often follows</t>
-        </is>
-      </c>
-      <c r="E74" s="26" t="n">
-        <v>-0.04163168907292192</v>
-      </c>
-      <c r="F74" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="G74" s="23" t="inlineStr">
-        <is>
-          <t>Very Weak</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="B5:G74"/>
+  <autoFilter ref="B5:G71"/>
   <mergeCells count="1">
     <mergeCell ref="B2:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="E6:E74">
+  <conditionalFormatting sqref="E6:E71">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="-0.05"/>

</xml_diff>

<commit_message>
Daily workbook: 2026-09-18 23:16 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -28,7 +28,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'09-15'!$5:$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'09-14'!$A$6:$AZ$48</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'09-14'!$5:$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Signals'!$B$5:$G$66</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Signals'!$B$5:$G$65</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 18 Sep 2026, 10:37 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 18 Sep 2026, 11:16 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -1376,21 +1376,21 @@
       <c r="D8" s="6" t="n"/>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>20</t>
         </is>
       </c>
       <c r="F8" s="8" t="n"/>
       <c r="G8" s="8" t="n"/>
       <c r="H8" s="14" t="inlineStr">
         <is>
-          <t>48%</t>
+          <t>49%</t>
         </is>
       </c>
       <c r="I8" s="8" t="n"/>
       <c r="J8" s="8" t="n"/>
       <c r="K8" s="15" t="inlineStr">
         <is>
-          <t>5.2</t>
+          <t>5.3</t>
         </is>
       </c>
       <c r="L8" s="10" t="n"/>
@@ -1404,7 +1404,7 @@
       <c r="P8" s="10" t="n"/>
       <c r="Q8" s="16" t="inlineStr">
         <is>
-          <t>61</t>
+          <t>60</t>
         </is>
       </c>
       <c r="R8" s="12" t="n"/>
@@ -1413,14 +1413,14 @@
     <row r="9" ht="15" customHeight="1">
       <c r="B9" s="17" t="inlineStr">
         <is>
-          <t>of 40 names</t>
+          <t>of 39 names</t>
         </is>
       </c>
       <c r="C9" s="6" t="n"/>
       <c r="D9" s="6" t="n"/>
       <c r="E9" s="18" t="inlineStr">
         <is>
-          <t>of 40 names</t>
+          <t>of 39 names</t>
         </is>
       </c>
       <c r="F9" s="8" t="n"/>
@@ -1441,7 +1441,7 @@
       <c r="M9" s="10" t="n"/>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>of 40 names</t>
+          <t>of 39 names</t>
         </is>
       </c>
       <c r="O9" s="10" t="n"/>
@@ -2117,11 +2117,11 @@
       </c>
       <c r="H33" s="24" t="inlineStr">
         <is>
-          <t>CCJ</t>
+          <t>XLRE</t>
         </is>
       </c>
       <c r="I33" s="26" t="n">
-        <v>-0.01271552011175747</v>
+        <v>-0.009548203552039447</v>
       </c>
       <c r="J33" s="27" t="n">
         <v>1</v>
@@ -2132,7 +2132,7 @@
         </is>
       </c>
       <c r="L33" s="28" t="n">
-        <v>40.00608558948002</v>
+        <v>31.05187129641278</v>
       </c>
     </row>
     <row r="34">
@@ -2157,11 +2157,11 @@
       </c>
       <c r="H34" s="31" t="inlineStr">
         <is>
-          <t>XLRE</t>
+          <t>XLP</t>
         </is>
       </c>
       <c r="I34" s="33" t="n">
-        <v>-0.009548203552039447</v>
+        <v>-0.008264400882337819</v>
       </c>
       <c r="J34" s="34" t="n">
         <v>1</v>
@@ -2172,7 +2172,7 @@
         </is>
       </c>
       <c r="L34" s="35" t="n">
-        <v>31.05187129641278</v>
+        <v>39.26120983046337</v>
       </c>
     </row>
     <row r="35">
@@ -2197,11 +2197,11 @@
       </c>
       <c r="H35" s="24" t="inlineStr">
         <is>
-          <t>XLP</t>
+          <t>XLY</t>
         </is>
       </c>
       <c r="I35" s="26" t="n">
-        <v>-0.008264400882337819</v>
+        <v>-0.003231893458336965</v>
       </c>
       <c r="J35" s="27" t="n">
         <v>1</v>
@@ -2212,7 +2212,7 @@
         </is>
       </c>
       <c r="L35" s="28" t="n">
-        <v>39.26120983046337</v>
+        <v>38.01124802917117</v>
       </c>
     </row>
     <row r="36">
@@ -2237,11 +2237,11 @@
       </c>
       <c r="H36" s="31" t="inlineStr">
         <is>
-          <t>XLY</t>
+          <t>CRWV</t>
         </is>
       </c>
       <c r="I36" s="33" t="n">
-        <v>-0.003231893458336965</v>
+        <v>0.0185278343492965</v>
       </c>
       <c r="J36" s="34" t="n">
         <v>1</v>
@@ -2252,7 +2252,7 @@
         </is>
       </c>
       <c r="L36" s="35" t="n">
-        <v>38.01124802917117</v>
+        <v>44.16457104126275</v>
       </c>
     </row>
     <row r="37">
@@ -2277,22 +2277,22 @@
       </c>
       <c r="H37" s="24" t="inlineStr">
         <is>
-          <t>CRWV</t>
+          <t>ASTS</t>
         </is>
       </c>
       <c r="I37" s="26" t="n">
-        <v>0.0185278343492965</v>
+        <v>-0.0668154789966573</v>
       </c>
       <c r="J37" s="27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K37" s="23" t="inlineStr">
         <is>
-          <t>Very Weak</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="L37" s="28" t="n">
-        <v>44.16457104126275</v>
+        <v>43.68463137542</v>
       </c>
     </row>
     <row r="38">
@@ -2317,11 +2317,11 @@
       </c>
       <c r="H38" s="31" t="inlineStr">
         <is>
-          <t>ASTS</t>
+          <t>IWM</t>
         </is>
       </c>
       <c r="I38" s="33" t="n">
-        <v>-0.0668154789966573</v>
+        <v>-0.004659589413843923</v>
       </c>
       <c r="J38" s="34" t="n">
         <v>2</v>
@@ -2332,7 +2332,7 @@
         </is>
       </c>
       <c r="L38" s="35" t="n">
-        <v>43.68463137542</v>
+        <v>34.36229466876138</v>
       </c>
     </row>
     <row r="41" ht="22" customHeight="1">
@@ -2741,11 +2741,11 @@
       </c>
       <c r="H51" s="24" t="inlineStr">
         <is>
-          <t>CCJ</t>
+          <t>XLRE</t>
         </is>
       </c>
       <c r="I51" s="26" t="n">
-        <v>-0.01271552011175747</v>
+        <v>-0.009548203552039447</v>
       </c>
       <c r="J51" s="27" t="n">
         <v>1</v>
@@ -2756,7 +2756,7 @@
         </is>
       </c>
       <c r="L51" s="28" t="n">
-        <v>40.00608558948002</v>
+        <v>31.05187129641278</v>
       </c>
     </row>
     <row r="52">
@@ -2781,11 +2781,11 @@
       </c>
       <c r="H52" s="31" t="inlineStr">
         <is>
-          <t>XLRE</t>
+          <t>XLP</t>
         </is>
       </c>
       <c r="I52" s="33" t="n">
-        <v>-0.009548203552039447</v>
+        <v>-0.008264400882337819</v>
       </c>
       <c r="J52" s="34" t="n">
         <v>1</v>
@@ -2796,7 +2796,7 @@
         </is>
       </c>
       <c r="L52" s="35" t="n">
-        <v>31.05187129641278</v>
+        <v>39.26120983046337</v>
       </c>
     </row>
   </sheetData>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 18 Sep 2026, 10:37 PM · Yahoo Finance data</t>
+          <t>Built 18 Sep 2026, 11:16 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -3132,22 +3132,22 @@
       </c>
       <c r="Y3" s="44" t="inlineStr">
         <is>
-          <t>19 of 40</t>
+          <t>19 of 39</t>
         </is>
       </c>
       <c r="AA3" s="45" t="inlineStr">
         <is>
-          <t>21 of 40</t>
+          <t>20 of 39</t>
         </is>
       </c>
       <c r="AC3" s="46" t="inlineStr">
         <is>
-          <t>5.2 / 9</t>
+          <t>5.3 / 9</t>
         </is>
       </c>
       <c r="AE3" s="47" t="inlineStr">
         <is>
-          <t>20 of 40</t>
+          <t>20 of 39</t>
         </is>
       </c>
     </row>
@@ -6772,17 +6772,17 @@
       </c>
       <c r="AX25" s="90" t="inlineStr">
         <is>
+          <t>Dow Jones Futures: Market Still Choppy; Robinhood, Sandisk, AMD, Moderna Surge Into Buy Areas</t>
+        </is>
+      </c>
+      <c r="AY25" s="90" t="inlineStr">
+        <is>
           <t>Top Research Reports for AMD, Linde &amp; Amgen</t>
         </is>
       </c>
-      <c r="AY25" s="90" t="inlineStr">
+      <c r="AZ25" s="90" t="inlineStr">
         <is>
           <t>AMD stock rises on a rumor that could give it a 2027 GPU edge</t>
-        </is>
-      </c>
-      <c r="AZ25" s="90" t="inlineStr">
-        <is>
-          <t>Prediction: AMD’s Biggest Growth Opportunity May Still Be Ahead</t>
         </is>
       </c>
     </row>
@@ -7361,7 +7361,7 @@
         <v>-0.0668154789966573</v>
       </c>
       <c r="D29" s="34" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E29" s="30" t="inlineStr">
         <is>
@@ -7733,171 +7733,57 @@
           <t>CCJ</t>
         </is>
       </c>
-      <c r="C31" s="33" t="n">
-        <v>-0.01271552011175747</v>
-      </c>
-      <c r="D31" s="34" t="n">
-        <v>20</v>
-      </c>
-      <c r="E31" s="30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F31" s="30" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G31" s="30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H31" s="30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I31" s="30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J31" s="30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K31" s="30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L31" s="30" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M31" s="30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N31" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="O31" s="30" t="inlineStr">
-        <is>
-          <t>Very Weak</t>
-        </is>
-      </c>
-      <c r="P31" s="32" t="inlineStr">
-        <is>
-          <t>Below every average</t>
-        </is>
-      </c>
+      <c r="C31" s="33" t="n"/>
+      <c r="D31" s="34" t="n"/>
+      <c r="E31" s="30" t="n"/>
+      <c r="F31" s="30" t="n"/>
+      <c r="G31" s="30" t="n"/>
+      <c r="H31" s="30" t="n"/>
+      <c r="I31" s="30" t="n"/>
+      <c r="J31" s="30" t="n"/>
+      <c r="K31" s="30" t="n"/>
+      <c r="L31" s="30" t="n"/>
+      <c r="M31" s="30" t="n"/>
+      <c r="N31" s="80" t="n"/>
+      <c r="O31" s="30" t="n"/>
+      <c r="P31" s="32" t="n"/>
       <c r="Q31" s="32" t="inlineStr">
         <is>
           <t>Cameco Corporation</t>
         </is>
       </c>
-      <c r="R31" s="81" t="n">
-        <v>91.62000274658203</v>
-      </c>
-      <c r="S31" s="82" t="n">
-        <v>-1.180000305175781</v>
-      </c>
-      <c r="T31" s="83" t="n">
-        <v>94.18000030517578</v>
-      </c>
-      <c r="U31" s="83" t="n">
-        <v>96.08999633789062</v>
-      </c>
-      <c r="V31" s="83" t="n">
-        <v>90.68000030517578</v>
-      </c>
-      <c r="W31" s="84" t="n">
-        <v>8101775</v>
-      </c>
-      <c r="X31" s="85" t="n">
-        <v>2.739799336758741</v>
-      </c>
-      <c r="Y31" s="35" t="n">
-        <v>40.00608558948002</v>
-      </c>
-      <c r="Z31" s="35" t="n">
-        <v>13.07374300727498</v>
-      </c>
-      <c r="AA31" s="35" t="n">
-        <v>14.50333255219578</v>
-      </c>
-      <c r="AB31" s="86" t="n">
-        <v>-1.396879006427824</v>
-      </c>
-      <c r="AC31" s="86" t="n">
-        <v>-0.2132073037071444</v>
-      </c>
-      <c r="AD31" s="86" t="n">
-        <v>-1.183671702720679</v>
-      </c>
-      <c r="AE31" s="83" t="n">
-        <v>93.93853850673425</v>
-      </c>
-      <c r="AF31" s="83" t="n">
-        <v>96.28604398207875</v>
-      </c>
-      <c r="AG31" s="83" t="n">
-        <v>94.79200027465821</v>
-      </c>
-      <c r="AH31" s="83" t="n">
-        <v>101.4737998962402</v>
-      </c>
-      <c r="AI31" s="83" t="n">
-        <v>105.8177498245239</v>
-      </c>
-      <c r="AJ31" s="83" t="n">
-        <v>108.7274959824728</v>
-      </c>
-      <c r="AK31" s="83" t="n">
-        <v>98.7235008239746</v>
-      </c>
-      <c r="AL31" s="83" t="n">
-        <v>88.7195056654764</v>
-      </c>
-      <c r="AM31" s="87" t="n">
-        <v>0.1449669374660638</v>
-      </c>
-      <c r="AN31" s="36" t="n">
-        <v>20.26669450536497</v>
-      </c>
-      <c r="AO31" s="88" t="n">
-        <v>4.056557870564574</v>
-      </c>
-      <c r="AP31" s="83" t="n">
-        <v>135.2400054931641</v>
-      </c>
-      <c r="AQ31" s="83" t="n">
-        <v>77.69999694824219</v>
-      </c>
-      <c r="AR31" s="36" t="n">
-        <v>-32.25377179446127</v>
-      </c>
-      <c r="AS31" s="89" t="n">
-        <v>24.19187301210149</v>
-      </c>
-      <c r="AT31" s="33" t="n">
-        <v>-0.05233758318805948</v>
-      </c>
-      <c r="AU31" s="33" t="n">
-        <v>-0.06491121037404513</v>
-      </c>
-      <c r="AV31" s="33" t="n">
-        <v>-0.1396374815990735</v>
-      </c>
-      <c r="AW31" s="33" t="n">
-        <v>0.001420973722243257</v>
-      </c>
+      <c r="R31" s="81" t="n"/>
+      <c r="S31" s="82" t="n"/>
+      <c r="T31" s="83" t="n"/>
+      <c r="U31" s="83" t="n"/>
+      <c r="V31" s="83" t="n"/>
+      <c r="W31" s="84" t="n"/>
+      <c r="X31" s="85" t="n"/>
+      <c r="Y31" s="35" t="n"/>
+      <c r="Z31" s="35" t="n"/>
+      <c r="AA31" s="35" t="n"/>
+      <c r="AB31" s="86" t="n"/>
+      <c r="AC31" s="86" t="n"/>
+      <c r="AD31" s="86" t="n"/>
+      <c r="AE31" s="83" t="n"/>
+      <c r="AF31" s="83" t="n"/>
+      <c r="AG31" s="83" t="n"/>
+      <c r="AH31" s="83" t="n"/>
+      <c r="AI31" s="83" t="n"/>
+      <c r="AJ31" s="83" t="n"/>
+      <c r="AK31" s="83" t="n"/>
+      <c r="AL31" s="83" t="n"/>
+      <c r="AM31" s="87" t="n"/>
+      <c r="AN31" s="36" t="n"/>
+      <c r="AO31" s="88" t="n"/>
+      <c r="AP31" s="83" t="n"/>
+      <c r="AQ31" s="83" t="n"/>
+      <c r="AR31" s="36" t="n"/>
+      <c r="AS31" s="89" t="n"/>
+      <c r="AT31" s="33" t="n"/>
+      <c r="AU31" s="33" t="n"/>
+      <c r="AV31" s="33" t="n"/>
+      <c r="AW31" s="33" t="n"/>
       <c r="AX31" s="90" t="inlineStr">
         <is>
           <t>Cameco (CCJ) Stock Declines While Market Improves: Some Information for Investors</t>
@@ -8113,7 +7999,7 @@
         <v>-0.03456836507735306</v>
       </c>
       <c r="D33" s="34" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E33" s="30" t="inlineStr">
         <is>
@@ -9216,17 +9102,17 @@
       </c>
       <c r="AX38" s="79" t="inlineStr">
         <is>
+          <t>Strategy (MSTR) Surges 16% on Growing Digital Asset Adoption — A New Catalyst Looms Next Week</t>
+        </is>
+      </c>
+      <c r="AY38" s="79" t="inlineStr">
+        <is>
           <t>Strategy, Circle, and Coinbase Lead Crypto Stock Rally on Tokenized Stock Approval</t>
         </is>
       </c>
-      <c r="AY38" s="79" t="inlineStr">
+      <c r="AZ38" s="79" t="inlineStr">
         <is>
           <t>Tom Lee Says Q4 Could Bring One of the Biggest Rallies of Our Lifetime. Can Bitcoin, Ethereum, and XRP Reac...</t>
-        </is>
-      </c>
-      <c r="AZ38" s="79" t="inlineStr">
-        <is>
-          <t>Strategy (MSTR) After Its AI Forum Launch And The Case For A Pricey Narrative</t>
         </is>
       </c>
     </row>
@@ -9617,7 +9503,7 @@
         <v>-0.04674009769191312</v>
       </c>
       <c r="D41" s="34" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E41" s="30" t="inlineStr">
         <is>
@@ -9785,12 +9671,12 @@
       </c>
       <c r="AY41" s="90" t="inlineStr">
         <is>
+          <t>Netflix (NFLX) Stock Trades Down, Here Is Why</t>
+        </is>
+      </c>
+      <c r="AZ41" s="90" t="inlineStr">
+        <is>
           <t>Stock Market Today, Sept. 18: Netflix Falls on Analyst Downgrade and Slashed Price Target</t>
-        </is>
-      </c>
-      <c r="AZ41" s="90" t="inlineStr">
-        <is>
-          <t>Netflix Stock Gets Downgraded by Wells Fargo on ‘Worrying’ Engagement Trends</t>
         </is>
       </c>
     </row>
@@ -10156,17 +10042,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
+          <t>NVIDIA Vs Intel Corporation (NASDAQ:INTC): Here’s The One Jim Cramer Likes</t>
+        </is>
+      </c>
+      <c r="AY43" s="90" t="inlineStr">
+        <is>
           <t>Jensen Huang Maintained His Prediction That AI Infrastructure Spending Will Hit $3 Trillion to $4 Trillion ...</t>
         </is>
       </c>
-      <c r="AY43" s="90" t="inlineStr">
+      <c r="AZ43" s="90" t="inlineStr">
         <is>
           <t>Nvidia-Backed Cloud Platform Nscale Files For IPO — NVDA Stock In Focus</t>
-        </is>
-      </c>
-      <c r="AZ43" s="90" t="inlineStr">
-        <is>
-          <t>Nvidia Stock Is Up 21% in Six Months. Here’s What the Street Still Isn’t Pricing In</t>
         </is>
       </c>
     </row>
@@ -10344,17 +10230,17 @@
       </c>
       <c r="AX44" s="79" t="inlineStr">
         <is>
+          <t>Jim Cramer Says His Palantir Technologies Inc. (NASDAQ:PLTR) Price Target Is $250</t>
+        </is>
+      </c>
+      <c r="AY44" s="79" t="inlineStr">
+        <is>
           <t>Palantir CEO offers surprising solution to AI threats that involves Washington, D.C.</t>
         </is>
       </c>
-      <c r="AY44" s="79" t="inlineStr">
+      <c r="AZ44" s="79" t="inlineStr">
         <is>
           <t>The 3 Tech Laggards Are Top Stock Picks, UBS Says</t>
-        </is>
-      </c>
-      <c r="AZ44" s="79" t="inlineStr">
-        <is>
-          <t>PLTR's 110% Commercial Revenue Surge Defines Its Q2 Growth</t>
         </is>
       </c>
     </row>
@@ -10369,7 +10255,7 @@
         <v>-0.05823753432337975</v>
       </c>
       <c r="D45" s="34" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E45" s="30" t="inlineStr">
         <is>
@@ -10557,7 +10443,7 @@
         <v>-0.04792096748192742</v>
       </c>
       <c r="D46" s="27" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E46" s="23" t="inlineStr">
         <is>
@@ -10908,17 +10794,17 @@
       </c>
       <c r="AX47" s="90" t="inlineStr">
         <is>
+          <t>Dow Jones Futures: Market Still Choppy; Robinhood, Sandisk, AMD, Moderna Surge Into Buy Areas</t>
+        </is>
+      </c>
+      <c r="AY47" s="90" t="inlineStr">
+        <is>
           <t>Stock Market Today: Nasdaq, S&amp;P Reverse Slightly Higher; Sandisk, Lumentum Lead This Tech Rally</t>
         </is>
       </c>
-      <c r="AY47" s="90" t="inlineStr">
+      <c r="AZ47" s="90" t="inlineStr">
         <is>
           <t>Credo Technology Group vs. Sandisk: Which Technology Stock Is a Better Buy in 2026?</t>
-        </is>
-      </c>
-      <c r="AZ47" s="90" t="inlineStr">
-        <is>
-          <t>Is Sandisk (SNDK) Stock At Risk As New NAND Competition Targets AI Memory?</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11529,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 18 Sep 2026, 10:37 PM · Yahoo Finance data</t>
+          <t>Built 18 Sep 2026, 11:16 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -11668,22 +11554,22 @@
       </c>
       <c r="Y3" s="44" t="inlineStr">
         <is>
-          <t>36 of 40</t>
+          <t>35 of 39</t>
         </is>
       </c>
       <c r="AA3" s="45" t="inlineStr">
         <is>
-          <t>4 of 40</t>
+          <t>4 of 39</t>
         </is>
       </c>
       <c r="AC3" s="46" t="inlineStr">
         <is>
-          <t>5.4 / 9</t>
+          <t>5.5 / 9</t>
         </is>
       </c>
       <c r="AE3" s="47" t="inlineStr">
         <is>
-          <t>24 of 40</t>
+          <t>24 of 39</t>
         </is>
       </c>
     </row>
@@ -14777,7 +14663,7 @@
         <v>0.01380823768034456</v>
       </c>
       <c r="D24" s="27" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E24" s="23" t="inlineStr">
         <is>
@@ -16005,171 +15891,57 @@
           <t>CCJ</t>
         </is>
       </c>
-      <c r="C31" s="33" t="n">
-        <v>0.02090210664449743</v>
-      </c>
-      <c r="D31" s="34" t="n">
-        <v>18</v>
-      </c>
-      <c r="E31" s="30" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F31" s="30" t="inlineStr">
-        <is>
-          <t>Same</t>
-        </is>
-      </c>
-      <c r="G31" s="30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H31" s="30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I31" s="30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J31" s="30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K31" s="30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L31" s="30" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M31" s="30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N31" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="O31" s="30" t="inlineStr">
-        <is>
-          <t>Weak</t>
-        </is>
-      </c>
-      <c r="P31" s="32" t="inlineStr">
-        <is>
-          <t>Below every average</t>
-        </is>
-      </c>
+      <c r="C31" s="33" t="n"/>
+      <c r="D31" s="34" t="n"/>
+      <c r="E31" s="30" t="n"/>
+      <c r="F31" s="30" t="n"/>
+      <c r="G31" s="30" t="n"/>
+      <c r="H31" s="30" t="n"/>
+      <c r="I31" s="30" t="n"/>
+      <c r="J31" s="30" t="n"/>
+      <c r="K31" s="30" t="n"/>
+      <c r="L31" s="30" t="n"/>
+      <c r="M31" s="30" t="n"/>
+      <c r="N31" s="80" t="n"/>
+      <c r="O31" s="30" t="n"/>
+      <c r="P31" s="32" t="n"/>
       <c r="Q31" s="32" t="inlineStr">
         <is>
           <t>Cameco Corporation</t>
         </is>
       </c>
-      <c r="R31" s="81" t="n">
-        <v>92.80000305175781</v>
-      </c>
-      <c r="S31" s="82" t="n">
-        <v>1.900001525878906</v>
-      </c>
-      <c r="T31" s="83" t="n">
-        <v>92.62000274658203</v>
-      </c>
-      <c r="U31" s="83" t="n">
-        <v>93.09999847412109</v>
-      </c>
-      <c r="V31" s="83" t="n">
-        <v>91.59999847412109</v>
-      </c>
-      <c r="W31" s="84" t="n">
-        <v>2120600</v>
-      </c>
-      <c r="X31" s="85" t="n">
-        <v>0.7980265720344485</v>
-      </c>
-      <c r="Y31" s="35" t="n">
-        <v>41.86387168601648</v>
-      </c>
-      <c r="Z31" s="35" t="n">
-        <v>18.2905234547971</v>
-      </c>
-      <c r="AA31" s="35" t="n">
-        <v>14.90419385253837</v>
-      </c>
-      <c r="AB31" s="86" t="n">
-        <v>-1.151972671185007</v>
-      </c>
-      <c r="AC31" s="86" t="n">
-        <v>0.08271062197302553</v>
-      </c>
-      <c r="AD31" s="86" t="n">
-        <v>-1.234683293158032</v>
-      </c>
-      <c r="AE31" s="83" t="n">
-        <v>94.60097729534917</v>
-      </c>
-      <c r="AF31" s="83" t="n">
-        <v>96.75264810562842</v>
-      </c>
-      <c r="AG31" s="83" t="n">
-        <v>94.87440017700196</v>
-      </c>
-      <c r="AH31" s="83" t="n">
-        <v>101.7886998748779</v>
-      </c>
-      <c r="AI31" s="83" t="n">
-        <v>105.7972998046875</v>
-      </c>
-      <c r="AJ31" s="83" t="n">
-        <v>108.5029265405086</v>
-      </c>
-      <c r="AK31" s="83" t="n">
-        <v>98.92200050354003</v>
-      </c>
-      <c r="AL31" s="83" t="n">
-        <v>89.34107446657144</v>
-      </c>
-      <c r="AM31" s="87" t="n">
-        <v>0.180511182939931</v>
-      </c>
-      <c r="AN31" s="36" t="n">
-        <v>19.37066777501276</v>
-      </c>
-      <c r="AO31" s="88" t="n">
-        <v>3.864610451597756</v>
-      </c>
-      <c r="AP31" s="83" t="n">
-        <v>135.2400054931641</v>
-      </c>
-      <c r="AQ31" s="83" t="n">
-        <v>77.69999694824219</v>
-      </c>
-      <c r="AR31" s="36" t="n">
-        <v>-31.38124868203399</v>
-      </c>
-      <c r="AS31" s="89" t="n">
-        <v>26.24262054415051</v>
-      </c>
-      <c r="AT31" s="33" t="n">
-        <v>-0.04742347776660316</v>
-      </c>
-      <c r="AU31" s="33" t="n">
-        <v>-0.03363527823177914</v>
-      </c>
-      <c r="AV31" s="33" t="n">
-        <v>-0.1217942210674683</v>
-      </c>
-      <c r="AW31" s="33" t="n">
-        <v>0.01431856179446966</v>
-      </c>
+      <c r="R31" s="81" t="n"/>
+      <c r="S31" s="82" t="n"/>
+      <c r="T31" s="83" t="n"/>
+      <c r="U31" s="83" t="n"/>
+      <c r="V31" s="83" t="n"/>
+      <c r="W31" s="84" t="n"/>
+      <c r="X31" s="85" t="n"/>
+      <c r="Y31" s="35" t="n"/>
+      <c r="Z31" s="35" t="n"/>
+      <c r="AA31" s="35" t="n"/>
+      <c r="AB31" s="86" t="n"/>
+      <c r="AC31" s="86" t="n"/>
+      <c r="AD31" s="86" t="n"/>
+      <c r="AE31" s="83" t="n"/>
+      <c r="AF31" s="83" t="n"/>
+      <c r="AG31" s="83" t="n"/>
+      <c r="AH31" s="83" t="n"/>
+      <c r="AI31" s="83" t="n"/>
+      <c r="AJ31" s="83" t="n"/>
+      <c r="AK31" s="83" t="n"/>
+      <c r="AL31" s="83" t="n"/>
+      <c r="AM31" s="87" t="n"/>
+      <c r="AN31" s="36" t="n"/>
+      <c r="AO31" s="88" t="n"/>
+      <c r="AP31" s="83" t="n"/>
+      <c r="AQ31" s="83" t="n"/>
+      <c r="AR31" s="36" t="n"/>
+      <c r="AS31" s="89" t="n"/>
+      <c r="AT31" s="33" t="n"/>
+      <c r="AU31" s="33" t="n"/>
+      <c r="AV31" s="33" t="n"/>
+      <c r="AW31" s="33" t="n"/>
       <c r="AX31" s="32" t="n"/>
       <c r="AY31" s="32" t="n"/>
       <c r="AZ31" s="32" t="n"/>
@@ -16185,7 +15957,7 @@
         <v>-0.04163168907292192</v>
       </c>
       <c r="D32" s="27" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E32" s="23" t="inlineStr">
         <is>
@@ -16537,7 +16309,7 @@
         <v>0.01272986654494157</v>
       </c>
       <c r="D34" s="27" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E34" s="23" t="inlineStr">
         <is>
@@ -16713,7 +16485,7 @@
         <v>0.02017833486401566</v>
       </c>
       <c r="D35" s="34" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E35" s="30" t="inlineStr">
         <is>
@@ -17065,7 +16837,7 @@
         <v>0.01519480398228579</v>
       </c>
       <c r="D37" s="34" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E37" s="30" t="inlineStr">
         <is>
@@ -17769,7 +17541,7 @@
         <v>-0.01439610065168861</v>
       </c>
       <c r="D41" s="34" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E41" s="30" t="inlineStr">
         <is>
@@ -18297,7 +18069,7 @@
         <v>0.01089829755181948</v>
       </c>
       <c r="D44" s="27" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E44" s="23" t="inlineStr">
         <is>
@@ -19579,7 +19351,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 18 Sep 2026, 10:37 PM · Yahoo Finance data</t>
+          <t>Built 18 Sep 2026, 11:16 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19604,22 +19376,22 @@
       </c>
       <c r="Y3" s="44" t="inlineStr">
         <is>
-          <t>19 of 40</t>
+          <t>19 of 39</t>
         </is>
       </c>
       <c r="AA3" s="45" t="inlineStr">
         <is>
-          <t>20 of 40</t>
+          <t>19 of 39</t>
         </is>
       </c>
       <c r="AC3" s="46" t="inlineStr">
         <is>
-          <t>3.5 / 9</t>
+          <t>3.6 / 9</t>
         </is>
       </c>
       <c r="AE3" s="47" t="inlineStr">
         <is>
-          <t>9 of 40</t>
+          <t>9 of 39</t>
         </is>
       </c>
     </row>
@@ -23065,7 +22837,7 @@
         <v>-0.009902550008897171</v>
       </c>
       <c r="D26" s="27" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E26" s="23" t="inlineStr">
         <is>
@@ -23241,7 +23013,7 @@
         <v>-0.00371299037639905</v>
       </c>
       <c r="D27" s="34" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E27" s="30" t="inlineStr">
         <is>
@@ -23941,171 +23713,57 @@
           <t>CCJ</t>
         </is>
       </c>
-      <c r="C31" s="33" t="n">
-        <v>-0.003398723404290926</v>
-      </c>
-      <c r="D31" s="34" t="n">
-        <v>17</v>
-      </c>
-      <c r="E31" s="30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F31" s="30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G31" s="30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H31" s="30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I31" s="30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J31" s="30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K31" s="30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L31" s="30" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M31" s="30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N31" s="80" t="n">
-        <v>0</v>
-      </c>
-      <c r="O31" s="30" t="inlineStr">
-        <is>
-          <t>Very Weak</t>
-        </is>
-      </c>
-      <c r="P31" s="32" t="inlineStr">
-        <is>
-          <t>Below every average</t>
-        </is>
-      </c>
+      <c r="C31" s="33" t="n"/>
+      <c r="D31" s="34" t="n"/>
+      <c r="E31" s="30" t="n"/>
+      <c r="F31" s="30" t="n"/>
+      <c r="G31" s="30" t="n"/>
+      <c r="H31" s="30" t="n"/>
+      <c r="I31" s="30" t="n"/>
+      <c r="J31" s="30" t="n"/>
+      <c r="K31" s="30" t="n"/>
+      <c r="L31" s="30" t="n"/>
+      <c r="M31" s="30" t="n"/>
+      <c r="N31" s="80" t="n"/>
+      <c r="O31" s="30" t="n"/>
+      <c r="P31" s="32" t="n"/>
       <c r="Q31" s="32" t="inlineStr">
         <is>
           <t>Cameco Corporation</t>
         </is>
       </c>
-      <c r="R31" s="81" t="n">
-        <v>90.90000152587891</v>
-      </c>
-      <c r="S31" s="82" t="n">
-        <v>-0.30999755859375</v>
-      </c>
-      <c r="T31" s="83" t="n">
-        <v>92.55000305175781</v>
-      </c>
-      <c r="U31" s="83" t="n">
-        <v>92.93000030517578</v>
-      </c>
-      <c r="V31" s="83" t="n">
-        <v>89.73999786376953</v>
-      </c>
-      <c r="W31" s="84" t="n">
-        <v>2114600</v>
-      </c>
-      <c r="X31" s="85" t="n">
-        <v>0.7986524203934721</v>
-      </c>
-      <c r="Y31" s="35" t="n">
-        <v>37.52622102985752</v>
-      </c>
-      <c r="Z31" s="35" t="n">
-        <v>6.032259280345485</v>
-      </c>
-      <c r="AA31" s="35" t="n">
-        <v>14.35227414280901</v>
-      </c>
-      <c r="AB31" s="86" t="n">
-        <v>-0.9427726500575631</v>
-      </c>
-      <c r="AC31" s="86" t="n">
-        <v>0.3913814452625337</v>
-      </c>
-      <c r="AD31" s="86" t="n">
-        <v>-1.334154095320097</v>
-      </c>
-      <c r="AE31" s="83" t="n">
-        <v>95.11554136494669</v>
-      </c>
-      <c r="AF31" s="83" t="n">
-        <v>97.1479126110155</v>
-      </c>
-      <c r="AG31" s="83" t="n">
-        <v>94.91300018310547</v>
-      </c>
-      <c r="AH31" s="83" t="n">
-        <v>102.0821998596191</v>
-      </c>
-      <c r="AI31" s="83" t="n">
-        <v>105.7758498001099</v>
-      </c>
-      <c r="AJ31" s="83" t="n">
-        <v>108.3574661161388</v>
-      </c>
-      <c r="AK31" s="83" t="n">
-        <v>99.18100051879883</v>
-      </c>
-      <c r="AL31" s="83" t="n">
-        <v>90.00453492145886</v>
-      </c>
-      <c r="AM31" s="87" t="n">
-        <v>0.0487914761364999</v>
-      </c>
-      <c r="AN31" s="36" t="n">
-        <v>18.50448281291669</v>
-      </c>
-      <c r="AO31" s="88" t="n">
-        <v>4.062708207172672</v>
-      </c>
-      <c r="AP31" s="83" t="n">
-        <v>135.2400054931641</v>
-      </c>
-      <c r="AQ31" s="83" t="n">
-        <v>77.69999694824219</v>
-      </c>
-      <c r="AR31" s="36" t="n">
-        <v>-32.78615954324729</v>
-      </c>
-      <c r="AS31" s="89" t="n">
-        <v>22.94056763535477</v>
-      </c>
-      <c r="AT31" s="33" t="n">
-        <v>-0.0947116999241695</v>
-      </c>
-      <c r="AU31" s="33" t="n">
-        <v>-0.07790627066874756</v>
-      </c>
-      <c r="AV31" s="33" t="n">
-        <v>-0.1573970723011033</v>
-      </c>
-      <c r="AW31" s="33" t="n">
-        <v>-0.006448752340874941</v>
-      </c>
+      <c r="R31" s="81" t="n"/>
+      <c r="S31" s="82" t="n"/>
+      <c r="T31" s="83" t="n"/>
+      <c r="U31" s="83" t="n"/>
+      <c r="V31" s="83" t="n"/>
+      <c r="W31" s="84" t="n"/>
+      <c r="X31" s="85" t="n"/>
+      <c r="Y31" s="35" t="n"/>
+      <c r="Z31" s="35" t="n"/>
+      <c r="AA31" s="35" t="n"/>
+      <c r="AB31" s="86" t="n"/>
+      <c r="AC31" s="86" t="n"/>
+      <c r="AD31" s="86" t="n"/>
+      <c r="AE31" s="83" t="n"/>
+      <c r="AF31" s="83" t="n"/>
+      <c r="AG31" s="83" t="n"/>
+      <c r="AH31" s="83" t="n"/>
+      <c r="AI31" s="83" t="n"/>
+      <c r="AJ31" s="83" t="n"/>
+      <c r="AK31" s="83" t="n"/>
+      <c r="AL31" s="83" t="n"/>
+      <c r="AM31" s="87" t="n"/>
+      <c r="AN31" s="36" t="n"/>
+      <c r="AO31" s="88" t="n"/>
+      <c r="AP31" s="83" t="n"/>
+      <c r="AQ31" s="83" t="n"/>
+      <c r="AR31" s="36" t="n"/>
+      <c r="AS31" s="89" t="n"/>
+      <c r="AT31" s="33" t="n"/>
+      <c r="AU31" s="33" t="n"/>
+      <c r="AV31" s="33" t="n"/>
+      <c r="AW31" s="33" t="n"/>
       <c r="AX31" s="32" t="n"/>
       <c r="AY31" s="32" t="n"/>
       <c r="AZ31" s="32" t="n"/>
@@ -24473,7 +24131,7 @@
         <v>-0.00606275772083209</v>
       </c>
       <c r="D34" s="27" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E34" s="23" t="inlineStr">
         <is>
@@ -25001,7 +24659,7 @@
         <v>-0.01371903643226224</v>
       </c>
       <c r="D37" s="34" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E37" s="30" t="inlineStr">
         <is>
@@ -25177,7 +24835,7 @@
         <v>-0.02638893238637796</v>
       </c>
       <c r="D38" s="27" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E38" s="23" t="inlineStr">
         <is>
@@ -25705,7 +25363,7 @@
         <v>-0.01912705821032035</v>
       </c>
       <c r="D41" s="34" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E41" s="30" t="inlineStr">
         <is>
@@ -26409,7 +26067,7 @@
         <v>-0.01576148384327447</v>
       </c>
       <c r="D45" s="34" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E45" s="30" t="inlineStr">
         <is>
@@ -26761,7 +26419,7 @@
         <v>-0.007136380149352251</v>
       </c>
       <c r="D47" s="34" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E47" s="30" t="inlineStr">
         <is>
@@ -27515,7 +27173,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 18 Sep 2026, 10:37 PM · Yahoo Finance data</t>
+          <t>Built 18 Sep 2026, 11:16 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27540,22 +27198,22 @@
       </c>
       <c r="Y3" s="44" t="inlineStr">
         <is>
-          <t>11 of 40</t>
+          <t>11 of 39</t>
         </is>
       </c>
       <c r="AA3" s="45" t="inlineStr">
         <is>
-          <t>29 of 40</t>
+          <t>28 of 39</t>
         </is>
       </c>
       <c r="AC3" s="46" t="inlineStr">
         <is>
-          <t>3.1 / 9</t>
+          <t>3.2 / 9</t>
         </is>
       </c>
       <c r="AE3" s="47" t="inlineStr">
         <is>
-          <t>8 of 40</t>
+          <t>8 of 39</t>
         </is>
       </c>
     </row>
@@ -31877,171 +31535,57 @@
           <t>CCJ</t>
         </is>
       </c>
-      <c r="C31" s="33" t="n">
-        <v>-0.02198158915719572</v>
-      </c>
-      <c r="D31" s="34" t="n">
-        <v>20</v>
-      </c>
-      <c r="E31" s="30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F31" s="30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G31" s="30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H31" s="30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I31" s="30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J31" s="30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K31" s="30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L31" s="30" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M31" s="30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N31" s="80" t="n">
-        <v>0</v>
-      </c>
-      <c r="O31" s="30" t="inlineStr">
-        <is>
-          <t>Very Weak</t>
-        </is>
-      </c>
-      <c r="P31" s="32" t="inlineStr">
-        <is>
-          <t>Below every average</t>
-        </is>
-      </c>
+      <c r="C31" s="33" t="n"/>
+      <c r="D31" s="34" t="n"/>
+      <c r="E31" s="30" t="n"/>
+      <c r="F31" s="30" t="n"/>
+      <c r="G31" s="30" t="n"/>
+      <c r="H31" s="30" t="n"/>
+      <c r="I31" s="30" t="n"/>
+      <c r="J31" s="30" t="n"/>
+      <c r="K31" s="30" t="n"/>
+      <c r="L31" s="30" t="n"/>
+      <c r="M31" s="30" t="n"/>
+      <c r="N31" s="80" t="n"/>
+      <c r="O31" s="30" t="n"/>
+      <c r="P31" s="32" t="n"/>
       <c r="Q31" s="32" t="inlineStr">
         <is>
           <t>Cameco Corporation</t>
         </is>
       </c>
-      <c r="R31" s="81" t="n">
-        <v>91.20999908447266</v>
-      </c>
-      <c r="S31" s="82" t="n">
-        <v>-2.050003051757812</v>
-      </c>
-      <c r="T31" s="83" t="n">
-        <v>93.75</v>
-      </c>
-      <c r="U31" s="83" t="n">
-        <v>94.40000152587891</v>
-      </c>
-      <c r="V31" s="83" t="n">
-        <v>91.01000213623047</v>
-      </c>
-      <c r="W31" s="84" t="n">
-        <v>2264700</v>
-      </c>
-      <c r="X31" s="85" t="n">
-        <v>0.8477989869986935</v>
-      </c>
-      <c r="Y31" s="35" t="n">
-        <v>37.95526333336542</v>
-      </c>
-      <c r="Z31" s="35" t="n">
-        <v>0.9741693138524246</v>
-      </c>
-      <c r="AA31" s="35" t="n">
-        <v>13.69953333397874</v>
-      </c>
-      <c r="AB31" s="86" t="n">
-        <v>-0.4685895928191144</v>
-      </c>
-      <c r="AC31" s="86" t="n">
-        <v>0.7249199690925578</v>
-      </c>
-      <c r="AD31" s="86" t="n">
-        <v>-1.193509561911672</v>
-      </c>
-      <c r="AE31" s="83" t="n">
-        <v>96.31998131896607</v>
-      </c>
-      <c r="AF31" s="83" t="n">
-        <v>97.77270371952916</v>
-      </c>
-      <c r="AG31" s="83" t="n">
-        <v>94.9884001159668</v>
-      </c>
-      <c r="AH31" s="83" t="n">
-        <v>102.4116998291016</v>
-      </c>
-      <c r="AI31" s="83" t="n">
-        <v>105.7653997802734</v>
-      </c>
-      <c r="AJ31" s="83" t="n">
-        <v>107.9354487026402</v>
-      </c>
-      <c r="AK31" s="83" t="n">
-        <v>99.43750038146973</v>
-      </c>
-      <c r="AL31" s="83" t="n">
-        <v>90.93955206029926</v>
-      </c>
-      <c r="AM31" s="87" t="n">
-        <v>0.01591248934167105</v>
-      </c>
-      <c r="AN31" s="36" t="n">
-        <v>17.09203929819231</v>
-      </c>
-      <c r="AO31" s="88" t="n">
-        <v>4.091321258457188</v>
-      </c>
-      <c r="AP31" s="83" t="n">
-        <v>135.2400054931641</v>
-      </c>
-      <c r="AQ31" s="83" t="n">
-        <v>77.69999694824219</v>
-      </c>
-      <c r="AR31" s="36" t="n">
-        <v>-32.55693923416543</v>
-      </c>
-      <c r="AS31" s="89" t="n">
-        <v>23.47931896062045</v>
-      </c>
-      <c r="AT31" s="33" t="n">
-        <v>-0.1055212514212057</v>
-      </c>
-      <c r="AU31" s="33" t="n">
-        <v>-0.06680989279740335</v>
-      </c>
-      <c r="AV31" s="33" t="n">
-        <v>-0.1477293781957715</v>
-      </c>
-      <c r="AW31" s="33" t="n">
-        <v>-0.003060430493328936</v>
-      </c>
+      <c r="R31" s="81" t="n"/>
+      <c r="S31" s="82" t="n"/>
+      <c r="T31" s="83" t="n"/>
+      <c r="U31" s="83" t="n"/>
+      <c r="V31" s="83" t="n"/>
+      <c r="W31" s="84" t="n"/>
+      <c r="X31" s="85" t="n"/>
+      <c r="Y31" s="35" t="n"/>
+      <c r="Z31" s="35" t="n"/>
+      <c r="AA31" s="35" t="n"/>
+      <c r="AB31" s="86" t="n"/>
+      <c r="AC31" s="86" t="n"/>
+      <c r="AD31" s="86" t="n"/>
+      <c r="AE31" s="83" t="n"/>
+      <c r="AF31" s="83" t="n"/>
+      <c r="AG31" s="83" t="n"/>
+      <c r="AH31" s="83" t="n"/>
+      <c r="AI31" s="83" t="n"/>
+      <c r="AJ31" s="83" t="n"/>
+      <c r="AK31" s="83" t="n"/>
+      <c r="AL31" s="83" t="n"/>
+      <c r="AM31" s="87" t="n"/>
+      <c r="AN31" s="36" t="n"/>
+      <c r="AO31" s="88" t="n"/>
+      <c r="AP31" s="83" t="n"/>
+      <c r="AQ31" s="83" t="n"/>
+      <c r="AR31" s="36" t="n"/>
+      <c r="AS31" s="89" t="n"/>
+      <c r="AT31" s="33" t="n"/>
+      <c r="AU31" s="33" t="n"/>
+      <c r="AV31" s="33" t="n"/>
+      <c r="AW31" s="33" t="n"/>
       <c r="AX31" s="32" t="n"/>
       <c r="AY31" s="32" t="n"/>
       <c r="AZ31" s="32" t="n"/>
@@ -32057,7 +31601,7 @@
         <v>-0.02482532061522447</v>
       </c>
       <c r="D32" s="27" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E32" s="23" t="inlineStr">
         <is>
@@ -32585,7 +32129,7 @@
         <v>-0.03683104946329141</v>
       </c>
       <c r="D35" s="34" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E35" s="30" t="inlineStr">
         <is>
@@ -33113,7 +32657,7 @@
         <v>-0.05360008914145631</v>
       </c>
       <c r="D38" s="27" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E38" s="23" t="inlineStr">
         <is>
@@ -33465,7 +33009,7 @@
         <v>-0.02271552508959385</v>
       </c>
       <c r="D40" s="27" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E40" s="23" t="inlineStr">
         <is>
@@ -33641,7 +33185,7 @@
         <v>-0.03012945938919442</v>
       </c>
       <c r="D41" s="34" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E41" s="30" t="inlineStr">
         <is>
@@ -35451,7 +34995,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 18 Sep 2026, 10:37 PM · Yahoo Finance data</t>
+          <t>Built 18 Sep 2026, 11:16 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35476,22 +35020,22 @@
       </c>
       <c r="Y3" s="44" t="inlineStr">
         <is>
-          <t>11 of 40</t>
+          <t>11 of 39</t>
         </is>
       </c>
       <c r="AA3" s="45" t="inlineStr">
         <is>
-          <t>29 of 40</t>
+          <t>28 of 39</t>
         </is>
       </c>
       <c r="AC3" s="46" t="inlineStr">
         <is>
-          <t>3.9 / 9</t>
+          <t>4.0 / 9</t>
         </is>
       </c>
       <c r="AE3" s="47" t="inlineStr">
         <is>
-          <t>15 of 40</t>
+          <t>15 of 39</t>
         </is>
       </c>
     </row>
@@ -38761,7 +38305,7 @@
         <v>-0.04401991941131522</v>
       </c>
       <c r="D25" s="34" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E25" s="30" t="inlineStr">
         <is>
@@ -39289,7 +38833,7 @@
         <v>-0.09736022208599437</v>
       </c>
       <c r="D28" s="27" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E28" s="23" t="inlineStr">
         <is>
@@ -39641,7 +39185,7 @@
         <v>-0.04770847117206256</v>
       </c>
       <c r="D30" s="27" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E30" s="23" t="inlineStr">
         <is>
@@ -39813,171 +39357,57 @@
           <t>CCJ</t>
         </is>
       </c>
-      <c r="C31" s="33" t="n">
-        <v>-0.03537441206195591</v>
-      </c>
-      <c r="D31" s="34" t="n">
-        <v>15</v>
-      </c>
-      <c r="E31" s="30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F31" s="30" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G31" s="30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H31" s="30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I31" s="30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J31" s="30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K31" s="30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L31" s="30" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M31" s="30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N31" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="O31" s="30" t="inlineStr">
-        <is>
-          <t>Very Weak</t>
-        </is>
-      </c>
-      <c r="P31" s="32" t="inlineStr">
-        <is>
-          <t>Below every average</t>
-        </is>
-      </c>
+      <c r="C31" s="33" t="n"/>
+      <c r="D31" s="34" t="n"/>
+      <c r="E31" s="30" t="n"/>
+      <c r="F31" s="30" t="n"/>
+      <c r="G31" s="30" t="n"/>
+      <c r="H31" s="30" t="n"/>
+      <c r="I31" s="30" t="n"/>
+      <c r="J31" s="30" t="n"/>
+      <c r="K31" s="30" t="n"/>
+      <c r="L31" s="30" t="n"/>
+      <c r="M31" s="30" t="n"/>
+      <c r="N31" s="80" t="n"/>
+      <c r="O31" s="30" t="n"/>
+      <c r="P31" s="32" t="n"/>
       <c r="Q31" s="32" t="inlineStr">
         <is>
           <t>Cameco Corporation</t>
         </is>
       </c>
-      <c r="R31" s="81" t="n">
-        <v>93.26000213623047</v>
-      </c>
-      <c r="S31" s="82" t="n">
-        <v>-3.419998168945312</v>
-      </c>
-      <c r="T31" s="83" t="n">
-        <v>93.09999847412109</v>
-      </c>
-      <c r="U31" s="83" t="n">
-        <v>94.43000030517578</v>
-      </c>
-      <c r="V31" s="83" t="n">
-        <v>91.97000122070312</v>
-      </c>
-      <c r="W31" s="84" t="n">
-        <v>3466900</v>
-      </c>
-      <c r="X31" s="85" t="n">
-        <v>1.291722787623396</v>
-      </c>
-      <c r="Y31" s="35" t="n">
-        <v>40.82117169989679</v>
-      </c>
-      <c r="Z31" s="35" t="n">
-        <v>6.591726804515573</v>
-      </c>
-      <c r="AA31" s="35" t="n">
-        <v>13.26402845480098</v>
-      </c>
-      <c r="AB31" s="86" t="n">
-        <v>0.1118928792585194</v>
-      </c>
-      <c r="AC31" s="86" t="n">
-        <v>1.023297359570476</v>
-      </c>
-      <c r="AD31" s="86" t="n">
-        <v>-0.9114044803119563</v>
-      </c>
-      <c r="AE31" s="83" t="n">
-        <v>97.77997624310704</v>
-      </c>
-      <c r="AF31" s="83" t="n">
-        <v>98.42897418303481</v>
-      </c>
-      <c r="AG31" s="83" t="n">
-        <v>95.11420013427734</v>
-      </c>
-      <c r="AH31" s="83" t="n">
-        <v>102.7642998504639</v>
-      </c>
-      <c r="AI31" s="83" t="n">
-        <v>105.7460997772217</v>
-      </c>
-      <c r="AJ31" s="83" t="n">
-        <v>107.4401777173457</v>
-      </c>
-      <c r="AK31" s="83" t="n">
-        <v>99.80600051879883</v>
-      </c>
-      <c r="AL31" s="83" t="n">
-        <v>92.17182332025196</v>
-      </c>
-      <c r="AM31" s="87" t="n">
-        <v>0.07127020945922236</v>
-      </c>
-      <c r="AN31" s="36" t="n">
-        <v>15.29803250077923</v>
-      </c>
-      <c r="AO31" s="88" t="n">
-        <v>4.029571309708374</v>
-      </c>
-      <c r="AP31" s="83" t="n">
-        <v>135.2400054931641</v>
-      </c>
-      <c r="AQ31" s="83" t="n">
-        <v>77.52999877929688</v>
-      </c>
-      <c r="AR31" s="36" t="n">
-        <v>-31.04111331839272</v>
-      </c>
-      <c r="AS31" s="89" t="n">
-        <v>27.25697717368974</v>
-      </c>
-      <c r="AT31" s="33" t="n">
-        <v>-0.07425050512363762</v>
-      </c>
-      <c r="AU31" s="33" t="n">
-        <v>-0.04593348198229696</v>
-      </c>
-      <c r="AV31" s="33" t="n">
-        <v>-0.07626779930732408</v>
-      </c>
-      <c r="AW31" s="33" t="n">
-        <v>0.01934642380357809</v>
-      </c>
+      <c r="R31" s="81" t="n"/>
+      <c r="S31" s="82" t="n"/>
+      <c r="T31" s="83" t="n"/>
+      <c r="U31" s="83" t="n"/>
+      <c r="V31" s="83" t="n"/>
+      <c r="W31" s="84" t="n"/>
+      <c r="X31" s="85" t="n"/>
+      <c r="Y31" s="35" t="n"/>
+      <c r="Z31" s="35" t="n"/>
+      <c r="AA31" s="35" t="n"/>
+      <c r="AB31" s="86" t="n"/>
+      <c r="AC31" s="86" t="n"/>
+      <c r="AD31" s="86" t="n"/>
+      <c r="AE31" s="83" t="n"/>
+      <c r="AF31" s="83" t="n"/>
+      <c r="AG31" s="83" t="n"/>
+      <c r="AH31" s="83" t="n"/>
+      <c r="AI31" s="83" t="n"/>
+      <c r="AJ31" s="83" t="n"/>
+      <c r="AK31" s="83" t="n"/>
+      <c r="AL31" s="83" t="n"/>
+      <c r="AM31" s="87" t="n"/>
+      <c r="AN31" s="36" t="n"/>
+      <c r="AO31" s="88" t="n"/>
+      <c r="AP31" s="83" t="n"/>
+      <c r="AQ31" s="83" t="n"/>
+      <c r="AR31" s="36" t="n"/>
+      <c r="AS31" s="89" t="n"/>
+      <c r="AT31" s="33" t="n"/>
+      <c r="AU31" s="33" t="n"/>
+      <c r="AV31" s="33" t="n"/>
+      <c r="AW31" s="33" t="n"/>
       <c r="AX31" s="32" t="n"/>
       <c r="AY31" s="32" t="n"/>
       <c r="AZ31" s="32" t="n"/>
@@ -39993,7 +39423,7 @@
         <v>-0.06753561805941777</v>
       </c>
       <c r="D32" s="27" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E32" s="23" t="inlineStr">
         <is>
@@ -40169,7 +39599,7 @@
         <v>-0.05818884522736567</v>
       </c>
       <c r="D33" s="34" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E33" s="30" t="inlineStr">
         <is>
@@ -40697,7 +40127,7 @@
         <v>-0.05585777990701835</v>
       </c>
       <c r="D36" s="27" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E36" s="23" t="inlineStr">
         <is>
@@ -41225,7 +40655,7 @@
         <v>-0.05252956130238706</v>
       </c>
       <c r="D39" s="34" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E39" s="30" t="inlineStr">
         <is>
@@ -41401,7 +40831,7 @@
         <v>-0.05504342214372016</v>
       </c>
       <c r="D40" s="27" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E40" s="23" t="inlineStr">
         <is>
@@ -41753,7 +41183,7 @@
         <v>-0.132973987483646</v>
       </c>
       <c r="D42" s="27" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E42" s="23" t="inlineStr">
         <is>
@@ -42633,7 +42063,7 @@
         <v>-0.04981172839114034</v>
       </c>
       <c r="D47" s="34" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E47" s="30" t="inlineStr">
         <is>
@@ -43864,7 +43294,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:G66"/>
+  <dimension ref="B2:G65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -45386,21 +44816,21 @@
     <row r="58">
       <c r="B58" s="24" t="inlineStr">
         <is>
-          <t>CCJ</t>
+          <t>XLC</t>
         </is>
       </c>
       <c r="C58" s="101" t="inlineStr">
         <is>
-          <t>Cameco Corporation</t>
+          <t>State Street Communication Services Select Sector SPDR ETF</t>
         </is>
       </c>
       <c r="D58" s="106" t="inlineStr">
         <is>
-          <t>Volume 2.7x its 20-day average</t>
+          <t>MACD crossed down</t>
         </is>
       </c>
       <c r="E58" s="26" t="n">
-        <v>-0.01271552011175747</v>
+        <v>-0.0137071734440839</v>
       </c>
       <c r="F58" s="27" t="n">
         <v>1</v>
@@ -45424,7 +44854,7 @@
       </c>
       <c r="D59" s="107" t="inlineStr">
         <is>
-          <t>MACD crossed down</t>
+          <t>RSI dropped below 50</t>
         </is>
       </c>
       <c r="E59" s="33" t="n">
@@ -45452,7 +44882,7 @@
       </c>
       <c r="D60" s="106" t="inlineStr">
         <is>
-          <t>RSI dropped below 50</t>
+          <t>Lost the 50 DMA</t>
         </is>
       </c>
       <c r="E60" s="26" t="n">
@@ -45470,21 +44900,21 @@
     <row r="61">
       <c r="B61" s="31" t="inlineStr">
         <is>
-          <t>XLC</t>
+          <t>XLU</t>
         </is>
       </c>
       <c r="C61" s="102" t="inlineStr">
         <is>
-          <t>State Street Communication Services Select Sector SPDR ETF</t>
+          <t>State Street Utilities Select Sector SPDR ETF</t>
         </is>
       </c>
       <c r="D61" s="107" t="inlineStr">
         <is>
-          <t>Lost the 50 DMA</t>
+          <t>New 52-week low</t>
         </is>
       </c>
       <c r="E61" s="33" t="n">
-        <v>-0.0137071734440839</v>
+        <v>-0.01415207896432746</v>
       </c>
       <c r="F61" s="34" t="n">
         <v>1</v>
@@ -45498,21 +44928,21 @@
     <row r="62">
       <c r="B62" s="24" t="inlineStr">
         <is>
-          <t>XLU</t>
+          <t>XLB</t>
         </is>
       </c>
       <c r="C62" s="101" t="inlineStr">
         <is>
-          <t>State Street Utilities Select Sector SPDR ETF</t>
+          <t>State Street Materials Select Sector SPDR ETF</t>
         </is>
       </c>
       <c r="D62" s="106" t="inlineStr">
         <is>
-          <t>New 52-week low</t>
+          <t>Lost the 200 DMA</t>
         </is>
       </c>
       <c r="E62" s="26" t="n">
-        <v>-0.01415207896432746</v>
+        <v>-0.01419833206477661</v>
       </c>
       <c r="F62" s="27" t="n">
         <v>1</v>
@@ -45526,21 +44956,21 @@
     <row r="63">
       <c r="B63" s="31" t="inlineStr">
         <is>
-          <t>XLB</t>
+          <t>NFLX</t>
         </is>
       </c>
       <c r="C63" s="102" t="inlineStr">
         <is>
-          <t>State Street Materials Select Sector SPDR ETF</t>
+          <t>Netflix, Inc.</t>
         </is>
       </c>
       <c r="D63" s="107" t="inlineStr">
         <is>
-          <t>Lost the 200 DMA</t>
+          <t>Closed below lower band</t>
         </is>
       </c>
       <c r="E63" s="33" t="n">
-        <v>-0.01419833206477661</v>
+        <v>-0.04674009769191312</v>
       </c>
       <c r="F63" s="34" t="n">
         <v>1</v>
@@ -45564,7 +44994,7 @@
       </c>
       <c r="D64" s="106" t="inlineStr">
         <is>
-          <t>Closed below lower band</t>
+          <t>Volume 3.7x its 20-day average</t>
         </is>
       </c>
       <c r="E64" s="26" t="n">
@@ -45592,7 +45022,7 @@
       </c>
       <c r="D65" s="107" t="inlineStr">
         <is>
-          <t>Volume 3.7x its 20-day average</t>
+          <t>Gapped down 5.4% at the open</t>
         </is>
       </c>
       <c r="E65" s="33" t="n">
@@ -45607,40 +45037,12 @@
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="B66" s="24" t="inlineStr">
-        <is>
-          <t>NFLX</t>
-        </is>
-      </c>
-      <c r="C66" s="101" t="inlineStr">
-        <is>
-          <t>Netflix, Inc.</t>
-        </is>
-      </c>
-      <c r="D66" s="106" t="inlineStr">
-        <is>
-          <t>Gapped down 5.4% at the open</t>
-        </is>
-      </c>
-      <c r="E66" s="26" t="n">
-        <v>-0.04674009769191312</v>
-      </c>
-      <c r="F66" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="G66" s="23" t="inlineStr">
-        <is>
-          <t>Very Weak</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="B5:G66"/>
+  <autoFilter ref="B5:G65"/>
   <mergeCells count="1">
     <mergeCell ref="B2:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="E6:E66">
+  <conditionalFormatting sqref="E6:E65">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="-0.05"/>

</xml_diff>

<commit_message>
Daily workbook: 2026-09-21 23:20 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 21 Sep 2026, 09:10 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 21 Sep 2026, 11:20 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 21 Sep 2026, 09:10 PM · Yahoo Finance data</t>
+          <t>Built 21 Sep 2026, 11:20 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -5816,12 +5816,12 @@
       </c>
       <c r="AY19" s="79" t="inlineStr">
         <is>
+          <t>Nasdaq Ends Nearly 3% Higher As AI Stocks Pop, AMD Enters $1 Trillion Club — AMD, ARM, META, AMZN, PSKY In ...</t>
+        </is>
+      </c>
+      <c r="AZ19" s="79" t="inlineStr">
+        <is>
           <t>Opendoor Gains 5% but Is Still Down 24% in a Month. Will the Bulls or Bears Win?</t>
-        </is>
-      </c>
-      <c r="AZ19" s="79" t="inlineStr">
-        <is>
-          <t>Rocket Lab Climbs 7% as Cantor Reiterates $122 Target on Launch Record; Intuitive Machines Jumps 10%, AST S...</t>
         </is>
       </c>
     </row>
@@ -6493,7 +6493,7 @@
         <v>2.850006103515625</v>
       </c>
       <c r="T24" s="72" t="n">
-        <v>335.2799987792969</v>
+        <v>335.2000122070312</v>
       </c>
       <c r="U24" s="72" t="n">
         <v>339.6400146484375</v>
@@ -6681,7 +6681,7 @@
         <v>55.70001220703125</v>
       </c>
       <c r="T25" s="83" t="n">
-        <v>583.8800048828125</v>
+        <v>583.9400024414062</v>
       </c>
       <c r="U25" s="83" t="n">
         <v>616.6799926757812</v>
@@ -6772,17 +6772,17 @@
       </c>
       <c r="AX25" s="90" t="inlineStr">
         <is>
-          <t>Chip Stocks Rise As Four New Names Join SOX Index. AMD Breaks Out.</t>
+          <t>Dow Jones Futures: Falling Oil Prices, Yields Spark Market Rally; AMD, Intel, Micron, Nvidia, Sandisk Are K...</t>
         </is>
       </c>
       <c r="AY25" s="90" t="inlineStr">
         <is>
-          <t>Stock Market Today: Dow Up, Nasdaq Roars To Record As Micron Does This; AMD Hits New High (Live Coverage)</t>
+          <t>Advanced Micro Devices (AMD) Is Up 24.7% After Expanding Its Role In Regulated AI Infrastructure – Has The ...</t>
         </is>
       </c>
       <c r="AZ25" s="90" t="inlineStr">
         <is>
-          <t>AMD Storms Into $1 Trillion Club as Chip Stocks Charge Higher</t>
+          <t>Nasdaq Ends Nearly 3% Higher As AI Stocks Pop, AMD Enters $1 Trillion Club — AMD, ARM, META, AMZN, PSKY In ...</t>
         </is>
       </c>
     </row>
@@ -6869,7 +6869,7 @@
         <v>4.740005493164062</v>
       </c>
       <c r="T26" s="72" t="n">
-        <v>256.3999938964844</v>
+        <v>256.5199890136719</v>
       </c>
       <c r="U26" s="72" t="n">
         <v>259.489990234375</v>
@@ -6965,12 +6965,12 @@
       </c>
       <c r="AY26" s="79" t="inlineStr">
         <is>
-          <t>Amazon Takes Wearable AI Deeper Into Logistics</t>
+          <t>Amazon (AMZN) Laps the Stock Market: Here's Why</t>
         </is>
       </c>
       <c r="AZ26" s="79" t="inlineStr">
         <is>
-          <t>Sector Update: Tech Stocks Gain Late Afternoon</t>
+          <t>Amazon kicks out Meta's Muse in split over AI shopping</t>
         </is>
       </c>
     </row>
@@ -7245,7 +7245,7 @@
         <v>47.29000854492188</v>
       </c>
       <c r="T28" s="72" t="n">
-        <v>294.3599853515625</v>
+        <v>294.2200012207031</v>
       </c>
       <c r="U28" s="72" t="n">
         <v>324.1600036621094</v>
@@ -7346,7 +7346,7 @@
       </c>
       <c r="AZ28" s="79" t="inlineStr">
         <is>
-          <t>Intel, AMD, and Arm Stock Are Jumping. Thank Meta’s Muse AI Agent.</t>
+          <t>Arm Stock Surges As Meta’s Muse Reportedly Fuels CPU Rally — Meta Is Lead Partner On AGI CPU</t>
         </is>
       </c>
     </row>
@@ -7433,7 +7433,7 @@
         <v>3.369998931884766</v>
       </c>
       <c r="T29" s="83" t="n">
-        <v>59.54499816894531</v>
+        <v>59.55500030517578</v>
       </c>
       <c r="U29" s="83" t="n">
         <v>62.36000061035156</v>
@@ -7621,7 +7621,7 @@
         <v>5.050018310546875</v>
       </c>
       <c r="T30" s="72" t="n">
-        <v>358.6549987792969</v>
+        <v>358.8599853515625</v>
       </c>
       <c r="U30" s="72" t="n">
         <v>363.9700012207031</v>
@@ -8464,17 +8464,17 @@
       </c>
       <c r="AX34" s="79" t="inlineStr">
         <is>
+          <t>Google just disclosed something troubling about its AI</t>
+        </is>
+      </c>
+      <c r="AY34" s="79" t="inlineStr">
+        <is>
           <t>Google, Apple's new job postings go viral</t>
         </is>
       </c>
-      <c r="AY34" s="79" t="inlineStr">
+      <c r="AZ34" s="79" t="inlineStr">
         <is>
           <t>Sector Update: Tech Stocks Gain Late Afternoon</t>
-        </is>
-      </c>
-      <c r="AZ34" s="79" t="inlineStr">
-        <is>
-          <t>Google Just Got Hit With Another Massive Legal Setback</t>
         </is>
       </c>
     </row>
@@ -8840,17 +8840,17 @@
       </c>
       <c r="AX36" s="79" t="inlineStr">
         <is>
-          <t>Update: Nasdaq Composite Rallies to Record as AI Trade Lifts Chipmakers</t>
+          <t>Dow Jones Futures: Falling Oil Prices, Yields Spark Market Rally; AMD, Intel, Micron, Nvidia, Sandisk Are K...</t>
         </is>
       </c>
       <c r="AY36" s="79" t="inlineStr">
         <is>
-          <t>Intel's CEO Just Gave Micron Technology Investors Great News</t>
+          <t>AMD, Intel, Meta, Warner Bros., Moderna, Grail, Strategy, and More Stocks That Explain Today’s Market</t>
         </is>
       </c>
       <c r="AZ36" s="79" t="inlineStr">
         <is>
-          <t>AMD Hits $1 Trillion Market Cap: 3 Reasons Nvidia Sat Out the AI Rally</t>
+          <t>Meta’s Muse AI Agent Triggers Intel, Chip Stock Rally. AMD Hits $1T Market Cap.</t>
         </is>
       </c>
     </row>
@@ -9028,17 +9028,17 @@
       </c>
       <c r="AX37" s="90" t="inlineStr">
         <is>
+          <t>Microsoft (MSFT) Laps the Stock Market: Here's Why</t>
+        </is>
+      </c>
+      <c r="AY37" s="90" t="inlineStr">
+        <is>
+          <t>Microsoft (MSFT) Stock Looks Reasonable Despite Its 75% Five Year Run</t>
+        </is>
+      </c>
+      <c r="AZ37" s="90" t="inlineStr">
+        <is>
           <t>Microsoft Patent Hints At Contextual In-Game Ads</t>
-        </is>
-      </c>
-      <c r="AY37" s="90" t="inlineStr">
-        <is>
-          <t>Microsoft's Nadella Is Joining Trump and Xi and Tech Giants Are Coming Too</t>
-        </is>
-      </c>
-      <c r="AZ37" s="90" t="inlineStr">
-        <is>
-          <t>Microsoft Stays Flat as Hyderabad Adds AI Capacity Without Water Cooling</t>
         </is>
       </c>
     </row>
@@ -9404,17 +9404,17 @@
       </c>
       <c r="AX39" s="90" t="inlineStr">
         <is>
+          <t>Dow Jones Futures: Falling Oil Prices, Yields Spark Market Rally; AMD, Intel, Micron, Nvidia, Sandisk Are K...</t>
+        </is>
+      </c>
+      <c r="AY39" s="90" t="inlineStr">
+        <is>
+          <t>Micron (MU) Beats Stock Market Upswing: What Investors Need to Know</t>
+        </is>
+      </c>
+      <c r="AZ39" s="90" t="inlineStr">
+        <is>
           <t>Micron Stock Is Back Above $1,000. Is a Stock Split Coming?</t>
-        </is>
-      </c>
-      <c r="AY39" s="90" t="inlineStr">
-        <is>
-          <t>Stock Market Today: Dow Up, Nasdaq Roars To Record As Micron Does This; AMD Hits New High (Live Coverage)</t>
-        </is>
-      </c>
-      <c r="AZ39" s="90" t="inlineStr">
-        <is>
-          <t>Intel's CEO Just Gave Micron Technology Investors Great News</t>
         </is>
       </c>
     </row>
@@ -9780,17 +9780,17 @@
       </c>
       <c r="AX41" s="90" t="inlineStr">
         <is>
+          <t>Netflix (NFLX) Laps the Stock Market: Here's Why</t>
+        </is>
+      </c>
+      <c r="AY41" s="90" t="inlineStr">
+        <is>
           <t>Wells Fargo Cuts Netflix (NFLX) to Underweight as its 2026 Slide Deepens</t>
         </is>
       </c>
-      <c r="AY41" s="90" t="inlineStr">
+      <c r="AZ41" s="90" t="inlineStr">
         <is>
           <t>This Bearish Netflix Stock Trade Can Cash In On Video Streaming Giant's Woes</t>
-        </is>
-      </c>
-      <c r="AZ41" s="90" t="inlineStr">
-        <is>
-          <t>Ackman Bets $1 Billion on Netflix Redemption After $400 Million 2022 Loss</t>
         </is>
       </c>
     </row>
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
-          <t>Stock Market Today: Dow Up, Nasdaq Roars To Record As Micron Does This; AMD Hits New High (Live Coverage)</t>
+          <t>$500 a Month in Nvidia Stock Since ChatGPT Launched Is Now Worth About $79,000</t>
         </is>
       </c>
       <c r="AY43" s="90" t="inlineStr">
         <is>
-          <t>Nvidia Stock Can Surge on Trump’s China Talks. Why They Are Crucial.</t>
+          <t>Dow Jones Futures: Falling Oil Prices, Yields Spark Market Rally; AMD, Intel, Micron, Nvidia, Sandisk Are K...</t>
         </is>
       </c>
       <c r="AZ43" s="90" t="inlineStr">
         <is>
-          <t>Better AI Data Center Stock: Nebius vs. CoreWeave</t>
+          <t>Should You Forget Nvidia and Buy These 3 Millionaire-Maker AI Infrastructure Stocks Instead?</t>
         </is>
       </c>
     </row>
@@ -10344,17 +10344,17 @@
       </c>
       <c r="AX44" s="79" t="inlineStr">
         <is>
+          <t>Palantir's Alex Karp says AI's biggest names may never IPO — the play is telling Washington 'nationalize us...</t>
+        </is>
+      </c>
+      <c r="AY44" s="79" t="inlineStr">
+        <is>
           <t>Palantir Climbs as CEO Sends Blunt Message to AI Industry</t>
         </is>
       </c>
-      <c r="AY44" s="79" t="inlineStr">
+      <c r="AZ44" s="79" t="inlineStr">
         <is>
           <t>Palantir Stock Gets a Bullish Options Signal as Shares Jump 2.7%</t>
-        </is>
-      </c>
-      <c r="AZ44" s="79" t="inlineStr">
-        <is>
-          <t>OpenAI and Anthropic Weighed Mutual AI Tests. Palantir CEO Says One May Never List</t>
         </is>
       </c>
     </row>
@@ -10720,12 +10720,12 @@
       </c>
       <c r="AX46" s="79" t="inlineStr">
         <is>
+          <t>Rocket Lab Looks More and More Like a SpaceX Competitor. The Stock Is Up.</t>
+        </is>
+      </c>
+      <c r="AY46" s="79" t="inlineStr">
+        <is>
           <t>Archer Aviation vs. Rocket Lab: Which Aerospace Stock Is a Better Buy in 2026?</t>
-        </is>
-      </c>
-      <c r="AY46" s="79" t="inlineStr">
-        <is>
-          <t>Rocket Lab Looks More and More Like a SpaceX Competitor. The Stock Is Up.</t>
         </is>
       </c>
       <c r="AZ46" s="79" t="inlineStr">
@@ -10817,7 +10817,7 @@
         <v>-25.179931640625</v>
       </c>
       <c r="T47" s="83" t="n">
-        <v>1826</v>
+        <v>1826.660034179688</v>
       </c>
       <c r="U47" s="83" t="n">
         <v>1834.489990234375</v>
@@ -10908,17 +10908,17 @@
       </c>
       <c r="AX47" s="90" t="inlineStr">
         <is>
+          <t>Dow Jones Futures: Falling Oil Prices, Yields Spark Market Rally; AMD, Intel, Micron, Nvidia, Sandisk Are K...</t>
+        </is>
+      </c>
+      <c r="AY47" s="90" t="inlineStr">
+        <is>
+          <t>Top Stock Reports for Procter &amp; Gamble, Sandisk &amp; Analog Devices</t>
+        </is>
+      </c>
+      <c r="AZ47" s="90" t="inlineStr">
+        <is>
           <t>SanDisk Faces a Make-or-Break Test at $1,832</t>
-        </is>
-      </c>
-      <c r="AY47" s="90" t="inlineStr">
-        <is>
-          <t>SanDisk Falls 2% Despite Memory Rally; Micron Advances 3%, Western Digital Nudges Higher</t>
-        </is>
-      </c>
-      <c r="AZ47" s="90" t="inlineStr">
-        <is>
-          <t>Should You Buy Sandisk Stock Now or Wait for a Dip?</t>
         </is>
       </c>
     </row>
@@ -11005,7 +11005,7 @@
         <v>11.02999877929688</v>
       </c>
       <c r="T48" s="72" t="n">
-        <v>371.635009765625</v>
+        <v>371.6400146484375</v>
       </c>
       <c r="U48" s="72" t="n">
         <v>378.3599853515625</v>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 21 Sep 2026, 09:10 PM · Yahoo Finance data</t>
+          <t>Built 21 Sep 2026, 11:20 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 21 Sep 2026, 09:10 PM · Yahoo Finance data</t>
+          <t>Built 21 Sep 2026, 11:20 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 21 Sep 2026, 09:10 PM · Yahoo Finance data</t>
+          <t>Built 21 Sep 2026, 11:20 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 21 Sep 2026, 09:10 PM · Yahoo Finance data</t>
+          <t>Built 21 Sep 2026, 11:20 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-09-22 22:59 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 22 Sep 2026, 08:20 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 22 Sep 2026, 10:59 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -1589,22 +1589,22 @@
         </is>
       </c>
       <c r="E16" s="26" t="n">
-        <v>0.007236275900198041</v>
+        <v>0.007287647546651455</v>
       </c>
       <c r="F16" s="27" t="n">
         <v>8</v>
       </c>
       <c r="G16" s="28" t="n">
-        <v>66.8485297926847</v>
+        <v>66.85946474007164</v>
       </c>
       <c r="H16" s="29" t="n">
-        <v>6.89658601122014</v>
+        <v>6.901921446771309</v>
       </c>
       <c r="I16" s="26" t="n">
-        <v>0.06813970087824828</v>
+        <v>0.06819417875636802</v>
       </c>
       <c r="J16" s="26" t="n">
-        <v>0.07064533915616256</v>
+        <v>0.07069994482829345</v>
       </c>
     </row>
     <row r="17">
@@ -1853,22 +1853,22 @@
         </is>
       </c>
       <c r="E24" s="26" t="n">
-        <v>-0.01985689767535492</v>
+        <v>-0.01967803682991154</v>
       </c>
       <c r="F24" s="27" t="n">
         <v>2</v>
       </c>
       <c r="G24" s="28" t="n">
-        <v>29.82927985143608</v>
+        <v>29.88421862900658</v>
       </c>
       <c r="H24" s="29" t="n">
-        <v>-4.141559014976792</v>
+        <v>-4.124401767059894</v>
       </c>
       <c r="I24" s="26" t="n">
-        <v>-0.03623566603139816</v>
+        <v>-0.03605979405599691</v>
       </c>
       <c r="J24" s="26" t="n">
-        <v>-0.04679886305030978</v>
+        <v>-0.04662491869378871</v>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
@@ -2121,7 +2121,7 @@
         </is>
       </c>
       <c r="I33" s="26" t="n">
-        <v>-0.01985689767535492</v>
+        <v>-0.01967803682991154</v>
       </c>
       <c r="J33" s="27" t="n">
         <v>2</v>
@@ -2132,7 +2132,7 @@
         </is>
       </c>
       <c r="L33" s="28" t="n">
-        <v>29.82927985143608</v>
+        <v>29.88421862900658</v>
       </c>
     </row>
     <row r="34">
@@ -2465,7 +2465,7 @@
         </is>
       </c>
       <c r="I44" s="33" t="n">
-        <v>-0.01985689767535492</v>
+        <v>-0.01967803682991154</v>
       </c>
       <c r="J44" s="34" t="n">
         <v>2</v>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="L44" s="35" t="n">
-        <v>29.82927985143608</v>
+        <v>29.88421862900658</v>
       </c>
     </row>
     <row r="45">
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 22 Sep 2026, 08:20 PM · Yahoo Finance data</t>
+          <t>Built 22 Sep 2026, 10:59 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -3620,10 +3620,10 @@
         <v>169.1300048828125</v>
       </c>
       <c r="W7" s="73" t="n">
-        <v>7147580</v>
+        <v>7147653</v>
       </c>
       <c r="X7" s="74" t="n">
-        <v>0.9452421624465278</v>
+        <v>0.9452513601657703</v>
       </c>
       <c r="Y7" s="28" t="n">
         <v>36.46038369995261</v>
@@ -3810,10 +3810,10 @@
         <v>167.8699951171875</v>
       </c>
       <c r="W8" s="84" t="n">
-        <v>7035707</v>
+        <v>7037068</v>
       </c>
       <c r="X8" s="85" t="n">
-        <v>0.9541694326266994</v>
+        <v>0.9543452014286316</v>
       </c>
       <c r="Y8" s="35" t="n">
         <v>54.36945963073954</v>
@@ -3916,7 +3916,7 @@
         </is>
       </c>
       <c r="C9" s="26" t="n">
-        <v>-0.01985689767535492</v>
+        <v>-0.01967803682991154</v>
       </c>
       <c r="D9" s="27" t="n">
         <v>11</v>
@@ -3985,10 +3985,10 @@
         </is>
       </c>
       <c r="R9" s="70" t="n">
-        <v>54.79000091552734</v>
+        <v>54.79999923706055</v>
       </c>
       <c r="S9" s="71" t="n">
-        <v>-1.110000610351562</v>
+        <v>-1.100002288818359</v>
       </c>
       <c r="T9" s="72" t="n">
         <v>56</v>
@@ -4000,61 +4000,61 @@
         <v>54.54999923706055</v>
       </c>
       <c r="W9" s="73" t="n">
-        <v>68684300</v>
+        <v>69564269</v>
       </c>
       <c r="X9" s="74" t="n">
-        <v>2.098257559348897</v>
+        <v>2.122287386605865</v>
       </c>
       <c r="Y9" s="28" t="n">
-        <v>29.82927985143608</v>
+        <v>29.88421862900658</v>
       </c>
       <c r="Z9" s="28" t="n">
-        <v>5.925968485885146</v>
+        <v>6.172840669013255</v>
       </c>
       <c r="AA9" s="28" t="n">
         <v>23.08539275263411</v>
       </c>
       <c r="AB9" s="75" t="n">
-        <v>-0.4655087674763365</v>
+        <v>-0.4647111805734028</v>
       </c>
       <c r="AC9" s="75" t="n">
-        <v>-0.1701045364519713</v>
+        <v>-0.1699450190713845</v>
       </c>
       <c r="AD9" s="75" t="n">
-        <v>-0.2954042310243652</v>
+        <v>-0.2947661615020182</v>
       </c>
       <c r="AE9" s="72" t="n">
-        <v>56.02598939753015</v>
+        <v>56.02821124675975</v>
       </c>
       <c r="AF9" s="72" t="n">
-        <v>56.74248976901416</v>
+        <v>56.74339870733536</v>
       </c>
       <c r="AG9" s="72" t="n">
-        <v>57.15720008850098</v>
+        <v>57.15740005493164</v>
       </c>
       <c r="AH9" s="72" t="n">
-        <v>54.97070003509521</v>
+        <v>54.97080001831055</v>
       </c>
       <c r="AI9" s="72" t="n">
-        <v>53.71280002593994</v>
+        <v>53.71285001754761</v>
       </c>
       <c r="AJ9" s="72" t="n">
-        <v>59.10430726018718</v>
+        <v>59.10245155817658</v>
       </c>
       <c r="AK9" s="72" t="n">
-        <v>57.125</v>
+        <v>57.12549991607666</v>
       </c>
       <c r="AL9" s="72" t="n">
-        <v>55.14569273981282</v>
+        <v>55.14854827397675</v>
       </c>
       <c r="AM9" s="76" t="n">
-        <v>-0.08985260435305889</v>
+        <v>-0.08815315192686651</v>
       </c>
       <c r="AN9" s="29" t="n">
-        <v>6.929740954703489</v>
+        <v>6.92143314283205</v>
       </c>
       <c r="AO9" s="77" t="n">
-        <v>1.370974103459627</v>
+        <v>1.370723967691545</v>
       </c>
       <c r="AP9" s="72" t="n">
         <v>58.59999847412109</v>
@@ -4063,22 +4063,22 @@
         <v>47.66999816894531</v>
       </c>
       <c r="AR9" s="29" t="n">
-        <v>-6.501702487716477</v>
+        <v>-6.484640505133632</v>
       </c>
       <c r="AS9" s="78" t="n">
-        <v>65.14183483792249</v>
+        <v>65.23331078718178</v>
       </c>
       <c r="AT9" s="26" t="n">
-        <v>-0.03623566603139816</v>
+        <v>-0.03605979405599691</v>
       </c>
       <c r="AU9" s="26" t="n">
-        <v>-0.04679886305030978</v>
+        <v>-0.04662491869378871</v>
       </c>
       <c r="AV9" s="26" t="n">
-        <v>0.01688938064907775</v>
+        <v>0.01707494711780444</v>
       </c>
       <c r="AW9" s="26" t="n">
-        <v>0.0003651717655013265</v>
+        <v>0.0005477228235557519</v>
       </c>
       <c r="AX9" s="79" t="inlineStr">
         <is>
@@ -4190,10 +4190,10 @@
         <v>61.41999816894531</v>
       </c>
       <c r="W10" s="84" t="n">
-        <v>37931419</v>
+        <v>39244284</v>
       </c>
       <c r="X10" s="85" t="n">
-        <v>1.201810723574533</v>
+        <v>1.240826545371343</v>
       </c>
       <c r="Y10" s="35" t="n">
         <v>42.73137840954573</v>
@@ -4380,10 +4380,10 @@
         <v>82.28949737548828</v>
       </c>
       <c r="W11" s="73" t="n">
-        <v>9812934</v>
+        <v>9853525</v>
       </c>
       <c r="X11" s="74" t="n">
-        <v>1.0180430541219</v>
+        <v>1.022038972170681</v>
       </c>
       <c r="Y11" s="28" t="n">
         <v>41.2260809859164</v>
@@ -4570,10 +4570,10 @@
         <v>111.9749984741211</v>
       </c>
       <c r="W12" s="84" t="n">
-        <v>7338513</v>
+        <v>7641365</v>
       </c>
       <c r="X12" s="85" t="n">
-        <v>1.244677406468663</v>
+        <v>1.292723684460392</v>
       </c>
       <c r="Y12" s="35" t="n">
         <v>43.56414387982772</v>
@@ -4760,10 +4760,10 @@
         <v>113.4400024414062</v>
       </c>
       <c r="W13" s="73" t="n">
-        <v>7335454</v>
+        <v>7335475</v>
       </c>
       <c r="X13" s="74" t="n">
-        <v>1.543632529022546</v>
+        <v>1.543636607070755</v>
       </c>
       <c r="Y13" s="28" t="n">
         <v>53.72756049695191</v>
@@ -4950,10 +4950,10 @@
         <v>49.90999984741211</v>
       </c>
       <c r="W14" s="84" t="n">
-        <v>10097764</v>
+        <v>10098095</v>
       </c>
       <c r="X14" s="85" t="n">
-        <v>0.9305658700751868</v>
+        <v>0.9305949542700238</v>
       </c>
       <c r="Y14" s="35" t="n">
         <v>42.33556072918565</v>
@@ -5056,7 +5056,7 @@
         </is>
       </c>
       <c r="C15" s="26" t="n">
-        <v>0.007236275900198041</v>
+        <v>0.007287647546651455</v>
       </c>
       <c r="D15" s="27" t="n">
         <v>3</v>
@@ -5125,10 +5125,10 @@
         </is>
       </c>
       <c r="R15" s="70" t="n">
-        <v>196.2599945068359</v>
+        <v>196.2700042724609</v>
       </c>
       <c r="S15" s="71" t="n">
-        <v>1.409988403320312</v>
+        <v>1.419998168945312</v>
       </c>
       <c r="T15" s="72" t="n">
         <v>194.5899963378906</v>
@@ -5140,61 +5140,61 @@
         <v>194.4700012207031</v>
       </c>
       <c r="W15" s="73" t="n">
-        <v>8506555</v>
+        <v>8568988</v>
       </c>
       <c r="X15" s="74" t="n">
-        <v>1.259596326900781</v>
+        <v>1.268254776268384</v>
       </c>
       <c r="Y15" s="28" t="n">
-        <v>66.8485297926847</v>
+        <v>66.85946474007164</v>
       </c>
       <c r="Z15" s="28" t="n">
-        <v>98.30148822085202</v>
+        <v>98.37087999559955</v>
       </c>
       <c r="AA15" s="28" t="n">
         <v>12.01865653533205</v>
       </c>
       <c r="AB15" s="75" t="n">
-        <v>2.072475494809538</v>
+        <v>2.073273994631478</v>
       </c>
       <c r="AC15" s="75" t="n">
-        <v>1.14197352954448</v>
+        <v>1.142133229508867</v>
       </c>
       <c r="AD15" s="75" t="n">
-        <v>0.9305019652650586</v>
+        <v>0.9311407651226107</v>
       </c>
       <c r="AE15" s="72" t="n">
-        <v>190.1935840256214</v>
+        <v>190.1958084179824</v>
       </c>
       <c r="AF15" s="72" t="n">
-        <v>187.4334523063111</v>
+        <v>187.4343622850043</v>
       </c>
       <c r="AG15" s="72" t="n">
-        <v>183.5980004882813</v>
+        <v>183.5982006835937</v>
       </c>
       <c r="AH15" s="72" t="n">
-        <v>182.5355006408691</v>
+        <v>182.5356007385254</v>
       </c>
       <c r="AI15" s="72" t="n">
-        <v>162.9489751434326</v>
+        <v>162.9490251922607</v>
       </c>
       <c r="AJ15" s="72" t="n">
-        <v>193.9750630063005</v>
+        <v>193.9782003697751</v>
       </c>
       <c r="AK15" s="72" t="n">
-        <v>186.7610000610352</v>
+        <v>186.7615005493164</v>
       </c>
       <c r="AL15" s="72" t="n">
-        <v>179.5469371157698</v>
+        <v>179.5448007288577</v>
       </c>
       <c r="AM15" s="76" t="n">
-        <v>1.158366479324599</v>
+        <v>1.158784760326931</v>
       </c>
       <c r="AN15" s="29" t="n">
-        <v>7.72544904226013</v>
+        <v>7.728252128230277</v>
       </c>
       <c r="AO15" s="77" t="n">
-        <v>1.765976314326021</v>
+        <v>1.765886249575316</v>
       </c>
       <c r="AP15" s="72" t="n">
         <v>198.7299957275391</v>
@@ -5203,22 +5203,22 @@
         <v>126.6800003051758</v>
       </c>
       <c r="AR15" s="29" t="n">
-        <v>-1.242893007500245</v>
+        <v>-1.237856140474536</v>
       </c>
       <c r="AS15" s="78" t="n">
-        <v>96.57182320939263</v>
+        <v>96.58571601475137</v>
       </c>
       <c r="AT15" s="26" t="n">
-        <v>0.06813970087824828</v>
+        <v>0.06819417875636802</v>
       </c>
       <c r="AU15" s="26" t="n">
-        <v>0.07064533915616256</v>
+        <v>0.07069994482829345</v>
       </c>
       <c r="AV15" s="26" t="n">
-        <v>0.06553011512809626</v>
+        <v>0.06558445991061612</v>
       </c>
       <c r="AW15" s="26" t="n">
-        <v>0.3632006170922601</v>
+        <v>0.363270143837694</v>
       </c>
       <c r="AX15" s="79" t="inlineStr">
         <is>
@@ -5330,10 +5330,10 @@
         <v>42.41999816894531</v>
       </c>
       <c r="W16" s="84" t="n">
-        <v>4309823</v>
+        <v>4316302</v>
       </c>
       <c r="X16" s="85" t="n">
-        <v>0.8499905871016638</v>
+        <v>0.8512140024135633</v>
       </c>
       <c r="Y16" s="35" t="n">
         <v>31.35359492523786</v>
@@ -5520,10 +5520,10 @@
         <v>40.45000076293945</v>
       </c>
       <c r="W17" s="73" t="n">
-        <v>18131748</v>
+        <v>18147509</v>
       </c>
       <c r="X17" s="74" t="n">
-        <v>0.8588695768337393</v>
+        <v>0.8595840611324987</v>
       </c>
       <c r="Y17" s="28" t="n">
         <v>27.70088497571194</v>
@@ -5612,7 +5612,7 @@
       </c>
       <c r="AZ17" s="79" t="inlineStr">
         <is>
-          <t>Should You Invest in the State Street Utilities Select Sector SPDR ETF (XLU)?</t>
+          <t>Stock Market News for Sep 21, 2026</t>
         </is>
       </c>
     </row>
@@ -5729,10 +5729,10 @@
         <v>772.5900268554688</v>
       </c>
       <c r="W19" s="73" t="n">
-        <v>33575401</v>
+        <v>34483102</v>
       </c>
       <c r="X19" s="74" t="n">
-        <v>0.8101301117240773</v>
+        <v>0.8311215930668289</v>
       </c>
       <c r="Y19" s="28" t="n">
         <v>58.31343174753219</v>
@@ -5811,17 +5811,17 @@
       </c>
       <c r="AX19" s="79" t="inlineStr">
         <is>
-          <t>Skyworks Just Surged 33% in a Month: Is It Too Late to Buy SWKS Stock Now?</t>
+          <t>VGT Holders Bought ‘Tech’ and Own No Google, Meta, or Amazon: The Sector Rule That Decides What’s Inside</t>
         </is>
       </c>
       <c r="AY19" s="79" t="inlineStr">
         <is>
-          <t>Bloom Energy Just Ripped 38% in a Month: Take Profits, or Buy More?</t>
+          <t>The Market Is Near Another All-Time High and You’re 66 With Cash to Invest. Buying Now Feels Like the Top. ...</t>
         </is>
       </c>
       <c r="AZ19" s="79" t="inlineStr">
         <is>
-          <t>Adobe Is Down 32% This Year: Is ADBE Stock Dead Money or Due for a Bounce?</t>
+          <t>Nasdaq Jumps To Close At Record As Chipmakers Climb, Oil Prices Cool — AAPL, META, SPCX, MSFT, VKTX In Focus</t>
         </is>
       </c>
     </row>
@@ -5908,7 +5908,7 @@
         <v>5.99005126953125</v>
       </c>
       <c r="T20" s="83" t="n">
-        <v>740.97998046875</v>
+        <v>741.0050048828125</v>
       </c>
       <c r="U20" s="83" t="n">
         <v>748.3489990234375</v>
@@ -5917,10 +5917,10 @@
         <v>741</v>
       </c>
       <c r="W20" s="84" t="n">
-        <v>38676822</v>
+        <v>39451977</v>
       </c>
       <c r="X20" s="85" t="n">
-        <v>1.204463816950354</v>
+        <v>1.227122380926987</v>
       </c>
       <c r="Y20" s="35" t="n">
         <v>67.96300700369569</v>
@@ -6105,10 +6105,10 @@
         <v>286.0599975585938</v>
       </c>
       <c r="W21" s="73" t="n">
-        <v>24936918</v>
+        <v>25435821</v>
       </c>
       <c r="X21" s="74" t="n">
-        <v>1.18585833816299</v>
+        <v>1.208150166370825</v>
       </c>
       <c r="Y21" s="28" t="n">
         <v>41.67362648552117</v>
@@ -6293,10 +6293,10 @@
         <v>137.4600067138672</v>
       </c>
       <c r="W22" s="84" t="n">
-        <v>64657557</v>
+        <v>65009024</v>
       </c>
       <c r="X22" s="85" t="n">
-        <v>1.142291694927831</v>
+        <v>1.148144531373491</v>
       </c>
       <c r="Y22" s="35" t="n">
         <v>62.72892087930219</v>
@@ -6493,7 +6493,7 @@
         <v>0.769989013671875</v>
       </c>
       <c r="T24" s="72" t="n">
-        <v>340.135009765625</v>
+        <v>340.3299865722656</v>
       </c>
       <c r="U24" s="72" t="n">
         <v>345.3399963378906</v>
@@ -6502,10 +6502,10 @@
         <v>338.75</v>
       </c>
       <c r="W24" s="73" t="n">
-        <v>39489843</v>
+        <v>40599377</v>
       </c>
       <c r="X24" s="74" t="n">
-        <v>0.9155963748235209</v>
+        <v>0.9401123748153288</v>
       </c>
       <c r="Y24" s="28" t="n">
         <v>66.87815401332701</v>
@@ -6584,17 +6584,17 @@
       </c>
       <c r="AX24" s="79" t="inlineStr">
         <is>
+          <t>Meta’s new AI agent just got me $250 in flight credits</t>
+        </is>
+      </c>
+      <c r="AY24" s="79" t="inlineStr">
+        <is>
           <t>Apple doesn't need to be in first place for AI. Here's why.</t>
         </is>
       </c>
-      <c r="AY24" s="79" t="inlineStr">
-        <is>
-          <t>Apple Takes Aim at Nvidia’s AI Economics: New Macs Have ‘No Cost per Token,’ Hardware Chief Says</t>
-        </is>
-      </c>
       <c r="AZ24" s="79" t="inlineStr">
         <is>
-          <t>Apple’s New CEO Is Already Being Pressured to Drop the Chinese Chip Deal Tim Cook Fought to Keep</t>
+          <t>Stock Market Today: Dow Skids But Apple Eyes A Buy Point; Filing Says Trump Makes These Trades</t>
         </is>
       </c>
     </row>
@@ -6681,7 +6681,7 @@
         <v>8.25</v>
       </c>
       <c r="T25" s="83" t="n">
-        <v>606.5650024414062</v>
+        <v>607.0999755859375</v>
       </c>
       <c r="U25" s="83" t="n">
         <v>624.52001953125</v>
@@ -6690,10 +6690,10 @@
         <v>606.3125</v>
       </c>
       <c r="W25" s="84" t="n">
-        <v>27878184</v>
+        <v>28045099</v>
       </c>
       <c r="X25" s="85" t="n">
-        <v>1.319229329464831</v>
+        <v>1.326604031799133</v>
       </c>
       <c r="Y25" s="35" t="n">
         <v>73.87799261709131</v>
@@ -6772,17 +6772,17 @@
       </c>
       <c r="AX25" s="90" t="inlineStr">
         <is>
-          <t>AMD Stock Just Sent a Huge AI Signal</t>
+          <t>Advanced Micro Devices (AMD) Stock Moves 1.34%: What You Should Know</t>
         </is>
       </c>
       <c r="AY25" s="90" t="inlineStr">
         <is>
-          <t>Here's How AMD Joined the Rule Breakers $1 Trillion Club</t>
+          <t>Sandisk, Lennar, Viking Therapeutics, Shopify, GameStop, and More Stocks That Explain Today’s Market</t>
         </is>
       </c>
       <c r="AZ25" s="90" t="inlineStr">
         <is>
-          <t>AMD Stock Just Entered Rarefied Territory</t>
+          <t>AMD Stock Has Blown Past Nvidia This Year. Is It Still the Better Buy?</t>
         </is>
       </c>
     </row>
@@ -6869,7 +6869,7 @@
         <v>-3.470016479492188</v>
       </c>
       <c r="T26" s="72" t="n">
-        <v>255.1100006103516</v>
+        <v>255.3800048828125</v>
       </c>
       <c r="U26" s="72" t="n">
         <v>259</v>
@@ -6878,10 +6878,10 @@
         <v>253.7899932861328</v>
       </c>
       <c r="W26" s="73" t="n">
-        <v>41032595</v>
+        <v>41258805</v>
       </c>
       <c r="X26" s="74" t="n">
-        <v>1.211289677790828</v>
+        <v>1.217560909189923</v>
       </c>
       <c r="Y26" s="28" t="n">
         <v>49.21923987802839</v>
@@ -6960,17 +6960,17 @@
       </c>
       <c r="AX26" s="79" t="inlineStr">
         <is>
-          <t>Shopify Just Gave Meta's AI Agent a Major Boost</t>
+          <t>VGT Holders Bought ‘Tech’ and Own No Google, Meta, or Amazon: The Sector Rule That Decides What’s Inside</t>
         </is>
       </c>
       <c r="AY26" s="79" t="inlineStr">
         <is>
-          <t>Meta Platforms Just Hit an Amazon Roadblock</t>
+          <t>Amazon.com (AMZN) Blocks Rival AI Shopping Agent On Its Platform</t>
         </is>
       </c>
       <c r="AZ26" s="79" t="inlineStr">
         <is>
-          <t>Sector Update: Tech Stocks Higher in Afternoon Trading</t>
+          <t>GREEN FUEL FORWARD EXPANDS INDUSTRY ALLIANCE TO SUPPORT SUSTAINABLE AVIATION FUEL ADOPTION IN ASIA</t>
         </is>
       </c>
     </row>
@@ -7066,10 +7066,10 @@
         <v>90.48000335693359</v>
       </c>
       <c r="W27" s="84" t="n">
-        <v>4933373</v>
+        <v>4934486</v>
       </c>
       <c r="X27" s="85" t="n">
-        <v>1.081379988615571</v>
+        <v>1.081610760927659</v>
       </c>
       <c r="Y27" s="35" t="n">
         <v>66.93057679090926</v>
@@ -7148,17 +7148,17 @@
       </c>
       <c r="AX27" s="90" t="inlineStr">
         <is>
+          <t>Daily ETF Flows: ARKK Enters Top 10</t>
+        </is>
+      </c>
+      <c r="AY27" s="90" t="inlineStr">
+        <is>
           <t>Cathie Wood buys $19.2 million of tumbling AI stock</t>
         </is>
       </c>
-      <c r="AY27" s="90" t="inlineStr">
+      <c r="AZ27" s="90" t="inlineStr">
         <is>
           <t>Cathie Wood buys $27.9 million of surging megacap stock</t>
-        </is>
-      </c>
-      <c r="AZ27" s="90" t="inlineStr">
-        <is>
-          <t>Cathie Wood Sold Palantir and AMD, Then Poured $3.35 Million Into Archer Aviation. Is ARK Betting Big on Fl...</t>
         </is>
       </c>
     </row>
@@ -7254,10 +7254,10 @@
         <v>318.6849975585938</v>
       </c>
       <c r="W28" s="73" t="n">
-        <v>7348709</v>
+        <v>7363146</v>
       </c>
       <c r="X28" s="74" t="n">
-        <v>1.549675470998797</v>
+        <v>1.552483583966011</v>
       </c>
       <c r="Y28" s="28" t="n">
         <v>71.35819310240269</v>
@@ -7433,7 +7433,7 @@
         <v>1.799999237060547</v>
       </c>
       <c r="T29" s="83" t="n">
-        <v>61.90999984741211</v>
+        <v>61.97499847412109</v>
       </c>
       <c r="U29" s="83" t="n">
         <v>65.41000366210938</v>
@@ -7442,10 +7442,10 @@
         <v>60.99050140380859</v>
       </c>
       <c r="W29" s="84" t="n">
-        <v>10374650</v>
+        <v>10426708</v>
       </c>
       <c r="X29" s="85" t="n">
-        <v>1.059759423941309</v>
+        <v>1.064793981971666</v>
       </c>
       <c r="Y29" s="35" t="n">
         <v>51.8558068104839</v>
@@ -7524,17 +7524,17 @@
       </c>
       <c r="AX29" s="90" t="inlineStr">
         <is>
+          <t>AST SpaceMobile, Inc. (ASTS) Stock Moves 2.91%: What You Should Know</t>
+        </is>
+      </c>
+      <c r="AY29" s="90" t="inlineStr">
+        <is>
           <t>Prediction: AST SpaceMobile Will Be the Best-Performing Space Stock of 2027</t>
         </is>
       </c>
-      <c r="AY29" s="90" t="inlineStr">
+      <c r="AZ29" s="90" t="inlineStr">
         <is>
           <t>AST SpaceMobile Is Building Something the World Has Never Had. Here’s My Price Prediction</t>
-        </is>
-      </c>
-      <c r="AZ29" s="90" t="inlineStr">
-        <is>
-          <t>Rocket Lab Slides 5% as Space Names Give Back Gains; AST SpaceMobile Drops 6%, Planet Labs Sinks 4%</t>
         </is>
       </c>
     </row>
@@ -7630,10 +7630,10 @@
         <v>359.2901000976562</v>
       </c>
       <c r="W30" s="73" t="n">
-        <v>20382974</v>
+        <v>20440459</v>
       </c>
       <c r="X30" s="74" t="n">
-        <v>0.7468996999634524</v>
+        <v>0.7489272622727374</v>
       </c>
       <c r="Y30" s="28" t="n">
         <v>49.75937580567621</v>
@@ -7818,10 +7818,10 @@
         <v>92.25</v>
       </c>
       <c r="W31" s="84" t="n">
-        <v>3089392</v>
+        <v>3099259</v>
       </c>
       <c r="X31" s="85" t="n">
-        <v>1.037682126381237</v>
+        <v>1.04082383507031</v>
       </c>
       <c r="Y31" s="35" t="n">
         <v>46.64944348885832</v>
@@ -7997,7 +7997,7 @@
         <v>1.330001831054688</v>
       </c>
       <c r="T32" s="72" t="n">
-        <v>85.70999908447266</v>
+        <v>85.80000305175781</v>
       </c>
       <c r="U32" s="72" t="n">
         <v>89.23000335693359</v>
@@ -8006,10 +8006,10 @@
         <v>84.59999847412109</v>
       </c>
       <c r="W32" s="73" t="n">
-        <v>25786320</v>
+        <v>26353529</v>
       </c>
       <c r="X32" s="74" t="n">
-        <v>0.9531852000039478</v>
+        <v>0.9731317757539442</v>
       </c>
       <c r="Y32" s="28" t="n">
         <v>50.15792891131577</v>
@@ -8194,10 +8194,10 @@
         <v>547.7100219726562</v>
       </c>
       <c r="W33" s="84" t="n">
-        <v>9377999</v>
+        <v>9687163</v>
       </c>
       <c r="X33" s="85" t="n">
-        <v>0.8788859799438442</v>
+        <v>0.9065468449076659</v>
       </c>
       <c r="Y33" s="35" t="n">
         <v>56.97901373253364</v>
@@ -8373,7 +8373,7 @@
         <v>-3.459991455078125</v>
       </c>
       <c r="T34" s="72" t="n">
-        <v>353.239990234375</v>
+        <v>353.5</v>
       </c>
       <c r="U34" s="72" t="n">
         <v>359.9800109863281</v>
@@ -8382,10 +8382,10 @@
         <v>345.739990234375</v>
       </c>
       <c r="W34" s="73" t="n">
-        <v>19455169</v>
+        <v>19629631</v>
       </c>
       <c r="X34" s="74" t="n">
-        <v>1.125814739856203</v>
+        <v>1.135337258228878</v>
       </c>
       <c r="Y34" s="28" t="n">
         <v>55.09178007552627</v>
@@ -8464,17 +8464,17 @@
       </c>
       <c r="AX34" s="79" t="inlineStr">
         <is>
+          <t>INTEGRITY Global Security Launches AI Dome™, Nuclear-Grade Security That Neutralizes All AI Cyberattacks</t>
+        </is>
+      </c>
+      <c r="AY34" s="79" t="inlineStr">
+        <is>
+          <t>Google Appeals $425M Privacy Verdict</t>
+        </is>
+      </c>
+      <c r="AZ34" s="79" t="inlineStr">
+        <is>
           <t>Bill Ackman ditches a major AI stock after just one quarter</t>
-        </is>
-      </c>
-      <c r="AY34" s="79" t="inlineStr">
-        <is>
-          <t>IDrive Secures Educational Data with Cloud-to-Cloud Data Protection for Academic Institutions</t>
-        </is>
-      </c>
-      <c r="AZ34" s="79" t="inlineStr">
-        <is>
-          <t>Anthropic Unveils More Cost-Efficient Opus 5.5 Model Before IPO</t>
         </is>
       </c>
     </row>
@@ -8561,7 +8561,7 @@
         <v>1.319999694824219</v>
       </c>
       <c r="T35" s="83" t="n">
-        <v>46.97999954223633</v>
+        <v>46.98500061035156</v>
       </c>
       <c r="U35" s="83" t="n">
         <v>49.34999847412109</v>
@@ -8570,10 +8570,10 @@
         <v>46.86000061035156</v>
       </c>
       <c r="W35" s="84" t="n">
-        <v>33578434</v>
+        <v>33625427</v>
       </c>
       <c r="X35" s="85" t="n">
-        <v>0.8216752435935969</v>
+        <v>0.8227778706325699</v>
       </c>
       <c r="Y35" s="35" t="n">
         <v>62.34497022921656</v>
@@ -8652,17 +8652,17 @@
       </c>
       <c r="AX35" s="90" t="inlineStr">
         <is>
+          <t>Iren (IREN) Stock Looks Stretched With AI Hopes Already Priced In</t>
+        </is>
+      </c>
+      <c r="AY35" s="90" t="inlineStr">
+        <is>
           <t>IREN’s Energy Pipeline Optionality is Very Appealing So Should You Buy It?</t>
         </is>
       </c>
-      <c r="AY35" s="90" t="inlineStr">
+      <c r="AZ35" s="90" t="inlineStr">
         <is>
           <t>IREN Broadens Its AI Customer Base: Can Diversification Pay Off?</t>
-        </is>
-      </c>
-      <c r="AZ35" s="90" t="inlineStr">
-        <is>
-          <t>Iris Energy Is Sitting on $7.6 Billion in Cash and Building One of the Largest AI Data Centers in the World...</t>
         </is>
       </c>
     </row>
@@ -8749,7 +8749,7 @@
         <v>2.080001831054688</v>
       </c>
       <c r="T36" s="72" t="n">
-        <v>120.1500015258789</v>
+        <v>120.1100006103516</v>
       </c>
       <c r="U36" s="72" t="n">
         <v>124.0899963378906</v>
@@ -8758,10 +8758,10 @@
         <v>120.0749969482422</v>
       </c>
       <c r="W36" s="73" t="n">
-        <v>107356649</v>
+        <v>107684537</v>
       </c>
       <c r="X36" s="74" t="n">
-        <v>1.037883309860537</v>
+        <v>1.040888231110729</v>
       </c>
       <c r="Y36" s="28" t="n">
         <v>72.05534146051558</v>
@@ -8845,12 +8845,12 @@
       </c>
       <c r="AY36" s="79" t="inlineStr">
         <is>
+          <t>Intel (INTC) Stock Moves 1.71%: What You Should Know</t>
+        </is>
+      </c>
+      <c r="AZ36" s="79" t="inlineStr">
+        <is>
           <t>Intel Is Up 25% in 5 Days. The $145 Price Target Just Moved Too</t>
-        </is>
-      </c>
-      <c r="AZ36" s="79" t="inlineStr">
-        <is>
-          <t>Intel Drops as Muse Revives the Server CPU Thesis</t>
         </is>
       </c>
     </row>
@@ -8937,7 +8937,7 @@
         <v>-3.6099853515625</v>
       </c>
       <c r="T37" s="83" t="n">
-        <v>507.3200073242188</v>
+        <v>507.5150146484375</v>
       </c>
       <c r="U37" s="83" t="n">
         <v>508.5</v>
@@ -8946,10 +8946,10 @@
         <v>493.6499938964844</v>
       </c>
       <c r="W37" s="84" t="n">
-        <v>20581454</v>
+        <v>20867650</v>
       </c>
       <c r="X37" s="85" t="n">
-        <v>0.9575511595234667</v>
+        <v>0.9702204780257161</v>
       </c>
       <c r="Y37" s="35" t="n">
         <v>54.81814757076656</v>
@@ -9028,17 +9028,17 @@
       </c>
       <c r="AX37" s="90" t="inlineStr">
         <is>
-          <t>Microsoft Azure, M365 Commercial Can Sustain Acceleration in Fiscal 2027 Despite Some Risks, Oppenheimer Says</t>
+          <t>Oppenheimer Revamps Microsoft Stock Price Target For 2027</t>
         </is>
       </c>
       <c r="AY37" s="90" t="inlineStr">
         <is>
-          <t>Microsoft (MSFT) Raises Its Dividend 8%. Does AI Spending Change the Investment Case?</t>
+          <t>$223 Billion Back To Shareholders: Inside The MSFT Machine</t>
         </is>
       </c>
       <c r="AZ37" s="90" t="inlineStr">
         <is>
-          <t>BNP Paribas Spots What Could Move Microsoft Stock Next</t>
+          <t>Microsoft Scores Positive Reviews On AI Momentum</t>
         </is>
       </c>
     </row>
@@ -9125,7 +9125,7 @@
         <v>-1.169998168945312</v>
       </c>
       <c r="T38" s="72" t="n">
-        <v>167.5449981689453</v>
+        <v>167.4900054931641</v>
       </c>
       <c r="U38" s="72" t="n">
         <v>171.1699981689453</v>
@@ -9134,10 +9134,10 @@
         <v>167.25</v>
       </c>
       <c r="W38" s="73" t="n">
-        <v>23346006</v>
+        <v>23484383</v>
       </c>
       <c r="X38" s="74" t="n">
-        <v>0.8775918569871625</v>
+        <v>0.8825639993197634</v>
       </c>
       <c r="Y38" s="28" t="n">
         <v>70.04315352722058</v>
@@ -9313,7 +9313,7 @@
         <v>52.2000732421875</v>
       </c>
       <c r="T39" s="83" t="n">
-        <v>1032.849975585938</v>
+        <v>1033.280029296875</v>
       </c>
       <c r="U39" s="83" t="n">
         <v>1097.25</v>
@@ -9322,10 +9322,10 @@
         <v>1030.015014648438</v>
       </c>
       <c r="W39" s="84" t="n">
-        <v>28578068</v>
+        <v>28773640</v>
       </c>
       <c r="X39" s="85" t="n">
-        <v>1.13939492061999</v>
+        <v>1.146745209905541</v>
       </c>
       <c r="Y39" s="35" t="n">
         <v>66.06200731108626</v>
@@ -9404,17 +9404,17 @@
       </c>
       <c r="AX39" s="90" t="inlineStr">
         <is>
-          <t>Micron Stock Climbs Despite $25 Billion Plant Labor Dispute</t>
+          <t>Micron's Memory Boom Is Facing a New Test</t>
         </is>
       </c>
       <c r="AY39" s="90" t="inlineStr">
         <is>
-          <t>Micron, IBD Stock Of The Day, Surges Past Early Buy Point With Earnings Ahead</t>
+          <t>Dow Jones Futures: Nasdaq Hits New High; Sandisk, Micron Trigger Buy Signals</t>
         </is>
       </c>
       <c r="AZ39" s="90" t="inlineStr">
         <is>
-          <t>Michael Burry Adds To Micron, Nebius, Palantir Shorts As Acer Flags Rising Memory Supply</t>
+          <t>Micron vs. SanDisk: Comparing Two Red-Hot AI Memory Stocks</t>
         </is>
       </c>
     </row>
@@ -9501,7 +9501,7 @@
         <v>3.319992065429688</v>
       </c>
       <c r="T40" s="72" t="n">
-        <v>233.2400054931641</v>
+        <v>233.5099945068359</v>
       </c>
       <c r="U40" s="72" t="n">
         <v>246.6100006103516</v>
@@ -9510,10 +9510,10 @@
         <v>231.7550048828125</v>
       </c>
       <c r="W40" s="73" t="n">
-        <v>15179652</v>
+        <v>15303929</v>
       </c>
       <c r="X40" s="74" t="n">
-        <v>1.02370417761672</v>
+        <v>1.031653002172532</v>
       </c>
       <c r="Y40" s="28" t="n">
         <v>56.55373500283283</v>
@@ -9689,7 +9689,7 @@
         <v>-1.199996948242188</v>
       </c>
       <c r="T41" s="83" t="n">
-        <v>73.69000244140625</v>
+        <v>73.75299835205078</v>
       </c>
       <c r="U41" s="83" t="n">
         <v>73.76000213623047</v>
@@ -9698,10 +9698,10 @@
         <v>71.58010101318359</v>
       </c>
       <c r="W41" s="84" t="n">
-        <v>33976652</v>
+        <v>34214890</v>
       </c>
       <c r="X41" s="85" t="n">
-        <v>1.05587996384271</v>
+        <v>1.062890136336951</v>
       </c>
       <c r="Y41" s="35" t="n">
         <v>38.55205799342562</v>
@@ -9780,17 +9780,17 @@
       </c>
       <c r="AX41" s="90" t="inlineStr">
         <is>
+          <t>Netflix Stock Drops on HSBC Downgrade, Citing YouTube Threat</t>
+        </is>
+      </c>
+      <c r="AY41" s="90" t="inlineStr">
+        <is>
+          <t>Netflix Stock Downgraded As YouTube Swipes Viewers</t>
+        </is>
+      </c>
+      <c r="AZ41" s="90" t="inlineStr">
+        <is>
           <t>HSBC Resets Netflix Stock Target For 2026</t>
-        </is>
-      </c>
-      <c r="AY41" s="90" t="inlineStr">
-        <is>
-          <t>Netflix Stock Downgraded As YouTube Swipes Viewers</t>
-        </is>
-      </c>
-      <c r="AZ41" s="90" t="inlineStr">
-        <is>
-          <t>Netflix stock has a strange stock price target problem</t>
         </is>
       </c>
     </row>
@@ -9886,10 +9886,10 @@
         <v>10.47999954223633</v>
       </c>
       <c r="W42" s="73" t="n">
-        <v>105978380</v>
+        <v>106907601</v>
       </c>
       <c r="X42" s="74" t="n">
-        <v>1.261842906515133</v>
+        <v>1.272203001273955</v>
       </c>
       <c r="Y42" s="28" t="n">
         <v>55.23938997408226</v>
@@ -10065,7 +10065,7 @@
         <v>1.489990234375</v>
       </c>
       <c r="T43" s="83" t="n">
-        <v>226.8500061035156</v>
+        <v>226.9100036621094</v>
       </c>
       <c r="U43" s="83" t="n">
         <v>229.9799957275391</v>
@@ -10074,10 +10074,10 @@
         <v>226.5</v>
       </c>
       <c r="W43" s="84" t="n">
-        <v>91975117</v>
+        <v>93296546</v>
       </c>
       <c r="X43" s="85" t="n">
-        <v>0.6910921354270751</v>
+        <v>0.7006733727155737</v>
       </c>
       <c r="Y43" s="35" t="n">
         <v>59.36025833517122</v>
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
-          <t>Americans Stopped Drinking Wine. California Lost Legacy Vineyards.</t>
+          <t>Nvidia’s Cooling Stock Valuations Are Being Looked At As A Warning Signal</t>
         </is>
       </c>
       <c r="AY43" s="90" t="inlineStr">
         <is>
-          <t>3 Big Tech Stocks With the Most Upside Right Now</t>
+          <t>Nvidia Backed SB Energy’s $50 Billion Valuation Push. Wall Street Just Hit the Brakes</t>
         </is>
       </c>
       <c r="AZ43" s="90" t="inlineStr">
         <is>
-          <t>Is NVIDIA Funding Its Own Stock Rally?</t>
+          <t>JEPI’s 4.42% Gain Looks Modest Next to FYEE’s 12.4% Run in 2026</t>
         </is>
       </c>
     </row>
@@ -10253,7 +10253,7 @@
         <v>1.900009155273438</v>
       </c>
       <c r="T44" s="72" t="n">
-        <v>185.125</v>
+        <v>185.0850067138672</v>
       </c>
       <c r="U44" s="72" t="n">
         <v>185.5399932861328</v>
@@ -10262,10 +10262,10 @@
         <v>182.0299987792969</v>
       </c>
       <c r="W44" s="73" t="n">
-        <v>21799289</v>
+        <v>21859169</v>
       </c>
       <c r="X44" s="74" t="n">
-        <v>0.8004552256558806</v>
+        <v>0.8025657467642598</v>
       </c>
       <c r="Y44" s="28" t="n">
         <v>62.47361240756932</v>
@@ -10344,17 +10344,17 @@
       </c>
       <c r="AX44" s="79" t="inlineStr">
         <is>
+          <t>Palantir's Huge Rally Has Wall Street Asking a New Question</t>
+        </is>
+      </c>
+      <c r="AY44" s="79" t="inlineStr">
+        <is>
+          <t>Palantir Gains as Karp Puts Liability Before AI Listings</t>
+        </is>
+      </c>
+      <c r="AZ44" s="79" t="inlineStr">
+        <is>
           <t>Prediction: 3 Stocks That Will Be Worth More Than Palantir 5 Years From Now</t>
-        </is>
-      </c>
-      <c r="AY44" s="79" t="inlineStr">
-        <is>
-          <t>Is Palantir a Millionaire-Maker Stock?</t>
-        </is>
-      </c>
-      <c r="AZ44" s="79" t="inlineStr">
-        <is>
-          <t>Michael Burry Adds To Micron, Nebius, Palantir Shorts As Acer Flags Rising Memory Supply</t>
         </is>
       </c>
     </row>
@@ -10441,7 +10441,7 @@
         <v>4.040008544921875</v>
       </c>
       <c r="T45" s="83" t="n">
-        <v>192</v>
+        <v>192.1199951171875</v>
       </c>
       <c r="U45" s="83" t="n">
         <v>199.1499938964844</v>
@@ -10450,10 +10450,10 @@
         <v>191.6600036621094</v>
       </c>
       <c r="W45" s="84" t="n">
-        <v>11428427</v>
+        <v>11465322</v>
       </c>
       <c r="X45" s="85" t="n">
-        <v>0.7840978385261814</v>
+        <v>0.786529634482675</v>
       </c>
       <c r="Y45" s="35" t="n">
         <v>67.57176020386714</v>
@@ -10532,17 +10532,17 @@
       </c>
       <c r="AX45" s="90" t="inlineStr">
         <is>
-          <t>Qualcomm reveals two new smartphone chips focusing on agentic AI</t>
+          <t>Meta’s Muse just changed the AI game</t>
         </is>
       </c>
       <c r="AY45" s="90" t="inlineStr">
         <is>
-          <t>Qualcomm Slips as Googlebook Opens a New PC Lane</t>
+          <t>Qualcomm CFO on agentic AI and the race to the edge</t>
         </is>
       </c>
       <c r="AZ45" s="90" t="inlineStr">
         <is>
-          <t>Qualcomm Stock Jumped 9% on Monday. Can It Bring More Meaningful Upside in 2026?</t>
+          <t>Qualcomm reveals 2 new smartphone chips focusing on agentic AI</t>
         </is>
       </c>
     </row>
@@ -10629,7 +10629,7 @@
         <v>2.090003967285156</v>
       </c>
       <c r="T46" s="72" t="n">
-        <v>71.64499664306641</v>
+        <v>71.73999786376953</v>
       </c>
       <c r="U46" s="72" t="n">
         <v>72.5</v>
@@ -10638,10 +10638,10 @@
         <v>70.09999847412109</v>
       </c>
       <c r="W46" s="73" t="n">
-        <v>21150576</v>
+        <v>21927781</v>
       </c>
       <c r="X46" s="74" t="n">
-        <v>1.125609680656573</v>
+        <v>1.164563218403716</v>
       </c>
       <c r="Y46" s="28" t="n">
         <v>57.2022118839521</v>
@@ -10720,17 +10720,17 @@
       </c>
       <c r="AX46" s="79" t="inlineStr">
         <is>
+          <t>Rocket Lab Corporation (RKLB) Stock Moves 2.99%: What You Should Know</t>
+        </is>
+      </c>
+      <c r="AY46" s="79" t="inlineStr">
+        <is>
+          <t>Why Rocket Lab Is Up Today</t>
+        </is>
+      </c>
+      <c r="AZ46" s="79" t="inlineStr">
+        <is>
           <t>Wall Street Thinks Rocket Lab Is a Buy. Here's Why I'm Not So Sure.</t>
-        </is>
-      </c>
-      <c r="AY46" s="79" t="inlineStr">
-        <is>
-          <t>Redwire vs. Rocket Lab: Which Space Stock Is a Better Buy in 2026?</t>
-        </is>
-      </c>
-      <c r="AZ46" s="79" t="inlineStr">
-        <is>
-          <t>Rocket Lab Stock Breaks Above Key Trendline</t>
         </is>
       </c>
     </row>
@@ -10817,7 +10817,7 @@
         <v>120.4000244140625</v>
       </c>
       <c r="T47" s="83" t="n">
-        <v>1757.505004882812</v>
+        <v>1758.550048828125</v>
       </c>
       <c r="U47" s="83" t="n">
         <v>1909.47998046875</v>
@@ -10826,10 +10826,10 @@
         <v>1758.140014648438</v>
       </c>
       <c r="W47" s="84" t="n">
-        <v>12728127</v>
+        <v>12806071</v>
       </c>
       <c r="X47" s="85" t="n">
-        <v>1.175844740932823</v>
+        <v>1.182619554372934</v>
       </c>
       <c r="Y47" s="35" t="n">
         <v>64.68501912101556</v>
@@ -10908,17 +10908,17 @@
       </c>
       <c r="AX47" s="90" t="inlineStr">
         <is>
-          <t>Sandisk Jumps 6.6% as $2,400 Target Prices AI Storage Scarcity</t>
+          <t>Dow Jones Futures: Nasdaq Hits New High; Sandisk, Micron Trigger Buy Signals</t>
         </is>
       </c>
       <c r="AY47" s="90" t="inlineStr">
         <is>
-          <t>What Are You Really Paying For SanDisk's AI Flash Boom?</t>
+          <t>5-star analyst sets jaw-dropping price target on SanDisk stock</t>
         </is>
       </c>
       <c r="AZ47" s="90" t="inlineStr">
         <is>
-          <t>Sandisk, Lennar, Viking Therapeutics, Shopify, GameStop, and More Stocks That Explain Today’s Market</t>
+          <t>Micron vs. SanDisk: Comparing Two Red-Hot AI Memory Stocks</t>
         </is>
       </c>
     </row>
@@ -11014,10 +11014,10 @@
         <v>372.8800048828125</v>
       </c>
       <c r="W48" s="73" t="n">
-        <v>27978205</v>
+        <v>28089930</v>
       </c>
       <c r="X48" s="74" t="n">
-        <v>0.7212223316849438</v>
+        <v>0.7239981219302735</v>
       </c>
       <c r="Y48" s="28" t="n">
         <v>60.08354763375358</v>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 22 Sep 2026, 08:20 PM · Yahoo Finance data</t>
+          <t>Built 22 Sep 2026, 10:59 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 22 Sep 2026, 08:20 PM · Yahoo Finance data</t>
+          <t>Built 22 Sep 2026, 10:59 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 22 Sep 2026, 08:20 PM · Yahoo Finance data</t>
+          <t>Built 22 Sep 2026, 10:59 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 22 Sep 2026, 08:20 PM · Yahoo Finance data</t>
+          <t>Built 22 Sep 2026, 10:59 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -43355,22 +43355,22 @@
         </is>
       </c>
       <c r="D6" s="26" t="n">
-        <v>0.007236275900198041</v>
+        <v>0.007287647546651455</v>
       </c>
       <c r="E6" s="26" t="n">
-        <v>0.06813970087824828</v>
+        <v>0.06819417875636802</v>
       </c>
       <c r="F6" s="26" t="n">
-        <v>0.07064533915616256</v>
+        <v>0.07069994482829345</v>
       </c>
       <c r="G6" s="26" t="n">
-        <v>0.06553011512809626</v>
+        <v>0.06558445991061612</v>
       </c>
       <c r="H6" s="26" t="n">
-        <v>0.4330777574314872</v>
+        <v>0.433150848091203</v>
       </c>
       <c r="I6" s="26" t="n">
-        <v>0.3632006170922601</v>
+        <v>0.363270143837694</v>
       </c>
       <c r="J6" s="27" t="n">
         <v>8</v>
@@ -43545,22 +43545,22 @@
         </is>
       </c>
       <c r="D11" s="33" t="n">
-        <v>-0.01985689767535492</v>
+        <v>-0.01967803682991154</v>
       </c>
       <c r="E11" s="33" t="n">
-        <v>-0.03623566603139816</v>
+        <v>-0.03605979405599691</v>
       </c>
       <c r="F11" s="33" t="n">
-        <v>-0.04679886305030978</v>
+        <v>-0.04662491869378871</v>
       </c>
       <c r="G11" s="33" t="n">
-        <v>0.01688938064907775</v>
+        <v>0.01707494711780444</v>
       </c>
       <c r="H11" s="33" t="n">
-        <v>0.1120357297844081</v>
+        <v>0.1122386589794619</v>
       </c>
       <c r="I11" s="33" t="n">
-        <v>0.0003651717655013265</v>
+        <v>0.0005477228235557519</v>
       </c>
       <c r="J11" s="34" t="n">
         <v>2</v>
@@ -44364,7 +44364,7 @@
         </is>
       </c>
       <c r="E21" s="33" t="n">
-        <v>0.007236275900198041</v>
+        <v>0.007287647546651455</v>
       </c>
       <c r="F21" s="34" t="n">
         <v>8</v>
@@ -44500,7 +44500,7 @@
       </c>
       <c r="D26" s="107" t="inlineStr">
         <is>
-          <t>Gapped up 2.5% at the open</t>
+          <t>Gapped up 2.6% at the open</t>
         </is>
       </c>
       <c r="E26" s="26" t="n">
@@ -44952,7 +44952,7 @@
         </is>
       </c>
       <c r="E42" s="26" t="n">
-        <v>-0.01985689767535492</v>
+        <v>-0.01967803682991154</v>
       </c>
       <c r="F42" s="27" t="n">
         <v>2</v>
@@ -44980,7 +44980,7 @@
         </is>
       </c>
       <c r="E43" s="33" t="n">
-        <v>-0.01985689767535492</v>
+        <v>-0.01967803682991154</v>
       </c>
       <c r="F43" s="34" t="n">
         <v>2</v>
@@ -45008,7 +45008,7 @@
         </is>
       </c>
       <c r="E44" s="26" t="n">
-        <v>-0.01985689767535492</v>
+        <v>-0.01967803682991154</v>
       </c>
       <c r="F44" s="27" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
Daily workbook: 2026-09-22 23:35 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 22 Sep 2026, 10:59 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 22 Sep 2026, 11:35 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 22 Sep 2026, 10:59 PM · Yahoo Finance data</t>
+          <t>Built 22 Sep 2026, 11:35 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -9028,17 +9028,17 @@
       </c>
       <c r="AX37" s="90" t="inlineStr">
         <is>
+          <t>Microsoft kills 35-year-old Office app Oct. 1</t>
+        </is>
+      </c>
+      <c r="AY37" s="90" t="inlineStr">
+        <is>
           <t>Oppenheimer Revamps Microsoft Stock Price Target For 2027</t>
         </is>
       </c>
-      <c r="AY37" s="90" t="inlineStr">
+      <c r="AZ37" s="90" t="inlineStr">
         <is>
           <t>$223 Billion Back To Shareholders: Inside The MSFT Machine</t>
-        </is>
-      </c>
-      <c r="AZ37" s="90" t="inlineStr">
-        <is>
-          <t>Microsoft Scores Positive Reviews On AI Momentum</t>
         </is>
       </c>
     </row>
@@ -9216,17 +9216,17 @@
       </c>
       <c r="AX38" s="79" t="inlineStr">
         <is>
+          <t>Strategy CEO Phong Le Reveals the One Mistake Behind STRC's 25% Collapse</t>
+        </is>
+      </c>
+      <c r="AY38" s="79" t="inlineStr">
+        <is>
           <t>Analyst predicts 35% upside for Saylor's Strategy</t>
         </is>
       </c>
-      <c r="AY38" s="79" t="inlineStr">
+      <c r="AZ38" s="79" t="inlineStr">
         <is>
           <t>MicroStrategy CEO Says Jamie Dimon Is a Bitcoiner Behind the Scenes</t>
-        </is>
-      </c>
-      <c r="AZ38" s="79" t="inlineStr">
-        <is>
-          <t>MSTR, HOOD, RIOT Stocks Lead Gains In Fundstrat's Granny Shots ETF Last Week, Says Tom Lee</t>
         </is>
       </c>
     </row>
@@ -9404,12 +9404,12 @@
       </c>
       <c r="AX39" s="90" t="inlineStr">
         <is>
+          <t>Dow Jones Futures: Nasdaq Hits New High; Sandisk, Micron Trigger Buy Signals</t>
+        </is>
+      </c>
+      <c r="AY39" s="90" t="inlineStr">
+        <is>
           <t>Micron's Memory Boom Is Facing a New Test</t>
-        </is>
-      </c>
-      <c r="AY39" s="90" t="inlineStr">
-        <is>
-          <t>Dow Jones Futures: Nasdaq Hits New High; Sandisk, Micron Trigger Buy Signals</t>
         </is>
       </c>
       <c r="AZ39" s="90" t="inlineStr">
@@ -10908,17 +10908,17 @@
       </c>
       <c r="AX47" s="90" t="inlineStr">
         <is>
+          <t>Sandisk (SNDK) Has Signed Away Two Thirds of Next Year’s Output. Can the AI Storage Boom Keep Paying?</t>
+        </is>
+      </c>
+      <c r="AY47" s="90" t="inlineStr">
+        <is>
           <t>Dow Jones Futures: Nasdaq Hits New High; Sandisk, Micron Trigger Buy Signals</t>
         </is>
       </c>
-      <c r="AY47" s="90" t="inlineStr">
+      <c r="AZ47" s="90" t="inlineStr">
         <is>
           <t>5-star analyst sets jaw-dropping price target on SanDisk stock</t>
-        </is>
-      </c>
-      <c r="AZ47" s="90" t="inlineStr">
-        <is>
-          <t>Micron vs. SanDisk: Comparing Two Red-Hot AI Memory Stocks</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 22 Sep 2026, 10:59 PM · Yahoo Finance data</t>
+          <t>Built 22 Sep 2026, 11:35 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 22 Sep 2026, 10:59 PM · Yahoo Finance data</t>
+          <t>Built 22 Sep 2026, 11:35 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 22 Sep 2026, 10:59 PM · Yahoo Finance data</t>
+          <t>Built 22 Sep 2026, 11:35 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 22 Sep 2026, 10:59 PM · Yahoo Finance data</t>
+          <t>Built 22 Sep 2026, 11:35 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-09-23 22:58 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 23 Sep 2026, 08:35 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 23 Sep 2026, 10:58 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 23 Sep 2026, 08:35 PM · Yahoo Finance data</t>
+          <t>Built 23 Sep 2026, 10:58 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -3620,10 +3620,10 @@
         <v>169.5800018310547</v>
       </c>
       <c r="W7" s="73" t="n">
-        <v>7995282</v>
+        <v>7996530</v>
       </c>
       <c r="X7" s="74" t="n">
-        <v>1.051454058384691</v>
+        <v>1.051609552311116</v>
       </c>
       <c r="Y7" s="28" t="n">
         <v>35.7636190327093</v>
@@ -3810,10 +3810,10 @@
         <v>168.1900024414062</v>
       </c>
       <c r="W8" s="84" t="n">
-        <v>7326274</v>
+        <v>7327832</v>
       </c>
       <c r="X8" s="85" t="n">
-        <v>0.9916217860443644</v>
+        <v>0.9918222059465328</v>
       </c>
       <c r="Y8" s="35" t="n">
         <v>50.98298281616719</v>
@@ -3892,17 +3892,17 @@
       </c>
       <c r="AX8" s="90" t="inlineStr">
         <is>
+          <t>Ocular Therapeutix and ANI Pharmaceuticals Stocks Trade Down, What You Need To Know</t>
+        </is>
+      </c>
+      <c r="AY8" s="90" t="inlineStr">
+        <is>
           <t>Biotech Week Ahead: XLV Beats The Market — Here Are The Stocks, Readouts And Events To Watch Next</t>
         </is>
       </c>
-      <c r="AY8" s="90" t="inlineStr">
+      <c r="AZ8" s="90" t="inlineStr">
         <is>
           <t>Sector Update: Healthcare Stocks Softer Late Afternoon</t>
-        </is>
-      </c>
-      <c r="AZ8" s="90" t="inlineStr">
-        <is>
-          <t>Sector Update: Healthcare Stocks Higher Late Afternoon</t>
         </is>
       </c>
     </row>
@@ -4000,10 +4000,10 @@
         <v>54.46500015258789</v>
       </c>
       <c r="W9" s="73" t="n">
-        <v>42351137</v>
+        <v>42573909</v>
       </c>
       <c r="X9" s="74" t="n">
-        <v>1.255781433963288</v>
+        <v>1.261970192199754</v>
       </c>
       <c r="Y9" s="28" t="n">
         <v>28.41845219426713</v>
@@ -4190,10 +4190,10 @@
         <v>62.04999923706055</v>
       </c>
       <c r="W10" s="84" t="n">
-        <v>36474514</v>
+        <v>36479755</v>
       </c>
       <c r="X10" s="85" t="n">
-        <v>1.13690881368298</v>
+        <v>1.137062887769043</v>
       </c>
       <c r="Y10" s="35" t="n">
         <v>46.03843778048065</v>
@@ -4380,10 +4380,10 @@
         <v>82.25</v>
       </c>
       <c r="W11" s="73" t="n">
-        <v>10645507</v>
+        <v>10700163</v>
       </c>
       <c r="X11" s="74" t="n">
-        <v>1.099669145507949</v>
+        <v>1.105003112989035</v>
       </c>
       <c r="Y11" s="28" t="n">
         <v>39.12980497413955</v>
@@ -4462,17 +4462,17 @@
       </c>
       <c r="AX11" s="79" t="inlineStr">
         <is>
+          <t>Better Consumer Staples ETF: Vanguard's VDC vs. State Street's XLP</t>
+        </is>
+      </c>
+      <c r="AY11" s="79" t="inlineStr">
+        <is>
           <t>Should You Invest in the State Street Consumer Staples Select Sector SPDR ETF (XLP)?</t>
         </is>
       </c>
-      <c r="AY11" s="79" t="inlineStr">
+      <c r="AZ11" s="79" t="inlineStr">
         <is>
           <t>Sector Update: Consumer Stocks Mixed Late Afternoon</t>
-        </is>
-      </c>
-      <c r="AZ11" s="79" t="inlineStr">
-        <is>
-          <t>Sector Update: Consumer Stocks Mixed Monday Afternoon</t>
         </is>
       </c>
     </row>
@@ -4570,10 +4570,10 @@
         <v>110.3600006103516</v>
       </c>
       <c r="W12" s="84" t="n">
-        <v>6827615</v>
+        <v>6905601</v>
       </c>
       <c r="X12" s="85" t="n">
-        <v>1.16306367872932</v>
+        <v>1.175567507319484</v>
       </c>
       <c r="Y12" s="35" t="n">
         <v>38.61086937080812</v>
@@ -4760,10 +4760,10 @@
         <v>112.2750015258789</v>
       </c>
       <c r="W13" s="73" t="n">
-        <v>5613704</v>
+        <v>5613884</v>
       </c>
       <c r="X13" s="74" t="n">
-        <v>1.203112260193196</v>
+        <v>1.203148516558379</v>
       </c>
       <c r="Y13" s="28" t="n">
         <v>51.01089682481231</v>
@@ -4950,10 +4950,10 @@
         <v>50.04499816894531</v>
       </c>
       <c r="W14" s="84" t="n">
-        <v>10464790</v>
+        <v>10466595</v>
       </c>
       <c r="X14" s="85" t="n">
-        <v>0.9627611864123841</v>
+        <v>0.9629192513769821</v>
       </c>
       <c r="Y14" s="35" t="n">
         <v>39.95979749615056</v>
@@ -5140,10 +5140,10 @@
         <v>193.8249969482422</v>
       </c>
       <c r="W15" s="73" t="n">
-        <v>5811224</v>
+        <v>5821732</v>
       </c>
       <c r="X15" s="74" t="n">
-        <v>0.8780099425996118</v>
+        <v>0.879527763401156</v>
       </c>
       <c r="Y15" s="28" t="n">
         <v>65.81172395108267</v>
@@ -5330,10 +5330,10 @@
         <v>41.81010055541992</v>
       </c>
       <c r="W16" s="84" t="n">
-        <v>6710833</v>
+        <v>6710964</v>
       </c>
       <c r="X16" s="85" t="n">
-        <v>1.292910174424589</v>
+        <v>1.29293378132159</v>
       </c>
       <c r="Y16" s="35" t="n">
         <v>26.34240846268446</v>
@@ -5520,10 +5520,10 @@
         <v>39.70999908447266</v>
       </c>
       <c r="W17" s="73" t="n">
-        <v>27663389</v>
+        <v>27794894</v>
       </c>
       <c r="X17" s="74" t="n">
-        <v>1.281438634892701</v>
+        <v>1.287138241864891</v>
       </c>
       <c r="Y17" s="28" t="n">
         <v>23.73754057047114</v>
@@ -5729,10 +5729,10 @@
         <v>766.5</v>
       </c>
       <c r="W19" s="73" t="n">
-        <v>43595781</v>
+        <v>54730992</v>
       </c>
       <c r="X19" s="74" t="n">
-        <v>1.030280583151902</v>
+        <v>1.276636712486932</v>
       </c>
       <c r="Y19" s="28" t="n">
         <v>53.0448459345421</v>
@@ -5811,17 +5811,17 @@
       </c>
       <c r="AX19" s="79" t="inlineStr">
         <is>
-          <t>VGT Holders Bought ‘Tech’ and Own No Google, Meta, or Amazon: The Sector Rule That Decides What’s Inside</t>
+          <t>Vanguard Will Put $1,500 Into Your Kid’s Trump Account Starting in 2027. Here’s What to Buy With It</t>
         </is>
       </c>
       <c r="AY19" s="79" t="inlineStr">
         <is>
-          <t>SpaceX Drops 4% Amid Share Supply and Valuation Concerns; AST SpaceMobile Falls 6%</t>
+          <t>Steve Weiss Dumped an Energy Stock That Tripled the S&amp;P 500 Over a Decade</t>
         </is>
       </c>
       <c r="AZ19" s="79" t="inlineStr">
         <is>
-          <t>Domino’s Pizza Is Down 28% This Year. Is It Time to Sell or Load Up?</t>
+          <t>S&amp;P 500, Dow, Nasdaq Drop As Yields Spike Amid Calls For More Rate Hikes — AMZN, GOOGL, NFLX, SPCX, RKLB In...</t>
         </is>
       </c>
     </row>
@@ -5917,10 +5917,10 @@
         <v>738.1909790039062</v>
       </c>
       <c r="W20" s="84" t="n">
-        <v>32027122</v>
+        <v>32952535</v>
       </c>
       <c r="X20" s="85" t="n">
-        <v>0.9826769113696519</v>
+        <v>1.009637644031099</v>
       </c>
       <c r="Y20" s="35" t="n">
         <v>63.21738526937805</v>
@@ -6105,10 +6105,10 @@
         <v>281.8399963378906</v>
       </c>
       <c r="W21" s="73" t="n">
-        <v>24006903</v>
+        <v>24267666</v>
       </c>
       <c r="X21" s="74" t="n">
-        <v>1.114764917605888</v>
+        <v>1.126191666101312</v>
       </c>
       <c r="Y21" s="28" t="n">
         <v>34.40622208588071</v>
@@ -6293,10 +6293,10 @@
         <v>139.5800018310547</v>
       </c>
       <c r="W22" s="84" t="n">
-        <v>60802103</v>
+        <v>61043803</v>
       </c>
       <c r="X22" s="85" t="n">
-        <v>1.059869815551021</v>
+        <v>1.06385888924159</v>
       </c>
       <c r="Y22" s="35" t="n">
         <v>59.63106202420396</v>
@@ -6502,10 +6502,10 @@
         <v>335.6099853515625</v>
       </c>
       <c r="W24" s="73" t="n">
-        <v>31020770</v>
+        <v>31482942</v>
       </c>
       <c r="X24" s="74" t="n">
-        <v>0.7139609398259219</v>
+        <v>0.7242129170944033</v>
       </c>
       <c r="Y24" s="28" t="n">
         <v>62.9037747705856</v>
@@ -6681,7 +6681,7 @@
         <v>-9.1600341796875</v>
       </c>
       <c r="T25" s="83" t="n">
-        <v>621.5</v>
+        <v>622.1500244140625</v>
       </c>
       <c r="U25" s="83" t="n">
         <v>624.6898803710938</v>
@@ -6690,10 +6690,10 @@
         <v>608.0900268554688</v>
       </c>
       <c r="W25" s="84" t="n">
-        <v>16163572</v>
+        <v>16270327</v>
       </c>
       <c r="X25" s="85" t="n">
-        <v>0.7693087521668199</v>
+        <v>0.77419309496591</v>
       </c>
       <c r="Y25" s="35" t="n">
         <v>71.00438492046516</v>
@@ -6777,12 +6777,12 @@
       </c>
       <c r="AY25" s="90" t="inlineStr">
         <is>
+          <t>Marvell and 2 More Stocks to Play the AI Data-Center Boom</t>
+        </is>
+      </c>
+      <c r="AZ25" s="90" t="inlineStr">
+        <is>
           <t>AMD Is Up 187% This Year: Take Profits, or Buy More?</t>
-        </is>
-      </c>
-      <c r="AZ25" s="90" t="inlineStr">
-        <is>
-          <t>AMD Just Hit $1 Trillion. Can Oracle’s 50,000-GPU Deployment Help Justify It?</t>
         </is>
       </c>
     </row>
@@ -6869,7 +6869,7 @@
         <v>-5.709991455078125</v>
       </c>
       <c r="T26" s="72" t="n">
-        <v>253</v>
+        <v>253.3300018310547</v>
       </c>
       <c r="U26" s="72" t="n">
         <v>253.8099975585938</v>
@@ -6878,10 +6878,10 @@
         <v>247.7599945068359</v>
       </c>
       <c r="W26" s="73" t="n">
-        <v>43386392</v>
+        <v>43691413</v>
       </c>
       <c r="X26" s="74" t="n">
-        <v>1.246218307647267</v>
+        <v>1.254430119378623</v>
       </c>
       <c r="Y26" s="28" t="n">
         <v>44.0741573683181</v>
@@ -6960,17 +6960,17 @@
       </c>
       <c r="AX26" s="79" t="inlineStr">
         <is>
-          <t>Sector Update: Tech Stocks Fall Late Afternoon</t>
+          <t>Beloved travel brand closing after 22 years, final sale swamped</t>
         </is>
       </c>
       <c r="AY26" s="79" t="inlineStr">
         <is>
-          <t>AMZN Stock In Focus — Amazon Reportedly Taps Former Employees And Laid-Off Staff In Accelerated Push For AI...</t>
+          <t>Why UPS Slashed Its Amazon Business by 50%</t>
         </is>
       </c>
       <c r="AZ26" s="79" t="inlineStr">
         <is>
-          <t>Amazon blocks Meta's Muse but Shopify opens the door</t>
+          <t>If Amazon doesn’t know how to eliminate carbon emissions, then who does?</t>
         </is>
       </c>
     </row>
@@ -7066,10 +7066,10 @@
         <v>89.66999816894531</v>
       </c>
       <c r="W27" s="84" t="n">
-        <v>3852015</v>
+        <v>3852963</v>
       </c>
       <c r="X27" s="85" t="n">
-        <v>0.8544765261937795</v>
+        <v>0.8546778305566185</v>
       </c>
       <c r="Y27" s="35" t="n">
         <v>62.6884650695654</v>
@@ -7245,7 +7245,7 @@
         <v>-0.6400146484375</v>
       </c>
       <c r="T28" s="72" t="n">
-        <v>331.7799987792969</v>
+        <v>331.7200012207031</v>
       </c>
       <c r="U28" s="72" t="n">
         <v>336.9798889160156</v>
@@ -7254,10 +7254,10 @@
         <v>324.5599975585938</v>
       </c>
       <c r="W28" s="73" t="n">
-        <v>6930976</v>
+        <v>6946312</v>
       </c>
       <c r="X28" s="74" t="n">
-        <v>1.409471551474218</v>
+        <v>1.412370016353152</v>
       </c>
       <c r="Y28" s="28" t="n">
         <v>71.06681661915931</v>
@@ -7442,10 +7442,10 @@
         <v>59.91999816894531</v>
       </c>
       <c r="W29" s="84" t="n">
-        <v>8330034</v>
+        <v>8428910</v>
       </c>
       <c r="X29" s="85" t="n">
-        <v>0.8529940229119813</v>
+        <v>0.8626821801006705</v>
       </c>
       <c r="Y29" s="35" t="n">
         <v>46.39897420427741</v>
@@ -7630,10 +7630,10 @@
         <v>354.010009765625</v>
       </c>
       <c r="W30" s="73" t="n">
-        <v>22060703</v>
+        <v>22438949</v>
       </c>
       <c r="X30" s="74" t="n">
-        <v>0.8021551644339051</v>
+        <v>0.8153479745209047</v>
       </c>
       <c r="Y30" s="28" t="n">
         <v>44.37179877049647</v>
@@ -7818,10 +7818,10 @@
         <v>90.76999664306641</v>
       </c>
       <c r="W31" s="84" t="n">
-        <v>2428853</v>
+        <v>2434924</v>
       </c>
       <c r="X31" s="85" t="n">
-        <v>0.8249682216017095</v>
+        <v>0.8269449979847043</v>
       </c>
       <c r="Y31" s="35" t="n">
         <v>39.72589313624533</v>
@@ -7997,7 +7997,7 @@
         <v>0.1399993896484375</v>
       </c>
       <c r="T32" s="72" t="n">
-        <v>88.98500061035156</v>
+        <v>89.04499816894531</v>
       </c>
       <c r="U32" s="72" t="n">
         <v>90.36000061035156</v>
@@ -8006,10 +8006,10 @@
         <v>86.55000305175781</v>
       </c>
       <c r="W32" s="73" t="n">
-        <v>31398469</v>
+        <v>31585491</v>
       </c>
       <c r="X32" s="74" t="n">
-        <v>1.123323322192016</v>
+        <v>1.129636372843098</v>
       </c>
       <c r="Y32" s="28" t="n">
         <v>50.31530309964712</v>
@@ -8088,17 +8088,17 @@
       </c>
       <c r="AX32" s="79" t="inlineStr">
         <is>
+          <t>CoreWeave Becomes the Only Provider to Earn SemiAnalysis' Platinum ClusterMAX™ Rating Three Consecutive Times</t>
+        </is>
+      </c>
+      <c r="AY32" s="79" t="inlineStr">
+        <is>
           <t>CoreWeave Just Scored Another Big AI Win</t>
         </is>
       </c>
-      <c r="AY32" s="79" t="inlineStr">
+      <c r="AZ32" s="79" t="inlineStr">
         <is>
           <t>CoreWeave gets 'buy' rating from UBS as AI compute demand strengthens</t>
-        </is>
-      </c>
-      <c r="AZ32" s="79" t="inlineStr">
-        <is>
-          <t>CoreWeave Just Got a Big Vote of Confidence But There's a Catch</t>
         </is>
       </c>
     </row>
@@ -8194,10 +8194,10 @@
         <v>542.2302856445312</v>
       </c>
       <c r="W33" s="84" t="n">
-        <v>8206204</v>
+        <v>8218969</v>
       </c>
       <c r="X33" s="85" t="n">
-        <v>0.7524461318445039</v>
+        <v>0.7535724836430305</v>
       </c>
       <c r="Y33" s="35" t="n">
         <v>57.12654796990839</v>
@@ -8382,10 +8382,10 @@
         <v>334.2000122070312</v>
       </c>
       <c r="W34" s="73" t="n">
-        <v>22829247</v>
+        <v>23055710</v>
       </c>
       <c r="X34" s="74" t="n">
-        <v>1.285692827428</v>
+        <v>1.297619238910516</v>
       </c>
       <c r="Y34" s="28" t="n">
         <v>44.93718158640226</v>
@@ -8464,17 +8464,17 @@
       </c>
       <c r="AX34" s="79" t="inlineStr">
         <is>
-          <t>Google Is Helping Upgrade Southern’s Nuclear Plants. Can 96 MW Ease Its AI Power Bottleneck?</t>
+          <t>Alphabet Inc. (GOOG) Dips More Than Broader Market: What You Should Know</t>
         </is>
       </c>
       <c r="AY34" s="79" t="inlineStr">
         <is>
-          <t>GOOGL, NFLX Stocks In Focus — Alphabet's YouTube Reportedly Rolls Out Fresh Tools To Prevent Creators From ...</t>
+          <t>Why Alphabet (GOOGL) Stock Is Down Today</t>
         </is>
       </c>
       <c r="AZ34" s="79" t="inlineStr">
         <is>
-          <t>Nvidia Stock Falls. It Has a Google AI Chip Conundrum.</t>
+          <t>Alphabet vs. Amazon: Which Anthropic Backer Will Benefit More From the $2 Trillion IPO?</t>
         </is>
       </c>
     </row>
@@ -8570,10 +8570,10 @@
         <v>47.0099983215332</v>
       </c>
       <c r="W35" s="84" t="n">
-        <v>31986735</v>
+        <v>32093751</v>
       </c>
       <c r="X35" s="85" t="n">
-        <v>0.7830486231212633</v>
+        <v>0.7855655183828868</v>
       </c>
       <c r="Y35" s="35" t="n">
         <v>58.36047210248843</v>
@@ -8758,10 +8758,10 @@
         <v>119.4400024414062</v>
       </c>
       <c r="W36" s="73" t="n">
-        <v>84199525</v>
+        <v>84944757</v>
       </c>
       <c r="X36" s="74" t="n">
-        <v>0.8126857682439965</v>
+        <v>0.8195839166979799</v>
       </c>
       <c r="Y36" s="28" t="n">
         <v>70.25971337460517</v>
@@ -8840,17 +8840,17 @@
       </c>
       <c r="AX36" s="79" t="inlineStr">
         <is>
+          <t>VYM’s Index Buys on Forecast Yield, So It Held Intel and Walgreens Right Into Their Dividend Cuts</t>
+        </is>
+      </c>
+      <c r="AY36" s="79" t="inlineStr">
+        <is>
+          <t>Prediction: Intel Names a Major Outside Customer for Its Next Factory Process Before 2027</t>
+        </is>
+      </c>
+      <c r="AZ36" s="79" t="inlineStr">
+        <is>
           <t>Intel Falls 2.24% as Muse Keeps the CPU Thesis Alive</t>
-        </is>
-      </c>
-      <c r="AY36" s="79" t="inlineStr">
-        <is>
-          <t>Not Intel. Not Nvidia. This Chip Giant Holds an Unbreakable Moat in Next-Gen Data Centers.</t>
-        </is>
-      </c>
-      <c r="AZ36" s="79" t="inlineStr">
-        <is>
-          <t>Intel’s Price Targets Reveal Just How Much Is Riding on Its Turnaround</t>
         </is>
       </c>
     </row>
@@ -8946,10 +8946,10 @@
         <v>495.8999938964844</v>
       </c>
       <c r="W37" s="84" t="n">
-        <v>19061882</v>
+        <v>19296597</v>
       </c>
       <c r="X37" s="85" t="n">
-        <v>0.8855877762410882</v>
+        <v>0.8960037747634604</v>
       </c>
       <c r="Y37" s="35" t="n">
         <v>56.19452966281882</v>
@@ -9028,17 +9028,17 @@
       </c>
       <c r="AX37" s="90" t="inlineStr">
         <is>
+          <t>Microsoft President Brad Smith: AI Systems Need an ‘Emergency Brake’</t>
+        </is>
+      </c>
+      <c r="AY37" s="90" t="inlineStr">
+        <is>
+          <t>Microsoft President Brad Smith: AI’s Power Is Advancing Faster Than Its Safety</t>
+        </is>
+      </c>
+      <c r="AZ37" s="90" t="inlineStr">
+        <is>
           <t>Microsoft Stock Gets Another Upgrade, Price-Target Hike</t>
-        </is>
-      </c>
-      <c r="AY37" s="90" t="inlineStr">
-        <is>
-          <t>Sector Update: Tech Stocks Fall Late Afternoon</t>
-        </is>
-      </c>
-      <c r="AZ37" s="90" t="inlineStr">
-        <is>
-          <t>Update: Market Chatter: Microsoft Agrees to Keep Shareholder Proposal Rights Through 2027</t>
         </is>
       </c>
     </row>
@@ -9134,10 +9134,10 @@
         <v>161.8370056152344</v>
       </c>
       <c r="W38" s="73" t="n">
-        <v>20798984</v>
+        <v>20981397</v>
       </c>
       <c r="X38" s="74" t="n">
-        <v>0.7974561684602933</v>
+        <v>0.8041688711407238</v>
       </c>
       <c r="Y38" s="28" t="n">
         <v>66.24656919420906</v>
@@ -9216,17 +9216,17 @@
       </c>
       <c r="AX38" s="79" t="inlineStr">
         <is>
+          <t>Strategy (MSTR) Registers a Bigger Fall Than the Market: Important Facts to Note</t>
+        </is>
+      </c>
+      <c r="AY38" s="79" t="inlineStr">
+        <is>
           <t>Gary Cardone made $750K without chasing Bitcoin, here's what he bought</t>
         </is>
       </c>
-      <c r="AY38" s="79" t="inlineStr">
+      <c r="AZ38" s="79" t="inlineStr">
         <is>
           <t>Strategy (MSTR) Is Up 29.1% After Resuming Bitcoin Buys and Preferred Stock Buybacks – What's Changed</t>
-        </is>
-      </c>
-      <c r="AZ38" s="79" t="inlineStr">
-        <is>
-          <t>Trump's stock accounts quietly loaded up on Strategy and Tesla, filing shows</t>
         </is>
       </c>
     </row>
@@ -9322,10 +9322,10 @@
         <v>1064.25</v>
       </c>
       <c r="W39" s="84" t="n">
-        <v>21310328</v>
+        <v>21405071</v>
       </c>
       <c r="X39" s="85" t="n">
-        <v>0.8449863189264578</v>
+        <v>0.8485836265517673</v>
       </c>
       <c r="Y39" s="35" t="n">
         <v>62.18920104505369</v>
@@ -9404,17 +9404,17 @@
       </c>
       <c r="AX39" s="90" t="inlineStr">
         <is>
+          <t>Top Research Reports for Micron, Costco &amp; Interactive Brokers</t>
+        </is>
+      </c>
+      <c r="AY39" s="90" t="inlineStr">
+        <is>
+          <t>Own ON Semiconductor For AI Power, Or Own Micron's Contracts?</t>
+        </is>
+      </c>
+      <c r="AZ39" s="90" t="inlineStr">
+        <is>
           <t>Chip Stocks Drop After Six-Day Climb For SOX Index</t>
-        </is>
-      </c>
-      <c r="AY39" s="90" t="inlineStr">
-        <is>
-          <t>Micron (MU) vs Western Digital (WDC): Which is a Better Stock to Buy</t>
-        </is>
-      </c>
-      <c r="AZ39" s="90" t="inlineStr">
-        <is>
-          <t>Citi Resets Micron Target After Surprise</t>
         </is>
       </c>
     </row>
@@ -9510,10 +9510,10 @@
         <v>226.3899993896484</v>
       </c>
       <c r="W40" s="73" t="n">
-        <v>10843967</v>
+        <v>10887468</v>
       </c>
       <c r="X40" s="74" t="n">
-        <v>0.737512575591741</v>
+        <v>0.7403616160484731</v>
       </c>
       <c r="Y40" s="28" t="n">
         <v>52.27681782849186</v>
@@ -9689,7 +9689,7 @@
         <v>-0.8000030517578125</v>
       </c>
       <c r="T41" s="83" t="n">
-        <v>72.07499694824219</v>
+        <v>72.05999755859375</v>
       </c>
       <c r="U41" s="83" t="n">
         <v>72.36949920654297</v>
@@ -9698,10 +9698,10 @@
         <v>71.06999969482422</v>
       </c>
       <c r="W41" s="84" t="n">
-        <v>32373153</v>
+        <v>32606518</v>
       </c>
       <c r="X41" s="85" t="n">
-        <v>1.000905437479429</v>
+        <v>1.007757006429308</v>
       </c>
       <c r="Y41" s="35" t="n">
         <v>37.08249449749585</v>
@@ -9790,7 +9790,7 @@
       </c>
       <c r="AZ41" s="90" t="inlineStr">
         <is>
-          <t>GOOGL, NFLX Stocks In Focus — Alphabet's YouTube Reportedly Rolls Out Fresh Tools To Prevent Creators From ...</t>
+          <t>Is Netflix (NFLX) Worth More Than Its Cash Flow Suggests?</t>
         </is>
       </c>
     </row>
@@ -9886,10 +9886,10 @@
         <v>10.57499980926514</v>
       </c>
       <c r="W42" s="73" t="n">
-        <v>63322484</v>
+        <v>63469410</v>
       </c>
       <c r="X42" s="74" t="n">
-        <v>0.7405146432417938</v>
+        <v>0.7421690859660737</v>
       </c>
       <c r="Y42" s="28" t="n">
         <v>52.76075715448685</v>
@@ -10074,10 +10074,10 @@
         <v>224.0200042724609</v>
       </c>
       <c r="W43" s="84" t="n">
-        <v>85801410</v>
+        <v>86851377</v>
       </c>
       <c r="X43" s="85" t="n">
-        <v>0.6527312831134676</v>
+        <v>0.6604550988874065</v>
       </c>
       <c r="Y43" s="35" t="n">
         <v>55.71799631755795</v>
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
-          <t>How the Trump-Xi Meeting Could Move Nvidia, Boeing and Your 401(k)</t>
+          <t>Stock Market Today, Sept. 23: IonQ Surges on Quantum Breakthrough and Nvidia Partnership</t>
         </is>
       </c>
       <c r="AY43" s="90" t="inlineStr">
         <is>
-          <t>Forget Waiting for a Dip: Nvidia (NVDA) Is Worth Buying Today Based on The Motley Fool's Long-Term Convicti...</t>
+          <t>IonQ Wants to Be the Nvidia of Quantum. Now They Are Partners.</t>
         </is>
       </c>
       <c r="AZ43" s="90" t="inlineStr">
         <is>
-          <t>Grid Dynamics Co-Hosts Physical AI Summit Alongside NVIDIA, EAIGG, and BGV to Accelerate Manufacturing Auto...</t>
+          <t>Here's How Much You'd Need to Invest in SCHD to Generate $500 Per Month in Dividends</t>
         </is>
       </c>
     </row>
@@ -10262,10 +10262,10 @@
         <v>182.9499969482422</v>
       </c>
       <c r="W44" s="73" t="n">
-        <v>34597606</v>
+        <v>34908712</v>
       </c>
       <c r="X44" s="74" t="n">
-        <v>1.24697670572474</v>
+        <v>1.257484669287845</v>
       </c>
       <c r="Y44" s="28" t="n">
         <v>66.88183818591999</v>
@@ -10344,17 +10344,17 @@
       </c>
       <c r="AX44" s="79" t="inlineStr">
         <is>
-          <t>Palantir Stock Rises 3% Despite Losing $875 Million FAA AI Deal: Here’s Why</t>
+          <t>Dow Jones Futures: Stocks Fall As Treasury Yields Soar; Palantir, Palo Alto Flash Buy Signals</t>
         </is>
       </c>
       <c r="AY44" s="79" t="inlineStr">
         <is>
-          <t>Palantir Could Be Big Winner as Air Traffic Control Goes AI. The Stock Is Rising.</t>
+          <t>Palantir's CEO just sent a message Silicon Valley won't ignore</t>
         </is>
       </c>
       <c r="AZ44" s="79" t="inlineStr">
         <is>
-          <t>Palantir Jumps Over 4% as Karp Makes AI Liability the Product Test</t>
+          <t>Palantir, IBD Stock Of The Day, Flashes Buy Signal Amid Earnings, AI Momentum</t>
         </is>
       </c>
     </row>
@@ -10450,10 +10450,10 @@
         <v>193.2299957275391</v>
       </c>
       <c r="W45" s="84" t="n">
-        <v>9606665</v>
+        <v>9685834</v>
       </c>
       <c r="X45" s="85" t="n">
-        <v>0.6629937107777658</v>
+        <v>0.6682749098273952</v>
       </c>
       <c r="Y45" s="35" t="n">
         <v>66.44760389438214</v>
@@ -10532,17 +10532,17 @@
       </c>
       <c r="AX45" s="90" t="inlineStr">
         <is>
+          <t>How Qualcomm is transforming the car into a 'digital computer on wheels': CEO explains</t>
+        </is>
+      </c>
+      <c r="AY45" s="90" t="inlineStr">
+        <is>
           <t>How Qualcomm is targeting agentic AI with its 2 new smartphone chips</t>
         </is>
       </c>
-      <c r="AY45" s="90" t="inlineStr">
+      <c r="AZ45" s="90" t="inlineStr">
         <is>
           <t>Qualcomm Takes AI To The Edge With New Mobile Chips</t>
-        </is>
-      </c>
-      <c r="AZ45" s="90" t="inlineStr">
-        <is>
-          <t>QUALCOMM (QCOM) Draws Fresh AI Focus As Valuation Looks Close To Fair Value</t>
         </is>
       </c>
     </row>
@@ -10629,7 +10629,7 @@
         <v>-1.670005798339844</v>
       </c>
       <c r="T46" s="72" t="n">
-        <v>72.87000274658203</v>
+        <v>72.80000305175781</v>
       </c>
       <c r="U46" s="72" t="n">
         <v>73.56999969482422</v>
@@ -10638,10 +10638,10 @@
         <v>70.08000183105469</v>
       </c>
       <c r="W46" s="73" t="n">
-        <v>19014723</v>
+        <v>19110310</v>
       </c>
       <c r="X46" s="74" t="n">
-        <v>0.999040972370472</v>
+        <v>1.003811084767845</v>
       </c>
       <c r="Y46" s="28" t="n">
         <v>53.93604009674983</v>
@@ -10720,17 +10720,17 @@
       </c>
       <c r="AX46" s="79" t="inlineStr">
         <is>
+          <t>Rocket Lab Readies For Mission, Cathie Wood Buys $25 Million In Shares</t>
+        </is>
+      </c>
+      <c r="AY46" s="79" t="inlineStr">
+        <is>
+          <t>Rocket Lab (RKLB) Neutron Could Fill A Medium Lift Launch Gap</t>
+        </is>
+      </c>
+      <c r="AZ46" s="79" t="inlineStr">
+        <is>
           <t>Peter Beck’s Iridium Deal Faces Its Next Big Test</t>
-        </is>
-      </c>
-      <c r="AY46" s="79" t="inlineStr">
-        <is>
-          <t>SPCX, RKLB, LUNR, ASTS In Focus — Space Economy Investment Surges To $23B In Year Ending June, A Near 140% ...</t>
-        </is>
-      </c>
-      <c r="AZ46" s="79" t="inlineStr">
-        <is>
-          <t>What Could Surprise RKLB Stock Investors On The Upside?</t>
         </is>
       </c>
     </row>
@@ -10817,7 +10817,7 @@
         <v>-70.4700927734375</v>
       </c>
       <c r="T47" s="83" t="n">
-        <v>1895.410034179688</v>
+        <v>1895</v>
       </c>
       <c r="U47" s="83" t="n">
         <v>1902.219970703125</v>
@@ -10826,10 +10826,10 @@
         <v>1803.670043945312</v>
       </c>
       <c r="W47" s="84" t="n">
-        <v>7646795</v>
+        <v>7672720</v>
       </c>
       <c r="X47" s="85" t="n">
-        <v>0.7103161792919727</v>
+        <v>0.7126385623141713</v>
       </c>
       <c r="Y47" s="35" t="n">
         <v>60.05657264950232</v>
@@ -11005,7 +11005,7 @@
         <v>1.220001220703125</v>
       </c>
       <c r="T48" s="72" t="n">
-        <v>380.1000061035156</v>
+        <v>379.9349975585938</v>
       </c>
       <c r="U48" s="72" t="n">
         <v>386.7000122070312</v>
@@ -11014,10 +11014,10 @@
         <v>377.5750122070312</v>
       </c>
       <c r="W48" s="73" t="n">
-        <v>32715439</v>
+        <v>32914670</v>
       </c>
       <c r="X48" s="74" t="n">
-        <v>0.8399281689923684</v>
+        <v>0.8448271120276751</v>
       </c>
       <c r="Y48" s="28" t="n">
         <v>60.59414491377634</v>
@@ -11096,17 +11096,17 @@
       </c>
       <c r="AX48" s="79" t="inlineStr">
         <is>
+          <t>Tesla wins lead role in 2,500-truck electric Class 8 order</t>
+        </is>
+      </c>
+      <c r="AY48" s="79" t="inlineStr">
+        <is>
           <t>3 Things You Need to Know Before Buying Tesla</t>
         </is>
       </c>
-      <c r="AY48" s="79" t="inlineStr">
+      <c r="AZ48" s="79" t="inlineStr">
         <is>
           <t>Tesla Rises as BBB Rating Meets a $25 Billion Buildout</t>
-        </is>
-      </c>
-      <c r="AZ48" s="79" t="inlineStr">
-        <is>
-          <t>Tesla Is Supplying the Trucks. Nvidia Is Supplying the Compute. This $4 Stock Sits in the Middle</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 23 Sep 2026, 08:35 PM · Yahoo Finance data</t>
+          <t>Built 23 Sep 2026, 10:58 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 23 Sep 2026, 08:35 PM · Yahoo Finance data</t>
+          <t>Built 23 Sep 2026, 10:58 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 23 Sep 2026, 08:35 PM · Yahoo Finance data</t>
+          <t>Built 23 Sep 2026, 10:58 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 23 Sep 2026, 08:35 PM · Yahoo Finance data</t>
+          <t>Built 23 Sep 2026, 10:58 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-09-23 23:39 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 23 Sep 2026, 10:58 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 23 Sep 2026, 11:39 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 23 Sep 2026, 10:58 PM · Yahoo Finance data</t>
+          <t>Built 23 Sep 2026, 11:39 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -6772,17 +6772,17 @@
       </c>
       <c r="AX25" s="90" t="inlineStr">
         <is>
-          <t>Nasdaq rally hasn't stopped these tech stocks from flashing warning signs</t>
+          <t>Marvell and 2 More Stocks to Play the AI Data-Center Boom</t>
         </is>
       </c>
       <c r="AY25" s="90" t="inlineStr">
         <is>
-          <t>Marvell and 2 More Stocks to Play the AI Data-Center Boom</t>
+          <t>AMD Is Up 187% This Year: Take Profits, or Buy More?</t>
         </is>
       </c>
       <c r="AZ25" s="90" t="inlineStr">
         <is>
-          <t>AMD Is Up 187% This Year: Take Profits, or Buy More?</t>
+          <t>AMD Just Hit $1 Trillion. Can Oracle’s 50,000-GPU Deployment Help Justify It?</t>
         </is>
       </c>
     </row>
@@ -7712,17 +7712,17 @@
       </c>
       <c r="AX30" s="79" t="inlineStr">
         <is>
+          <t>3 Companies With a Strong History of Dividend Growth</t>
+        </is>
+      </c>
+      <c r="AY30" s="79" t="inlineStr">
+        <is>
           <t>Broadcom Just Made a Move That Further Solidifies My Decision to Buy on Repeat</t>
         </is>
       </c>
-      <c r="AY30" s="79" t="inlineStr">
+      <c r="AZ30" s="79" t="inlineStr">
         <is>
           <t>Two Chip Giants, Two Very Different Dividends. Which One Pays You Better?</t>
-        </is>
-      </c>
-      <c r="AZ30" s="79" t="inlineStr">
-        <is>
-          <t>AVGO Stock Falls Premarket: China Reportedly Audits Broadcom’s Grip On State-Backed Data Centers</t>
         </is>
       </c>
     </row>
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
+          <t>Why IonQ (IONQ) Is Up 15.5% After NVIDIA Deal And Real-Time Error Correction Breakthrough</t>
+        </is>
+      </c>
+      <c r="AY43" s="90" t="inlineStr">
+        <is>
           <t>Stock Market Today, Sept. 23: IonQ Surges on Quantum Breakthrough and Nvidia Partnership</t>
         </is>
       </c>
-      <c r="AY43" s="90" t="inlineStr">
+      <c r="AZ43" s="90" t="inlineStr">
         <is>
           <t>IonQ Wants to Be the Nvidia of Quantum. Now They Are Partners.</t>
-        </is>
-      </c>
-      <c r="AZ43" s="90" t="inlineStr">
-        <is>
-          <t>Here's How Much You'd Need to Invest in SCHD to Generate $500 Per Month in Dividends</t>
         </is>
       </c>
     </row>
@@ -11096,17 +11096,17 @@
       </c>
       <c r="AX48" s="79" t="inlineStr">
         <is>
+          <t>Is Tesla (TSLA) Quietly Shifting From Automaker To Physical AI Platform With FSD Subscriptions?</t>
+        </is>
+      </c>
+      <c r="AY48" s="79" t="inlineStr">
+        <is>
           <t>Tesla wins lead role in 2,500-truck electric Class 8 order</t>
         </is>
       </c>
-      <c r="AY48" s="79" t="inlineStr">
+      <c r="AZ48" s="79" t="inlineStr">
         <is>
           <t>3 Things You Need to Know Before Buying Tesla</t>
-        </is>
-      </c>
-      <c r="AZ48" s="79" t="inlineStr">
-        <is>
-          <t>Tesla Rises as BBB Rating Meets a $25 Billion Buildout</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 23 Sep 2026, 10:58 PM · Yahoo Finance data</t>
+          <t>Built 23 Sep 2026, 11:39 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 23 Sep 2026, 10:58 PM · Yahoo Finance data</t>
+          <t>Built 23 Sep 2026, 11:39 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 23 Sep 2026, 10:58 PM · Yahoo Finance data</t>
+          <t>Built 23 Sep 2026, 11:39 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 23 Sep 2026, 10:58 PM · Yahoo Finance data</t>
+          <t>Built 23 Sep 2026, 11:39 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-09-24 23:14 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -28,7 +28,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'09-21'!$5:$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'09-18'!$A$6:$AZ$48</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'09-18'!$5:$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Signals'!$B$5:$G$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Signals'!$B$5:$G$45</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 24 Sep 2026, 08:38 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 24 Sep 2026, 11:14 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -1404,7 +1404,7 @@
       <c r="P8" s="10" t="n"/>
       <c r="Q8" s="16" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>40</t>
         </is>
       </c>
       <c r="R8" s="12" t="n"/>
@@ -1592,7 +1592,7 @@
         <v>0.003687663078005166</v>
       </c>
       <c r="F16" s="27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G16" s="28" t="n">
         <v>47.31565963045056</v>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 24 Sep 2026, 08:38 PM · Yahoo Finance data</t>
+          <t>Built 24 Sep 2026, 11:14 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -3620,10 +3620,10 @@
         <v>168.2449951171875</v>
       </c>
       <c r="W7" s="73" t="n">
-        <v>8519488</v>
+        <v>8522853</v>
       </c>
       <c r="X7" s="74" t="n">
-        <v>1.106090962441878</v>
+        <v>1.106503672216411</v>
       </c>
       <c r="Y7" s="28" t="n">
         <v>32.86420470607366</v>
@@ -3810,10 +3810,10 @@
         <v>168.7299957275391</v>
       </c>
       <c r="W8" s="84" t="n">
-        <v>8736640</v>
+        <v>8783505</v>
       </c>
       <c r="X8" s="85" t="n">
-        <v>1.155877655820038</v>
+        <v>1.161717850855603</v>
       </c>
       <c r="Y8" s="35" t="n">
         <v>54.43098224798918</v>
@@ -4000,10 +4000,10 @@
         <v>54.25</v>
       </c>
       <c r="W9" s="73" t="n">
-        <v>28611370</v>
+        <v>28667342</v>
       </c>
       <c r="X9" s="74" t="n">
-        <v>0.8373142510134171</v>
+        <v>0.8388835708662532</v>
       </c>
       <c r="Y9" s="28" t="n">
         <v>28.36082219832512</v>
@@ -4118,7 +4118,7 @@
       </c>
       <c r="F10" s="30" t="inlineStr">
         <is>
-          <t>Same</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G10" s="30" t="inlineStr">
@@ -4157,11 +4157,11 @@
         </is>
       </c>
       <c r="N10" s="80" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O10" s="30" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="P10" s="32" t="inlineStr">
@@ -4190,10 +4190,10 @@
         <v>62.45500183105469</v>
       </c>
       <c r="W10" s="84" t="n">
-        <v>35683279</v>
+        <v>37713159</v>
       </c>
       <c r="X10" s="85" t="n">
-        <v>1.092886177777691</v>
+        <v>1.151476768377846</v>
       </c>
       <c r="Y10" s="35" t="n">
         <v>47.31565963045056</v>
@@ -4380,10 +4380,10 @@
         <v>81.69999694824219</v>
       </c>
       <c r="W11" s="73" t="n">
-        <v>10583167</v>
+        <v>10608620</v>
       </c>
       <c r="X11" s="74" t="n">
-        <v>1.072762699517549</v>
+        <v>1.075204039157924</v>
       </c>
       <c r="Y11" s="28" t="n">
         <v>35.78515562955096</v>
@@ -4570,10 +4570,10 @@
         <v>109.625</v>
       </c>
       <c r="W12" s="84" t="n">
-        <v>4949539</v>
+        <v>4949775</v>
       </c>
       <c r="X12" s="85" t="n">
-        <v>0.8365304519234171</v>
+        <v>0.8365686703044973</v>
       </c>
       <c r="Y12" s="35" t="n">
         <v>37.71931638384608</v>
@@ -4760,10 +4760,10 @@
         <v>112.5149993896484</v>
       </c>
       <c r="W13" s="73" t="n">
-        <v>5461680</v>
+        <v>5482442</v>
       </c>
       <c r="X13" s="74" t="n">
-        <v>1.136713523292025</v>
+        <v>1.140788146980679</v>
       </c>
       <c r="Y13" s="28" t="n">
         <v>54.65132051167176</v>
@@ -4950,10 +4950,10 @@
         <v>49.56999969482422</v>
       </c>
       <c r="W14" s="84" t="n">
-        <v>12777970</v>
+        <v>12806366</v>
       </c>
       <c r="X14" s="85" t="n">
-        <v>1.151227741140006</v>
+        <v>1.153638501662976</v>
       </c>
       <c r="Y14" s="35" t="n">
         <v>36.11416737497208</v>
@@ -5140,10 +5140,10 @@
         <v>192.6199951171875</v>
       </c>
       <c r="W15" s="73" t="n">
-        <v>6248431</v>
+        <v>6324299</v>
       </c>
       <c r="X15" s="74" t="n">
-        <v>0.9375051364738455</v>
+        <v>0.948348498206924</v>
       </c>
       <c r="Y15" s="28" t="n">
         <v>64.32809115927992</v>
@@ -5330,10 +5330,10 @@
         <v>41.625</v>
       </c>
       <c r="W16" s="84" t="n">
-        <v>5651437</v>
+        <v>5673101</v>
       </c>
       <c r="X16" s="85" t="n">
-        <v>1.06235173798894</v>
+        <v>1.066207016146866</v>
       </c>
       <c r="Y16" s="35" t="n">
         <v>25.09876229664819</v>
@@ -5520,10 +5520,10 @@
         <v>39.36000061035156</v>
       </c>
       <c r="W17" s="73" t="n">
-        <v>25403549</v>
+        <v>25543115</v>
       </c>
       <c r="X17" s="74" t="n">
-        <v>1.14446008604205</v>
+        <v>1.150386041096763</v>
       </c>
       <c r="Y17" s="28" t="n">
         <v>22.03958519090727</v>
@@ -5729,10 +5729,10 @@
         <v>763.2449951171875</v>
       </c>
       <c r="W19" s="73" t="n">
-        <v>41127903</v>
+        <v>42694185</v>
       </c>
       <c r="X19" s="74" t="n">
-        <v>0.9454671837579151</v>
+        <v>0.9797098042787793</v>
       </c>
       <c r="Y19" s="28" t="n">
         <v>52.4674308976979</v>
@@ -5811,17 +5811,17 @@
       </c>
       <c r="AX19" s="79" t="inlineStr">
         <is>
+          <t>SPY’s 9.45 Basis Points Hides $6,450 a Decade on $100,000 Versus Cheaper Peers</t>
+        </is>
+      </c>
+      <c r="AY19" s="79" t="inlineStr">
+        <is>
           <t>Solar Stocks Slide as High Borrowing Costs Weigh on Project Financing: First Solar Sinks 8%, SolarEdge Fall...</t>
         </is>
       </c>
-      <c r="AY19" s="79" t="inlineStr">
+      <c r="AZ19" s="79" t="inlineStr">
         <is>
           <t>Wells Fargo Says the AI Spending Math Breaks in 2028 and Just Cut Its S&amp;P 500 Target to 7,700</t>
-        </is>
-      </c>
-      <c r="AZ19" s="79" t="inlineStr">
-        <is>
-          <t>Coherent Has Ripped 59% in 2026: Is It Too Late to Buy COHR Stock Now?</t>
         </is>
       </c>
     </row>
@@ -5908,7 +5908,7 @@
         <v>-0.11004638671875</v>
       </c>
       <c r="T20" s="83" t="n">
-        <v>735.2890014648438</v>
+        <v>735.1599731445312</v>
       </c>
       <c r="U20" s="83" t="n">
         <v>742.6500244140625</v>
@@ -5917,10 +5917,10 @@
         <v>734.630126953125</v>
       </c>
       <c r="W20" s="84" t="n">
-        <v>27956147</v>
+        <v>28622284</v>
       </c>
       <c r="X20" s="85" t="n">
-        <v>0.846434388228434</v>
+        <v>0.8657301282879422</v>
       </c>
       <c r="Y20" s="35" t="n">
         <v>63.13379362429247</v>
@@ -6105,10 +6105,10 @@
         <v>279.0450134277344</v>
       </c>
       <c r="W21" s="73" t="n">
-        <v>26906508</v>
+        <v>27088934</v>
       </c>
       <c r="X21" s="74" t="n">
-        <v>1.202785653696073</v>
+        <v>1.210446982308641</v>
       </c>
       <c r="Y21" s="28" t="n">
         <v>34.09153058946279</v>
@@ -6293,10 +6293,10 @@
         <v>136.8999938964844</v>
       </c>
       <c r="W22" s="84" t="n">
-        <v>64169008</v>
+        <v>64553899</v>
       </c>
       <c r="X22" s="85" t="n">
-        <v>1.094240467577254</v>
+        <v>1.100442682886356</v>
       </c>
       <c r="Y22" s="35" t="n">
         <v>59.66117315470079</v>
@@ -6493,7 +6493,7 @@
         <v>-1.0999755859375</v>
       </c>
       <c r="T24" s="72" t="n">
-        <v>336.7200012207031</v>
+        <v>336.3200073242188</v>
       </c>
       <c r="U24" s="72" t="n">
         <v>338.9100036621094</v>
@@ -6502,10 +6502,10 @@
         <v>334.2999877929688</v>
       </c>
       <c r="W24" s="73" t="n">
-        <v>24228667</v>
+        <v>24364559</v>
       </c>
       <c r="X24" s="74" t="n">
-        <v>0.5635760723543183</v>
+        <v>0.5666474601136546</v>
       </c>
       <c r="Y24" s="28" t="n">
         <v>61.32249689905161</v>
@@ -6589,12 +6589,12 @@
       </c>
       <c r="AY24" s="79" t="inlineStr">
         <is>
-          <t>Welcome to the age of listening devices</t>
+          <t>Meta's new AI device changes everything</t>
         </is>
       </c>
       <c r="AZ24" s="79" t="inlineStr">
         <is>
-          <t>Apple stock is giving new CEO John Ternus plenty to smile about</t>
+          <t>Could John Ternus’ Product Strategy Reshape Apple’s (AAPL) Next Growth Phase?</t>
         </is>
       </c>
     </row>
@@ -6681,7 +6681,7 @@
         <v>14.6500244140625</v>
       </c>
       <c r="T25" s="83" t="n">
-        <v>600.27001953125</v>
+        <v>600.7550048828125</v>
       </c>
       <c r="U25" s="83" t="n">
         <v>630.7899780273438</v>
@@ -6690,10 +6690,10 @@
         <v>599.3499755859375</v>
       </c>
       <c r="W25" s="84" t="n">
-        <v>25072938</v>
+        <v>25202032</v>
       </c>
       <c r="X25" s="85" t="n">
-        <v>1.163181240874684</v>
+        <v>1.168820158570506</v>
       </c>
       <c r="Y25" s="35" t="n">
         <v>72.82495971578706</v>
@@ -6869,7 +6869,7 @@
         <v>0.1100006103515625</v>
       </c>
       <c r="T26" s="72" t="n">
-        <v>246.0200042724609</v>
+        <v>245.9700012207031</v>
       </c>
       <c r="U26" s="72" t="n">
         <v>250.4299926757812</v>
@@ -6878,10 +6878,10 @@
         <v>245.6049957275391</v>
       </c>
       <c r="W26" s="73" t="n">
-        <v>32625365</v>
+        <v>32701576</v>
       </c>
       <c r="X26" s="74" t="n">
-        <v>0.9213490661469196</v>
+        <v>0.9234019170842662</v>
       </c>
       <c r="Y26" s="28" t="n">
         <v>44.1951819131943</v>
@@ -6960,17 +6960,17 @@
       </c>
       <c r="AX26" s="79" t="inlineStr">
         <is>
-          <t>Amazon Stock Dips After $100 Million Indiana Manufacturing Push</t>
+          <t>Beloved travel brand closing after 22 years, final sale swamped</t>
         </is>
       </c>
       <c r="AY26" s="79" t="inlineStr">
         <is>
-          <t>Amazon Opens Seller Data to Claude Days After Blocking Meta’s Muse</t>
+          <t>Blue Origin raises $10B as Bezos’ total investment hits $32B - WSJ</t>
         </is>
       </c>
       <c r="AZ26" s="79" t="inlineStr">
         <is>
-          <t>Amazon Faces Another Worker Lawsuit. Is Employment Scrutiny Becoming an Investor Risk?</t>
+          <t>Shopify Opens Its Doors to Muse, Here’s Why Amazon Won’t</t>
         </is>
       </c>
     </row>
@@ -7066,10 +7066,10 @@
         <v>88.77999877929688</v>
       </c>
       <c r="W27" s="84" t="n">
-        <v>5466694</v>
+        <v>5473192</v>
       </c>
       <c r="X27" s="85" t="n">
-        <v>1.209981045372801</v>
+        <v>1.211332182729855</v>
       </c>
       <c r="Y27" s="35" t="n">
         <v>65.91902600686896</v>
@@ -7254,10 +7254,10 @@
         <v>303.6499938964844</v>
       </c>
       <c r="W28" s="73" t="n">
-        <v>9433302</v>
+        <v>9485249</v>
       </c>
       <c r="X28" s="74" t="n">
-        <v>1.818625580655178</v>
+        <v>1.827725118398938</v>
       </c>
       <c r="Y28" s="28" t="n">
         <v>60.21837912066924</v>
@@ -7433,7 +7433,7 @@
         <v>1.080001831054688</v>
       </c>
       <c r="T29" s="83" t="n">
-        <v>59.20999908447266</v>
+        <v>59.04999923706055</v>
       </c>
       <c r="U29" s="83" t="n">
         <v>63.20000076293945</v>
@@ -7442,10 +7442,10 @@
         <v>58.31999969482422</v>
       </c>
       <c r="W29" s="84" t="n">
-        <v>8660388</v>
+        <v>8732321</v>
       </c>
       <c r="X29" s="85" t="n">
-        <v>0.8801100523231455</v>
+        <v>0.8870959864796181</v>
       </c>
       <c r="Y29" s="35" t="n">
         <v>48.1107848022371</v>
@@ -7524,17 +7524,17 @@
       </c>
       <c r="AX29" s="90" t="inlineStr">
         <is>
+          <t>AST SpaceMobile, Inc. (ASTS) Increases Despite Market Slip: Here's What You Need to Know</t>
+        </is>
+      </c>
+      <c r="AY29" s="90" t="inlineStr">
+        <is>
           <t>AST SpaceMobile vs. Intuitive Machines: Which Space Infrastructure Stock Is a Better Buy in 2026?</t>
         </is>
       </c>
-      <c r="AY29" s="90" t="inlineStr">
+      <c r="AZ29" s="90" t="inlineStr">
         <is>
           <t>Space Stocks Rally as Buying Spreads Across the Pure Plays: Rocket Lab and Planet Labs Jump 6%, AST SpaceMo...</t>
-        </is>
-      </c>
-      <c r="AZ29" s="90" t="inlineStr">
-        <is>
-          <t>Is AST SpaceMobile (ASTS) A Bargain As Lawsuit And Financing Questions Test Its Valuation?</t>
         </is>
       </c>
     </row>
@@ -7630,10 +7630,10 @@
         <v>346.8900146484375</v>
       </c>
       <c r="W30" s="73" t="n">
-        <v>20822871</v>
+        <v>20865350</v>
       </c>
       <c r="X30" s="74" t="n">
-        <v>0.7531020338544626</v>
+        <v>0.7545804097901414</v>
       </c>
       <c r="Y30" s="28" t="n">
         <v>41.9976626366506</v>
@@ -7712,17 +7712,17 @@
       </c>
       <c r="AX30" s="79" t="inlineStr">
         <is>
+          <t>Broadcom (AVGO) Stock May Be 24% Undervalued Following Fresh AI Demand Fears</t>
+        </is>
+      </c>
+      <c r="AY30" s="79" t="inlineStr">
+        <is>
+          <t>Broadcom's Latest Prediction Makes the Stock a No-Brainer Buy Right Now</t>
+        </is>
+      </c>
+      <c r="AZ30" s="79" t="inlineStr">
+        <is>
           <t>Broadcom Falls 2% as $230 Billion AI Target Doubles the Delivery Test</t>
-        </is>
-      </c>
-      <c r="AY30" s="79" t="inlineStr">
-        <is>
-          <t>Where Will Broadcom Stock Be in 5 Years?</t>
-        </is>
-      </c>
-      <c r="AZ30" s="79" t="inlineStr">
-        <is>
-          <t>3 Companies With a Strong History of Dividend Growth</t>
         </is>
       </c>
     </row>
@@ -7818,10 +7818,10 @@
         <v>88.04000091552734</v>
       </c>
       <c r="W31" s="84" t="n">
-        <v>3453523</v>
+        <v>3455423</v>
       </c>
       <c r="X31" s="85" t="n">
-        <v>1.175070908260476</v>
+        <v>1.175679385920688</v>
       </c>
       <c r="Y31" s="35" t="n">
         <v>35.8704697325515</v>
@@ -7900,17 +7900,17 @@
       </c>
       <c r="AX31" s="90" t="inlineStr">
         <is>
+          <t>Here's Why Cameco (CCJ) Fell More Than Broader Market</t>
+        </is>
+      </c>
+      <c r="AY31" s="90" t="inlineStr">
+        <is>
           <t>Is the Options Market Predicting a Spike in Cameco Stock?</t>
         </is>
       </c>
-      <c r="AY31" s="90" t="inlineStr">
+      <c r="AZ31" s="90" t="inlineStr">
         <is>
           <t>Cameco vs. MP Materials: Does Uranium or Rare Earths Make a Better Stock Buy in 2026?</t>
-        </is>
-      </c>
-      <c r="AZ31" s="90" t="inlineStr">
-        <is>
-          <t>Westinghouse Electric Is Taking Nuclear Back to the Stock Market. At 63, Where He Buys the IPO Decides How ...</t>
         </is>
       </c>
     </row>
@@ -7997,7 +7997,7 @@
         <v>3.229995727539062</v>
       </c>
       <c r="T32" s="72" t="n">
-        <v>88.90499877929688</v>
+        <v>88.80999755859375</v>
       </c>
       <c r="U32" s="72" t="n">
         <v>91.12249755859375</v>
@@ -8006,10 +8006,10 @@
         <v>85.93620300292969</v>
       </c>
       <c r="W32" s="73" t="n">
-        <v>33527903</v>
+        <v>33605545</v>
       </c>
       <c r="X32" s="74" t="n">
-        <v>1.158519732650342</v>
+        <v>1.161046821602089</v>
       </c>
       <c r="Y32" s="28" t="n">
         <v>53.92956966968482</v>
@@ -8194,10 +8194,10 @@
         <v>530.4500122070312</v>
       </c>
       <c r="W33" s="84" t="n">
-        <v>7910073</v>
+        <v>7927868</v>
       </c>
       <c r="X33" s="85" t="n">
-        <v>0.7138498631376986</v>
+        <v>0.7153983412047411</v>
       </c>
       <c r="Y33" s="35" t="n">
         <v>54.0948300199157</v>
@@ -8276,17 +8276,17 @@
       </c>
       <c r="AX33" s="90" t="inlineStr">
         <is>
-          <t>Why These S&amp;P 500 Stocks Are Earning The Biggest EPS Upgrades</t>
+          <t>Is Dell Technologies (DELL) Stock a Buy After its $5 Billion AI-Fueled Bond Sale?</t>
         </is>
       </c>
       <c r="AY33" s="90" t="inlineStr">
         <is>
-          <t>Dell Slips 2.34% as $999 Googlebook Tests Premium AI PCs</t>
+          <t>What Changed In Dell's Story?</t>
         </is>
       </c>
       <c r="AZ33" s="90" t="inlineStr">
         <is>
-          <t>BairesDev’s Rodrigo Outumuro Named to HR’s Rising Stars 2026</t>
+          <t>Dell Top Executives Sell $32 Million in Stock as AI Rally Accelerates</t>
         </is>
       </c>
     </row>
@@ -8382,10 +8382,10 @@
         <v>332.8099975585938</v>
       </c>
       <c r="W34" s="73" t="n">
-        <v>15615617</v>
+        <v>15687193</v>
       </c>
       <c r="X34" s="74" t="n">
-        <v>0.8797012374344129</v>
+        <v>0.8835553163890739</v>
       </c>
       <c r="Y34" s="28" t="n">
         <v>48.26658070404994</v>
@@ -8464,17 +8464,17 @@
       </c>
       <c r="AX34" s="79" t="inlineStr">
         <is>
-          <t>Google Prepares to Put AI Chips Into Space</t>
+          <t>Meta's new AI device changes everything</t>
         </is>
       </c>
       <c r="AY34" s="79" t="inlineStr">
         <is>
-          <t>Google Is Taking a Major Step Forward Toward Space-Based AI Data Centers</t>
+          <t>Google is Changing Search to Avoid More EU Fines. Could Compliance Become the Bigger Risk?</t>
         </is>
       </c>
       <c r="AZ34" s="79" t="inlineStr">
         <is>
-          <t>Alphabet Drops Below $350: Buying Opportunity or the Start of Something Worse?</t>
+          <t>Alphabet Reportedly Values Its Anthropic Stake at $124 Billion. A $2 Trillion IPO Could Double It -- on Paper.</t>
         </is>
       </c>
     </row>
@@ -8570,10 +8570,10 @@
         <v>45.14289855957031</v>
       </c>
       <c r="W35" s="84" t="n">
-        <v>30192685</v>
+        <v>30279081</v>
       </c>
       <c r="X35" s="85" t="n">
-        <v>0.7472709170642213</v>
+        <v>0.7493291089125886</v>
       </c>
       <c r="Y35" s="35" t="n">
         <v>56.04600150230382</v>
@@ -8758,10 +8758,10 @@
         <v>119.5500030517578</v>
       </c>
       <c r="W36" s="73" t="n">
-        <v>117876418</v>
+        <v>118581605</v>
       </c>
       <c r="X36" s="74" t="n">
-        <v>1.11431492479272</v>
+        <v>1.120607716107054</v>
       </c>
       <c r="Y36" s="28" t="n">
         <v>73.01301375737832</v>
@@ -8937,7 +8937,7 @@
         <v>-2.660003662109375</v>
       </c>
       <c r="T37" s="83" t="n">
-        <v>495.0700073242188</v>
+        <v>495.3900146484375</v>
       </c>
       <c r="U37" s="83" t="n">
         <v>498.8800048828125</v>
@@ -8946,10 +8946,10 @@
         <v>491.2200012207031</v>
       </c>
       <c r="W37" s="84" t="n">
-        <v>16459047</v>
+        <v>16611248</v>
       </c>
       <c r="X37" s="85" t="n">
-        <v>0.7716837154058181</v>
+        <v>0.7785418892542548</v>
       </c>
       <c r="Y37" s="35" t="n">
         <v>54.36286859766769</v>
@@ -9134,10 +9134,10 @@
         <v>158.2899932861328</v>
       </c>
       <c r="W38" s="73" t="n">
-        <v>16614443</v>
+        <v>16738047</v>
       </c>
       <c r="X38" s="74" t="n">
-        <v>0.6369902542955521</v>
+        <v>0.6415771567374591</v>
       </c>
       <c r="Y38" s="28" t="n">
         <v>65.8047942135762</v>
@@ -9322,10 +9322,10 @@
         <v>1044</v>
       </c>
       <c r="W39" s="84" t="n">
-        <v>21812855</v>
+        <v>21938990</v>
       </c>
       <c r="X39" s="85" t="n">
-        <v>0.8591996047332551</v>
+        <v>0.8639533881596195</v>
       </c>
       <c r="Y39" s="35" t="n">
         <v>63.02093183680572</v>
@@ -9404,17 +9404,17 @@
       </c>
       <c r="AX39" s="90" t="inlineStr">
         <is>
-          <t>Micron Just Rallied 17% in a Month: Take Profits, or Buy More?</t>
+          <t>Forget Betting on Micron Alone: The $26B Memory ETF Owns MU, SK Hynix, and Samsung at a September Discount</t>
         </is>
       </c>
       <c r="AY39" s="90" t="inlineStr">
         <is>
-          <t>Michael Burry keeps pointing at unloved stocks for a reason</t>
+          <t>3 Reasons Why Micron and Sandisk Investors Can Ignore What History Says Will Happen</t>
         </is>
       </c>
       <c r="AZ39" s="90" t="inlineStr">
         <is>
-          <t>Micron Stock Gets a Big Wall Street Boost Ahead of Earnings</t>
+          <t>5-star analyst resets Micron stock price target by 8%</t>
         </is>
       </c>
     </row>
@@ -9510,10 +9510,10 @@
         <v>229.5</v>
       </c>
       <c r="W40" s="73" t="n">
-        <v>24044028</v>
+        <v>24256977</v>
       </c>
       <c r="X40" s="74" t="n">
-        <v>1.5627245877776</v>
+        <v>1.575474791815994</v>
       </c>
       <c r="Y40" s="28" t="n">
         <v>58.30119956465312</v>
@@ -9698,10 +9698,10 @@
         <v>71.20999908447266</v>
       </c>
       <c r="W41" s="84" t="n">
-        <v>28040664</v>
+        <v>28121254</v>
       </c>
       <c r="X41" s="85" t="n">
-        <v>0.8595136398458048</v>
+        <v>0.861877462936041</v>
       </c>
       <c r="Y41" s="35" t="n">
         <v>38.22368736291582</v>
@@ -9780,17 +9780,17 @@
       </c>
       <c r="AX41" s="90" t="inlineStr">
         <is>
+          <t>Netflix's Revenue Growth Has Slowed for 2 Straight Quarters. Should You Buy the Stock Anyway?</t>
+        </is>
+      </c>
+      <c r="AY41" s="90" t="inlineStr">
+        <is>
           <t>Netflix Edges Higher Despite HSBC Engagement Expectations Cut</t>
         </is>
       </c>
-      <c r="AY41" s="90" t="inlineStr">
+      <c r="AZ41" s="90" t="inlineStr">
         <is>
           <t>What Would A Real Market Crash Do To Netflix Stock After This Fall?</t>
-        </is>
-      </c>
-      <c r="AZ41" s="90" t="inlineStr">
-        <is>
-          <t>Zacks Investment Ideas feature highlights: Netflix</t>
         </is>
       </c>
     </row>
@@ -9886,10 +9886,10 @@
         <v>10.17010021209717</v>
       </c>
       <c r="W42" s="73" t="n">
-        <v>74782160</v>
+        <v>74815291</v>
       </c>
       <c r="X42" s="74" t="n">
-        <v>0.8526787163480846</v>
+        <v>0.853040369111612</v>
       </c>
       <c r="Y42" s="28" t="n">
         <v>50.20694616599592</v>
@@ -10074,10 +10074,10 @@
         <v>221.0908050537109</v>
       </c>
       <c r="W43" s="84" t="n">
-        <v>75752682</v>
+        <v>76420503</v>
       </c>
       <c r="X43" s="85" t="n">
-        <v>0.5991681747314328</v>
+        <v>0.6042907277911681</v>
       </c>
       <c r="Y43" s="35" t="n">
         <v>54.71724882425972</v>
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
-          <t>Soaring Defense Spending Means Great News for These 2 Stocks</t>
+          <t>Why Semiconductor Investors Are Rotating From SMH’s Nvidia Concentration to PSI’s Equal-Weight Approach</t>
         </is>
       </c>
       <c r="AY43" s="90" t="inlineStr">
         <is>
-          <t>Amazon Blocks Meta's Muse. It Could Be a Gift for Walmart and Shopify</t>
+          <t>Darden Restaurants, Inc. Q1 2027 Earnings Call Summary</t>
         </is>
       </c>
       <c r="AZ43" s="90" t="inlineStr">
         <is>
-          <t>Nvidia, AMD Love This High-Tech Facilitator. So Does Wall Street.</t>
+          <t>TD SYNNEX Corporation Q3 2026 Earnings Call Summary</t>
         </is>
       </c>
     </row>
@@ -10262,10 +10262,10 @@
         <v>188.2400054931641</v>
       </c>
       <c r="W44" s="73" t="n">
-        <v>22557318</v>
+        <v>22612777</v>
       </c>
       <c r="X44" s="74" t="n">
-        <v>0.8201782486144512</v>
+        <v>0.8221118351175177</v>
       </c>
       <c r="Y44" s="28" t="n">
         <v>67.36751284030443</v>
@@ -10344,17 +10344,17 @@
       </c>
       <c r="AX44" s="79" t="inlineStr">
         <is>
+          <t>Anthropic proposes supervoting shares to give co-founders majority control -report</t>
+        </is>
+      </c>
+      <c r="AY44" s="79" t="inlineStr">
+        <is>
+          <t>Does Palantir (PLTR) Have a Moat Strong Enough to Protect Its AI Dominance?</t>
+        </is>
+      </c>
+      <c r="AZ44" s="79" t="inlineStr">
+        <is>
           <t>Rosenblatt Has Message For Palantir Stock Investors</t>
-        </is>
-      </c>
-      <c r="AY44" s="79" t="inlineStr">
-        <is>
-          <t>Palantir Slips as Karp Puts Liability Before AI Listings</t>
-        </is>
-      </c>
-      <c r="AZ44" s="79" t="inlineStr">
-        <is>
-          <t>Inside the $600 Billion Sovereign AI Gold Rush -- and Why Palantir Is Positioned to Win</t>
         </is>
       </c>
     </row>
@@ -10450,10 +10450,10 @@
         <v>191.75</v>
       </c>
       <c r="W45" s="84" t="n">
-        <v>9042129</v>
+        <v>9058984</v>
       </c>
       <c r="X45" s="85" t="n">
-        <v>0.6268568579995603</v>
+        <v>0.6279886618280421</v>
       </c>
       <c r="Y45" s="35" t="n">
         <v>63.17299974059192</v>
@@ -10532,17 +10532,17 @@
       </c>
       <c r="AX45" s="90" t="inlineStr">
         <is>
-          <t>What's Going On With Qualcomm Stock Thursday</t>
+          <t>Meta's new AI device changes everything</t>
         </is>
       </c>
       <c r="AY45" s="90" t="inlineStr">
         <is>
-          <t>Qualcomm CFO says look beyond the Apple deal</t>
+          <t>Qualcomm (QCOM) Registers a Bigger Fall Than the Market: Important Facts to Note</t>
         </is>
       </c>
       <c r="AZ45" s="90" t="inlineStr">
         <is>
-          <t>3 Reasons to Avoid QCOM and 1 Stock to Buy Instead</t>
+          <t>Chip Stocks Retreat. Qualcomm Secures Apple Licensing Deal.</t>
         </is>
       </c>
     </row>
@@ -10638,10 +10638,10 @@
         <v>68.92160034179688</v>
       </c>
       <c r="W46" s="73" t="n">
-        <v>24896036</v>
+        <v>25020442</v>
       </c>
       <c r="X46" s="74" t="n">
-        <v>1.261730002454734</v>
+        <v>1.267635277942186</v>
       </c>
       <c r="Y46" s="28" t="n">
         <v>58.92679087340188</v>
@@ -10720,17 +10720,17 @@
       </c>
       <c r="AX46" s="79" t="inlineStr">
         <is>
+          <t>IRDM Shareholders Approve Acquisition By RKLB In $54-A-Share Deal — Iridium-Rocket Lab Merger Expected To C...</t>
+        </is>
+      </c>
+      <c r="AY46" s="79" t="inlineStr">
+        <is>
           <t>Iridium Stockholders Approve Acquisition by Rocket Lab</t>
         </is>
       </c>
-      <c r="AY46" s="79" t="inlineStr">
+      <c r="AZ46" s="79" t="inlineStr">
         <is>
           <t>Space Stocks Rally as Buying Spreads Across the Pure Plays: Rocket Lab and Planet Labs Jump 6%, AST SpaceMo...</t>
-        </is>
-      </c>
-      <c r="AZ46" s="79" t="inlineStr">
-        <is>
-          <t>Why Cathie Wood Is Trimming the World’s Biggest Tech Stock to Bet on a Space Company</t>
         </is>
       </c>
     </row>
@@ -10826,10 +10826,10 @@
         <v>1726.390014648438</v>
       </c>
       <c r="W47" s="84" t="n">
-        <v>8115290</v>
+        <v>8145414</v>
       </c>
       <c r="X47" s="85" t="n">
-        <v>0.7565339380043758</v>
+        <v>0.7592355895670841</v>
       </c>
       <c r="Y47" s="35" t="n">
         <v>56.18883673359787</v>
@@ -10908,17 +10908,17 @@
       </c>
       <c r="AX47" s="90" t="inlineStr">
         <is>
+          <t>Micron vs. Sandisk: Which AI Memory Stock Is the Better Buy?</t>
+        </is>
+      </c>
+      <c r="AY47" s="90" t="inlineStr">
+        <is>
           <t>Sandisk (SNDK) Stock May Still Look Reasonable After AI Slowdown Fears</t>
         </is>
       </c>
-      <c r="AY47" s="90" t="inlineStr">
+      <c r="AZ47" s="90" t="inlineStr">
         <is>
           <t>Will Sandisk or Micron Perform a Stock Split Next Year?</t>
-        </is>
-      </c>
-      <c r="AZ47" s="90" t="inlineStr">
-        <is>
-          <t>Why Rosenblatt Thinks Sandisk Stock Is Headed for $2,400</t>
         </is>
       </c>
     </row>
@@ -11014,10 +11014,10 @@
         <v>375.7000122070312</v>
       </c>
       <c r="W48" s="73" t="n">
-        <v>25844378</v>
+        <v>25925858</v>
       </c>
       <c r="X48" s="74" t="n">
-        <v>0.6651629786706298</v>
+        <v>0.6671900918182481</v>
       </c>
       <c r="Y48" s="28" t="n">
         <v>59.13843172330105</v>
@@ -11096,17 +11096,17 @@
       </c>
       <c r="AX48" s="79" t="inlineStr">
         <is>
-          <t>Tesla to open doors of its Nevada Semi truck factory</t>
+          <t>Dow Jones Futures: Market Rally Resilient As Yields, Oil Prices Keep Rising; Tesla Event On Deck</t>
         </is>
       </c>
       <c r="AY48" s="79" t="inlineStr">
         <is>
-          <t>Is Tesla (TSLA) Priced For Too Much Sales Growth After Recent Expansion Bets?</t>
+          <t>Tesla's Roadster Reveal Is Oct. 1. The Real Story Is Optimus.</t>
         </is>
       </c>
       <c r="AZ48" s="79" t="inlineStr">
         <is>
-          <t>Elon Musk Has Left the Door Open to a Tesla-SpaceX Merger. Here's What Shareholders of Both Stocks Should Do.</t>
+          <t>Top Stock Reports for Tesla, Bank of America &amp; Coca-Cola</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 24 Sep 2026, 08:38 PM · Yahoo Finance data</t>
+          <t>Built 24 Sep 2026, 11:14 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 24 Sep 2026, 08:38 PM · Yahoo Finance data</t>
+          <t>Built 24 Sep 2026, 11:14 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 24 Sep 2026, 08:38 PM · Yahoo Finance data</t>
+          <t>Built 24 Sep 2026, 11:14 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 24 Sep 2026, 08:38 PM · Yahoo Finance data</t>
+          <t>Built 24 Sep 2026, 11:14 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -43449,7 +43449,7 @@
         <v>0.400134192708169</v>
       </c>
       <c r="J8" s="27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K8" s="101" t="inlineStr">
         <is>
@@ -43864,7 +43864,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:G44"/>
+  <dimension ref="B2:G45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -44304,7 +44304,7 @@
       </c>
       <c r="D19" s="105" t="inlineStr">
         <is>
-          <t>Gapped up 2.3% at the open</t>
+          <t>Gapped up 2.2% at the open</t>
         </is>
       </c>
       <c r="E19" s="33" t="n">
@@ -44668,7 +44668,7 @@
       </c>
       <c r="D32" s="104" t="inlineStr">
         <is>
-          <t>Bands squeezing — a big move often follows</t>
+          <t>Gapped down 1.6% at the open</t>
         </is>
       </c>
       <c r="E32" s="26" t="n">
@@ -44686,21 +44686,21 @@
     <row r="33">
       <c r="B33" s="31" t="inlineStr">
         <is>
-          <t>DELL</t>
+          <t>ASTS</t>
         </is>
       </c>
       <c r="C33" s="102" t="inlineStr">
         <is>
-          <t>Dell Technologies Inc.</t>
+          <t>AST SpaceMobile, Inc.</t>
         </is>
       </c>
       <c r="D33" s="105" t="inlineStr">
         <is>
-          <t>MACD crossed down</t>
+          <t>Bands squeezing — a big move often follows</t>
         </is>
       </c>
       <c r="E33" s="33" t="n">
-        <v>-0.025116849079444</v>
+        <v>0.01800603266584178</v>
       </c>
       <c r="F33" s="34" t="n">
         <v>5</v>
@@ -44724,7 +44724,7 @@
       </c>
       <c r="D34" s="104" t="inlineStr">
         <is>
-          <t>Gapped down 2.5% at the open</t>
+          <t>MACD crossed down</t>
         </is>
       </c>
       <c r="E34" s="26" t="n">
@@ -44742,24 +44742,24 @@
     <row r="35">
       <c r="B35" s="31" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>DELL</t>
         </is>
       </c>
       <c r="C35" s="102" t="inlineStr">
         <is>
-          <t>Alphabet Inc.</t>
+          <t>Dell Technologies Inc.</t>
         </is>
       </c>
       <c r="D35" s="105" t="inlineStr">
         <is>
-          <t>Reclaimed the 200 DMA</t>
+          <t>Gapped down 2.5% at the open</t>
         </is>
       </c>
       <c r="E35" s="33" t="n">
-        <v>0.01203056495051991</v>
+        <v>-0.025116849079444</v>
       </c>
       <c r="F35" s="34" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G35" s="30" t="inlineStr">
         <is>
@@ -44770,21 +44770,21 @@
     <row r="36">
       <c r="B36" s="24" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="C36" s="101" t="inlineStr">
         <is>
-          <t>Microsoft Corporation</t>
+          <t>Alphabet Inc.</t>
         </is>
       </c>
       <c r="D36" s="104" t="inlineStr">
         <is>
-          <t>Bands squeezing — a big move often follows</t>
+          <t>Reclaimed the 200 DMA</t>
         </is>
       </c>
       <c r="E36" s="26" t="n">
-        <v>-0.00531373715329686</v>
+        <v>0.01203056495051991</v>
       </c>
       <c r="F36" s="27" t="n">
         <v>4</v>
@@ -44815,60 +44815,60 @@
         <v>0.003687663078005166</v>
       </c>
       <c r="F37" s="34" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G37" s="30" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="24" t="inlineStr">
         <is>
-          <t>XLF</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="C38" s="101" t="inlineStr">
         <is>
-          <t>State Street Financial Select Sector SPDR ETF</t>
-        </is>
-      </c>
-      <c r="D38" s="106" t="inlineStr">
-        <is>
-          <t>RSI oversold (28)</t>
+          <t>Microsoft Corporation</t>
+        </is>
+      </c>
+      <c r="D38" s="104" t="inlineStr">
+        <is>
+          <t>Bands squeezing — a big move often follows</t>
         </is>
       </c>
       <c r="E38" s="26" t="n">
-        <v>-0.0001833908335637791</v>
+        <v>-0.00531373715329686</v>
       </c>
       <c r="F38" s="27" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G38" s="23" t="inlineStr">
         <is>
-          <t>Very Weak</t>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="31" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>XLF</t>
         </is>
       </c>
       <c r="C39" s="102" t="inlineStr">
         <is>
-          <t>Broadcom Inc.</t>
-        </is>
-      </c>
-      <c r="D39" s="105" t="inlineStr">
-        <is>
-          <t>Gapped down 1.6% at the open</t>
+          <t>State Street Financial Select Sector SPDR ETF</t>
+        </is>
+      </c>
+      <c r="D39" s="107" t="inlineStr">
+        <is>
+          <t>RSI oversold (28)</t>
         </is>
       </c>
       <c r="E39" s="33" t="n">
-        <v>-0.01304263503248537</v>
+        <v>-0.0001833908335637791</v>
       </c>
       <c r="F39" s="34" t="n">
         <v>1</v>
@@ -44882,24 +44882,24 @@
     <row r="40">
       <c r="B40" s="24" t="inlineStr">
         <is>
-          <t>XLRE</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="C40" s="101" t="inlineStr">
         <is>
-          <t>State Street Real Estate Select Sector SPDR ETF</t>
+          <t>Broadcom Inc.</t>
         </is>
       </c>
       <c r="D40" s="104" t="inlineStr">
         <is>
-          <t>Closed below lower band</t>
+          <t>Gapped down 1.6% at the open</t>
         </is>
       </c>
       <c r="E40" s="26" t="n">
-        <v>-0.004541076147611678</v>
+        <v>-0.01304263503248537</v>
       </c>
       <c r="F40" s="27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G40" s="23" t="inlineStr">
         <is>
@@ -44918,9 +44918,9 @@
           <t>State Street Real Estate Select Sector SPDR ETF</t>
         </is>
       </c>
-      <c r="D41" s="107" t="inlineStr">
-        <is>
-          <t>RSI oversold (25)</t>
+      <c r="D41" s="105" t="inlineStr">
+        <is>
+          <t>Closed below lower band</t>
         </is>
       </c>
       <c r="E41" s="33" t="n">
@@ -44938,21 +44938,21 @@
     <row r="42">
       <c r="B42" s="24" t="inlineStr">
         <is>
-          <t>XLU</t>
+          <t>XLRE</t>
         </is>
       </c>
       <c r="C42" s="101" t="inlineStr">
         <is>
-          <t>State Street Utilities Select Sector SPDR ETF</t>
-        </is>
-      </c>
-      <c r="D42" s="104" t="inlineStr">
-        <is>
-          <t>Closed below lower band</t>
+          <t>State Street Real Estate Select Sector SPDR ETF</t>
+        </is>
+      </c>
+      <c r="D42" s="106" t="inlineStr">
+        <is>
+          <t>RSI oversold (25)</t>
         </is>
       </c>
       <c r="E42" s="26" t="n">
-        <v>-0.009811305399960668</v>
+        <v>-0.004541076147611678</v>
       </c>
       <c r="F42" s="27" t="n">
         <v>0</v>
@@ -44974,9 +44974,9 @@
           <t>State Street Utilities Select Sector SPDR ETF</t>
         </is>
       </c>
-      <c r="D43" s="107" t="inlineStr">
-        <is>
-          <t>RSI oversold (22)</t>
+      <c r="D43" s="105" t="inlineStr">
+        <is>
+          <t>Closed below lower band</t>
         </is>
       </c>
       <c r="E43" s="33" t="n">
@@ -45002,9 +45002,9 @@
           <t>State Street Utilities Select Sector SPDR ETF</t>
         </is>
       </c>
-      <c r="D44" s="104" t="inlineStr">
-        <is>
-          <t>New 52-week low</t>
+      <c r="D44" s="106" t="inlineStr">
+        <is>
+          <t>RSI oversold (22)</t>
         </is>
       </c>
       <c r="E44" s="26" t="n">
@@ -45019,12 +45019,40 @@
         </is>
       </c>
     </row>
+    <row r="45">
+      <c r="B45" s="31" t="inlineStr">
+        <is>
+          <t>XLU</t>
+        </is>
+      </c>
+      <c r="C45" s="102" t="inlineStr">
+        <is>
+          <t>State Street Utilities Select Sector SPDR ETF</t>
+        </is>
+      </c>
+      <c r="D45" s="105" t="inlineStr">
+        <is>
+          <t>New 52-week low</t>
+        </is>
+      </c>
+      <c r="E45" s="33" t="n">
+        <v>-0.009811305399960668</v>
+      </c>
+      <c r="F45" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" s="30" t="inlineStr">
+        <is>
+          <t>Very Weak</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="B5:G44"/>
+  <autoFilter ref="B5:G45"/>
   <mergeCells count="1">
     <mergeCell ref="B2:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="E6:E44">
+  <conditionalFormatting sqref="E6:E45">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="-0.05"/>

</xml_diff>

<commit_message>
Daily workbook: 2026-09-24 23:52 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 24 Sep 2026, 11:14 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 24 Sep 2026, 11:52 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 24 Sep 2026, 11:14 PM · Yahoo Finance data</t>
+          <t>Built 24 Sep 2026, 11:52 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -6594,7 +6594,7 @@
       </c>
       <c r="AZ24" s="79" t="inlineStr">
         <is>
-          <t>Could John Ternus’ Product Strategy Reshape Apple’s (AAPL) Next Growth Phase?</t>
+          <t>Here is Why Garmin (GRMN) is a Good Investment at Today’s Price</t>
         </is>
       </c>
     </row>
@@ -7336,17 +7336,17 @@
       </c>
       <c r="AX28" s="79" t="inlineStr">
         <is>
+          <t>Arm Holdings (ARM) Stock Gains On AI CPU Demand Surge</t>
+        </is>
+      </c>
+      <c r="AY28" s="79" t="inlineStr">
+        <is>
           <t>Arm Drops 3.3% as More AI Cores Test Royalty Economics</t>
         </is>
       </c>
-      <c r="AY28" s="79" t="inlineStr">
+      <c r="AZ28" s="79" t="inlineStr">
         <is>
           <t>Critical Role of ARM Holdings (ARM) In Powering the Next Wave of Agentic AI</t>
-        </is>
-      </c>
-      <c r="AZ28" s="79" t="inlineStr">
-        <is>
-          <t>SoftBank Is Raising $11 Billion for OpenAI. Its Arm Stake Backs a $25 Billion Loan Facility</t>
         </is>
       </c>
     </row>
@@ -8469,12 +8469,12 @@
       </c>
       <c r="AY34" s="79" t="inlineStr">
         <is>
+          <t>Waymo is scaling fast. Here’s what the fleet data shows.</t>
+        </is>
+      </c>
+      <c r="AZ34" s="79" t="inlineStr">
+        <is>
           <t>Google is Changing Search to Avoid More EU Fines. Could Compliance Become the Bigger Risk?</t>
-        </is>
-      </c>
-      <c r="AZ34" s="79" t="inlineStr">
-        <is>
-          <t>Alphabet Reportedly Values Its Anthropic Stake at $124 Billion. A $2 Trillion IPO Could Double It -- on Paper.</t>
         </is>
       </c>
     </row>
@@ -10720,17 +10720,17 @@
       </c>
       <c r="AX46" s="79" t="inlineStr">
         <is>
+          <t>Cathie Wood buys $25 million in tumbling tech stock</t>
+        </is>
+      </c>
+      <c r="AY46" s="79" t="inlineStr">
+        <is>
           <t>IRDM Shareholders Approve Acquisition By RKLB In $54-A-Share Deal — Iridium-Rocket Lab Merger Expected To C...</t>
         </is>
       </c>
-      <c r="AY46" s="79" t="inlineStr">
+      <c r="AZ46" s="79" t="inlineStr">
         <is>
           <t>Iridium Stockholders Approve Acquisition by Rocket Lab</t>
-        </is>
-      </c>
-      <c r="AZ46" s="79" t="inlineStr">
-        <is>
-          <t>Space Stocks Rally as Buying Spreads Across the Pure Plays: Rocket Lab and Planet Labs Jump 6%, AST SpaceMo...</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 24 Sep 2026, 11:14 PM · Yahoo Finance data</t>
+          <t>Built 24 Sep 2026, 11:52 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 24 Sep 2026, 11:14 PM · Yahoo Finance data</t>
+          <t>Built 24 Sep 2026, 11:52 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 24 Sep 2026, 11:14 PM · Yahoo Finance data</t>
+          <t>Built 24 Sep 2026, 11:52 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 24 Sep 2026, 11:14 PM · Yahoo Finance data</t>
+          <t>Built 24 Sep 2026, 11:52 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-09-25 23:19 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 25 Sep 2026, 08:37 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 25 Sep 2026, 11:19 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -1592,7 +1592,7 @@
         <v>0.005684969378886295</v>
       </c>
       <c r="F16" s="27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G16" s="28" t="n">
         <v>32.90243851206939</v>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 25 Sep 2026, 08:37 PM · Yahoo Finance data</t>
+          <t>Built 25 Sep 2026, 11:19 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -3620,10 +3620,10 @@
         <v>169.0299987792969</v>
       </c>
       <c r="W7" s="73" t="n">
-        <v>7280522</v>
+        <v>7280606</v>
       </c>
       <c r="X7" s="74" t="n">
-        <v>0.9393832727782079</v>
+        <v>0.9393936019691974</v>
       </c>
       <c r="Y7" s="28" t="n">
         <v>39.90619649923384</v>
@@ -3810,10 +3810,10 @@
         <v>168.6849975585938</v>
       </c>
       <c r="W8" s="84" t="n">
-        <v>5931829</v>
+        <v>5937318</v>
       </c>
       <c r="X8" s="85" t="n">
-        <v>0.7823973770097233</v>
+        <v>0.7830930185147065</v>
       </c>
       <c r="Y8" s="35" t="n">
         <v>56.44211234772722</v>
@@ -3967,7 +3967,7 @@
         </is>
       </c>
       <c r="N9" s="69" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O9" s="23" t="inlineStr">
         <is>
@@ -4000,10 +4000,10 @@
         <v>54.31000137329102</v>
       </c>
       <c r="W9" s="73" t="n">
-        <v>28767254</v>
+        <v>29036071</v>
       </c>
       <c r="X9" s="74" t="n">
-        <v>0.8383411073506694</v>
+        <v>0.8458437129193708</v>
       </c>
       <c r="Y9" s="28" t="n">
         <v>32.90243851206939</v>
@@ -4190,10 +4190,10 @@
         <v>61.65999984741211</v>
       </c>
       <c r="W10" s="84" t="n">
-        <v>37398357</v>
+        <v>37439924</v>
       </c>
       <c r="X10" s="85" t="n">
-        <v>1.127654402317913</v>
+        <v>1.128837010414797</v>
       </c>
       <c r="Y10" s="35" t="n">
         <v>44.55075150375365</v>
@@ -4380,10 +4380,10 @@
         <v>81.33000183105469</v>
       </c>
       <c r="W11" s="73" t="n">
-        <v>8496303</v>
+        <v>8509504</v>
       </c>
       <c r="X11" s="74" t="n">
-        <v>0.8481748192874804</v>
+        <v>0.8494366868353258</v>
       </c>
       <c r="Y11" s="28" t="n">
         <v>39.1162395405759</v>
@@ -4570,10 +4570,10 @@
         <v>109.6500015258789</v>
       </c>
       <c r="W12" s="84" t="n">
-        <v>6082819</v>
+        <v>6082861</v>
       </c>
       <c r="X12" s="85" t="n">
-        <v>0.9842046949740697</v>
+        <v>0.9842111561888756</v>
       </c>
       <c r="Y12" s="35" t="n">
         <v>38.66771778342982</v>
@@ -4950,10 +4950,10 @@
         <v>49.45000076293945</v>
       </c>
       <c r="W14" s="84" t="n">
-        <v>9914471</v>
+        <v>9918906</v>
       </c>
       <c r="X14" s="85" t="n">
-        <v>0.8714452886136662</v>
+        <v>0.8718181160810233</v>
       </c>
       <c r="Y14" s="35" t="n">
         <v>38.00148336198168</v>
@@ -5140,10 +5140,10 @@
         <v>195.0500030517578</v>
       </c>
       <c r="W15" s="73" t="n">
-        <v>5965183</v>
+        <v>5968181</v>
       </c>
       <c r="X15" s="74" t="n">
-        <v>0.8817414558677587</v>
+        <v>0.8821650576991692</v>
       </c>
       <c r="Y15" s="28" t="n">
         <v>65.35355037531475</v>
@@ -5330,10 +5330,10 @@
         <v>41.34000015258789</v>
       </c>
       <c r="W16" s="84" t="n">
-        <v>5753402</v>
+        <v>5753403</v>
       </c>
       <c r="X16" s="85" t="n">
-        <v>1.055708813980168</v>
+        <v>1.055708987787378</v>
       </c>
       <c r="Y16" s="35" t="n">
         <v>24.10372046044128</v>
@@ -5520,10 +5520,10 @@
         <v>39.125</v>
       </c>
       <c r="W17" s="73" t="n">
-        <v>29642115</v>
+        <v>29656584</v>
       </c>
       <c r="X17" s="74" t="n">
-        <v>1.276683497350225</v>
+        <v>1.277266877737724</v>
       </c>
       <c r="Y17" s="28" t="n">
         <v>24.08322061547351</v>
@@ -5729,10 +5729,10 @@
         <v>766.2899780273438</v>
       </c>
       <c r="W19" s="73" t="n">
-        <v>34116693</v>
+        <v>35238956</v>
       </c>
       <c r="X19" s="74" t="n">
-        <v>0.7821188574534268</v>
+        <v>0.8068086631233591</v>
       </c>
       <c r="Y19" s="28" t="n">
         <v>55.89003490300169</v>
@@ -5811,17 +5811,17 @@
       </c>
       <c r="AX19" s="79" t="inlineStr">
         <is>
+          <t>S&amp;P 500, Dow, Nasdaq End Week Higher On Chipmaker Strength, Easing Oil Amid Signs Of Easing US-Iran Conflic...</t>
+        </is>
+      </c>
+      <c r="AY19" s="79" t="inlineStr">
+        <is>
           <t>Dell Rises 7% as Morgan Stanley Lifts Odds on $756 Bull Case; Hewlett Packard Enterprise Edges Higher</t>
         </is>
       </c>
-      <c r="AY19" s="79" t="inlineStr">
+      <c r="AZ19" s="79" t="inlineStr">
         <is>
           <t>Whether You Buy Tesla Depends On The Chances That Tesla Actually Becomes an AI Firm</t>
-        </is>
-      </c>
-      <c r="AZ19" s="79" t="inlineStr">
-        <is>
-          <t>Micron at $1080: The Street Loves What It Sees Underneath The Headlines</t>
         </is>
       </c>
     </row>
@@ -5845,7 +5845,7 @@
       </c>
       <c r="F20" s="30" t="inlineStr">
         <is>
-          <t>Same</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G20" s="30" t="inlineStr">
@@ -5917,10 +5917,10 @@
         <v>739.6400146484375</v>
       </c>
       <c r="W20" s="84" t="n">
-        <v>29536154</v>
+        <v>30017218</v>
       </c>
       <c r="X20" s="85" t="n">
-        <v>0.8917650913992408</v>
+        <v>0.9056318411579448</v>
       </c>
       <c r="Y20" s="35" t="n">
         <v>64.68742047332788</v>
@@ -5999,17 +5999,17 @@
       </c>
       <c r="AX20" s="90" t="inlineStr">
         <is>
+          <t>You’re 45, Make $150K, and Have Never Opened a Brokerage Account. These 3 ETFs Are the First Deposit</t>
+        </is>
+      </c>
+      <c r="AY20" s="90" t="inlineStr">
+        <is>
           <t>The Case For and Against Fidelity’s Fundamental Large Cap Growth ETF</t>
         </is>
       </c>
-      <c r="AY20" s="90" t="inlineStr">
+      <c r="AZ20" s="90" t="inlineStr">
         <is>
           <t>Exchange-Traded Funds Rise US Equities Advance After Midday</t>
-        </is>
-      </c>
-      <c r="AZ20" s="90" t="inlineStr">
-        <is>
-          <t>VGT vs. QQQ: Where Should You Invest $1,000 Right Now for Maximum Long-Term Growth?</t>
         </is>
       </c>
     </row>
@@ -6105,10 +6105,10 @@
         <v>280.4549865722656</v>
       </c>
       <c r="W21" s="73" t="n">
-        <v>22126129</v>
+        <v>22409666</v>
       </c>
       <c r="X21" s="74" t="n">
-        <v>0.9698656763375693</v>
+        <v>0.9816840563936964</v>
       </c>
       <c r="Y21" s="28" t="n">
         <v>34.85654933315288</v>
@@ -6293,10 +6293,10 @@
         <v>147.3899993896484</v>
       </c>
       <c r="W22" s="84" t="n">
-        <v>55598722</v>
+        <v>55809520</v>
       </c>
       <c r="X22" s="85" t="n">
-        <v>0.9474496056457952</v>
+        <v>0.9508709983401613</v>
       </c>
       <c r="Y22" s="35" t="n">
         <v>61.63353168880354</v>
@@ -6502,10 +6502,10 @@
         <v>334.5299987792969</v>
       </c>
       <c r="W24" s="73" t="n">
-        <v>29403008</v>
+        <v>29649787</v>
       </c>
       <c r="X24" s="74" t="n">
-        <v>0.6859387429691065</v>
+        <v>0.6914967665466368</v>
       </c>
       <c r="Y24" s="28" t="n">
         <v>65.67332189493369</v>
@@ -6589,12 +6589,12 @@
       </c>
       <c r="AY24" s="79" t="inlineStr">
         <is>
+          <t>Apple (AAPL) Rises Higher Than Market: Key Facts</t>
+        </is>
+      </c>
+      <c r="AZ24" s="79" t="inlineStr">
+        <is>
           <t>Deer Park Town Center Trades For $125M, Suburban Retail Buying Spree Rolls On</t>
-        </is>
-      </c>
-      <c r="AZ24" s="79" t="inlineStr">
-        <is>
-          <t>Apple Just Gained 10% in a Month. What Will It Take for AAPL Stock to Finally Hit $350?</t>
         </is>
       </c>
     </row>
@@ -6681,7 +6681,7 @@
         <v>1.3699951171875</v>
       </c>
       <c r="T25" s="83" t="n">
-        <v>634.5349731445312</v>
+        <v>635.0679931640625</v>
       </c>
       <c r="U25" s="83" t="n">
         <v>638.9500122070312</v>
@@ -6690,10 +6690,10 @@
         <v>625.52001953125</v>
       </c>
       <c r="W25" s="84" t="n">
-        <v>17354993</v>
+        <v>17516535</v>
       </c>
       <c r="X25" s="85" t="n">
-        <v>0.8029720982027732</v>
+        <v>0.8101434858533951</v>
       </c>
       <c r="Y25" s="35" t="n">
         <v>72.99571503316014</v>
@@ -6782,7 +6782,7 @@
       </c>
       <c r="AZ25" s="90" t="inlineStr">
         <is>
-          <t>AMD CEO Lisa Su is having a September to remember</t>
+          <t>Microsoft, Meta, Akamai, Zscaler, Comcast, and More Stocks That Explain Today’s Market</t>
         </is>
       </c>
     </row>
@@ -6878,10 +6878,10 @@
         <v>247.1799926757812</v>
       </c>
       <c r="W26" s="73" t="n">
-        <v>32663542</v>
+        <v>32976800</v>
       </c>
       <c r="X26" s="74" t="n">
-        <v>0.9261536339673093</v>
+        <v>0.9346207864471937</v>
       </c>
       <c r="Y26" s="28" t="n">
         <v>44.53594307206563</v>
@@ -6965,12 +6965,12 @@
       </c>
       <c r="AY26" s="79" t="inlineStr">
         <is>
+          <t>Interrupted authority and written vetting rules at center of New Mexico crash lawsuit</t>
+        </is>
+      </c>
+      <c r="AZ26" s="79" t="inlineStr">
+        <is>
           <t>Amazon Stocks Move Lower as Anthropic Commits $11.6 Billion Elsewhere</t>
-        </is>
-      </c>
-      <c r="AZ26" s="79" t="inlineStr">
-        <is>
-          <t>Should SpaceX Investors Be Worried About Competition From Amazon?</t>
         </is>
       </c>
     </row>
@@ -7066,10 +7066,10 @@
         <v>89.72000122070312</v>
       </c>
       <c r="W27" s="84" t="n">
-        <v>3969018</v>
+        <v>3981024</v>
       </c>
       <c r="X27" s="85" t="n">
-        <v>0.850175161207495</v>
+        <v>0.8526372439983352</v>
       </c>
       <c r="Y27" s="35" t="n">
         <v>61.92665807874</v>
@@ -7245,7 +7245,7 @@
         <v>3.980010986328125</v>
       </c>
       <c r="T28" s="72" t="n">
-        <v>318.5</v>
+        <v>318.1099853515625</v>
       </c>
       <c r="U28" s="72" t="n">
         <v>325.4800109863281</v>
@@ -7254,10 +7254,10 @@
         <v>310.0799865722656</v>
       </c>
       <c r="W28" s="73" t="n">
-        <v>6972303</v>
+        <v>6983681</v>
       </c>
       <c r="X28" s="74" t="n">
-        <v>1.316031654093357</v>
+        <v>1.318037735290698</v>
       </c>
       <c r="Y28" s="28" t="n">
         <v>61.18691287964294</v>
@@ -7433,7 +7433,7 @@
         <v>0.75</v>
       </c>
       <c r="T29" s="83" t="n">
-        <v>61.97999954223633</v>
+        <v>62.1077995300293</v>
       </c>
       <c r="U29" s="83" t="n">
         <v>63.21500015258789</v>
@@ -7442,10 +7442,10 @@
         <v>61.02000045776367</v>
       </c>
       <c r="W29" s="84" t="n">
-        <v>6394394</v>
+        <v>6415940</v>
       </c>
       <c r="X29" s="85" t="n">
-        <v>0.6501420580641132</v>
+        <v>0.6522612765958312</v>
       </c>
       <c r="Y29" s="35" t="n">
         <v>49.32118916493694</v>
@@ -7621,7 +7621,7 @@
         <v>2.45001220703125</v>
       </c>
       <c r="T30" s="72" t="n">
-        <v>352.6199951171875</v>
+        <v>352.6300048828125</v>
       </c>
       <c r="U30" s="72" t="n">
         <v>354.4299926757812</v>
@@ -7630,10 +7630,10 @@
         <v>349.4299926757812</v>
       </c>
       <c r="W30" s="73" t="n">
-        <v>15582394</v>
+        <v>15753539</v>
       </c>
       <c r="X30" s="74" t="n">
-        <v>0.5693765999449705</v>
+        <v>0.5754502618668451</v>
       </c>
       <c r="Y30" s="28" t="n">
         <v>43.71387649680234</v>
@@ -7818,10 +7818,10 @@
         <v>87.80000305175781</v>
       </c>
       <c r="W31" s="84" t="n">
-        <v>1938319</v>
+        <v>1938592</v>
       </c>
       <c r="X31" s="85" t="n">
-        <v>0.6712198099704374</v>
+        <v>0.6713111738554212</v>
       </c>
       <c r="Y31" s="35" t="n">
         <v>36.40840968595577</v>
@@ -7997,7 +7997,7 @@
         <v>-2.540000915527344</v>
       </c>
       <c r="T32" s="72" t="n">
-        <v>90.36499786376953</v>
+        <v>90.63420104980469</v>
       </c>
       <c r="U32" s="72" t="n">
         <v>90.90000152587891</v>
@@ -8006,10 +8006,10 @@
         <v>86.80000305175781</v>
       </c>
       <c r="W32" s="73" t="n">
-        <v>22765799</v>
+        <v>23199906</v>
       </c>
       <c r="X32" s="74" t="n">
-        <v>0.7824367431331888</v>
+        <v>0.7967621707108126</v>
       </c>
       <c r="Y32" s="28" t="n">
         <v>50.80004593494216</v>
@@ -8194,10 +8194,10 @@
         <v>541.235107421875</v>
       </c>
       <c r="W33" s="84" t="n">
-        <v>8680957</v>
+        <v>8694381</v>
       </c>
       <c r="X33" s="85" t="n">
-        <v>0.7692182445701428</v>
+        <v>0.7703619258950238</v>
       </c>
       <c r="Y33" s="35" t="n">
         <v>58.68869662331603</v>
@@ -8382,10 +8382,10 @@
         <v>337.9100036621094</v>
       </c>
       <c r="W34" s="73" t="n">
-        <v>13304415</v>
+        <v>13336367</v>
       </c>
       <c r="X34" s="74" t="n">
-        <v>0.7586512822376287</v>
+        <v>0.760403993645225</v>
       </c>
       <c r="Y34" s="28" t="n">
         <v>49.94089039770569</v>
@@ -8464,17 +8464,17 @@
       </c>
       <c r="AX34" s="79" t="inlineStr">
         <is>
+          <t>Market Chatter: US Appeals Court Upholds Pentagon's Anthropic Ban</t>
+        </is>
+      </c>
+      <c r="AY34" s="79" t="inlineStr">
+        <is>
           <t>Sundar Pichai Reported Alphabet's Cloud Backlog Hit $514 Billion After 82% Revenue Growth Last Quarter, Wit...</t>
         </is>
       </c>
-      <c r="AY34" s="79" t="inlineStr">
+      <c r="AZ34" s="79" t="inlineStr">
         <is>
           <t>Google’s New Initiative Aims to Match 25,000 Veterans With These In-Demand Jobs</t>
-        </is>
-      </c>
-      <c r="AZ34" s="79" t="inlineStr">
-        <is>
-          <t>Alphabet Moved Higher as TPUs Chase Power Beyond Earth</t>
         </is>
       </c>
     </row>
@@ -8570,10 +8570,10 @@
         <v>43.40999984741211</v>
       </c>
       <c r="W35" s="84" t="n">
-        <v>39992363</v>
+        <v>40140584</v>
       </c>
       <c r="X35" s="85" t="n">
-        <v>1.002413140096293</v>
+        <v>1.005941453876306</v>
       </c>
       <c r="Y35" s="35" t="n">
         <v>51.13242321382663</v>
@@ -8652,17 +8652,17 @@
       </c>
       <c r="AX35" s="90" t="inlineStr">
         <is>
+          <t>Is It Too Late to Buy IREN Stock After Its Monster Run?</t>
+        </is>
+      </c>
+      <c r="AY35" s="90" t="inlineStr">
+        <is>
           <t>Is IREN (IREN) Cheap As Sector Selling And Mixed Views Test Its AI Buildout?</t>
         </is>
       </c>
-      <c r="AY35" s="90" t="inlineStr">
+      <c r="AZ35" s="90" t="inlineStr">
         <is>
           <t>The IREN Story Is Changing Fast. We See 82% Upside Potential</t>
-        </is>
-      </c>
-      <c r="AZ35" s="90" t="inlineStr">
-        <is>
-          <t>Neocloud Stocks Fall as Selling Extends After a Week of Research Notes: IREN Drops 4%, CoreWeave Slides 3%,...</t>
         </is>
       </c>
     </row>
@@ -8758,10 +8758,10 @@
         <v>122.8399963378906</v>
       </c>
       <c r="W36" s="73" t="n">
-        <v>96075541</v>
+        <v>96982345</v>
       </c>
       <c r="X36" s="74" t="n">
-        <v>0.909541777037646</v>
+        <v>0.9177325186148084</v>
       </c>
       <c r="Y36" s="28" t="n">
         <v>66.90009367487519</v>
@@ -8850,7 +8850,7 @@
       </c>
       <c r="AZ36" s="79" t="inlineStr">
         <is>
-          <t>ARM vs. Intel: What Revenue Growth Trends Reveal About These Artificial Intelligence Companies</t>
+          <t>Is Now the Time to Bet on Intel’s (INTC) Server CPU Comeback and AI Ambitions?</t>
         </is>
       </c>
     </row>
@@ -8946,10 +8946,10 @@
         <v>497.2999877929688</v>
       </c>
       <c r="W37" s="84" t="n">
-        <v>37897460</v>
+        <v>37985485</v>
       </c>
       <c r="X37" s="85" t="n">
-        <v>1.73848673074146</v>
+        <v>1.742172994468769</v>
       </c>
       <c r="Y37" s="35" t="n">
         <v>63.21665999043974</v>
@@ -9033,12 +9033,12 @@
       </c>
       <c r="AY37" s="90" t="inlineStr">
         <is>
-          <t>Microsoft CEO: We 'have to earn that permission' to build data centers from communities</t>
+          <t>S&amp;P 500, Dow, Nasdaq End Week Higher On Chipmaker Strength, Easing Oil Amid Signs Of Easing US-Iran Conflic...</t>
         </is>
       </c>
       <c r="AZ37" s="90" t="inlineStr">
         <is>
-          <t>Microsoft CEO Satya Nadella on AI: 'Trust is going to be the biggest issue for us'</t>
+          <t>Goldman Sachs Outweighs Microsoft in This Popular Dow ETF, and Share Price Is the Only Reason</t>
         </is>
       </c>
     </row>
@@ -9125,7 +9125,7 @@
         <v>-3</v>
       </c>
       <c r="T38" s="72" t="n">
-        <v>162.8399963378906</v>
+        <v>162.75</v>
       </c>
       <c r="U38" s="72" t="n">
         <v>162.75</v>
@@ -9134,10 +9134,10 @@
         <v>156.7805938720703</v>
       </c>
       <c r="W38" s="73" t="n">
-        <v>18224447</v>
+        <v>18304905</v>
       </c>
       <c r="X38" s="74" t="n">
-        <v>0.7351206258725775</v>
+        <v>0.7382462684366292</v>
       </c>
       <c r="Y38" s="28" t="n">
         <v>63.48646301858243</v>
@@ -9216,17 +9216,17 @@
       </c>
       <c r="AX38" s="79" t="inlineStr">
         <is>
+          <t>Strategy (MSTR) Stock Drops Despite Market Gains: Important Facts to Note</t>
+        </is>
+      </c>
+      <c r="AY38" s="79" t="inlineStr">
+        <is>
           <t>Strategy's Bitcoin Buying Struggle Has A New Fix</t>
         </is>
       </c>
-      <c r="AY38" s="79" t="inlineStr">
+      <c r="AZ38" s="79" t="inlineStr">
         <is>
           <t>Strategy Proposes Daily Dividends on Its Preferred Stock</t>
-        </is>
-      </c>
-      <c r="AZ38" s="79" t="inlineStr">
-        <is>
-          <t>MSTR, ASST Stocks Slide With Bitcoin: Strategy Proposes Daily Dividends, Matt Cole Challenges MSCI Rules</t>
         </is>
       </c>
     </row>
@@ -9322,10 +9322,10 @@
         <v>1073</v>
       </c>
       <c r="W39" s="84" t="n">
-        <v>19510574</v>
+        <v>20493572</v>
       </c>
       <c r="X39" s="85" t="n">
-        <v>0.7824928507785076</v>
+        <v>0.820300073746893</v>
       </c>
       <c r="Y39" s="35" t="n">
         <v>63.19731285863126</v>
@@ -9404,17 +9404,17 @@
       </c>
       <c r="AX39" s="90" t="inlineStr">
         <is>
-          <t>Stock Market Today: Dow Surges 450 Points On Iran Peace Hopes; Micron Rises (Live Coverage)</t>
+          <t>Dow Jones Futures: Growth Stocks Shrug Off Surging Yields; Micron, SpaceX, Tesla, Key Economic Data Due</t>
         </is>
       </c>
       <c r="AY39" s="90" t="inlineStr">
         <is>
+          <t>Stock Market Today: Dow Surges 450 Points On U.S.-Iran Peace Hopes; Micron Rises</t>
+        </is>
+      </c>
+      <c r="AZ39" s="90" t="inlineStr">
+        <is>
           <t>Micron Technology Stock Wavers Ahead Of Fiscal Q4 Earnings Report</t>
-        </is>
-      </c>
-      <c r="AZ39" s="90" t="inlineStr">
-        <is>
-          <t>Two Numbers to Watch in Micron’s Earnings Report Next Week</t>
         </is>
       </c>
     </row>
@@ -9501,7 +9501,7 @@
         <v>-6.149993896484375</v>
       </c>
       <c r="T40" s="72" t="n">
-        <v>245.6000061035156</v>
+        <v>246.8999938964844</v>
       </c>
       <c r="U40" s="72" t="n">
         <v>246.8999938964844</v>
@@ -9510,10 +9510,10 @@
         <v>235.4113006591797</v>
       </c>
       <c r="W40" s="73" t="n">
-        <v>10972739</v>
+        <v>10990560</v>
       </c>
       <c r="X40" s="74" t="n">
-        <v>0.7244768223454382</v>
+        <v>0.7256107677528069</v>
       </c>
       <c r="Y40" s="28" t="n">
         <v>55.5482522571431</v>
@@ -9698,10 +9698,10 @@
         <v>70.98000335693359</v>
       </c>
       <c r="W41" s="84" t="n">
-        <v>22320107</v>
+        <v>23135069</v>
       </c>
       <c r="X41" s="85" t="n">
-        <v>0.6890980625944936</v>
+        <v>0.7133612953784753</v>
       </c>
       <c r="Y41" s="35" t="n">
         <v>37.06722791404464</v>
@@ -9785,12 +9785,12 @@
       </c>
       <c r="AY41" s="90" t="inlineStr">
         <is>
-          <t>1 Wall Street Analyst Just Called Netflix a Sell. Is It Time To Dump the Streaming Stock?</t>
+          <t>Netflix (NFLX)’s YouTube Problem Is Becoming Harder to Dismiss</t>
         </is>
       </c>
       <c r="AZ41" s="90" t="inlineStr">
         <is>
-          <t>Netflix's Revenue Growth Has Slowed for 2 Straight Quarters. Should You Buy the Stock Anyway?</t>
+          <t>Walt Disney vs. Netflix: Which Stock Is a Better Buy in 2026?</t>
         </is>
       </c>
     </row>
@@ -9886,10 +9886,10 @@
         <v>10.31999969482422</v>
       </c>
       <c r="W42" s="73" t="n">
-        <v>44541549</v>
+        <v>44577714</v>
       </c>
       <c r="X42" s="74" t="n">
-        <v>0.51531994150577</v>
+        <v>0.5157275603937559</v>
       </c>
       <c r="Y42" s="28" t="n">
         <v>49.68891967958996</v>
@@ -10074,10 +10074,10 @@
         <v>223.1329040527344</v>
       </c>
       <c r="W43" s="84" t="n">
-        <v>87234141</v>
+        <v>87931936</v>
       </c>
       <c r="X43" s="85" t="n">
-        <v>0.752460676414398</v>
+        <v>0.7582514916900709</v>
       </c>
       <c r="Y43" s="35" t="n">
         <v>55.17408895732846</v>
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
-          <t>Trump says China's Xi 'seemed to like' renaming AI as super intelligence</t>
+          <t>This Stock May Be the Best Artificial Intelligence (AI) and Quantum Computing Investment</t>
         </is>
       </c>
       <c r="AY43" s="90" t="inlineStr">
         <is>
-          <t>Meet the Magnificent Semiconductor Stock Crushing Nvidia in 2026</t>
+          <t>Does IonQ's NVIDIA Quantum Tie-Up Reframe the Long-Term Hardware Opportunity for Rigetti Computing (RGTI)?</t>
         </is>
       </c>
       <c r="AZ43" s="90" t="inlineStr">
         <is>
-          <t>Nvidia, AMD Love This High-Tech Facilitator. So Does Wall Street.</t>
+          <t>Microsoft, Meta, Akamai, Zscaler, Comcast, and More Stocks That Explain Today’s Market</t>
         </is>
       </c>
     </row>
@@ -10262,10 +10262,10 @@
         <v>189.3500061035156</v>
       </c>
       <c r="W44" s="73" t="n">
-        <v>17578636</v>
+        <v>17677784</v>
       </c>
       <c r="X44" s="74" t="n">
-        <v>0.6670997256527352</v>
+        <v>0.6707361525838595</v>
       </c>
       <c r="Y44" s="28" t="n">
         <v>63.69582459518597</v>
@@ -10349,12 +10349,12 @@
       </c>
       <c r="AY44" s="79" t="inlineStr">
         <is>
-          <t>Why Is a Stock Down 97% This Year Paying to Appear Next to Palantir?</t>
+          <t>Commercial AI Momentum Meets Valuation Risk: What Comes Next for Palantir (PLTR)?</t>
         </is>
       </c>
       <c r="AZ44" s="79" t="inlineStr">
         <is>
-          <t>Palantir's Latest $250 Target Comes With a Catch</t>
+          <t>Palantir Co-Founder and FTC Chairman Put AI Accountability in Focus at Reuters Momentum AI Austin 2026</t>
         </is>
       </c>
     </row>
@@ -10441,7 +10441,7 @@
         <v>7.710006713867188</v>
       </c>
       <c r="T45" s="83" t="n">
-        <v>195.0299987792969</v>
+        <v>195.3999938964844</v>
       </c>
       <c r="U45" s="83" t="n">
         <v>205.8531951904297</v>
@@ -10450,10 +10450,10 @@
         <v>194.5299987792969</v>
       </c>
       <c r="W45" s="84" t="n">
-        <v>17551795</v>
+        <v>17757473</v>
       </c>
       <c r="X45" s="85" t="n">
-        <v>1.20620698741974</v>
+        <v>1.219479885595547</v>
       </c>
       <c r="Y45" s="35" t="n">
         <v>67.61919651176316</v>
@@ -10629,7 +10629,7 @@
         <v>0.339996337890625</v>
       </c>
       <c r="T46" s="72" t="n">
-        <v>74.15000152587891</v>
+        <v>74.09999847412109</v>
       </c>
       <c r="U46" s="72" t="n">
         <v>75.31999969482422</v>
@@ -10638,10 +10638,10 @@
         <v>72.78009796142578</v>
       </c>
       <c r="W46" s="73" t="n">
-        <v>18729138</v>
+        <v>18756601</v>
       </c>
       <c r="X46" s="74" t="n">
-        <v>0.9311511125016102</v>
+        <v>0.9324528253383479</v>
       </c>
       <c r="Y46" s="28" t="n">
         <v>59.41467670309203</v>
@@ -10817,7 +10817,7 @@
         <v>24.1800537109375</v>
       </c>
       <c r="T47" s="83" t="n">
-        <v>1791.93994140625</v>
+        <v>1791.800048828125</v>
       </c>
       <c r="U47" s="83" t="n">
         <v>1815.000244140625</v>
@@ -10826,10 +10826,10 @@
         <v>1742.949951171875</v>
       </c>
       <c r="W47" s="84" t="n">
-        <v>7199542</v>
+        <v>7213004</v>
       </c>
       <c r="X47" s="85" t="n">
-        <v>0.676012247905217</v>
+        <v>0.6772334810752453</v>
       </c>
       <c r="Y47" s="35" t="n">
         <v>57.32570252002956</v>
@@ -11005,7 +11005,7 @@
         <v>-5.83001708984375</v>
       </c>
       <c r="T48" s="72" t="n">
-        <v>384.6199951171875</v>
+        <v>384.8989868164062</v>
       </c>
       <c r="U48" s="72" t="n">
         <v>386.8299865722656</v>
@@ -11014,10 +11014,10 @@
         <v>367.6700134277344</v>
       </c>
       <c r="W48" s="73" t="n">
-        <v>44502151</v>
+        <v>44753533</v>
       </c>
       <c r="X48" s="74" t="n">
-        <v>1.124116222285492</v>
+        <v>1.130107284433211</v>
       </c>
       <c r="Y48" s="28" t="n">
         <v>55.31142289856894</v>
@@ -11101,12 +11101,12 @@
       </c>
       <c r="AY48" s="79" t="inlineStr">
         <is>
-          <t>Tesla Semi: Diesel's surge gives the electric truck an opening as high prices improve the math for fleets</t>
+          <t>Stock Market Today, Sept. 25: Tesla Stock Under Pressure Despite Plans to Ramp Semi Truck Production</t>
         </is>
       </c>
       <c r="AZ48" s="79" t="inlineStr">
         <is>
-          <t>Musk’s ‘Zuckerberg moment,’ mortgage rates, and Google’s space bet</t>
+          <t>Dow Jones Futures: Growth Stocks Shrug Off Surging Yields; Micron, SpaceX, Tesla, Key Economic Data Due</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 25 Sep 2026, 08:37 PM · Yahoo Finance data</t>
+          <t>Built 25 Sep 2026, 11:19 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 25 Sep 2026, 08:37 PM · Yahoo Finance data</t>
+          <t>Built 25 Sep 2026, 11:19 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 25 Sep 2026, 08:37 PM · Yahoo Finance data</t>
+          <t>Built 25 Sep 2026, 11:19 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 25 Sep 2026, 08:37 PM · Yahoo Finance data</t>
+          <t>Built 25 Sep 2026, 11:19 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -43639,7 +43639,7 @@
         <v>0.001278066354558405</v>
       </c>
       <c r="J13" s="34" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K13" s="102" t="inlineStr">
         <is>
@@ -44136,7 +44136,7 @@
       </c>
       <c r="D13" s="105" t="inlineStr">
         <is>
-          <t>Gapped up 4.0% at the open</t>
+          <t>Gapped up 3.8% at the open</t>
         </is>
       </c>
       <c r="E13" s="33" t="n">
@@ -44416,7 +44416,7 @@
       </c>
       <c r="D23" s="105" t="inlineStr">
         <is>
-          <t>Gapped up 1.5% at the open</t>
+          <t>Gapped up 1.7% at the open</t>
         </is>
       </c>
       <c r="E23" s="33" t="n">

</xml_diff>

<commit_message>
Daily workbook: 2026-09-25 23:56 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 25 Sep 2026, 11:19 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 25 Sep 2026, 11:56 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 25 Sep 2026, 11:19 PM · Yahoo Finance data</t>
+          <t>Built 25 Sep 2026, 11:56 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -6965,12 +6965,12 @@
       </c>
       <c r="AY26" s="79" t="inlineStr">
         <is>
+          <t>Let’s Take a Closer Look at Amazon’s (AMZN) Debt-Fueled AI Buildout</t>
+        </is>
+      </c>
+      <c r="AZ26" s="79" t="inlineStr">
+        <is>
           <t>Interrupted authority and written vetting rules at center of New Mexico crash lawsuit</t>
-        </is>
-      </c>
-      <c r="AZ26" s="79" t="inlineStr">
-        <is>
-          <t>Amazon Stocks Move Lower as Anthropic Commits $11.6 Billion Elsewhere</t>
         </is>
       </c>
     </row>
@@ -7712,17 +7712,17 @@
       </c>
       <c r="AX30" s="79" t="inlineStr">
         <is>
+          <t>Nvidia Would Have to Add Almost a Whole Broadcom to Reach $7 Trillion</t>
+        </is>
+      </c>
+      <c r="AY30" s="79" t="inlineStr">
+        <is>
           <t>Jim Cramer Couldn’t Believe People Didn’t Take Broadcom Inc. (AVGO)’s CEO Seriously</t>
         </is>
       </c>
-      <c r="AY30" s="79" t="inlineStr">
+      <c r="AZ30" s="79" t="inlineStr">
         <is>
           <t>Broadcom And 2 Other High Growth Stocks To Own</t>
-        </is>
-      </c>
-      <c r="AZ30" s="79" t="inlineStr">
-        <is>
-          <t>Broadcom vs. Marvell: Which Custom AI Chip Stock Has the Better Risk-Reward?</t>
         </is>
       </c>
     </row>
@@ -9033,12 +9033,12 @@
       </c>
       <c r="AY37" s="90" t="inlineStr">
         <is>
+          <t>What Is Microsoft (MSFT) Planning With Its $10 Billion Gulf Cloud And AI Push?</t>
+        </is>
+      </c>
+      <c r="AZ37" s="90" t="inlineStr">
+        <is>
           <t>S&amp;P 500, Dow, Nasdaq End Week Higher On Chipmaker Strength, Easing Oil Amid Signs Of Easing US-Iran Conflic...</t>
-        </is>
-      </c>
-      <c r="AZ37" s="90" t="inlineStr">
-        <is>
-          <t>Goldman Sachs Outweighs Microsoft in This Popular Dow ETF, and Share Price Is the Only Reason</t>
         </is>
       </c>
     </row>
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
+          <t>Nvidia Would Have to Add Almost a Whole Broadcom to Reach $7 Trillion</t>
+        </is>
+      </c>
+      <c r="AY43" s="90" t="inlineStr">
+        <is>
           <t>This Stock May Be the Best Artificial Intelligence (AI) and Quantum Computing Investment</t>
         </is>
       </c>
-      <c r="AY43" s="90" t="inlineStr">
+      <c r="AZ43" s="90" t="inlineStr">
         <is>
           <t>Does IonQ's NVIDIA Quantum Tie-Up Reframe the Long-Term Hardware Opportunity for Rigetti Computing (RGTI)?</t>
-        </is>
-      </c>
-      <c r="AZ43" s="90" t="inlineStr">
-        <is>
-          <t>Microsoft, Meta, Akamai, Zscaler, Comcast, and More Stocks That Explain Today’s Market</t>
         </is>
       </c>
     </row>
@@ -11101,12 +11101,12 @@
       </c>
       <c r="AY48" s="79" t="inlineStr">
         <is>
+          <t>Tesla (TSLA), Ford (F), and GM (GM) Face a Weaker EV Market. Who Can Protect Profits?</t>
+        </is>
+      </c>
+      <c r="AZ48" s="79" t="inlineStr">
+        <is>
           <t>Stock Market Today, Sept. 25: Tesla Stock Under Pressure Despite Plans to Ramp Semi Truck Production</t>
-        </is>
-      </c>
-      <c r="AZ48" s="79" t="inlineStr">
-        <is>
-          <t>Dow Jones Futures: Growth Stocks Shrug Off Surging Yields; Micron, SpaceX, Tesla, Key Economic Data Due</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 25 Sep 2026, 11:19 PM · Yahoo Finance data</t>
+          <t>Built 25 Sep 2026, 11:56 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 25 Sep 2026, 11:19 PM · Yahoo Finance data</t>
+          <t>Built 25 Sep 2026, 11:56 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 25 Sep 2026, 11:19 PM · Yahoo Finance data</t>
+          <t>Built 25 Sep 2026, 11:56 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 25 Sep 2026, 11:19 PM · Yahoo Finance data</t>
+          <t>Built 25 Sep 2026, 11:56 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-09-29 00:58 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 29 Sep 2026, 12:23 AM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 29 Sep 2026, 12:58 AM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 29 Sep 2026, 12:23 AM · Yahoo Finance data</t>
+          <t>Built 29 Sep 2026, 12:58 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -9404,17 +9404,17 @@
       </c>
       <c r="AX39" s="90" t="inlineStr">
         <is>
+          <t>Marvell Technology, Semtech, Lattice Semiconductor, and Micron Stocks Trade Down, What You Need To Know</t>
+        </is>
+      </c>
+      <c r="AY39" s="90" t="inlineStr">
+        <is>
           <t>Sandisk Jumped 22% the Day After Micron's Last Report. Micron Reports Again Wednesday.</t>
         </is>
       </c>
-      <c r="AY39" s="90" t="inlineStr">
+      <c r="AZ39" s="90" t="inlineStr">
         <is>
           <t>Is Micron Stock a Sell After This Weekend's Negative AI News?</t>
-        </is>
-      </c>
-      <c r="AZ39" s="90" t="inlineStr">
-        <is>
-          <t>Michael Burry Swaps MU, NBIS, NVDA, PLTR Shorts For Puts — Says AI Bubble May Burst ‘Sooner Than Later’</t>
         </is>
       </c>
     </row>
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
+          <t>Use This Zacks Tool to Find Strong AI Stocks</t>
+        </is>
+      </c>
+      <c r="AY43" s="90" t="inlineStr">
+        <is>
           <t>Nvidia’s Glass Packaging Push Could Reshape AI Chips</t>
         </is>
       </c>
-      <c r="AY43" s="90" t="inlineStr">
+      <c r="AZ43" s="90" t="inlineStr">
         <is>
           <t>Why Nvidia (NVDA) Stock Is Trading Up Today</t>
-        </is>
-      </c>
-      <c r="AZ43" s="90" t="inlineStr">
-        <is>
-          <t>Nvidia’s Latest $150 Billion Move Delivers a Clear Message to Investors About What’s Next for the Stock.</t>
         </is>
       </c>
     </row>
@@ -10720,17 +10720,17 @@
       </c>
       <c r="AX46" s="79" t="inlineStr">
         <is>
+          <t>Prediction: Rocket Lab Stock Trades Above $100 Again Before 2029</t>
+        </is>
+      </c>
+      <c r="AY46" s="79" t="inlineStr">
+        <is>
           <t>Rocket Lab (RKLB) Nails Back To Back September Launches With 100% Mission Record</t>
         </is>
       </c>
-      <c r="AY46" s="79" t="inlineStr">
+      <c r="AZ46" s="79" t="inlineStr">
         <is>
           <t>Rocket Lab Corporation (RKLB) Declines More Than Market: Some Information for Investors</t>
-        </is>
-      </c>
-      <c r="AZ46" s="79" t="inlineStr">
-        <is>
-          <t>Cathie Wood Makes $64 Million Bet on Two Stocks</t>
         </is>
       </c>
     </row>
@@ -11106,7 +11106,7 @@
       </c>
       <c r="AZ48" s="79" t="inlineStr">
         <is>
-          <t>TSLA Heads Into Friday’s Delivery Print With Family-Targeted Model Y L Already Sold Into Next Year</t>
+          <t>Dow Jones Futures: Trump Sparks Stock Market Losses; Elon Musk-Led SpaceX, Tesla In Focus</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 29 Sep 2026, 12:23 AM · Yahoo Finance data</t>
+          <t>Built 29 Sep 2026, 12:58 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 29 Sep 2026, 12:23 AM · Yahoo Finance data</t>
+          <t>Built 29 Sep 2026, 12:58 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 29 Sep 2026, 12:23 AM · Yahoo Finance data</t>
+          <t>Built 29 Sep 2026, 12:58 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 29 Sep 2026, 12:23 AM · Yahoo Finance data</t>
+          <t>Built 29 Sep 2026, 12:58 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-09-29 23:45 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 29 Sep 2026, 09:29 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 29 Sep 2026, 11:45 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 29 Sep 2026, 09:29 PM · Yahoo Finance data</t>
+          <t>Built 29 Sep 2026, 11:45 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -5811,17 +5811,17 @@
       </c>
       <c r="AX19" s="79" t="inlineStr">
         <is>
+          <t>Forget SPY’s Dividend. Here Is What $100,000 in State Street’s High-Dividend Version Pays</t>
+        </is>
+      </c>
+      <c r="AY19" s="79" t="inlineStr">
+        <is>
           <t>Exchange-Traded Funds, Equity Futures Higher Pre-Bell Tuesday as Investors Weigh Tech Rebound</t>
         </is>
       </c>
-      <c r="AY19" s="79" t="inlineStr">
-        <is>
-          <t>AMC Sinks 7%, Gives Back Part of Sharp Rally; Cinemark and IMAX Dip</t>
-        </is>
-      </c>
       <c r="AZ19" s="79" t="inlineStr">
         <is>
-          <t>September Has Been One of the S&amp;P 500’s Weakest Months. What History Says About Q4</t>
+          <t>S&amp;P 500, Dow Extend Losses From Elevated Yield Pressure — SPCX, TGT, AAPL, MU, NTAP In Focus</t>
         </is>
       </c>
     </row>
@@ -5999,17 +5999,17 @@
       </c>
       <c r="AX20" s="90" t="inlineStr">
         <is>
-          <t>Exchange-Traded Funds Lower as US Equities Drop After Midday</t>
+          <t>QQQM Charges 0.15% and QQQ Charges 0.18%. A Wide Spread Can Take That Back on a Single Trade</t>
         </is>
       </c>
       <c r="AY20" s="90" t="inlineStr">
         <is>
-          <t>The Biggest Names in Food and Social Media Come Together at the 2026 Food Network New York City Wine &amp; Food...</t>
+          <t>S&amp;P 500, Dow Extend Losses From Elevated Yield Pressure — SPCX, TGT, AAPL, MU, NTAP In Focus</t>
         </is>
       </c>
       <c r="AZ20" s="90" t="inlineStr">
         <is>
-          <t>Exchange-Traded Funds, Equity Futures Higher Pre-Bell Tuesday as Investors Weigh Tech Rebound</t>
+          <t>If You'd Invested $1,000 in the Invesco QQQ Trust (QQQ) 10 Years Ago, Here's How Much You'd Have Today</t>
         </is>
       </c>
     </row>
@@ -6589,12 +6589,12 @@
       </c>
       <c r="AY24" s="79" t="inlineStr">
         <is>
-          <t>Apple, Meta, Iovance, Carnival, Fair Isaac, Bloom Energy, SpaceX, and More Stocks That Explain Today’s Market</t>
+          <t>Apple is betting $1,999 that consumers are ready for this shift</t>
         </is>
       </c>
       <c r="AZ24" s="79" t="inlineStr">
         <is>
-          <t>Billionaire Investor: Meta’s Muse Puts Apple’s “30% Rev Share on Notice”</t>
+          <t>Own an iPhone? You could be owed money. How to claim it in Arizona</t>
         </is>
       </c>
     </row>
@@ -6772,7 +6772,7 @@
       </c>
       <c r="AX25" s="90" t="inlineStr">
         <is>
-          <t>Are Meta, AMD, and Micron to thank for the September rally?</t>
+          <t>AMD takes on Nvidia with aggressive $8.2 billion bet on AI’s next era</t>
         </is>
       </c>
       <c r="AY25" s="90" t="inlineStr">
@@ -7712,17 +7712,17 @@
       </c>
       <c r="AX30" s="79" t="inlineStr">
         <is>
+          <t>3 Dividend ETFs for a 40-Year Retirement. One Has Paid Every Quarter Since 2005</t>
+        </is>
+      </c>
+      <c r="AY30" s="79" t="inlineStr">
+        <is>
           <t>Broadcom Stock Jumps Nearly 3.2% as $16.7 Billion AI Engine Faces Margin Test</t>
         </is>
       </c>
-      <c r="AY30" s="79" t="inlineStr">
+      <c r="AZ30" s="79" t="inlineStr">
         <is>
           <t>Reflecting On Processors and Graphics Chips Stocks’ Q2 Earnings: Broadcom (NASDAQ:AVGO)</t>
-        </is>
-      </c>
-      <c r="AZ30" s="79" t="inlineStr">
-        <is>
-          <t>3 Stocks to Buy Before the End of September</t>
         </is>
       </c>
     </row>
@@ -9409,12 +9409,12 @@
       </c>
       <c r="AY39" s="90" t="inlineStr">
         <is>
-          <t>Dow Jones Futures: Stocks Dip As Yields Rise But Bloom Energy Soars; Micron, Inflation Data Due</t>
+          <t>Dow Jones Futures Rise With Micron, Inflation Data Due; Yields Pressure Stocks But Bloom Energy Soars</t>
         </is>
       </c>
       <c r="AZ39" s="90" t="inlineStr">
         <is>
-          <t>Bullish on Micron? When a 2X ETF makes sense — and when it doesn’t</t>
+          <t>Micron Technology (MU) Could Be 47% Undervalued On Its Enterprise Memory Narrative</t>
         </is>
       </c>
     </row>
@@ -9592,17 +9592,17 @@
       </c>
       <c r="AX40" s="79" t="inlineStr">
         <is>
+          <t>Innodata vs. Nebius Group N.V.: Which AI Stock Is a Better Buy in 2026?</t>
+        </is>
+      </c>
+      <c r="AY40" s="79" t="inlineStr">
+        <is>
           <t>Cerebras Systems vs. Nebius: What Revenue Growth Trends Reveal to Investors About These Artificial Intellig...</t>
         </is>
       </c>
-      <c r="AY40" s="79" t="inlineStr">
+      <c r="AZ40" s="79" t="inlineStr">
         <is>
           <t>Nebius Climbs 4% Despite Michael Burry’s Bigger Bearish Bet; CoreWeave Ticks Up, Cloudflare Slips</t>
-        </is>
-      </c>
-      <c r="AZ40" s="79" t="inlineStr">
-        <is>
-          <t>Nebius’ Strong Signal Is Going to Move Markets in the Coming Days</t>
         </is>
       </c>
     </row>
@@ -10156,12 +10156,12 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
-          <t>How Nvidia is tackling the AI safety problem</t>
+          <t>Jensen Huang: AI data center push will create 1 million US jobs</t>
         </is>
       </c>
       <c r="AY43" s="90" t="inlineStr">
         <is>
-          <t>What we know about Trump's meeting with Alex Karp, Jensen Huang, &amp; other AI leaders</t>
+          <t>Elon Musk: 'Scaling energy' is the long-term challenge with AI</t>
         </is>
       </c>
       <c r="AZ43" s="90" t="inlineStr">
@@ -10908,17 +10908,17 @@
       </c>
       <c r="AX47" s="90" t="inlineStr">
         <is>
+          <t>Is Sandisk a Millionaire-Maker Stock After Its 2026 Run?</t>
+        </is>
+      </c>
+      <c r="AY47" s="90" t="inlineStr">
+        <is>
+          <t>Sandisk to Report First Quarter Fiscal Year 2027 Results on October 29, 2026</t>
+        </is>
+      </c>
+      <c r="AZ47" s="90" t="inlineStr">
+        <is>
           <t>SanDisk Could Have a Much Bigger Opportunity Than Investors Expect</t>
-        </is>
-      </c>
-      <c r="AY47" s="90" t="inlineStr">
-        <is>
-          <t>Examine Sandisk Carefully Before You Jump in on The Buyback News</t>
-        </is>
-      </c>
-      <c r="AZ47" s="90" t="inlineStr">
-        <is>
-          <t>What Does Sandisk (SNDK) AI Data Center Momentum Mean For Its Stock?</t>
         </is>
       </c>
     </row>
@@ -11106,7 +11106,7 @@
       </c>
       <c r="AZ48" s="79" t="inlineStr">
         <is>
-          <t>How Tesla Semi could add billions to the EV maker's financials</t>
+          <t>Tesla (TSLA), What Is Drawing Fresh Attention Now?</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 29 Sep 2026, 09:29 PM · Yahoo Finance data</t>
+          <t>Built 29 Sep 2026, 11:45 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 29 Sep 2026, 09:29 PM · Yahoo Finance data</t>
+          <t>Built 29 Sep 2026, 11:45 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 29 Sep 2026, 09:29 PM · Yahoo Finance data</t>
+          <t>Built 29 Sep 2026, 11:45 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 29 Sep 2026, 09:29 PM · Yahoo Finance data</t>
+          <t>Built 29 Sep 2026, 11:45 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-09-30 23:54 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1299,7 +1299,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 30 Sep 2026, 09:29 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 30 Sep 2026, 11:54 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3104,7 +3104,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 30 Sep 2026, 09:29 PM · Yahoo Finance data</t>
+          <t>Built 30 Sep 2026, 11:54 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -5808,17 +5808,17 @@
       </c>
       <c r="AX19" s="79" t="inlineStr">
         <is>
+          <t>Forget Waiting Three Months for SPY’s Dividend. Invesco’s High-Dividend Fund Pays Every Month</t>
+        </is>
+      </c>
+      <c r="AY19" s="79" t="inlineStr">
+        <is>
+          <t>Wall Street Now Sells 11 Weekly-Pay ETFs. Only Three Have Beaten the S&amp;P. Here They Are</t>
+        </is>
+      </c>
+      <c r="AZ19" s="79" t="inlineStr">
+        <is>
           <t>Which Airline Stock Dominated in September: American, United, or Delta?</t>
-        </is>
-      </c>
-      <c r="AY19" s="79" t="inlineStr">
-        <is>
-          <t>MP Materials Surges 6% as Traders Weigh Critical Minerals Growth Story; USA Rare Earth Rises 3%, Critical M...</t>
-        </is>
-      </c>
-      <c r="AZ19" s="79" t="inlineStr">
-        <is>
-          <t>ChargePoint Jumps 7% as Electric September Run Persists; EVgo Falls 3%, Blink Charging Slips</t>
         </is>
       </c>
     </row>
@@ -6581,17 +6581,17 @@
       </c>
       <c r="AX24" s="79" t="inlineStr">
         <is>
+          <t>Mynd.ai's Promethean Brand Launches On-Device AI Companion to Help Teachers Create Lesson Content in Seconds</t>
+        </is>
+      </c>
+      <c r="AY24" s="79" t="inlineStr">
+        <is>
           <t>Apple Predicted To Sell 6 Million iPhone Duo Handsets This Year</t>
         </is>
       </c>
-      <c r="AY24" s="79" t="inlineStr">
+      <c r="AZ24" s="79" t="inlineStr">
         <is>
           <t>Top Analyst Reports for Apple, Microsoft &amp; Broadcom</t>
-        </is>
-      </c>
-      <c r="AZ24" s="79" t="inlineStr">
-        <is>
-          <t>TSMC's next move could ripple far beyond Apple, Nvidia</t>
         </is>
       </c>
     </row>
@@ -6774,12 +6774,12 @@
       </c>
       <c r="AY25" s="90" t="inlineStr">
         <is>
-          <t>Dow Jones Futures: Micron Rises On Hot Earnings After Treasury Yields Pressure Stocks</t>
+          <t>Dow Jones Futures: Micron Earnings Crush Views, S&amp;P 500 At Critical Level As Treasury Yields Rise</t>
         </is>
       </c>
       <c r="AZ25" s="90" t="inlineStr">
         <is>
-          <t>Intel Rises 3% as Chip Contender Caps Off Surprisingly Strong September; NVIDIA Ticks Up, AMD Slips</t>
+          <t>Advanced Micro Devices vs. Arm: Which Tech Stock Is a Better Buy in 2026?</t>
         </is>
       </c>
     </row>
@@ -6967,7 +6967,7 @@
       </c>
       <c r="AZ26" s="79" t="inlineStr">
         <is>
-          <t>Amazon Signs $1 Billion Synopsys Deal as AWS Steps Up Nvidia Challenge</t>
+          <t>Amazon deal with Calvert Cliffs would extend nuclear plant’s life, explore new reactors</t>
         </is>
       </c>
     </row>
@@ -7897,17 +7897,17 @@
       </c>
       <c r="AX31" s="90" t="inlineStr">
         <is>
+          <t>Cameco Acknowledges United States and Republic of Korea Announcement of Framework for the Deployment of Nuc...</t>
+        </is>
+      </c>
+      <c r="AY31" s="90" t="inlineStr">
+        <is>
           <t>Is Cameco Stock a Buy Now?</t>
         </is>
       </c>
-      <c r="AY31" s="90" t="inlineStr">
+      <c r="AZ31" s="90" t="inlineStr">
         <is>
           <t>Cameco’s Westinghouse Stake Could Be Worth More Than $24.5 Billion</t>
-        </is>
-      </c>
-      <c r="AZ31" s="90" t="inlineStr">
-        <is>
-          <t>Here's Why Cameco (CCJ) Fell More Than Broader Market</t>
         </is>
       </c>
     </row>
@@ -8466,12 +8466,12 @@
       </c>
       <c r="AY34" s="79" t="inlineStr">
         <is>
-          <t>Dow Jones Futures: Micron Rises On Hot Earnings After Treasury Yields Pressure Stocks</t>
+          <t>Dow Jones Futures: Micron Earnings Crush Views, S&amp;P 500 At Critical Level As Treasury Yields Rise</t>
         </is>
       </c>
       <c r="AZ34" s="79" t="inlineStr">
         <is>
-          <t>Google Stock Rises On Gemini 4 Argon Release After New AI Model Delays</t>
+          <t>The $30M company run with zero employees</t>
         </is>
       </c>
     </row>
@@ -9030,12 +9030,12 @@
       </c>
       <c r="AY37" s="90" t="inlineStr">
         <is>
-          <t>Dow Jones Futures: Micron Rises On Hot Earnings After Treasury Yields Pressure Stocks</t>
+          <t>Dow Jones Futures: Micron Earnings Crush Views, S&amp;P 500 At Critical Level As Treasury Yields Rise</t>
         </is>
       </c>
       <c r="AZ37" s="90" t="inlineStr">
         <is>
-          <t>Top Analyst Reports for Apple, Microsoft &amp; Broadcom</t>
+          <t>Patriot Consulting Launches Free ISOC Cost Evaluation and Agentic MXDR365 Operations for Microsoft's New In...</t>
         </is>
       </c>
     </row>
@@ -9213,17 +9213,17 @@
       </c>
       <c r="AX38" s="79" t="inlineStr">
         <is>
+          <t>Michael Saylor Wants His Bitcoin Rival to Win: What's in It for MicroStrategy?</t>
+        </is>
+      </c>
+      <c r="AY38" s="79" t="inlineStr">
+        <is>
           <t>How Daily Dividends Could Shake Up the MicroStrategy Stock Story</t>
         </is>
       </c>
-      <c r="AY38" s="79" t="inlineStr">
+      <c r="AZ38" s="79" t="inlineStr">
         <is>
           <t>Can Strategy (MSTR) Be A Bargain Based On Book Value?</t>
-        </is>
-      </c>
-      <c r="AZ38" s="79" t="inlineStr">
-        <is>
-          <t>Michael Saylor's Strategy just bought more Bitcoin, this purchase was 75% bigger</t>
         </is>
       </c>
     </row>
@@ -9406,12 +9406,12 @@
       </c>
       <c r="AY39" s="90" t="inlineStr">
         <is>
-          <t>AI spending will fuel wins for Micron, Nvidia, Intel, and other chip stocks: BofA analyst</t>
+          <t>Dow Jones Futures: Micron Earnings Crush Views, S&amp;P 500 At Critical Level As Treasury Yields Rise</t>
         </is>
       </c>
       <c r="AZ39" s="90" t="inlineStr">
         <is>
-          <t>Dow Jones Futures: Micron Rises On Hot Earnings After Treasury Yields Pressure Stocks</t>
+          <t>Micron’s Revenue More Than Quadrupled. Here’s What Comes Next for the AI Chipmaker.</t>
         </is>
       </c>
     </row>
@@ -9589,17 +9589,17 @@
       </c>
       <c r="AX40" s="79" t="inlineStr">
         <is>
+          <t>Nebius Chief Revenue Officer Liquidates Entire Directly-Held Shares for $1.5 Million</t>
+        </is>
+      </c>
+      <c r="AY40" s="79" t="inlineStr">
+        <is>
           <t>I've Changed My Mind on Nebius Stock. The AI Supercycle Has Room for More Than Just Hyperscalers.</t>
         </is>
       </c>
-      <c r="AY40" s="79" t="inlineStr">
+      <c r="AZ40" s="79" t="inlineStr">
         <is>
           <t>Stock-Split Watch: Is Nebius Next?</t>
-        </is>
-      </c>
-      <c r="AZ40" s="79" t="inlineStr">
-        <is>
-          <t>Nebius Could Stand Apart In AI Cloud, Says William Blair – Sees Valuation Understating Long-Term Earnings P...</t>
         </is>
       </c>
     </row>
@@ -9777,17 +9777,17 @@
       </c>
       <c r="AX41" s="90" t="inlineStr">
         <is>
+          <t>Wall Street bank backs Netflix despite U.S. drift to YouTube</t>
+        </is>
+      </c>
+      <c r="AY41" s="90" t="inlineStr">
+        <is>
           <t>Netflix Stock Has Turned $1,000 Into About $654,000 Since Its IPO. It Has Gone Nowhere Since 2021.</t>
         </is>
       </c>
-      <c r="AY41" s="90" t="inlineStr">
+      <c r="AZ41" s="90" t="inlineStr">
         <is>
           <t>Netflix's Content Commitments Rise: Is Cash Flow Under Pressure?</t>
-        </is>
-      </c>
-      <c r="AZ41" s="90" t="inlineStr">
-        <is>
-          <t>What You Need To Know Ahead of Netflix's Earnings Release</t>
         </is>
       </c>
     </row>
@@ -10153,17 +10153,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
-          <t>Why today's headwinds could set up a major stock rally in coming months</t>
+          <t>Nvidia, Broadcom, and AMD Investors Need to Have Oct. 15 Circled on Their Calendars</t>
         </is>
       </c>
       <c r="AY43" s="90" t="inlineStr">
         <is>
-          <t>AI spending will fuel wins for Micron, Nvidia, Intel, and other chip stocks: BofA analyst</t>
+          <t>Nvidia Stock Can Top $400 in 5 Years If One Assumption Holds Up</t>
         </is>
       </c>
       <c r="AZ43" s="90" t="inlineStr">
         <is>
-          <t>Nvidia, AMD Collaborator Teases Breakout To Record High. These Clues Bode Well.</t>
+          <t>Nvidia's record buyback exposes strange Wall Street gap</t>
         </is>
       </c>
     </row>
@@ -10717,17 +10717,17 @@
       </c>
       <c r="AX46" s="79" t="inlineStr">
         <is>
+          <t>Rocket Lab Secures Largest-Ever Electron Commercial Deal: 20-Launch Contract for Synspective</t>
+        </is>
+      </c>
+      <c r="AY46" s="79" t="inlineStr">
+        <is>
           <t>3 Space Stocks to Buy in October</t>
         </is>
       </c>
-      <c r="AY46" s="79" t="inlineStr">
+      <c r="AZ46" s="79" t="inlineStr">
         <is>
           <t>AST SpaceMobile Jumps 5% on Takeover Speculation; Rocket Lab Rises 5%, SpaceX Treads Water</t>
-        </is>
-      </c>
-      <c r="AZ46" s="79" t="inlineStr">
-        <is>
-          <t>Rocket Lab Sold Kepler a Dedicated Neutron Flight. Here's How Many More It Needs to Justify Its Valuation</t>
         </is>
       </c>
     </row>
@@ -11640,7 +11640,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 30 Sep 2026, 09:29 PM · Yahoo Finance data</t>
+          <t>Built 30 Sep 2026, 11:54 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19576,7 +19576,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 30 Sep 2026, 09:29 PM · Yahoo Finance data</t>
+          <t>Built 30 Sep 2026, 11:54 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27512,7 +27512,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 30 Sep 2026, 09:29 PM · Yahoo Finance data</t>
+          <t>Built 30 Sep 2026, 11:54 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35448,7 +35448,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 30 Sep 2026, 09:29 PM · Yahoo Finance data</t>
+          <t>Built 30 Sep 2026, 11:54 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-10-01 23:55 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 1 Oct 2026, 09:54 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 1 Oct 2026, 11:55 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 1 Oct 2026, 09:54 PM · Yahoo Finance data</t>
+          <t>Built 1 Oct 2026, 11:55 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -5811,17 +5811,17 @@
       </c>
       <c r="AX19" s="79" t="inlineStr">
         <is>
+          <t>S&amp;P 500, Nasdaq, Dow Futures Inch Higher As Investors Cheer Cooling Yields — GOOGL, MU, MAT, NVDA In Focus</t>
+        </is>
+      </c>
+      <c r="AY19" s="79" t="inlineStr">
+        <is>
           <t>Accenture Soars 23% as Record Bookings Dispel AI Demand Fears; Infosys Jumps 8%, IBM Climbs 5%</t>
         </is>
       </c>
-      <c r="AY19" s="79" t="inlineStr">
+      <c r="AZ19" s="79" t="inlineStr">
         <is>
           <t>Exchange-Traded Funds, Equity Futures up Pre-Bell Thursday as Traders Assess Micron's Fiscal Q4 Results</t>
-        </is>
-      </c>
-      <c r="AZ19" s="79" t="inlineStr">
-        <is>
-          <t>Tesla Is Down 20% in 2026. These Two Other EV Makers Are Doing Even Worse.</t>
         </is>
       </c>
     </row>
@@ -7524,17 +7524,17 @@
       </c>
       <c r="AX29" s="90" t="inlineStr">
         <is>
+          <t>AST SpaceMobile, Inc. (ASTS) Stock Sinks As Market Gains: Here's Why</t>
+        </is>
+      </c>
+      <c r="AY29" s="90" t="inlineStr">
+        <is>
           <t>Rocket Lab Climbs 5% as Largest-Ever Electron Deal Lifts Backlog Past 100 Missions; AST SpaceMobile Ticks U...</t>
         </is>
       </c>
-      <c r="AY29" s="90" t="inlineStr">
+      <c r="AZ29" s="90" t="inlineStr">
         <is>
           <t>ASTS Climbs Overnight As BlueBird Convoy Heads To Cape Canaveral, CEO Pitches Spectrum To FCC Chief</t>
-        </is>
-      </c>
-      <c r="AZ29" s="90" t="inlineStr">
-        <is>
-          <t>ASTS Stock Alert: What to Know as Takeover Speculation Swirls Around AST SpaceMobile</t>
         </is>
       </c>
     </row>
@@ -7712,17 +7712,17 @@
       </c>
       <c r="AX30" s="79" t="inlineStr">
         <is>
-          <t>Broadcom to lend Anthropic up to $42 billion to lease chips, in latest circular investing deal</t>
+          <t>Broadcom lends Anthropic $42B, Nike releases Caitlin 1s, and Micron earnings takeaways</t>
         </is>
       </c>
       <c r="AY30" s="79" t="inlineStr">
         <is>
-          <t>Broadcom lends Anthropic $42B, Nike releases Caitlin 1s, and Micron earnings takeaways</t>
+          <t>Broadcom to lend Anthropic $42 billion in finance infrastructure spending</t>
         </is>
       </c>
       <c r="AZ30" s="79" t="inlineStr">
         <is>
-          <t>Broadcom to lend Anthropic $42 billion in finance infrastructure spending</t>
+          <t>Anthropic and Broadcom Are Becoming More Intertwined. What It Means for Broadcom Stock.</t>
         </is>
       </c>
     </row>
@@ -7900,17 +7900,17 @@
       </c>
       <c r="AX31" s="90" t="inlineStr">
         <is>
+          <t>Forget URA’s Concentration. This Nuclear Fund Spreads the Bet Across Utilities, Miners and Reactor Builders</t>
+        </is>
+      </c>
+      <c r="AY31" s="90" t="inlineStr">
+        <is>
           <t>Cameco Stock Slips Even as a $120 Billion U.S. Reactor Framework Takes Shape</t>
         </is>
       </c>
-      <c r="AY31" s="90" t="inlineStr">
+      <c r="AZ31" s="90" t="inlineStr">
         <is>
           <t>Cameco Acknowledges United States and Republic of Korea Announcement of Framework for the Deployment of Nuc...</t>
-        </is>
-      </c>
-      <c r="AZ31" s="90" t="inlineStr">
-        <is>
-          <t>Is Cameco Stock a Buy Now?</t>
         </is>
       </c>
     </row>
@@ -8464,17 +8464,17 @@
       </c>
       <c r="AX34" s="79" t="inlineStr">
         <is>
+          <t>Planet Launches Suncatcher, Tanager-2, and 18 SuperDove Satellites</t>
+        </is>
+      </c>
+      <c r="AY34" s="79" t="inlineStr">
+        <is>
           <t>BAG Ventures Closes $11.3M Fund With Support From Google, Amazon, And More</t>
         </is>
       </c>
-      <c r="AY34" s="79" t="inlineStr">
+      <c r="AZ34" s="79" t="inlineStr">
         <is>
           <t>How Much Must Google Cloud Be Worth to Justify Alphabet’s Valuation?</t>
-        </is>
-      </c>
-      <c r="AZ34" s="79" t="inlineStr">
-        <is>
-          <t>Zuckerberg’s Free AI Agent Hit 5 Million Downloads And Google Still Has Its Own Locked Behind A Paywall</t>
         </is>
       </c>
     </row>
@@ -8840,17 +8840,17 @@
       </c>
       <c r="AX36" s="79" t="inlineStr">
         <is>
+          <t>Intel vs. Taiwan Semiconductor Manufacturing: Which Technology Stock Is a Better Buy in 2026?</t>
+        </is>
+      </c>
+      <c r="AY36" s="79" t="inlineStr">
+        <is>
           <t>Intel (INTC) Rides AI Optimism But Is It Already Fully Valued</t>
         </is>
       </c>
-      <c r="AY36" s="79" t="inlineStr">
+      <c r="AZ36" s="79" t="inlineStr">
         <is>
           <t>3 Top AI Stocks for October</t>
-        </is>
-      </c>
-      <c r="AZ36" s="79" t="inlineStr">
-        <is>
-          <t>Not Intel. Not Nvidia. These 2 Chip Stocks Maintain an Unbreachable Moat in Advanced Chip Tech.</t>
         </is>
       </c>
     </row>
@@ -9404,12 +9404,12 @@
       </c>
       <c r="AX39" s="90" t="inlineStr">
         <is>
-          <t>Should Apple join the consumer AI agent race? And should Big Tech self-police on AI?</t>
+          <t>Dow Jones Futures: Stocks Rise Off Support As Yields Tumble, Micron, Meta In Focus; Tesla, Jobs Report Due</t>
         </is>
       </c>
       <c r="AY39" s="90" t="inlineStr">
         <is>
-          <t>Dow Jones Futures: Stocks Rise Off Support As Yields Tumble, Micron, Meta In Focus; Tesla, Jobs Report Due</t>
+          <t>S&amp;P 500, Nasdaq, Dow Futures Inch Higher As Investors Cheer Cooling Yields — GOOGL, MU, MAT, NVDA In Focus</t>
         </is>
       </c>
       <c r="AZ39" s="90" t="inlineStr">
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
-          <t>Michael Burry Warns Nvidia, AI Infrastructure Expansion Mirroring 1960s Computer Leasing Bubble</t>
+          <t>SpaceX's Terafab Will Be Bigger Than Any Building on Earth. Here's When Investors Will Profit.</t>
         </is>
       </c>
       <c r="AY43" s="90" t="inlineStr">
         <is>
-          <t>Better Quantum Computing Stock: IonQ vs. D-Wave</t>
+          <t>Prediction: Taiwan Semiconductor Manufacturing Stock Will Skyrocket After Oct. 15</t>
         </is>
       </c>
       <c r="AZ43" s="90" t="inlineStr">
         <is>
-          <t>Acuity Brands, Inc. Q4 2026 Earnings Call Summary</t>
+          <t>What Is the Worst-Performing "Magnificent Seven" Stock in 2026?</t>
         </is>
       </c>
     </row>
@@ -10720,17 +10720,17 @@
       </c>
       <c r="AX46" s="79" t="inlineStr">
         <is>
+          <t>Intuitive Machines vs. Rocket Lab: Which Space Stock Can Send Your Returns Into Orbit in 2026?</t>
+        </is>
+      </c>
+      <c r="AY46" s="79" t="inlineStr">
+        <is>
           <t>Elon Musk Lowers Starship Expectations, Rocket Lab Surges On Electron Deal</t>
         </is>
       </c>
-      <c r="AY46" s="79" t="inlineStr">
-        <is>
-          <t>Rocket Lab Stock Rises on Record Electron Launch Deal and Citi Buy Rating</t>
-        </is>
-      </c>
       <c r="AZ46" s="79" t="inlineStr">
         <is>
-          <t>Rocket Lab (RKLB) Stock Fair Value Edges Lower As Neutron And Deal Risks Weigh</t>
+          <t>Citi Just Upgraded Rocket Lab Stock. Here's Why.</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 1 Oct 2026, 09:54 PM · Yahoo Finance data</t>
+          <t>Built 1 Oct 2026, 11:55 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 1 Oct 2026, 09:54 PM · Yahoo Finance data</t>
+          <t>Built 1 Oct 2026, 11:55 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 1 Oct 2026, 09:54 PM · Yahoo Finance data</t>
+          <t>Built 1 Oct 2026, 11:55 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 1 Oct 2026, 09:54 PM · Yahoo Finance data</t>
+          <t>Built 1 Oct 2026, 11:55 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-10-02 23:49 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 2 Oct 2026, 09:24 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 2 Oct 2026, 11:49 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 2 Oct 2026, 09:24 PM · Yahoo Finance data</t>
+          <t>Built 2 Oct 2026, 11:49 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -6584,17 +6584,17 @@
       </c>
       <c r="AX24" s="79" t="inlineStr">
         <is>
+          <t>Apple Says Some AT&amp;T iPhone 18 Pro Max Users Must Replace Phones After Service-Loss Bug</t>
+        </is>
+      </c>
+      <c r="AY24" s="79" t="inlineStr">
+        <is>
           <t>Jefferies Sees Signs of Softer iPhone 18 Demand in Resale Pricing</t>
         </is>
       </c>
-      <c r="AY24" s="79" t="inlineStr">
+      <c r="AZ24" s="79" t="inlineStr">
         <is>
           <t>How Much Upside Is Left In Apple Stock?</t>
-        </is>
-      </c>
-      <c r="AZ24" s="79" t="inlineStr">
-        <is>
-          <t>How to Pretend to Understand Muse and Other ‘Persistent Agents’</t>
         </is>
       </c>
     </row>
@@ -6960,17 +6960,17 @@
       </c>
       <c r="AX26" s="79" t="inlineStr">
         <is>
+          <t>Should You Buy Amazon Stock (AMZN) in October?</t>
+        </is>
+      </c>
+      <c r="AY26" s="79" t="inlineStr">
+        <is>
           <t>What Are Amazon Investors Paying for AWS Without Investment Gains?</t>
         </is>
       </c>
-      <c r="AY26" s="79" t="inlineStr">
+      <c r="AZ26" s="79" t="inlineStr">
         <is>
           <t>How Much Could Better Retail Margins Add to Amazon’s Value?</t>
-        </is>
-      </c>
-      <c r="AZ26" s="79" t="inlineStr">
-        <is>
-          <t>More Amazon Prime settlement payments are on the way. Who qualifies?</t>
         </is>
       </c>
     </row>
@@ -8469,12 +8469,12 @@
       </c>
       <c r="AY34" s="79" t="inlineStr">
         <is>
+          <t>HigherVisibility Analysis: Google's AI Fact-Check Rule Now Covers Metadata</t>
+        </is>
+      </c>
+      <c r="AZ34" s="79" t="inlineStr">
+        <is>
           <t>SPCX Stock Climbs As Three Thursday Launches Meet Start Of Google’s $920 Million AI Pact</t>
-        </is>
-      </c>
-      <c r="AZ34" s="79" t="inlineStr">
-        <is>
-          <t>I Sold NVIDIA, Google and Microsoft Over a $2 Trillion AI Gap. Was I Wrong?</t>
         </is>
       </c>
     </row>
@@ -9409,12 +9409,12 @@
       </c>
       <c r="AY39" s="90" t="inlineStr">
         <is>
+          <t>Micron's Last 5 Post-Earnings Dips Turned Into Gains. This Time, the Stock Rose Instead.</t>
+        </is>
+      </c>
+      <c r="AZ39" s="90" t="inlineStr">
+        <is>
           <t>US Equity Indexes Closed Mixed This Week as Treasury Yields Traded Close to Two-Decade High While October R...</t>
-        </is>
-      </c>
-      <c r="AZ39" s="90" t="inlineStr">
-        <is>
-          <t>Micron just sent a stark memory chip warning to tech stock investors</t>
         </is>
       </c>
     </row>
@@ -9592,17 +9592,17 @@
       </c>
       <c r="AX40" s="79" t="inlineStr">
         <is>
+          <t>Nebius Group (NBIS) Stock Fair Value Falls As Analyst Views Split On AI Growth</t>
+        </is>
+      </c>
+      <c r="AY40" s="79" t="inlineStr">
+        <is>
           <t>This AI Infrastructure Stock Is Up 177% in 2026, and It Is Significantly Cheaper Than Nebius</t>
         </is>
       </c>
-      <c r="AY40" s="79" t="inlineStr">
+      <c r="AZ40" s="79" t="inlineStr">
         <is>
           <t>The Bull Case For Nebius Group (NBIS) Could Change Following Inferize Deal And New AI Capacity Commitments</t>
-        </is>
-      </c>
-      <c r="AZ40" s="79" t="inlineStr">
-        <is>
-          <t>Nvidia-Backed Nebius Acquires Inferize To Reduce Idle GPU Costs Across AI Inference Workloads</t>
         </is>
       </c>
     </row>
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
+          <t>Nvidia Stock Is Back at Its May Record. Its Quarterly Revenue Is 41% Higher.</t>
+        </is>
+      </c>
+      <c r="AY43" s="90" t="inlineStr">
+        <is>
+          <t>The Copper Shortage Is Real, and It Is the Metal AI Can't Live Without. Here's the Best Way to Invest.</t>
+        </is>
+      </c>
+      <c r="AZ43" s="90" t="inlineStr">
+        <is>
           <t>Stock Market Today: Nasdaq Leads Charge On Rate Hopes; Nvidia Hits Highs</t>
-        </is>
-      </c>
-      <c r="AY43" s="90" t="inlineStr">
-        <is>
-          <t>Dow Jones Futures: Nasdaq Hits High As Nvidia, SpaceX, Bloom Energy Flash Buy Signals. What To Do Now.</t>
-        </is>
-      </c>
-      <c r="AZ43" s="90" t="inlineStr">
-        <is>
-          <t>Paramount and Warner Bros. Discovery to Merge Into Skydance (SKYD). Will Skydance Achieve David Ellison’s “...</t>
         </is>
       </c>
     </row>
@@ -10537,12 +10537,12 @@
       </c>
       <c r="AY45" s="90" t="inlineStr">
         <is>
+          <t>Why Qualcomm (QCOM) Outpaced the Stock Market Today</t>
+        </is>
+      </c>
+      <c r="AZ45" s="90" t="inlineStr">
+        <is>
           <t>Investors Heavily Search QUALCOMM Incorporated (QCOM): Here is What You Need to Know</t>
-        </is>
-      </c>
-      <c r="AZ45" s="90" t="inlineStr">
-        <is>
-          <t>Qualcomm (QCOM): Can Its AI Strategy Overcome Skepticism Around Its Current Market Position?</t>
         </is>
       </c>
     </row>
@@ -11096,17 +11096,17 @@
       </c>
       <c r="AX48" s="79" t="inlineStr">
         <is>
+          <t>Stock Market Today, Oct. 2: Tesla Rises on Q3 Delivery Beat</t>
+        </is>
+      </c>
+      <c r="AY48" s="79" t="inlineStr">
+        <is>
           <t>Nvidia, Tesla, Rivian, On Semi, Seagate, HPE, Nike, and More Stocks That Explain Today’s Market</t>
         </is>
       </c>
-      <c r="AY48" s="79" t="inlineStr">
+      <c r="AZ48" s="79" t="inlineStr">
         <is>
           <t>Tesla Just Lined Up $30 Billion in Credit: What It Means for AI, Capex, and the Investment Case</t>
-        </is>
-      </c>
-      <c r="AZ48" s="79" t="inlineStr">
-        <is>
-          <t>Sector Update: Consumer Stocks Rise Late Afternoon</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 2 Oct 2026, 09:24 PM · Yahoo Finance data</t>
+          <t>Built 2 Oct 2026, 11:49 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 2 Oct 2026, 09:24 PM · Yahoo Finance data</t>
+          <t>Built 2 Oct 2026, 11:49 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 2 Oct 2026, 09:24 PM · Yahoo Finance data</t>
+          <t>Built 2 Oct 2026, 11:49 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 2 Oct 2026, 09:24 PM · Yahoo Finance data</t>
+          <t>Built 2 Oct 2026, 11:49 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-10-06 23:51 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -28,7 +28,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'10-01'!$5:$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'09-30'!$A$6:$AZ$48</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'09-30'!$5:$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Signals'!$B$5:$G$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Signals'!$B$5:$G$49</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 6 Oct 2026, 09:47 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 6 Oct 2026, 11:51 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -1369,7 +1369,7 @@
     <row r="8" ht="32" customHeight="1">
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>32</t>
         </is>
       </c>
       <c r="C8" s="6" t="n"/>
@@ -1383,28 +1383,28 @@
       <c r="G8" s="8" t="n"/>
       <c r="H8" s="13" t="inlineStr">
         <is>
-          <t>79%</t>
+          <t>80%</t>
         </is>
       </c>
       <c r="I8" s="6" t="n"/>
       <c r="J8" s="6" t="n"/>
       <c r="K8" s="15" t="inlineStr">
         <is>
-          <t>5.9</t>
+          <t>6.0</t>
         </is>
       </c>
       <c r="L8" s="10" t="n"/>
       <c r="M8" s="10" t="n"/>
       <c r="N8" s="15" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="O8" s="10" t="n"/>
       <c r="P8" s="10" t="n"/>
       <c r="Q8" s="16" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>44</t>
         </is>
       </c>
       <c r="R8" s="12" t="n"/>
@@ -1413,14 +1413,14 @@
     <row r="9" ht="15" customHeight="1">
       <c r="B9" s="17" t="inlineStr">
         <is>
-          <t>of 39 names</t>
+          <t>of 40 names</t>
         </is>
       </c>
       <c r="C9" s="6" t="n"/>
       <c r="D9" s="6" t="n"/>
       <c r="E9" s="18" t="inlineStr">
         <is>
-          <t>of 39 names</t>
+          <t>of 40 names</t>
         </is>
       </c>
       <c r="F9" s="8" t="n"/>
@@ -1441,7 +1441,7 @@
       <c r="M9" s="10" t="n"/>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>of 39 names</t>
+          <t>of 40 names</t>
         </is>
       </c>
       <c r="O9" s="10" t="n"/>
@@ -2037,11 +2037,11 @@
       </c>
       <c r="H31" s="24" t="inlineStr">
         <is>
-          <t>SNDK</t>
+          <t>IWM</t>
         </is>
       </c>
       <c r="I31" s="26" t="n">
-        <v>-0.02564317456442577</v>
+        <v>-0.007198844342477528</v>
       </c>
       <c r="J31" s="27" t="n">
         <v>2</v>
@@ -2052,7 +2052,7 @@
         </is>
       </c>
       <c r="L31" s="28" t="n">
-        <v>48.72377558873259</v>
+        <v>40.4971772462138</v>
       </c>
     </row>
     <row r="32">
@@ -2077,11 +2077,11 @@
       </c>
       <c r="H32" s="31" t="inlineStr">
         <is>
-          <t>IWM</t>
+          <t>XLV</t>
         </is>
       </c>
       <c r="I32" s="33" t="n">
-        <v>-0.007198844342477528</v>
+        <v>-0.001672932947753392</v>
       </c>
       <c r="J32" s="34" t="n">
         <v>2</v>
@@ -2092,7 +2092,7 @@
         </is>
       </c>
       <c r="L32" s="35" t="n">
-        <v>40.4971772462138</v>
+        <v>44.92808228521599</v>
       </c>
     </row>
     <row r="33">
@@ -2117,11 +2117,11 @@
       </c>
       <c r="H33" s="24" t="inlineStr">
         <is>
-          <t>XLV</t>
+          <t>XLC</t>
         </is>
       </c>
       <c r="I33" s="26" t="n">
-        <v>-0.001672932947753392</v>
+        <v>0.0003583990261499803</v>
       </c>
       <c r="J33" s="27" t="n">
         <v>2</v>
@@ -2132,7 +2132,7 @@
         </is>
       </c>
       <c r="L33" s="28" t="n">
-        <v>44.92808228521599</v>
+        <v>49.16525991657925</v>
       </c>
     </row>
     <row r="34">
@@ -2157,11 +2157,11 @@
       </c>
       <c r="H34" s="31" t="inlineStr">
         <is>
-          <t>XLC</t>
+          <t>XLF</t>
         </is>
       </c>
       <c r="I34" s="33" t="n">
-        <v>0.0003583990261499803</v>
+        <v>0.002412718092815735</v>
       </c>
       <c r="J34" s="34" t="n">
         <v>2</v>
@@ -2172,7 +2172,7 @@
         </is>
       </c>
       <c r="L34" s="35" t="n">
-        <v>49.16525991657925</v>
+        <v>34.07886570787851</v>
       </c>
     </row>
     <row r="35">
@@ -2197,11 +2197,11 @@
       </c>
       <c r="H35" s="24" t="inlineStr">
         <is>
-          <t>XLF</t>
+          <t>IREN</t>
         </is>
       </c>
       <c r="I35" s="26" t="n">
-        <v>0.002412718092815735</v>
+        <v>0.01976282722596956</v>
       </c>
       <c r="J35" s="27" t="n">
         <v>2</v>
@@ -2212,7 +2212,7 @@
         </is>
       </c>
       <c r="L35" s="28" t="n">
-        <v>34.07886570787851</v>
+        <v>46.18333312452347</v>
       </c>
     </row>
     <row r="36">
@@ -2237,14 +2237,14 @@
       </c>
       <c r="H36" s="31" t="inlineStr">
         <is>
-          <t>IREN</t>
+          <t>SNDK</t>
         </is>
       </c>
       <c r="I36" s="33" t="n">
-        <v>0.01976282722596956</v>
+        <v>-0.02564317456442577</v>
       </c>
       <c r="J36" s="34" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K36" s="30" t="inlineStr">
         <is>
@@ -2252,7 +2252,7 @@
         </is>
       </c>
       <c r="L36" s="35" t="n">
-        <v>46.18333312452347</v>
+        <v>48.72377558873259</v>
       </c>
     </row>
     <row r="37">
@@ -2468,7 +2468,7 @@
         <v>-0.02564317456442577</v>
       </c>
       <c r="J44" s="34" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K44" s="30" t="inlineStr">
         <is>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 6 Oct 2026, 09:47 PM · Yahoo Finance data</t>
+          <t>Built 6 Oct 2026, 11:51 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -3132,22 +3132,22 @@
       </c>
       <c r="Y3" s="44" t="inlineStr">
         <is>
-          <t>31 of 39</t>
+          <t>32 of 40</t>
         </is>
       </c>
       <c r="AA3" s="45" t="inlineStr">
         <is>
-          <t>8 of 39</t>
+          <t>8 of 40</t>
         </is>
       </c>
       <c r="AC3" s="46" t="inlineStr">
         <is>
-          <t>5.9 / 9</t>
+          <t>6.0 / 9</t>
         </is>
       </c>
       <c r="AE3" s="47" t="inlineStr">
         <is>
-          <t>25 of 39</t>
+          <t>26 of 40</t>
         </is>
       </c>
     </row>
@@ -3620,10 +3620,10 @@
         <v>170.2599945068359</v>
       </c>
       <c r="W7" s="73" t="n">
-        <v>5730436</v>
+        <v>5846368</v>
       </c>
       <c r="X7" s="74" t="n">
-        <v>0.7712677592424697</v>
+        <v>0.7862577996140881</v>
       </c>
       <c r="Y7" s="28" t="n">
         <v>49.39410836699721</v>
@@ -3810,10 +3810,10 @@
         <v>165.8200073242188</v>
       </c>
       <c r="W8" s="84" t="n">
-        <v>7334206</v>
+        <v>7339458</v>
       </c>
       <c r="X8" s="85" t="n">
-        <v>0.9181207624875156</v>
+        <v>0.9187480234975016</v>
       </c>
       <c r="Y8" s="35" t="n">
         <v>44.92808228521599</v>
@@ -4000,10 +4000,10 @@
         <v>53.88000106811523</v>
       </c>
       <c r="W9" s="73" t="n">
-        <v>21644486</v>
+        <v>21721482</v>
       </c>
       <c r="X9" s="74" t="n">
-        <v>0.5800568896967935</v>
+        <v>0.5820602756733966</v>
       </c>
       <c r="Y9" s="28" t="n">
         <v>34.07886570787851</v>
@@ -4190,10 +4190,10 @@
         <v>62.93000030517578</v>
       </c>
       <c r="W10" s="84" t="n">
-        <v>25864195</v>
+        <v>27825597</v>
       </c>
       <c r="X10" s="85" t="n">
-        <v>0.745620376362049</v>
+        <v>0.7999027523103013</v>
       </c>
       <c r="Y10" s="35" t="n">
         <v>55.85599293509511</v>
@@ -4380,10 +4380,10 @@
         <v>81.02999877929688</v>
       </c>
       <c r="W11" s="73" t="n">
-        <v>12020078</v>
+        <v>12023395</v>
       </c>
       <c r="X11" s="74" t="n">
-        <v>1.098957570538379</v>
+        <v>1.099244165325627</v>
       </c>
       <c r="Y11" s="28" t="n">
         <v>43.88948885873197</v>
@@ -4570,10 +4570,10 @@
         <v>110.6500015258789</v>
       </c>
       <c r="W12" s="84" t="n">
-        <v>5896631</v>
+        <v>5896683</v>
       </c>
       <c r="X12" s="85" t="n">
-        <v>0.8760263377302074</v>
+        <v>0.8760337246694887</v>
       </c>
       <c r="Y12" s="35" t="n">
         <v>49.27062209355519</v>
@@ -4760,10 +4760,10 @@
         <v>111.0699996948242</v>
       </c>
       <c r="W13" s="73" t="n">
-        <v>5807159</v>
+        <v>5814099</v>
       </c>
       <c r="X13" s="74" t="n">
-        <v>0.9490019079939651</v>
+        <v>0.9500821621606252</v>
       </c>
       <c r="Y13" s="28" t="n">
         <v>49.16525991657925</v>
@@ -4950,10 +4950,10 @@
         <v>49.44499969482422</v>
       </c>
       <c r="W14" s="84" t="n">
-        <v>12917689</v>
+        <v>12921980</v>
       </c>
       <c r="X14" s="85" t="n">
-        <v>1.091258411368361</v>
+        <v>1.091601120797821</v>
       </c>
       <c r="Y14" s="35" t="n">
         <v>44.1974046121752</v>
@@ -5140,10 +5140,10 @@
         <v>201.8699951171875</v>
       </c>
       <c r="W15" s="73" t="n">
-        <v>6120023</v>
+        <v>6124005</v>
       </c>
       <c r="X15" s="74" t="n">
-        <v>0.8382908565624466</v>
+        <v>0.8388134155659276</v>
       </c>
       <c r="Y15" s="28" t="n">
         <v>71.578365200105</v>
@@ -5330,10 +5330,10 @@
         <v>40.7400016784668</v>
       </c>
       <c r="W16" s="84" t="n">
-        <v>7355121</v>
+        <v>7384955</v>
       </c>
       <c r="X16" s="85" t="n">
-        <v>1.169731526221423</v>
+        <v>1.174197656193388</v>
       </c>
       <c r="Y16" s="35" t="n">
         <v>30.5775918915937</v>
@@ -5520,10 +5520,10 @@
         <v>40.40999984741211</v>
       </c>
       <c r="W17" s="73" t="n">
-        <v>51897785</v>
+        <v>52063230</v>
       </c>
       <c r="X17" s="74" t="n">
-        <v>1.610573578202585</v>
+        <v>1.615293253328431</v>
       </c>
       <c r="Y17" s="28" t="n">
         <v>50.68515236988998</v>
@@ -5729,10 +5729,10 @@
         <v>777.9600219726562</v>
       </c>
       <c r="W19" s="73" t="n">
-        <v>35461764</v>
+        <v>36017885</v>
       </c>
       <c r="X19" s="74" t="n">
-        <v>0.7688621013640179</v>
+        <v>0.7804490919452431</v>
       </c>
       <c r="Y19" s="28" t="n">
         <v>62.00057962316311</v>
@@ -5845,7 +5845,7 @@
       </c>
       <c r="F20" s="30" t="inlineStr">
         <is>
-          <t>Same</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G20" s="30" t="inlineStr">
@@ -5917,10 +5917,10 @@
         <v>759.0999755859375</v>
       </c>
       <c r="W20" s="84" t="n">
-        <v>26242293</v>
+        <v>26482253</v>
       </c>
       <c r="X20" s="85" t="n">
-        <v>0.7854957379931203</v>
+        <v>0.7923937533129014</v>
       </c>
       <c r="Y20" s="35" t="n">
         <v>69.93257050295246</v>
@@ -6105,10 +6105,10 @@
         <v>280.760009765625</v>
       </c>
       <c r="W21" s="73" t="n">
-        <v>21673253</v>
+        <v>21803061</v>
       </c>
       <c r="X21" s="74" t="n">
-        <v>0.8678443888565941</v>
+        <v>0.8728153489035568</v>
       </c>
       <c r="Y21" s="28" t="n">
         <v>40.4971772462138</v>
@@ -6293,10 +6293,10 @@
         <v>163.4199981689453</v>
       </c>
       <c r="W22" s="84" t="n">
-        <v>44283353</v>
+        <v>44634151</v>
       </c>
       <c r="X22" s="85" t="n">
-        <v>0.745939875415895</v>
+        <v>0.7516268916524619</v>
       </c>
       <c r="Y22" s="35" t="n">
         <v>65.32555246622047</v>
@@ -6421,7 +6421,7 @@
         <v>0.002222927098478822</v>
       </c>
       <c r="D24" s="27" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E24" s="23" t="inlineStr">
         <is>
@@ -6502,10 +6502,10 @@
         <v>330.6199951171875</v>
       </c>
       <c r="W24" s="73" t="n">
-        <v>29565965</v>
+        <v>30438844</v>
       </c>
       <c r="X24" s="74" t="n">
-        <v>0.7093561107147947</v>
+        <v>0.729534593514634</v>
       </c>
       <c r="Y24" s="28" t="n">
         <v>54.55918363854356</v>
@@ -6584,17 +6584,17 @@
       </c>
       <c r="AX24" s="79" t="inlineStr">
         <is>
+          <t>Apple Reportedly Partners With LG Electronics To Enter Smart Home Device Market</t>
+        </is>
+      </c>
+      <c r="AY24" s="79" t="inlineStr">
+        <is>
+          <t>XLK Does Not Own Alphabet, Amazon, Meta, Netflix or Tesla. Three Stocks Are 35.87% of It</t>
+        </is>
+      </c>
+      <c r="AZ24" s="79" t="inlineStr">
+        <is>
           <t>Scott Galloway: “Apple Wins by Showing Up Late” in AI, and Its New Home Hub Is the Test</t>
-        </is>
-      </c>
-      <c r="AY24" s="79" t="inlineStr">
-        <is>
-          <t>Apple's Market Value Grew From $350 Billion to $4.75 Trillion During Tim Cook's 15 Years as CEO. Here's Wha...</t>
-        </is>
-      </c>
-      <c r="AZ24" s="79" t="inlineStr">
-        <is>
-          <t>The Magnificent Seven's Combined Value Nears $25 Trillion</t>
         </is>
       </c>
     </row>
@@ -6690,10 +6690,10 @@
         <v>628</v>
       </c>
       <c r="W25" s="84" t="n">
-        <v>24147205</v>
+        <v>24224687</v>
       </c>
       <c r="X25" s="85" t="n">
-        <v>1.087477284321567</v>
+        <v>1.090776402318854</v>
       </c>
       <c r="Y25" s="35" t="n">
         <v>72.15736583910612</v>
@@ -6777,12 +6777,12 @@
       </c>
       <c r="AY25" s="90" t="inlineStr">
         <is>
+          <t>Why Advanced Micro Devices (AMD) Outpaced the Stock Market Today</t>
+        </is>
+      </c>
+      <c r="AZ25" s="90" t="inlineStr">
+        <is>
           <t>AMD Rallies On Bullish Takes For AI Hardware Sales</t>
-        </is>
-      </c>
-      <c r="AZ25" s="90" t="inlineStr">
-        <is>
-          <t>AMD to Report Fiscal Third Quarter 2026 Financial Results</t>
         </is>
       </c>
     </row>
@@ -6878,10 +6878,10 @@
         <v>251.0800018310547</v>
       </c>
       <c r="W26" s="73" t="n">
-        <v>32758669</v>
+        <v>34067715</v>
       </c>
       <c r="X26" s="74" t="n">
-        <v>0.9156606383490937</v>
+        <v>0.9505117410058717</v>
       </c>
       <c r="Y26" s="28" t="n">
         <v>54.52229902057779</v>
@@ -6965,12 +6965,12 @@
       </c>
       <c r="AY26" s="79" t="inlineStr">
         <is>
-          <t>Pinterest swipes Amazon exec for CFO</t>
+          <t>Amazon (AMZN) Surpasses Market Returns: Some Facts Worth Knowing</t>
         </is>
       </c>
       <c r="AZ26" s="79" t="inlineStr">
         <is>
-          <t>Better Cloud Investment: Amazon or Nebius Group?</t>
+          <t>She Quit Her 6-Figure Amazon Job at 5 Months Pregnant to Launch Her Own Business: ‘Massive Opportunity Ahea...</t>
         </is>
       </c>
     </row>
@@ -6985,7 +6985,7 @@
         <v>-0.02468205373633114</v>
       </c>
       <c r="D27" s="34" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E27" s="30" t="inlineStr">
         <is>
@@ -7066,10 +7066,10 @@
         <v>90.26999664306641</v>
       </c>
       <c r="W27" s="84" t="n">
-        <v>4769117</v>
+        <v>4769498</v>
       </c>
       <c r="X27" s="85" t="n">
-        <v>1.042447980274894</v>
+        <v>1.042526919315377</v>
       </c>
       <c r="Y27" s="35" t="n">
         <v>57.45099815016937</v>
@@ -7173,7 +7173,7 @@
         <v>-0.001122470600005365</v>
       </c>
       <c r="D28" s="27" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E28" s="23" t="inlineStr">
         <is>
@@ -7254,10 +7254,10 @@
         <v>301.0700073242188</v>
       </c>
       <c r="W28" s="73" t="n">
-        <v>3384633</v>
+        <v>3395305</v>
       </c>
       <c r="X28" s="74" t="n">
-        <v>0.5829431475021669</v>
+        <v>0.58472747237314</v>
       </c>
       <c r="Y28" s="28" t="n">
         <v>56.65331032664491</v>
@@ -7442,10 +7442,10 @@
         <v>60.06399917602539</v>
       </c>
       <c r="W29" s="84" t="n">
-        <v>17536845</v>
+        <v>17587380</v>
       </c>
       <c r="X29" s="85" t="n">
-        <v>1.676055116102631</v>
+        <v>1.68047909675173</v>
       </c>
       <c r="Y29" s="35" t="n">
         <v>53.75819025328347</v>
@@ -7630,10 +7630,10 @@
         <v>364.010009765625</v>
       </c>
       <c r="W30" s="73" t="n">
-        <v>30710804</v>
+        <v>30811427</v>
       </c>
       <c r="X30" s="74" t="n">
-        <v>1.254459423184676</v>
+        <v>1.258311025364968</v>
       </c>
       <c r="Y30" s="28" t="n">
         <v>58.83882486173181</v>
@@ -7818,10 +7818,10 @@
         <v>89.40000152587891</v>
       </c>
       <c r="W31" s="84" t="n">
-        <v>5972023</v>
+        <v>6053875</v>
       </c>
       <c r="X31" s="85" t="n">
-        <v>1.893019064216636</v>
+        <v>1.916478406130705</v>
       </c>
       <c r="Y31" s="35" t="n">
         <v>52.43504338294215</v>
@@ -8006,10 +8006,10 @@
         <v>88.59999847412109</v>
       </c>
       <c r="W32" s="73" t="n">
-        <v>31927260</v>
+        <v>32015876</v>
       </c>
       <c r="X32" s="74" t="n">
-        <v>1.078085407224731</v>
+        <v>1.080915976391645</v>
       </c>
       <c r="Y32" s="28" t="n">
         <v>56.12174380786062</v>
@@ -8194,10 +8194,10 @@
         <v>561.7750244140625</v>
       </c>
       <c r="W33" s="84" t="n">
-        <v>5380201</v>
+        <v>5389831</v>
       </c>
       <c r="X33" s="85" t="n">
-        <v>0.6617151763152009</v>
+        <v>0.6628603229998266</v>
       </c>
       <c r="Y33" s="35" t="n">
         <v>59.76450182072013</v>
@@ -8301,7 +8301,7 @@
         <v>0.002210423160590835</v>
       </c>
       <c r="D34" s="27" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E34" s="23" t="inlineStr">
         <is>
@@ -8382,10 +8382,10 @@
         <v>341.7000122070312</v>
       </c>
       <c r="W34" s="73" t="n">
-        <v>12516486</v>
+        <v>13164921</v>
       </c>
       <c r="X34" s="74" t="n">
-        <v>0.7004475555136437</v>
+        <v>0.7354009720774396</v>
       </c>
       <c r="Y34" s="28" t="n">
         <v>53.55252150253348</v>
@@ -8464,17 +8464,17 @@
       </c>
       <c r="AX34" s="79" t="inlineStr">
         <is>
+          <t>XLK Does Not Own Alphabet, Amazon, Meta, Netflix or Tesla. Three Stocks Are 35.87% of It</t>
+        </is>
+      </c>
+      <c r="AY34" s="79" t="inlineStr">
+        <is>
+          <t>AI borrowing binge rattles US markets</t>
+        </is>
+      </c>
+      <c r="AZ34" s="79" t="inlineStr">
+        <is>
           <t>Google and Constellation Energy sign latest nuclear energy deal</t>
-        </is>
-      </c>
-      <c r="AY34" s="79" t="inlineStr">
-        <is>
-          <t>Google Joins Microsoft, Amazon, and Meta on Constellation’s Energy Roster</t>
-        </is>
-      </c>
-      <c r="AZ34" s="79" t="inlineStr">
-        <is>
-          <t>US Equity Markets End Higher as Big Tech Gains, Government Bond Yields Fall</t>
         </is>
       </c>
     </row>
@@ -8570,10 +8570,10 @@
         <v>40.5</v>
       </c>
       <c r="W35" s="84" t="n">
-        <v>35584234</v>
+        <v>35863050</v>
       </c>
       <c r="X35" s="85" t="n">
-        <v>1.020483007456523</v>
+        <v>1.0280678647684</v>
       </c>
       <c r="Y35" s="35" t="n">
         <v>46.18333312452347</v>
@@ -8677,7 +8677,7 @@
         <v>-0.03175834722326554</v>
       </c>
       <c r="D36" s="27" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E36" s="23" t="inlineStr">
         <is>
@@ -8758,10 +8758,10 @@
         <v>112.0999984741211</v>
       </c>
       <c r="W36" s="73" t="n">
-        <v>101146493</v>
+        <v>101730627</v>
       </c>
       <c r="X36" s="74" t="n">
-        <v>0.9249470509921963</v>
+        <v>0.9300403398465671</v>
       </c>
       <c r="Y36" s="28" t="n">
         <v>51.98853989406195</v>
@@ -8861,70 +8861,184 @@
           <t>MSFT</t>
         </is>
       </c>
-      <c r="C37" s="33" t="n"/>
-      <c r="D37" s="34" t="n"/>
-      <c r="E37" s="30" t="n"/>
-      <c r="F37" s="30" t="n"/>
-      <c r="G37" s="30" t="n"/>
-      <c r="H37" s="30" t="n"/>
-      <c r="I37" s="30" t="n"/>
-      <c r="J37" s="30" t="n"/>
-      <c r="K37" s="30" t="n"/>
-      <c r="L37" s="30" t="n"/>
-      <c r="M37" s="30" t="n"/>
-      <c r="N37" s="80" t="n"/>
-      <c r="O37" s="30" t="n"/>
-      <c r="P37" s="32" t="n"/>
+      <c r="C37" s="33" t="n">
+        <v>0.007844920169552072</v>
+      </c>
+      <c r="D37" s="34" t="n">
+        <v>14</v>
+      </c>
+      <c r="E37" s="30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F37" s="30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G37" s="30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H37" s="30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I37" s="30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J37" s="30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K37" s="30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L37" s="30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M37" s="30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N37" s="80" t="n">
+        <v>8</v>
+      </c>
+      <c r="O37" s="30" t="inlineStr">
+        <is>
+          <t>Very Strong</t>
+        </is>
+      </c>
+      <c r="P37" s="32" t="inlineStr">
+        <is>
+          <t>Above every average</t>
+        </is>
+      </c>
       <c r="Q37" s="32" t="inlineStr">
         <is>
           <t>Microsoft Corporation</t>
         </is>
       </c>
-      <c r="R37" s="81" t="n"/>
-      <c r="S37" s="82" t="n"/>
-      <c r="T37" s="83" t="n"/>
-      <c r="U37" s="83" t="n"/>
-      <c r="V37" s="83" t="n"/>
-      <c r="W37" s="84" t="n"/>
-      <c r="X37" s="85" t="n"/>
-      <c r="Y37" s="35" t="n"/>
-      <c r="Z37" s="35" t="n"/>
-      <c r="AA37" s="35" t="n"/>
-      <c r="AB37" s="86" t="n"/>
-      <c r="AC37" s="86" t="n"/>
-      <c r="AD37" s="86" t="n"/>
-      <c r="AE37" s="83" t="n"/>
-      <c r="AF37" s="83" t="n"/>
-      <c r="AG37" s="83" t="n"/>
-      <c r="AH37" s="83" t="n"/>
-      <c r="AI37" s="83" t="n"/>
-      <c r="AJ37" s="83" t="n"/>
-      <c r="AK37" s="83" t="n"/>
-      <c r="AL37" s="83" t="n"/>
-      <c r="AM37" s="87" t="n"/>
-      <c r="AN37" s="36" t="n"/>
-      <c r="AO37" s="88" t="n"/>
-      <c r="AP37" s="83" t="n"/>
-      <c r="AQ37" s="83" t="n"/>
-      <c r="AR37" s="36" t="n"/>
-      <c r="AS37" s="89" t="n"/>
-      <c r="AT37" s="33" t="n"/>
-      <c r="AU37" s="33" t="n"/>
-      <c r="AV37" s="33" t="n"/>
-      <c r="AW37" s="33" t="n"/>
+      <c r="R37" s="81" t="n">
+        <v>529.2999877929688</v>
+      </c>
+      <c r="S37" s="82" t="n">
+        <v>4.1199951171875</v>
+      </c>
+      <c r="T37" s="83" t="n">
+        <v>531.6799926757812</v>
+      </c>
+      <c r="U37" s="83" t="n">
+        <v>535.6900024414062</v>
+      </c>
+      <c r="V37" s="83" t="n">
+        <v>528.8200073242188</v>
+      </c>
+      <c r="W37" s="84" t="n">
+        <v>21098949</v>
+      </c>
+      <c r="X37" s="85" t="n">
+        <v>0.9682446535794419</v>
+      </c>
+      <c r="Y37" s="35" t="n">
+        <v>67.93773216705935</v>
+      </c>
+      <c r="Z37" s="35" t="n">
+        <v>85.66939857986141</v>
+      </c>
+      <c r="AA37" s="35" t="n">
+        <v>39.22214136949519</v>
+      </c>
+      <c r="AB37" s="86" t="n">
+        <v>9.507712489119115</v>
+      </c>
+      <c r="AC37" s="86" t="n">
+        <v>8.047404945628641</v>
+      </c>
+      <c r="AD37" s="86" t="n">
+        <v>1.460307543490474</v>
+      </c>
+      <c r="AE37" s="83" t="n">
+        <v>516.9904477691638</v>
+      </c>
+      <c r="AF37" s="83" t="n">
+        <v>507.0594827080815</v>
+      </c>
+      <c r="AG37" s="83" t="n">
+        <v>493.3977990722656</v>
+      </c>
+      <c r="AH37" s="83" t="n">
+        <v>446.1273986816406</v>
+      </c>
+      <c r="AI37" s="83" t="n">
+        <v>433.3407992553711</v>
+      </c>
+      <c r="AJ37" s="83" t="n">
+        <v>526.8272599034109</v>
+      </c>
+      <c r="AK37" s="83" t="n">
+        <v>504.7134979248047</v>
+      </c>
+      <c r="AL37" s="83" t="n">
+        <v>482.5997359461985</v>
+      </c>
+      <c r="AM37" s="87" t="n">
+        <v>1.055909254426046</v>
+      </c>
+      <c r="AN37" s="36" t="n">
+        <v>8.762896997813545</v>
+      </c>
+      <c r="AO37" s="88" t="n">
+        <v>2.214887133372449</v>
+      </c>
+      <c r="AP37" s="83" t="n">
+        <v>553.719970703125</v>
+      </c>
+      <c r="AQ37" s="83" t="n">
+        <v>349.2000122070312</v>
+      </c>
+      <c r="AR37" s="36" t="n">
+        <v>-4.410168352632693</v>
+      </c>
+      <c r="AS37" s="89" t="n">
+        <v>88.05985338070433</v>
+      </c>
+      <c r="AT37" s="33" t="n">
+        <v>0.03996384132226205</v>
+      </c>
+      <c r="AU37" s="33" t="n">
+        <v>0.05923549102030812</v>
+      </c>
+      <c r="AV37" s="33" t="n">
+        <v>0.3807585768494226</v>
+      </c>
+      <c r="AW37" s="33" t="n">
+        <v>0.09445430945160238</v>
+      </c>
       <c r="AX37" s="90" t="inlineStr">
         <is>
-          <t>Marvell stock surges after company raises 2028 revenue outlook to $20 billion</t>
+          <t>Google Joins Microsoft, Amazon, and Meta on Constellation’s Energy Roster</t>
         </is>
       </c>
       <c r="AY37" s="90" t="inlineStr">
         <is>
-          <t>Google Joins Microsoft, Amazon, and Meta on Constellation’s Energy Roster</t>
+          <t>A $1,000 Bet on Microsoft a Decade Ago Crushed the Market by Over 3x</t>
         </is>
       </c>
       <c r="AZ37" s="90" t="inlineStr">
         <is>
-          <t>A $1,000 Bet on Microsoft a Decade Ago Crushed the Market by Over 3x</t>
+          <t>Jim Cramer: Microsoft’s “Monster” Data Center Play Is Starting to Pay Off</t>
         </is>
       </c>
     </row>
@@ -8939,7 +9053,7 @@
         <v>0.000729856968449738</v>
       </c>
       <c r="D38" s="27" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E38" s="23" t="inlineStr">
         <is>
@@ -8948,7 +9062,7 @@
       </c>
       <c r="F38" s="23" t="inlineStr">
         <is>
-          <t>Same</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G38" s="23" t="inlineStr">
@@ -9020,10 +9134,10 @@
         <v>163.1799926757812</v>
       </c>
       <c r="W38" s="73" t="n">
-        <v>17800689</v>
+        <v>17466665</v>
       </c>
       <c r="X38" s="74" t="n">
-        <v>0.8013136281163082</v>
+        <v>0.7868688278539158</v>
       </c>
       <c r="Y38" s="28" t="n">
         <v>65.04416257626946</v>
@@ -9127,7 +9241,7 @@
         <v>-0.0172937920779811</v>
       </c>
       <c r="D39" s="34" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E39" s="30" t="inlineStr">
         <is>
@@ -9208,10 +9322,10 @@
         <v>1045.260009765625</v>
       </c>
       <c r="W39" s="84" t="n">
-        <v>20839091</v>
+        <v>21725080</v>
       </c>
       <c r="X39" s="85" t="n">
-        <v>0.8258840890752386</v>
+        <v>0.8594881844843747</v>
       </c>
       <c r="Y39" s="35" t="n">
         <v>53.94384414684087</v>
@@ -9295,12 +9409,12 @@
       </c>
       <c r="AY39" s="90" t="inlineStr">
         <is>
+          <t>NLST Stock Jumps 18% After Micron’s $600M License Deal — Retail Now Awaits SK Hynix</t>
+        </is>
+      </c>
+      <c r="AZ39" s="90" t="inlineStr">
+        <is>
           <t>5 Surging ETFs Up More than 50% in 2026</t>
-        </is>
-      </c>
-      <c r="AZ39" s="90" t="inlineStr">
-        <is>
-          <t>Micron Stock Drops. Why It Needs a Memory Price Test.</t>
         </is>
       </c>
     </row>
@@ -9396,10 +9510,10 @@
         <v>237</v>
       </c>
       <c r="W40" s="73" t="n">
-        <v>21348395</v>
+        <v>21398036</v>
       </c>
       <c r="X40" s="74" t="n">
-        <v>1.391291577186505</v>
+        <v>1.394301181763071</v>
       </c>
       <c r="Y40" s="28" t="n">
         <v>58.73547651017797</v>
@@ -9584,10 +9698,10 @@
         <v>67.30999755859375</v>
       </c>
       <c r="W41" s="84" t="n">
-        <v>34792314</v>
+        <v>35156434</v>
       </c>
       <c r="X41" s="85" t="n">
-        <v>0.974910086497915</v>
+        <v>0.9846107403523489</v>
       </c>
       <c r="Y41" s="35" t="n">
         <v>37.36148507175925</v>
@@ -9772,10 +9886,10 @@
         <v>10.26000022888184</v>
       </c>
       <c r="W42" s="73" t="n">
-        <v>87302057</v>
+        <v>89196650</v>
       </c>
       <c r="X42" s="74" t="n">
-        <v>1.015489740460704</v>
+        <v>1.036385497715088</v>
       </c>
       <c r="Y42" s="28" t="n">
         <v>56.87277379073492</v>
@@ -9879,7 +9993,7 @@
         <v>0.001423238197431731</v>
       </c>
       <c r="D43" s="34" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E43" s="30" t="inlineStr">
         <is>
@@ -9960,10 +10074,10 @@
         <v>238.9299926757812</v>
       </c>
       <c r="W43" s="84" t="n">
-        <v>100677088</v>
+        <v>101482897</v>
       </c>
       <c r="X43" s="85" t="n">
-        <v>0.9283915668018391</v>
+        <v>0.9354747529303267</v>
       </c>
       <c r="Y43" s="35" t="n">
         <v>67.16310870159653</v>
@@ -10042,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
-          <t>Markets climb as a handful of tech stocks power the rally</t>
+          <t>SPCX Stock Slips After-Hours As SpaceX Reportedly Seeks $40B For Nvidia Chips</t>
         </is>
       </c>
       <c r="AY43" s="90" t="inlineStr">
         <is>
-          <t>Lamb Weston Holdings, Inc. Q1 2027 Earnings Call Summary</t>
+          <t>Is Nvidia’s (NVDA) Free Cash Flow Keeping Pace With Its Reported Earnings?</t>
         </is>
       </c>
       <c r="AZ43" s="90" t="inlineStr">
         <is>
-          <t>$5,100 Split Across These 5 AI Infrastructure Stocks Could Be Worth This Much by 2030</t>
+          <t>XLK Does Not Own Alphabet, Amazon, Meta, Netflix or Tesla. Three Stocks Are 35.87% of It</t>
         </is>
       </c>
     </row>
@@ -10148,10 +10262,10 @@
         <v>190.25</v>
       </c>
       <c r="W44" s="73" t="n">
-        <v>17488501</v>
+        <v>17636801</v>
       </c>
       <c r="X44" s="74" t="n">
-        <v>0.7889763456234195</v>
+        <v>0.7954006750510053</v>
       </c>
       <c r="Y44" s="28" t="n">
         <v>64.31868245367329</v>
@@ -10255,7 +10369,7 @@
         <v>0.001327537485906083</v>
       </c>
       <c r="D45" s="34" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E45" s="30" t="inlineStr">
         <is>
@@ -10336,10 +10450,10 @@
         <v>179.3311004638672</v>
       </c>
       <c r="W45" s="84" t="n">
-        <v>8210457</v>
+        <v>8222272</v>
       </c>
       <c r="X45" s="85" t="n">
-        <v>0.5693911581602681</v>
+        <v>0.5701871630497433</v>
       </c>
       <c r="Y45" s="35" t="n">
         <v>49.1466119946765</v>
@@ -10524,10 +10638,10 @@
         <v>73.66000366210938</v>
       </c>
       <c r="W46" s="73" t="n">
-        <v>26870720</v>
+        <v>26990034</v>
       </c>
       <c r="X46" s="74" t="n">
-        <v>1.242604746068015</v>
+        <v>1.247778048275746</v>
       </c>
       <c r="Y46" s="28" t="n">
         <v>59.77533414754705</v>
@@ -10631,7 +10745,7 @@
         <v>-0.02564317456442577</v>
       </c>
       <c r="D47" s="34" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E47" s="30" t="inlineStr">
         <is>
@@ -10679,7 +10793,7 @@
         </is>
       </c>
       <c r="N47" s="80" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O47" s="30" t="inlineStr">
         <is>
@@ -10712,10 +10826,10 @@
         <v>1650</v>
       </c>
       <c r="W47" s="84" t="n">
-        <v>6501257</v>
+        <v>6521635</v>
       </c>
       <c r="X47" s="85" t="n">
-        <v>0.7489998306838814</v>
+        <v>0.751259361496903</v>
       </c>
       <c r="Y47" s="35" t="n">
         <v>48.72377558873259</v>
@@ -10819,7 +10933,7 @@
         <v>0.00514873823802553</v>
       </c>
       <c r="D48" s="27" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E48" s="23" t="inlineStr">
         <is>
@@ -10900,10 +11014,10 @@
         <v>378.5199890136719</v>
       </c>
       <c r="W48" s="73" t="n">
-        <v>27592528</v>
+        <v>27702813</v>
       </c>
       <c r="X48" s="74" t="n">
-        <v>0.7705928838583525</v>
+        <v>0.7735537513531296</v>
       </c>
       <c r="Y48" s="28" t="n">
         <v>59.64583596842736</v>
@@ -11529,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 6 Oct 2026, 09:47 PM · Yahoo Finance data</t>
+          <t>Built 6 Oct 2026, 11:51 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -11554,22 +11668,22 @@
       </c>
       <c r="Y3" s="44" t="inlineStr">
         <is>
-          <t>23 of 39</t>
+          <t>24 of 40</t>
         </is>
       </c>
       <c r="AA3" s="45" t="inlineStr">
         <is>
-          <t>16 of 39</t>
+          <t>16 of 40</t>
         </is>
       </c>
       <c r="AC3" s="46" t="inlineStr">
         <is>
-          <t>4.9 / 9</t>
+          <t>5.0 / 9</t>
         </is>
       </c>
       <c r="AE3" s="47" t="inlineStr">
         <is>
-          <t>19 of 39</t>
+          <t>20 of 40</t>
         </is>
       </c>
     </row>
@@ -14663,7 +14777,7 @@
         <v>-0.002397398145331686</v>
       </c>
       <c r="D24" s="27" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E24" s="23" t="inlineStr">
         <is>
@@ -14839,7 +14953,7 @@
         <v>-0.003407381546336352</v>
       </c>
       <c r="D25" s="34" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E25" s="30" t="inlineStr">
         <is>
@@ -15015,7 +15129,7 @@
         <v>-0.0004771404816237279</v>
       </c>
       <c r="D26" s="27" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E26" s="23" t="inlineStr">
         <is>
@@ -15367,7 +15481,7 @@
         <v>-0.01492730327381397</v>
       </c>
       <c r="D28" s="27" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E28" s="23" t="inlineStr">
         <is>
@@ -15543,7 +15657,7 @@
         <v>-0.0001711229443954743</v>
       </c>
       <c r="D29" s="34" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E29" s="30" t="inlineStr">
         <is>
@@ -16071,7 +16185,7 @@
         <v>-0.02488287534691735</v>
       </c>
       <c r="D32" s="27" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E32" s="23" t="inlineStr">
         <is>
@@ -16247,7 +16361,7 @@
         <v>-0.01818609320328013</v>
       </c>
       <c r="D33" s="34" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E33" s="30" t="inlineStr">
         <is>
@@ -16423,7 +16537,7 @@
         <v>0.01022471105139799</v>
       </c>
       <c r="D34" s="27" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E34" s="23" t="inlineStr">
         <is>
@@ -16599,7 +16713,7 @@
         <v>-0.03065131299674539</v>
       </c>
       <c r="D35" s="34" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E35" s="30" t="inlineStr">
         <is>
@@ -16775,7 +16889,7 @@
         <v>-0.02631357865974049</v>
       </c>
       <c r="D36" s="27" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E36" s="23" t="inlineStr">
         <is>
@@ -16947,57 +17061,171 @@
           <t>MSFT</t>
         </is>
       </c>
-      <c r="C37" s="33" t="n"/>
-      <c r="D37" s="34" t="n"/>
-      <c r="E37" s="30" t="n"/>
-      <c r="F37" s="30" t="n"/>
-      <c r="G37" s="30" t="n"/>
-      <c r="H37" s="30" t="n"/>
-      <c r="I37" s="30" t="n"/>
-      <c r="J37" s="30" t="n"/>
-      <c r="K37" s="30" t="n"/>
-      <c r="L37" s="30" t="n"/>
-      <c r="M37" s="30" t="n"/>
-      <c r="N37" s="80" t="n"/>
-      <c r="O37" s="30" t="n"/>
-      <c r="P37" s="32" t="n"/>
+      <c r="C37" s="33" t="n">
+        <v>0.01478168018443227</v>
+      </c>
+      <c r="D37" s="34" t="n">
+        <v>7</v>
+      </c>
+      <c r="E37" s="30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F37" s="30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G37" s="30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H37" s="30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I37" s="30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J37" s="30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K37" s="30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L37" s="30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M37" s="30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N37" s="80" t="n">
+        <v>9</v>
+      </c>
+      <c r="O37" s="30" t="inlineStr">
+        <is>
+          <t>Very Strong</t>
+        </is>
+      </c>
+      <c r="P37" s="32" t="inlineStr">
+        <is>
+          <t>Above every average</t>
+        </is>
+      </c>
       <c r="Q37" s="32" t="inlineStr">
         <is>
           <t>Microsoft Corporation</t>
         </is>
       </c>
-      <c r="R37" s="81" t="n"/>
-      <c r="S37" s="82" t="n"/>
-      <c r="T37" s="83" t="n"/>
-      <c r="U37" s="83" t="n"/>
-      <c r="V37" s="83" t="n"/>
-      <c r="W37" s="84" t="n"/>
-      <c r="X37" s="85" t="n"/>
-      <c r="Y37" s="35" t="n"/>
-      <c r="Z37" s="35" t="n"/>
-      <c r="AA37" s="35" t="n"/>
-      <c r="AB37" s="86" t="n"/>
-      <c r="AC37" s="86" t="n"/>
-      <c r="AD37" s="86" t="n"/>
-      <c r="AE37" s="83" t="n"/>
-      <c r="AF37" s="83" t="n"/>
-      <c r="AG37" s="83" t="n"/>
-      <c r="AH37" s="83" t="n"/>
-      <c r="AI37" s="83" t="n"/>
-      <c r="AJ37" s="83" t="n"/>
-      <c r="AK37" s="83" t="n"/>
-      <c r="AL37" s="83" t="n"/>
-      <c r="AM37" s="87" t="n"/>
-      <c r="AN37" s="36" t="n"/>
-      <c r="AO37" s="88" t="n"/>
-      <c r="AP37" s="83" t="n"/>
-      <c r="AQ37" s="83" t="n"/>
-      <c r="AR37" s="36" t="n"/>
-      <c r="AS37" s="89" t="n"/>
-      <c r="AT37" s="33" t="n"/>
-      <c r="AU37" s="33" t="n"/>
-      <c r="AV37" s="33" t="n"/>
-      <c r="AW37" s="33" t="n"/>
+      <c r="R37" s="81" t="n">
+        <v>525.1799926757812</v>
+      </c>
+      <c r="S37" s="82" t="n">
+        <v>7.64996337890625</v>
+      </c>
+      <c r="T37" s="83" t="n">
+        <v>521.6199951171875</v>
+      </c>
+      <c r="U37" s="83" t="n">
+        <v>532.3499755859375</v>
+      </c>
+      <c r="V37" s="83" t="n">
+        <v>521.469970703125</v>
+      </c>
+      <c r="W37" s="84" t="n">
+        <v>26604800</v>
+      </c>
+      <c r="X37" s="85" t="n">
+        <v>1.227153294300602</v>
+      </c>
+      <c r="Y37" s="35" t="n">
+        <v>66.17154210418117</v>
+      </c>
+      <c r="Z37" s="35" t="n">
+        <v>84.10906796186111</v>
+      </c>
+      <c r="AA37" s="35" t="n">
+        <v>37.7752728220594</v>
+      </c>
+      <c r="AB37" s="86" t="n">
+        <v>8.630325702191044</v>
+      </c>
+      <c r="AC37" s="86" t="n">
+        <v>7.682328059756022</v>
+      </c>
+      <c r="AD37" s="86" t="n">
+        <v>0.9479976424350225</v>
+      </c>
+      <c r="AE37" s="83" t="n">
+        <v>513.4734363337909</v>
+      </c>
+      <c r="AF37" s="83" t="n">
+        <v>504.8354321995928</v>
+      </c>
+      <c r="AG37" s="83" t="n">
+        <v>490.5937994384765</v>
+      </c>
+      <c r="AH37" s="83" t="n">
+        <v>444.8864987182617</v>
+      </c>
+      <c r="AI37" s="83" t="n">
+        <v>433.0748992919922</v>
+      </c>
+      <c r="AJ37" s="83" t="n">
+        <v>522.4086220226808</v>
+      </c>
+      <c r="AK37" s="83" t="n">
+        <v>502.9459991455078</v>
+      </c>
+      <c r="AL37" s="83" t="n">
+        <v>483.4833762683348</v>
+      </c>
+      <c r="AM37" s="87" t="n">
+        <v>1.071197255133349</v>
+      </c>
+      <c r="AN37" s="36" t="n">
+        <v>7.73944833450886</v>
+      </c>
+      <c r="AO37" s="88" t="n">
+        <v>2.250035225266358</v>
+      </c>
+      <c r="AP37" s="83" t="n">
+        <v>553.719970703125</v>
+      </c>
+      <c r="AQ37" s="83" t="n">
+        <v>349.2000122070312</v>
+      </c>
+      <c r="AR37" s="36" t="n">
+        <v>-5.154225879031071</v>
+      </c>
+      <c r="AS37" s="89" t="n">
+        <v>86.04538244716647</v>
+      </c>
+      <c r="AT37" s="33" t="n">
+        <v>0.03134203569541416</v>
+      </c>
+      <c r="AU37" s="33" t="n">
+        <v>0.02952246079892262</v>
+      </c>
+      <c r="AV37" s="33" t="n">
+        <v>0.3506326448460697</v>
+      </c>
+      <c r="AW37" s="33" t="n">
+        <v>0.0859352342297659</v>
+      </c>
       <c r="AX37" s="32" t="n"/>
       <c r="AY37" s="32" t="n"/>
       <c r="AZ37" s="32" t="n"/>
@@ -17189,7 +17417,7 @@
         <v>-0.0101685321865348</v>
       </c>
       <c r="D39" s="34" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E39" s="30" t="inlineStr">
         <is>
@@ -17365,7 +17593,7 @@
         <v>-0.04217285258982773</v>
       </c>
       <c r="D40" s="27" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E40" s="23" t="inlineStr">
         <is>
@@ -17541,7 +17769,7 @@
         <v>0.006561325043619393</v>
       </c>
       <c r="D41" s="34" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E41" s="30" t="inlineStr">
         <is>
@@ -17717,7 +17945,7 @@
         <v>-0.03773590168014018</v>
       </c>
       <c r="D42" s="27" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E42" s="23" t="inlineStr">
         <is>
@@ -18069,7 +18297,7 @@
         <v>0.003443676272764984</v>
       </c>
       <c r="D44" s="27" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E44" s="23" t="inlineStr">
         <is>
@@ -18245,7 +18473,7 @@
         <v>-0.02206957288265421</v>
       </c>
       <c r="D45" s="34" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E45" s="30" t="inlineStr">
         <is>
@@ -18421,7 +18649,7 @@
         <v>-0.01217534561921851</v>
       </c>
       <c r="D46" s="27" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E46" s="23" t="inlineStr">
         <is>
@@ -18597,7 +18825,7 @@
         <v>-0.009203516383563648</v>
       </c>
       <c r="D47" s="34" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E47" s="30" t="inlineStr">
         <is>
@@ -19351,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 6 Oct 2026, 09:47 PM · Yahoo Finance data</t>
+          <t>Built 6 Oct 2026, 11:51 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19376,22 +19604,22 @@
       </c>
       <c r="Y3" s="44" t="inlineStr">
         <is>
-          <t>31 of 39</t>
+          <t>32 of 40</t>
         </is>
       </c>
       <c r="AA3" s="45" t="inlineStr">
         <is>
-          <t>8 of 39</t>
+          <t>8 of 40</t>
         </is>
       </c>
       <c r="AC3" s="46" t="inlineStr">
         <is>
-          <t>5.1 / 9</t>
+          <t>5.2 / 9</t>
         </is>
       </c>
       <c r="AE3" s="47" t="inlineStr">
         <is>
-          <t>20 of 39</t>
+          <t>21 of 40</t>
         </is>
       </c>
     </row>
@@ -23717,7 +23945,7 @@
         <v>-0.005951711071302657</v>
       </c>
       <c r="D31" s="34" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E31" s="30" t="inlineStr">
         <is>
@@ -24597,7 +24825,7 @@
         <v>-0.005583318074544263</v>
       </c>
       <c r="D36" s="27" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E36" s="23" t="inlineStr">
         <is>
@@ -24769,57 +24997,171 @@
           <t>MSFT</t>
         </is>
       </c>
-      <c r="C37" s="33" t="n"/>
-      <c r="D37" s="34" t="n"/>
-      <c r="E37" s="30" t="n"/>
-      <c r="F37" s="30" t="n"/>
-      <c r="G37" s="30" t="n"/>
-      <c r="H37" s="30" t="n"/>
-      <c r="I37" s="30" t="n"/>
-      <c r="J37" s="30" t="n"/>
-      <c r="K37" s="30" t="n"/>
-      <c r="L37" s="30" t="n"/>
-      <c r="M37" s="30" t="n"/>
-      <c r="N37" s="80" t="n"/>
-      <c r="O37" s="30" t="n"/>
-      <c r="P37" s="32" t="n"/>
+      <c r="C37" s="33" t="n">
+        <v>0.009223950110185841</v>
+      </c>
+      <c r="D37" s="34" t="n">
+        <v>18</v>
+      </c>
+      <c r="E37" s="30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F37" s="30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G37" s="30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H37" s="30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I37" s="30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J37" s="30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K37" s="30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L37" s="30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M37" s="30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N37" s="80" t="n">
+        <v>8</v>
+      </c>
+      <c r="O37" s="30" t="inlineStr">
+        <is>
+          <t>Very Strong</t>
+        </is>
+      </c>
+      <c r="P37" s="32" t="inlineStr">
+        <is>
+          <t>Above every average</t>
+        </is>
+      </c>
       <c r="Q37" s="32" t="inlineStr">
         <is>
           <t>Microsoft Corporation</t>
         </is>
       </c>
-      <c r="R37" s="81" t="n"/>
-      <c r="S37" s="82" t="n"/>
-      <c r="T37" s="83" t="n"/>
-      <c r="U37" s="83" t="n"/>
-      <c r="V37" s="83" t="n"/>
-      <c r="W37" s="84" t="n"/>
-      <c r="X37" s="85" t="n"/>
-      <c r="Y37" s="35" t="n"/>
-      <c r="Z37" s="35" t="n"/>
-      <c r="AA37" s="35" t="n"/>
-      <c r="AB37" s="86" t="n"/>
-      <c r="AC37" s="86" t="n"/>
-      <c r="AD37" s="86" t="n"/>
-      <c r="AE37" s="83" t="n"/>
-      <c r="AF37" s="83" t="n"/>
-      <c r="AG37" s="83" t="n"/>
-      <c r="AH37" s="83" t="n"/>
-      <c r="AI37" s="83" t="n"/>
-      <c r="AJ37" s="83" t="n"/>
-      <c r="AK37" s="83" t="n"/>
-      <c r="AL37" s="83" t="n"/>
-      <c r="AM37" s="87" t="n"/>
-      <c r="AN37" s="36" t="n"/>
-      <c r="AO37" s="88" t="n"/>
-      <c r="AP37" s="83" t="n"/>
-      <c r="AQ37" s="83" t="n"/>
-      <c r="AR37" s="36" t="n"/>
-      <c r="AS37" s="89" t="n"/>
-      <c r="AT37" s="33" t="n"/>
-      <c r="AU37" s="33" t="n"/>
-      <c r="AV37" s="33" t="n"/>
-      <c r="AW37" s="33" t="n"/>
+      <c r="R37" s="81" t="n">
+        <v>517.530029296875</v>
+      </c>
+      <c r="S37" s="82" t="n">
+        <v>4.73004150390625</v>
+      </c>
+      <c r="T37" s="83" t="n">
+        <v>519.3900146484375</v>
+      </c>
+      <c r="U37" s="83" t="n">
+        <v>522.5</v>
+      </c>
+      <c r="V37" s="83" t="n">
+        <v>513.6599731445312</v>
+      </c>
+      <c r="W37" s="84" t="n">
+        <v>17822300</v>
+      </c>
+      <c r="X37" s="85" t="n">
+        <v>0.8385013463925689</v>
+      </c>
+      <c r="Y37" s="35" t="n">
+        <v>62.62141386896888</v>
+      </c>
+      <c r="Z37" s="35" t="n">
+        <v>85.06470641152507</v>
+      </c>
+      <c r="AA37" s="35" t="n">
+        <v>36.37480485709369</v>
+      </c>
+      <c r="AB37" s="86" t="n">
+        <v>7.804419514048277</v>
+      </c>
+      <c r="AC37" s="86" t="n">
+        <v>7.445328649147266</v>
+      </c>
+      <c r="AD37" s="86" t="n">
+        <v>0.3590908649010114</v>
+      </c>
+      <c r="AE37" s="83" t="n">
+        <v>510.1287059503651</v>
+      </c>
+      <c r="AF37" s="83" t="n">
+        <v>502.8009761519739</v>
+      </c>
+      <c r="AG37" s="83" t="n">
+        <v>487.7241998291016</v>
+      </c>
+      <c r="AH37" s="83" t="n">
+        <v>443.7123986816407</v>
+      </c>
+      <c r="AI37" s="83" t="n">
+        <v>432.8309494018555</v>
+      </c>
+      <c r="AJ37" s="83" t="n">
+        <v>518.2713551635253</v>
+      </c>
+      <c r="AK37" s="83" t="n">
+        <v>501.6720001220703</v>
+      </c>
+      <c r="AL37" s="83" t="n">
+        <v>485.0726450806154</v>
+      </c>
+      <c r="AM37" s="87" t="n">
+        <v>0.9776700400467692</v>
+      </c>
+      <c r="AN37" s="36" t="n">
+        <v>6.617612718037244</v>
+      </c>
+      <c r="AO37" s="88" t="n">
+        <v>2.238656292275798</v>
+      </c>
+      <c r="AP37" s="83" t="n">
+        <v>553.719970703125</v>
+      </c>
+      <c r="AQ37" s="83" t="n">
+        <v>349.2000122070312</v>
+      </c>
+      <c r="AR37" s="36" t="n">
+        <v>-6.535784028214708</v>
+      </c>
+      <c r="AS37" s="89" t="n">
+        <v>82.30493411383065</v>
+      </c>
+      <c r="AT37" s="33" t="n">
+        <v>0.002634880817847796</v>
+      </c>
+      <c r="AU37" s="33" t="n">
+        <v>0.04168516095838526</v>
+      </c>
+      <c r="AV37" s="33" t="n">
+        <v>0.3381859708462982</v>
+      </c>
+      <c r="AW37" s="33" t="n">
+        <v>0.07011710541759264</v>
+      </c>
       <c r="AX37" s="32" t="n"/>
       <c r="AY37" s="32" t="n"/>
       <c r="AZ37" s="32" t="n"/>
@@ -24835,7 +25177,7 @@
         <v>-0.003052993726878839</v>
       </c>
       <c r="D38" s="27" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E38" s="23" t="inlineStr">
         <is>
@@ -25011,7 +25353,7 @@
         <v>-0.02050319366830411</v>
       </c>
       <c r="D39" s="34" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E39" s="30" t="inlineStr">
         <is>
@@ -25363,7 +25705,7 @@
         <v>-0.01164334463218386</v>
       </c>
       <c r="D41" s="34" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E41" s="30" t="inlineStr">
         <is>
@@ -25891,7 +26233,7 @@
         <v>-0.006788009533290951</v>
       </c>
       <c r="D44" s="27" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E44" s="23" t="inlineStr">
         <is>
@@ -26419,7 +26761,7 @@
         <v>-0.037870074448492</v>
       </c>
       <c r="D47" s="34" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E47" s="30" t="inlineStr">
         <is>
@@ -27173,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 6 Oct 2026, 09:47 PM · Yahoo Finance data</t>
+          <t>Built 6 Oct 2026, 11:51 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27198,12 +27540,12 @@
       </c>
       <c r="Y3" s="44" t="inlineStr">
         <is>
-          <t>20 of 39</t>
+          <t>20 of 40</t>
         </is>
       </c>
       <c r="AA3" s="45" t="inlineStr">
         <is>
-          <t>19 of 39</t>
+          <t>20 of 40</t>
         </is>
       </c>
       <c r="AC3" s="46" t="inlineStr">
@@ -27213,7 +27555,7 @@
       </c>
       <c r="AE3" s="47" t="inlineStr">
         <is>
-          <t>15 of 39</t>
+          <t>16 of 40</t>
         </is>
       </c>
     </row>
@@ -30307,7 +30649,7 @@
         <v>-0.008107566448037673</v>
       </c>
       <c r="D24" s="27" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E24" s="23" t="inlineStr">
         <is>
@@ -30659,7 +31001,7 @@
         <v>-0.003692547427183723</v>
       </c>
       <c r="D26" s="27" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E26" s="23" t="inlineStr">
         <is>
@@ -30835,7 +31177,7 @@
         <v>-0.005836101593396092</v>
       </c>
       <c r="D27" s="34" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E27" s="30" t="inlineStr">
         <is>
@@ -31187,7 +31529,7 @@
         <v>-0.03092082358055803</v>
       </c>
       <c r="D29" s="34" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E29" s="30" t="inlineStr">
         <is>
@@ -31363,7 +31705,7 @@
         <v>-0.02149829932652603</v>
       </c>
       <c r="D30" s="27" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E30" s="23" t="inlineStr">
         <is>
@@ -31539,7 +31881,7 @@
         <v>-0.0113072083563307</v>
       </c>
       <c r="D31" s="34" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E31" s="30" t="inlineStr">
         <is>
@@ -32067,7 +32409,7 @@
         <v>-0.01705111734785636</v>
       </c>
       <c r="D34" s="27" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E34" s="23" t="inlineStr">
         <is>
@@ -32243,7 +32585,7 @@
         <v>-0.00562621174723299</v>
       </c>
       <c r="D35" s="34" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E35" s="30" t="inlineStr">
         <is>
@@ -32419,7 +32761,7 @@
         <v>-0.001913027950691926</v>
       </c>
       <c r="D36" s="27" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E36" s="23" t="inlineStr">
         <is>
@@ -32591,57 +32933,171 @@
           <t>MSFT</t>
         </is>
       </c>
-      <c r="C37" s="33" t="n"/>
-      <c r="D37" s="34" t="n"/>
-      <c r="E37" s="30" t="n"/>
-      <c r="F37" s="30" t="n"/>
-      <c r="G37" s="30" t="n"/>
-      <c r="H37" s="30" t="n"/>
-      <c r="I37" s="30" t="n"/>
-      <c r="J37" s="30" t="n"/>
-      <c r="K37" s="30" t="n"/>
-      <c r="L37" s="30" t="n"/>
-      <c r="M37" s="30" t="n"/>
-      <c r="N37" s="80" t="n"/>
-      <c r="O37" s="30" t="n"/>
-      <c r="P37" s="32" t="n"/>
+      <c r="C37" s="33" t="n">
+        <v>-0.0001950411704659816</v>
+      </c>
+      <c r="D37" s="34" t="n">
+        <v>12</v>
+      </c>
+      <c r="E37" s="30" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="F37" s="30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G37" s="30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H37" s="30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I37" s="30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J37" s="30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K37" s="30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L37" s="30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M37" s="30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N37" s="80" t="n">
+        <v>7</v>
+      </c>
+      <c r="O37" s="30" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="P37" s="32" t="inlineStr">
+        <is>
+          <t>Above every average</t>
+        </is>
+      </c>
       <c r="Q37" s="32" t="inlineStr">
         <is>
           <t>Microsoft Corporation</t>
         </is>
       </c>
-      <c r="R37" s="81" t="n"/>
-      <c r="S37" s="82" t="n"/>
-      <c r="T37" s="83" t="n"/>
-      <c r="U37" s="83" t="n"/>
-      <c r="V37" s="83" t="n"/>
-      <c r="W37" s="84" t="n"/>
-      <c r="X37" s="85" t="n"/>
-      <c r="Y37" s="35" t="n"/>
-      <c r="Z37" s="35" t="n"/>
-      <c r="AA37" s="35" t="n"/>
-      <c r="AB37" s="86" t="n"/>
-      <c r="AC37" s="86" t="n"/>
-      <c r="AD37" s="86" t="n"/>
-      <c r="AE37" s="83" t="n"/>
-      <c r="AF37" s="83" t="n"/>
-      <c r="AG37" s="83" t="n"/>
-      <c r="AH37" s="83" t="n"/>
-      <c r="AI37" s="83" t="n"/>
-      <c r="AJ37" s="83" t="n"/>
-      <c r="AK37" s="83" t="n"/>
-      <c r="AL37" s="83" t="n"/>
-      <c r="AM37" s="87" t="n"/>
-      <c r="AN37" s="36" t="n"/>
-      <c r="AO37" s="88" t="n"/>
-      <c r="AP37" s="83" t="n"/>
-      <c r="AQ37" s="83" t="n"/>
-      <c r="AR37" s="36" t="n"/>
-      <c r="AS37" s="89" t="n"/>
-      <c r="AT37" s="33" t="n"/>
-      <c r="AU37" s="33" t="n"/>
-      <c r="AV37" s="33" t="n"/>
-      <c r="AW37" s="33" t="n"/>
+      <c r="R37" s="81" t="n">
+        <v>512.7999877929688</v>
+      </c>
+      <c r="S37" s="82" t="n">
+        <v>-0.10003662109375</v>
+      </c>
+      <c r="T37" s="83" t="n">
+        <v>519.8800048828125</v>
+      </c>
+      <c r="U37" s="83" t="n">
+        <v>522.8499755859375</v>
+      </c>
+      <c r="V37" s="83" t="n">
+        <v>512.1699829101562</v>
+      </c>
+      <c r="W37" s="84" t="n">
+        <v>19731900</v>
+      </c>
+      <c r="X37" s="85" t="n">
+        <v>0.9147791215859898</v>
+      </c>
+      <c r="Y37" s="35" t="n">
+        <v>60.22481728807202</v>
+      </c>
+      <c r="Z37" s="35" t="n">
+        <v>71.78551998594922</v>
+      </c>
+      <c r="AA37" s="35" t="n">
+        <v>35.3894915907883</v>
+      </c>
+      <c r="AB37" s="86" t="n">
+        <v>7.415649421375804</v>
+      </c>
+      <c r="AC37" s="86" t="n">
+        <v>7.355555932922011</v>
+      </c>
+      <c r="AD37" s="86" t="n">
+        <v>0.06009348845379225</v>
+      </c>
+      <c r="AE37" s="83" t="n">
+        <v>508.0140421370766</v>
+      </c>
+      <c r="AF37" s="83" t="n">
+        <v>501.3280708374839</v>
+      </c>
+      <c r="AG37" s="83" t="n">
+        <v>485.0051989746094</v>
+      </c>
+      <c r="AH37" s="83" t="n">
+        <v>442.663698425293</v>
+      </c>
+      <c r="AI37" s="83" t="n">
+        <v>432.6173992919922</v>
+      </c>
+      <c r="AJ37" s="83" t="n">
+        <v>516.7600820400728</v>
+      </c>
+      <c r="AK37" s="83" t="n">
+        <v>501.3014984130859</v>
+      </c>
+      <c r="AL37" s="83" t="n">
+        <v>485.8429147860991</v>
+      </c>
+      <c r="AM37" s="87" t="n">
+        <v>0.8719127721316361</v>
+      </c>
+      <c r="AN37" s="36" t="n">
+        <v>6.167379780799529</v>
+      </c>
+      <c r="AO37" s="88" t="n">
+        <v>2.287592273745634</v>
+      </c>
+      <c r="AP37" s="83" t="n">
+        <v>553.719970703125</v>
+      </c>
+      <c r="AQ37" s="83" t="n">
+        <v>349.2000122070312</v>
+      </c>
+      <c r="AR37" s="36" t="n">
+        <v>-7.390013919526006</v>
+      </c>
+      <c r="AS37" s="89" t="n">
+        <v>79.9921811000476</v>
+      </c>
+      <c r="AT37" s="33" t="n">
+        <v>0.02986362608381743</v>
+      </c>
+      <c r="AU37" s="33" t="n">
+        <v>0.02351203352682085</v>
+      </c>
+      <c r="AV37" s="33" t="n">
+        <v>0.31322185105227</v>
+      </c>
+      <c r="AW37" s="33" t="n">
+        <v>0.06033661339562801</v>
+      </c>
       <c r="AX37" s="32" t="n"/>
       <c r="AY37" s="32" t="n"/>
       <c r="AZ37" s="32" t="n"/>
@@ -33009,7 +33465,7 @@
         <v>-0.01526202318549275</v>
       </c>
       <c r="D40" s="27" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E40" s="23" t="inlineStr">
         <is>
@@ -33185,7 +33641,7 @@
         <v>-0.02486351410473042</v>
       </c>
       <c r="D41" s="34" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E41" s="30" t="inlineStr">
         <is>
@@ -33889,7 +34345,7 @@
         <v>-0.01059550651694752</v>
       </c>
       <c r="D45" s="34" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E45" s="30" t="inlineStr">
         <is>
@@ -34417,7 +34873,7 @@
         <v>-0.001972921315205212</v>
       </c>
       <c r="D48" s="27" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E48" s="23" t="inlineStr">
         <is>
@@ -34995,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 6 Oct 2026, 09:47 PM · Yahoo Finance data</t>
+          <t>Built 6 Oct 2026, 11:51 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35020,22 +35476,22 @@
       </c>
       <c r="Y3" s="44" t="inlineStr">
         <is>
-          <t>14 of 39</t>
+          <t>15 of 40</t>
         </is>
       </c>
       <c r="AA3" s="45" t="inlineStr">
         <is>
-          <t>25 of 39</t>
+          <t>25 of 40</t>
         </is>
       </c>
       <c r="AC3" s="46" t="inlineStr">
         <is>
-          <t>4.3 / 9</t>
+          <t>4.4 / 9</t>
         </is>
       </c>
       <c r="AE3" s="47" t="inlineStr">
         <is>
-          <t>17 of 39</t>
+          <t>18 of 40</t>
         </is>
       </c>
     </row>
@@ -38305,7 +38761,7 @@
         <v>0.006896328638504201</v>
       </c>
       <c r="D25" s="34" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E25" s="30" t="inlineStr">
         <is>
@@ -38657,7 +39113,7 @@
         <v>-0.003912783522213137</v>
       </c>
       <c r="D27" s="34" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E27" s="30" t="inlineStr">
         <is>
@@ -38833,7 +39289,7 @@
         <v>-0.01365481520847134</v>
       </c>
       <c r="D28" s="27" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E28" s="23" t="inlineStr">
         <is>
@@ -39009,7 +39465,7 @@
         <v>-0.009090924270297895</v>
       </c>
       <c r="D29" s="34" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E29" s="30" t="inlineStr">
         <is>
@@ -39185,7 +39641,7 @@
         <v>-0.01101099294537766</v>
       </c>
       <c r="D30" s="27" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E30" s="23" t="inlineStr">
         <is>
@@ -39361,7 +39817,7 @@
         <v>-0.002417116610399006</v>
       </c>
       <c r="D31" s="34" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E31" s="30" t="inlineStr">
         <is>
@@ -39713,7 +40169,7 @@
         <v>-0.003039371683711267</v>
       </c>
       <c r="D33" s="34" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E33" s="30" t="inlineStr">
         <is>
@@ -40065,7 +40521,7 @@
         <v>-0.0120831316359068</v>
       </c>
       <c r="D35" s="34" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E35" s="30" t="inlineStr">
         <is>
@@ -40413,57 +40869,171 @@
           <t>MSFT</t>
         </is>
       </c>
-      <c r="C37" s="33" t="n"/>
-      <c r="D37" s="34" t="n"/>
-      <c r="E37" s="30" t="n"/>
-      <c r="F37" s="30" t="n"/>
-      <c r="G37" s="30" t="n"/>
-      <c r="H37" s="30" t="n"/>
-      <c r="I37" s="30" t="n"/>
-      <c r="J37" s="30" t="n"/>
-      <c r="K37" s="30" t="n"/>
-      <c r="L37" s="30" t="n"/>
-      <c r="M37" s="30" t="n"/>
-      <c r="N37" s="80" t="n"/>
-      <c r="O37" s="30" t="n"/>
-      <c r="P37" s="32" t="n"/>
+      <c r="C37" s="33" t="n">
+        <v>0.007741341215681929</v>
+      </c>
+      <c r="D37" s="34" t="n">
+        <v>6</v>
+      </c>
+      <c r="E37" s="30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F37" s="30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G37" s="30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H37" s="30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I37" s="30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J37" s="30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K37" s="30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L37" s="30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M37" s="30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N37" s="80" t="n">
+        <v>8</v>
+      </c>
+      <c r="O37" s="30" t="inlineStr">
+        <is>
+          <t>Very Strong</t>
+        </is>
+      </c>
+      <c r="P37" s="32" t="inlineStr">
+        <is>
+          <t>Above every average</t>
+        </is>
+      </c>
       <c r="Q37" s="32" t="inlineStr">
         <is>
           <t>Microsoft Corporation</t>
         </is>
       </c>
-      <c r="R37" s="81" t="n"/>
-      <c r="S37" s="82" t="n"/>
-      <c r="T37" s="83" t="n"/>
-      <c r="U37" s="83" t="n"/>
-      <c r="V37" s="83" t="n"/>
-      <c r="W37" s="84" t="n"/>
-      <c r="X37" s="85" t="n"/>
-      <c r="Y37" s="35" t="n"/>
-      <c r="Z37" s="35" t="n"/>
-      <c r="AA37" s="35" t="n"/>
-      <c r="AB37" s="86" t="n"/>
-      <c r="AC37" s="86" t="n"/>
-      <c r="AD37" s="86" t="n"/>
-      <c r="AE37" s="83" t="n"/>
-      <c r="AF37" s="83" t="n"/>
-      <c r="AG37" s="83" t="n"/>
-      <c r="AH37" s="83" t="n"/>
-      <c r="AI37" s="83" t="n"/>
-      <c r="AJ37" s="83" t="n"/>
-      <c r="AK37" s="83" t="n"/>
-      <c r="AL37" s="83" t="n"/>
-      <c r="AM37" s="87" t="n"/>
-      <c r="AN37" s="36" t="n"/>
-      <c r="AO37" s="88" t="n"/>
-      <c r="AP37" s="83" t="n"/>
-      <c r="AQ37" s="83" t="n"/>
-      <c r="AR37" s="36" t="n"/>
-      <c r="AS37" s="89" t="n"/>
-      <c r="AT37" s="33" t="n"/>
-      <c r="AU37" s="33" t="n"/>
-      <c r="AV37" s="33" t="n"/>
-      <c r="AW37" s="33" t="n"/>
+      <c r="R37" s="81" t="n">
+        <v>512.9000244140625</v>
+      </c>
+      <c r="S37" s="82" t="n">
+        <v>3.940032958984375</v>
+      </c>
+      <c r="T37" s="83" t="n">
+        <v>511.6099853515625</v>
+      </c>
+      <c r="U37" s="83" t="n">
+        <v>519.8300170898438</v>
+      </c>
+      <c r="V37" s="83" t="n">
+        <v>510.3099975585938</v>
+      </c>
+      <c r="W37" s="84" t="n">
+        <v>27223300</v>
+      </c>
+      <c r="X37" s="85" t="n">
+        <v>1.275076011687873</v>
+      </c>
+      <c r="Y37" s="35" t="n">
+        <v>60.30074566695022</v>
+      </c>
+      <c r="Z37" s="35" t="n">
+        <v>78.74235773522167</v>
+      </c>
+      <c r="AA37" s="35" t="n">
+        <v>34.32838499630556</v>
+      </c>
+      <c r="AB37" s="86" t="n">
+        <v>7.293177646451511</v>
+      </c>
+      <c r="AC37" s="86" t="n">
+        <v>7.340532560808563</v>
+      </c>
+      <c r="AD37" s="86" t="n">
+        <v>-0.04735491435705175</v>
+      </c>
+      <c r="AE37" s="83" t="n">
+        <v>506.6466290925359</v>
+      </c>
+      <c r="AF37" s="83" t="n">
+        <v>500.1808791419355</v>
+      </c>
+      <c r="AG37" s="83" t="n">
+        <v>482.5559991455078</v>
+      </c>
+      <c r="AH37" s="83" t="n">
+        <v>441.6868984985351</v>
+      </c>
+      <c r="AI37" s="83" t="n">
+        <v>432.4460493469238</v>
+      </c>
+      <c r="AJ37" s="83" t="n">
+        <v>515.1308250240739</v>
+      </c>
+      <c r="AK37" s="83" t="n">
+        <v>500.5024993896484</v>
+      </c>
+      <c r="AL37" s="83" t="n">
+        <v>485.8741737552229</v>
+      </c>
+      <c r="AM37" s="87" t="n">
+        <v>0.9237506511079574</v>
+      </c>
+      <c r="AN37" s="36" t="n">
+        <v>5.845455578049834</v>
+      </c>
+      <c r="AO37" s="88" t="n">
+        <v>2.302905359006555</v>
+      </c>
+      <c r="AP37" s="83" t="n">
+        <v>553.719970703125</v>
+      </c>
+      <c r="AQ37" s="83" t="n">
+        <v>349.2000122070312</v>
+      </c>
+      <c r="AR37" s="36" t="n">
+        <v>-7.3719476357749</v>
+      </c>
+      <c r="AS37" s="89" t="n">
+        <v>80.04109398944449</v>
+      </c>
+      <c r="AT37" s="33" t="n">
+        <v>0.02459103890654424</v>
+      </c>
+      <c r="AU37" s="33" t="n">
+        <v>0.01105879432798607</v>
+      </c>
+      <c r="AV37" s="33" t="n">
+        <v>0.3347039295392416</v>
+      </c>
+      <c r="AW37" s="33" t="n">
+        <v>0.06054346303398828</v>
+      </c>
       <c r="AX37" s="32" t="n"/>
       <c r="AY37" s="32" t="n"/>
       <c r="AZ37" s="32" t="n"/>
@@ -40479,7 +41049,7 @@
         <v>-0.01021530904350865</v>
       </c>
       <c r="D38" s="27" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E38" s="23" t="inlineStr">
         <is>
@@ -40655,7 +41225,7 @@
         <v>2.819440616108615e-05</v>
       </c>
       <c r="D39" s="34" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E39" s="30" t="inlineStr">
         <is>
@@ -40831,7 +41401,7 @@
         <v>-0.006214281861670612</v>
       </c>
       <c r="D40" s="27" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E40" s="23" t="inlineStr">
         <is>
@@ -41007,7 +41577,7 @@
         <v>-0.01024183768773135</v>
       </c>
       <c r="D41" s="34" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E41" s="30" t="inlineStr">
         <is>
@@ -41183,7 +41753,7 @@
         <v>-0.0212354556607246</v>
       </c>
       <c r="D42" s="27" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E42" s="23" t="inlineStr">
         <is>
@@ -41359,7 +41929,7 @@
         <v>0.00514941302923666</v>
       </c>
       <c r="D43" s="34" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E43" s="30" t="inlineStr">
         <is>
@@ -41535,7 +42105,7 @@
         <v>0.000427885920374127</v>
       </c>
       <c r="D44" s="27" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E44" s="23" t="inlineStr">
         <is>
@@ -41711,7 +42281,7 @@
         <v>-0.0003259794426572205</v>
       </c>
       <c r="D45" s="34" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E45" s="30" t="inlineStr">
         <is>
@@ -41887,7 +42457,7 @@
         <v>-0.0002868958958671675</v>
       </c>
       <c r="D46" s="27" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E46" s="23" t="inlineStr">
         <is>
@@ -42063,7 +42633,7 @@
         <v>0.00585630655444791</v>
       </c>
       <c r="D47" s="34" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E47" s="30" t="inlineStr">
         <is>
@@ -42239,7 +42809,7 @@
         <v>0.005583270720864064</v>
       </c>
       <c r="D48" s="27" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E48" s="23" t="inlineStr">
         <is>
@@ -43294,7 +43864,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:G48"/>
+  <dimension ref="B2:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -43976,12 +44546,12 @@
     <row r="28">
       <c r="B28" s="24" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="C28" s="101" t="inlineStr">
         <is>
-          <t>State Street SPDR S&amp;P 500 ETF Trust</t>
+          <t>Microsoft Corporation</t>
         </is>
       </c>
       <c r="D28" s="104" t="inlineStr">
@@ -43990,7 +44560,7 @@
         </is>
       </c>
       <c r="E28" s="26" t="n">
-        <v>0.005497992684414754</v>
+        <v>0.007844920169552072</v>
       </c>
       <c r="F28" s="27" t="n">
         <v>8</v>
@@ -44004,21 +44574,21 @@
     <row r="29">
       <c r="B29" s="31" t="inlineStr">
         <is>
-          <t>XLK</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="C29" s="102" t="inlineStr">
         <is>
-          <t>State Street Technology Select Sector SPDR ETF</t>
-        </is>
-      </c>
-      <c r="D29" s="107" t="inlineStr">
-        <is>
-          <t>RSI overbought (72)</t>
+          <t>State Street SPDR S&amp;P 500 ETF Trust</t>
+        </is>
+      </c>
+      <c r="D29" s="105" t="inlineStr">
+        <is>
+          <t>Closed above upper band</t>
         </is>
       </c>
       <c r="E29" s="33" t="n">
-        <v>0.005325274290659543</v>
+        <v>0.005497992684414754</v>
       </c>
       <c r="F29" s="34" t="n">
         <v>8</v>
@@ -44032,21 +44602,21 @@
     <row r="30">
       <c r="B30" s="24" t="inlineStr">
         <is>
-          <t>SOXL</t>
+          <t>XLK</t>
         </is>
       </c>
       <c r="C30" s="101" t="inlineStr">
         <is>
-          <t>Direxion Daily Semiconductor Bull 3X Shares</t>
+          <t>State Street Technology Select Sector SPDR ETF</t>
         </is>
       </c>
       <c r="D30" s="106" t="inlineStr">
         <is>
-          <t>Gapped up 1.9% at the open</t>
+          <t>RSI overbought (72)</t>
         </is>
       </c>
       <c r="E30" s="26" t="n">
-        <v>-6.093483511693254e-05</v>
+        <v>0.005325274290659543</v>
       </c>
       <c r="F30" s="27" t="n">
         <v>8</v>
@@ -44060,28 +44630,28 @@
     <row r="31">
       <c r="B31" s="31" t="inlineStr">
         <is>
-          <t>CCJ</t>
+          <t>SOXL</t>
         </is>
       </c>
       <c r="C31" s="102" t="inlineStr">
         <is>
-          <t>Cameco Corporation</t>
-        </is>
-      </c>
-      <c r="D31" s="105" t="inlineStr">
-        <is>
-          <t>MACD crossed up</t>
+          <t>Direxion Daily Semiconductor Bull 3X Shares</t>
+        </is>
+      </c>
+      <c r="D31" s="107" t="inlineStr">
+        <is>
+          <t>Gapped up 1.9% at the open</t>
         </is>
       </c>
       <c r="E31" s="33" t="n">
-        <v>0.06345027260671476</v>
+        <v>-6.093483511693254e-05</v>
       </c>
       <c r="F31" s="34" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G31" s="30" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Very Strong</t>
         </is>
       </c>
     </row>
@@ -44096,9 +44666,9 @@
           <t>Cameco Corporation</t>
         </is>
       </c>
-      <c r="D32" s="106" t="inlineStr">
-        <is>
-          <t>Volume 1.9x its 20-day average</t>
+      <c r="D32" s="104" t="inlineStr">
+        <is>
+          <t>MACD crossed up</t>
         </is>
       </c>
       <c r="E32" s="26" t="n">
@@ -44126,7 +44696,7 @@
       </c>
       <c r="D33" s="107" t="inlineStr">
         <is>
-          <t>RSI crossed back above 50</t>
+          <t>Volume 1.9x its 20-day average</t>
         </is>
       </c>
       <c r="E33" s="33" t="n">
@@ -44154,7 +44724,7 @@
       </c>
       <c r="D34" s="106" t="inlineStr">
         <is>
-          <t>Gapped up 2.4% at the open</t>
+          <t>RSI crossed back above 50</t>
         </is>
       </c>
       <c r="E34" s="26" t="n">
@@ -44172,21 +44742,21 @@
     <row r="35">
       <c r="B35" s="31" t="inlineStr">
         <is>
-          <t>XLU</t>
+          <t>CCJ</t>
         </is>
       </c>
       <c r="C35" s="102" t="inlineStr">
         <is>
-          <t>State Street Utilities Select Sector SPDR ETF</t>
+          <t>Cameco Corporation</t>
         </is>
       </c>
       <c r="D35" s="107" t="inlineStr">
         <is>
-          <t>RSI crossed back above 50</t>
+          <t>Gapped up 2.4% at the open</t>
         </is>
       </c>
       <c r="E35" s="33" t="n">
-        <v>0.02977229397963099</v>
+        <v>0.06345027260671476</v>
       </c>
       <c r="F35" s="34" t="n">
         <v>7</v>
@@ -44200,12 +44770,12 @@
     <row r="36">
       <c r="B36" s="24" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>XLU</t>
         </is>
       </c>
       <c r="C36" s="101" t="inlineStr">
         <is>
-          <t>Amazon.com, Inc.</t>
+          <t>State Street Utilities Select Sector SPDR ETF</t>
         </is>
       </c>
       <c r="D36" s="106" t="inlineStr">
@@ -44214,7 +44784,7 @@
         </is>
       </c>
       <c r="E36" s="26" t="n">
-        <v>0.01945113272536902</v>
+        <v>0.02977229397963099</v>
       </c>
       <c r="F36" s="27" t="n">
         <v>7</v>
@@ -44238,7 +44808,7 @@
       </c>
       <c r="D37" s="107" t="inlineStr">
         <is>
-          <t>Bands squeezing — a big move often follows</t>
+          <t>RSI crossed back above 50</t>
         </is>
       </c>
       <c r="E37" s="33" t="n">
@@ -44256,21 +44826,21 @@
     <row r="38">
       <c r="B38" s="24" t="inlineStr">
         <is>
-          <t>TSLA</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="C38" s="101" t="inlineStr">
         <is>
-          <t>Tesla, Inc.</t>
-        </is>
-      </c>
-      <c r="D38" s="104" t="inlineStr">
-        <is>
-          <t>MACD crossed up</t>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="D38" s="106" t="inlineStr">
+        <is>
+          <t>Bands squeezing — a big move often follows</t>
         </is>
       </c>
       <c r="E38" s="26" t="n">
-        <v>0.00514873823802553</v>
+        <v>0.01945113272536902</v>
       </c>
       <c r="F38" s="27" t="n">
         <v>7</v>
@@ -44284,21 +44854,21 @@
     <row r="39">
       <c r="B39" s="31" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>TSLA</t>
         </is>
       </c>
       <c r="C39" s="102" t="inlineStr">
         <is>
-          <t>Apple Inc.</t>
-        </is>
-      </c>
-      <c r="D39" s="107" t="inlineStr">
-        <is>
-          <t>Bands squeezing — a big move often follows</t>
+          <t>Tesla, Inc.</t>
+        </is>
+      </c>
+      <c r="D39" s="105" t="inlineStr">
+        <is>
+          <t>MACD crossed up</t>
         </is>
       </c>
       <c r="E39" s="33" t="n">
-        <v>0.002222927098478822</v>
+        <v>0.00514873823802553</v>
       </c>
       <c r="F39" s="34" t="n">
         <v>7</v>
@@ -44312,21 +44882,21 @@
     <row r="40">
       <c r="B40" s="24" t="inlineStr">
         <is>
-          <t>ARKK</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="C40" s="101" t="inlineStr">
         <is>
-          <t>ARK Innovation ETF</t>
+          <t>Apple Inc.</t>
         </is>
       </c>
       <c r="D40" s="106" t="inlineStr">
         <is>
-          <t>MACD crossed down</t>
+          <t>Bands squeezing — a big move often follows</t>
         </is>
       </c>
       <c r="E40" s="26" t="n">
-        <v>-0.02468205373633114</v>
+        <v>0.002222927098478822</v>
       </c>
       <c r="F40" s="27" t="n">
         <v>7</v>
@@ -44340,12 +44910,12 @@
     <row r="41">
       <c r="B41" s="31" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>ARKK</t>
         </is>
       </c>
       <c r="C41" s="102" t="inlineStr">
         <is>
-          <t>Micron Technology, Inc.</t>
+          <t>ARK Innovation ETF</t>
         </is>
       </c>
       <c r="D41" s="107" t="inlineStr">
@@ -44354,10 +44924,10 @@
         </is>
       </c>
       <c r="E41" s="33" t="n">
-        <v>-0.0172937920779811</v>
+        <v>-0.02468205373633114</v>
       </c>
       <c r="F41" s="34" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G41" s="30" t="inlineStr">
         <is>
@@ -44368,80 +44938,80 @@
     <row r="42">
       <c r="B42" s="24" t="inlineStr">
         <is>
-          <t>XLI</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="C42" s="101" t="inlineStr">
         <is>
-          <t>State Street Industrial Select Sector SPDR ETF</t>
+          <t>Micron Technology, Inc.</t>
         </is>
       </c>
       <c r="D42" s="106" t="inlineStr">
         <is>
-          <t>Bands squeezing — a big move often follows</t>
+          <t>MACD crossed down</t>
         </is>
       </c>
       <c r="E42" s="26" t="n">
-        <v>0.008700738826772358</v>
+        <v>-0.0172937920779811</v>
       </c>
       <c r="F42" s="27" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G42" s="23" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Strong</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="31" t="inlineStr">
         <is>
-          <t>XLB</t>
+          <t>XLI</t>
         </is>
       </c>
       <c r="C43" s="102" t="inlineStr">
         <is>
-          <t>State Street Materials Select Sector SPDR ETF</t>
-        </is>
-      </c>
-      <c r="D43" s="105" t="inlineStr">
-        <is>
-          <t>MACD crossed up</t>
+          <t>State Street Industrial Select Sector SPDR ETF</t>
+        </is>
+      </c>
+      <c r="D43" s="107" t="inlineStr">
+        <is>
+          <t>Bands squeezing — a big move often follows</t>
         </is>
       </c>
       <c r="E43" s="33" t="n">
-        <v>0.004646455398713778</v>
+        <v>0.008700738826772358</v>
       </c>
       <c r="F43" s="34" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G43" s="30" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="B44" s="24" t="inlineStr">
         <is>
-          <t>IREN</t>
+          <t>XLB</t>
         </is>
       </c>
       <c r="C44" s="101" t="inlineStr">
         <is>
-          <t>IREN Limited</t>
-        </is>
-      </c>
-      <c r="D44" s="106" t="inlineStr">
-        <is>
-          <t>Bands squeezing — a big move often follows</t>
+          <t>State Street Materials Select Sector SPDR ETF</t>
+        </is>
+      </c>
+      <c r="D44" s="104" t="inlineStr">
+        <is>
+          <t>MACD crossed up</t>
         </is>
       </c>
       <c r="E44" s="26" t="n">
-        <v>0.01976282722596956</v>
+        <v>0.004646455398713778</v>
       </c>
       <c r="F44" s="27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G44" s="23" t="inlineStr">
         <is>
@@ -44452,24 +45022,24 @@
     <row r="45">
       <c r="B45" s="31" t="inlineStr">
         <is>
-          <t>XLC</t>
+          <t>SNDK</t>
         </is>
       </c>
       <c r="C45" s="102" t="inlineStr">
         <is>
-          <t>State Street Communication Services Select Sector SPDR ETF</t>
+          <t>Sandisk Corporation</t>
         </is>
       </c>
       <c r="D45" s="107" t="inlineStr">
         <is>
-          <t>Lost the 50 DMA</t>
+          <t>RSI dropped below 50</t>
         </is>
       </c>
       <c r="E45" s="33" t="n">
-        <v>0.0003583990261499803</v>
+        <v>-0.02564317456442577</v>
       </c>
       <c r="F45" s="34" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G45" s="30" t="inlineStr">
         <is>
@@ -44480,12 +45050,12 @@
     <row r="46">
       <c r="B46" s="24" t="inlineStr">
         <is>
-          <t>XLV</t>
+          <t>SNDK</t>
         </is>
       </c>
       <c r="C46" s="101" t="inlineStr">
         <is>
-          <t>State Street Health Care Select Sector SPDR ETF</t>
+          <t>Sandisk Corporation</t>
         </is>
       </c>
       <c r="D46" s="106" t="inlineStr">
@@ -44494,10 +45064,10 @@
         </is>
       </c>
       <c r="E46" s="26" t="n">
-        <v>-0.001672932947753392</v>
+        <v>-0.02564317456442577</v>
       </c>
       <c r="F46" s="27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G46" s="23" t="inlineStr">
         <is>
@@ -44508,21 +45078,21 @@
     <row r="47">
       <c r="B47" s="31" t="inlineStr">
         <is>
-          <t>SNDK</t>
+          <t>IREN</t>
         </is>
       </c>
       <c r="C47" s="102" t="inlineStr">
         <is>
-          <t>Sandisk Corporation</t>
+          <t>IREN Limited</t>
         </is>
       </c>
       <c r="D47" s="107" t="inlineStr">
         <is>
-          <t>RSI dropped below 50</t>
+          <t>Bands squeezing — a big move often follows</t>
         </is>
       </c>
       <c r="E47" s="33" t="n">
-        <v>-0.02564317456442577</v>
+        <v>0.01976282722596956</v>
       </c>
       <c r="F47" s="34" t="n">
         <v>2</v>
@@ -44536,21 +45106,21 @@
     <row r="48">
       <c r="B48" s="24" t="inlineStr">
         <is>
-          <t>SNDK</t>
+          <t>XLC</t>
         </is>
       </c>
       <c r="C48" s="101" t="inlineStr">
         <is>
-          <t>Sandisk Corporation</t>
+          <t>State Street Communication Services Select Sector SPDR ETF</t>
         </is>
       </c>
       <c r="D48" s="106" t="inlineStr">
         <is>
-          <t>Bands squeezing — a big move often follows</t>
+          <t>Lost the 50 DMA</t>
         </is>
       </c>
       <c r="E48" s="26" t="n">
-        <v>-0.02564317456442577</v>
+        <v>0.0003583990261499803</v>
       </c>
       <c r="F48" s="27" t="n">
         <v>2</v>
@@ -44561,12 +45131,40 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="B49" s="31" t="inlineStr">
+        <is>
+          <t>XLV</t>
+        </is>
+      </c>
+      <c r="C49" s="102" t="inlineStr">
+        <is>
+          <t>State Street Health Care Select Sector SPDR ETF</t>
+        </is>
+      </c>
+      <c r="D49" s="107" t="inlineStr">
+        <is>
+          <t>Bands squeezing — a big move often follows</t>
+        </is>
+      </c>
+      <c r="E49" s="33" t="n">
+        <v>-0.001672932947753392</v>
+      </c>
+      <c r="F49" s="34" t="n">
+        <v>2</v>
+      </c>
+      <c r="G49" s="30" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="B5:G48"/>
+  <autoFilter ref="B5:G49"/>
   <mergeCells count="1">
     <mergeCell ref="B2:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="E6:E48">
+  <conditionalFormatting sqref="E6:E49">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="-0.05"/>

</xml_diff>

<commit_message>
Daily workbook: 2026-10-08 00:57 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 8 Oct 2026, 12:14 AM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 8 Oct 2026, 12:57 AM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 8 Oct 2026, 12:14 AM · Yahoo Finance data</t>
+          <t>Built 8 Oct 2026, 12:57 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
+          <t>Jensen Huang Said Nvidia Now Has "a Lot Greater Visibility" Into Demand, Letting It Forecast a Full Year Ah...</t>
+        </is>
+      </c>
+      <c r="AY43" s="90" t="inlineStr">
+        <is>
           <t>Think You Missed Out on Nvidia's Stock Rise? Think Again.</t>
         </is>
       </c>
-      <c r="AY43" s="90" t="inlineStr">
+      <c r="AZ43" s="90" t="inlineStr">
         <is>
           <t>Robot data startup Mecka AI nabs $60M from Sequoia</t>
-        </is>
-      </c>
-      <c r="AZ43" s="90" t="inlineStr">
-        <is>
-          <t>Why NorthWestern Energy Group Stock Soared on Wednesday</t>
         </is>
       </c>
     </row>
@@ -10537,12 +10537,12 @@
       </c>
       <c r="AY45" s="90" t="inlineStr">
         <is>
+          <t>Why Did QUALCOMM (QCOM) Stock Drop After Its Latest Update?</t>
+        </is>
+      </c>
+      <c r="AZ45" s="90" t="inlineStr">
+        <is>
           <t>Broadcom vs. Qualcomm: Rapid Growth vs. Flat Revenue</t>
-        </is>
-      </c>
-      <c r="AZ45" s="90" t="inlineStr">
-        <is>
-          <t>Processors and Graphics Chips Stocks Q2 Results: Benchmarking Qualcomm (NASDAQ:QCOM)</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 8 Oct 2026, 12:14 AM · Yahoo Finance data</t>
+          <t>Built 8 Oct 2026, 12:57 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 8 Oct 2026, 12:14 AM · Yahoo Finance data</t>
+          <t>Built 8 Oct 2026, 12:57 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 8 Oct 2026, 12:14 AM · Yahoo Finance data</t>
+          <t>Built 8 Oct 2026, 12:57 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 8 Oct 2026, 12:14 AM · Yahoo Finance data</t>
+          <t>Built 8 Oct 2026, 12:57 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-10-09 01:12 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 9 Oct 2026, 12:25 AM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 9 Oct 2026, 01:12 AM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 9 Oct 2026, 12:25 AM · Yahoo Finance data</t>
+          <t>Built 9 Oct 2026, 01:12 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -7524,17 +7524,17 @@
       </c>
       <c r="AX29" s="90" t="inlineStr">
         <is>
+          <t>AST SpaceMobile (ASTS) Could Be 67% Undervalued On TELUS Integration Progress</t>
+        </is>
+      </c>
+      <c r="AY29" s="90" t="inlineStr">
+        <is>
           <t>ASTS, SPCX And NN Stocks Slide: Clear Street Calls FCC Meeting Agenda Mixed For AST SpaceMobile</t>
         </is>
       </c>
-      <c r="AY29" s="90" t="inlineStr">
+      <c r="AZ29" s="90" t="inlineStr">
         <is>
           <t>AST SpaceMobile Sinks 7% as Satellite Rival Clears Regulatory Hurdle; Rocket Lab Drops 4%, Planet Labs Fall...</t>
-        </is>
-      </c>
-      <c r="AZ29" s="90" t="inlineStr">
-        <is>
-          <t>AST SpaceMobile Got U.S.-Japan Backing. Wall Street Still Sees $3.2 Billion of Cash Burn Before 2029</t>
         </is>
       </c>
     </row>
@@ -8840,17 +8840,17 @@
       </c>
       <c r="AX36" s="79" t="inlineStr">
         <is>
+          <t>AMD CEO delivers stark warning on chip market’s future</t>
+        </is>
+      </c>
+      <c r="AY36" s="79" t="inlineStr">
+        <is>
+          <t>Intel CEO Lip-Bu Tan Says Company Will Keep Working on Terafab — Elon Musk Confirms TSMC May Only Sublease ...</t>
+        </is>
+      </c>
+      <c r="AZ36" s="79" t="inlineStr">
+        <is>
           <t>Prediction: This Will Happen to Intel Stock in 2027</t>
-        </is>
-      </c>
-      <c r="AY36" s="79" t="inlineStr">
-        <is>
-          <t>Anaconda Expands Collaboration with Intel to Give Enterprises a Secure Path to Production AI</t>
-        </is>
-      </c>
-      <c r="AZ36" s="79" t="inlineStr">
-        <is>
-          <t>Intel (INTC): Buy, Sell, or Hold Post Q2 Earnings?</t>
         </is>
       </c>
     </row>
@@ -10720,17 +10720,17 @@
       </c>
       <c r="AX46" s="79" t="inlineStr">
         <is>
+          <t>BA, SPCX, RKLB, RTX, PLTR Stock In Focus: Why Barclays Is Overweight On Aerospace And Defense Stocks?</t>
+        </is>
+      </c>
+      <c r="AY46" s="79" t="inlineStr">
+        <is>
           <t>Rocket Lab Fell Hard Over The Last 3 Months: Wall Street Pro Predicts It Doubles From Today</t>
         </is>
       </c>
-      <c r="AY46" s="79" t="inlineStr">
+      <c r="AZ46" s="79" t="inlineStr">
         <is>
           <t>AST SpaceMobile Sinks 7% as Satellite Rival Clears Regulatory Hurdle; Rocket Lab Drops 4%, Planet Labs Fall...</t>
-        </is>
-      </c>
-      <c r="AZ46" s="79" t="inlineStr">
-        <is>
-          <t>Not SpaceX. Not Blue Origin. The Space Titan That Morgan Stanley Calls an Undervalued Launch Play.</t>
         </is>
       </c>
     </row>
@@ -11096,17 +11096,17 @@
       </c>
       <c r="AX48" s="79" t="inlineStr">
         <is>
-          <t>Securitize's tokenized US stock trading is here, bringing Nvidia, Tesla, &amp; Apple to Solana</t>
+          <t>Cathie Wood Says Follow the AI Agents. Her Own Filings Show Where ARK Was Looking</t>
         </is>
       </c>
       <c r="AY48" s="79" t="inlineStr">
         <is>
-          <t>Cathie Wood Says Follow the AI Agents. Her Own Filings Show Where ARK Was Looking</t>
+          <t>Pilot and Tesla Open First Megacharger Site, Announce Three Additional Locations Opening Soon</t>
         </is>
       </c>
       <c r="AZ48" s="79" t="inlineStr">
         <is>
-          <t>Pilot and Tesla Open First Megacharger Site, Announce Three Additional Locations Opening Soon</t>
+          <t>Tesla (TSLA) Deliveries Beat Expectations. But TSLA’s 159x Forward P/E Is Betting on Much More</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 9 Oct 2026, 12:25 AM · Yahoo Finance data</t>
+          <t>Built 9 Oct 2026, 01:12 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 9 Oct 2026, 12:25 AM · Yahoo Finance data</t>
+          <t>Built 9 Oct 2026, 01:12 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 9 Oct 2026, 12:25 AM · Yahoo Finance data</t>
+          <t>Built 9 Oct 2026, 01:12 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 9 Oct 2026, 12:25 AM · Yahoo Finance data</t>
+          <t>Built 9 Oct 2026, 01:12 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-10-10 00:47 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1299,7 +1299,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 10 Oct 2026, 12:04 AM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 10 Oct 2026, 12:47 AM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3104,7 +3104,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 10 Oct 2026, 12:04 AM · Yahoo Finance data</t>
+          <t>Built 10 Oct 2026, 12:47 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -10158,12 +10158,12 @@
       </c>
       <c r="AY43" s="90" t="inlineStr">
         <is>
+          <t>What Is Physical AI? Nvidia Is the Stock I'd Buy to Own It.</t>
+        </is>
+      </c>
+      <c r="AZ43" s="90" t="inlineStr">
+        <is>
           <t>Why CrowdStrike Holdings Stock Crushed it on Friday</t>
-        </is>
-      </c>
-      <c r="AZ43" s="90" t="inlineStr">
-        <is>
-          <t>Elon Musk Just Made a Surprising Statement About AI Chips. Here's the Stock It Helps.</t>
         </is>
       </c>
     </row>
@@ -10341,17 +10341,17 @@
       </c>
       <c r="AX44" s="79" t="inlineStr">
         <is>
+          <t>Why Palantir Stock Powered to a More Than 5% Gain Today</t>
+        </is>
+      </c>
+      <c r="AY44" s="79" t="inlineStr">
+        <is>
+          <t>Why Goldman Sachs Thinks You Should Buy the Palantir Stock Dip</t>
+        </is>
+      </c>
+      <c r="AZ44" s="79" t="inlineStr">
+        <is>
           <t>Better High-Growth AI Stock: CrowdStrike vs. Palantir Technologies</t>
-        </is>
-      </c>
-      <c r="AY44" s="79" t="inlineStr">
-        <is>
-          <t>Goldman Predicts a “Step Function Change” in Palantir’s AI Opportunity</t>
-        </is>
-      </c>
-      <c r="AZ44" s="79" t="inlineStr">
-        <is>
-          <t>Goldman Sachs Upgrades Palantir to Buy, Sees 18% Upside and Further Outperformance Into 2027</t>
         </is>
       </c>
     </row>
@@ -11103,7 +11103,7 @@
       </c>
       <c r="AZ48" s="79" t="inlineStr">
         <is>
-          <t>Tesla’s China-Made EV Sales Hit 2026 High In September – Yorkville Says TSLA Is One Of The Clearest Ways To...</t>
+          <t>Elon Musk Sees SpaceX Stock Rising to Crazy Levels. He Once Made Similar Predictions for TSLA Too</t>
         </is>
       </c>
     </row>
@@ -11640,7 +11640,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 10 Oct 2026, 12:04 AM · Yahoo Finance data</t>
+          <t>Built 10 Oct 2026, 12:47 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19576,7 +19576,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 10 Oct 2026, 12:04 AM · Yahoo Finance data</t>
+          <t>Built 10 Oct 2026, 12:47 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27512,7 +27512,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 10 Oct 2026, 12:04 AM · Yahoo Finance data</t>
+          <t>Built 10 Oct 2026, 12:47 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35448,7 +35448,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 10 Oct 2026, 12:04 AM · Yahoo Finance data</t>
+          <t>Built 10 Oct 2026, 12:47 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-10-13 02:03 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 12 Oct 2026, 11:43 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 13 Oct 2026, 02:03 AM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 12 Oct 2026, 11:43 PM · Yahoo Finance data</t>
+          <t>Built 13 Oct 2026, 02:03 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -3548,7 +3548,7 @@
       </c>
       <c r="F7" s="23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Same</t>
         </is>
       </c>
       <c r="G7" s="23" t="inlineStr">
@@ -3614,16 +3614,16 @@
         <v>169.0200042724609</v>
       </c>
       <c r="U7" s="72" t="n">
-        <v>170.0399932861328</v>
+        <v>170.0599975585938</v>
       </c>
       <c r="V7" s="72" t="n">
         <v>168.8300018310547</v>
       </c>
       <c r="W7" s="73" t="n">
-        <v>3648383</v>
+        <v>3802400</v>
       </c>
       <c r="X7" s="74" t="n">
-        <v>0.4984603625195709</v>
+        <v>0.5189569271482686</v>
       </c>
       <c r="Y7" s="28" t="n">
         <v>43.99992293313758</v>
@@ -3632,7 +3632,7 @@
         <v>48.21427686759045</v>
       </c>
       <c r="AA7" s="28" t="n">
-        <v>27.3159441369652</v>
+        <v>27.30530429066492</v>
       </c>
       <c r="AB7" s="75" t="n">
         <v>-1.483424470630837</v>
@@ -3674,7 +3674,7 @@
         <v>2.346229976245372</v>
       </c>
       <c r="AO7" s="77" t="n">
-        <v>1.384599275672566</v>
+        <v>1.385444015049398</v>
       </c>
       <c r="AP7" s="72" t="n">
         <v>188.1900024414062</v>
@@ -3810,10 +3810,10 @@
         <v>170.8500061035156</v>
       </c>
       <c r="W8" s="84" t="n">
-        <v>5822841</v>
+        <v>5826800</v>
       </c>
       <c r="X8" s="85" t="n">
-        <v>0.7243531446508353</v>
+        <v>0.724827789958172</v>
       </c>
       <c r="Y8" s="35" t="n">
         <v>60.04508064742269</v>
@@ -4000,10 +4000,10 @@
         <v>54.83000183105469</v>
       </c>
       <c r="W9" s="73" t="n">
-        <v>19551603</v>
+        <v>19644200</v>
       </c>
       <c r="X9" s="74" t="n">
-        <v>0.5143801647813432</v>
+        <v>0.5167370978157795</v>
       </c>
       <c r="Y9" s="28" t="n">
         <v>49.2757119428642</v>
@@ -4187,13 +4187,13 @@
         <v>66.41999816894531</v>
       </c>
       <c r="V10" s="83" t="n">
-        <v>65.66500091552734</v>
+        <v>65.66999816894531</v>
       </c>
       <c r="W10" s="84" t="n">
-        <v>19840595</v>
+        <v>19855300</v>
       </c>
       <c r="X10" s="85" t="n">
-        <v>0.5827383665659366</v>
+        <v>0.5831576739952614</v>
       </c>
       <c r="Y10" s="35" t="n">
         <v>65.4654781708585</v>
@@ -4380,10 +4380,10 @@
         <v>83.38999938964844</v>
       </c>
       <c r="W11" s="73" t="n">
-        <v>7274524</v>
+        <v>7324100</v>
       </c>
       <c r="X11" s="74" t="n">
-        <v>0.680214165441079</v>
+        <v>0.6846248939635772</v>
       </c>
       <c r="Y11" s="28" t="n">
         <v>59.91834597677683</v>
@@ -4567,13 +4567,13 @@
         <v>112.8600006103516</v>
       </c>
       <c r="V12" s="83" t="n">
-        <v>112.0950012207031</v>
+        <v>112.0999984741211</v>
       </c>
       <c r="W12" s="84" t="n">
-        <v>3919370</v>
+        <v>3936600</v>
       </c>
       <c r="X12" s="85" t="n">
-        <v>0.5827779139546224</v>
+        <v>0.5852649012776188</v>
       </c>
       <c r="Y12" s="35" t="n">
         <v>51.66799137565226</v>
@@ -4582,7 +4582,7 @@
         <v>85.5999755859375</v>
       </c>
       <c r="AA12" s="35" t="n">
-        <v>19.31633569508231</v>
+        <v>19.320228603571</v>
       </c>
       <c r="AB12" s="86" t="n">
         <v>-0.5566494184845112</v>
@@ -4624,7 +4624,7 @@
         <v>4.296566230942043</v>
       </c>
       <c r="AO12" s="88" t="n">
-        <v>1.232295292532498</v>
+        <v>1.231977356589338</v>
       </c>
       <c r="AP12" s="83" t="n">
         <v>125.0100021362305</v>
@@ -4760,10 +4760,10 @@
         <v>110.9499969482422</v>
       </c>
       <c r="W13" s="73" t="n">
-        <v>7157995</v>
+        <v>7171200</v>
       </c>
       <c r="X13" s="74" t="n">
-        <v>1.121120444608048</v>
+        <v>1.12307253803243</v>
       </c>
       <c r="Y13" s="28" t="n">
         <v>48.98612684691692</v>
@@ -4944,16 +4944,16 @@
         <v>49.2400016784668</v>
       </c>
       <c r="U14" s="83" t="n">
-        <v>49.76010131835938</v>
+        <v>49.7599983215332</v>
       </c>
       <c r="V14" s="83" t="n">
         <v>49.15999984741211</v>
       </c>
       <c r="W14" s="84" t="n">
-        <v>5789367</v>
+        <v>5798000</v>
       </c>
       <c r="X14" s="85" t="n">
-        <v>0.5035467680641833</v>
+        <v>0.5042787153156177</v>
       </c>
       <c r="Y14" s="35" t="n">
         <v>43.46793716284411</v>
@@ -4962,7 +4962,7 @@
         <v>59.70686911114744</v>
       </c>
       <c r="AA14" s="35" t="n">
-        <v>20.19546303103422</v>
+        <v>20.19563015662768</v>
       </c>
       <c r="AB14" s="86" t="n">
         <v>-0.5747866114742095</v>
@@ -5004,7 +5004,7 @@
         <v>5.068976114256403</v>
       </c>
       <c r="AO14" s="88" t="n">
-        <v>1.483343570683938</v>
+        <v>1.483328690189683</v>
       </c>
       <c r="AP14" s="83" t="n">
         <v>54.18999862670898</v>
@@ -5140,10 +5140,10 @@
         <v>195.8200073242188</v>
       </c>
       <c r="W15" s="73" t="n">
-        <v>5115645</v>
+        <v>5200700</v>
       </c>
       <c r="X15" s="74" t="n">
-        <v>0.7030565601594686</v>
+        <v>0.7143283916245281</v>
       </c>
       <c r="Y15" s="28" t="n">
         <v>55.14458776420557</v>
@@ -5330,10 +5330,10 @@
         <v>41.46500015258789</v>
       </c>
       <c r="W16" s="84" t="n">
-        <v>8317565</v>
+        <v>8421800</v>
       </c>
       <c r="X16" s="85" t="n">
-        <v>1.213984628746734</v>
+        <v>1.228263865695739</v>
       </c>
       <c r="Y16" s="35" t="n">
         <v>48.01817642289245</v>
@@ -5520,10 +5520,10 @@
         <v>41.20000076293945</v>
       </c>
       <c r="W17" s="73" t="n">
-        <v>16544305</v>
+        <v>16550400</v>
       </c>
       <c r="X17" s="74" t="n">
-        <v>0.4897661332118749</v>
+        <v>0.4899421452997108</v>
       </c>
       <c r="Y17" s="28" t="n">
         <v>55.66455029895977</v>
@@ -5723,16 +5723,16 @@
         <v>778.780029296875</v>
       </c>
       <c r="U19" s="72" t="n">
-        <v>779.39697265625</v>
+        <v>779.4000244140625</v>
       </c>
       <c r="V19" s="72" t="n">
         <v>777.0499877929688</v>
       </c>
       <c r="W19" s="73" t="n">
-        <v>18392278</v>
+        <v>18639800</v>
       </c>
       <c r="X19" s="74" t="n">
-        <v>0.4226207227132978</v>
+        <v>0.4281727851927809</v>
       </c>
       <c r="Y19" s="28" t="n">
         <v>59.33134082336289</v>
@@ -5783,7 +5783,7 @@
         <v>3.687166529766521</v>
       </c>
       <c r="AO19" s="77" t="n">
-        <v>0.8107424405553274</v>
+        <v>0.810770455297357</v>
       </c>
       <c r="AP19" s="72" t="n">
         <v>781.6199951171875</v>
@@ -5811,7 +5811,7 @@
       </c>
       <c r="AX19" s="79" t="inlineStr">
         <is>
-          <t>Salesforce at $229: One Of The Most Unpredictable AI Plays There Is</t>
+          <t>ServiceNow (NOW) Grew Revenue 24% While Earnings Fell 22.60%. Where Did the Profit Go?</t>
         </is>
       </c>
       <c r="AY19" s="79" t="inlineStr">
@@ -5908,19 +5908,19 @@
         <v>-5.23004150390625</v>
       </c>
       <c r="T20" s="83" t="n">
-        <v>749.6400146484375</v>
+        <v>749.6900024414062</v>
       </c>
       <c r="U20" s="83" t="n">
         <v>749.7899780273438</v>
       </c>
       <c r="V20" s="83" t="n">
-        <v>744.844970703125</v>
+        <v>744.8499755859375</v>
       </c>
       <c r="W20" s="84" t="n">
-        <v>24781235</v>
+        <v>24936300</v>
       </c>
       <c r="X20" s="85" t="n">
-        <v>0.7403319110313271</v>
+        <v>0.7447474299937327</v>
       </c>
       <c r="Y20" s="35" t="n">
         <v>56.5645773947613</v>
@@ -5929,7 +5929,7 @@
         <v>46.14147344392502</v>
       </c>
       <c r="AA20" s="35" t="n">
-        <v>13.31929729783367</v>
+        <v>13.31879357883253</v>
       </c>
       <c r="AB20" s="86" t="n">
         <v>8.835868629033371</v>
@@ -5971,7 +5971,7 @@
         <v>8.3359753790364</v>
       </c>
       <c r="AO20" s="88" t="n">
-        <v>1.201475384996289</v>
+        <v>1.201427466434283</v>
       </c>
       <c r="AP20" s="83" t="n">
         <v>762.8599853515625</v>
@@ -6102,13 +6102,13 @@
         <v>279.1400146484375</v>
       </c>
       <c r="V21" s="72" t="n">
-        <v>277.7950134277344</v>
+        <v>277.7900085449219</v>
       </c>
       <c r="W21" s="73" t="n">
-        <v>16630340</v>
+        <v>16752600</v>
       </c>
       <c r="X21" s="74" t="n">
-        <v>0.6693551142857224</v>
+        <v>0.6740901647804125</v>
       </c>
       <c r="Y21" s="28" t="n">
         <v>36.83536917654311</v>
@@ -6159,7 +6159,7 @@
         <v>4.159398668760494</v>
       </c>
       <c r="AO21" s="77" t="n">
-        <v>1.242214717860557</v>
+        <v>1.242343358248221</v>
       </c>
       <c r="AP21" s="72" t="n">
         <v>305.1799926757812</v>
@@ -6293,10 +6293,10 @@
         <v>127.2699966430664</v>
       </c>
       <c r="W22" s="84" t="n">
-        <v>57087700</v>
+        <v>57428800</v>
       </c>
       <c r="X22" s="85" t="n">
-        <v>0.9455709174461302</v>
+        <v>0.9507201942867028</v>
       </c>
       <c r="Y22" s="35" t="n">
         <v>43.37185951842583</v>
@@ -6493,7 +6493,7 @@
         <v>4.329986572265625</v>
       </c>
       <c r="T24" s="72" t="n">
-        <v>338.1600036621094</v>
+        <v>338.2200012207031</v>
       </c>
       <c r="U24" s="72" t="n">
         <v>342.6300048828125</v>
@@ -6502,10 +6502,10 @@
         <v>337.6000061035156</v>
       </c>
       <c r="W24" s="73" t="n">
-        <v>25796997</v>
+        <v>25848300</v>
       </c>
       <c r="X24" s="74" t="n">
-        <v>0.6953579348242687</v>
+        <v>0.6966680367358214</v>
       </c>
       <c r="Y24" s="28" t="n">
         <v>60.20673859193633</v>
@@ -6589,12 +6589,12 @@
       </c>
       <c r="AY24" s="79" t="inlineStr">
         <is>
+          <t>Dow Jones Futures: Micron, Nvidia Lead AI Trade Lower; Apple, Meta Rally Near Buy Points</t>
+        </is>
+      </c>
+      <c r="AZ24" s="79" t="inlineStr">
+        <is>
           <t>Apple Stock Scores Price-Target Hike Ahead Of Smart Home Launch</t>
-        </is>
-      </c>
-      <c r="AZ24" s="79" t="inlineStr">
-        <is>
-          <t>Apple co-founder's forgotten company lands Nasdaq deal</t>
         </is>
       </c>
     </row>
@@ -6681,7 +6681,7 @@
         <v>-13.8599853515625</v>
       </c>
       <c r="T25" s="83" t="n">
-        <v>599.8599853515625</v>
+        <v>599.9299926757812</v>
       </c>
       <c r="U25" s="83" t="n">
         <v>601.77001953125</v>
@@ -6690,10 +6690,10 @@
         <v>586.5399780273438</v>
       </c>
       <c r="W25" s="84" t="n">
-        <v>15252527</v>
+        <v>15327700</v>
       </c>
       <c r="X25" s="85" t="n">
-        <v>0.7041851007268116</v>
+        <v>0.7074694226266331</v>
       </c>
       <c r="Y25" s="35" t="n">
         <v>52.9837528694086</v>
@@ -6772,17 +6772,17 @@
       </c>
       <c r="AX25" s="90" t="inlineStr">
         <is>
+          <t>SNDK, MU, INTC, AMD, SKHY: Chip Stocks Extend Slide As AI Funding Concerns, China Competition Weigh On Sector</t>
+        </is>
+      </c>
+      <c r="AY25" s="90" t="inlineStr">
+        <is>
           <t>Why Advanced Micro Devices (AMD) Dipped More Than Broader Market Today</t>
         </is>
       </c>
-      <c r="AY25" s="90" t="inlineStr">
+      <c r="AZ25" s="90" t="inlineStr">
         <is>
           <t>Intel Is Up 174% in 2026 and AMD Is Up 175%: Take Profits, or Hold On for the Ride?</t>
-        </is>
-      </c>
-      <c r="AZ25" s="90" t="inlineStr">
-        <is>
-          <t>2 Reasons to Like AMD (and 1 Not So Much)</t>
         </is>
       </c>
     </row>
@@ -6869,7 +6869,7 @@
         <v>-2.899993896484375</v>
       </c>
       <c r="T26" s="72" t="n">
-        <v>262.5450134277344</v>
+        <v>262.5</v>
       </c>
       <c r="U26" s="72" t="n">
         <v>263.7000122070312</v>
@@ -6878,10 +6878,10 @@
         <v>259.2699890136719</v>
       </c>
       <c r="W26" s="73" t="n">
-        <v>25322105</v>
+        <v>26524900</v>
       </c>
       <c r="X26" s="74" t="n">
-        <v>0.6916972182418528</v>
+        <v>0.7233056926349615</v>
       </c>
       <c r="Y26" s="28" t="n">
         <v>55.57687470546155</v>
@@ -6960,17 +6960,17 @@
       </c>
       <c r="AX26" s="79" t="inlineStr">
         <is>
-          <t>The bull market’s four-year run, EV demand, and interest rates threaten earnings</t>
+          <t>/C O R R E C T I O N - Duracell/</t>
         </is>
       </c>
       <c r="AY26" s="79" t="inlineStr">
         <is>
-          <t>/C O R R E C T I O N - Duracell/</t>
+          <t>The Staggering Costs of a Single Data Center, From Land to Chips</t>
         </is>
       </c>
       <c r="AZ26" s="79" t="inlineStr">
         <is>
-          <t>The Staggering Costs of a Single Data Center, From Land to Chips</t>
+          <t>Better High-Yield Dividend Stock: UPS vs. Energy Transfer</t>
         </is>
       </c>
     </row>
@@ -7063,13 +7063,13 @@
         <v>89.48799896240234</v>
       </c>
       <c r="V27" s="83" t="n">
-        <v>87.58999633789062</v>
+        <v>87.58499908447266</v>
       </c>
       <c r="W27" s="84" t="n">
-        <v>2434618</v>
+        <v>2440700</v>
       </c>
       <c r="X27" s="85" t="n">
-        <v>0.523175935958719</v>
+        <v>0.5244486273700858</v>
       </c>
       <c r="Y27" s="35" t="n">
         <v>50.54385468883044</v>
@@ -7078,7 +7078,7 @@
         <v>17.32517552248608</v>
       </c>
       <c r="AA27" s="35" t="n">
-        <v>19.34269163790259</v>
+        <v>19.34022330840291</v>
       </c>
       <c r="AB27" s="86" t="n">
         <v>1.132883624033255</v>
@@ -7120,7 +7120,7 @@
         <v>10.60893842135828</v>
       </c>
       <c r="AO27" s="88" t="n">
-        <v>2.718703695019072</v>
+        <v>2.719109224087835</v>
       </c>
       <c r="AP27" s="83" t="n">
         <v>94.81999969482422</v>
@@ -7245,19 +7245,19 @@
         <v>-11.03999328613281</v>
       </c>
       <c r="T28" s="72" t="n">
-        <v>260.6499938964844</v>
+        <v>260.2999877929688</v>
       </c>
       <c r="U28" s="72" t="n">
-        <v>263.1199951171875</v>
+        <v>263.239990234375</v>
       </c>
       <c r="V28" s="72" t="n">
         <v>253.3399963378906</v>
       </c>
       <c r="W28" s="73" t="n">
-        <v>3581107</v>
+        <v>3585600</v>
       </c>
       <c r="X28" s="74" t="n">
-        <v>0.6185787076905389</v>
+        <v>0.6192339708274759</v>
       </c>
       <c r="Y28" s="28" t="n">
         <v>40.62046217058992</v>
@@ -7336,17 +7336,17 @@
       </c>
       <c r="AX28" s="79" t="inlineStr">
         <is>
+          <t>What Does Arm Holdings (ARM) Winning An AI Ecosystem Award Really Signal?</t>
+        </is>
+      </c>
+      <c r="AY28" s="79" t="inlineStr">
+        <is>
+          <t>AI Is Blowing Up Tech’s Money Rules. How Arm Could Make Qualcomm Pay More.</t>
+        </is>
+      </c>
+      <c r="AZ28" s="79" t="inlineStr">
+        <is>
           <t>Arm Holdings (ARM) Is Helping Reshape the Future of Computing: Here’s Why</t>
-        </is>
-      </c>
-      <c r="AY28" s="79" t="inlineStr">
-        <is>
-          <t>Arm Holdings plc (ARM) is Positioned as Specialized Computing Demand Outlasts Near-Term Shortages</t>
-        </is>
-      </c>
-      <c r="AZ28" s="79" t="inlineStr">
-        <is>
-          <t>Qualcomm and Arm Trial Ends in Hung Jury Over Licensing Breach Allegations</t>
         </is>
       </c>
     </row>
@@ -7433,7 +7433,7 @@
         <v>0.4949989318847656</v>
       </c>
       <c r="T29" s="83" t="n">
-        <v>53.35499954223633</v>
+        <v>53.2599983215332</v>
       </c>
       <c r="U29" s="83" t="n">
         <v>54.66999816894531</v>
@@ -7442,10 +7442,10 @@
         <v>51.31999969482422</v>
       </c>
       <c r="W29" s="84" t="n">
-        <v>21662884</v>
+        <v>21706700</v>
       </c>
       <c r="X29" s="85" t="n">
-        <v>1.520795314709436</v>
+        <v>1.522581079597644</v>
       </c>
       <c r="Y29" s="35" t="n">
         <v>36.68568372368077</v>
@@ -7621,19 +7621,19 @@
         <v>-6.80999755859375</v>
       </c>
       <c r="T30" s="72" t="n">
-        <v>359.7049865722656</v>
+        <v>359.4299926757812</v>
       </c>
       <c r="U30" s="72" t="n">
-        <v>360.6899108886719</v>
+        <v>360.6900024414062</v>
       </c>
       <c r="V30" s="72" t="n">
         <v>354.2200012207031</v>
       </c>
       <c r="W30" s="73" t="n">
-        <v>15703894</v>
+        <v>16284100</v>
       </c>
       <c r="X30" s="74" t="n">
-        <v>0.6772885848539576</v>
+        <v>0.7014071560836704</v>
       </c>
       <c r="Y30" s="28" t="n">
         <v>46.39896153805817</v>
@@ -7818,10 +7818,10 @@
         <v>85.69000244140625</v>
       </c>
       <c r="W31" s="84" t="n">
-        <v>1820192</v>
+        <v>1821500</v>
       </c>
       <c r="X31" s="85" t="n">
-        <v>0.5619247362072525</v>
+        <v>0.5623171851726081</v>
       </c>
       <c r="Y31" s="35" t="n">
         <v>40.65344038497854</v>
@@ -8006,10 +8006,10 @@
         <v>79.02999877929688</v>
       </c>
       <c r="W32" s="73" t="n">
-        <v>18858147</v>
+        <v>18873400</v>
       </c>
       <c r="X32" s="74" t="n">
-        <v>0.6293056874716687</v>
+        <v>0.6297221697177554</v>
       </c>
       <c r="Y32" s="28" t="n">
         <v>41.65623250329339</v>
@@ -8188,16 +8188,16 @@
         <v>581.72998046875</v>
       </c>
       <c r="U33" s="83" t="n">
-        <v>585.32373046875</v>
+        <v>585.3200073242188</v>
       </c>
       <c r="V33" s="83" t="n">
-        <v>565.3499755859375</v>
+        <v>565</v>
       </c>
       <c r="W33" s="84" t="n">
-        <v>5231750</v>
+        <v>5238700</v>
       </c>
       <c r="X33" s="85" t="n">
-        <v>0.7182555386195779</v>
+        <v>0.7190983782641133</v>
       </c>
       <c r="Y33" s="35" t="n">
         <v>58.78614127460222</v>
@@ -8206,7 +8206,7 @@
         <v>75.56091533165856</v>
       </c>
       <c r="AA33" s="35" t="n">
-        <v>24.23902966953202</v>
+        <v>24.21656319255873</v>
       </c>
       <c r="AB33" s="86" t="n">
         <v>19.10070682905246</v>
@@ -8248,7 +8248,7 @@
         <v>11.84204764311698</v>
       </c>
       <c r="AO33" s="88" t="n">
-        <v>4.740488034214399</v>
+        <v>4.744822290354756</v>
       </c>
       <c r="AP33" s="83" t="n">
         <v>595.510009765625</v>
@@ -8310,7 +8310,7 @@
       </c>
       <c r="F34" s="23" t="inlineStr">
         <is>
-          <t>Same</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G34" s="23" t="inlineStr">
@@ -8373,19 +8373,19 @@
         <v>1.110015869140625</v>
       </c>
       <c r="T34" s="72" t="n">
-        <v>348.4100036621094</v>
+        <v>348.3399963378906</v>
       </c>
       <c r="U34" s="72" t="n">
         <v>352.6600036621094</v>
       </c>
       <c r="V34" s="72" t="n">
-        <v>347.1600952148438</v>
+        <v>347.1600036621094</v>
       </c>
       <c r="W34" s="73" t="n">
-        <v>11454890</v>
+        <v>11833900</v>
       </c>
       <c r="X34" s="74" t="n">
-        <v>0.6902372133985398</v>
+        <v>0.7122335909990825</v>
       </c>
       <c r="Y34" s="28" t="n">
         <v>56.90493123908869</v>
@@ -8436,7 +8436,7 @@
         <v>5.153845797822692</v>
       </c>
       <c r="AO34" s="77" t="n">
-        <v>2.287660075599462</v>
+        <v>2.287661949537338</v>
       </c>
       <c r="AP34" s="72" t="n">
         <v>404.4700012207031</v>
@@ -8474,7 +8474,7 @@
       </c>
       <c r="AZ34" s="79" t="inlineStr">
         <is>
-          <t>The Staggering Costs of a Single Data Center, From Land to Chips</t>
+          <t>Alphabet vs. Meta Platforms: Which Stock Is a Better Buy in 2026?</t>
         </is>
       </c>
     </row>
@@ -8561,19 +8561,19 @@
         <v>-0.3899993896484375</v>
       </c>
       <c r="T35" s="83" t="n">
-        <v>36.33000183105469</v>
+        <v>36.30500030517578</v>
       </c>
       <c r="U35" s="83" t="n">
-        <v>36.69409942626953</v>
+        <v>36.69400024414062</v>
       </c>
       <c r="V35" s="83" t="n">
         <v>34.65499877929688</v>
       </c>
       <c r="W35" s="84" t="n">
-        <v>48998732</v>
+        <v>49217800</v>
       </c>
       <c r="X35" s="85" t="n">
-        <v>1.283553312034913</v>
+        <v>1.288568288728647</v>
       </c>
       <c r="Y35" s="35" t="n">
         <v>33.22700907063553</v>
@@ -8582,7 +8582,7 @@
         <v>1.086217599351113</v>
       </c>
       <c r="AA35" s="35" t="n">
-        <v>14.65202384202304</v>
+        <v>14.65206996014311</v>
       </c>
       <c r="AB35" s="86" t="n">
         <v>-1.697365071663903</v>
@@ -8624,7 +8624,7 @@
         <v>36.71972171768799</v>
       </c>
       <c r="AO35" s="88" t="n">
-        <v>7.436199194240606</v>
+        <v>7.436178836660334</v>
       </c>
       <c r="AP35" s="83" t="n">
         <v>76.87000274658203</v>
@@ -8749,28 +8749,28 @@
         <v>-3.349998474121094</v>
       </c>
       <c r="T36" s="72" t="n">
-        <v>102.6100006103516</v>
+        <v>102.5199966430664</v>
       </c>
       <c r="U36" s="72" t="n">
         <v>103.1900024414062</v>
       </c>
       <c r="V36" s="72" t="n">
-        <v>100.7102966308594</v>
+        <v>100.7099990844727</v>
       </c>
       <c r="W36" s="73" t="n">
-        <v>73592416</v>
+        <v>73728400</v>
       </c>
       <c r="X36" s="74" t="n">
-        <v>0.6807752651389222</v>
+        <v>0.6818985306862616</v>
       </c>
       <c r="Y36" s="28" t="n">
         <v>40.25962164832117</v>
       </c>
       <c r="Z36" s="28" t="n">
-        <v>2.393224406567574</v>
+        <v>2.394310921335615</v>
       </c>
       <c r="AA36" s="28" t="n">
-        <v>20.06331807027038</v>
+        <v>20.06336022710883</v>
       </c>
       <c r="AB36" s="75" t="n">
         <v>1.212809672425195</v>
@@ -8812,7 +8812,7 @@
         <v>29.48812679331235</v>
       </c>
       <c r="AO36" s="77" t="n">
-        <v>5.687597679555839</v>
+        <v>5.687618649771583</v>
       </c>
       <c r="AP36" s="72" t="n">
         <v>142.3500061035156</v>
@@ -8845,12 +8845,12 @@
       </c>
       <c r="AY36" s="79" t="inlineStr">
         <is>
+          <t>SNDK, MU, INTC, AMD, SKHY: Chip Stocks Extend Slide As AI Funding Concerns, China Competition Weigh On Sector</t>
+        </is>
+      </c>
+      <c r="AZ36" s="79" t="inlineStr">
+        <is>
           <t>Intel (INTC) Sees a More Significant Dip Than Broader Market: Some Facts to Know</t>
-        </is>
-      </c>
-      <c r="AZ36" s="79" t="inlineStr">
-        <is>
-          <t>Chip Stocks Fall As Broadcom, Intel CEOs Warn About AI Funding</t>
         </is>
       </c>
     </row>
@@ -8937,19 +8937,19 @@
         <v>6.08001708984375</v>
       </c>
       <c r="T37" s="83" t="n">
-        <v>538.0700073242188</v>
+        <v>537.530029296875</v>
       </c>
       <c r="U37" s="83" t="n">
         <v>542.739990234375</v>
       </c>
       <c r="V37" s="83" t="n">
-        <v>535.7012939453125</v>
+        <v>535.7000122070312</v>
       </c>
       <c r="W37" s="84" t="n">
-        <v>18227041</v>
+        <v>18292000</v>
       </c>
       <c r="X37" s="85" t="n">
-        <v>0.8228432435840689</v>
+        <v>0.8256230199513527</v>
       </c>
       <c r="Y37" s="35" t="n">
         <v>69.85523672407514</v>
@@ -9038,7 +9038,7 @@
       </c>
       <c r="AZ37" s="90" t="inlineStr">
         <is>
-          <t>Chamath Palihapitiya, Elon Musk Highlight Power, Cooling As Real Barriers In The AI Race Where ‘Everyone Co...</t>
+          <t>Microsoft Sues JLL For Protection Against Lawsuit At NYC Office Project</t>
         </is>
       </c>
     </row>
@@ -9125,19 +9125,19 @@
         <v>-1.660003662109375</v>
       </c>
       <c r="T38" s="72" t="n">
-        <v>153.2200012207031</v>
+        <v>153.3999938964844</v>
       </c>
       <c r="U38" s="72" t="n">
-        <v>158.4035034179688</v>
+        <v>158.3999938964844</v>
       </c>
       <c r="V38" s="72" t="n">
-        <v>150.8406982421875</v>
+        <v>150.8399963378906</v>
       </c>
       <c r="W38" s="73" t="n">
-        <v>12882016</v>
+        <v>12925900</v>
       </c>
       <c r="X38" s="74" t="n">
-        <v>0.5748803021440733</v>
+        <v>0.5767252141431285</v>
       </c>
       <c r="Y38" s="28" t="n">
         <v>53.92997434164897</v>
@@ -9146,7 +9146,7 @@
         <v>23.28945985901684</v>
       </c>
       <c r="AA38" s="28" t="n">
-        <v>33.44636146369641</v>
+        <v>33.44601028410538</v>
       </c>
       <c r="AB38" s="75" t="n">
         <v>6.559865089732028</v>
@@ -9188,7 +9188,7 @@
         <v>30.07636567451442</v>
       </c>
       <c r="AO38" s="77" t="n">
-        <v>5.697988755541677</v>
+        <v>5.697857406252678</v>
       </c>
       <c r="AP38" s="72" t="n">
         <v>323.4299926757812</v>
@@ -9313,7 +9313,7 @@
         <v>-39.96002197265625</v>
       </c>
       <c r="T39" s="83" t="n">
-        <v>1002.409973144531</v>
+        <v>1002.450012207031</v>
       </c>
       <c r="U39" s="83" t="n">
         <v>1002.669982910156</v>
@@ -9322,10 +9322,10 @@
         <v>978.5</v>
       </c>
       <c r="W39" s="84" t="n">
-        <v>23566935</v>
+        <v>23711800</v>
       </c>
       <c r="X39" s="85" t="n">
-        <v>0.9226436057459436</v>
+        <v>0.9279318571688252</v>
       </c>
       <c r="Y39" s="35" t="n">
         <v>44.65626981841611</v>
@@ -9404,17 +9404,17 @@
       </c>
       <c r="AX39" s="90" t="inlineStr">
         <is>
-          <t>Wall Street’s Biggest Micron Bull Just Raised Its Target Again. It Now Sees the Stock Nearly Tripling</t>
+          <t>SNDK, MU, INTC, AMD, SKHY: Chip Stocks Extend Slide As AI Funding Concerns, China Competition Weigh On Sector</t>
         </is>
       </c>
       <c r="AY39" s="90" t="inlineStr">
         <is>
-          <t>Micron Stock Falls On Competition From China Rival CXMT</t>
+          <t>Dow Jones Futures: Micron, Nvidia Lead AI Trade Lower; Apple, Meta Rally Near Buy Points</t>
         </is>
       </c>
       <c r="AZ39" s="90" t="inlineStr">
         <is>
-          <t>Micron, Fannie Mae, eBay, IonQ, Salesforce, and More Stocks That Explain Today’s Market</t>
+          <t>Monolithic Power Systems, MACOM, Micron, Seagate, and Vishay Intertechnology Shares Plummet, What You Need ...</t>
         </is>
       </c>
     </row>
@@ -9501,19 +9501,19 @@
         <v>-11.010009765625</v>
       </c>
       <c r="T40" s="72" t="n">
-        <v>217.0299987792969</v>
+        <v>217.1950073242188</v>
       </c>
       <c r="U40" s="72" t="n">
-        <v>217.0299987792969</v>
+        <v>217.1950073242188</v>
       </c>
       <c r="V40" s="72" t="n">
         <v>206.8999938964844</v>
       </c>
       <c r="W40" s="73" t="n">
-        <v>13918067</v>
+        <v>13962800</v>
       </c>
       <c r="X40" s="74" t="n">
-        <v>0.8672180016891728</v>
+        <v>0.8698149397512305</v>
       </c>
       <c r="Y40" s="28" t="n">
         <v>42.7886627198356</v>
@@ -9698,10 +9698,10 @@
         <v>70.55999755859375</v>
       </c>
       <c r="W41" s="84" t="n">
-        <v>23989230</v>
+        <v>24166800</v>
       </c>
       <c r="X41" s="85" t="n">
-        <v>0.6417704615677575</v>
+        <v>0.6463262240069643</v>
       </c>
       <c r="Y41" s="35" t="n">
         <v>44.8741901085375</v>
@@ -9886,10 +9886,10 @@
         <v>9.890000343322754</v>
       </c>
       <c r="W42" s="73" t="n">
-        <v>69793134</v>
+        <v>70924000</v>
       </c>
       <c r="X42" s="74" t="n">
-        <v>0.8612880378250057</v>
+        <v>0.8745827561786736</v>
       </c>
       <c r="Y42" s="28" t="n">
         <v>44.46653425690072</v>
@@ -10071,13 +10071,13 @@
         <v>228.8600006103516</v>
       </c>
       <c r="V43" s="83" t="n">
-        <v>224.9199981689453</v>
+        <v>224.8999938964844</v>
       </c>
       <c r="W43" s="84" t="n">
-        <v>69908781</v>
+        <v>70089000</v>
       </c>
       <c r="X43" s="85" t="n">
-        <v>0.6611783927762186</v>
+        <v>0.6627713362295281</v>
       </c>
       <c r="Y43" s="35" t="n">
         <v>49.35441364676441</v>
@@ -10086,7 +10086,7 @@
         <v>23.47401828041382</v>
       </c>
       <c r="AA43" s="35" t="n">
-        <v>16.98020105164052</v>
+        <v>16.98340086069082</v>
       </c>
       <c r="AB43" s="86" t="n">
         <v>3.277854124125412</v>
@@ -10128,7 +10128,7 @@
         <v>12.24728024689279</v>
       </c>
       <c r="AO43" s="88" t="n">
-        <v>2.471116984057208</v>
+        <v>2.471748336371679</v>
       </c>
       <c r="AP43" s="83" t="n">
         <v>243.3699951171875</v>
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
+          <t>Dow Jones Futures: Micron, Nvidia Lead AI Trade Lower; Apple, Meta Rally Near Buy Points</t>
+        </is>
+      </c>
+      <c r="AY43" s="90" t="inlineStr">
+        <is>
+          <t>Nvidia’s 'Reflection' move could put customers on edge</t>
+        </is>
+      </c>
+      <c r="AZ43" s="90" t="inlineStr">
+        <is>
           <t>Why Harmony Biosciences Stock Got Mashed on Monday</t>
-        </is>
-      </c>
-      <c r="AY43" s="90" t="inlineStr">
-        <is>
-          <t>$10,000 Invested Equally in Alphabet and Nvidia Could Be Worth This Much by 2030</t>
-        </is>
-      </c>
-      <c r="AZ43" s="90" t="inlineStr">
-        <is>
-          <t>You Bought VOO to Own the S&amp;P 500. On $500,000, One Chipmaker Is $40,400 of It</t>
         </is>
       </c>
     </row>
@@ -10256,25 +10256,25 @@
         <v>208.8999938964844</v>
       </c>
       <c r="U44" s="72" t="n">
-        <v>212.9398956298828</v>
+        <v>212.9400024414062</v>
       </c>
       <c r="V44" s="72" t="n">
         <v>206.0500030517578</v>
       </c>
       <c r="W44" s="73" t="n">
-        <v>24215062</v>
+        <v>24259200</v>
       </c>
       <c r="X44" s="74" t="n">
-        <v>1.016316801710124</v>
+        <v>1.017769814913756</v>
       </c>
       <c r="Y44" s="28" t="n">
         <v>76.20477587472955</v>
       </c>
       <c r="Z44" s="28" t="n">
-        <v>86.86696780841811</v>
+        <v>86.86665852864583</v>
       </c>
       <c r="AA44" s="28" t="n">
-        <v>35.10682715195058</v>
+        <v>35.10683374262661</v>
       </c>
       <c r="AB44" s="75" t="n">
         <v>7.909426863004427</v>
@@ -10316,19 +10316,19 @@
         <v>20.06242725926203</v>
       </c>
       <c r="AO44" s="77" t="n">
-        <v>3.197751075121628</v>
+        <v>3.197754725549633</v>
       </c>
       <c r="AP44" s="72" t="n">
-        <v>212.9398956298828</v>
+        <v>212.9400024414062</v>
       </c>
       <c r="AQ44" s="72" t="n">
         <v>106.370002746582</v>
       </c>
       <c r="AR44" s="29" t="n">
-        <v>-1.85023835868261</v>
+        <v>-1.850287590980193</v>
       </c>
       <c r="AS44" s="78" t="n">
-        <v>96.30299372244167</v>
+        <v>96.30289720119272</v>
       </c>
       <c r="AT44" s="26" t="n">
         <v>0.1034847240503498</v>
@@ -10441,19 +10441,19 @@
         <v>-1.07000732421875</v>
       </c>
       <c r="T45" s="83" t="n">
-        <v>175</v>
+        <v>175.1900024414062</v>
       </c>
       <c r="U45" s="83" t="n">
-        <v>175.2153015136719</v>
+        <v>175.2299957275391</v>
       </c>
       <c r="V45" s="83" t="n">
-        <v>172.1600952148438</v>
+        <v>172.1600036621094</v>
       </c>
       <c r="W45" s="84" t="n">
-        <v>6899324</v>
+        <v>6904700</v>
       </c>
       <c r="X45" s="85" t="n">
-        <v>0.5214492248925675</v>
+        <v>0.521825023447248</v>
       </c>
       <c r="Y45" s="35" t="n">
         <v>43.44088976069265</v>
@@ -10504,7 +10504,7 @@
         <v>17.01121841686022</v>
       </c>
       <c r="AO45" s="88" t="n">
-        <v>4.042656169835966</v>
+        <v>4.042659918893641</v>
       </c>
       <c r="AP45" s="83" t="n">
         <v>259.9200134277344</v>
@@ -10629,7 +10629,7 @@
         <v>-2.5</v>
       </c>
       <c r="T46" s="72" t="n">
-        <v>67.90000152587891</v>
+        <v>67.87999725341797</v>
       </c>
       <c r="U46" s="72" t="n">
         <v>68.06999969482422</v>
@@ -10638,10 +10638,10 @@
         <v>65.11499786376953</v>
       </c>
       <c r="W46" s="73" t="n">
-        <v>14390631</v>
+        <v>14430600</v>
       </c>
       <c r="X46" s="74" t="n">
-        <v>0.6690192097746087</v>
+        <v>0.6707190106306634</v>
       </c>
       <c r="Y46" s="28" t="n">
         <v>42.11483736151887</v>
@@ -10720,17 +10720,17 @@
       </c>
       <c r="AX46" s="79" t="inlineStr">
         <is>
+          <t>RKLB Stock Slips Overnight Despite Electron’s Push Toward 100th Launch — Retail Still Frets Over Neutron De...</t>
+        </is>
+      </c>
+      <c r="AY46" s="79" t="inlineStr">
+        <is>
           <t>AST SpaceMobile Rallies 4% as Next BlueBird Satellites Reach Cape Canaveral; Rocket Lab and Intuitive Machi...</t>
         </is>
       </c>
-      <c r="AY46" s="79" t="inlineStr">
+      <c r="AZ46" s="79" t="inlineStr">
         <is>
           <t>How Could RKLB Manage Orbital Collision Risks as Space Activity Grows?</t>
-        </is>
-      </c>
-      <c r="AZ46" s="79" t="inlineStr">
-        <is>
-          <t>RKLB Stock Rises Overnight: NASA Chief Warns Moon Race With China Is ‘Months, Not Years’ As Neutron Opportu...</t>
         </is>
       </c>
     </row>
@@ -10817,19 +10817,19 @@
         <v>-94.489990234375</v>
       </c>
       <c r="T47" s="83" t="n">
-        <v>1537.150024414062</v>
+        <v>1538.114990234375</v>
       </c>
       <c r="U47" s="83" t="n">
-        <v>1538.089965820312</v>
+        <v>1539.099975585938</v>
       </c>
       <c r="V47" s="83" t="n">
         <v>1464.430053710938</v>
       </c>
       <c r="W47" s="84" t="n">
-        <v>8663985</v>
+        <v>8687300</v>
       </c>
       <c r="X47" s="85" t="n">
-        <v>1.024585330624319</v>
+        <v>1.027021179880916</v>
       </c>
       <c r="Y47" s="35" t="n">
         <v>38.56381407509831</v>
@@ -10913,12 +10913,12 @@
       </c>
       <c r="AY47" s="90" t="inlineStr">
         <is>
-          <t>Micron, SK Hynix stocks fall as Chinese memory maker announces progress in new design</t>
+          <t>SNDK, MU, INTC, AMD, SKHY: Chip Stocks Extend Slide As AI Funding Concerns, China Competition Weigh On Sector</t>
         </is>
       </c>
       <c r="AZ47" s="90" t="inlineStr">
         <is>
-          <t>S&amp;P upgrades SanDisk to BBB as AI memory demand drives cash flow past $23B</t>
+          <t>Dow Jones Futures: Micron, Nvidia Lead AI Trade Lower; Apple, Meta Rally Near Buy Points</t>
         </is>
       </c>
     </row>
@@ -11005,19 +11005,19 @@
         <v>-4.670013427734375</v>
       </c>
       <c r="T48" s="72" t="n">
-        <v>382.6050109863281</v>
+        <v>382.6099853515625</v>
       </c>
       <c r="U48" s="72" t="n">
-        <v>382.6050109863281</v>
+        <v>382.7000122070312</v>
       </c>
       <c r="V48" s="72" t="n">
         <v>377.5799865722656</v>
       </c>
       <c r="W48" s="73" t="n">
-        <v>20131780</v>
+        <v>20164200</v>
       </c>
       <c r="X48" s="74" t="n">
-        <v>0.5715701392392668</v>
+        <v>0.5724197966601322</v>
       </c>
       <c r="Y48" s="28" t="n">
         <v>56.44703643496045</v>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 12 Oct 2026, 11:43 PM · Yahoo Finance data</t>
+          <t>Built 13 Oct 2026, 02:03 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -12512,10 +12512,10 @@
         <v>54.20999908447266</v>
       </c>
       <c r="W9" s="73" t="n">
-        <v>35459400</v>
+        <v>35483300</v>
       </c>
       <c r="X9" s="74" t="n">
-        <v>0.91060312042211</v>
+        <v>0.9111889139063052</v>
       </c>
       <c r="Y9" s="28" t="n">
         <v>45.595534981943</v>
@@ -12868,10 +12868,10 @@
         <v>82.95999908447266</v>
       </c>
       <c r="W11" s="73" t="n">
-        <v>7726700</v>
+        <v>7747400</v>
       </c>
       <c r="X11" s="74" t="n">
-        <v>0.7116954889815092</v>
+        <v>0.7135341140020731</v>
       </c>
       <c r="Y11" s="28" t="n">
         <v>54.64969965581181</v>
@@ -14133,10 +14133,10 @@
         <v>775.1400146484375</v>
       </c>
       <c r="W19" s="73" t="n">
-        <v>22596500</v>
+        <v>22624500</v>
       </c>
       <c r="X19" s="74" t="n">
-        <v>0.5043907767905912</v>
+        <v>0.5050000011160468</v>
       </c>
       <c r="Y19" s="28" t="n">
         <v>59.89154933765729</v>
@@ -14309,10 +14309,10 @@
         <v>748.3699951171875</v>
       </c>
       <c r="W20" s="84" t="n">
-        <v>21122000</v>
+        <v>21162000</v>
       </c>
       <c r="X20" s="85" t="n">
-        <v>0.6213261173765695</v>
+        <v>0.6224661389539028</v>
       </c>
       <c r="Y20" s="35" t="n">
         <v>60.89658268019971</v>
@@ -14485,10 +14485,10 @@
         <v>277.4599914550781</v>
       </c>
       <c r="W21" s="73" t="n">
-        <v>18705600</v>
+        <v>18720300</v>
       </c>
       <c r="X21" s="74" t="n">
-        <v>0.7388598381828383</v>
+        <v>0.7394190124016592</v>
       </c>
       <c r="Y21" s="28" t="n">
         <v>38.48230289287564</v>
@@ -14661,10 +14661,10 @@
         <v>137.7100067138672</v>
       </c>
       <c r="W22" s="84" t="n">
-        <v>59031400</v>
+        <v>59326000</v>
       </c>
       <c r="X22" s="85" t="n">
-        <v>0.9433522649186112</v>
+        <v>0.9478370108895969</v>
       </c>
       <c r="Y22" s="35" t="n">
         <v>49.17747649665148</v>
@@ -14858,10 +14858,10 @@
         <v>330.7000122070312</v>
       </c>
       <c r="W24" s="73" t="n">
-        <v>37855000</v>
+        <v>37881200</v>
       </c>
       <c r="X24" s="74" t="n">
-        <v>1.002184659307517</v>
+        <v>1.002843506039505</v>
       </c>
       <c r="Y24" s="28" t="n">
         <v>56.12381782112851</v>
@@ -15034,10 +15034,10 @@
         <v>606</v>
       </c>
       <c r="W25" s="84" t="n">
-        <v>13694400</v>
+        <v>13733300</v>
       </c>
       <c r="X25" s="85" t="n">
-        <v>0.6186007086100388</v>
+        <v>0.6203033923300504</v>
       </c>
       <c r="Y25" s="35" t="n">
         <v>57.18735511557669</v>
@@ -15210,10 +15210,10 @@
         <v>256</v>
       </c>
       <c r="W26" s="73" t="n">
-        <v>34710500</v>
+        <v>34770000</v>
       </c>
       <c r="X26" s="74" t="n">
-        <v>0.9365980044894535</v>
+        <v>0.9381281927757654</v>
       </c>
       <c r="Y26" s="28" t="n">
         <v>59.04749876615112</v>
@@ -15562,10 +15562,10 @@
         <v>265.6000061035156</v>
       </c>
       <c r="W28" s="73" t="n">
-        <v>4253900</v>
+        <v>4272000</v>
       </c>
       <c r="X28" s="74" t="n">
-        <v>0.7167819206297854</v>
+        <v>0.7197220174792039</v>
       </c>
       <c r="Y28" s="28" t="n">
         <v>43.85047833091154</v>
@@ -15738,10 +15738,10 @@
         <v>47.56999969482422</v>
       </c>
       <c r="W29" s="84" t="n">
-        <v>54119500</v>
+        <v>54317100</v>
       </c>
       <c r="X29" s="85" t="n">
-        <v>4.007182192604933</v>
+        <v>4.018873138665555</v>
       </c>
       <c r="Y29" s="35" t="n">
         <v>35.70422191116761</v>
@@ -15914,10 +15914,10 @@
         <v>361.1000061035156</v>
       </c>
       <c r="W30" s="73" t="n">
-        <v>16825700</v>
+        <v>16843800</v>
       </c>
       <c r="X30" s="74" t="n">
-        <v>0.7000685684994317</v>
+        <v>0.7007952689516841</v>
       </c>
       <c r="Y30" s="28" t="n">
         <v>50.07284791885349</v>
@@ -16266,10 +16266,10 @@
         <v>81.20999908447266</v>
       </c>
       <c r="W32" s="73" t="n">
-        <v>19938600</v>
+        <v>20011400</v>
       </c>
       <c r="X32" s="74" t="n">
-        <v>0.6569595234765022</v>
+        <v>0.6592791496058686</v>
       </c>
       <c r="Y32" s="28" t="n">
         <v>43.70681166286358</v>
@@ -16442,10 +16442,10 @@
         <v>566.2000122070312</v>
       </c>
       <c r="W33" s="84" t="n">
-        <v>5500400</v>
+        <v>5516000</v>
       </c>
       <c r="X33" s="85" t="n">
-        <v>0.735242418531039</v>
+        <v>0.737250813635665</v>
       </c>
       <c r="Y33" s="35" t="n">
         <v>61.69074540880679</v>
@@ -16618,10 +16618,10 @@
         <v>346.8800048828125</v>
       </c>
       <c r="W34" s="73" t="n">
-        <v>11129700</v>
+        <v>11142900</v>
       </c>
       <c r="X34" s="74" t="n">
-        <v>0.649073368845738</v>
+        <v>0.6498181682462741</v>
       </c>
       <c r="Y34" s="28" t="n">
         <v>55.93129419756334</v>
@@ -16794,10 +16794,10 @@
         <v>34.63999938964844</v>
       </c>
       <c r="W35" s="84" t="n">
-        <v>38317000</v>
+        <v>38526700</v>
       </c>
       <c r="X35" s="85" t="n">
-        <v>1.022281178148576</v>
+        <v>1.027588431718528</v>
       </c>
       <c r="Y35" s="35" t="n">
         <v>33.89940439795105</v>
@@ -16970,10 +16970,10 @@
         <v>104</v>
       </c>
       <c r="W36" s="73" t="n">
-        <v>74726800</v>
+        <v>75017800</v>
       </c>
       <c r="X36" s="74" t="n">
-        <v>0.684034108519752</v>
+        <v>0.6866064164528243</v>
       </c>
       <c r="Y36" s="28" t="n">
         <v>43.44448480797771</v>
@@ -17146,10 +17146,10 @@
         <v>526.239990234375</v>
       </c>
       <c r="W37" s="84" t="n">
-        <v>18483600</v>
+        <v>18500600</v>
       </c>
       <c r="X37" s="85" t="n">
-        <v>0.8253620805254496</v>
+        <v>0.8260898394914845</v>
       </c>
       <c r="Y37" s="35" t="n">
         <v>67.46788699912219</v>
@@ -17322,10 +17322,10 @@
         <v>150.5</v>
       </c>
       <c r="W38" s="73" t="n">
-        <v>15997900</v>
+        <v>16042200</v>
       </c>
       <c r="X38" s="74" t="n">
-        <v>0.70476215230015</v>
+        <v>0.7066447654450525</v>
       </c>
       <c r="Y38" s="28" t="n">
         <v>55.38217278703281</v>
@@ -17498,10 +17498,10 @@
         <v>1017</v>
       </c>
       <c r="W39" s="84" t="n">
-        <v>19852800</v>
+        <v>19918900</v>
       </c>
       <c r="X39" s="85" t="n">
-        <v>0.7718342396084845</v>
+        <v>0.7743045742858375</v>
       </c>
       <c r="Y39" s="35" t="n">
         <v>50.20250913285658</v>
@@ -17674,10 +17674,10 @@
         <v>218.5</v>
       </c>
       <c r="W40" s="73" t="n">
-        <v>9535900</v>
+        <v>9561400</v>
       </c>
       <c r="X40" s="74" t="n">
-        <v>0.5945278672273675</v>
+        <v>0.5960703147769194</v>
       </c>
       <c r="Y40" s="28" t="n">
         <v>46.74180659969193</v>
@@ -17850,10 +17850,10 @@
         <v>70.19000244140625</v>
       </c>
       <c r="W41" s="84" t="n">
-        <v>29076700</v>
+        <v>29124300</v>
       </c>
       <c r="X41" s="85" t="n">
-        <v>0.7707018423666943</v>
+        <v>0.7719148241423125</v>
       </c>
       <c r="Y41" s="35" t="n">
         <v>43.84449031248121</v>
@@ -18026,10 +18026,10 @@
         <v>10.1899995803833</v>
       </c>
       <c r="W42" s="73" t="n">
-        <v>50633700</v>
+        <v>50727400</v>
       </c>
       <c r="X42" s="74" t="n">
-        <v>0.6040073069642512</v>
+        <v>0.6050912335404482</v>
       </c>
       <c r="Y42" s="28" t="n">
         <v>49.43061884585565</v>
@@ -18202,10 +18202,10 @@
         <v>229.1100006103516</v>
       </c>
       <c r="W43" s="84" t="n">
-        <v>84470000</v>
+        <v>84645600</v>
       </c>
       <c r="X43" s="85" t="n">
-        <v>0.7760111054014994</v>
+        <v>0.7775615934971344</v>
       </c>
       <c r="Y43" s="35" t="n">
         <v>52.96326731274894</v>
@@ -18378,10 +18378,10 @@
         <v>198.3000030517578</v>
       </c>
       <c r="W44" s="73" t="n">
-        <v>37479600</v>
+        <v>37622500</v>
       </c>
       <c r="X44" s="74" t="n">
-        <v>1.556913415290939</v>
+        <v>1.562385798101009</v>
       </c>
       <c r="Y44" s="28" t="n">
         <v>76.28889898945955</v>
@@ -18554,10 +18554,10 @@
         <v>171.7899932861328</v>
       </c>
       <c r="W45" s="84" t="n">
-        <v>7565100</v>
+        <v>7575200</v>
       </c>
       <c r="X45" s="85" t="n">
-        <v>0.5572682211040174</v>
+        <v>0.5579914605620944</v>
       </c>
       <c r="Y45" s="35" t="n">
         <v>44.42080071853557</v>
@@ -18730,10 +18730,10 @@
         <v>66.98000335693359</v>
       </c>
       <c r="W46" s="73" t="n">
-        <v>14873000</v>
+        <v>14934600</v>
       </c>
       <c r="X46" s="74" t="n">
-        <v>0.6913502200416261</v>
+        <v>0.6941142323720589</v>
       </c>
       <c r="Y46" s="28" t="n">
         <v>46.26963594603323</v>
@@ -18906,10 +18906,10 @@
         <v>1575.68994140625</v>
       </c>
       <c r="W47" s="84" t="n">
-        <v>5577200</v>
+        <v>5606800</v>
       </c>
       <c r="X47" s="85" t="n">
-        <v>0.6559694668160393</v>
+        <v>0.6593361364252406</v>
       </c>
       <c r="Y47" s="35" t="n">
         <v>43.80204422392227</v>
@@ -19082,10 +19082,10 @@
         <v>379.7099914550781</v>
       </c>
       <c r="W48" s="73" t="n">
-        <v>38897700</v>
+        <v>38952400</v>
       </c>
       <c r="X48" s="74" t="n">
-        <v>1.085340727851881</v>
+        <v>1.086784055363144</v>
       </c>
       <c r="Y48" s="28" t="n">
         <v>59.73255255639365</v>
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 12 Oct 2026, 11:43 PM · Yahoo Finance data</t>
+          <t>Built 13 Oct 2026, 02:03 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 12 Oct 2026, 11:43 PM · Yahoo Finance data</t>
+          <t>Built 13 Oct 2026, 02:03 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 12 Oct 2026, 11:43 PM · Yahoo Finance data</t>
+          <t>Built 13 Oct 2026, 02:03 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -44556,7 +44556,7 @@
       </c>
       <c r="D28" s="104" t="inlineStr">
         <is>
-          <t>Gapped up 4.7% at the open</t>
+          <t>Gapped up 4.5% at the open</t>
         </is>
       </c>
       <c r="E28" s="26" t="n">
@@ -44780,7 +44780,7 @@
       </c>
       <c r="D36" s="104" t="inlineStr">
         <is>
-          <t>Gapped down 2.0% at the open</t>
+          <t>Gapped down 2.1% at the open</t>
         </is>
       </c>
       <c r="E36" s="26" t="n">
@@ -44836,7 +44836,7 @@
       </c>
       <c r="D38" s="104" t="inlineStr">
         <is>
-          <t>Gapped down 2.1% at the open</t>
+          <t>Gapped down 2.2% at the open</t>
         </is>
       </c>
       <c r="E38" s="26" t="n">

</xml_diff>

<commit_message>
Daily workbook: 2026-10-13 02:33 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 13 Oct 2026, 02:03 AM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 13 Oct 2026, 02:33 AM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 13 Oct 2026, 02:03 AM · Yahoo Finance data</t>
+          <t>Built 13 Oct 2026, 02:33 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -5811,17 +5811,17 @@
       </c>
       <c r="AX19" s="79" t="inlineStr">
         <is>
+          <t>Ventas (VTR) Pays Out Over 370% of Its Earnings as Dividends, So What Actually Funds It?</t>
+        </is>
+      </c>
+      <c r="AY19" s="79" t="inlineStr">
+        <is>
+          <t>Charter Communications (CHTR) Trades at 2.69 Times Earnings With 41.52% of Its Float Sold Short. Which Side...</t>
+        </is>
+      </c>
+      <c r="AZ19" s="79" t="inlineStr">
+        <is>
           <t>ServiceNow (NOW) Grew Revenue 24% While Earnings Fell 22.60%. Where Did the Profit Go?</t>
-        </is>
-      </c>
-      <c r="AY19" s="79" t="inlineStr">
-        <is>
-          <t>Jefferies Financial Group (JEF): Record Banking Revenue Is Not Enough to Resolve the Valuation Discount</t>
-        </is>
-      </c>
-      <c r="AZ19" s="79" t="inlineStr">
-        <is>
-          <t>Dow Rises 200 Points, Nasdaq Wavers: China Chip Competition Hits Tech Stocks, Oil Climbs</t>
         </is>
       </c>
     </row>
@@ -7712,17 +7712,17 @@
       </c>
       <c r="AX30" s="79" t="inlineStr">
         <is>
+          <t>Broadcom CEO follows a proven blueprint for labs buying its chips</t>
+        </is>
+      </c>
+      <c r="AY30" s="79" t="inlineStr">
+        <is>
           <t>Broadcom vs. Qualcomm: Which Chip Stock Is a Better Buy in 2026?</t>
         </is>
       </c>
-      <c r="AY30" s="79" t="inlineStr">
+      <c r="AZ30" s="79" t="inlineStr">
         <is>
           <t>3 Dividend Paying Stocks Offering AI Exposure</t>
-        </is>
-      </c>
-      <c r="AZ30" s="79" t="inlineStr">
-        <is>
-          <t>Chip Stocks Fall As Broadcom, Intel CEOs Warn About AI Funding</t>
         </is>
       </c>
     </row>
@@ -9038,7 +9038,7 @@
       </c>
       <c r="AZ37" s="90" t="inlineStr">
         <is>
-          <t>Microsoft Sues JLL For Protection Against Lawsuit At NYC Office Project</t>
+          <t>Microsoft Now Has 3 Generations of Its Own AI Chips. Nvidia Is Still the Chip Stock to Buy.</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 13 Oct 2026, 02:03 AM · Yahoo Finance data</t>
+          <t>Built 13 Oct 2026, 02:33 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 13 Oct 2026, 02:03 AM · Yahoo Finance data</t>
+          <t>Built 13 Oct 2026, 02:33 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 13 Oct 2026, 02:03 AM · Yahoo Finance data</t>
+          <t>Built 13 Oct 2026, 02:33 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 13 Oct 2026, 02:03 AM · Yahoo Finance data</t>
+          <t>Built 13 Oct 2026, 02:33 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-10-13 23:44 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 13 Oct 2026, 09:55 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 13 Oct 2026, 11:44 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 13 Oct 2026, 09:55 PM · Yahoo Finance data</t>
+          <t>Built 13 Oct 2026, 11:44 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -3620,10 +3620,10 @@
         <v>166.5599975585938</v>
       </c>
       <c r="W7" s="73" t="n">
-        <v>7278251</v>
+        <v>7284575</v>
       </c>
       <c r="X7" s="74" t="n">
-        <v>1.004393684430788</v>
+        <v>1.00522252885483</v>
       </c>
       <c r="Y7" s="28" t="n">
         <v>42.6555295735747</v>
@@ -3810,10 +3810,10 @@
         <v>169.4799957275391</v>
       </c>
       <c r="W8" s="84" t="n">
-        <v>8724335</v>
+        <v>8745019</v>
       </c>
       <c r="X8" s="85" t="n">
-        <v>1.076591702510288</v>
+        <v>1.07900642466421</v>
       </c>
       <c r="Y8" s="35" t="n">
         <v>52.16656581728714</v>
@@ -4000,10 +4000,10 @@
         <v>54.63999938964844</v>
       </c>
       <c r="W9" s="73" t="n">
-        <v>44344074</v>
+        <v>44490388</v>
       </c>
       <c r="X9" s="74" t="n">
-        <v>1.145041546251567</v>
+        <v>1.148602653797858</v>
       </c>
       <c r="Y9" s="28" t="n">
         <v>46.82402511867949</v>
@@ -4190,10 +4190,10 @@
         <v>66.29000091552734</v>
       </c>
       <c r="W10" s="84" t="n">
-        <v>27389584</v>
+        <v>27490546</v>
       </c>
       <c r="X10" s="85" t="n">
-        <v>0.8129815638388761</v>
+        <v>0.8158560858211086</v>
       </c>
       <c r="Y10" s="35" t="n">
         <v>69.75320591506099</v>
@@ -4380,10 +4380,10 @@
         <v>84.11000061035156</v>
       </c>
       <c r="W11" s="73" t="n">
-        <v>9983583</v>
+        <v>10004762</v>
       </c>
       <c r="X11" s="74" t="n">
-        <v>0.9528097855934305</v>
+        <v>0.954734570747758</v>
       </c>
       <c r="Y11" s="28" t="n">
         <v>58.2814120345096</v>
@@ -4570,10 +4570,10 @@
         <v>112.1600036621094</v>
       </c>
       <c r="W12" s="84" t="n">
-        <v>5684041</v>
+        <v>5684050</v>
       </c>
       <c r="X12" s="85" t="n">
-        <v>0.8914979182991497</v>
+        <v>0.8914992669584717</v>
       </c>
       <c r="Y12" s="35" t="n">
         <v>52.09238182280671</v>
@@ -4760,10 +4760,10 @@
         <v>111.4449996948242</v>
       </c>
       <c r="W13" s="73" t="n">
-        <v>6922405</v>
+        <v>6929000</v>
       </c>
       <c r="X13" s="74" t="n">
-        <v>1.072444608095515</v>
+        <v>1.073411493512127</v>
       </c>
       <c r="Y13" s="28" t="n">
         <v>51.93524468671532</v>
@@ -4950,10 +4950,10 @@
         <v>49.34500122070312</v>
       </c>
       <c r="W14" s="84" t="n">
-        <v>7897796</v>
+        <v>7897808</v>
       </c>
       <c r="X14" s="85" t="n">
-        <v>0.6927715118259538</v>
+        <v>0.6927725279699892</v>
       </c>
       <c r="Y14" s="35" t="n">
         <v>46.60967502075996</v>
@@ -5140,10 +5140,10 @@
         <v>193.9199981689453</v>
       </c>
       <c r="W15" s="73" t="n">
-        <v>6667321</v>
+        <v>6753008</v>
       </c>
       <c r="X15" s="74" t="n">
-        <v>0.9125152489429303</v>
+        <v>0.9237010689669445</v>
       </c>
       <c r="Y15" s="28" t="n">
         <v>54.95228149986838</v>
@@ -5330,10 +5330,10 @@
         <v>41.58499908447266</v>
       </c>
       <c r="W16" s="84" t="n">
-        <v>5830515</v>
+        <v>5853296</v>
       </c>
       <c r="X16" s="85" t="n">
-        <v>0.8430307343229925</v>
+        <v>0.8461852635954263</v>
       </c>
       <c r="Y16" s="35" t="n">
         <v>46.95003749617617</v>
@@ -5520,10 +5520,10 @@
         <v>41.09000015258789</v>
       </c>
       <c r="W17" s="73" t="n">
-        <v>27179321</v>
+        <v>27226247</v>
       </c>
       <c r="X17" s="74" t="n">
-        <v>0.8010703652072149</v>
+        <v>0.8023979509760902</v>
       </c>
       <c r="Y17" s="28" t="n">
         <v>58.06159776627418</v>
@@ -5729,10 +5729,10 @@
         <v>775.9500122070312</v>
       </c>
       <c r="W19" s="73" t="n">
-        <v>25344746</v>
+        <v>25825560</v>
       </c>
       <c r="X19" s="74" t="n">
-        <v>0.5964436966463029</v>
+        <v>0.6074151539985702</v>
       </c>
       <c r="Y19" s="28" t="n">
         <v>59.21716692586363</v>
@@ -5811,17 +5811,17 @@
       </c>
       <c r="AX19" s="79" t="inlineStr">
         <is>
-          <t>Becton Dickinson (BDX) Grew Revenue 5.4% While Earnings Fell 34.3%. Why Did Profit Fall So Much Further?</t>
+          <t>If You Own SPY, This Lower-Cost Fund Tracks Identical Holdings for Less Than Half the Fee</t>
         </is>
       </c>
       <c r="AY19" s="79" t="inlineStr">
         <is>
-          <t>Pfizer (PFE) Pays Out Over 226% of Earnings and Trades at 36.7x Trailing Against 9.8 Forward. What Is the Y...</t>
+          <t>Is Spotify (SPOT) a Good or Bad Investment at Today’s Price?</t>
         </is>
       </c>
       <c r="AZ19" s="79" t="inlineStr">
         <is>
-          <t>What is MSCI’s (MSCI) Economic Moat, and is it Widening or Narrowing?</t>
+          <t>Humana (HUM) Will Have 95% of Its Members in Four-Star Plans, Up From 20%. What Changed?</t>
         </is>
       </c>
     </row>
@@ -6102,13 +6102,13 @@
         <v>278.7000122070312</v>
       </c>
       <c r="V21" s="72" t="n">
-        <v>275.7000122070312</v>
+        <v>275.6000061035156</v>
       </c>
       <c r="W21" s="73" t="n">
-        <v>27654822</v>
+        <v>27728271</v>
       </c>
       <c r="X21" s="74" t="n">
-        <v>1.107487262382833</v>
+        <v>1.110265373554089</v>
       </c>
       <c r="Y21" s="28" t="n">
         <v>34.97542275219583</v>
@@ -6117,7 +6117,7 @@
         <v>21.54167659289594</v>
       </c>
       <c r="AA21" s="28" t="n">
-        <v>39.00457017094627</v>
+        <v>39.02043464694359</v>
       </c>
       <c r="AB21" s="75" t="n">
         <v>-3.451122107332139</v>
@@ -6159,7 +6159,7 @@
         <v>4.252906971479913</v>
       </c>
       <c r="AO21" s="77" t="n">
-        <v>1.236050787477307</v>
+        <v>1.238632389498674</v>
       </c>
       <c r="AP21" s="72" t="n">
         <v>305.1799926757812</v>
@@ -6293,10 +6293,10 @@
         <v>115.8399963378906</v>
       </c>
       <c r="W22" s="84" t="n">
-        <v>77745448</v>
+        <v>78745280</v>
       </c>
       <c r="X22" s="85" t="n">
-        <v>1.264144532397705</v>
+        <v>1.279361896944545</v>
       </c>
       <c r="Y22" s="35" t="n">
         <v>42.97269118559336</v>
@@ -6589,12 +6589,12 @@
       </c>
       <c r="AY24" s="79" t="inlineStr">
         <is>
+          <t>Apple Takes on Amazon With New Smart Home Gadgets. It Still Isn’t Worth $5 Trillion.</t>
+        </is>
+      </c>
+      <c r="AZ24" s="79" t="inlineStr">
+        <is>
           <t>Judge orders OpenAI to turn over hiring records in Apple trade secrets case</t>
-        </is>
-      </c>
-      <c r="AZ24" s="79" t="inlineStr">
-        <is>
-          <t>Apple Introduces HomeView Smart Home Hub, Other Gadgets</t>
         </is>
       </c>
     </row>
@@ -6777,12 +6777,12 @@
       </c>
       <c r="AY25" s="90" t="inlineStr">
         <is>
+          <t>Dow Jones Futures: Stock Market Holds Up As Meta, AMD Lead Buys; ASML, CPI Inflation Due</t>
+        </is>
+      </c>
+      <c r="AZ25" s="90" t="inlineStr">
+        <is>
           <t>Stock Market Today, Oct. 13: Fermi Surges 14% on AMD Credit Support for Project Matador</t>
-        </is>
-      </c>
-      <c r="AZ25" s="90" t="inlineStr">
-        <is>
-          <t>Dow Jones Futures: Stock Market Holds Up As Meta, AMD Lead Buys; ASML, CPI Inflation Due</t>
         </is>
       </c>
     </row>
@@ -6960,17 +6960,17 @@
       </c>
       <c r="AX26" s="79" t="inlineStr">
         <is>
+          <t>Jeff Bezos Aims for the Moon But Advises Retirees to Stick With Index Funds</t>
+        </is>
+      </c>
+      <c r="AY26" s="79" t="inlineStr">
+        <is>
           <t>Sector Update: Tech Stocks Fall Tuesday Afternoon</t>
         </is>
       </c>
-      <c r="AY26" s="79" t="inlineStr">
-        <is>
-          <t>Data Reveals Next Big AI Robotics Stock Investments</t>
-        </is>
-      </c>
       <c r="AZ26" s="79" t="inlineStr">
         <is>
-          <t>Investors Are Paying More for Walmart Than Amazon. Here’s Why That Doesn’t Add Up.</t>
+          <t>Franklin Templeton CEO says AI is hiding a bigger tech story</t>
         </is>
       </c>
     </row>
@@ -7066,10 +7066,10 @@
         <v>86.50099945068359</v>
       </c>
       <c r="W27" s="84" t="n">
-        <v>3517475</v>
+        <v>3521445</v>
       </c>
       <c r="X27" s="85" t="n">
-        <v>0.758692332973936</v>
+        <v>0.75951611284733</v>
       </c>
       <c r="Y27" s="35" t="n">
         <v>48.46664549859157</v>
@@ -7341,12 +7341,12 @@
       </c>
       <c r="AY28" s="79" t="inlineStr">
         <is>
+          <t>Heavy Unusual Call Option Activity in Chip Designer Arm Holdings Plc - Are Investors Still Bullish?</t>
+        </is>
+      </c>
+      <c r="AZ28" s="79" t="inlineStr">
+        <is>
           <t>What Does Arm Holdings (ARM) Winning An AI Ecosystem Award Really Signal?</t>
-        </is>
-      </c>
-      <c r="AZ28" s="79" t="inlineStr">
-        <is>
-          <t>AI Is Blowing Up Tech’s Money Rules. How Arm Could Make Qualcomm Pay More.</t>
         </is>
       </c>
     </row>
@@ -7818,10 +7818,10 @@
         <v>85.22000122070312</v>
       </c>
       <c r="W31" s="84" t="n">
-        <v>2374493</v>
+        <v>2425015</v>
       </c>
       <c r="X31" s="85" t="n">
-        <v>0.7317920577074828</v>
+        <v>0.7467809896603808</v>
       </c>
       <c r="Y31" s="35" t="n">
         <v>40.72524564751583</v>
@@ -7900,17 +7900,17 @@
       </c>
       <c r="AX31" s="90" t="inlineStr">
         <is>
+          <t>Cameco Heads 3 Canadian Nuclear Stocks To Watch</t>
+        </is>
+      </c>
+      <c r="AY31" s="90" t="inlineStr">
+        <is>
           <t>3 Stocks to Buy If You Think the Nuclear Fuel Shortage Is the Real Story, Not the Reactors</t>
         </is>
       </c>
-      <c r="AY31" s="90" t="inlineStr">
+      <c r="AZ31" s="90" t="inlineStr">
         <is>
           <t>IsoEnergy Announces the Appointment of Nathan Bridge as Vice President, Exploration and Dr. Dan Brisbin as ...</t>
-        </is>
-      </c>
-      <c r="AZ31" s="90" t="inlineStr">
-        <is>
-          <t>Cameco And 2 Other Canadian Growth Stocks To Watch</t>
         </is>
       </c>
     </row>
@@ -8194,10 +8194,10 @@
         <v>548.4000244140625</v>
       </c>
       <c r="W33" s="84" t="n">
-        <v>5531687</v>
+        <v>5542069</v>
       </c>
       <c r="X33" s="85" t="n">
-        <v>0.7823117839190858</v>
+        <v>0.7837225095729586</v>
       </c>
       <c r="Y33" s="35" t="n">
         <v>57.44255900581597</v>
@@ -8652,17 +8652,17 @@
       </c>
       <c r="AX35" s="90" t="inlineStr">
         <is>
+          <t>Stock Market Today, Oct. 13: IREN Holds Moderate Buy Rating as Analysts Eye AI Cloud Execution</t>
+        </is>
+      </c>
+      <c r="AY35" s="90" t="inlineStr">
+        <is>
           <t>IREN's Global Expansion Accelerates: Can It Drive Future Growth?</t>
         </is>
       </c>
-      <c r="AY35" s="90" t="inlineStr">
+      <c r="AZ35" s="90" t="inlineStr">
         <is>
           <t>IREN Slides 5% as Anthropic Cloud Report Buzz Fades; Core Scientific Falls 3%</t>
-        </is>
-      </c>
-      <c r="AZ35" s="90" t="inlineStr">
-        <is>
-          <t>IREN reportedly inks multiyear deal with Anthropic. Here’s what we know</t>
         </is>
       </c>
     </row>
@@ -9028,17 +9028,17 @@
       </c>
       <c r="AX37" s="90" t="inlineStr">
         <is>
-          <t>Microsoft Reports $130 Billion in Data Center Leases</t>
+          <t>Microsoft Weighs 20% Cost Cuts In Azure Vertical Amid Soaring AI Data Center Spending: Report</t>
         </is>
       </c>
       <c r="AY37" s="90" t="inlineStr">
         <is>
-          <t>Marvell Stock Is on a Bad Run, but Microsoft’s New AI Chips Can Revive It</t>
+          <t>How much MSFT stock does Microsoft founder Bill Gates actually own?</t>
         </is>
       </c>
       <c r="AZ37" s="90" t="inlineStr">
         <is>
-          <t>Is Microsoft’s New Maia 300 Chip a Threat to Nvidia’s Dominance? What the Stock Says.</t>
+          <t>Franklin Templeton CEO says AI is hiding a bigger tech story</t>
         </is>
       </c>
     </row>
@@ -9216,17 +9216,17 @@
       </c>
       <c r="AX38" s="79" t="inlineStr">
         <is>
+          <t>Strategy (MSTR) Stock Still Looks Like A Bargain Despite Its 354% Run</t>
+        </is>
+      </c>
+      <c r="AY38" s="79" t="inlineStr">
+        <is>
           <t>Strategy’s Bitcoin-Backed Preferred Shares Pay Up to About 10%. A Solana Treasury Company’s Preferred Pays ...</t>
         </is>
       </c>
-      <c r="AY38" s="79" t="inlineStr">
+      <c r="AZ38" s="79" t="inlineStr">
         <is>
           <t>Peter Schiff Calls Strategy’s 2026 a ‘Failure’ as MSTR Bulls Push Back</t>
-        </is>
-      </c>
-      <c r="AZ38" s="79" t="inlineStr">
-        <is>
-          <t>Strategy Bought 250 Bitcoin Last Week and Spent Nearly Nine Times That Buying Back Its Own Preferred Shares...</t>
         </is>
       </c>
     </row>
@@ -9404,12 +9404,12 @@
       </c>
       <c r="AX39" s="90" t="inlineStr">
         <is>
+          <t>Dow Jones Futures: Stock Market Holds Up As Meta, AMD Lead Buys; ASML, CPI Inflation Due</t>
+        </is>
+      </c>
+      <c r="AY39" s="90" t="inlineStr">
+        <is>
           <t>Micron Just Raised Its Buyback Authorization to $35 Billion. Prediction: It Spends More Buying Back Stock i...</t>
-        </is>
-      </c>
-      <c r="AY39" s="90" t="inlineStr">
-        <is>
-          <t>Dow Jones Futures: Stock Market Holds Up As Meta, AMD Lead Buys; ASML, CPI Inflation Due</t>
         </is>
       </c>
       <c r="AZ39" s="90" t="inlineStr">
@@ -9790,7 +9790,7 @@
       </c>
       <c r="AZ41" s="90" t="inlineStr">
         <is>
-          <t>Netflix Stock Downgraded To Sell Before Q3 Report</t>
+          <t>Netflix faces unexpected challenge as streaming prices soar, customer interest shifts</t>
         </is>
       </c>
     </row>
@@ -9886,10 +9886,10 @@
         <v>9.550000190734863</v>
       </c>
       <c r="W42" s="73" t="n">
-        <v>76413109</v>
+        <v>76721489</v>
       </c>
       <c r="X42" s="74" t="n">
-        <v>0.9468737408542213</v>
+        <v>0.9505134249086967</v>
       </c>
       <c r="Y42" s="28" t="n">
         <v>44.05225077148548</v>
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
+          <t>If You Own SPY, This Lower-Cost Fund Tracks Identical Holdings for Less Than Half the Fee</t>
+        </is>
+      </c>
+      <c r="AY43" s="90" t="inlineStr">
+        <is>
+          <t>Nvidia in 5 Years: Where the Stock Could Be Headed</t>
+        </is>
+      </c>
+      <c r="AZ43" s="90" t="inlineStr">
+        <is>
           <t>You Bought a Semiconductor Fund. On $500,000, $87,743 of It Is NVIDIA</t>
-        </is>
-      </c>
-      <c r="AY43" s="90" t="inlineStr">
-        <is>
-          <t>Citigroup Inc. Q3 2026 Earnings Call Summary</t>
-        </is>
-      </c>
-      <c r="AZ43" s="90" t="inlineStr">
-        <is>
-          <t>The Goldman Sachs Group, Inc. Q3 2026 Earnings Call Summary</t>
         </is>
       </c>
     </row>
@@ -10349,12 +10349,12 @@
       </c>
       <c r="AY44" s="79" t="inlineStr">
         <is>
+          <t>After a 60% Rally in Just 3 Months, Palantir Stock Can Still Soar Higher</t>
+        </is>
+      </c>
+      <c r="AZ44" s="79" t="inlineStr">
+        <is>
           <t>When Palantir's CEO and the Chart Say the Same Thing, Pay Attention</t>
-        </is>
-      </c>
-      <c r="AZ44" s="79" t="inlineStr">
-        <is>
-          <t>Palantir Stock Has Become a Wall Street Sensation. Here’s My Price Prediction For Next Year</t>
         </is>
       </c>
     </row>
@@ -10537,12 +10537,12 @@
       </c>
       <c r="AY45" s="90" t="inlineStr">
         <is>
+          <t>Qualcomm (QCOM) Rises As Market Takes a Dip: Key Facts</t>
+        </is>
+      </c>
+      <c r="AZ45" s="90" t="inlineStr">
+        <is>
           <t>ARM-QCOM Lawsuit: Delaware Jury Delivers Verdict In High-Stakes Qualcomm-ARM Licensing Battle</t>
-        </is>
-      </c>
-      <c r="AZ45" s="90" t="inlineStr">
-        <is>
-          <t>Is Qualcomm (QCOM) a Good or Bad Investment at Today’s Price?</t>
         </is>
       </c>
     </row>
@@ -10720,17 +10720,17 @@
       </c>
       <c r="AX46" s="79" t="inlineStr">
         <is>
+          <t>Here's Why Rocket Lab Corporation (RKLB) Fell More Than Broader Market</t>
+        </is>
+      </c>
+      <c r="AY46" s="79" t="inlineStr">
+        <is>
           <t>AST SpaceMobile vs. Rocket Lab: Which Space-Focused Stock Is a Better Buy in 2026?</t>
         </is>
       </c>
-      <c r="AY46" s="79" t="inlineStr">
+      <c r="AZ46" s="79" t="inlineStr">
         <is>
           <t>AST SpaceMobile Sinks 9% as Piper Sandler Cuts to Neutral on SpaceX Direct-to-Cell Threat; Planet Labs Drop...</t>
-        </is>
-      </c>
-      <c r="AZ46" s="79" t="inlineStr">
-        <is>
-          <t>Air Launch Is Back on the Space Industry's Flight Plan</t>
         </is>
       </c>
     </row>
@@ -11096,17 +11096,17 @@
       </c>
       <c r="AX48" s="79" t="inlineStr">
         <is>
+          <t>Tesla Robotaxi Fleet in Austin Soars 8x in a Month While Elon Musk Admits TSLA Is Still Working on Not Runn...</t>
+        </is>
+      </c>
+      <c r="AY48" s="79" t="inlineStr">
+        <is>
           <t>Tesla target lowered by analysts worried about runaway $25 billion spending</t>
         </is>
       </c>
-      <c r="AY48" s="79" t="inlineStr">
+      <c r="AZ48" s="79" t="inlineStr">
         <is>
           <t>EXCLUSIVE: Ross Gerber Says Tesla May Make Just ‘a Few Hundred’ Roadsters: ‘Hovering Is a Gimmick’</t>
-        </is>
-      </c>
-      <c r="AZ48" s="79" t="inlineStr">
-        <is>
-          <t>Electric Trucks: The REALITY for Tesla Semi &amp; Volvo Fleets</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 13 Oct 2026, 09:55 PM · Yahoo Finance data</t>
+          <t>Built 13 Oct 2026, 11:44 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 13 Oct 2026, 09:55 PM · Yahoo Finance data</t>
+          <t>Built 13 Oct 2026, 11:44 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 13 Oct 2026, 09:55 PM · Yahoo Finance data</t>
+          <t>Built 13 Oct 2026, 11:44 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 13 Oct 2026, 09:55 PM · Yahoo Finance data</t>
+          <t>Built 13 Oct 2026, 11:44 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-10-14 23:16 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 14 Oct 2026, 08:51 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 14 Oct 2026, 11:16 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 14 Oct 2026, 08:51 PM · Yahoo Finance data</t>
+          <t>Built 14 Oct 2026, 11:16 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -3620,10 +3620,10 @@
         <v>165.6900024414062</v>
       </c>
       <c r="W7" s="73" t="n">
-        <v>10818554</v>
+        <v>10822507</v>
       </c>
       <c r="X7" s="74" t="n">
-        <v>1.47348127618954</v>
+        <v>1.473979993395457</v>
       </c>
       <c r="Y7" s="28" t="n">
         <v>38.368242485176</v>
@@ -3810,10 +3810,10 @@
         <v>170.6699981689453</v>
       </c>
       <c r="W8" s="84" t="n">
-        <v>11784062</v>
+        <v>11816834</v>
       </c>
       <c r="X8" s="85" t="n">
-        <v>1.413663380568404</v>
+        <v>1.41731623508839</v>
       </c>
       <c r="Y8" s="35" t="n">
         <v>62.06025959405533</v>
@@ -4000,10 +4000,10 @@
         <v>54.01499938964844</v>
       </c>
       <c r="W9" s="73" t="n">
-        <v>43883616</v>
+        <v>44049658</v>
       </c>
       <c r="X9" s="74" t="n">
-        <v>1.146535883584759</v>
+        <v>1.15062444167997</v>
       </c>
       <c r="Y9" s="28" t="n">
         <v>43.76530390030472</v>
@@ -4190,10 +4190,10 @@
         <v>67.11499786376953</v>
       </c>
       <c r="W10" s="84" t="n">
-        <v>25120661</v>
+        <v>25205402</v>
       </c>
       <c r="X10" s="85" t="n">
-        <v>0.7724477879278754</v>
+        <v>0.7749525650045778</v>
       </c>
       <c r="Y10" s="35" t="n">
         <v>71.14722807096484</v>
@@ -4380,10 +4380,10 @@
         <v>84.61000061035156</v>
       </c>
       <c r="W11" s="73" t="n">
-        <v>14143977</v>
+        <v>14288954</v>
       </c>
       <c r="X11" s="74" t="n">
-        <v>1.32136577332065</v>
+        <v>1.334006491102856</v>
       </c>
       <c r="Y11" s="28" t="n">
         <v>66.627149302189</v>
@@ -4570,10 +4570,10 @@
         <v>110.6750030517578</v>
       </c>
       <c r="W12" s="84" t="n">
-        <v>8295122</v>
+        <v>8302448</v>
       </c>
       <c r="X12" s="85" t="n">
-        <v>1.30696550690664</v>
+        <v>1.308044287214514</v>
       </c>
       <c r="Y12" s="35" t="n">
         <v>47.77561280222257</v>
@@ -4760,10 +4760,10 @@
         <v>110.4100036621094</v>
       </c>
       <c r="W13" s="73" t="n">
-        <v>6773350</v>
+        <v>6777028</v>
       </c>
       <c r="X13" s="74" t="n">
-        <v>1.030325179105391</v>
+        <v>1.030855819445307</v>
       </c>
       <c r="Y13" s="28" t="n">
         <v>46.80908430193281</v>
@@ -4950,10 +4950,10 @@
         <v>49.22999954223633</v>
       </c>
       <c r="W14" s="84" t="n">
-        <v>8893588</v>
+        <v>8895844</v>
       </c>
       <c r="X14" s="85" t="n">
-        <v>0.7825002249770369</v>
+        <v>0.7826909506423405</v>
       </c>
       <c r="Y14" s="35" t="n">
         <v>46.11678135110024</v>
@@ -5140,10 +5140,10 @@
         <v>189.7299957275391</v>
       </c>
       <c r="W15" s="73" t="n">
-        <v>11842878</v>
+        <v>11921254</v>
       </c>
       <c r="X15" s="74" t="n">
-        <v>1.579108532248767</v>
+        <v>1.588728898298956</v>
       </c>
       <c r="Y15" s="28" t="n">
         <v>43.11268966576086</v>
@@ -5330,10 +5330,10 @@
         <v>41.31499862670898</v>
       </c>
       <c r="W16" s="84" t="n">
-        <v>7805384</v>
+        <v>7826350</v>
       </c>
       <c r="X16" s="85" t="n">
-        <v>1.108405343475006</v>
+        <v>1.111217204780462</v>
       </c>
       <c r="Y16" s="35" t="n">
         <v>43.05357700497292</v>
@@ -5520,10 +5520,10 @@
         <v>41.2400016784668</v>
       </c>
       <c r="W17" s="73" t="n">
-        <v>35286119</v>
+        <v>35403779</v>
       </c>
       <c r="X17" s="74" t="n">
-        <v>1.022289700763391</v>
+        <v>1.025523691247782</v>
       </c>
       <c r="Y17" s="28" t="n">
         <v>56.02289911757695</v>
@@ -5729,10 +5729,10 @@
         <v>766.7100219726562</v>
       </c>
       <c r="W19" s="73" t="n">
-        <v>54511707</v>
+        <v>55376546</v>
       </c>
       <c r="X19" s="74" t="n">
-        <v>1.289211863518004</v>
+        <v>1.308327464019265</v>
       </c>
       <c r="Y19" s="28" t="n">
         <v>49.60700748923982</v>
@@ -5917,10 +5917,10 @@
         <v>726.3900146484375</v>
       </c>
       <c r="W20" s="84" t="n">
-        <v>49885770</v>
+        <v>51534028</v>
       </c>
       <c r="X20" s="85" t="n">
-        <v>1.454026884756354</v>
+        <v>1.498469398113142</v>
       </c>
       <c r="Y20" s="35" t="n">
         <v>44.65135113476836</v>
@@ -6105,10 +6105,10 @@
         <v>270.3500061035156</v>
       </c>
       <c r="W21" s="73" t="n">
-        <v>37130334</v>
+        <v>37947395</v>
       </c>
       <c r="X21" s="74" t="n">
-        <v>1.45880681511796</v>
+        <v>1.488518999322167</v>
       </c>
       <c r="Y21" s="28" t="n">
         <v>28.17118867433366</v>
@@ -6293,10 +6293,10 @@
         <v>109</v>
       </c>
       <c r="W22" s="84" t="n">
-        <v>99172281</v>
+        <v>102344094</v>
       </c>
       <c r="X22" s="85" t="n">
-        <v>1.579153338839553</v>
+        <v>1.625554177401734</v>
       </c>
       <c r="Y22" s="35" t="n">
         <v>35.71049260039442</v>
@@ -6502,10 +6502,10 @@
         <v>341.7200012207031</v>
       </c>
       <c r="W24" s="73" t="n">
-        <v>49732645</v>
+        <v>49893047</v>
       </c>
       <c r="X24" s="74" t="n">
-        <v>1.303446481851079</v>
+        <v>1.307375659892054</v>
       </c>
       <c r="Y24" s="28" t="n">
         <v>62.06788775406566</v>
@@ -6584,17 +6584,17 @@
       </c>
       <c r="AX24" s="79" t="inlineStr">
         <is>
-          <t>Apple retakes $5 trillion market cap, only second company to eclipse milestone number</t>
+          <t>Apple doubled the price of its TV streaming box from $150 to $300, and even the company's hardcore fans are...</t>
         </is>
       </c>
       <c r="AY24" s="79" t="inlineStr">
         <is>
-          <t>OpenAI Employee Allegedly Took Secret AI Device Files to Apple, Presented it to Top Executives.</t>
+          <t>Here's What a $10,000 Investment in Apple Stock Could Be Worth in 5 Years</t>
         </is>
       </c>
       <c r="AZ24" s="79" t="inlineStr">
         <is>
-          <t>Gene Munster Warns Apple Can Sell Millions of iPhones and Still Lose the AI Game as Users Could Lock Into M...</t>
+          <t>Apple Hits $5 Trillion Milestone as Rest of Tech Trade Falters. Can It Hold?</t>
         </is>
       </c>
     </row>
@@ -6690,10 +6690,10 @@
         <v>567</v>
       </c>
       <c r="W25" s="84" t="n">
-        <v>21880824</v>
+        <v>22119483</v>
       </c>
       <c r="X25" s="85" t="n">
-        <v>1.008973103634531</v>
+        <v>1.019417257934239</v>
       </c>
       <c r="Y25" s="35" t="n">
         <v>46.50479793939365</v>
@@ -6772,17 +6772,17 @@
       </c>
       <c r="AX25" s="90" t="inlineStr">
         <is>
+          <t>Dow Jones Futures: Techs Fall On Anthropic News After Dell, AMD, CoreWeave Dive In AI-Led Sell-Off</t>
+        </is>
+      </c>
+      <c r="AY25" s="90" t="inlineStr">
+        <is>
           <t>KBW keeps Core Scientific at outperform, says AMD’s 1.9 GW reservation is overlooked</t>
         </is>
       </c>
-      <c r="AY25" s="90" t="inlineStr">
+      <c r="AZ25" s="90" t="inlineStr">
         <is>
           <t>Advanced Micro Devices Just Unveiled Its Helion Blueprint for Agentic AI. What That Means for AMD Stock.</t>
-        </is>
-      </c>
-      <c r="AZ25" s="90" t="inlineStr">
-        <is>
-          <t>AMD Is Paying $8.2 Billion to Bring In the ‘Godmother of AI.’ Here’s Why It Makes Sense</t>
         </is>
       </c>
     </row>
@@ -6878,10 +6878,10 @@
         <v>252.6600036621094</v>
       </c>
       <c r="W26" s="73" t="n">
-        <v>33260130</v>
+        <v>34598204</v>
       </c>
       <c r="X26" s="74" t="n">
-        <v>0.9209708096452293</v>
+        <v>0.9562504801193192</v>
       </c>
       <c r="Y26" s="28" t="n">
         <v>49.33534011995938</v>
@@ -6960,17 +6960,17 @@
       </c>
       <c r="AX26" s="79" t="inlineStr">
         <is>
+          <t>Amazon.com (AMZN) Could See Blue Origin Go Public</t>
+        </is>
+      </c>
+      <c r="AY26" s="79" t="inlineStr">
+        <is>
+          <t>Amazon Is the Most Crowded Stock for Hedge Funds. Tesla, Not So Much.</t>
+        </is>
+      </c>
+      <c r="AZ26" s="79" t="inlineStr">
+        <is>
           <t>Amazon (AMZN) Has a $25B Chip Business. Is the Cash Burn Worth It?</t>
-        </is>
-      </c>
-      <c r="AY26" s="79" t="inlineStr">
-        <is>
-          <t>Amazon customers could be eligible for payments in $309.5M lawsuit</t>
-        </is>
-      </c>
-      <c r="AZ26" s="79" t="inlineStr">
-        <is>
-          <t>Amazon’s $550 tablet breaks its oldest hardware rule</t>
         </is>
       </c>
     </row>
@@ -7066,10 +7066,10 @@
         <v>83.98000335693359</v>
       </c>
       <c r="W27" s="84" t="n">
-        <v>4098503</v>
+        <v>4111664</v>
       </c>
       <c r="X27" s="85" t="n">
-        <v>0.8971104386137938</v>
+        <v>0.8998615999559837</v>
       </c>
       <c r="Y27" s="35" t="n">
         <v>42.51217461477839</v>
@@ -7182,7 +7182,7 @@
       </c>
       <c r="F28" s="23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Same</t>
         </is>
       </c>
       <c r="G28" s="23" t="inlineStr">
@@ -7254,10 +7254,10 @@
         <v>237.5500030517578</v>
       </c>
       <c r="W28" s="73" t="n">
-        <v>6549262</v>
+        <v>6604374</v>
       </c>
       <c r="X28" s="74" t="n">
-        <v>1.068151487341851</v>
+        <v>1.076656100090873</v>
       </c>
       <c r="Y28" s="28" t="n">
         <v>35.86605857400195</v>
@@ -7433,7 +7433,7 @@
         <v>-4.924999237060547</v>
       </c>
       <c r="T29" s="83" t="n">
-        <v>45.5</v>
+        <v>45.54000091552734</v>
       </c>
       <c r="U29" s="83" t="n">
         <v>45.97999954223633</v>
@@ -7442,10 +7442,10 @@
         <v>42</v>
       </c>
       <c r="W29" s="84" t="n">
-        <v>26702718</v>
+        <v>27212216</v>
       </c>
       <c r="X29" s="85" t="n">
-        <v>1.665547567971422</v>
+        <v>1.694634135429711</v>
       </c>
       <c r="Y29" s="35" t="n">
         <v>27.74802911954028</v>
@@ -7630,10 +7630,10 @@
         <v>342.8200988769531</v>
       </c>
       <c r="W30" s="73" t="n">
-        <v>22727383</v>
+        <v>22989932</v>
       </c>
       <c r="X30" s="74" t="n">
-        <v>0.9958607144680036</v>
+        <v>1.006785879517827</v>
       </c>
       <c r="Y30" s="28" t="n">
         <v>42.28325957381871</v>
@@ -7712,17 +7712,17 @@
       </c>
       <c r="AX30" s="79" t="inlineStr">
         <is>
+          <t>Broadcom vs. Marvell Technology: Which Technology Stock Is a Better Buy in 2026?</t>
+        </is>
+      </c>
+      <c r="AY30" s="79" t="inlineStr">
+        <is>
+          <t>A $10,000 Broadcom investment in 2016 now pays $1,991 a year in dividends</t>
+        </is>
+      </c>
+      <c r="AZ30" s="79" t="inlineStr">
+        <is>
           <t>Broadcom is The Steady Hand The Market Keeps Discounting</t>
-        </is>
-      </c>
-      <c r="AY30" s="79" t="inlineStr">
-        <is>
-          <t>Broadcom vs. Nvidia: If I Could Only Own One for the Next 5 Years, It Would Be This One</t>
-        </is>
-      </c>
-      <c r="AZ30" s="79" t="inlineStr">
-        <is>
-          <t>Broadcom And 2 Cash Flow Stocks To Watch</t>
         </is>
       </c>
     </row>
@@ -7818,10 +7818,10 @@
         <v>81.22000122070312</v>
       </c>
       <c r="W31" s="84" t="n">
-        <v>5584707</v>
+        <v>5695409</v>
       </c>
       <c r="X31" s="85" t="n">
-        <v>1.632580366376978</v>
+        <v>1.662252285830416</v>
       </c>
       <c r="Y31" s="35" t="n">
         <v>33.84528591909125</v>
@@ -7900,17 +7900,17 @@
       </c>
       <c r="AX31" s="90" t="inlineStr">
         <is>
+          <t>Why Cameco (CCJ) Dipped More Than Broader Market Today</t>
+        </is>
+      </c>
+      <c r="AY31" s="90" t="inlineStr">
+        <is>
           <t>Is Cameco (CCJ) a Buy Before the Westinghouse Spin-Off?</t>
         </is>
       </c>
-      <c r="AY31" s="90" t="inlineStr">
+      <c r="AZ31" s="90" t="inlineStr">
         <is>
           <t>Cameco Heads 3 Canadian Nuclear Stocks To Watch</t>
-        </is>
-      </c>
-      <c r="AZ31" s="90" t="inlineStr">
-        <is>
-          <t>3 Stocks to Buy If You Think the Nuclear Fuel Shortage Is the Real Story, Not the Reactors</t>
         </is>
       </c>
     </row>
@@ -8006,10 +8006,10 @@
         <v>64.41000366210938</v>
       </c>
       <c r="W32" s="73" t="n">
-        <v>107287990</v>
+        <v>109419566</v>
       </c>
       <c r="X32" s="74" t="n">
-        <v>3.036391432630929</v>
+        <v>3.08740523759355</v>
       </c>
       <c r="Y32" s="28" t="n">
         <v>29.17768071148392</v>
@@ -8093,12 +8093,12 @@
       </c>
       <c r="AY32" s="79" t="inlineStr">
         <is>
-          <t>Why CoreWeave Stock Tumbled Today</t>
+          <t>Dow Jones Futures: Techs Fall On Anthropic News After Dell, AMD, CoreWeave Dive In AI-Led Sell-Off</t>
         </is>
       </c>
       <c r="AZ32" s="79" t="inlineStr">
         <is>
-          <t>Stock Market Midday, Oct. 14: Hot Inflation Weighs on Markets, CoreWeave Plummets 15%</t>
+          <t>CoreWeave Stock Sinks on Credit Market’s Warning Sign. Even Elon Musk Says ‘Yikes.’</t>
         </is>
       </c>
     </row>
@@ -8194,10 +8194,10 @@
         <v>502.3432006835938</v>
       </c>
       <c r="W33" s="84" t="n">
-        <v>11615461</v>
+        <v>11672615</v>
       </c>
       <c r="X33" s="85" t="n">
-        <v>1.660042137100161</v>
+        <v>1.667529351923906</v>
       </c>
       <c r="Y33" s="35" t="n">
         <v>41.92001266731174</v>
@@ -8276,17 +8276,17 @@
       </c>
       <c r="AX33" s="90" t="inlineStr">
         <is>
-          <t>Why Dell Stock Is Having Its Worst Day in More Than a Year</t>
+          <t>Dow Jones Futures: Techs Fall On Anthropic News After Dell, AMD, CoreWeave Dive In AI-Led Sell-Off</t>
         </is>
       </c>
       <c r="AY33" s="90" t="inlineStr">
         <is>
-          <t>Top Midday Decliners</t>
+          <t>Dell leads CIO spending plans as hardware prices jump</t>
         </is>
       </c>
       <c r="AZ33" s="90" t="inlineStr">
         <is>
-          <t>Why Dell (DELL) Stock Is Falling Today</t>
+          <t>Dell Just Found Out What Gravity Feels Like</t>
         </is>
       </c>
     </row>
@@ -8382,10 +8382,10 @@
         <v>342.3999938964844</v>
       </c>
       <c r="W34" s="73" t="n">
-        <v>19020009</v>
+        <v>20028772</v>
       </c>
       <c r="X34" s="74" t="n">
-        <v>1.120278414145583</v>
+        <v>1.176200284976213</v>
       </c>
       <c r="Y34" s="28" t="n">
         <v>50.62695058808003</v>
@@ -8469,12 +8469,12 @@
       </c>
       <c r="AY34" s="79" t="inlineStr">
         <is>
-          <t>3 Cloud Leaders That Will Make a Fortune From AI</t>
+          <t>Gene Munster Flags Meta’s Muse As A Bigger Risk To Google Search Than ChatGPT</t>
         </is>
       </c>
       <c r="AZ34" s="79" t="inlineStr">
         <is>
-          <t>Google's Gemini 4 Argon Is the Most Accurate and Most Consistent AI Model on Accounting Work, DualEntry Ben...</t>
+          <t>Alphabet (GOOGL) Falls More Steeply Than Broader Market: What Investors Need to Know</t>
         </is>
       </c>
     </row>
@@ -8570,10 +8570,10 @@
         <v>30.3799991607666</v>
       </c>
       <c r="W35" s="84" t="n">
-        <v>75919983</v>
+        <v>77249064</v>
       </c>
       <c r="X35" s="85" t="n">
-        <v>1.83066037387632</v>
+        <v>1.859728491950499</v>
       </c>
       <c r="Y35" s="35" t="n">
         <v>26.5796008944031</v>
@@ -8758,10 +8758,10 @@
         <v>97.66999816894531</v>
       </c>
       <c r="W36" s="73" t="n">
-        <v>102340556</v>
+        <v>103750027</v>
       </c>
       <c r="X36" s="74" t="n">
-        <v>0.9526440834512875</v>
+        <v>0.965131107303464</v>
       </c>
       <c r="Y36" s="28" t="n">
         <v>37.8870839720441</v>
@@ -8946,10 +8946,10 @@
         <v>532.5399780273438</v>
       </c>
       <c r="W37" s="84" t="n">
-        <v>21176641</v>
+        <v>22251503</v>
       </c>
       <c r="X37" s="85" t="n">
-        <v>0.9335199679028027</v>
+        <v>0.9785842119603223</v>
       </c>
       <c r="Y37" s="35" t="n">
         <v>62.44641478118911</v>
@@ -9028,17 +9028,17 @@
       </c>
       <c r="AX37" s="90" t="inlineStr">
         <is>
+          <t>Microsoft Just Unveiled a Brand-New AI Chip. Could It Be the "Nvidia Killer" Everyone's Been Looking For?</t>
+        </is>
+      </c>
+      <c r="AY37" s="90" t="inlineStr">
+        <is>
           <t>Sara Eisen Went on Bill Maher and Said What Wall Street Will Not About the AI Race</t>
         </is>
       </c>
-      <c r="AY37" s="90" t="inlineStr">
+      <c r="AZ37" s="90" t="inlineStr">
         <is>
           <t>Citi Says the S&amp;P 500 Hits 8,100. Half the Market Has to Cooperate First.</t>
-        </is>
-      </c>
-      <c r="AZ37" s="90" t="inlineStr">
-        <is>
-          <t>Microsoft (MSFT) Built a $100B Azure. Can It Outrun Its Own Spending?</t>
         </is>
       </c>
     </row>
@@ -9131,22 +9131,22 @@
         <v>152.1799926757812</v>
       </c>
       <c r="V38" s="72" t="n">
-        <v>141.7599945068359</v>
+        <v>141.7400054931641</v>
       </c>
       <c r="W38" s="73" t="n">
-        <v>20524146</v>
+        <v>20701924</v>
       </c>
       <c r="X38" s="74" t="n">
-        <v>0.94141834820574</v>
+        <v>0.9491858099804279</v>
       </c>
       <c r="Y38" s="28" t="n">
         <v>46.00424202192021</v>
       </c>
       <c r="Z38" s="28" t="n">
-        <v>5.209471297260079</v>
+        <v>5.276118137300155</v>
       </c>
       <c r="AA38" s="28" t="n">
-        <v>30.01535600724731</v>
+        <v>30.01768782058695</v>
       </c>
       <c r="AB38" s="75" t="n">
         <v>4.489594668743763</v>
@@ -9188,7 +9188,7 @@
         <v>20.93576226223079</v>
       </c>
       <c r="AO38" s="77" t="n">
-        <v>6.000360045882449</v>
+        <v>6.001356825159252</v>
       </c>
       <c r="AP38" s="72" t="n">
         <v>312.7099914550781</v>
@@ -9319,22 +9319,22 @@
         <v>949.4199829101562</v>
       </c>
       <c r="V39" s="83" t="n">
-        <v>913.5999755859375</v>
+        <v>913.5599975585938</v>
       </c>
       <c r="W39" s="84" t="n">
-        <v>26415343</v>
+        <v>27296988</v>
       </c>
       <c r="X39" s="85" t="n">
-        <v>1.003747268778443</v>
+        <v>1.03551403091591</v>
       </c>
       <c r="Y39" s="35" t="n">
         <v>36.24755467790129</v>
       </c>
       <c r="Z39" s="35" t="n">
-        <v>0.2716427378735166</v>
+        <v>0.2920718398524348</v>
       </c>
       <c r="AA39" s="35" t="n">
-        <v>17.77651915022507</v>
+        <v>17.77703541450669</v>
       </c>
       <c r="AB39" s="86" t="n">
         <v>-2.211312594369929</v>
@@ -9376,7 +9376,7 @@
         <v>18.60696339676301</v>
       </c>
       <c r="AO39" s="88" t="n">
-        <v>5.111058142523979</v>
+        <v>5.111370524063415</v>
       </c>
       <c r="AP39" s="83" t="n">
         <v>1255</v>
@@ -9510,10 +9510,10 @@
         <v>183.1300048828125</v>
       </c>
       <c r="W40" s="73" t="n">
-        <v>32885932</v>
+        <v>33609105</v>
       </c>
       <c r="X40" s="74" t="n">
-        <v>1.893951446277898</v>
+        <v>1.931577712706544</v>
       </c>
       <c r="Y40" s="28" t="n">
         <v>35.29776511268888</v>
@@ -9698,10 +9698,10 @@
         <v>69.37000274658203</v>
       </c>
       <c r="W41" s="84" t="n">
-        <v>38228573</v>
+        <v>39920482</v>
       </c>
       <c r="X41" s="85" t="n">
-        <v>1.005399704214988</v>
+        <v>1.047565730026242</v>
       </c>
       <c r="Y41" s="35" t="n">
         <v>44.86160952076844</v>
@@ -9785,12 +9785,12 @@
       </c>
       <c r="AY41" s="90" t="inlineStr">
         <is>
+          <t>Netflix to Cut 6% of Staff After Steep Stock Decline. How We Got Here.</t>
+        </is>
+      </c>
+      <c r="AZ41" s="90" t="inlineStr">
+        <is>
           <t>Netflix to Reportedly Cut About 1,000 Roles as Streamer Reallocates Resources</t>
-        </is>
-      </c>
-      <c r="AZ41" s="90" t="inlineStr">
-        <is>
-          <t>Netflix to lay off roughly 1,000 employees</t>
         </is>
       </c>
     </row>
@@ -9814,7 +9814,7 @@
       </c>
       <c r="F42" s="23" t="inlineStr">
         <is>
-          <t>Same</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G42" s="23" t="inlineStr">
@@ -9886,10 +9886,10 @@
         <v>9.300000190734863</v>
       </c>
       <c r="W42" s="73" t="n">
-        <v>78512645</v>
+        <v>85996980</v>
       </c>
       <c r="X42" s="74" t="n">
-        <v>1.005016821575992</v>
+        <v>1.095573493243081</v>
       </c>
       <c r="Y42" s="28" t="n">
         <v>39.49512696120658</v>
@@ -10074,10 +10074,10 @@
         <v>219.6399993896484</v>
       </c>
       <c r="W43" s="84" t="n">
-        <v>115959194</v>
+        <v>117762243</v>
       </c>
       <c r="X43" s="85" t="n">
-        <v>1.088306659903889</v>
+        <v>1.104294387745933</v>
       </c>
       <c r="Y43" s="35" t="n">
         <v>43.94171792913651</v>
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
-          <t>Nvidia stock sinks as chip sell-off deepens on hot inflation data</t>
+          <t>Nvidia, Anthropic Weigh In On AI Safeguards</t>
         </is>
       </c>
       <c r="AY43" s="90" t="inlineStr">
         <is>
-          <t>Bank of America Corporation Q3 2026 Earnings Call Summary</t>
+          <t>Got $5,000? 2 Stocks Supplying the AI Data Center Power Crunch.</t>
         </is>
       </c>
       <c r="AZ43" s="90" t="inlineStr">
         <is>
-          <t>What Is the Worth of Rare Earth?</t>
+          <t>Dell Just Found Out What Gravity Feels Like</t>
         </is>
       </c>
     </row>
@@ -10262,10 +10262,10 @@
         <v>199.7400054931641</v>
       </c>
       <c r="W44" s="73" t="n">
-        <v>23865536</v>
+        <v>24103301</v>
       </c>
       <c r="X44" s="74" t="n">
-        <v>1.022206162355125</v>
+        <v>1.031864666510699</v>
       </c>
       <c r="Y44" s="28" t="n">
         <v>63.25256875049414</v>
@@ -10450,10 +10450,10 @@
         <v>171.0200042724609</v>
       </c>
       <c r="W45" s="84" t="n">
-        <v>11121441</v>
+        <v>11157772</v>
       </c>
       <c r="X45" s="85" t="n">
-        <v>0.8409453570483022</v>
+        <v>0.8435766457285828</v>
       </c>
       <c r="Y45" s="35" t="n">
         <v>42.27019369380251</v>
@@ -10638,10 +10638,10 @@
         <v>58.84000015258789</v>
       </c>
       <c r="W46" s="73" t="n">
-        <v>20897306</v>
+        <v>24121394</v>
       </c>
       <c r="X46" s="74" t="n">
-        <v>0.9749963179812783</v>
+        <v>1.117019782661722</v>
       </c>
       <c r="Y46" s="28" t="n">
         <v>33.22450083013594</v>
@@ -10720,17 +10720,17 @@
       </c>
       <c r="AX46" s="79" t="inlineStr">
         <is>
+          <t>RKLB Stock Slides 8% After Hours As Neutron Debut Slips Into 2027 Over Manufacturing Issues: CEO Says ‘Poss...</t>
+        </is>
+      </c>
+      <c r="AY46" s="79" t="inlineStr">
+        <is>
+          <t>Rocket Lab stock falls after delaying Neutron rocket to 2027</t>
+        </is>
+      </c>
+      <c r="AZ46" s="79" t="inlineStr">
+        <is>
           <t>Rocket Lab Provides Update on Neutron Development and Adjusts Target Launch Timing</t>
-        </is>
-      </c>
-      <c r="AY46" s="79" t="inlineStr">
-        <is>
-          <t>AST SpaceMobile Falls 8% as Piper Sandler Cuts Target to $54 on SpaceX Competition; Rocket Lab Slips</t>
-        </is>
-      </c>
-      <c r="AZ46" s="79" t="inlineStr">
-        <is>
-          <t>Is Rocket Lab Stock Ready For A Neutron Delay?</t>
         </is>
       </c>
     </row>
@@ -10823,13 +10823,13 @@
         <v>1461.799926757812</v>
       </c>
       <c r="V47" s="83" t="n">
-        <v>1402.06005859375</v>
+        <v>1402.02001953125</v>
       </c>
       <c r="W47" s="84" t="n">
-        <v>7073146</v>
+        <v>7345106</v>
       </c>
       <c r="X47" s="85" t="n">
-        <v>0.8298325458768667</v>
+        <v>0.860366741932345</v>
       </c>
       <c r="Y47" s="35" t="n">
         <v>34.34738914248405</v>
@@ -10880,7 +10880,7 @@
         <v>28.51545091468194</v>
       </c>
       <c r="AO47" s="88" t="n">
-        <v>6.757778980979887</v>
+        <v>6.75798277571996</v>
       </c>
       <c r="AP47" s="83" t="n">
         <v>2354.389892578125</v>
@@ -10908,17 +10908,17 @@
       </c>
       <c r="AX47" s="90" t="inlineStr">
         <is>
+          <t>Top Research Reports for Mastercard, AstraZeneca &amp; Sandisk</t>
+        </is>
+      </c>
+      <c r="AY47" s="90" t="inlineStr">
+        <is>
           <t>Why SandiskStock Keeps Going Down</t>
         </is>
       </c>
-      <c r="AY47" s="90" t="inlineStr">
+      <c r="AZ47" s="90" t="inlineStr">
         <is>
           <t>AI Memory Chip Selloff Looks Overblown: 2 Stocks to Buy on the Dip</t>
-        </is>
-      </c>
-      <c r="AZ47" s="90" t="inlineStr">
-        <is>
-          <t>Arm vs. Sandisk: Which Tech Stock Is a Better Buy in October?</t>
         </is>
       </c>
     </row>
@@ -11014,10 +11014,10 @@
         <v>363.8200073242188</v>
       </c>
       <c r="W48" s="73" t="n">
-        <v>29381134</v>
+        <v>30868569</v>
       </c>
       <c r="X48" s="74" t="n">
-        <v>0.8517702266465265</v>
+        <v>0.8929662383855183</v>
       </c>
       <c r="Y48" s="28" t="n">
         <v>49.26645898543141</v>
@@ -11106,7 +11106,7 @@
       </c>
       <c r="AZ48" s="79" t="inlineStr">
         <is>
-          <t>Tesla Just Launched the Cybercab in Austin. Here's How Many People Can Actually Hail One.</t>
+          <t>Tesla's Elon Musk Might Have Gone Back on His Word, but It's Working in China</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 14 Oct 2026, 08:51 PM · Yahoo Finance data</t>
+          <t>Built 14 Oct 2026, 11:16 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 14 Oct 2026, 08:51 PM · Yahoo Finance data</t>
+          <t>Built 14 Oct 2026, 11:16 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 14 Oct 2026, 08:51 PM · Yahoo Finance data</t>
+          <t>Built 14 Oct 2026, 11:16 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 14 Oct 2026, 08:51 PM · Yahoo Finance data</t>
+          <t>Built 14 Oct 2026, 11:16 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -45564,7 +45564,7 @@
       </c>
       <c r="D64" s="107" t="inlineStr">
         <is>
-          <t>Gapped down 3.3% at the open</t>
+          <t>Gapped down 3.2% at the open</t>
         </is>
       </c>
       <c r="E64" s="26" t="n">
@@ -45620,7 +45620,7 @@
       </c>
       <c r="D66" s="107" t="inlineStr">
         <is>
-          <t>Volume 1.8x its 20-day average</t>
+          <t>Volume 1.9x its 20-day average</t>
         </is>
       </c>
       <c r="E66" s="26" t="n">
@@ -45844,7 +45844,7 @@
       </c>
       <c r="D74" s="107" t="inlineStr">
         <is>
-          <t>Volume 3.0x its 20-day average</t>
+          <t>Volume 3.1x its 20-day average</t>
         </is>
       </c>
       <c r="E74" s="26" t="n">

</xml_diff>

<commit_message>
Daily workbook: 2026-10-14 23:54 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 14 Oct 2026, 11:16 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 14 Oct 2026, 11:54 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 14 Oct 2026, 11:16 PM · Yahoo Finance data</t>
+          <t>Built 14 Oct 2026, 11:54 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -5999,17 +5999,17 @@
       </c>
       <c r="AX20" s="90" t="inlineStr">
         <is>
+          <t>Invesco QQQ Doesn't Own a Single Bank, and That's Not the Only Thing the Nasdaq-100 Leaves Out</t>
+        </is>
+      </c>
+      <c r="AY20" s="90" t="inlineStr">
+        <is>
           <t>Exchange-Traded Funds Lower as US Equities Drop After Midday</t>
         </is>
       </c>
-      <c r="AY20" s="90" t="inlineStr">
+      <c r="AZ20" s="90" t="inlineStr">
         <is>
           <t>Exchange-Traded Funds Higher, Equity Futures Mixed Pre-Bell Wednesday Amid September Consumer Inflation Data</t>
-        </is>
-      </c>
-      <c r="AZ20" s="90" t="inlineStr">
-        <is>
-          <t>Southern Glazer’s Wine &amp; Spirits Continues Longstanding Partnership as Exclusive Provider of Wine and Spiri...</t>
         </is>
       </c>
     </row>
@@ -8469,12 +8469,12 @@
       </c>
       <c r="AY34" s="79" t="inlineStr">
         <is>
+          <t>Prediction: Alphabet Will Soar After Oct. 28</t>
+        </is>
+      </c>
+      <c r="AZ34" s="79" t="inlineStr">
+        <is>
           <t>Gene Munster Flags Meta’s Muse As A Bigger Risk To Google Search Than ChatGPT</t>
-        </is>
-      </c>
-      <c r="AZ34" s="79" t="inlineStr">
-        <is>
-          <t>Alphabet (GOOGL) Falls More Steeply Than Broader Market: What Investors Need to Know</t>
         </is>
       </c>
     </row>
@@ -9414,7 +9414,7 @@
       </c>
       <c r="AZ39" s="90" t="inlineStr">
         <is>
-          <t>'Smart move': What Elon Musk had to say about Micron</t>
+          <t>China's Competitive Threat To Micron Called 'Paper Tiger'</t>
         </is>
       </c>
     </row>
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
+          <t>Britain lacks entrepreneurial spirit, Nvidia boss warns</t>
+        </is>
+      </c>
+      <c r="AY43" s="90" t="inlineStr">
+        <is>
           <t>Nvidia, Anthropic Weigh In On AI Safeguards</t>
         </is>
       </c>
-      <c r="AY43" s="90" t="inlineStr">
+      <c r="AZ43" s="90" t="inlineStr">
         <is>
           <t>Got $5,000? 2 Stocks Supplying the AI Data Center Power Crunch.</t>
-        </is>
-      </c>
-      <c r="AZ43" s="90" t="inlineStr">
-        <is>
-          <t>Dell Just Found Out What Gravity Feels Like</t>
         </is>
       </c>
     </row>
@@ -11106,7 +11106,7 @@
       </c>
       <c r="AZ48" s="79" t="inlineStr">
         <is>
-          <t>Tesla's Elon Musk Might Have Gone Back on His Word, but It's Working in China</t>
+          <t>Tesla-SpaceX Merger Could Be Announced As Early As Before December AGM, Says Barclays</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 14 Oct 2026, 11:16 PM · Yahoo Finance data</t>
+          <t>Built 14 Oct 2026, 11:54 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 14 Oct 2026, 11:16 PM · Yahoo Finance data</t>
+          <t>Built 14 Oct 2026, 11:54 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 14 Oct 2026, 11:16 PM · Yahoo Finance data</t>
+          <t>Built 14 Oct 2026, 11:54 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 14 Oct 2026, 11:16 PM · Yahoo Finance data</t>
+          <t>Built 14 Oct 2026, 11:54 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-10-15 23:05 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 15 Oct 2026, 08:27 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 15 Oct 2026, 11:05 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -1390,7 +1390,7 @@
       <c r="J8" s="6" t="n"/>
       <c r="K8" s="15" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="L8" s="10" t="n"/>
@@ -1658,7 +1658,7 @@
         <v>0.01375641954700679</v>
       </c>
       <c r="F18" s="27" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G18" s="28" t="n">
         <v>52.17617960272845</v>
@@ -2058,11 +2058,11 @@
     <row r="32">
       <c r="B32" s="31" t="inlineStr">
         <is>
-          <t>XLE</t>
+          <t>XLF</t>
         </is>
       </c>
       <c r="C32" s="33" t="n">
-        <v>-0.01582137717401932</v>
+        <v>0.01375641954700679</v>
       </c>
       <c r="D32" s="34" t="n">
         <v>8</v>
@@ -2073,7 +2073,7 @@
         </is>
       </c>
       <c r="F32" s="35" t="n">
-        <v>63.32604798826599</v>
+        <v>52.17617960272845</v>
       </c>
       <c r="H32" s="31" t="inlineStr">
         <is>
@@ -2098,22 +2098,22 @@
     <row r="33">
       <c r="B33" s="24" t="inlineStr">
         <is>
-          <t>XLB</t>
+          <t>XLE</t>
         </is>
       </c>
       <c r="C33" s="26" t="n">
-        <v>0.01791832569267449</v>
+        <v>-0.01582137717401932</v>
       </c>
       <c r="D33" s="27" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E33" s="23" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Very Strong</t>
         </is>
       </c>
       <c r="F33" s="28" t="n">
-        <v>55.19817695478138</v>
+        <v>63.32604798826599</v>
       </c>
       <c r="H33" s="24" t="inlineStr">
         <is>
@@ -2138,11 +2138,11 @@
     <row r="34">
       <c r="B34" s="31" t="inlineStr">
         <is>
-          <t>XLC</t>
+          <t>NFLX</t>
         </is>
       </c>
       <c r="C34" s="33" t="n">
-        <v>0.01461832477028691</v>
+        <v>0.02890748086083605</v>
       </c>
       <c r="D34" s="34" t="n">
         <v>7</v>
@@ -2153,7 +2153,7 @@
         </is>
       </c>
       <c r="F34" s="35" t="n">
-        <v>52.4207922981891</v>
+        <v>51.97743826050299</v>
       </c>
       <c r="H34" s="31" t="inlineStr">
         <is>
@@ -2161,7 +2161,7 @@
         </is>
       </c>
       <c r="I34" s="33" t="n">
-        <v>0.01356079427348655</v>
+        <v>0.01367133994853043</v>
       </c>
       <c r="J34" s="34" t="n">
         <v>1</v>
@@ -2172,17 +2172,17 @@
         </is>
       </c>
       <c r="L34" s="35" t="n">
-        <v>37.24824783586103</v>
+        <v>37.31282542253678</v>
       </c>
     </row>
     <row r="35">
       <c r="B35" s="24" t="inlineStr">
         <is>
-          <t>XLF</t>
+          <t>XLB</t>
         </is>
       </c>
       <c r="C35" s="26" t="n">
-        <v>0.01375641954700679</v>
+        <v>0.01791832569267449</v>
       </c>
       <c r="D35" s="27" t="n">
         <v>7</v>
@@ -2193,7 +2193,7 @@
         </is>
       </c>
       <c r="F35" s="28" t="n">
-        <v>52.17617960272845</v>
+        <v>55.19817695478138</v>
       </c>
       <c r="H35" s="24" t="inlineStr">
         <is>
@@ -2218,11 +2218,11 @@
     <row r="36">
       <c r="B36" s="31" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>XLC</t>
         </is>
       </c>
       <c r="C36" s="33" t="n">
-        <v>0.003666549652273643</v>
+        <v>0.01461832477028691</v>
       </c>
       <c r="D36" s="34" t="n">
         <v>7</v>
@@ -2233,7 +2233,7 @@
         </is>
       </c>
       <c r="F36" s="35" t="n">
-        <v>51.9391021227524</v>
+        <v>52.4207922981891</v>
       </c>
       <c r="H36" s="31" t="inlineStr">
         <is>
@@ -2258,11 +2258,11 @@
     <row r="37">
       <c r="B37" s="24" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="C37" s="26" t="n">
-        <v>-0.002338663570922606</v>
+        <v>0.003666549652273643</v>
       </c>
       <c r="D37" s="27" t="n">
         <v>7</v>
@@ -2273,7 +2273,7 @@
         </is>
       </c>
       <c r="F37" s="28" t="n">
-        <v>62.58014496903483</v>
+        <v>51.9391021227524</v>
       </c>
       <c r="H37" s="24" t="inlineStr">
         <is>
@@ -2298,11 +2298,11 @@
     <row r="38">
       <c r="B38" s="31" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="C38" s="33" t="n">
-        <v>-0.00279913540645127</v>
+        <v>-0.002338663570922606</v>
       </c>
       <c r="D38" s="34" t="n">
         <v>7</v>
@@ -2313,7 +2313,7 @@
         </is>
       </c>
       <c r="F38" s="35" t="n">
-        <v>60.57988770507023</v>
+        <v>62.58014496903483</v>
       </c>
       <c r="H38" s="31" t="inlineStr">
         <is>
@@ -2569,7 +2569,7 @@
         <v>0.02890748086083605</v>
       </c>
       <c r="D47" s="27" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E47" s="23" t="inlineStr">
         <is>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 15 Oct 2026, 08:27 PM · Yahoo Finance data</t>
+          <t>Built 15 Oct 2026, 11:05 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -3142,7 +3142,7 @@
       </c>
       <c r="AC3" s="46" t="inlineStr">
         <is>
-          <t>4.0 / 9</t>
+          <t>4.1 / 9</t>
         </is>
       </c>
       <c r="AE3" s="47" t="inlineStr">
@@ -3620,10 +3620,10 @@
         <v>164.6600036621094</v>
       </c>
       <c r="W7" s="73" t="n">
-        <v>7543373</v>
+        <v>7618716</v>
       </c>
       <c r="X7" s="74" t="n">
-        <v>1.01567114665723</v>
+        <v>1.025295586550958</v>
       </c>
       <c r="Y7" s="28" t="n">
         <v>41.66117426398795</v>
@@ -3810,10 +3810,10 @@
         <v>176.3000030517578</v>
       </c>
       <c r="W8" s="84" t="n">
-        <v>11338999</v>
+        <v>11462690</v>
       </c>
       <c r="X8" s="85" t="n">
-        <v>1.316417202450199</v>
+        <v>1.329822466857806</v>
       </c>
       <c r="Y8" s="35" t="n">
         <v>67.49839028620065</v>
@@ -3967,11 +3967,11 @@
         </is>
       </c>
       <c r="N9" s="69" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="O9" s="23" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Very Strong</t>
         </is>
       </c>
       <c r="P9" s="25" t="inlineStr">
@@ -4000,10 +4000,10 @@
         <v>54.59000015258789</v>
       </c>
       <c r="W9" s="73" t="n">
-        <v>43693291</v>
+        <v>45293407</v>
       </c>
       <c r="X9" s="74" t="n">
-        <v>1.119713337663497</v>
+        <v>1.158344042830177</v>
       </c>
       <c r="Y9" s="28" t="n">
         <v>52.17617960272845</v>
@@ -4190,10 +4190,10 @@
         <v>66.16999816894531</v>
       </c>
       <c r="W10" s="84" t="n">
-        <v>31265312</v>
+        <v>31312005</v>
       </c>
       <c r="X10" s="85" t="n">
-        <v>0.9675476761825617</v>
+        <v>0.9689226510628638</v>
       </c>
       <c r="Y10" s="35" t="n">
         <v>63.32604798826599</v>
@@ -4380,10 +4380,10 @@
         <v>86.59500122070312</v>
       </c>
       <c r="W11" s="73" t="n">
-        <v>23369861</v>
+        <v>23959739</v>
       </c>
       <c r="X11" s="74" t="n">
-        <v>2.032349500308857</v>
+        <v>2.078317251115838</v>
       </c>
       <c r="Y11" s="28" t="n">
         <v>68.85201064323559</v>
@@ -4570,10 +4570,10 @@
         <v>111.7149963378906</v>
       </c>
       <c r="W12" s="84" t="n">
-        <v>6103298</v>
+        <v>6107725</v>
       </c>
       <c r="X12" s="85" t="n">
-        <v>0.9496407077634853</v>
+        <v>0.9502967963574984</v>
       </c>
       <c r="Y12" s="35" t="n">
         <v>56.41431654327126</v>
@@ -4760,10 +4760,10 @@
         <v>110.2799987792969</v>
       </c>
       <c r="W13" s="73" t="n">
-        <v>6521177</v>
+        <v>6525994</v>
       </c>
       <c r="X13" s="74" t="n">
-        <v>0.9751039219713145</v>
+        <v>0.975789060228295</v>
       </c>
       <c r="Y13" s="28" t="n">
         <v>52.4207922981891</v>
@@ -4950,10 +4950,10 @@
         <v>49.90000152587891</v>
       </c>
       <c r="W14" s="84" t="n">
-        <v>14833292</v>
+        <v>14847401</v>
       </c>
       <c r="X14" s="85" t="n">
-        <v>1.27278185766994</v>
+        <v>1.27391537887635</v>
       </c>
       <c r="Y14" s="35" t="n">
         <v>55.19817695478138</v>
@@ -5140,10 +5140,10 @@
         <v>184.8399963378906</v>
       </c>
       <c r="W15" s="73" t="n">
-        <v>13577943</v>
+        <v>13670787</v>
       </c>
       <c r="X15" s="74" t="n">
-        <v>1.737356892894204</v>
+        <v>1.748198274962676</v>
       </c>
       <c r="Y15" s="28" t="n">
         <v>41.09175478737813</v>
@@ -5330,10 +5330,10 @@
         <v>41.81999969482422</v>
       </c>
       <c r="W16" s="84" t="n">
-        <v>9511506</v>
+        <v>9638982</v>
       </c>
       <c r="X16" s="85" t="n">
-        <v>1.302800524209947</v>
+        <v>1.319109423348576</v>
       </c>
       <c r="Y16" s="35" t="n">
         <v>49.66883642661386</v>
@@ -5520,10 +5520,10 @@
         <v>41.42499923706055</v>
       </c>
       <c r="W17" s="73" t="n">
-        <v>35140180</v>
+        <v>35197018</v>
       </c>
       <c r="X17" s="74" t="n">
-        <v>0.9974325185291868</v>
+        <v>0.9989652482740143</v>
       </c>
       <c r="Y17" s="28" t="n">
         <v>55.05143031771929</v>
@@ -5729,10 +5729,10 @@
         <v>764.4400024414062</v>
       </c>
       <c r="W19" s="73" t="n">
-        <v>41462196</v>
+        <v>42916599</v>
       </c>
       <c r="X19" s="74" t="n">
-        <v>0.988757737919189</v>
+        <v>1.021669441868448</v>
       </c>
       <c r="Y19" s="28" t="n">
         <v>51.80060080068652</v>
@@ -5917,10 +5917,10 @@
         <v>715.4349975585938</v>
       </c>
       <c r="W20" s="84" t="n">
-        <v>48600043</v>
+        <v>49058351</v>
       </c>
       <c r="X20" s="85" t="n">
-        <v>1.388569596338733</v>
+        <v>1.400746978715844</v>
       </c>
       <c r="Y20" s="35" t="n">
         <v>44.08965566451499</v>
@@ -6021,7 +6021,7 @@
         </is>
       </c>
       <c r="C21" s="26" t="n">
-        <v>0.01356079427348655</v>
+        <v>0.01367133994853043</v>
       </c>
       <c r="D21" s="27" t="n">
         <v>1</v>
@@ -6090,10 +6090,10 @@
         </is>
       </c>
       <c r="R21" s="70" t="n">
-        <v>275.0499877929688</v>
+        <v>275.0799865722656</v>
       </c>
       <c r="S21" s="71" t="n">
-        <v>3.67999267578125</v>
+        <v>3.709991455078125</v>
       </c>
       <c r="T21" s="72" t="n">
         <v>271.4200134277344</v>
@@ -6105,61 +6105,61 @@
         <v>270.8500061035156</v>
       </c>
       <c r="W21" s="73" t="n">
-        <v>31666168</v>
+        <v>31921315</v>
       </c>
       <c r="X21" s="74" t="n">
-        <v>1.219174343601148</v>
+        <v>1.228394370656753</v>
       </c>
       <c r="Y21" s="28" t="n">
-        <v>37.24824783586103</v>
+        <v>37.31282542253678</v>
       </c>
       <c r="Z21" s="28" t="n">
-        <v>32.88998515765982</v>
+        <v>33.09991350866515</v>
       </c>
       <c r="AA21" s="28" t="n">
         <v>40.75090195987555</v>
       </c>
       <c r="AB21" s="75" t="n">
-        <v>-3.837141804246642</v>
+        <v>-3.834748739231543</v>
       </c>
       <c r="AC21" s="75" t="n">
-        <v>-3.649657730119999</v>
+        <v>-3.649179117116979</v>
       </c>
       <c r="AD21" s="75" t="n">
-        <v>-0.187484074126643</v>
+        <v>-0.185569622114564</v>
       </c>
       <c r="AE21" s="72" t="n">
-        <v>276.6451755397707</v>
+        <v>276.65184193517</v>
       </c>
       <c r="AF21" s="72" t="n">
-        <v>280.4321417274671</v>
+        <v>280.4348688892214</v>
       </c>
       <c r="AG21" s="72" t="n">
-        <v>289.6254022216797</v>
+        <v>289.6260021972656</v>
       </c>
       <c r="AH21" s="72" t="n">
-        <v>291.5599014282226</v>
+        <v>291.5602014160156</v>
       </c>
       <c r="AI21" s="72" t="n">
-        <v>277.5382008361817</v>
+        <v>277.5383508300781</v>
       </c>
       <c r="AJ21" s="72" t="n">
-        <v>287.1865729154478</v>
+        <v>287.1839615772174</v>
       </c>
       <c r="AK21" s="72" t="n">
-        <v>279.9925003051758</v>
+        <v>279.9940002441406</v>
       </c>
       <c r="AL21" s="72" t="n">
-        <v>272.7984276949038</v>
+        <v>272.8040389110639</v>
       </c>
       <c r="AM21" s="76" t="n">
-        <v>0.1564871679811848</v>
+        <v>0.1582725939520337</v>
       </c>
       <c r="AN21" s="29" t="n">
-        <v>5.138760932832734</v>
+        <v>5.1357967147921</v>
       </c>
       <c r="AO21" s="77" t="n">
-        <v>1.343155463934949</v>
+        <v>1.343008986450978</v>
       </c>
       <c r="AP21" s="72" t="n">
         <v>305.1799926757812</v>
@@ -6168,22 +6168,22 @@
         <v>228.8999938964844</v>
       </c>
       <c r="AR21" s="29" t="n">
-        <v>-9.872863754480187</v>
+        <v>-9.863033890132311</v>
       </c>
       <c r="AS21" s="78" t="n">
-        <v>60.50077954250037</v>
+        <v>60.54010673151053</v>
       </c>
       <c r="AT21" s="26" t="n">
-        <v>-0.009078861061189714</v>
+        <v>-0.008970784617390648</v>
       </c>
       <c r="AU21" s="26" t="n">
-        <v>-0.03124128351389821</v>
+        <v>-0.03113562425115479</v>
       </c>
       <c r="AV21" s="26" t="n">
-        <v>-0.06458311862364108</v>
+        <v>-0.06448109584298167</v>
       </c>
       <c r="AW21" s="26" t="n">
-        <v>0.1173626247199571</v>
+        <v>0.1174844917123627</v>
       </c>
       <c r="AX21" s="79" t="inlineStr">
         <is>
@@ -6293,10 +6293,10 @@
         <v>95.23000335693359</v>
       </c>
       <c r="W22" s="84" t="n">
-        <v>135527534</v>
+        <v>136485535</v>
       </c>
       <c r="X22" s="85" t="n">
-        <v>2.018368794832909</v>
+        <v>2.0311870331558</v>
       </c>
       <c r="Y22" s="35" t="n">
         <v>34.53322867937399</v>
@@ -6502,10 +6502,10 @@
         <v>341.6000061035156</v>
       </c>
       <c r="W24" s="73" t="n">
-        <v>38900835</v>
+        <v>39605715</v>
       </c>
       <c r="X24" s="74" t="n">
-        <v>1.016186889267074</v>
+        <v>1.033648473853279</v>
       </c>
       <c r="Y24" s="28" t="n">
         <v>60.57988770507023</v>
@@ -6594,7 +6594,7 @@
       </c>
       <c r="AZ24" s="79" t="inlineStr">
         <is>
-          <t>Apple sets preorder date for its ambitious and expensive iPhone Duo</t>
+          <t>iPhone Duo Preorders Begin Friday. Is Apple’s First Foldable Phone Reason Alone to Buy the Stock?</t>
         </is>
       </c>
     </row>
@@ -6690,10 +6690,10 @@
         <v>530.0900268554688</v>
       </c>
       <c r="W25" s="84" t="n">
-        <v>28467521</v>
+        <v>28525288</v>
       </c>
       <c r="X25" s="85" t="n">
-        <v>1.31136537942812</v>
+        <v>1.313851623013426</v>
       </c>
       <c r="Y25" s="35" t="n">
         <v>44.52251866572423</v>
@@ -6772,7 +6772,7 @@
       </c>
       <c r="AX25" s="90" t="inlineStr">
         <is>
-          <t>Nvidia stock falls amid concerns over AI financing</t>
+          <t>Nvidia stock trims losses as chip sell-off eases amid AI financing concerns</t>
         </is>
       </c>
       <c r="AY25" s="90" t="inlineStr">
@@ -6878,10 +6878,10 @@
         <v>248.6499938964844</v>
       </c>
       <c r="W26" s="73" t="n">
-        <v>33990059</v>
+        <v>34045521</v>
       </c>
       <c r="X26" s="74" t="n">
-        <v>0.9345678804212821</v>
+        <v>0.9360214572920091</v>
       </c>
       <c r="Y26" s="28" t="n">
         <v>50.09785874375949</v>
@@ -6960,17 +6960,17 @@
       </c>
       <c r="AX26" s="79" t="inlineStr">
         <is>
-          <t>Amazon’s New Devices Show Push to Avoid Getting Shut Out of Personal AI</t>
+          <t>Elon Musk wants to start an Amazon competitor after Grok bot users say the company blocked them from placin...</t>
         </is>
       </c>
       <c r="AY26" s="79" t="inlineStr">
         <is>
-          <t>Sector Update: Tech Stocks Fall Thursday Afternoon</t>
+          <t>Elon Musk has shopping advice after Amazon blocks his AI</t>
         </is>
       </c>
       <c r="AZ26" s="79" t="inlineStr">
         <is>
-          <t>SpaceX CEO Elon Musk Teases ‘X Shop’ After Amazon Shuts Out Grok Agents</t>
+          <t>Amazon’s Reinvestment Model Is Dave Ellison’s Market Playbook</t>
         </is>
       </c>
     </row>
@@ -7066,10 +7066,10 @@
         <v>81.51000213623047</v>
       </c>
       <c r="W27" s="84" t="n">
-        <v>6800311</v>
+        <v>6802662</v>
       </c>
       <c r="X27" s="85" t="n">
-        <v>1.487383556180408</v>
+        <v>1.48785951948564</v>
       </c>
       <c r="Y27" s="35" t="n">
         <v>45.74132085614958</v>
@@ -7254,10 +7254,10 @@
         <v>226.5399932861328</v>
       </c>
       <c r="W28" s="73" t="n">
-        <v>6505847</v>
+        <v>6550887</v>
       </c>
       <c r="X28" s="74" t="n">
-        <v>1.056894225411485</v>
+        <v>1.063821914601169</v>
       </c>
       <c r="Y28" s="28" t="n">
         <v>38.90577727957994</v>
@@ -7433,7 +7433,7 @@
         <v>2.319999694824219</v>
       </c>
       <c r="T29" s="83" t="n">
-        <v>40.79000091552734</v>
+        <v>40.83000183105469</v>
       </c>
       <c r="U29" s="83" t="n">
         <v>44.93500137329102</v>
@@ -7442,10 +7442,10 @@
         <v>39.86999893188477</v>
       </c>
       <c r="W29" s="84" t="n">
-        <v>22996790</v>
+        <v>23115152</v>
       </c>
       <c r="X29" s="85" t="n">
-        <v>1.372038820157551</v>
+        <v>1.378613785787168</v>
       </c>
       <c r="Y29" s="35" t="n">
         <v>32.32218064297044</v>
@@ -7630,10 +7630,10 @@
         <v>334.6099853515625</v>
       </c>
       <c r="W30" s="73" t="n">
-        <v>25945420</v>
+        <v>28198872</v>
       </c>
       <c r="X30" s="74" t="n">
-        <v>1.132016858379239</v>
+        <v>1.224317821028627</v>
       </c>
       <c r="Y30" s="28" t="n">
         <v>41.36828271555768</v>
@@ -7818,10 +7818,10 @@
         <v>78.55000305175781</v>
       </c>
       <c r="W31" s="84" t="n">
-        <v>5395748</v>
+        <v>5397770</v>
       </c>
       <c r="X31" s="85" t="n">
-        <v>1.502961468184502</v>
+        <v>1.503482347743991</v>
       </c>
       <c r="Y31" s="35" t="n">
         <v>38.08165253913529</v>
@@ -8006,10 +8006,10 @@
         <v>59.5099983215332</v>
       </c>
       <c r="W32" s="73" t="n">
-        <v>128180879</v>
+        <v>128884246</v>
       </c>
       <c r="X32" s="74" t="n">
-        <v>3.376554564195051</v>
+        <v>3.391940411360233</v>
       </c>
       <c r="Y32" s="28" t="n">
         <v>34.91657821894675</v>
@@ -8088,17 +8088,17 @@
       </c>
       <c r="AX32" s="79" t="inlineStr">
         <is>
-          <t>As chip stocks fall, investors are turning elsewhere in the market: Chart of the Day</t>
+          <t>CoreWeave’s Debt Insurance Costs Just Hit a Record. Can It Keep Funding Its AI Boom?</t>
         </is>
       </c>
       <c r="AY32" s="79" t="inlineStr">
         <is>
-          <t>CoreWeave Contract Structure Limits Financing Risk, Capacity Adds Support Growth, BofA Says</t>
+          <t>Deutsche Bank has blunt advice after NVIDIA-linked stock sinks 15%</t>
         </is>
       </c>
       <c r="AZ32" s="79" t="inlineStr">
         <is>
-          <t>CoreWeave’s Freakout Hurt Constellation and NRG Stocks. It Shouldn’t Have.</t>
+          <t>CoreWeave three co-founders sold $3.3 billion in shares since IPO</t>
         </is>
       </c>
     </row>
@@ -8191,22 +8191,22 @@
         <v>482</v>
       </c>
       <c r="V33" s="83" t="n">
-        <v>452.4200439453125</v>
+        <v>452.4201049804688</v>
       </c>
       <c r="W33" s="84" t="n">
-        <v>16123394</v>
+        <v>16314848</v>
       </c>
       <c r="X33" s="85" t="n">
-        <v>2.196006025323908</v>
+        <v>2.219188675560352</v>
       </c>
       <c r="Y33" s="35" t="n">
         <v>36.27106647072114</v>
       </c>
       <c r="Z33" s="35" t="n">
-        <v>14.70133028785034</v>
+        <v>14.70129378882094</v>
       </c>
       <c r="AA33" s="35" t="n">
-        <v>23.36391343914559</v>
+        <v>23.36391208856758</v>
       </c>
       <c r="AB33" s="86" t="n">
         <v>4.680171083725213</v>
@@ -8248,7 +8248,7 @@
         <v>19.02167238060184</v>
       </c>
       <c r="AO33" s="88" t="n">
-        <v>6.85670067652379</v>
+        <v>6.856699755580406</v>
       </c>
       <c r="AP33" s="83" t="n">
         <v>595.510009765625</v>
@@ -8281,12 +8281,12 @@
       </c>
       <c r="AY33" s="90" t="inlineStr">
         <is>
-          <t>Stock Market Today: Nasdaq Higher As Yields Plunge; Dell Triggers Sell Signals (Live Coverage)</t>
+          <t>Dell stock tumbles 8% in a day. Here’s why</t>
         </is>
       </c>
       <c r="AZ33" s="90" t="inlineStr">
         <is>
-          <t>Michael Dell Loses Title of World’s Fourth Richest Person After $36 Billion Drop in Net Worth in Two Days</t>
+          <t>Dell Technologies (DELL) Stock Drops Despite Market Gains: Important Facts to Note</t>
         </is>
       </c>
     </row>
@@ -8382,10 +8382,10 @@
         <v>336.8200073242188</v>
       </c>
       <c r="W34" s="73" t="n">
-        <v>15094771</v>
+        <v>15220969</v>
       </c>
       <c r="X34" s="74" t="n">
-        <v>0.8868216019894786</v>
+        <v>0.893904388605842</v>
       </c>
       <c r="Y34" s="28" t="n">
         <v>51.9391021227524</v>
@@ -8464,17 +8464,17 @@
       </c>
       <c r="AX34" s="79" t="inlineStr">
         <is>
+          <t>Here Are the 3 Magnificent Seven Stocks I'd Buy Today</t>
+        </is>
+      </c>
+      <c r="AY34" s="79" t="inlineStr">
+        <is>
           <t>Google’s $180 Fitbit Edge makes a bet on smartwatch fatigue</t>
         </is>
       </c>
-      <c r="AY34" s="79" t="inlineStr">
+      <c r="AZ34" s="79" t="inlineStr">
         <is>
           <t>Sector Update: Consumer Stocks Rise Late Afternoon</t>
-        </is>
-      </c>
-      <c r="AZ34" s="79" t="inlineStr">
-        <is>
-          <t>Sector Update: Tech Stocks Fall Late Afternoon</t>
         </is>
       </c>
     </row>
@@ -8561,7 +8561,7 @@
         <v>-0.1700000762939453</v>
       </c>
       <c r="T35" s="83" t="n">
-        <v>28.8799991607666</v>
+        <v>28.8700008392334</v>
       </c>
       <c r="U35" s="83" t="n">
         <v>30.45999908447266</v>
@@ -8570,10 +8570,10 @@
         <v>26.60000038146973</v>
       </c>
       <c r="W35" s="84" t="n">
-        <v>105304368</v>
+        <v>105793791</v>
       </c>
       <c r="X35" s="85" t="n">
-        <v>2.364491345224895</v>
+        <v>2.374176245317949</v>
       </c>
       <c r="Y35" s="35" t="n">
         <v>26.35196431182526</v>
@@ -8652,17 +8652,17 @@
       </c>
       <c r="AX35" s="90" t="inlineStr">
         <is>
+          <t>Stock Market Today, Oct. 15: Iren Stock Recovers, but Still Slides on Concerns Over Neocloud Provider Viabi...</t>
+        </is>
+      </c>
+      <c r="AY35" s="90" t="inlineStr">
+        <is>
           <t>AI Cloud Stocks Sink as Gartner Warns Most Neoclouds Won’t Survive Independently: IREN and CoreWeave Fall 5...</t>
         </is>
       </c>
-      <c r="AY35" s="90" t="inlineStr">
+      <c r="AZ35" s="90" t="inlineStr">
         <is>
           <t>IREN Expands Liquid Cooling Across AI Data Centers: Can Returns Rise?</t>
-        </is>
-      </c>
-      <c r="AZ35" s="90" t="inlineStr">
-        <is>
-          <t>AI Stocks Selloff and CoreWeave Debt, IREN Proposes 900 MW Aussie Site, Keel’s New 80 MW Site</t>
         </is>
       </c>
     </row>
@@ -8749,7 +8749,7 @@
         <v>-2.75</v>
       </c>
       <c r="T36" s="72" t="n">
-        <v>93.61000061035156</v>
+        <v>93.55999755859375</v>
       </c>
       <c r="U36" s="72" t="n">
         <v>96.87000274658203</v>
@@ -8758,10 +8758,10 @@
         <v>90.01999664306641</v>
       </c>
       <c r="W36" s="73" t="n">
-        <v>145656686</v>
+        <v>146124769</v>
       </c>
       <c r="X36" s="74" t="n">
-        <v>1.357002889029483</v>
+        <v>1.361066987930089</v>
       </c>
       <c r="Y36" s="28" t="n">
         <v>35.56926485156553</v>
@@ -8840,7 +8840,7 @@
       </c>
       <c r="AX36" s="79" t="inlineStr">
         <is>
-          <t>Nvidia stock falls amid concerns over AI financing</t>
+          <t>Nvidia stock trims losses as chip sell-off eases amid AI financing concerns</t>
         </is>
       </c>
       <c r="AY36" s="79" t="inlineStr">
@@ -8874,7 +8874,7 @@
       </c>
       <c r="F37" s="30" t="inlineStr">
         <is>
-          <t>Same</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G37" s="30" t="inlineStr">
@@ -8937,7 +8937,7 @@
         <v>5.75</v>
       </c>
       <c r="T37" s="83" t="n">
-        <v>533.3150024414062</v>
+        <v>533.655029296875</v>
       </c>
       <c r="U37" s="83" t="n">
         <v>541.1331176757812</v>
@@ -8946,10 +8946,10 @@
         <v>531.219970703125</v>
       </c>
       <c r="W37" s="84" t="n">
-        <v>22475489</v>
+        <v>23481292</v>
       </c>
       <c r="X37" s="85" t="n">
-        <v>0.9783096195696964</v>
+        <v>1.019857566919823</v>
       </c>
       <c r="Y37" s="35" t="n">
         <v>65.04389805101135</v>
@@ -9028,17 +9028,17 @@
       </c>
       <c r="AX37" s="90" t="inlineStr">
         <is>
+          <t>3 Chip Stocks to Buy Before Big Tech Reports Its Spending Plans</t>
+        </is>
+      </c>
+      <c r="AY37" s="90" t="inlineStr">
+        <is>
           <t>These 2 Stocks Have Run Circles Around the Magnificent Seven This Year, and Wall Street Says There Is More ...</t>
         </is>
       </c>
-      <c r="AY37" s="90" t="inlineStr">
+      <c r="AZ37" s="90" t="inlineStr">
         <is>
           <t>Tucuvi joins the Microsoft Pegasus Program to scale clinically governed AI Care Management across health sy...</t>
-        </is>
-      </c>
-      <c r="AZ37" s="90" t="inlineStr">
-        <is>
-          <t>Microsoft can justify higher valuation as AI demand drives Azure growth, UBS says</t>
         </is>
       </c>
     </row>
@@ -9062,7 +9062,7 @@
       </c>
       <c r="F38" s="23" t="inlineStr">
         <is>
-          <t>Same</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G38" s="23" t="inlineStr">
@@ -9125,7 +9125,7 @@
         <v>8.04998779296875</v>
       </c>
       <c r="T38" s="72" t="n">
-        <v>137.7400054931641</v>
+        <v>137.7225036621094</v>
       </c>
       <c r="U38" s="72" t="n">
         <v>151.3300018310547</v>
@@ -9134,10 +9134,10 @@
         <v>134.8919982910156</v>
       </c>
       <c r="W38" s="73" t="n">
-        <v>20997477</v>
+        <v>21711948</v>
       </c>
       <c r="X38" s="74" t="n">
-        <v>0.9571329831949622</v>
+        <v>0.9880918806049387</v>
       </c>
       <c r="Y38" s="28" t="n">
         <v>52.4466077005222</v>
@@ -9216,17 +9216,17 @@
       </c>
       <c r="AX38" s="79" t="inlineStr">
         <is>
+          <t>Strategy CEO sees a historic Bitcoin banking boom coming. Here's what's driving it</t>
+        </is>
+      </c>
+      <c r="AY38" s="79" t="inlineStr">
+        <is>
           <t>Barclays Analyst Resets Strategy Stock Price Target. How to Play MSTR Here.</t>
         </is>
       </c>
-      <c r="AY38" s="79" t="inlineStr">
+      <c r="AZ38" s="79" t="inlineStr">
         <is>
           <t>Strategy’s Michael Saylor Says Bitcoin Bull Market Is Just Beginning</t>
-        </is>
-      </c>
-      <c r="AZ38" s="79" t="inlineStr">
-        <is>
-          <t>Is Trending Stock Strategy Inc (MSTR) a Buy Now?</t>
         </is>
       </c>
     </row>
@@ -9313,7 +9313,7 @@
         <v>17.1099853515625</v>
       </c>
       <c r="T39" s="83" t="n">
-        <v>871.5750122070312</v>
+        <v>871.5800170898438</v>
       </c>
       <c r="U39" s="83" t="n">
         <v>931.6500244140625</v>
@@ -9322,10 +9322,10 @@
         <v>858</v>
       </c>
       <c r="W39" s="84" t="n">
-        <v>38220845</v>
+        <v>38345136</v>
       </c>
       <c r="X39" s="85" t="n">
-        <v>1.405456774890544</v>
+        <v>1.409705055308292</v>
       </c>
       <c r="Y39" s="35" t="n">
         <v>39.16498851354567</v>
@@ -9404,17 +9404,17 @@
       </c>
       <c r="AX39" s="90" t="inlineStr">
         <is>
+          <t>Cathie Wood Says the Memory Chip Trend Is Up but the Cycles Are ‘Vicious’</t>
+        </is>
+      </c>
+      <c r="AY39" s="90" t="inlineStr">
+        <is>
+          <t>Prediction: This Is What $2,000 Invested in Micron Stock Today Could Be Worth by 2029</t>
+        </is>
+      </c>
+      <c r="AZ39" s="90" t="inlineStr">
+        <is>
           <t>I Just Bought Micron Stock. Here's Why</t>
-        </is>
-      </c>
-      <c r="AY39" s="90" t="inlineStr">
-        <is>
-          <t>DRAM Giants Get Rich as China Builds a Threat</t>
-        </is>
-      </c>
-      <c r="AZ39" s="90" t="inlineStr">
-        <is>
-          <t>Micron &amp; SanDisk Stocks Look Oversold: Time to Buy the Dip?</t>
         </is>
       </c>
     </row>
@@ -9510,10 +9510,10 @@
         <v>163.3600006103516</v>
       </c>
       <c r="W40" s="73" t="n">
-        <v>46845985</v>
+        <v>47084844</v>
       </c>
       <c r="X40" s="74" t="n">
-        <v>2.570375865465477</v>
+        <v>2.581789905682902</v>
       </c>
       <c r="Y40" s="28" t="n">
         <v>36.50386194892396</v>
@@ -9592,17 +9592,17 @@
       </c>
       <c r="AX40" s="79" t="inlineStr">
         <is>
+          <t>‘Huge’ AI correction ahead: Where to move your money now</t>
+        </is>
+      </c>
+      <c r="AY40" s="79" t="inlineStr">
+        <is>
           <t>Nebius stock breaks below $200 as CoreWeave’s debt scare spreads</t>
         </is>
       </c>
-      <c r="AY40" s="79" t="inlineStr">
-        <is>
-          <t>AI Cloud Stocks Sink as Gartner Warns Most Neoclouds Won’t Survive Independently: IREN and CoreWeave Fall 5...</t>
-        </is>
-      </c>
       <c r="AZ40" s="79" t="inlineStr">
         <is>
-          <t>IonQ vs. Nebius Group: Which Technology Stock Is a Better Buy in 2026?</t>
+          <t>Nebius Stock Just Scored a New Bullish Rating. What to Know.</t>
         </is>
       </c>
     </row>
@@ -9665,7 +9665,7 @@
         </is>
       </c>
       <c r="N41" s="80" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O41" s="30" t="inlineStr">
         <is>
@@ -9689,7 +9689,7 @@
         <v>2.040000915527344</v>
       </c>
       <c r="T41" s="83" t="n">
-        <v>71.55000305175781</v>
+        <v>71.5</v>
       </c>
       <c r="U41" s="83" t="n">
         <v>73.06999969482422</v>
@@ -9698,10 +9698,10 @@
         <v>71.33499908447266</v>
       </c>
       <c r="W41" s="84" t="n">
-        <v>40000311</v>
+        <v>40068614</v>
       </c>
       <c r="X41" s="85" t="n">
-        <v>1.033465962974657</v>
+        <v>1.035139334018433</v>
       </c>
       <c r="Y41" s="35" t="n">
         <v>51.97743826050299</v>
@@ -9790,7 +9790,7 @@
       </c>
       <c r="AZ41" s="90" t="inlineStr">
         <is>
-          <t>This Warning Signal Just Flashed Ahead of Netflix's Earnings -- Here's What It Means for the Stock</t>
+          <t>Why Netflix (NFLX) Outpaced the Stock Market Today</t>
         </is>
       </c>
     </row>
@@ -9814,7 +9814,7 @@
       </c>
       <c r="F42" s="23" t="inlineStr">
         <is>
-          <t>Same</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G42" s="23" t="inlineStr">
@@ -9886,10 +9886,10 @@
         <v>9.039999961853027</v>
       </c>
       <c r="W42" s="73" t="n">
-        <v>87259786</v>
+        <v>89092324</v>
       </c>
       <c r="X42" s="74" t="n">
-        <v>1.15332273418418</v>
+        <v>1.176119270469382</v>
       </c>
       <c r="Y42" s="28" t="n">
         <v>41.88770802710326</v>
@@ -10065,7 +10065,7 @@
         <v>-4.07000732421875</v>
       </c>
       <c r="T43" s="83" t="n">
-        <v>215.3000030517578</v>
+        <v>215.3399963378906</v>
       </c>
       <c r="U43" s="83" t="n">
         <v>218.4691925048828</v>
@@ -10074,10 +10074,10 @@
         <v>212.8500061035156</v>
       </c>
       <c r="W43" s="84" t="n">
-        <v>125363860</v>
+        <v>126396690</v>
       </c>
       <c r="X43" s="85" t="n">
-        <v>1.158124772517385</v>
+        <v>1.167109374202511</v>
       </c>
       <c r="Y43" s="35" t="n">
         <v>40.17280841550092</v>
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
-          <t>Chip stocks tumble; Are investors just repositioning?</t>
+          <t>IonQ Is Following Nvidia's Playbook. Why the Stock Could Be a Buy After a 60% Dip.</t>
         </is>
       </c>
       <c r="AY43" s="90" t="inlineStr">
         <is>
-          <t>These 2 Stocks Have Run Circles Around the Magnificent Seven This Year, and Wall Street Says There Is More ...</t>
+          <t>VGT Returned 799.70% and VOO Returned 324.46% Over a Decade. Adding VUG Does Not Make It Diversified</t>
         </is>
       </c>
       <c r="AZ43" s="90" t="inlineStr">
         <is>
-          <t>Anthropic Wants a $2T IPO on Cooling Growth</t>
+          <t>Here Are the 3 Magnificent Seven Stocks I'd Buy Today</t>
         </is>
       </c>
     </row>
@@ -10262,10 +10262,10 @@
         <v>192.6000061035156</v>
       </c>
       <c r="W44" s="73" t="n">
-        <v>24647119</v>
+        <v>24679424</v>
       </c>
       <c r="X44" s="74" t="n">
-        <v>1.052820971733687</v>
+        <v>1.054128173752671</v>
       </c>
       <c r="Y44" s="28" t="n">
         <v>62.58014496903483</v>
@@ -10344,17 +10344,17 @@
       </c>
       <c r="AX44" s="79" t="inlineStr">
         <is>
+          <t>Palantir Technologies (PLTR) Takes AI Onboarding Into Commercial Banking</t>
+        </is>
+      </c>
+      <c r="AY44" s="79" t="inlineStr">
+        <is>
           <t>ServiceNow vs. Palantir Technologies: Which Technology Stock Is a Better Buy in 2026?</t>
         </is>
       </c>
-      <c r="AY44" s="79" t="inlineStr">
+      <c r="AZ44" s="79" t="inlineStr">
         <is>
           <t>Figma vs. Palantir Technologies: Which Technology Stock Is a Better Buy in 2026?</t>
-        </is>
-      </c>
-      <c r="AZ44" s="79" t="inlineStr">
-        <is>
-          <t>Surf Air Mobility Expands Palantir-Powered AI Push With Fifth Aviation Software Deal</t>
         </is>
       </c>
     </row>
@@ -10450,10 +10450,10 @@
         <v>168.8399963378906</v>
       </c>
       <c r="W45" s="84" t="n">
-        <v>11726527</v>
+        <v>11764179</v>
       </c>
       <c r="X45" s="85" t="n">
-        <v>0.8884054723696477</v>
+        <v>0.8911309012705426</v>
       </c>
       <c r="Y45" s="35" t="n">
         <v>48.85834543989981</v>
@@ -10532,17 +10532,17 @@
       </c>
       <c r="AX45" s="90" t="inlineStr">
         <is>
+          <t>Qualcomm (QCOM) Unveils First AI Native Wi Fi 8 Gateway For Home Broadband</t>
+        </is>
+      </c>
+      <c r="AY45" s="90" t="inlineStr">
+        <is>
           <t>A 20% Drop in Smartphone Shipments Shows Who Wins When Memory Gets Expensive</t>
         </is>
       </c>
-      <c r="AY45" s="90" t="inlineStr">
+      <c r="AZ45" s="90" t="inlineStr">
         <is>
           <t>Intel vs. Qualcomm: Which Tech Stock Is a Better Buy in 2026?</t>
-        </is>
-      </c>
-      <c r="AZ45" s="90" t="inlineStr">
-        <is>
-          <t>QCOM, AVGO, NVDA Stocks In Focus As ByteDance Reportedly Closes In On A MediaTek Pact For AI Data Center Chips</t>
         </is>
       </c>
     </row>
@@ -10638,10 +10638,10 @@
         <v>49.69300079345703</v>
       </c>
       <c r="W46" s="73" t="n">
-        <v>47806392</v>
+        <v>48106607</v>
       </c>
       <c r="X46" s="74" t="n">
-        <v>2.083400842329233</v>
+        <v>2.095113645034586</v>
       </c>
       <c r="Y46" s="28" t="n">
         <v>29.1676807038621</v>
@@ -10730,7 +10730,7 @@
       </c>
       <c r="AZ46" s="79" t="inlineStr">
         <is>
-          <t>Why Rocket Lab Stock Plummeted as Much as 16% Today</t>
+          <t>Stock Market Today, Oct. 15: Rocket Lab Pushes Neutron Launch to 2027, Stock Falls 7%</t>
         </is>
       </c>
     </row>
@@ -10826,10 +10826,10 @@
         <v>1276.069946289062</v>
       </c>
       <c r="W47" s="84" t="n">
-        <v>13076757</v>
+        <v>13129814</v>
       </c>
       <c r="X47" s="85" t="n">
-        <v>1.49062318525694</v>
+        <v>1.496218712304483</v>
       </c>
       <c r="Y47" s="35" t="n">
         <v>33.94073657914728</v>
@@ -10908,7 +10908,7 @@
       </c>
       <c r="AX47" s="90" t="inlineStr">
         <is>
-          <t>Nvidia stock falls amid concerns over AI financing</t>
+          <t>Nvidia stock trims losses as chip sell-off eases amid AI financing concerns</t>
         </is>
       </c>
       <c r="AY47" s="90" t="inlineStr">
@@ -11014,10 +11014,10 @@
         <v>355.2300109863281</v>
       </c>
       <c r="W48" s="73" t="n">
-        <v>26422485</v>
+        <v>26484292</v>
       </c>
       <c r="X48" s="74" t="n">
-        <v>0.7782733583741278</v>
+        <v>0.7800228788873266</v>
       </c>
       <c r="Y48" s="28" t="n">
         <v>46.45144845315087</v>
@@ -11106,7 +11106,7 @@
       </c>
       <c r="AZ48" s="79" t="inlineStr">
         <is>
-          <t>Will SpaceX merge with Tesla? Speculation resurfaces it could happen before the end of 2026.</t>
+          <t>Dow Jones Futures: Disney, Salesforce Lead 12 Buys After Wild Session; Tesla Roadster On Tap</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 15 Oct 2026, 08:27 PM · Yahoo Finance data</t>
+          <t>Built 15 Oct 2026, 11:05 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 15 Oct 2026, 08:27 PM · Yahoo Finance data</t>
+          <t>Built 15 Oct 2026, 11:05 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 15 Oct 2026, 08:27 PM · Yahoo Finance data</t>
+          <t>Built 15 Oct 2026, 11:05 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 15 Oct 2026, 08:27 PM · Yahoo Finance data</t>
+          <t>Built 15 Oct 2026, 11:05 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -43715,7 +43715,7 @@
         <v>0.009129085189356179</v>
       </c>
       <c r="J15" s="34" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K15" s="102" t="inlineStr">
         <is>
@@ -43968,7 +43968,7 @@
       </c>
       <c r="D7" s="105" t="inlineStr">
         <is>
-          <t>Volume 2.0x its 20-day average</t>
+          <t>Volume 2.1x its 20-day average</t>
         </is>
       </c>
       <c r="E7" s="33" t="n">
@@ -44042,12 +44042,12 @@
     <row r="10">
       <c r="B10" s="24" t="inlineStr">
         <is>
-          <t>XLB</t>
+          <t>XLF</t>
         </is>
       </c>
       <c r="C10" s="101" t="inlineStr">
         <is>
-          <t>State Street Materials Select Sector SPDR ETF</t>
+          <t>State Street Financial Select Sector SPDR ETF</t>
         </is>
       </c>
       <c r="D10" s="106" t="inlineStr">
@@ -44056,35 +44056,35 @@
         </is>
       </c>
       <c r="E10" s="26" t="n">
-        <v>0.01791832569267449</v>
+        <v>0.01375641954700679</v>
       </c>
       <c r="F10" s="27" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G10" s="23" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Very Strong</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="31" t="inlineStr">
         <is>
-          <t>XLC</t>
+          <t>NFLX</t>
         </is>
       </c>
       <c r="C11" s="102" t="inlineStr">
         <is>
-          <t>State Street Communication Services Select Sector SPDR ETF</t>
-        </is>
-      </c>
-      <c r="D11" s="107" t="inlineStr">
-        <is>
-          <t>MACD crossed up</t>
+          <t>Netflix, Inc.</t>
+        </is>
+      </c>
+      <c r="D11" s="105" t="inlineStr">
+        <is>
+          <t>RSI crossed back above 50</t>
         </is>
       </c>
       <c r="E11" s="33" t="n">
-        <v>0.01461832477028691</v>
+        <v>0.02890748086083605</v>
       </c>
       <c r="F11" s="34" t="n">
         <v>7</v>
@@ -44098,21 +44098,21 @@
     <row r="12">
       <c r="B12" s="24" t="inlineStr">
         <is>
-          <t>XLC</t>
+          <t>NFLX</t>
         </is>
       </c>
       <c r="C12" s="101" t="inlineStr">
         <is>
-          <t>State Street Communication Services Select Sector SPDR ETF</t>
+          <t>Netflix, Inc.</t>
         </is>
       </c>
       <c r="D12" s="106" t="inlineStr">
         <is>
-          <t>RSI crossed back above 50</t>
+          <t>Bands squeezing — a big move often follows</t>
         </is>
       </c>
       <c r="E12" s="26" t="n">
-        <v>0.01461832477028691</v>
+        <v>0.02890748086083605</v>
       </c>
       <c r="F12" s="27" t="n">
         <v>7</v>
@@ -44126,21 +44126,21 @@
     <row r="13">
       <c r="B13" s="31" t="inlineStr">
         <is>
-          <t>XLC</t>
+          <t>XLB</t>
         </is>
       </c>
       <c r="C13" s="102" t="inlineStr">
         <is>
-          <t>State Street Communication Services Select Sector SPDR ETF</t>
+          <t>State Street Materials Select Sector SPDR ETF</t>
         </is>
       </c>
       <c r="D13" s="105" t="inlineStr">
         <is>
-          <t>Reclaimed the 50 DMA</t>
+          <t>RSI crossed back above 50</t>
         </is>
       </c>
       <c r="E13" s="33" t="n">
-        <v>0.01461832477028691</v>
+        <v>0.01791832569267449</v>
       </c>
       <c r="F13" s="34" t="n">
         <v>7</v>
@@ -44154,21 +44154,21 @@
     <row r="14">
       <c r="B14" s="24" t="inlineStr">
         <is>
-          <t>XLF</t>
+          <t>XLC</t>
         </is>
       </c>
       <c r="C14" s="101" t="inlineStr">
         <is>
-          <t>State Street Financial Select Sector SPDR ETF</t>
-        </is>
-      </c>
-      <c r="D14" s="106" t="inlineStr">
-        <is>
-          <t>RSI crossed back above 50</t>
+          <t>State Street Communication Services Select Sector SPDR ETF</t>
+        </is>
+      </c>
+      <c r="D14" s="104" t="inlineStr">
+        <is>
+          <t>MACD crossed up</t>
         </is>
       </c>
       <c r="E14" s="26" t="n">
-        <v>0.01375641954700679</v>
+        <v>0.01461832477028691</v>
       </c>
       <c r="F14" s="27" t="n">
         <v>7</v>
@@ -44182,21 +44182,21 @@
     <row r="15">
       <c r="B15" s="31" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>XLC</t>
         </is>
       </c>
       <c r="C15" s="102" t="inlineStr">
         <is>
-          <t>Alphabet Inc.</t>
+          <t>State Street Communication Services Select Sector SPDR ETF</t>
         </is>
       </c>
       <c r="D15" s="105" t="inlineStr">
         <is>
-          <t>Bands squeezing — a big move often follows</t>
+          <t>RSI crossed back above 50</t>
         </is>
       </c>
       <c r="E15" s="33" t="n">
-        <v>0.003666549652273643</v>
+        <v>0.01461832477028691</v>
       </c>
       <c r="F15" s="34" t="n">
         <v>7</v>
@@ -44210,21 +44210,21 @@
     <row r="16">
       <c r="B16" s="24" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>XLC</t>
         </is>
       </c>
       <c r="C16" s="101" t="inlineStr">
         <is>
-          <t>Palantir Technologies Inc.</t>
+          <t>State Street Communication Services Select Sector SPDR ETF</t>
         </is>
       </c>
       <c r="D16" s="106" t="inlineStr">
         <is>
-          <t>Gapped down 2.2% at the open</t>
+          <t>Reclaimed the 50 DMA</t>
         </is>
       </c>
       <c r="E16" s="26" t="n">
-        <v>-0.002338663570922606</v>
+        <v>0.01461832477028691</v>
       </c>
       <c r="F16" s="27" t="n">
         <v>7</v>
@@ -44238,12 +44238,12 @@
     <row r="17">
       <c r="B17" s="31" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="C17" s="102" t="inlineStr">
         <is>
-          <t>Apple Inc.</t>
+          <t>Alphabet Inc.</t>
         </is>
       </c>
       <c r="D17" s="105" t="inlineStr">
@@ -44252,7 +44252,7 @@
         </is>
       </c>
       <c r="E17" s="33" t="n">
-        <v>-0.00279913540645127</v>
+        <v>0.003666549652273643</v>
       </c>
       <c r="F17" s="34" t="n">
         <v>7</v>
@@ -44266,24 +44266,24 @@
     <row r="18">
       <c r="B18" s="24" t="inlineStr">
         <is>
-          <t>MSTR</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="C18" s="101" t="inlineStr">
         <is>
-          <t>Strategy Inc</t>
+          <t>Palantir Technologies Inc.</t>
         </is>
       </c>
       <c r="D18" s="106" t="inlineStr">
         <is>
-          <t>RSI crossed back above 50</t>
+          <t>Gapped down 2.2% at the open</t>
         </is>
       </c>
       <c r="E18" s="26" t="n">
-        <v>0.05619929827043268</v>
+        <v>-0.002338663570922606</v>
       </c>
       <c r="F18" s="27" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G18" s="23" t="inlineStr">
         <is>
@@ -44294,24 +44294,24 @@
     <row r="19">
       <c r="B19" s="31" t="inlineStr">
         <is>
-          <t>MSTR</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="C19" s="102" t="inlineStr">
         <is>
-          <t>Strategy Inc</t>
+          <t>Apple Inc.</t>
         </is>
       </c>
       <c r="D19" s="105" t="inlineStr">
         <is>
-          <t>Gapped down 3.8% at the open</t>
+          <t>Bands squeezing — a big move often follows</t>
         </is>
       </c>
       <c r="E19" s="33" t="n">
-        <v>0.05619929827043268</v>
+        <v>-0.00279913540645127</v>
       </c>
       <c r="F19" s="34" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G19" s="30" t="inlineStr">
         <is>
@@ -44322,12 +44322,12 @@
     <row r="20">
       <c r="B20" s="24" t="inlineStr">
         <is>
-          <t>NFLX</t>
+          <t>MSTR</t>
         </is>
       </c>
       <c r="C20" s="101" t="inlineStr">
         <is>
-          <t>Netflix, Inc.</t>
+          <t>Strategy Inc</t>
         </is>
       </c>
       <c r="D20" s="106" t="inlineStr">
@@ -44336,7 +44336,7 @@
         </is>
       </c>
       <c r="E20" s="26" t="n">
-        <v>0.02890748086083605</v>
+        <v>0.05619929827043268</v>
       </c>
       <c r="F20" s="27" t="n">
         <v>6</v>
@@ -44350,21 +44350,21 @@
     <row r="21">
       <c r="B21" s="31" t="inlineStr">
         <is>
-          <t>NFLX</t>
+          <t>MSTR</t>
         </is>
       </c>
       <c r="C21" s="102" t="inlineStr">
         <is>
-          <t>Netflix, Inc.</t>
+          <t>Strategy Inc</t>
         </is>
       </c>
       <c r="D21" s="105" t="inlineStr">
         <is>
-          <t>Bands squeezing — a big move often follows</t>
+          <t>Gapped down 3.9% at the open</t>
         </is>
       </c>
       <c r="E21" s="33" t="n">
-        <v>0.02890748086083605</v>
+        <v>0.05619929827043268</v>
       </c>
       <c r="F21" s="34" t="n">
         <v>6</v>
@@ -45368,7 +45368,7 @@
       </c>
       <c r="D57" s="105" t="inlineStr">
         <is>
-          <t>Gapped down 3.2% at the open</t>
+          <t>Gapped down 3.1% at the open</t>
         </is>
       </c>
       <c r="E57" s="33" t="n">

</xml_diff>

<commit_message>
Daily workbook: 2026-10-16 23:33 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 16 Oct 2026, 10:53 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 16 Oct 2026, 11:33 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 16 Oct 2026, 10:53 PM · Yahoo Finance data</t>
+          <t>Built 16 Oct 2026, 11:33 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -6772,7 +6772,7 @@
       </c>
       <c r="AX25" s="90" t="inlineStr">
         <is>
-          <t>Tesla pops, tech heads for losing week: AlphaCheck</t>
+          <t>How much AMD stock does CEO Lisa Su actually own?</t>
         </is>
       </c>
       <c r="AY25" s="90" t="inlineStr">
@@ -8469,12 +8469,12 @@
       </c>
       <c r="AY34" s="79" t="inlineStr">
         <is>
+          <t>Prediction: Alphabet Will Be a Larger Company Than Apple by the End of 2027</t>
+        </is>
+      </c>
+      <c r="AZ34" s="79" t="inlineStr">
+        <is>
           <t>Not Alphabet. Not Microsoft. This Is the Cloud Stock I'd Buy With $5,000 Right Now.</t>
-        </is>
-      </c>
-      <c r="AZ34" s="79" t="inlineStr">
-        <is>
-          <t>Google Partner Novacore Labs and AIBotics Complete Acquisition of Assets, Expanding AI, Drone, Mapping and ...</t>
         </is>
       </c>
     </row>
@@ -9978,7 +9978,7 @@
       </c>
       <c r="AZ42" s="79" t="inlineStr">
         <is>
-          <t>Nokia Corporation - Managers' transactions (Heard)</t>
+          <t>Nokia Corporation - Managers' transactions (Mahajan)</t>
         </is>
       </c>
     </row>
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
+          <t>1 Obvious Metric That Makes Nvidia a Top Stock to Buy Now</t>
+        </is>
+      </c>
+      <c r="AY43" s="90" t="inlineStr">
+        <is>
           <t>Prediction: $1,000 Invested in Taiwan Semi (TSMC) Today Will Be Worth This Much by 2030.</t>
         </is>
       </c>
-      <c r="AY43" s="90" t="inlineStr">
+      <c r="AZ43" s="90" t="inlineStr">
         <is>
           <t>Inflation Rose to 3.7% in September. Is It Time to Sell the S&amp;P 500?</t>
-        </is>
-      </c>
-      <c r="AZ43" s="90" t="inlineStr">
-        <is>
-          <t>Ladder Capital Corp Q3 2026 Earnings Call Summary</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 16 Oct 2026, 10:53 PM · Yahoo Finance data</t>
+          <t>Built 16 Oct 2026, 11:33 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 16 Oct 2026, 10:53 PM · Yahoo Finance data</t>
+          <t>Built 16 Oct 2026, 11:33 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 16 Oct 2026, 10:53 PM · Yahoo Finance data</t>
+          <t>Built 16 Oct 2026, 11:33 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 16 Oct 2026, 10:53 PM · Yahoo Finance data</t>
+          <t>Built 16 Oct 2026, 11:33 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-10-19 23:45 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 19 Oct 2026, 09:39 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 19 Oct 2026, 11:45 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 19 Oct 2026, 09:39 PM · Yahoo Finance data</t>
+          <t>Built 19 Oct 2026, 11:45 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -5821,7 +5821,7 @@
       </c>
       <c r="AZ19" s="79" t="inlineStr">
         <is>
-          <t>Trump Media Drops 7% While Rumble Climbs 3% Amid a Rising Market</t>
+          <t>Nasdaq 100 Sees Best Day In Nearly A Month As AI Rout Cools — AMZN, BE, CRWV, AAPL, PLTR In Focus</t>
         </is>
       </c>
     </row>
@@ -6584,7 +6584,7 @@
       </c>
       <c r="AX24" s="79" t="inlineStr">
         <is>
-          <t>Apple stock is at a record high — but is it warranted given slowing iPhone 18 demand?</t>
+          <t>Jim Cramer’s 4-word Apple rule could save you real money</t>
         </is>
       </c>
       <c r="AY24" s="79" t="inlineStr">
@@ -6772,17 +6772,17 @@
       </c>
       <c r="AX25" s="90" t="inlineStr">
         <is>
-          <t>Intel leads chip stocks higher as investors jump back into AI trade</t>
+          <t>Dow Jones Futures: AMD, Nvidia Lead AI Trade Higher; Meta, Netflix, SpaceX, Tesla Earnings On Deck</t>
         </is>
       </c>
       <c r="AY25" s="90" t="inlineStr">
         <is>
-          <t>Chip Stocks Catch A Break After Prolonged Slide. AI Names Among Leaders.</t>
+          <t>Will AI Rack Expansion Change AMD Stock Narrative</t>
         </is>
       </c>
       <c r="AZ25" s="90" t="inlineStr">
         <is>
-          <t>Here's What a $5,000 Investment in AMD Could Be Worth by 2032</t>
+          <t>AMD (AMD) Stock Trades Up, Here Is Why</t>
         </is>
       </c>
     </row>
@@ -6965,12 +6965,12 @@
       </c>
       <c r="AY26" s="79" t="inlineStr">
         <is>
-          <t>Stock Market Today, Oct. 19: Amazon Surges on Morgan Stanley Top Pick and $350 Price Target</t>
+          <t>3M Jumps On Expanded Amazon Data Center Deal; Earnings On Tap</t>
         </is>
       </c>
       <c r="AZ26" s="79" t="inlineStr">
         <is>
-          <t>Why Amazon (AMZN) Stock Is Up Today</t>
+          <t>Amazon vs. Home Depot: Which Consumer Stock Is a Better Buy in 2026?</t>
         </is>
       </c>
     </row>
@@ -8276,17 +8276,17 @@
       </c>
       <c r="AX33" s="90" t="inlineStr">
         <is>
+          <t>The AI Trade Is Working Again</t>
+        </is>
+      </c>
+      <c r="AY33" s="90" t="inlineStr">
+        <is>
           <t>Efosa Obano Walked Away From His Career At Dell Technologies To Support Black Canadian Founders</t>
         </is>
       </c>
-      <c r="AY33" s="90" t="inlineStr">
+      <c r="AZ33" s="90" t="inlineStr">
         <is>
           <t>Why 1 Analyst Is Cooling Their Stance on Red-Hot DELL Stock</t>
-        </is>
-      </c>
-      <c r="AZ33" s="90" t="inlineStr">
-        <is>
-          <t>Why Dell Technologies Stock Took a Dive Last Week</t>
         </is>
       </c>
     </row>
@@ -8464,17 +8464,17 @@
       </c>
       <c r="AX34" s="79" t="inlineStr">
         <is>
+          <t>Alphabet Stock Slipped After Q2 Earnings. Here's What Investors Need to See in Q3.</t>
+        </is>
+      </c>
+      <c r="AY34" s="79" t="inlineStr">
+        <is>
           <t>Update: Tech-Heavy Nasdaq Leads Wall Street's Relief Rally Ahead of Key Earnings</t>
         </is>
       </c>
-      <c r="AY34" s="79" t="inlineStr">
+      <c r="AZ34" s="79" t="inlineStr">
         <is>
           <t>Alphabet (GOOGL) Pushes Into Carbon Removal Power Markets And Quantum AI</t>
-        </is>
-      </c>
-      <c r="AZ34" s="79" t="inlineStr">
-        <is>
-          <t>A $1.5 Trillion Anthropic IPO Still Pays Off for Google: “They’re Gonna Be Fine”</t>
         </is>
       </c>
     </row>
@@ -8652,17 +8652,17 @@
       </c>
       <c r="AX35" s="90" t="inlineStr">
         <is>
+          <t>Stock Market Today, Oct. 19: IREN Rallies on AI Infrastructure Sentiment Rebound</t>
+        </is>
+      </c>
+      <c r="AY35" s="90" t="inlineStr">
+        <is>
           <t>Applied Digital Soars 10%, IREN Up 5%, CoreWeave Up 2% as AI Infrastructure Selloff Reverses</t>
         </is>
       </c>
-      <c r="AY35" s="90" t="inlineStr">
+      <c r="AZ35" s="90" t="inlineStr">
         <is>
           <t>Nebius, IREN rally as dip buyers return to AI infrastructure stocks</t>
-        </is>
-      </c>
-      <c r="AZ35" s="90" t="inlineStr">
-        <is>
-          <t>AI Infrastructure Stocks Rally as Selloff Reverses: Applied Digital Jumps 8%, TeraWulf and IREN Rise 6%</t>
         </is>
       </c>
     </row>
@@ -8840,17 +8840,17 @@
       </c>
       <c r="AX36" s="79" t="inlineStr">
         <is>
+          <t>Did Foundry Win Just Shift Intel (INTC) Investment Narrative?</t>
+        </is>
+      </c>
+      <c r="AY36" s="79" t="inlineStr">
+        <is>
+          <t>Applied Materials, Lam Research, Marvell Technology, Micron, and Semtech Shares Skyrocket, What You Need To...</t>
+        </is>
+      </c>
+      <c r="AZ36" s="79" t="inlineStr">
+        <is>
           <t>FormFactor, Teradyne, Entegris, Kulicke and Soffa, and Seagate Shares Skyrocket, What You Need To Know</t>
-        </is>
-      </c>
-      <c r="AY36" s="79" t="inlineStr">
-        <is>
-          <t>Why Intel (INTC) Stock Is Up Today</t>
-        </is>
-      </c>
-      <c r="AZ36" s="79" t="inlineStr">
-        <is>
-          <t>Tesla Rises on a Foundry Agreement With Intel as JPMorgan Upgrades the Stock</t>
         </is>
       </c>
     </row>
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
-          <t>2 Stocks Down About 70% to Buy Now and Hold for the Next Decade</t>
+          <t>Thinking Nvidia Stock Could Hit $10 Trillion? Here's 1 Reason I'd Be Cautious</t>
         </is>
       </c>
       <c r="AY43" s="90" t="inlineStr">
         <is>
-          <t>NVIDIA Deal Highlights Value of Tiny's Early Poolside Investment</t>
+          <t>Dow Jones Futures: AMD, Nvidia Lead AI Trade Higher; Meta, Netflix, SpaceX, Tesla Earnings On Deck</t>
         </is>
       </c>
       <c r="AZ43" s="90" t="inlineStr">
         <is>
-          <t>Cleveland-Cliffs Inc. Q3 2026 Earnings Call Summary</t>
+          <t>Where Will VTI Be in 20 Years? Here's What History Suggests</t>
         </is>
       </c>
     </row>
@@ -10720,17 +10720,17 @@
       </c>
       <c r="AX46" s="79" t="inlineStr">
         <is>
+          <t>Does Neutron Delay Change The Bull Case For Rocket Lab (RKLB)?</t>
+        </is>
+      </c>
+      <c r="AY46" s="79" t="inlineStr">
+        <is>
+          <t>Rocket Lab Corporation (RKLB) Rises Higher Than Market: Key Facts</t>
+        </is>
+      </c>
+      <c r="AZ46" s="79" t="inlineStr">
+        <is>
           <t>Rocket Lab Delays Neutron Again. Is the Stock in Trouble?</t>
-        </is>
-      </c>
-      <c r="AY46" s="79" t="inlineStr">
-        <is>
-          <t>Rocket Lab's Biggest Technological Advantage Is Fast Becoming Its Biggest Problem</t>
-        </is>
-      </c>
-      <c r="AZ46" s="79" t="inlineStr">
-        <is>
-          <t>AST SpaceMobile Rises 4% as Europe’s Largest Carriers Explore Joint Satellite Spectrum Bid; SpaceX and Rock...</t>
         </is>
       </c>
     </row>
@@ -11096,7 +11096,7 @@
       </c>
       <c r="AX48" s="79" t="inlineStr">
         <is>
-          <t>Tesla-SpaceX merger is 'not so easy': Analyst</t>
+          <t>Datadog, Intel, CoreWeave, Tesla, Amazon, Cleveland-Cliffs, and More Stocks That Explain Today’s Market</t>
         </is>
       </c>
       <c r="AY48" s="79" t="inlineStr">
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 19 Oct 2026, 09:39 PM · Yahoo Finance data</t>
+          <t>Built 19 Oct 2026, 11:45 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 19 Oct 2026, 09:39 PM · Yahoo Finance data</t>
+          <t>Built 19 Oct 2026, 11:45 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 19 Oct 2026, 09:39 PM · Yahoo Finance data</t>
+          <t>Built 19 Oct 2026, 11:45 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 19 Oct 2026, 09:39 PM · Yahoo Finance data</t>
+          <t>Built 19 Oct 2026, 11:45 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-10-20 23:12 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 20 Oct 2026, 08:46 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 20 Oct 2026, 11:12 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 20 Oct 2026, 08:46 PM · Yahoo Finance data</t>
+          <t>Built 20 Oct 2026, 11:12 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -3620,10 +3620,10 @@
         <v>164.9600067138672</v>
       </c>
       <c r="W7" s="73" t="n">
-        <v>9546463</v>
+        <v>9555363</v>
       </c>
       <c r="X7" s="74" t="n">
-        <v>1.280000183422934</v>
+        <v>1.281117065900471</v>
       </c>
       <c r="Y7" s="28" t="n">
         <v>38.83786429274229</v>
@@ -3810,10 +3810,10 @@
         <v>177.3999938964844</v>
       </c>
       <c r="W8" s="84" t="n">
-        <v>8129035</v>
+        <v>8131992</v>
       </c>
       <c r="X8" s="85" t="n">
-        <v>0.962312442587712</v>
+        <v>0.9626456426166723</v>
       </c>
       <c r="Y8" s="35" t="n">
         <v>69.24158925192168</v>
@@ -4000,10 +4000,10 @@
         <v>55.16999816894531</v>
       </c>
       <c r="W9" s="73" t="n">
-        <v>20161698</v>
+        <v>20206833</v>
       </c>
       <c r="X9" s="74" t="n">
-        <v>0.5463740068913585</v>
+        <v>0.54756366009582</v>
       </c>
       <c r="Y9" s="28" t="n">
         <v>55.85945311688045</v>
@@ -4190,10 +4190,10 @@
         <v>66.83499908447266</v>
       </c>
       <c r="W10" s="84" t="n">
-        <v>39307414</v>
+        <v>39326256</v>
       </c>
       <c r="X10" s="85" t="n">
-        <v>1.214745250590634</v>
+        <v>1.215292155957947</v>
       </c>
       <c r="Y10" s="35" t="n">
         <v>66.73595929299191</v>
@@ -4380,10 +4380,10 @@
         <v>87.48989868164062</v>
       </c>
       <c r="W11" s="73" t="n">
-        <v>15518806</v>
+        <v>15526822</v>
       </c>
       <c r="X11" s="74" t="n">
-        <v>1.222009970021994</v>
+        <v>1.222602594459063</v>
       </c>
       <c r="Y11" s="28" t="n">
         <v>70.57937149420148</v>
@@ -4570,10 +4570,10 @@
         <v>114.5599975585938</v>
       </c>
       <c r="W12" s="84" t="n">
-        <v>7396378</v>
+        <v>7396403</v>
       </c>
       <c r="X12" s="85" t="n">
-        <v>1.052827893400332</v>
+        <v>1.052831264663223</v>
       </c>
       <c r="Y12" s="35" t="n">
         <v>62.5914240337225</v>
@@ -4760,10 +4760,10 @@
         <v>109.6500015258789</v>
       </c>
       <c r="W13" s="73" t="n">
-        <v>4392869</v>
+        <v>4394896</v>
       </c>
       <c r="X13" s="74" t="n">
-        <v>0.6960143292915686</v>
+        <v>0.6963243093059902</v>
       </c>
       <c r="Y13" s="28" t="n">
         <v>45.33698882865465</v>
@@ -4950,10 +4950,10 @@
         <v>50.61000061035156</v>
       </c>
       <c r="W14" s="84" t="n">
-        <v>11264038</v>
+        <v>11265990</v>
       </c>
       <c r="X14" s="85" t="n">
-        <v>0.961613786012065</v>
+        <v>0.9617724151286953</v>
       </c>
       <c r="Y14" s="35" t="n">
         <v>60.91374473415699</v>
@@ -5140,10 +5140,10 @@
         <v>182.8099975585938</v>
       </c>
       <c r="W15" s="73" t="n">
-        <v>9173240</v>
+        <v>9190983</v>
       </c>
       <c r="X15" s="74" t="n">
-        <v>1.110043409512047</v>
+        <v>1.112071085709289</v>
       </c>
       <c r="Y15" s="28" t="n">
         <v>38.05726409483393</v>
@@ -5330,10 +5330,10 @@
         <v>41.86000061035156</v>
       </c>
       <c r="W16" s="84" t="n">
-        <v>6502647</v>
+        <v>6503408</v>
       </c>
       <c r="X16" s="85" t="n">
-        <v>0.8565528271014855</v>
+        <v>0.8566487752508817</v>
       </c>
       <c r="Y16" s="35" t="n">
         <v>53.98042056448287</v>
@@ -5520,10 +5520,10 @@
         <v>41.43999862670898</v>
       </c>
       <c r="W17" s="73" t="n">
-        <v>17893763</v>
+        <v>17912646</v>
       </c>
       <c r="X17" s="74" t="n">
-        <v>0.4994556805806482</v>
+        <v>0.4999695722324235</v>
       </c>
       <c r="Y17" s="28" t="n">
         <v>55.37500265255778</v>
@@ -5729,10 +5729,10 @@
         <v>764.260009765625</v>
       </c>
       <c r="W19" s="73" t="n">
-        <v>32501960</v>
+        <v>34504254</v>
       </c>
       <c r="X19" s="74" t="n">
-        <v>0.7875860085956072</v>
+        <v>0.8340820432051655</v>
       </c>
       <c r="Y19" s="28" t="n">
         <v>49.67709477004971</v>
@@ -5908,7 +5908,7 @@
         <v>-0.72998046875</v>
       </c>
       <c r="T20" s="83" t="n">
-        <v>715.1900024414062</v>
+        <v>715.25</v>
       </c>
       <c r="U20" s="83" t="n">
         <v>722.7465209960938</v>
@@ -5917,10 +5917,10 @@
         <v>710.3900146484375</v>
       </c>
       <c r="W20" s="84" t="n">
-        <v>28641296</v>
+        <v>29494120</v>
       </c>
       <c r="X20" s="85" t="n">
-        <v>0.8198960108591</v>
+        <v>0.8432798965652538</v>
       </c>
       <c r="Y20" s="35" t="n">
         <v>40.79309619213983</v>
@@ -6105,10 +6105,10 @@
         <v>271.2900085449219</v>
       </c>
       <c r="W21" s="73" t="n">
-        <v>25952826</v>
+        <v>26282083</v>
       </c>
       <c r="X21" s="74" t="n">
-        <v>0.9908753827049406</v>
+        <v>1.002816050972961</v>
       </c>
       <c r="Y21" s="28" t="n">
         <v>42.88316703090203</v>
@@ -6221,7 +6221,7 @@
       </c>
       <c r="F22" s="30" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Same</t>
         </is>
       </c>
       <c r="G22" s="30" t="inlineStr">
@@ -6293,10 +6293,10 @@
         <v>91.35369873046875</v>
       </c>
       <c r="W22" s="84" t="n">
-        <v>92467173</v>
+        <v>94282304</v>
       </c>
       <c r="X22" s="85" t="n">
-        <v>1.252822726756538</v>
+        <v>1.275846802593048</v>
       </c>
       <c r="Y22" s="35" t="n">
         <v>33.03223070019696</v>
@@ -6430,7 +6430,7 @@
       </c>
       <c r="F24" s="23" t="inlineStr">
         <is>
-          <t>Same</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G24" s="23" t="inlineStr">
@@ -6502,10 +6502,10 @@
         <v>338.7000122070312</v>
       </c>
       <c r="W24" s="73" t="n">
-        <v>35385537</v>
+        <v>35678066</v>
       </c>
       <c r="X24" s="74" t="n">
-        <v>0.9640574316300252</v>
+        <v>0.9716400186982215</v>
       </c>
       <c r="Y24" s="28" t="n">
         <v>55.53136087143232</v>
@@ -6584,17 +6584,17 @@
       </c>
       <c r="AX24" s="79" t="inlineStr">
         <is>
-          <t>Prediction: Apple’s Stock Is Due for a Reality Check on Nov. 2</t>
+          <t>Apple’s $1,999 foldable phone is set to hit stores Friday, are you buying one?</t>
         </is>
       </c>
       <c r="AY24" s="79" t="inlineStr">
         <is>
-          <t>Apple faces gross margin pressure as UBS flags slowing iPhone growth ahead of earnings</t>
+          <t>Apple Stock Downgraded As Analysts Turn Cautious On iPhone Maker</t>
         </is>
       </c>
       <c r="AZ24" s="79" t="inlineStr">
         <is>
-          <t>Laurene Powell Jobs Bought $250 Million of Skydance Stock. Now She Is Down $100 Million.</t>
+          <t>Apple (AAPL) Stock Sinks As Market Gains: What You Should Know</t>
         </is>
       </c>
     </row>
@@ -6690,10 +6690,10 @@
         <v>524.5999755859375</v>
       </c>
       <c r="W25" s="84" t="n">
-        <v>14760396</v>
+        <v>14863088</v>
       </c>
       <c r="X25" s="85" t="n">
-        <v>0.7619755571613512</v>
+        <v>0.7670735006787449</v>
       </c>
       <c r="Y25" s="35" t="n">
         <v>39.80580444458145</v>
@@ -6878,10 +6878,10 @@
         <v>260.4200134277344</v>
       </c>
       <c r="W26" s="73" t="n">
-        <v>34435852</v>
+        <v>34498734</v>
       </c>
       <c r="X26" s="74" t="n">
-        <v>0.9541849967391703</v>
+        <v>0.9558441244960677</v>
       </c>
       <c r="Y26" s="28" t="n">
         <v>57.40799983522404</v>
@@ -6960,17 +6960,17 @@
       </c>
       <c r="AX26" s="79" t="inlineStr">
         <is>
+          <t>Why Is 3M (MMM) Stock Rocketing Higher Today</t>
+        </is>
+      </c>
+      <c r="AY26" s="79" t="inlineStr">
+        <is>
+          <t>Amazon vs Alphabet: Which "Magnificent Seven" Stock Is the Better Buy Right Now?</t>
+        </is>
+      </c>
+      <c r="AZ26" s="79" t="inlineStr">
+        <is>
           <t>Amazon Stock Costs More Than the Market. I'd Still Buy It for the Next 5 Years.</t>
-        </is>
-      </c>
-      <c r="AY26" s="79" t="inlineStr">
-        <is>
-          <t>Amazon stockpiles Nvidia AI hardware ahead of power availability -Business Insider</t>
-        </is>
-      </c>
-      <c r="AZ26" s="79" t="inlineStr">
-        <is>
-          <t>Amazon’s $350 target rests on an AI bet beyond the cloud</t>
         </is>
       </c>
     </row>
@@ -7066,10 +7066,10 @@
         <v>81.23999786376953</v>
       </c>
       <c r="W27" s="84" t="n">
-        <v>3519623</v>
+        <v>3532967</v>
       </c>
       <c r="X27" s="85" t="n">
-        <v>0.8006811250360757</v>
+        <v>0.8035947885128817</v>
       </c>
       <c r="Y27" s="35" t="n">
         <v>42.80820999722767</v>
@@ -7254,10 +7254,10 @@
         <v>217.2599945068359</v>
       </c>
       <c r="W28" s="73" t="n">
-        <v>5066053</v>
+        <v>5083801</v>
       </c>
       <c r="X28" s="74" t="n">
-        <v>0.922877899221057</v>
+        <v>0.9259613470135818</v>
       </c>
       <c r="Y28" s="28" t="n">
         <v>32.83764745019016</v>
@@ -7370,7 +7370,7 @@
       </c>
       <c r="F29" s="30" t="inlineStr">
         <is>
-          <t>Same</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G29" s="30" t="inlineStr">
@@ -7433,7 +7433,7 @@
         <v>-0.7399978637695312</v>
       </c>
       <c r="T29" s="83" t="n">
-        <v>41.58499908447266</v>
+        <v>41.56000137329102</v>
       </c>
       <c r="U29" s="83" t="n">
         <v>42.36890029907227</v>
@@ -7442,10 +7442,10 @@
         <v>39.01670074462891</v>
       </c>
       <c r="W29" s="84" t="n">
-        <v>13907917</v>
+        <v>13975946</v>
       </c>
       <c r="X29" s="85" t="n">
-        <v>0.8243110577557955</v>
+        <v>0.8281761205811076</v>
       </c>
       <c r="Y29" s="35" t="n">
         <v>30.76241799256044</v>
@@ -7630,10 +7630,10 @@
         <v>330.8001098632812</v>
       </c>
       <c r="W30" s="73" t="n">
-        <v>15695935</v>
+        <v>15742796</v>
       </c>
       <c r="X30" s="74" t="n">
-        <v>0.7253303005134301</v>
+        <v>0.7274170490079919</v>
       </c>
       <c r="Y30" s="28" t="n">
         <v>38.6287317043238</v>
@@ -7818,10 +7818,10 @@
         <v>79.25</v>
       </c>
       <c r="W31" s="84" t="n">
-        <v>2303846</v>
+        <v>2304154</v>
       </c>
       <c r="X31" s="85" t="n">
-        <v>0.7162859904526748</v>
+        <v>0.7163783203462686</v>
       </c>
       <c r="Y31" s="35" t="n">
         <v>34.3003670433898</v>
@@ -8006,10 +8006,10 @@
         <v>57.23500061035156</v>
       </c>
       <c r="W32" s="73" t="n">
-        <v>90575820</v>
+        <v>91559625</v>
       </c>
       <c r="X32" s="74" t="n">
-        <v>1.9781175768029</v>
+        <v>1.99745740912122</v>
       </c>
       <c r="Y32" s="28" t="n">
         <v>30.81665986518259</v>
@@ -8194,10 +8194,10 @@
         <v>439.5</v>
       </c>
       <c r="W33" s="84" t="n">
-        <v>5028540</v>
+        <v>5244274</v>
       </c>
       <c r="X33" s="85" t="n">
-        <v>0.7288286280042473</v>
+        <v>0.7589102866578835</v>
       </c>
       <c r="Y33" s="35" t="n">
         <v>35.98291998634041</v>
@@ -8276,17 +8276,17 @@
       </c>
       <c r="AX33" s="90" t="inlineStr">
         <is>
+          <t>Super Micro Computer Surges On Blowout Preliminary Revenue; Dell, HPE Also Jump</t>
+        </is>
+      </c>
+      <c r="AY33" s="90" t="inlineStr">
+        <is>
           <t>How AI Server Demand Will Impact Dell Stock Investors</t>
         </is>
       </c>
-      <c r="AY33" s="90" t="inlineStr">
+      <c r="AZ33" s="90" t="inlineStr">
         <is>
           <t>Dell Technologies (DELL), What Is Driving The Latest Attention?</t>
-        </is>
-      </c>
-      <c r="AZ33" s="90" t="inlineStr">
-        <is>
-          <t>What Could Derail Dell Stock?</t>
         </is>
       </c>
     </row>
@@ -8382,10 +8382,10 @@
         <v>334.6000061035156</v>
       </c>
       <c r="W34" s="73" t="n">
-        <v>13598539</v>
+        <v>13651876</v>
       </c>
       <c r="X34" s="74" t="n">
-        <v>0.8700608214501634</v>
+        <v>0.8733244103145129</v>
       </c>
       <c r="Y34" s="28" t="n">
         <v>44.02745026472717</v>
@@ -8464,17 +8464,17 @@
       </c>
       <c r="AX34" s="79" t="inlineStr">
         <is>
-          <t>Microsoft, Alphabet, Goldman Sachs Join Growing List of Companies Objecting to Tokenized Stocks</t>
+          <t>Amazon vs Alphabet: Which "Magnificent Seven" Stock Is the Better Buy Right Now?</t>
         </is>
       </c>
       <c r="AY34" s="79" t="inlineStr">
         <is>
-          <t>Alphabet Stock And 2 More Undervalued Stocks To Watch</t>
+          <t>Alphabet (GOOGL) Stock Declines While Market Improves: Some Information for Investors</t>
         </is>
       </c>
       <c r="AZ34" s="79" t="inlineStr">
         <is>
-          <t>Bank of England investigates Google outage</t>
+          <t>Alphabet Inc. (GOOG) Stock Drops Despite Market Gains: Important Facts to Note</t>
         </is>
       </c>
     </row>
@@ -8570,10 +8570,10 @@
         <v>25.59000015258789</v>
       </c>
       <c r="W35" s="84" t="n">
-        <v>70092133</v>
+        <v>70908845</v>
       </c>
       <c r="X35" s="85" t="n">
-        <v>1.457529418108612</v>
+        <v>1.473261491568378</v>
       </c>
       <c r="Y35" s="35" t="n">
         <v>23.64130276579378</v>
@@ -8652,17 +8652,17 @@
       </c>
       <c r="AX35" s="90" t="inlineStr">
         <is>
+          <t>Stock Market Today, Oct. 20: IREN Slides on Funding Worries and Rate Fears</t>
+        </is>
+      </c>
+      <c r="AY35" s="90" t="inlineStr">
+        <is>
           <t>IREN Sinks 6%, Then Recovers After Co-CEO’s No-Debt Reassurance as Neocloud Worries Persist; TeraWulf and A...</t>
         </is>
       </c>
-      <c r="AY35" s="90" t="inlineStr">
+      <c r="AZ35" s="90" t="inlineStr">
         <is>
           <t>How Analyst Upgrade Optimism Will Impact IREN Stock Investors</t>
-        </is>
-      </c>
-      <c r="AZ35" s="90" t="inlineStr">
-        <is>
-          <t>IREN Co-CEO Daniel Roberts Says Firm’s Data Centers Carry No Debt As Funding Worries Hit Stock</t>
         </is>
       </c>
     </row>
@@ -8758,10 +8758,10 @@
         <v>88.76999664306641</v>
       </c>
       <c r="W36" s="73" t="n">
-        <v>80544770</v>
+        <v>81263600</v>
       </c>
       <c r="X36" s="74" t="n">
-        <v>0.8142480234261074</v>
+        <v>0.8212164803954115</v>
       </c>
       <c r="Y36" s="28" t="n">
         <v>34.38724006944398</v>
@@ -8943,13 +8943,13 @@
         <v>534.2100219726562</v>
       </c>
       <c r="V37" s="83" t="n">
-        <v>525.9000244140625</v>
+        <v>525.8599853515625</v>
       </c>
       <c r="W37" s="84" t="n">
-        <v>14411615</v>
+        <v>14432432</v>
       </c>
       <c r="X37" s="85" t="n">
-        <v>0.6716057242869046</v>
+        <v>0.6725432098641166</v>
       </c>
       <c r="Y37" s="35" t="n">
         <v>58.34264875143733</v>
@@ -8958,7 +8958,7 @@
         <v>50.53871531936947</v>
       </c>
       <c r="AA37" s="35" t="n">
-        <v>34.61752685422089</v>
+        <v>34.61275779218539</v>
       </c>
       <c r="AB37" s="86" t="n">
         <v>10.10718133012574</v>
@@ -9000,7 +9000,7 @@
         <v>9.946551332615911</v>
       </c>
       <c r="AO37" s="88" t="n">
-        <v>2.152086379664823</v>
+        <v>2.152624092463434</v>
       </c>
       <c r="AP37" s="83" t="n">
         <v>553.719970703125</v>
@@ -9028,17 +9028,17 @@
       </c>
       <c r="AX37" s="90" t="inlineStr">
         <is>
+          <t>Morgan Stanley sees new hurdle for Microsoft stock</t>
+        </is>
+      </c>
+      <c r="AY37" s="90" t="inlineStr">
+        <is>
           <t>Microsoft, Alphabet, Goldman Sachs Join Growing List of Companies Objecting to Tokenized Stocks</t>
         </is>
       </c>
-      <c r="AY37" s="90" t="inlineStr">
+      <c r="AZ37" s="90" t="inlineStr">
         <is>
           <t>Microsoft (MSFT) Withdraws From UK AI Data Center Project</t>
-        </is>
-      </c>
-      <c r="AZ37" s="90" t="inlineStr">
-        <is>
-          <t>Boeing, Microsoft Reveal AI Aircraft Platform, FAA Certifies 737 Max 10</t>
         </is>
       </c>
     </row>
@@ -9134,10 +9134,10 @@
         <v>133.5950012207031</v>
       </c>
       <c r="W38" s="73" t="n">
-        <v>18320150</v>
+        <v>18369195</v>
       </c>
       <c r="X38" s="74" t="n">
-        <v>0.959562648334561</v>
+        <v>0.9620079373322558</v>
       </c>
       <c r="Y38" s="28" t="n">
         <v>47.37837324748938</v>
@@ -9322,10 +9322,10 @@
         <v>881.52001953125</v>
       </c>
       <c r="W39" s="84" t="n">
-        <v>19165658</v>
+        <v>19362385</v>
       </c>
       <c r="X39" s="85" t="n">
-        <v>0.7273224573574555</v>
+        <v>0.7345139196525388</v>
       </c>
       <c r="Y39" s="35" t="n">
         <v>37.46133988311949</v>
@@ -9414,7 +9414,7 @@
       </c>
       <c r="AZ39" s="90" t="inlineStr">
         <is>
-          <t>Prediction: Micron Could Turn a $5,000 Investment Into This by 2030</t>
+          <t>SpaceX, GE Aerospace, Micron, GM, CoreWeave, Braze, and More Stocks That Explain Today’s Market</t>
         </is>
       </c>
     </row>
@@ -9501,7 +9501,7 @@
         <v>1.209991455078125</v>
       </c>
       <c r="T40" s="72" t="n">
-        <v>163.9949951171875</v>
+        <v>163.9575042724609</v>
       </c>
       <c r="U40" s="72" t="n">
         <v>174.7400054931641</v>
@@ -9510,10 +9510,10 @@
         <v>160.2799987792969</v>
       </c>
       <c r="W40" s="73" t="n">
-        <v>21052819</v>
+        <v>21380151</v>
       </c>
       <c r="X40" s="74" t="n">
-        <v>1.067973799104995</v>
+        <v>1.083679071865132</v>
       </c>
       <c r="Y40" s="28" t="n">
         <v>33.67150393657009</v>
@@ -9698,10 +9698,10 @@
         <v>68.19999694824219</v>
       </c>
       <c r="W41" s="84" t="n">
-        <v>58015098</v>
+        <v>62819587</v>
       </c>
       <c r="X41" s="85" t="n">
-        <v>1.600654501733236</v>
+        <v>1.721799978516279</v>
       </c>
       <c r="Y41" s="35" t="n">
         <v>40.50449479975881</v>
@@ -9785,12 +9785,12 @@
       </c>
       <c r="AY41" s="90" t="inlineStr">
         <is>
-          <t>Netflix stock sinks after announcing Q3 earnings, Q4 revenue forecast falls short of estimates</t>
+          <t>Netflix shares drop on slowing engagement, revenue growth</t>
         </is>
       </c>
       <c r="AZ41" s="90" t="inlineStr">
         <is>
-          <t>Have we hit AI IPO fatigue? More Netflix woes, and airlines try to stay afloat</t>
+          <t>Netflix Cut Its Ad Revenue Forecast by $300 Million. Does That Matter More Than Its Earnings Beat?</t>
         </is>
       </c>
     </row>
@@ -9886,10 +9886,10 @@
         <v>8.819999694824219</v>
       </c>
       <c r="W42" s="73" t="n">
-        <v>63124265</v>
+        <v>63221253</v>
       </c>
       <c r="X42" s="74" t="n">
-        <v>0.9326203224515613</v>
+        <v>0.9339863405343486</v>
       </c>
       <c r="Y42" s="28" t="n">
         <v>36.70067209134235</v>
@@ -10065,7 +10065,7 @@
         <v>-0.6199951171875</v>
       </c>
       <c r="T43" s="83" t="n">
-        <v>215.9700012207031</v>
+        <v>215.9799957275391</v>
       </c>
       <c r="U43" s="83" t="n">
         <v>218.4600067138672</v>
@@ -10074,10 +10074,10 @@
         <v>212.7700042724609</v>
       </c>
       <c r="W43" s="84" t="n">
-        <v>75939111</v>
+        <v>77454645</v>
       </c>
       <c r="X43" s="85" t="n">
-        <v>0.734880703347478</v>
+        <v>0.748997636904284</v>
       </c>
       <c r="Y43" s="35" t="n">
         <v>40.90296305103072</v>
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
-          <t>Unretired at 68 and the Paycheck Is Back? These 3 ETFs Decide What the New Money Should Do</t>
+          <t>This Nuclear Stock Could Be Your Ticket to Millionaire Status -- and It Didn't Even Need to Build a Reactor...</t>
         </is>
       </c>
       <c r="AY43" s="90" t="inlineStr">
         <is>
-          <t>Amazon stockpiles Nvidia AI hardware ahead of power availability -Business Insider</t>
+          <t>3 Stocks That Can Benefit From SpaceX’s Surprise Q3 Earnings</t>
         </is>
       </c>
       <c r="AZ43" s="90" t="inlineStr">
         <is>
-          <t>Market Chatter: Amazon is Buying More Nvidia AI Hardware Than It Can Power Up</t>
+          <t>SpaceX Crushes Q3 with Some Help From Musk</t>
         </is>
       </c>
     </row>
@@ -10253,7 +10253,7 @@
         <v>-1.54998779296875</v>
       </c>
       <c r="T44" s="72" t="n">
-        <v>192.1820068359375</v>
+        <v>192.4400024414062</v>
       </c>
       <c r="U44" s="72" t="n">
         <v>196.1100006103516</v>
@@ -10262,10 +10262,10 @@
         <v>189.4199981689453</v>
       </c>
       <c r="W44" s="73" t="n">
-        <v>14939515</v>
+        <v>14979559</v>
       </c>
       <c r="X44" s="74" t="n">
-        <v>0.6534170254754422</v>
+        <v>0.6551110810165154</v>
       </c>
       <c r="Y44" s="28" t="n">
         <v>52.12375921358297</v>
@@ -10450,10 +10450,10 @@
         <v>171.1300048828125</v>
       </c>
       <c r="W45" s="84" t="n">
-        <v>6690116</v>
+        <v>6822800</v>
       </c>
       <c r="X45" s="85" t="n">
-        <v>0.6390445149162152</v>
+        <v>0.651305847796349</v>
       </c>
       <c r="Y45" s="35" t="n">
         <v>47.11882413591954</v>
@@ -10537,12 +10537,12 @@
       </c>
       <c r="AY45" s="90" t="inlineStr">
         <is>
+          <t>Qualcomm (QCOM) Beats Stock Market Upswing: What Investors Need to Know</t>
+        </is>
+      </c>
+      <c r="AZ45" s="90" t="inlineStr">
+        <is>
           <t>Microsoft, Alphabet, Goldman Sachs Join Growing List of Companies Objecting to Tokenized Stocks</t>
-        </is>
-      </c>
-      <c r="AZ45" s="90" t="inlineStr">
-        <is>
-          <t>Qualcomm To Reportedly Conduct Global Layoffs In Performance-Driven Overhaul</t>
         </is>
       </c>
     </row>
@@ -10566,7 +10566,7 @@
       </c>
       <c r="F46" s="23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Same</t>
         </is>
       </c>
       <c r="G46" s="23" t="inlineStr">
@@ -10629,7 +10629,7 @@
         <v>-0.4599990844726562</v>
       </c>
       <c r="T46" s="72" t="n">
-        <v>50.56499862670898</v>
+        <v>50.53499984741211</v>
       </c>
       <c r="U46" s="72" t="n">
         <v>52.71500015258789</v>
@@ -10638,10 +10638,10 @@
         <v>49.25009918212891</v>
       </c>
       <c r="W46" s="73" t="n">
-        <v>16501835</v>
+        <v>16653261</v>
       </c>
       <c r="X46" s="74" t="n">
-        <v>0.7553631658611252</v>
+        <v>0.762030515789451</v>
       </c>
       <c r="Y46" s="28" t="n">
         <v>26.21422207872999</v>
@@ -10826,10 +10826,10 @@
         <v>1330.510009765625</v>
       </c>
       <c r="W47" s="84" t="n">
-        <v>6272528</v>
+        <v>6333961</v>
       </c>
       <c r="X47" s="85" t="n">
-        <v>0.7926813163377151</v>
+        <v>0.8001342273223002</v>
       </c>
       <c r="Y47" s="35" t="n">
         <v>35.87824519909739</v>
@@ -11014,10 +11014,10 @@
         <v>363.6400146484375</v>
       </c>
       <c r="W48" s="73" t="n">
-        <v>30572948</v>
+        <v>30761382</v>
       </c>
       <c r="X48" s="74" t="n">
-        <v>0.8810459340489499</v>
+        <v>0.8862355680997774</v>
       </c>
       <c r="Y48" s="28" t="n">
         <v>53.68072977604398</v>
@@ -11096,17 +11096,17 @@
       </c>
       <c r="AX48" s="79" t="inlineStr">
         <is>
+          <t>SpaceX-Tesla merger? Musk speaks on 'tap-dancing through a minefield'</t>
+        </is>
+      </c>
+      <c r="AY48" s="79" t="inlineStr">
+        <is>
           <t>Tesla Q3 earnings preview: 3 key things to watch</t>
         </is>
       </c>
-      <c r="AY48" s="79" t="inlineStr">
-        <is>
-          <t>Tesla Q3 preview: Delivery outlook, cash flow, and a dash of merger speculation on tap</t>
-        </is>
-      </c>
       <c r="AZ48" s="79" t="inlineStr">
         <is>
-          <t>What could a Tesla-SpaceX merger earn? Cathie Wood's Ark Invest has a $2.7 trillion answer.</t>
+          <t>SpaceX and Tesla boards form special committees to review merger</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 20 Oct 2026, 08:46 PM · Yahoo Finance data</t>
+          <t>Built 20 Oct 2026, 11:12 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 20 Oct 2026, 08:46 PM · Yahoo Finance data</t>
+          <t>Built 20 Oct 2026, 11:12 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 20 Oct 2026, 08:46 PM · Yahoo Finance data</t>
+          <t>Built 20 Oct 2026, 11:12 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 20 Oct 2026, 08:46 PM · Yahoo Finance data</t>
+          <t>Built 20 Oct 2026, 11:12 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -44836,7 +44836,7 @@
       </c>
       <c r="D38" s="107" t="inlineStr">
         <is>
-          <t>Gapped down 1.5% at the open</t>
+          <t>Gapped down 1.6% at the open</t>
         </is>
       </c>
       <c r="E38" s="26" t="n">

</xml_diff>

<commit_message>
Daily workbook: 2026-10-20 23:50 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 20 Oct 2026, 11:12 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 20 Oct 2026, 11:50 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 20 Oct 2026, 11:12 PM · Yahoo Finance data</t>
+          <t>Built 20 Oct 2026, 11:50 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -8469,12 +8469,12 @@
       </c>
       <c r="AY34" s="79" t="inlineStr">
         <is>
+          <t>Alphabet Inc. (GOOG) Stock Drops Despite Market Gains: Important Facts to Note</t>
+        </is>
+      </c>
+      <c r="AZ34" s="79" t="inlineStr">
+        <is>
           <t>Alphabet (GOOGL) Stock Declines While Market Improves: Some Information for Investors</t>
-        </is>
-      </c>
-      <c r="AZ34" s="79" t="inlineStr">
-        <is>
-          <t>Alphabet Inc. (GOOG) Stock Drops Despite Market Gains: Important Facts to Note</t>
         </is>
       </c>
     </row>
@@ -9785,12 +9785,12 @@
       </c>
       <c r="AY41" s="90" t="inlineStr">
         <is>
+          <t>Netflix Q3 Earnings Call Highlights</t>
+        </is>
+      </c>
+      <c r="AZ41" s="90" t="inlineStr">
+        <is>
           <t>Netflix shares drop on slowing engagement, revenue growth</t>
-        </is>
-      </c>
-      <c r="AZ41" s="90" t="inlineStr">
-        <is>
-          <t>Netflix Cut Its Ad Revenue Forecast by $300 Million. Does That Matter More Than Its Earnings Beat?</t>
         </is>
       </c>
     </row>
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
+          <t>2 Stocks to Buy From the 5 That Make Up Roughly 61.5% of Berkshire Hathaway's Portfolio</t>
+        </is>
+      </c>
+      <c r="AY43" s="90" t="inlineStr">
+        <is>
           <t>This Nuclear Stock Could Be Your Ticket to Millionaire Status -- and It Didn't Even Need to Build a Reactor...</t>
         </is>
       </c>
-      <c r="AY43" s="90" t="inlineStr">
+      <c r="AZ43" s="90" t="inlineStr">
         <is>
           <t>3 Stocks That Can Benefit From SpaceX’s Surprise Q3 Earnings</t>
-        </is>
-      </c>
-      <c r="AZ43" s="90" t="inlineStr">
-        <is>
-          <t>SpaceX Crushes Q3 with Some Help From Musk</t>
         </is>
       </c>
     </row>
@@ -11106,7 +11106,7 @@
       </c>
       <c r="AZ48" s="79" t="inlineStr">
         <is>
-          <t>SpaceX and Tesla boards form special committees to review merger</t>
+          <t>Dow Jones Futures: AI Stocks Jump On SpaceX, Supermicro; Tesla, Meta On Deck</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 20 Oct 2026, 11:12 PM · Yahoo Finance data</t>
+          <t>Built 20 Oct 2026, 11:50 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 20 Oct 2026, 11:12 PM · Yahoo Finance data</t>
+          <t>Built 20 Oct 2026, 11:50 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 20 Oct 2026, 11:12 PM · Yahoo Finance data</t>
+          <t>Built 20 Oct 2026, 11:50 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 20 Oct 2026, 11:12 PM · Yahoo Finance data</t>
+          <t>Built 20 Oct 2026, 11:50 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-10-21 23:24 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 21 Oct 2026, 08:47 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 21 Oct 2026, 11:24 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 21 Oct 2026, 08:47 PM · Yahoo Finance data</t>
+          <t>Built 21 Oct 2026, 11:24 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -3620,10 +3620,10 @@
         <v>167.3899993896484</v>
       </c>
       <c r="W7" s="73" t="n">
-        <v>7277283</v>
+        <v>7279725</v>
       </c>
       <c r="X7" s="74" t="n">
-        <v>0.9801029267379061</v>
+        <v>0.9804156924287467</v>
       </c>
       <c r="Y7" s="28" t="n">
         <v>45.21392022122898</v>
@@ -3810,10 +3810,10 @@
         <v>177.6399993896484</v>
       </c>
       <c r="W8" s="84" t="n">
-        <v>8461374</v>
+        <v>8461753</v>
       </c>
       <c r="X8" s="85" t="n">
-        <v>0.9954635293214111</v>
+        <v>0.9955058984946228</v>
       </c>
       <c r="Y8" s="35" t="n">
         <v>66.56956714312597</v>
@@ -4000,10 +4000,10 @@
         <v>55.63999938964844</v>
       </c>
       <c r="W9" s="73" t="n">
-        <v>27470174</v>
+        <v>27704785</v>
       </c>
       <c r="X9" s="74" t="n">
-        <v>0.7596361453848316</v>
+        <v>0.7658754330638647</v>
       </c>
       <c r="Y9" s="28" t="n">
         <v>58.54596315557711</v>
@@ -4190,10 +4190,10 @@
         <v>67.51499938964844</v>
       </c>
       <c r="W10" s="84" t="n">
-        <v>26375023</v>
+        <v>26380544</v>
       </c>
       <c r="X10" s="85" t="n">
-        <v>0.8280044543555628</v>
+        <v>0.8281706008312201</v>
       </c>
       <c r="Y10" s="35" t="n">
         <v>67.41490783867911</v>
@@ -4380,10 +4380,10 @@
         <v>86.91000366210938</v>
       </c>
       <c r="W11" s="73" t="n">
-        <v>13176329</v>
+        <v>13264011</v>
       </c>
       <c r="X11" s="74" t="n">
-        <v>1.027468864994847</v>
+        <v>1.033952693530864</v>
       </c>
       <c r="Y11" s="28" t="n">
         <v>65.64904786283529</v>
@@ -4570,10 +4570,10 @@
         <v>114.9599990844727</v>
       </c>
       <c r="W12" s="84" t="n">
-        <v>6440739</v>
+        <v>6440947</v>
       </c>
       <c r="X12" s="85" t="n">
-        <v>0.9200100283871234</v>
+        <v>0.920038372815115</v>
       </c>
       <c r="Y12" s="35" t="n">
         <v>62.68443449762388</v>
@@ -4760,10 +4760,10 @@
         <v>108.6100006103516</v>
       </c>
       <c r="W13" s="73" t="n">
-        <v>9297620</v>
+        <v>9306650</v>
       </c>
       <c r="X13" s="74" t="n">
-        <v>1.431475362082766</v>
+        <v>1.43276603753397</v>
       </c>
       <c r="Y13" s="28" t="n">
         <v>41.5549551834727</v>
@@ -4950,10 +4950,10 @@
         <v>50.95500183105469</v>
       </c>
       <c r="W14" s="84" t="n">
-        <v>7903422</v>
+        <v>7914807</v>
       </c>
       <c r="X14" s="85" t="n">
-        <v>0.6821185586833721</v>
+        <v>0.6830676016903501</v>
       </c>
       <c r="Y14" s="35" t="n">
         <v>61.68012088604651</v>
@@ -5140,10 +5140,10 @@
         <v>186.4700012207031</v>
       </c>
       <c r="W15" s="73" t="n">
-        <v>9558187</v>
+        <v>9569952</v>
       </c>
       <c r="X15" s="74" t="n">
-        <v>1.131003261735156</v>
+        <v>1.132316576573097</v>
       </c>
       <c r="Y15" s="28" t="n">
         <v>44.46304711724713</v>
@@ -5330,10 +5330,10 @@
         <v>41.97499847412109</v>
       </c>
       <c r="W16" s="84" t="n">
-        <v>6506774</v>
+        <v>6506802</v>
       </c>
       <c r="X16" s="85" t="n">
-        <v>0.8586843498530083</v>
+        <v>0.858687886303361</v>
       </c>
       <c r="Y16" s="35" t="n">
         <v>50.33456556372787</v>
@@ -5520,10 +5520,10 @@
         <v>41.8650016784668</v>
       </c>
       <c r="W17" s="73" t="n">
-        <v>37189135</v>
+        <v>40618387</v>
       </c>
       <c r="X17" s="74" t="n">
-        <v>1.024651394996892</v>
+        <v>1.113873478037085</v>
       </c>
       <c r="Y17" s="28" t="n">
         <v>56.49403929857731</v>
@@ -5729,10 +5729,10 @@
         <v>768.4000244140625</v>
       </c>
       <c r="W19" s="73" t="n">
-        <v>29996785</v>
+        <v>31623572</v>
       </c>
       <c r="X19" s="74" t="n">
-        <v>0.7471477209642424</v>
+        <v>0.786074508572621</v>
       </c>
       <c r="Y19" s="28" t="n">
         <v>53.48053970136419</v>
@@ -5845,7 +5845,7 @@
       </c>
       <c r="F20" s="30" t="inlineStr">
         <is>
-          <t>Same</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G20" s="30" t="inlineStr">
@@ -5917,10 +5917,10 @@
         <v>719.719970703125</v>
       </c>
       <c r="W20" s="84" t="n">
-        <v>30716866</v>
+        <v>31534625</v>
       </c>
       <c r="X20" s="85" t="n">
-        <v>0.8800649542742276</v>
+        <v>0.9024372785576342</v>
       </c>
       <c r="Y20" s="35" t="n">
         <v>45.98372421915985</v>
@@ -6105,10 +6105,10 @@
         <v>275.2999877929688</v>
       </c>
       <c r="W21" s="73" t="n">
-        <v>15496544</v>
+        <v>15740997</v>
       </c>
       <c r="X21" s="74" t="n">
-        <v>0.6012678593002827</v>
+        <v>0.6104631602253557</v>
       </c>
       <c r="Y21" s="28" t="n">
         <v>44.17332435036269</v>
@@ -6293,10 +6293,10 @@
         <v>99.30999755859375</v>
       </c>
       <c r="W22" s="84" t="n">
-        <v>75166315</v>
+        <v>76314129</v>
       </c>
       <c r="X22" s="85" t="n">
-        <v>1.004304535067795</v>
+        <v>1.018859326750166</v>
       </c>
       <c r="Y22" s="35" t="n">
         <v>37.09027381955874</v>
@@ -6496,16 +6496,16 @@
         <v>339.2049865722656</v>
       </c>
       <c r="U24" s="72" t="n">
-        <v>345.2200012207031</v>
+        <v>345.25</v>
       </c>
       <c r="V24" s="72" t="n">
         <v>338.8299865722656</v>
       </c>
       <c r="W24" s="73" t="n">
-        <v>35131228</v>
+        <v>35368592</v>
       </c>
       <c r="X24" s="74" t="n">
-        <v>0.9520215162674656</v>
+        <v>0.9581456903537892</v>
       </c>
       <c r="Y24" s="28" t="n">
         <v>60.64144034170997</v>
@@ -6514,7 +6514,7 @@
         <v>76.28277288773747</v>
       </c>
       <c r="AA24" s="28" t="n">
-        <v>18.17087497555117</v>
+        <v>18.17537445124041</v>
       </c>
       <c r="AB24" s="75" t="n">
         <v>3.853071122280767</v>
@@ -6556,7 +6556,7 @@
         <v>5.275490972590549</v>
       </c>
       <c r="AO24" s="77" t="n">
-        <v>1.881129911757746</v>
+        <v>1.881752828124677</v>
       </c>
       <c r="AP24" s="72" t="n">
         <v>348.1499938964844</v>
@@ -6690,10 +6690,10 @@
         <v>537.2999877929688</v>
       </c>
       <c r="W25" s="84" t="n">
-        <v>17657435</v>
+        <v>17756841</v>
       </c>
       <c r="X25" s="85" t="n">
-        <v>0.9074401591889473</v>
+        <v>0.9123157384883246</v>
       </c>
       <c r="Y25" s="35" t="n">
         <v>45.06717895559436</v>
@@ -6782,7 +6782,7 @@
       </c>
       <c r="AZ25" s="90" t="inlineStr">
         <is>
-          <t>AMD vs. Nvidia. 1 Metric Proves Which Is the Best Stock.</t>
+          <t>Teradyne, Vishay Intertechnology, Allegro MicroSystems, Entegris, and AMD shares are soaring, what you need...</t>
         </is>
       </c>
     </row>
@@ -6878,10 +6878,10 @@
         <v>259.2900085449219</v>
       </c>
       <c r="W26" s="73" t="n">
-        <v>30746898</v>
+        <v>30981629</v>
       </c>
       <c r="X26" s="74" t="n">
-        <v>0.867558138587019</v>
+        <v>0.8738919384984088</v>
       </c>
       <c r="Y26" s="28" t="n">
         <v>57.10063970368796</v>
@@ -6965,12 +6965,12 @@
       </c>
       <c r="AY26" s="79" t="inlineStr">
         <is>
+          <t>Amazon abandons $427 million GW campus data center plan and pledges land donations worth $65 million instead</t>
+        </is>
+      </c>
+      <c r="AZ26" s="79" t="inlineStr">
+        <is>
           <t>Amazon Ditches Ashburn Data Center Plan, Shifts To Mixed-Use Vision</t>
-        </is>
-      </c>
-      <c r="AZ26" s="79" t="inlineStr">
-        <is>
-          <t>Amazon's Nvidia Chips Are Sitting in Warehouses Without Power as AI Spending Soars, Business Insider Reports</t>
         </is>
       </c>
     </row>
@@ -7066,10 +7066,10 @@
         <v>84.375</v>
       </c>
       <c r="W27" s="84" t="n">
-        <v>3263503</v>
+        <v>3264054</v>
       </c>
       <c r="X27" s="85" t="n">
-        <v>0.7473819070972508</v>
+        <v>0.7475033765913983</v>
       </c>
       <c r="Y27" s="35" t="n">
         <v>47.81411691800711</v>
@@ -7254,10 +7254,10 @@
         <v>219.5</v>
       </c>
       <c r="W28" s="73" t="n">
-        <v>3218729</v>
+        <v>3239187</v>
       </c>
       <c r="X28" s="74" t="n">
-        <v>0.6062274215303758</v>
+        <v>0.6099630440038638</v>
       </c>
       <c r="Y28" s="28" t="n">
         <v>35.64726932516578</v>
@@ -7442,10 +7442,10 @@
         <v>40.58000183105469</v>
       </c>
       <c r="W29" s="84" t="n">
-        <v>10123545</v>
+        <v>10169707</v>
       </c>
       <c r="X29" s="85" t="n">
-        <v>0.5968050072327687</v>
+        <v>0.5994447926193853</v>
       </c>
       <c r="Y29" s="35" t="n">
         <v>30.54301423576503</v>
@@ -7524,17 +7524,17 @@
       </c>
       <c r="AX29" s="90" t="inlineStr">
         <is>
+          <t>Should You Sell Your AST SpaceMobile Stock Now?</t>
+        </is>
+      </c>
+      <c r="AY29" s="90" t="inlineStr">
+        <is>
           <t>AST SpaceMobile Hit a 52-Week Low Days After SpaceX Spent $8 Billion on Spectrum. That's Not a Coincidence.</t>
         </is>
       </c>
-      <c r="AY29" s="90" t="inlineStr">
-        <is>
-          <t>AST SpaceMobile Targets Initial Satellite Broadband Coverage in Five Countries by End of 2026</t>
-        </is>
-      </c>
       <c r="AZ29" s="90" t="inlineStr">
         <is>
-          <t>SpaceX Jumps 8% on Q3 Revenue Beat as Musk Backs Tesla Merger Idea; Rocket Lab and AST SpaceMobile Edge Higher</t>
+          <t>AST SpaceMobile Stock Gets a New Catalyst. Wall Street Sees 93% Upside.</t>
         </is>
       </c>
     </row>
@@ -7630,10 +7630,10 @@
         <v>332.2900085449219</v>
       </c>
       <c r="W30" s="73" t="n">
-        <v>16897548</v>
+        <v>16959641</v>
       </c>
       <c r="X30" s="74" t="n">
-        <v>0.7922709124746313</v>
+        <v>0.7950665153436166</v>
       </c>
       <c r="Y30" s="28" t="n">
         <v>41.04523544658122</v>
@@ -7818,10 +7818,10 @@
         <v>81.5</v>
       </c>
       <c r="W31" s="84" t="n">
-        <v>2721412</v>
+        <v>2739402</v>
       </c>
       <c r="X31" s="85" t="n">
-        <v>0.843171373717596</v>
+        <v>0.8485087192926501</v>
       </c>
       <c r="Y31" s="35" t="n">
         <v>38.40046348535039</v>
@@ -7900,17 +7900,17 @@
       </c>
       <c r="AX31" s="90" t="inlineStr">
         <is>
+          <t>Cameco (CCJ) Laps the Stock Market: Here's Why</t>
+        </is>
+      </c>
+      <c r="AY31" s="90" t="inlineStr">
+        <is>
           <t>Cameco Stock Is Nearly 40% Below Its Peak. Here’s What One AP1000 Reactor Pair Could Be Worth to Westinghouse</t>
         </is>
       </c>
-      <c r="AY31" s="90" t="inlineStr">
+      <c r="AZ31" s="90" t="inlineStr">
         <is>
           <t>Cameco Heads 3 Canadian Nuclear Stocks To Watch</t>
-        </is>
-      </c>
-      <c r="AZ31" s="90" t="inlineStr">
-        <is>
-          <t>Cameco Stock Is Down 36% From Its All-Time High. Here's What Needs to Happen to Make It a Buy</t>
         </is>
       </c>
     </row>
@@ -8006,10 +8006,10 @@
         <v>59.31000137329102</v>
       </c>
       <c r="W32" s="73" t="n">
-        <v>74067529</v>
+        <v>74632655</v>
       </c>
       <c r="X32" s="74" t="n">
-        <v>1.53931721962615</v>
+        <v>1.550151706899484</v>
       </c>
       <c r="Y32" s="28" t="n">
         <v>30.59954221346678</v>
@@ -8093,7 +8093,7 @@
       </c>
       <c r="AY32" s="79" t="inlineStr">
         <is>
-          <t>The bull case for CoreWeave as GPU demand surges</t>
+          <t>Did SpaceX Just Save CoreWeave, Nebius, and the Neocloud Sector?</t>
         </is>
       </c>
       <c r="AZ32" s="79" t="inlineStr">
@@ -8194,10 +8194,10 @@
         <v>480.5199890136719</v>
       </c>
       <c r="W33" s="84" t="n">
-        <v>6783524</v>
+        <v>6821140</v>
       </c>
       <c r="X33" s="85" t="n">
-        <v>0.9904369985013333</v>
+        <v>0.9956557545269221</v>
       </c>
       <c r="Y33" s="35" t="n">
         <v>42.43932574434353</v>
@@ -8281,12 +8281,12 @@
       </c>
       <c r="AY33" s="90" t="inlineStr">
         <is>
-          <t>Tech stocks lead market higher as SpaceX shares surge: AlphaCheck</t>
+          <t>Why Dell (DELL) stock is trading up today</t>
         </is>
       </c>
       <c r="AZ33" s="90" t="inlineStr">
         <is>
-          <t>Why Dell (DELL) stock is trading up today</t>
+          <t>2 Reasons Why Dell Stock Is Having a Super Day</t>
         </is>
       </c>
     </row>
@@ -8382,10 +8382,10 @@
         <v>326.260009765625</v>
       </c>
       <c r="W34" s="73" t="n">
-        <v>19054007</v>
+        <v>19130037</v>
       </c>
       <c r="X34" s="74" t="n">
-        <v>1.231075408616466</v>
+        <v>1.23568418953567</v>
       </c>
       <c r="Y34" s="28" t="n">
         <v>39.53381698725877</v>
@@ -8464,17 +8464,17 @@
       </c>
       <c r="AX34" s="79" t="inlineStr">
         <is>
+          <t>Why Meta didn't offer 2027 revenue guidance: Q3 earnings takeaways</t>
+        </is>
+      </c>
+      <c r="AY34" s="79" t="inlineStr">
+        <is>
+          <t>Prediction: This Artificial Intelligence (AI) Stock Will Be the Biggest Winner of 2027</t>
+        </is>
+      </c>
+      <c r="AZ34" s="79" t="inlineStr">
+        <is>
           <t>Kazakhstan’s AIFC Regulator Turns to Apple and Google to Enforce Coinbase, HTX Injunctions</t>
-        </is>
-      </c>
-      <c r="AY34" s="79" t="inlineStr">
-        <is>
-          <t>Bank of America sees a $300 billion test for Google stock</t>
-        </is>
-      </c>
-      <c r="AZ34" s="79" t="inlineStr">
-        <is>
-          <t>Sector Update: Tech Stocks Gain Late Afternoon</t>
         </is>
       </c>
     </row>
@@ -8570,10 +8570,10 @@
         <v>26.39999961853027</v>
       </c>
       <c r="W35" s="84" t="n">
-        <v>49746427</v>
+        <v>49884648</v>
       </c>
       <c r="X35" s="85" t="n">
-        <v>1.012732553493141</v>
+        <v>1.015403580511917</v>
       </c>
       <c r="Y35" s="35" t="n">
         <v>28.21488071612522</v>
@@ -8758,10 +8758,10 @@
         <v>90.76000213623047</v>
       </c>
       <c r="W36" s="73" t="n">
-        <v>73917997</v>
+        <v>74242457</v>
       </c>
       <c r="X36" s="74" t="n">
-        <v>0.7503622825595005</v>
+        <v>0.7535318720545814</v>
       </c>
       <c r="Y36" s="28" t="n">
         <v>36.40462449151186</v>
@@ -8946,10 +8946,10 @@
         <v>525.02001953125</v>
       </c>
       <c r="W37" s="84" t="n">
-        <v>13784913</v>
+        <v>13826924</v>
       </c>
       <c r="X37" s="85" t="n">
-        <v>0.6507342026377334</v>
+        <v>0.6526526684148622</v>
       </c>
       <c r="Y37" s="35" t="n">
         <v>58.93006414307374</v>
@@ -9134,10 +9134,10 @@
         <v>143.9299926757812</v>
       </c>
       <c r="W38" s="73" t="n">
-        <v>22253801</v>
+        <v>22318473</v>
       </c>
       <c r="X38" s="74" t="n">
-        <v>1.161852984755561</v>
+        <v>1.16503277258615</v>
       </c>
       <c r="Y38" s="28" t="n">
         <v>54.50776965078859</v>
@@ -9216,17 +9216,17 @@
       </c>
       <c r="AX38" s="79" t="inlineStr">
         <is>
+          <t>Why Strategy (MSTR) stock is up today</t>
+        </is>
+      </c>
+      <c r="AY38" s="79" t="inlineStr">
+        <is>
           <t>Strategy Soars 7%, Galaxy Up 8% as Crypto Stocks Rally on “Clear, Practical Framework” for Stablecoin Rules</t>
         </is>
       </c>
-      <c r="AY38" s="79" t="inlineStr">
+      <c r="AZ38" s="79" t="inlineStr">
         <is>
           <t>Strategy Increased Its Preferred Stock Buyback to $3 Billion and Shares Moved Higher. What This Means for MSTR</t>
-        </is>
-      </c>
-      <c r="AZ38" s="79" t="inlineStr">
-        <is>
-          <t>What Is Strategy (MSTR)? The Bitcoin Treasury Company</t>
         </is>
       </c>
     </row>
@@ -9322,10 +9322,10 @@
         <v>889.4500122070312</v>
       </c>
       <c r="W39" s="84" t="n">
-        <v>20635155</v>
+        <v>20724431</v>
       </c>
       <c r="X39" s="85" t="n">
-        <v>0.7827903794058977</v>
+        <v>0.7860439427392247</v>
       </c>
       <c r="Y39" s="35" t="n">
         <v>40.45069568571127</v>
@@ -9510,10 +9510,10 @@
         <v>164</v>
       </c>
       <c r="W40" s="73" t="n">
-        <v>19061611</v>
+        <v>19201416</v>
       </c>
       <c r="X40" s="74" t="n">
-        <v>0.9439520358783573</v>
+        <v>0.9505462881706782</v>
       </c>
       <c r="Y40" s="28" t="n">
         <v>33.73814615117286</v>
@@ -9597,12 +9597,12 @@
       </c>
       <c r="AY40" s="79" t="inlineStr">
         <is>
+          <t>Did SpaceX Just Save CoreWeave, Nebius, and the Neocloud Sector?</t>
+        </is>
+      </c>
+      <c r="AZ40" s="79" t="inlineStr">
+        <is>
           <t>Nebius Vs. DigitalOcean: The Cash Positive Neocloud Arguably Looks Better</t>
-        </is>
-      </c>
-      <c r="AZ40" s="79" t="inlineStr">
-        <is>
-          <t>AI Cloud Stocks Rise as Musk Calls Overcapacity Talk ‘Ridiculous’: Nebius and CoreWeave Gain 3%, Oracle Edg...</t>
         </is>
       </c>
     </row>
@@ -9698,10 +9698,10 @@
         <v>64.09999847412109</v>
       </c>
       <c r="W41" s="84" t="n">
-        <v>100741000</v>
+        <v>100931063</v>
       </c>
       <c r="X41" s="85" t="n">
-        <v>2.512714661434765</v>
+        <v>2.516858701715341</v>
       </c>
       <c r="Y41" s="35" t="n">
         <v>32.6116444740277</v>
@@ -9785,12 +9785,12 @@
       </c>
       <c r="AY41" s="90" t="inlineStr">
         <is>
-          <t>Why Netflix (NFLX) shares are falling today</t>
+          <t>Why Netflix Stock Dropped Today</t>
         </is>
       </c>
       <c r="AZ41" s="90" t="inlineStr">
         <is>
-          <t>Netflix Is Down 38% Since Completing Its 10-For-1 Stock Split. Here's Why the Sell-Off Is Worsening After I...</t>
+          <t>Netflix Stock Slammed With Price-Target Cuts After Q3 Report</t>
         </is>
       </c>
     </row>
@@ -9886,10 +9886,10 @@
         <v>9.135000228881836</v>
       </c>
       <c r="W42" s="73" t="n">
-        <v>73164202</v>
+        <v>73320711</v>
       </c>
       <c r="X42" s="74" t="n">
-        <v>1.075252584128057</v>
+        <v>1.077428796744912</v>
       </c>
       <c r="Y42" s="28" t="n">
         <v>40.45494644282233</v>
@@ -10074,10 +10074,10 @@
         <v>217.6600036621094</v>
       </c>
       <c r="W43" s="84" t="n">
-        <v>85740755</v>
+        <v>86111324</v>
       </c>
       <c r="X43" s="85" t="n">
-        <v>0.8297883537418639</v>
+        <v>0.8332252637462366</v>
       </c>
       <c r="Y43" s="35" t="n">
         <v>47.90964628179271</v>
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
-          <t>SpaceX, Tesla, Meta, Nvidia, Intel, Netflix, AT&amp;T, and More Stocks That Explain Today’s Market</t>
+          <t>Crypto Exchanges Want Your Next Stock Trade in 2027</t>
         </is>
       </c>
       <c r="AY43" s="90" t="inlineStr">
         <is>
-          <t>Savvy Investors Love This Often Overlooked Clue. It's Flashing Now For This Nvidia, Google Partner.</t>
+          <t>Everpure (P) stock trades up, here is why</t>
         </is>
       </c>
       <c r="AZ43" s="90" t="inlineStr">
         <is>
-          <t>YYForce Unveils "Workforce OS" Robotics Architecture Powered by NVIDIA Physical AI</t>
+          <t>Why Netflix Stock Dropped Today</t>
         </is>
       </c>
     </row>
@@ -10262,10 +10262,10 @@
         <v>189.8800048828125</v>
       </c>
       <c r="W44" s="73" t="n">
-        <v>21150939</v>
+        <v>21192659</v>
       </c>
       <c r="X44" s="74" t="n">
-        <v>0.9539039955029686</v>
+        <v>0.9556956506956598</v>
       </c>
       <c r="Y44" s="28" t="n">
         <v>59.16439524842366</v>
@@ -10344,17 +10344,17 @@
       </c>
       <c r="AX44" s="79" t="inlineStr">
         <is>
+          <t>Palantir Accelerates Delivery of Sovereign AI to New Wave of Customers</t>
+        </is>
+      </c>
+      <c r="AY44" s="79" t="inlineStr">
+        <is>
           <t>Palantir Rises 4% as Software Stocks Rally; ServiceNow Gains 3%, Salesforce Holds Flat</t>
         </is>
       </c>
-      <c r="AY44" s="79" t="inlineStr">
+      <c r="AZ44" s="79" t="inlineStr">
         <is>
           <t>What Could Surprise Palantir Stock Investors On The Upside?</t>
-        </is>
-      </c>
-      <c r="AZ44" s="79" t="inlineStr">
-        <is>
-          <t>The Zacks Analyst Blog Highlights Microsoft, Palantir Technologies, Micron Technology, Lam Research and IonQ</t>
         </is>
       </c>
     </row>
@@ -10450,10 +10450,10 @@
         <v>174.1000061035156</v>
       </c>
       <c r="W45" s="84" t="n">
-        <v>7112289</v>
+        <v>7164759</v>
       </c>
       <c r="X45" s="85" t="n">
-        <v>0.6873633389934612</v>
+        <v>0.6922587539245036</v>
       </c>
       <c r="Y45" s="35" t="n">
         <v>49.5878535118199</v>
@@ -10566,7 +10566,7 @@
       </c>
       <c r="F46" s="23" t="inlineStr">
         <is>
-          <t>Same</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G46" s="23" t="inlineStr">
@@ -10629,7 +10629,7 @@
         <v>2.769996643066406</v>
       </c>
       <c r="T46" s="72" t="n">
-        <v>52.22000122070312</v>
+        <v>52.20999908447266</v>
       </c>
       <c r="U46" s="72" t="n">
         <v>53.88999938964844</v>
@@ -10638,10 +10638,10 @@
         <v>52.02000045776367</v>
       </c>
       <c r="W46" s="73" t="n">
-        <v>17392971</v>
+        <v>17563720</v>
       </c>
       <c r="X46" s="74" t="n">
-        <v>0.7987547322697502</v>
+        <v>0.8062800873646221</v>
       </c>
       <c r="Y46" s="28" t="n">
         <v>32.78496651219285</v>
@@ -10826,10 +10826,10 @@
         <v>1327.619995117188</v>
       </c>
       <c r="W47" s="84" t="n">
-        <v>6821028</v>
+        <v>6859996</v>
       </c>
       <c r="X47" s="85" t="n">
-        <v>0.8652973838949091</v>
+        <v>0.8700257170113134</v>
       </c>
       <c r="Y47" s="35" t="n">
         <v>37.06977729100647</v>
@@ -11014,10 +11014,10 @@
         <v>380.510009765625</v>
       </c>
       <c r="W48" s="73" t="n">
-        <v>42923520</v>
+        <v>44779790</v>
       </c>
       <c r="X48" s="74" t="n">
-        <v>1.217746858849492</v>
+        <v>1.267073151563131</v>
       </c>
       <c r="Y48" s="28" t="n">
         <v>59.76728652545496</v>
@@ -11096,17 +11096,17 @@
       </c>
       <c r="AX48" s="79" t="inlineStr">
         <is>
-          <t>Full self-driving is a 'differentiator' for Tesla amid declining sales</t>
+          <t>Musk: Optimus will be 'the biggest product on earth,' but ramp-up will take a year</t>
         </is>
       </c>
       <c r="AY48" s="79" t="inlineStr">
         <is>
-          <t>Tesla stock gets boost after beating Q3 earnings expectations</t>
+          <t>S&amp;P 500, Nasdaq Gain, Powered By Meta, Tesla Stock — SPCX, META, TSLA, SKYD, IBM In Focus</t>
         </is>
       </c>
       <c r="AZ48" s="79" t="inlineStr">
         <is>
-          <t>Tesla's Third Quarter Was Just OK. These Numbers Show How.</t>
+          <t>Dow Jones Futures Fall; Meta, Tesla Are Earnings Movers After SpaceX, Super Micro Lead Bullish Nasdaq Move</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 21 Oct 2026, 08:47 PM · Yahoo Finance data</t>
+          <t>Built 21 Oct 2026, 11:24 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 21 Oct 2026, 08:47 PM · Yahoo Finance data</t>
+          <t>Built 21 Oct 2026, 11:24 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 21 Oct 2026, 08:47 PM · Yahoo Finance data</t>
+          <t>Built 21 Oct 2026, 11:24 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 21 Oct 2026, 08:47 PM · Yahoo Finance data</t>
+          <t>Built 21 Oct 2026, 11:24 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-10-21 23:59 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 21 Oct 2026, 11:24 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 21 Oct 2026, 11:59 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 21 Oct 2026, 11:24 PM · Yahoo Finance data</t>
+          <t>Built 21 Oct 2026, 11:59 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -6496,7 +6496,7 @@
         <v>339.2049865722656</v>
       </c>
       <c r="U24" s="72" t="n">
-        <v>345.25</v>
+        <v>345.2200012207031</v>
       </c>
       <c r="V24" s="72" t="n">
         <v>338.8299865722656</v>
@@ -6514,7 +6514,7 @@
         <v>76.28277288773747</v>
       </c>
       <c r="AA24" s="28" t="n">
-        <v>18.17537445124041</v>
+        <v>18.17087497555117</v>
       </c>
       <c r="AB24" s="75" t="n">
         <v>3.853071122280767</v>
@@ -6556,7 +6556,7 @@
         <v>5.275490972590549</v>
       </c>
       <c r="AO24" s="77" t="n">
-        <v>1.881752828124677</v>
+        <v>1.881129911757746</v>
       </c>
       <c r="AP24" s="72" t="n">
         <v>348.1499938964844</v>
@@ -6594,7 +6594,7 @@
       </c>
       <c r="AZ24" s="79" t="inlineStr">
         <is>
-          <t>Apple vs. SK hynix: Which Tech Stock Is a Better Buy in 2026?</t>
+          <t>Dear Apple Stock Fans, Mark Your Calendars for October 28</t>
         </is>
       </c>
     </row>
@@ -6782,7 +6782,7 @@
       </c>
       <c r="AZ25" s="90" t="inlineStr">
         <is>
-          <t>Teradyne, Vishay Intertechnology, Allegro MicroSystems, Entegris, and AMD shares are soaring, what you need...</t>
+          <t>Western Digital, Nova, Amtech, Monolithic Power Systems, and Texas Instruments shares skyrocket, what you n...</t>
         </is>
       </c>
     </row>
@@ -8469,12 +8469,12 @@
       </c>
       <c r="AY34" s="79" t="inlineStr">
         <is>
+          <t>Cathie Wood Trimmed Ark's Alphabet Stake Even as Google Search Revenue Grew, While Ark Piled Into Rocket La...</t>
+        </is>
+      </c>
+      <c r="AZ34" s="79" t="inlineStr">
+        <is>
           <t>Prediction: This Artificial Intelligence (AI) Stock Will Be the Biggest Winner of 2027</t>
-        </is>
-      </c>
-      <c r="AZ34" s="79" t="inlineStr">
-        <is>
-          <t>Kazakhstan’s AIFC Regulator Turns to Apple and Google to Enforce Coinbase, HTX Injunctions</t>
         </is>
       </c>
     </row>
@@ -9780,17 +9780,17 @@
       </c>
       <c r="AX41" s="90" t="inlineStr">
         <is>
-          <t>Is Netflix still making the prestige content subscribers are used to?</t>
+          <t>Netflix does everything but tell members prices are going up</t>
         </is>
       </c>
       <c r="AY41" s="90" t="inlineStr">
         <is>
+          <t>Netflix Stock Hits 26-Month Low, But Revenue Tells a Different Story</t>
+        </is>
+      </c>
+      <c r="AZ41" s="90" t="inlineStr">
+        <is>
           <t>Why Netflix Stock Dropped Today</t>
-        </is>
-      </c>
-      <c r="AZ41" s="90" t="inlineStr">
-        <is>
-          <t>Netflix Stock Slammed With Price-Target Cuts After Q3 Report</t>
         </is>
       </c>
     </row>
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
+          <t>History Says This ETF Is a Millionaire Maker. Here's What You'd Need to Invest Each Month to Get There.</t>
+        </is>
+      </c>
+      <c r="AY43" s="90" t="inlineStr">
+        <is>
           <t>Crypto Exchanges Want Your Next Stock Trade in 2027</t>
         </is>
       </c>
-      <c r="AY43" s="90" t="inlineStr">
-        <is>
-          <t>Everpure (P) stock trades up, here is why</t>
-        </is>
-      </c>
       <c r="AZ43" s="90" t="inlineStr">
         <is>
-          <t>Why Netflix Stock Dropped Today</t>
+          <t>SpaceX shares soar on possible tie-up with Tesla</t>
         </is>
       </c>
     </row>
@@ -10720,17 +10720,17 @@
       </c>
       <c r="AX46" s="79" t="inlineStr">
         <is>
+          <t>Cathie Wood Trimmed Ark's Alphabet Stake Even as Google Search Revenue Grew, While Ark Piled Into Rocket La...</t>
+        </is>
+      </c>
+      <c r="AY46" s="79" t="inlineStr">
+        <is>
           <t>Rocket Lab Just Had the Worst Week in Its History. Here's What I'd Do With the Stock Now.</t>
         </is>
       </c>
-      <c r="AY46" s="79" t="inlineStr">
+      <c r="AZ46" s="79" t="inlineStr">
         <is>
           <t>Rocket Lab Sets Another Spacecraft Milestone As Viasat Advances $81M NASA Program</t>
-        </is>
-      </c>
-      <c r="AZ46" s="79" t="inlineStr">
-        <is>
-          <t>SpaceX Jumps 8% on Q3 Revenue Beat as Musk Backs Tesla Merger Idea; Rocket Lab and AST SpaceMobile Edge Higher</t>
         </is>
       </c>
     </row>
@@ -11096,17 +11096,17 @@
       </c>
       <c r="AX48" s="79" t="inlineStr">
         <is>
-          <t>Musk: Optimus will be 'the biggest product on earth,' but ramp-up will take a year</t>
+          <t>Dow Jones Futures Fall; Meta, Tesla Are Earnings Movers After SpaceX Leads Bullish Nasdaq Move</t>
         </is>
       </c>
       <c r="AY48" s="79" t="inlineStr">
         <is>
-          <t>S&amp;P 500, Nasdaq Gain, Powered By Meta, Tesla Stock — SPCX, META, TSLA, SKYD, IBM In Focus</t>
+          <t>Tesla profits drop on tech spending spree as 'Elon Inc.' talk builds</t>
         </is>
       </c>
       <c r="AZ48" s="79" t="inlineStr">
         <is>
-          <t>Dow Jones Futures Fall; Meta, Tesla Are Earnings Movers After SpaceX, Super Micro Lead Bullish Nasdaq Move</t>
+          <t>SpaceX shares soar on possible tie-up with Tesla</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 21 Oct 2026, 11:24 PM · Yahoo Finance data</t>
+          <t>Built 21 Oct 2026, 11:59 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 21 Oct 2026, 11:24 PM · Yahoo Finance data</t>
+          <t>Built 21 Oct 2026, 11:59 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 21 Oct 2026, 11:24 PM · Yahoo Finance data</t>
+          <t>Built 21 Oct 2026, 11:59 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 21 Oct 2026, 11:24 PM · Yahoo Finance data</t>
+          <t>Built 21 Oct 2026, 11:59 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-10-22 23:26 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 22 Oct 2026, 08:41 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 22 Oct 2026, 11:26 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 22 Oct 2026, 08:41 PM · Yahoo Finance data</t>
+          <t>Built 22 Oct 2026, 11:26 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -3620,10 +3620,10 @@
         <v>164.7799987792969</v>
       </c>
       <c r="W7" s="73" t="n">
-        <v>10643877</v>
+        <v>10754826</v>
       </c>
       <c r="X7" s="74" t="n">
-        <v>1.41330165521724</v>
+        <v>1.426982436076355</v>
       </c>
       <c r="Y7" s="28" t="n">
         <v>40.46087787610487</v>
@@ -3810,10 +3810,10 @@
         <v>178.9499969482422</v>
       </c>
       <c r="W8" s="84" t="n">
-        <v>10064819</v>
+        <v>10108996</v>
       </c>
       <c r="X8" s="85" t="n">
-        <v>1.175651585363135</v>
+        <v>1.180507228971829</v>
       </c>
       <c r="Y8" s="35" t="n">
         <v>69.92181667403219</v>
@@ -4000,10 +4000,10 @@
         <v>55.81999969482422</v>
       </c>
       <c r="W9" s="73" t="n">
-        <v>32269443</v>
+        <v>32567843</v>
       </c>
       <c r="X9" s="74" t="n">
-        <v>0.8871217922943917</v>
+        <v>0.8949580479728818</v>
       </c>
       <c r="Y9" s="28" t="n">
         <v>63.15013993233266</v>
@@ -4080,9 +4080,21 @@
       <c r="AW9" s="26" t="n">
         <v>0.03432537981380901</v>
       </c>
-      <c r="AX9" s="25" t="n"/>
-      <c r="AY9" s="25" t="n"/>
-      <c r="AZ9" s="25" t="n"/>
+      <c r="AX9" s="79" t="inlineStr">
+        <is>
+          <t>Sector Update: Financial Stocks Rise Late Afternoon</t>
+        </is>
+      </c>
+      <c r="AY9" s="79" t="inlineStr">
+        <is>
+          <t>Sector Update: Financial Stocks Rise Wednesday Afternoon</t>
+        </is>
+      </c>
+      <c r="AZ9" s="79" t="inlineStr">
+        <is>
+          <t>Sector Update: Financial Stocks Higher Late Afternoon</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="17" customHeight="1">
       <c r="A10" s="67" t="n">
@@ -4178,10 +4190,10 @@
         <v>66.28500366210938</v>
       </c>
       <c r="W10" s="84" t="n">
-        <v>41473966</v>
+        <v>41617461</v>
       </c>
       <c r="X10" s="85" t="n">
-        <v>1.295101512306271</v>
+        <v>1.299291310268354</v>
       </c>
       <c r="Y10" s="35" t="n">
         <v>63.10743245733454</v>
@@ -4368,10 +4380,10 @@
         <v>87.86000061035156</v>
       </c>
       <c r="W11" s="73" t="n">
-        <v>22480539</v>
+        <v>22888564</v>
       </c>
       <c r="X11" s="74" t="n">
-        <v>1.674417420891511</v>
+        <v>1.702221732834791</v>
       </c>
       <c r="Y11" s="28" t="n">
         <v>74.33677346987844</v>
@@ -4558,10 +4570,10 @@
         <v>114.1699981689453</v>
       </c>
       <c r="W12" s="84" t="n">
-        <v>8035048</v>
+        <v>8039267</v>
       </c>
       <c r="X12" s="85" t="n">
-        <v>1.123390551669407</v>
+        <v>1.123947266772033</v>
       </c>
       <c r="Y12" s="35" t="n">
         <v>59.90408914596446</v>
@@ -4748,10 +4760,10 @@
         <v>106.7350006103516</v>
       </c>
       <c r="W13" s="73" t="n">
-        <v>6097094</v>
+        <v>6109139</v>
       </c>
       <c r="X13" s="74" t="n">
-        <v>0.9340698557968206</v>
+        <v>0.9358287965217555</v>
       </c>
       <c r="Y13" s="28" t="n">
         <v>37.29785787669868</v>
@@ -4938,10 +4950,10 @@
         <v>50.77000045776367</v>
       </c>
       <c r="W14" s="84" t="n">
-        <v>9608125</v>
+        <v>9619352</v>
       </c>
       <c r="X14" s="85" t="n">
-        <v>0.840933167229021</v>
+        <v>0.8418744271783214</v>
       </c>
       <c r="Y14" s="35" t="n">
         <v>64.7408938996829</v>
@@ -5128,10 +5140,10 @@
         <v>181.5099945068359</v>
       </c>
       <c r="W15" s="73" t="n">
-        <v>12021466</v>
+        <v>12099831</v>
       </c>
       <c r="X15" s="74" t="n">
-        <v>1.376050751903432</v>
+        <v>1.38439997759529</v>
       </c>
       <c r="Y15" s="28" t="n">
         <v>36.36346141284269</v>
@@ -5318,10 +5330,10 @@
         <v>41.97999954223633</v>
       </c>
       <c r="W16" s="84" t="n">
-        <v>10743977</v>
+        <v>10764185</v>
       </c>
       <c r="X16" s="85" t="n">
-        <v>1.372159134248492</v>
+        <v>1.374562607144429</v>
       </c>
       <c r="Y16" s="35" t="n">
         <v>55.03589974119432</v>
@@ -5508,10 +5520,10 @@
         <v>42.02000045776367</v>
       </c>
       <c r="W17" s="73" t="n">
-        <v>29867765</v>
+        <v>29955848</v>
       </c>
       <c r="X17" s="74" t="n">
-        <v>0.8141372940582958</v>
+        <v>0.8164402531572872</v>
       </c>
       <c r="Y17" s="28" t="n">
         <v>63.61741267074709</v>
@@ -5717,10 +5729,10 @@
         <v>761.1699829101562</v>
       </c>
       <c r="W19" s="73" t="n">
-        <v>49706495</v>
+        <v>54034474</v>
       </c>
       <c r="X19" s="74" t="n">
-        <v>1.226355230574957</v>
+        <v>1.326055049767035</v>
       </c>
       <c r="Y19" s="28" t="n">
         <v>45.17157701617262</v>
@@ -5905,10 +5917,10 @@
         <v>701.9000244140625</v>
       </c>
       <c r="W20" s="84" t="n">
-        <v>61029418</v>
+        <v>64223209</v>
       </c>
       <c r="X20" s="85" t="n">
-        <v>1.667819225550117</v>
+        <v>1.747473526666943</v>
       </c>
       <c r="Y20" s="35" t="n">
         <v>36.53721153980536</v>
@@ -6093,10 +6105,10 @@
         <v>274.489990234375</v>
       </c>
       <c r="W21" s="73" t="n">
-        <v>25455921</v>
+        <v>25711985</v>
       </c>
       <c r="X21" s="74" t="n">
-        <v>0.9903965532132107</v>
+        <v>0.9998610082726472</v>
       </c>
       <c r="Y21" s="28" t="n">
         <v>44.53950931719528</v>
@@ -6281,10 +6293,10 @@
         <v>80.21499633789062</v>
       </c>
       <c r="W22" s="84" t="n">
-        <v>173872206</v>
+        <v>177999401</v>
       </c>
       <c r="X22" s="85" t="n">
-        <v>2.159889890764436</v>
+        <v>2.205505355024982</v>
       </c>
       <c r="Y22" s="35" t="n">
         <v>29.855198707136</v>
@@ -6490,10 +6502,10 @@
         <v>342.2799987792969</v>
       </c>
       <c r="W24" s="73" t="n">
-        <v>43272015</v>
+        <v>46845411</v>
       </c>
       <c r="X24" s="74" t="n">
-        <v>1.143165325333909</v>
+        <v>1.231753707226329</v>
       </c>
       <c r="Y24" s="28" t="n">
         <v>64.75105176984249</v>
@@ -6582,7 +6594,7 @@
       </c>
       <c r="AZ24" s="79" t="inlineStr">
         <is>
-          <t>What Intel, Boeing, Nike Have In Common With Each Other — And Apple</t>
+          <t>Apple Reportedly Raised Its iPhone Duo Target 44%. Here’s What November 2 Has to Show</t>
         </is>
       </c>
     </row>
@@ -6669,7 +6681,7 @@
         <v>-44.78997802734375</v>
       </c>
       <c r="T25" s="83" t="n">
-        <v>524.094970703125</v>
+        <v>523.6199951171875</v>
       </c>
       <c r="U25" s="83" t="n">
         <v>529.97998046875</v>
@@ -6678,10 +6690,10 @@
         <v>502.6000061035156</v>
       </c>
       <c r="W25" s="84" t="n">
-        <v>27453314</v>
+        <v>27927104</v>
       </c>
       <c r="X25" s="85" t="n">
-        <v>1.401945993989355</v>
+        <v>1.424417637634868</v>
       </c>
       <c r="Y25" s="35" t="n">
         <v>36.50677294120715</v>
@@ -6770,7 +6782,7 @@
       </c>
       <c r="AZ25" s="90" t="inlineStr">
         <is>
-          <t>What Does an AI Agent Need a CPU For? Why Nvidia Wants In on the Business Dominated by AMD and Intel</t>
+          <t>Is nVent Electric (NVT) Undervalued On Its AMD AI Data Center Cooling Deal?</t>
         </is>
       </c>
     </row>
@@ -6866,10 +6878,10 @@
         <v>248.0001068115234</v>
       </c>
       <c r="W26" s="73" t="n">
-        <v>48226452</v>
+        <v>48711738</v>
       </c>
       <c r="X26" s="74" t="n">
-        <v>1.331360261158612</v>
+        <v>1.343857092377891</v>
       </c>
       <c r="Y26" s="28" t="n">
         <v>45.10739450903083</v>
@@ -6948,17 +6960,17 @@
       </c>
       <c r="AX26" s="79" t="inlineStr">
         <is>
+          <t>Amazon (AMZN) Suffers a Larger Drop Than the General Market: Key Insights</t>
+        </is>
+      </c>
+      <c r="AY26" s="79" t="inlineStr">
+        <is>
+          <t>Top Research Reports for Amazon, GE Aerospace &amp; TotalEnergies</t>
+        </is>
+      </c>
+      <c r="AZ26" s="79" t="inlineStr">
+        <is>
           <t>Alphabet (GOOGL) vs. MSFT and AMZN: Can AI Investments and Google Cloud Growth Unlock a 26% Upside?</t>
-        </is>
-      </c>
-      <c r="AY26" s="79" t="inlineStr">
-        <is>
-          <t>TEAMSTERS RALLY FOR DELIVERY PROTECTION ACT AT NEW YORK CITY HALL</t>
-        </is>
-      </c>
-      <c r="AZ26" s="79" t="inlineStr">
-        <is>
-          <t>Famous Billionaire Calls AI a Bubble — But That Is Not What His Money Says</t>
         </is>
       </c>
     </row>
@@ -7054,10 +7066,10 @@
         <v>81.09999847412109</v>
       </c>
       <c r="W27" s="84" t="n">
-        <v>6073049</v>
+        <v>6088141</v>
       </c>
       <c r="X27" s="85" t="n">
-        <v>1.38131915005455</v>
+        <v>1.384514205672531</v>
       </c>
       <c r="Y27" s="35" t="n">
         <v>40.94427621358847</v>
@@ -7242,10 +7254,10 @@
         <v>208.3103942871094</v>
       </c>
       <c r="W28" s="73" t="n">
-        <v>5714646</v>
+        <v>5736237</v>
       </c>
       <c r="X28" s="74" t="n">
-        <v>1.11606173252454</v>
+        <v>1.120042278677558</v>
       </c>
       <c r="Y28" s="28" t="n">
         <v>31.42558811221905</v>
@@ -7421,7 +7433,7 @@
         <v>-2.130001068115234</v>
       </c>
       <c r="T29" s="83" t="n">
-        <v>39.0099983215332</v>
+        <v>39.04000091552734</v>
       </c>
       <c r="U29" s="83" t="n">
         <v>40.43050003051758</v>
@@ -7430,10 +7442,10 @@
         <v>37.79999923706055</v>
       </c>
       <c r="W29" s="84" t="n">
-        <v>17057906</v>
+        <v>17193275</v>
       </c>
       <c r="X29" s="85" t="n">
-        <v>0.9811291045270212</v>
+        <v>0.9885303593570631</v>
       </c>
       <c r="Y29" s="35" t="n">
         <v>28.51472314558129</v>
@@ -7512,17 +7524,17 @@
       </c>
       <c r="AX29" s="90" t="inlineStr">
         <is>
+          <t>AST SpaceMobile, Inc. (ASTS) Falls More Steeply Than Broader Market: What Investors Need to Know</t>
+        </is>
+      </c>
+      <c r="AY29" s="90" t="inlineStr">
+        <is>
           <t>SpaceX and AST SpaceMobile Sink 6%, Rocket Lab Falls 5% as Tech Selloff Hits High-Flying Space Stocks</t>
         </is>
       </c>
-      <c r="AY29" s="90" t="inlineStr">
+      <c r="AZ29" s="90" t="inlineStr">
         <is>
           <t>Should You Sell Your AST SpaceMobile Stock Now?</t>
-        </is>
-      </c>
-      <c r="AZ29" s="90" t="inlineStr">
-        <is>
-          <t>AST SpaceMobile Hit a 52-Week Low Days After SpaceX Spent $8 Billion on Spectrum. That's Not a Coincidence.</t>
         </is>
       </c>
     </row>
@@ -7618,10 +7630,10 @@
         <v>321.0199890136719</v>
       </c>
       <c r="W30" s="73" t="n">
-        <v>27624434</v>
+        <v>28083824</v>
       </c>
       <c r="X30" s="74" t="n">
-        <v>1.274542687366931</v>
+        <v>1.294366398561288</v>
       </c>
       <c r="Y30" s="28" t="n">
         <v>34.78406532127708</v>
@@ -7705,12 +7717,12 @@
       </c>
       <c r="AY30" s="79" t="inlineStr">
         <is>
+          <t>Broadcom Inc. (AVGO) Suffers a Larger Drop Than the General Market: Key Insights</t>
+        </is>
+      </c>
+      <c r="AZ30" s="79" t="inlineStr">
+        <is>
           <t>Prediction: Broadcom Stock Could Crush the S&amp;P 500 Through 2030</t>
-        </is>
-      </c>
-      <c r="AZ30" s="79" t="inlineStr">
-        <is>
-          <t>Broadcom Has Lost 35% From Its High: Tigress Sees 83% Upside</t>
         </is>
       </c>
     </row>
@@ -7806,10 +7818,10 @@
         <v>78.27010345458984</v>
       </c>
       <c r="W31" s="84" t="n">
-        <v>4020573</v>
+        <v>4051654</v>
       </c>
       <c r="X31" s="85" t="n">
-        <v>1.234031904048725</v>
+        <v>1.242978695114943</v>
       </c>
       <c r="Y31" s="35" t="n">
         <v>33.75774981879118</v>
@@ -7994,10 +8006,10 @@
         <v>54.84999847412109</v>
       </c>
       <c r="W32" s="73" t="n">
-        <v>80066905</v>
+        <v>81234057</v>
       </c>
       <c r="X32" s="74" t="n">
-        <v>1.583629002399621</v>
+        <v>1.604861490572769</v>
       </c>
       <c r="Y32" s="28" t="n">
         <v>26.5566319771587</v>
@@ -8076,17 +8088,17 @@
       </c>
       <c r="AX32" s="79" t="inlineStr">
         <is>
+          <t>Stock Market Today, Oct. 22: CoreWeave Slides on Bernstein Downgrade and Financing Worries</t>
+        </is>
+      </c>
+      <c r="AY32" s="79" t="inlineStr">
+        <is>
+          <t>CoreWeave and Nebius Stocks Are Crashing. Time to Buy the Dip?</t>
+        </is>
+      </c>
+      <c r="AZ32" s="79" t="inlineStr">
+        <is>
           <t>CoreWeave Sinks 10% as Bernstein Slashes Target to $51: “The Fundamentals Are Probably Stuck”</t>
-        </is>
-      </c>
-      <c r="AY32" s="79" t="inlineStr">
-        <is>
-          <t>Companies Are Spending Billions To Build Data Centers. The Timeline For Them To Pay Off is Fuzzy.</t>
-        </is>
-      </c>
-      <c r="AZ32" s="79" t="inlineStr">
-        <is>
-          <t>CoreWeave capacity expansion to drive revenue growth, Bank of America says</t>
         </is>
       </c>
     </row>
@@ -8182,10 +8194,10 @@
         <v>446.9100036621094</v>
       </c>
       <c r="W33" s="84" t="n">
-        <v>6505768</v>
+        <v>6597846</v>
       </c>
       <c r="X33" s="85" t="n">
-        <v>0.9595034968999527</v>
+        <v>0.9724233433446541</v>
       </c>
       <c r="Y33" s="35" t="n">
         <v>36.99820650479885</v>
@@ -8264,17 +8276,17 @@
       </c>
       <c r="AX33" s="90" t="inlineStr">
         <is>
+          <t>Here's Why Dell Technologies (DELL) Fell More Than Broader Market</t>
+        </is>
+      </c>
+      <c r="AY33" s="90" t="inlineStr">
+        <is>
           <t>Dell Unveiled New AI Servers a Week After Barclays’ Downgrade. Here’s Where the Stock Could Go by 2031</t>
         </is>
       </c>
-      <c r="AY33" s="90" t="inlineStr">
+      <c r="AZ33" s="90" t="inlineStr">
         <is>
           <t>Are You Sure You Understand Dell Stock's Risk?</t>
-        </is>
-      </c>
-      <c r="AZ33" s="90" t="inlineStr">
-        <is>
-          <t>Apple Stock Could Have Another Major Growth Chapter Ahead</t>
         </is>
       </c>
     </row>
@@ -8370,10 +8382,10 @@
         <v>318.4500122070312</v>
       </c>
       <c r="W34" s="73" t="n">
-        <v>20957461</v>
+        <v>21055559</v>
       </c>
       <c r="X34" s="74" t="n">
-        <v>1.331532133230809</v>
+        <v>1.337348027460377</v>
       </c>
       <c r="Y34" s="28" t="n">
         <v>32.79420199742401</v>
@@ -8558,10 +8570,10 @@
         <v>24.86000061035156</v>
       </c>
       <c r="W35" s="84" t="n">
-        <v>65333028</v>
+        <v>66176624</v>
       </c>
       <c r="X35" s="85" t="n">
-        <v>1.283171177448194</v>
+        <v>1.298663943381078</v>
       </c>
       <c r="Y35" s="35" t="n">
         <v>25.12028993897121</v>
@@ -8746,10 +8758,10 @@
         <v>84.64499664306641</v>
       </c>
       <c r="W36" s="73" t="n">
-        <v>132334821</v>
+        <v>133529950</v>
       </c>
       <c r="X36" s="74" t="n">
-        <v>1.333427709397113</v>
+        <v>1.344660386899913</v>
       </c>
       <c r="Y36" s="28" t="n">
         <v>30.47020187170551</v>
@@ -8934,10 +8946,10 @@
         <v>520.2999877929688</v>
       </c>
       <c r="W37" s="84" t="n">
-        <v>21006593</v>
+        <v>21246740</v>
       </c>
       <c r="X37" s="85" t="n">
-        <v>0.9812111886222662</v>
+        <v>0.9918720767670858</v>
       </c>
       <c r="Y37" s="35" t="n">
         <v>50.50135119208441</v>
@@ -9016,17 +9028,17 @@
       </c>
       <c r="AX37" s="90" t="inlineStr">
         <is>
+          <t>Microsoft (MSFT) Falls More Steeply Than Broader Market: What Investors Need to Know</t>
+        </is>
+      </c>
+      <c r="AY37" s="90" t="inlineStr">
+        <is>
           <t>How much MSFT stock does Microsoft CEO Satya Nadella actually own?</t>
         </is>
       </c>
-      <c r="AY37" s="90" t="inlineStr">
+      <c r="AZ37" s="90" t="inlineStr">
         <is>
           <t>Microsoft, Google parent and McDonald’s protest new trading plan</t>
-        </is>
-      </c>
-      <c r="AZ37" s="90" t="inlineStr">
-        <is>
-          <t>Waymo, Google and Microsoft Alums Raise $30M to Build the Data Layer for Physical AI</t>
         </is>
       </c>
     </row>
@@ -9122,10 +9134,10 @@
         <v>143.4199981689453</v>
       </c>
       <c r="W38" s="73" t="n">
-        <v>20348310</v>
+        <v>20549884</v>
       </c>
       <c r="X38" s="74" t="n">
-        <v>1.052087272794582</v>
+        <v>1.061956043536041</v>
       </c>
       <c r="Y38" s="28" t="n">
         <v>49.36667274802698</v>
@@ -9204,17 +9216,17 @@
       </c>
       <c r="AX38" s="79" t="inlineStr">
         <is>
+          <t>Strategy (MSTR) Suffers a Larger Drop Than the General Market: Key Insights</t>
+        </is>
+      </c>
+      <c r="AY38" s="79" t="inlineStr">
+        <is>
           <t>Strategy (MSTR) Reports Next Week: Wall Street Expects Earnings Growth</t>
         </is>
       </c>
-      <c r="AY38" s="79" t="inlineStr">
+      <c r="AZ38" s="79" t="inlineStr">
         <is>
           <t>How Did Strategy Stock Leave Its Industry Behind?</t>
-        </is>
-      </c>
-      <c r="AZ38" s="79" t="inlineStr">
-        <is>
-          <t>Why Strategy (MSTR) stock is up today</t>
         </is>
       </c>
     </row>
@@ -9310,10 +9322,10 @@
         <v>849.25</v>
       </c>
       <c r="W39" s="84" t="n">
-        <v>30671226</v>
+        <v>31922936</v>
       </c>
       <c r="X39" s="85" t="n">
-        <v>1.143975718726421</v>
+        <v>1.187889104883893</v>
       </c>
       <c r="Y39" s="35" t="n">
         <v>34.65493049177566</v>
@@ -9392,17 +9404,17 @@
       </c>
       <c r="AX39" s="90" t="inlineStr">
         <is>
-          <t>Chip stocks fall as equipment maker Lam Research cites 'supply chain constraints'</t>
+          <t>Meta and chip stocks decline as AI trade comes under pressure: AlphaCheck</t>
         </is>
       </c>
       <c r="AY39" s="90" t="inlineStr">
         <is>
-          <t>Meta and chip stocks decline as AI trade comes under pressure: AlphaCheck</t>
+          <t>Why Micron Stock Dropped on Thursday</t>
         </is>
       </c>
       <c r="AZ39" s="90" t="inlineStr">
         <is>
-          <t>Micron Says Its Next AI Chips Need Even More Wafers. Here’s What That Means for the Stock</t>
+          <t>Micron (MU) Falls More Steeply Than Broader Market: What Investors Need to Know</t>
         </is>
       </c>
     </row>
@@ -9498,10 +9510,10 @@
         <v>155.7299957275391</v>
       </c>
       <c r="W40" s="73" t="n">
-        <v>25620100</v>
+        <v>26035828</v>
       </c>
       <c r="X40" s="74" t="n">
-        <v>1.262740718251214</v>
+        <v>1.28191742396273</v>
       </c>
       <c r="Y40" s="28" t="n">
         <v>30.34554991789557</v>
@@ -9686,10 +9698,10 @@
         <v>65.01999664306641</v>
       </c>
       <c r="W41" s="84" t="n">
-        <v>58334128</v>
+        <v>58691592</v>
       </c>
       <c r="X41" s="85" t="n">
-        <v>1.401231258104641</v>
+        <v>1.409212807418014</v>
       </c>
       <c r="Y41" s="35" t="n">
         <v>39.59251464499781</v>
@@ -9773,12 +9785,12 @@
       </c>
       <c r="AY41" s="90" t="inlineStr">
         <is>
+          <t>Stock Market Today, Oct. 22: Netflix Rises as Investors Capitalize on Post-Earnings Sell-Off</t>
+        </is>
+      </c>
+      <c r="AZ41" s="90" t="inlineStr">
+        <is>
           <t>Netflix CFO Eyes Double-Digit Revenue Growth Into 2027 Despite ‘Modest’ Viewership Gains, Points to 3 Key D...</t>
-        </is>
-      </c>
-      <c r="AZ41" s="90" t="inlineStr">
-        <is>
-          <t>The Truth About Netflix’s Massive Stock Buybacks</t>
         </is>
       </c>
     </row>
@@ -9874,10 +9886,10 @@
         <v>7.78000020980835</v>
       </c>
       <c r="W42" s="73" t="n">
-        <v>205214659</v>
+        <v>206826972</v>
       </c>
       <c r="X42" s="74" t="n">
-        <v>2.75225512067445</v>
+        <v>2.77088296883138</v>
       </c>
       <c r="Y42" s="28" t="n">
         <v>29.30548177405909</v>
@@ -9956,17 +9968,17 @@
       </c>
       <c r="AX42" s="79" t="inlineStr">
         <is>
+          <t>Nokia (NOK) Q3 2026 Earnings Call Transcript</t>
+        </is>
+      </c>
+      <c r="AY42" s="79" t="inlineStr">
+        <is>
           <t>Why Nokia Sank today</t>
         </is>
       </c>
-      <c r="AY42" s="79" t="inlineStr">
+      <c r="AZ42" s="79" t="inlineStr">
         <is>
           <t>What Is Nokia (HLSE:NOKIA) Building With Its New Push Into Agentic AI?</t>
-        </is>
-      </c>
-      <c r="AZ42" s="79" t="inlineStr">
-        <is>
-          <t>ICEYE and Nokia partner with the Ministry of Defence of Ukraine to develop sovereign satcom capability</t>
         </is>
       </c>
     </row>
@@ -10062,10 +10074,10 @@
         <v>211.2599945068359</v>
       </c>
       <c r="W43" s="84" t="n">
-        <v>121609814</v>
+        <v>124963035</v>
       </c>
       <c r="X43" s="85" t="n">
-        <v>1.151578581191599</v>
+        <v>1.181456005493145</v>
       </c>
       <c r="Y43" s="35" t="n">
         <v>39.0595901326795</v>
@@ -10144,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
-          <t>Is Nvidia a Top Quantum Computing Stock?</t>
+          <t>Nvidia CEO's new plan could dramatically reshape the AI race</t>
         </is>
       </c>
       <c r="AY43" s="90" t="inlineStr">
         <is>
-          <t>CrowdStrike Stock Rose 5% as It Expanded Its NVIDIA AI Security Deal. Here’s Where the Stock Could Go by 2031</t>
+          <t>FirstService Corporation Q3 2026 Earnings Call Summary</t>
         </is>
       </c>
       <c r="AZ43" s="90" t="inlineStr">
         <is>
-          <t>Oracle Is Down More Than a Third in 2026 Even as TD Cowen Flags Possible Nvidia Support. Here’s Where the S...</t>
+          <t>Valero Energy Corporation Q3 2026 Earnings Call Summary</t>
         </is>
       </c>
     </row>
@@ -10250,10 +10262,10 @@
         <v>194.5350036621094</v>
       </c>
       <c r="W44" s="73" t="n">
-        <v>22521314</v>
+        <v>22880756</v>
       </c>
       <c r="X44" s="74" t="n">
-        <v>1.015494784243779</v>
+        <v>1.030866781009203</v>
       </c>
       <c r="Y44" s="28" t="n">
         <v>53.98063449223372</v>
@@ -10332,17 +10344,17 @@
       </c>
       <c r="AX44" s="79" t="inlineStr">
         <is>
+          <t>Palantir Technologies Inc. (PLTR) Declines More Than Market: Some Information for Investors</t>
+        </is>
+      </c>
+      <c r="AY44" s="79" t="inlineStr">
+        <is>
           <t>All Eyes Will Be on Palantir on Nov. 2. Here's What It Must Say to Keep the Run Going.</t>
         </is>
       </c>
-      <c r="AY44" s="79" t="inlineStr">
+      <c r="AZ44" s="79" t="inlineStr">
         <is>
           <t>What Palantir Technologies Holders Got Right</t>
-        </is>
-      </c>
-      <c r="AZ44" s="79" t="inlineStr">
-        <is>
-          <t>Palantir Just Gained 7% in a Month: Take Profits, or Buy More?</t>
         </is>
       </c>
     </row>
@@ -10438,10 +10450,10 @@
         <v>171.9299926757812</v>
       </c>
       <c r="W45" s="84" t="n">
-        <v>14755157</v>
+        <v>15067396</v>
       </c>
       <c r="X45" s="85" t="n">
-        <v>1.387426878362656</v>
+        <v>1.41470991866519</v>
       </c>
       <c r="Y45" s="35" t="n">
         <v>44.48768101031819</v>
@@ -10525,12 +10537,12 @@
       </c>
       <c r="AY45" s="90" t="inlineStr">
         <is>
+          <t>Intel vs. Qualcomm: A Widening Gap in Revenue</t>
+        </is>
+      </c>
+      <c r="AZ45" s="90" t="inlineStr">
+        <is>
           <t>Qualcomm Schedules Fourth Quarter and Fiscal 2026 Earnings Release and Conference Call</t>
-        </is>
-      </c>
-      <c r="AZ45" s="90" t="inlineStr">
-        <is>
-          <t>Qualcomm (QCOM) Stock Stays Near Fair Value On Tokenized Trading Objections</t>
         </is>
       </c>
     </row>
@@ -10617,7 +10629,7 @@
         <v>-2.449996948242188</v>
       </c>
       <c r="T46" s="72" t="n">
-        <v>51.67499923706055</v>
+        <v>51.65000152587891</v>
       </c>
       <c r="U46" s="72" t="n">
         <v>52.97999954223633</v>
@@ -10626,10 +10638,10 @@
         <v>49.95500183105469</v>
       </c>
       <c r="W46" s="73" t="n">
-        <v>16513972</v>
+        <v>16609383</v>
       </c>
       <c r="X46" s="74" t="n">
-        <v>0.7731693361326661</v>
+        <v>0.7774627449218277</v>
       </c>
       <c r="Y46" s="28" t="n">
         <v>30.2214931054304</v>
@@ -10811,22 +10823,22 @@
         <v>1355</v>
       </c>
       <c r="V47" s="83" t="n">
-        <v>1244.609985351562</v>
+        <v>1244.599975585938</v>
       </c>
       <c r="W47" s="84" t="n">
-        <v>10115257</v>
+        <v>10345622</v>
       </c>
       <c r="X47" s="85" t="n">
-        <v>1.26690881858043</v>
+        <v>1.293894805810573</v>
       </c>
       <c r="Y47" s="35" t="n">
         <v>31.34063475112502</v>
       </c>
       <c r="Z47" s="35" t="n">
-        <v>3.27298160952238</v>
+        <v>3.274923320486705</v>
       </c>
       <c r="AA47" s="35" t="n">
-        <v>23.04829741362535</v>
+        <v>23.04836578405428</v>
       </c>
       <c r="AB47" s="86" t="n">
         <v>-89.87584662132895</v>
@@ -10868,7 +10880,7 @@
         <v>44.01613516137082</v>
       </c>
       <c r="AO47" s="88" t="n">
-        <v>7.777332300908771</v>
+        <v>7.777389003757341</v>
       </c>
       <c r="AP47" s="83" t="n">
         <v>2354.389892578125</v>
@@ -10896,17 +10908,17 @@
       </c>
       <c r="AX47" s="90" t="inlineStr">
         <is>
+          <t>Up 3,700%, Should You Buy Sandisk Right Now?</t>
+        </is>
+      </c>
+      <c r="AY47" s="90" t="inlineStr">
+        <is>
           <t>Why Does SanDisk Stock's High Cash Yield Get So Little Credit?</t>
         </is>
       </c>
-      <c r="AY47" s="90" t="inlineStr">
+      <c r="AZ47" s="90" t="inlineStr">
         <is>
           <t>Prediction: Sandisk Stock Will Soar After Oct. 29. Here Are 379 Billion Reasons Why</t>
-        </is>
-      </c>
-      <c r="AZ47" s="90" t="inlineStr">
-        <is>
-          <t>History Says This Will Happen to Sandisk Stock Heading Into Its Oct. 29 Report</t>
         </is>
       </c>
     </row>
@@ -11002,10 +11014,10 @@
         <v>373.7099914550781</v>
       </c>
       <c r="W48" s="73" t="n">
-        <v>51045424</v>
+        <v>51511993</v>
       </c>
       <c r="X48" s="74" t="n">
-        <v>1.387484294879189</v>
+        <v>1.399278995539313</v>
       </c>
       <c r="Y48" s="28" t="n">
         <v>52.80430327769546</v>
@@ -11084,17 +11096,17 @@
       </c>
       <c r="AX48" s="79" t="inlineStr">
         <is>
-          <t>This level-headed Tesla bull still expects 5 million Cybercabs by 2040</t>
+          <t>TSLA, SPCX Boards Confirm Special Committees On Potential Combination As Megapack Deals And Terafab Plans D...</t>
         </is>
       </c>
       <c r="AY48" s="79" t="inlineStr">
         <is>
-          <t>Global markets retreat as tech mood sours, oil prices jump</t>
+          <t>Musk wants to merge SpaceX and Tesla: Here's what to know</t>
         </is>
       </c>
       <c r="AZ48" s="79" t="inlineStr">
         <is>
-          <t>US Equity Markets End Lower After Meta, Tesla Fail to Meet Expectations, Higher Crude Oil Prices</t>
+          <t>Tesla, SpaceX, Meta, Lockheed Martin, Lam Research, Spotify, and More Stocks That Explain Today’s Market</t>
         </is>
       </c>
     </row>
@@ -11366,117 +11378,120 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX8" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY8" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX10" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ10" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX11" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY11" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ11" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX12" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY12" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ12" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX13" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY13" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ13" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX14" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY14" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ14" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX15" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY15" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ15" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX16" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY16" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ16" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX17" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY17" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ17" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX19" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY19" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ19" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX20" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY20" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ20" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX21" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY21" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ21" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX22" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY22" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ22" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX24" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY24" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ24" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX25" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY25" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ25" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX26" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY26" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ26" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX27" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY27" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ27" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX28" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY28" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ28" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX29" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY29" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ29" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX30" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY30" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ30" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX31" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY31" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ31" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX32" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY32" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ32" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX33" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY33" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ33" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX34" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY34" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ34" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX35" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY35" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ35" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX36" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY36" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ36" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX37" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY37" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ37" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX38" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY38" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ38" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX39" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY39" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ39" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX40" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY40" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ40" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX41" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY41" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ41" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX42" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY42" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ42" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX43" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY43" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ43" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX44" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY44" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ44" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX45" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY45" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ45" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX46" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY46" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ46" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX47" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY47" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ47" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX48" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY48" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ48" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY9" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ9" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX10" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY10" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ10" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX11" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY11" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ11" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX12" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY12" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ12" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX13" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY13" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ13" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX14" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY14" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX15" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY15" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ15" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX16" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY16" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ16" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX17" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY17" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ17" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX19" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY19" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ19" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX20" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY20" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ20" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX21" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY21" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ21" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX22" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY22" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ22" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX24" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY24" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ24" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX25" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY25" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ25" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX26" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY26" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ26" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX27" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY27" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ27" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX28" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY28" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ28" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX29" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY29" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ29" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX30" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY30" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ30" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX31" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY31" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ31" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX32" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY32" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ32" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX33" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY33" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ33" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX34" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY34" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ34" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX35" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY35" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ35" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX36" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY36" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ36" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX37" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY37" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ37" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX38" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY38" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ38" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX39" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY39" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ39" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX40" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY40" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ40" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX41" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY41" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ41" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX42" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY42" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ42" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX43" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY43" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ43" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX44" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY44" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ44" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX45" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY45" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ45" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX46" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY46" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ46" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX47" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY47" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ47" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AX48" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AY48" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AZ48" r:id="rId121"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11628,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 22 Oct 2026, 08:41 PM · Yahoo Finance data</t>
+          <t>Built 22 Oct 2026, 11:26 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19564,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 22 Oct 2026, 08:41 PM · Yahoo Finance data</t>
+          <t>Built 22 Oct 2026, 11:26 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27500,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 22 Oct 2026, 08:41 PM · Yahoo Finance data</t>
+          <t>Built 22 Oct 2026, 11:26 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35436,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 22 Oct 2026, 08:41 PM · Yahoo Finance data</t>
+          <t>Built 22 Oct 2026, 11:26 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -44681,7 +44696,7 @@
       </c>
       <c r="D33" s="105" t="inlineStr">
         <is>
-          <t>Gapped down 5.2% at the open</t>
+          <t>Gapped down 5.3% at the open</t>
         </is>
       </c>
       <c r="E33" s="33" t="n">
@@ -44849,7 +44864,7 @@
       </c>
       <c r="D39" s="105" t="inlineStr">
         <is>
-          <t>Gapped down 4.6% at the open</t>
+          <t>Gapped down 4.5% at the open</t>
         </is>
       </c>
       <c r="E39" s="33" t="n">
@@ -45381,7 +45396,7 @@
       </c>
       <c r="D58" s="107" t="inlineStr">
         <is>
-          <t>Gapped down 3.7% at the open</t>
+          <t>Gapped down 3.8% at the open</t>
         </is>
       </c>
       <c r="E58" s="26" t="n">

</xml_diff>

<commit_message>
Daily workbook: 2026-10-22 23:58 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 22 Oct 2026, 11:26 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 22 Oct 2026, 11:58 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 22 Oct 2026, 11:26 PM · Yahoo Finance data</t>
+          <t>Built 22 Oct 2026, 11:58 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 22 Oct 2026, 11:26 PM · Yahoo Finance data</t>
+          <t>Built 22 Oct 2026, 11:58 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 22 Oct 2026, 11:26 PM · Yahoo Finance data</t>
+          <t>Built 22 Oct 2026, 11:58 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 22 Oct 2026, 11:26 PM · Yahoo Finance data</t>
+          <t>Built 22 Oct 2026, 11:58 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 22 Oct 2026, 11:26 PM · Yahoo Finance data</t>
+          <t>Built 22 Oct 2026, 11:58 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-10-23 23:11 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -28,7 +28,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'10-20'!$5:$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'10-19'!$A$6:$AZ$48</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'10-19'!$5:$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Signals'!$B$5:$G$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Signals'!$B$5:$G$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -639,10 +639,10 @@
     <xf numFmtId="0" fontId="26" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="27" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 23 Oct 2026, 08:33 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 23 Oct 2026, 11:11 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -1404,7 +1404,7 @@
       <c r="P8" s="10" t="n"/>
       <c r="Q8" s="16" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="R8" s="12" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 23 Oct 2026, 08:33 PM · Yahoo Finance data</t>
+          <t>Built 23 Oct 2026, 11:11 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -3620,10 +3620,10 @@
         <v>162.9799957275391</v>
       </c>
       <c r="W7" s="73" t="n">
-        <v>7166526</v>
+        <v>7194295</v>
       </c>
       <c r="X7" s="74" t="n">
-        <v>0.9516728432995776</v>
+        <v>0.9551842894692495</v>
       </c>
       <c r="Y7" s="28" t="n">
         <v>35.14715001151464</v>
@@ -3810,10 +3810,10 @@
         <v>178.7100067138672</v>
       </c>
       <c r="W8" s="84" t="n">
-        <v>7688904</v>
+        <v>7704286</v>
       </c>
       <c r="X8" s="85" t="n">
-        <v>0.8890869338990013</v>
+        <v>0.89078637225605</v>
       </c>
       <c r="Y8" s="35" t="n">
         <v>64.00568608101659</v>
@@ -4000,10 +4000,10 @@
         <v>55.80500030517578</v>
       </c>
       <c r="W9" s="73" t="n">
-        <v>27556699</v>
+        <v>28504792</v>
       </c>
       <c r="X9" s="74" t="n">
-        <v>0.7588496443483019</v>
+        <v>0.7839346356169045</v>
       </c>
       <c r="Y9" s="28" t="n">
         <v>55.0538096737313</v>
@@ -4190,10 +4190,10 @@
         <v>67.76000213623047</v>
       </c>
       <c r="W10" s="84" t="n">
-        <v>38523494</v>
+        <v>38613173</v>
       </c>
       <c r="X10" s="85" t="n">
-        <v>1.200890934119784</v>
+        <v>1.203518267747853</v>
       </c>
       <c r="Y10" s="35" t="n">
         <v>69.39043172969249</v>
@@ -4380,10 +4380,10 @@
         <v>88.05999755859375</v>
       </c>
       <c r="W11" s="73" t="n">
-        <v>19688877</v>
+        <v>19689981</v>
       </c>
       <c r="X11" s="74" t="n">
-        <v>1.40609186087865</v>
+        <v>1.406165160342029</v>
       </c>
       <c r="Y11" s="28" t="n">
         <v>63.88471318191526</v>
@@ -4570,10 +4570,10 @@
         <v>112.8300018310547</v>
       </c>
       <c r="W12" s="84" t="n">
-        <v>6405861</v>
+        <v>6409956</v>
       </c>
       <c r="X12" s="85" t="n">
-        <v>0.8938533696055534</v>
+        <v>0.894399219687835</v>
       </c>
       <c r="Y12" s="35" t="n">
         <v>50.96261580288863</v>
@@ -4760,10 +4760,10 @@
         <v>105.5</v>
       </c>
       <c r="W13" s="73" t="n">
-        <v>5397841</v>
+        <v>5398530</v>
       </c>
       <c r="X13" s="74" t="n">
-        <v>0.8243046246233626</v>
+        <v>0.824405504771668</v>
       </c>
       <c r="Y13" s="28" t="n">
         <v>32.83410143665397</v>
@@ -4950,10 +4950,10 @@
         <v>50.83000183105469</v>
       </c>
       <c r="W14" s="84" t="n">
-        <v>8257465</v>
+        <v>8257885</v>
       </c>
       <c r="X14" s="85" t="n">
-        <v>0.728280485883106</v>
+        <v>0.7283161795271467</v>
       </c>
       <c r="Y14" s="35" t="n">
         <v>59.48575008043654</v>
@@ -5140,10 +5140,10 @@
         <v>181.5500030517578</v>
       </c>
       <c r="W15" s="73" t="n">
-        <v>7414569</v>
+        <v>7417778</v>
       </c>
       <c r="X15" s="74" t="n">
-        <v>0.8414642103645716</v>
+        <v>0.8418130644922439</v>
       </c>
       <c r="Y15" s="28" t="n">
         <v>38.10643965213546</v>
@@ -5330,10 +5330,10 @@
         <v>42.35499954223633</v>
       </c>
       <c r="W16" s="84" t="n">
-        <v>9526100</v>
+        <v>9526215</v>
       </c>
       <c r="X16" s="85" t="n">
-        <v>1.188061886823514</v>
+        <v>1.188075377228959</v>
       </c>
       <c r="Y16" s="35" t="n">
         <v>55.52866282616257</v>
@@ -5520,10 +5520,10 @@
         <v>42.38999938964844</v>
       </c>
       <c r="W17" s="73" t="n">
-        <v>18638126</v>
+        <v>18664387</v>
       </c>
       <c r="X17" s="74" t="n">
-        <v>0.5161673799248687</v>
+        <v>0.5168758608687153</v>
       </c>
       <c r="Y17" s="28" t="n">
         <v>59.85666904585845</v>
@@ -5729,10 +5729,10 @@
         <v>758.6799926757812</v>
       </c>
       <c r="W19" s="73" t="n">
-        <v>32468269</v>
+        <v>33133505</v>
       </c>
       <c r="X19" s="74" t="n">
-        <v>0.8008452917632164</v>
+        <v>0.816583713918213</v>
       </c>
       <c r="Y19" s="28" t="n">
         <v>42.09364045667231</v>
@@ -5917,10 +5917,10 @@
         <v>701.1599731445312</v>
       </c>
       <c r="W20" s="84" t="n">
-        <v>29201166</v>
+        <v>29960981</v>
       </c>
       <c r="X20" s="85" t="n">
-        <v>0.7953597341020291</v>
+        <v>0.8152114609765236</v>
       </c>
       <c r="Y20" s="35" t="n">
         <v>36.50995768802219</v>
@@ -6105,10 +6105,10 @@
         <v>273.3450012207031</v>
       </c>
       <c r="W21" s="73" t="n">
-        <v>20143343</v>
+        <v>20640183</v>
       </c>
       <c r="X21" s="74" t="n">
-        <v>0.7870202007899595</v>
+        <v>0.8056502624801092</v>
       </c>
       <c r="Y21" s="28" t="n">
         <v>43.06645901820595</v>
@@ -6293,10 +6293,10 @@
         <v>80.83000183105469</v>
       </c>
       <c r="W22" s="84" t="n">
-        <v>90727443</v>
+        <v>91390844</v>
       </c>
       <c r="X22" s="85" t="n">
-        <v>1.098967799168225</v>
+        <v>1.106558877744477</v>
       </c>
       <c r="Y22" s="35" t="n">
         <v>30.85201440463865</v>
@@ -6502,10 +6502,10 @@
         <v>345.75</v>
       </c>
       <c r="W24" s="73" t="n">
-        <v>39323315</v>
+        <v>39450857</v>
       </c>
       <c r="X24" s="74" t="n">
-        <v>1.021379744722434</v>
+        <v>1.024522807477374</v>
       </c>
       <c r="Y24" s="28" t="n">
         <v>63.91009221240459</v>
@@ -6584,7 +6584,7 @@
       </c>
       <c r="AX24" s="79" t="inlineStr">
         <is>
-          <t>Apple is taking Wall Street's top spot back from Nvidia — for the fifth time</t>
+          <t>Elon Musk's $1B Skydance Investment</t>
         </is>
       </c>
       <c r="AY24" s="79" t="inlineStr">
@@ -6594,7 +6594,7 @@
       </c>
       <c r="AZ24" s="79" t="inlineStr">
         <is>
-          <t>Apple is catching up to Nvidia's market cap, and investors are waiting on Anthropic's IPO</t>
+          <t>S&amp;P 500, Dow Drop As Elevated Oil Prices Stoke Inflation Fears Ahead Of Fed Meeting Next Week — AAPL, AXP, ...</t>
         </is>
       </c>
     </row>
@@ -6690,10 +6690,10 @@
         <v>508.3570861816406</v>
       </c>
       <c r="W25" s="84" t="n">
-        <v>15049021</v>
+        <v>15094156</v>
       </c>
       <c r="X25" s="85" t="n">
-        <v>0.7725036594351762</v>
+        <v>0.7747308028192519</v>
       </c>
       <c r="Y25" s="35" t="n">
         <v>38.97605722226721</v>
@@ -6772,17 +6772,17 @@
       </c>
       <c r="AX25" s="90" t="inlineStr">
         <is>
+          <t>AMD Stock Fell 8% in a Day as Lam Research’s Supply Warning Sank Chip Stocks. Here’s Where the Stock Could ...</t>
+        </is>
+      </c>
+      <c r="AY25" s="90" t="inlineStr">
+        <is>
           <t>TER vs. AMD: Which AI Component Supplier Stock Is the Better Buy?</t>
         </is>
       </c>
-      <c r="AY25" s="90" t="inlineStr">
+      <c r="AZ25" s="90" t="inlineStr">
         <is>
           <t>AMD or Broadcom: If I Could Only Own 1 AI Chip Stock Through 2030, Here's My Pick</t>
-        </is>
-      </c>
-      <c r="AZ25" s="90" t="inlineStr">
-        <is>
-          <t>AMD Stock Price Prediction: One Growth Opportunity Could Push Shares Much Higher</t>
         </is>
       </c>
     </row>
@@ -6878,10 +6878,10 @@
         <v>246.4515991210938</v>
       </c>
       <c r="W26" s="73" t="n">
-        <v>25336345</v>
+        <v>25470108</v>
       </c>
       <c r="X26" s="74" t="n">
-        <v>0.7075918021428114</v>
+        <v>0.7111946851761387</v>
       </c>
       <c r="Y26" s="28" t="n">
         <v>43.16913130836262</v>
@@ -6960,17 +6960,17 @@
       </c>
       <c r="AX26" s="79" t="inlineStr">
         <is>
+          <t>Dow Jones Futures: Microsoft, Google, Amazon Lead Earnings Wave; What To Do Amid Mixed Signals</t>
+        </is>
+      </c>
+      <c r="AY26" s="79" t="inlineStr">
+        <is>
           <t>Amazon Survived a 50% Crash. Here’s What a $1,000 Investment Became</t>
         </is>
       </c>
-      <c r="AY26" s="79" t="inlineStr">
+      <c r="AZ26" s="79" t="inlineStr">
         <is>
           <t>Amazon CEO Andy Jassy Says AI Inference Is Still 10 Times Too Expensive, Claims Amazon Chips Offer Answer</t>
-        </is>
-      </c>
-      <c r="AZ26" s="79" t="inlineStr">
-        <is>
-          <t>Prediction: Amazon Could Double by 2030 if This Part of Its Business Delivers</t>
         </is>
       </c>
     </row>
@@ -7066,10 +7066,10 @@
         <v>80.69999694824219</v>
       </c>
       <c r="W27" s="84" t="n">
-        <v>4894644</v>
+        <v>4901940</v>
       </c>
       <c r="X27" s="85" t="n">
-        <v>1.101664789461386</v>
+        <v>1.10321635840972</v>
       </c>
       <c r="Y27" s="35" t="n">
         <v>41.27607497698394</v>
@@ -7254,10 +7254,10 @@
         <v>208.5</v>
       </c>
       <c r="W28" s="73" t="n">
-        <v>2404782</v>
+        <v>2426422</v>
       </c>
       <c r="X28" s="74" t="n">
-        <v>0.4915212461383214</v>
+        <v>0.4958346608295048</v>
       </c>
       <c r="Y28" s="28" t="n">
         <v>31.54735618940262</v>
@@ -7433,7 +7433,7 @@
         <v>1.020000457763672</v>
       </c>
       <c r="T29" s="83" t="n">
-        <v>38.16999816894531</v>
+        <v>38.18999862670898</v>
       </c>
       <c r="U29" s="83" t="n">
         <v>40.15480041503906</v>
@@ -7442,10 +7442,10 @@
         <v>36.72000122070312</v>
       </c>
       <c r="W29" s="84" t="n">
-        <v>12883276</v>
+        <v>12901765</v>
       </c>
       <c r="X29" s="85" t="n">
-        <v>0.7270464069710806</v>
+        <v>0.7280518208306999</v>
       </c>
       <c r="Y29" s="35" t="n">
         <v>30.88181938202571</v>
@@ -7524,17 +7524,17 @@
       </c>
       <c r="AX29" s="90" t="inlineStr">
         <is>
+          <t>Why the Market Dipped But AST SpaceMobile, Inc. (ASTS) Gained Today</t>
+        </is>
+      </c>
+      <c r="AY29" s="90" t="inlineStr">
+        <is>
           <t>T-REX ETFs to Delist and Liquidate</t>
         </is>
       </c>
-      <c r="AY29" s="90" t="inlineStr">
+      <c r="AZ29" s="90" t="inlineStr">
         <is>
           <t>Stocktwits Space Race Weekly: RKLB, VSAT Beat SPCX With Modest Gains — ASTS And PL Sink Deeper</t>
-        </is>
-      </c>
-      <c r="AZ29" s="90" t="inlineStr">
-        <is>
-          <t>ASTS Slips Overnight: Retail Sees Upside In SpaceX’s 80,000-Site Push — FCC Adviser Sees Global Satellite P...</t>
         </is>
       </c>
     </row>
@@ -7630,10 +7630,10 @@
         <v>320.2300109863281</v>
       </c>
       <c r="W30" s="73" t="n">
-        <v>15680021</v>
+        <v>15826189</v>
       </c>
       <c r="X30" s="74" t="n">
-        <v>0.7235500346095713</v>
+        <v>0.7300487101493958</v>
       </c>
       <c r="Y30" s="28" t="n">
         <v>34.18241684792784</v>
@@ -7712,17 +7712,17 @@
       </c>
       <c r="AX30" s="79" t="inlineStr">
         <is>
+          <t>Prediction: Nvidia Will Outperform Broadcom Over the Next 5 Years</t>
+        </is>
+      </c>
+      <c r="AY30" s="79" t="inlineStr">
+        <is>
           <t>AMD or Broadcom: If I Could Only Own 1 AI Chip Stock Through 2030, Here's My Pick</t>
         </is>
       </c>
-      <c r="AY30" s="79" t="inlineStr">
+      <c r="AZ30" s="79" t="inlineStr">
         <is>
           <t>Same Playbook, Different Silicon: Broadcom Holds the Throne, Marvell Plays the AMD Challenger.</t>
-        </is>
-      </c>
-      <c r="AZ30" s="79" t="inlineStr">
-        <is>
-          <t>The Best Trillion-Dollar Stock To Sell Puts On Isn’t Tesla Or Broadcom</t>
         </is>
       </c>
     </row>
@@ -7818,10 +7818,10 @@
         <v>76.91999816894531</v>
       </c>
       <c r="W31" s="84" t="n">
-        <v>3103175</v>
+        <v>3103439</v>
       </c>
       <c r="X31" s="85" t="n">
-        <v>0.9358529771331355</v>
+        <v>0.9359288682491599</v>
       </c>
       <c r="Y31" s="35" t="n">
         <v>33.29477792719914</v>
@@ -8006,10 +8006,10 @@
         <v>54.0099983215332</v>
       </c>
       <c r="W32" s="73" t="n">
-        <v>45984246</v>
+        <v>46371125</v>
       </c>
       <c r="X32" s="74" t="n">
-        <v>0.8883205029783489</v>
+        <v>0.8954595850025938</v>
       </c>
       <c r="Y32" s="28" t="n">
         <v>25.75250463595559</v>
@@ -8093,12 +8093,12 @@
       </c>
       <c r="AY32" s="79" t="inlineStr">
         <is>
+          <t>CoreWeave appears to have a lender problem, not a customer one</t>
+        </is>
+      </c>
+      <c r="AZ32" s="79" t="inlineStr">
+        <is>
           <t>CoreWeave Heads for Third Weekly Loss, Weighing on Stocks and Bitcoin Over AI Financing Fears</t>
-        </is>
-      </c>
-      <c r="AZ32" s="79" t="inlineStr">
-        <is>
-          <t>CoreWeave Is Down 13% in a Week. Here's the Price at Which I'd Buy</t>
         </is>
       </c>
     </row>
@@ -8194,10 +8194,10 @@
         <v>449.7200927734375</v>
       </c>
       <c r="W33" s="84" t="n">
-        <v>4315923</v>
+        <v>4325290</v>
       </c>
       <c r="X33" s="85" t="n">
-        <v>0.6574259154714476</v>
+        <v>0.658805749792909</v>
       </c>
       <c r="Y33" s="35" t="n">
         <v>37.90682360461656</v>
@@ -8382,10 +8382,10 @@
         <v>316.9898986816406</v>
       </c>
       <c r="W34" s="73" t="n">
-        <v>10726436</v>
+        <v>10793024</v>
       </c>
       <c r="X34" s="74" t="n">
-        <v>0.6880517757223531</v>
+        <v>0.6921752662117598</v>
       </c>
       <c r="Y34" s="28" t="n">
         <v>30.85936519959294</v>
@@ -8464,17 +8464,17 @@
       </c>
       <c r="AX34" s="79" t="inlineStr">
         <is>
-          <t>Alphabet (GOOGL): Investing Behind AI Demand and TPU Growth</t>
+          <t>Eric Schmidt Rejects AI Bubble Fears, Says Anthropic Is Growing Twice as Fast as Google Did</t>
         </is>
       </c>
       <c r="AY34" s="79" t="inlineStr">
         <is>
-          <t>Apple and Alphabet are sending Wall Street different signals</t>
+          <t>Dow Jones Futures: Microsoft, Google, Amazon Lead Earnings Wave; What To Do Amid Mixed Signals</t>
         </is>
       </c>
       <c r="AZ34" s="79" t="inlineStr">
         <is>
-          <t>Hyperscalers Microsoft, Amazon Line Up With Earnings, Along With ServiceNow, Intel</t>
+          <t>Meta and Google About to Run the Old Playbook Again, Will “Sell Space Inside Their Models.”</t>
         </is>
       </c>
     </row>
@@ -8570,10 +8570,10 @@
         <v>24.8799991607666</v>
       </c>
       <c r="W35" s="84" t="n">
-        <v>38271117</v>
+        <v>38502015</v>
       </c>
       <c r="X35" s="85" t="n">
-        <v>0.7527560030423555</v>
+        <v>0.757125618407136</v>
       </c>
       <c r="Y35" s="35" t="n">
         <v>24.37278513044269</v>
@@ -8758,10 +8758,10 @@
         <v>84.73999786376953</v>
       </c>
       <c r="W36" s="73" t="n">
-        <v>71475768</v>
+        <v>71684828</v>
       </c>
       <c r="X36" s="74" t="n">
-        <v>0.7291873988051029</v>
+        <v>0.731242224520629</v>
       </c>
       <c r="Y36" s="28" t="n">
         <v>32.79200070565426</v>
@@ -8946,10 +8946,10 @@
         <v>515.7000122070312</v>
       </c>
       <c r="W37" s="84" t="n">
-        <v>13305533</v>
+        <v>13629072</v>
       </c>
       <c r="X37" s="85" t="n">
-        <v>0.6594255130203656</v>
+        <v>0.6749190807049503</v>
       </c>
       <c r="Y37" s="35" t="n">
         <v>52.61062363689017</v>
@@ -9033,12 +9033,12 @@
       </c>
       <c r="AY37" s="90" t="inlineStr">
         <is>
+          <t>Dow Jones Futures: Microsoft, Google, Amazon Lead Earnings Wave; What To Do Amid Mixed Signals</t>
+        </is>
+      </c>
+      <c r="AZ37" s="90" t="inlineStr">
+        <is>
           <t>Microsoft Earnings Report To Focus On AI Momentum, Capex</t>
-        </is>
-      </c>
-      <c r="AZ37" s="90" t="inlineStr">
-        <is>
-          <t>Sector Update: Tech Stocks Rise Late Afternoon</t>
         </is>
       </c>
     </row>
@@ -9134,10 +9134,10 @@
         <v>144.2050018310547</v>
       </c>
       <c r="W38" s="73" t="n">
-        <v>18332609</v>
+        <v>18365943</v>
       </c>
       <c r="X38" s="74" t="n">
-        <v>0.947731909827876</v>
+        <v>0.9493733608497387</v>
       </c>
       <c r="Y38" s="28" t="n">
         <v>49.50690724170995</v>
@@ -9322,10 +9322,10 @@
         <v>858.3400268554688</v>
       </c>
       <c r="W39" s="84" t="n">
-        <v>21056819</v>
+        <v>21123737</v>
       </c>
       <c r="X39" s="85" t="n">
-        <v>0.7830210570459022</v>
+        <v>0.7854117550360735</v>
       </c>
       <c r="Y39" s="35" t="n">
         <v>38.16884392635592</v>
@@ -9404,17 +9404,17 @@
       </c>
       <c r="AX39" s="90" t="inlineStr">
         <is>
+          <t>What Could Micron Technology (MU) Strike Risk And Supply Moves Mean For Investors?</t>
+        </is>
+      </c>
+      <c r="AY39" s="90" t="inlineStr">
+        <is>
           <t>Micron Stock Leads Chip Rebound. Dip Buyers Buckle Up.</t>
         </is>
       </c>
-      <c r="AY39" s="90" t="inlineStr">
+      <c r="AZ39" s="90" t="inlineStr">
         <is>
           <t>Micron, Sandisk gain as SK Hynix scraps Solidigm IPO, LYNX says</t>
-        </is>
-      </c>
-      <c r="AZ39" s="90" t="inlineStr">
-        <is>
-          <t>As the U.S. Pulls Chip Making Back Home, the Toolmakers Win First</t>
         </is>
       </c>
     </row>
@@ -9510,10 +9510,10 @@
         <v>155.8578033447266</v>
       </c>
       <c r="W40" s="73" t="n">
-        <v>13328081</v>
+        <v>13396970</v>
       </c>
       <c r="X40" s="74" t="n">
-        <v>0.6522716375479697</v>
+        <v>0.6555325379517466</v>
       </c>
       <c r="Y40" s="28" t="n">
         <v>30.23202220364797</v>
@@ -9698,10 +9698,10 @@
         <v>65.77999877929688</v>
       </c>
       <c r="W41" s="84" t="n">
-        <v>35460039</v>
+        <v>35672753</v>
       </c>
       <c r="X41" s="85" t="n">
-        <v>0.8390088387792213</v>
+        <v>0.8438294499281183</v>
       </c>
       <c r="Y41" s="35" t="n">
         <v>37.12018753285766</v>
@@ -9886,10 +9886,10 @@
         <v>8.038100242614746</v>
       </c>
       <c r="W42" s="73" t="n">
-        <v>84390159</v>
+        <v>84521485</v>
       </c>
       <c r="X42" s="74" t="n">
-        <v>1.101726632477473</v>
+        <v>1.103346530452715</v>
       </c>
       <c r="Y42" s="28" t="n">
         <v>33.07518734981166</v>
@@ -9968,17 +9968,17 @@
       </c>
       <c r="AX42" s="79" t="inlineStr">
         <is>
+          <t>Nokia says robots will drive the next wave of connectivity</t>
+        </is>
+      </c>
+      <c r="AY42" s="79" t="inlineStr">
+        <is>
           <t>Hop-on's Digitalage Targets Enterprise Licensing for AI-Assisted Moderation Technology</t>
         </is>
       </c>
-      <c r="AY42" s="79" t="inlineStr">
+      <c r="AZ42" s="79" t="inlineStr">
         <is>
           <t>Nokia: 3 Key Takeaways for Long-Term Investors</t>
-        </is>
-      </c>
-      <c r="AZ42" s="79" t="inlineStr">
-        <is>
-          <t>Nokia (HLSE:NOKIA) Stock Price Questions Q3 Earnings Margin Gains</t>
         </is>
       </c>
     </row>
@@ -10074,10 +10074,10 @@
         <v>210.1799926757812</v>
       </c>
       <c r="W43" s="84" t="n">
-        <v>77270084</v>
+        <v>79740563</v>
       </c>
       <c r="X43" s="85" t="n">
-        <v>0.7347948725679645</v>
+        <v>0.7573980606908288</v>
       </c>
       <c r="Y43" s="35" t="n">
         <v>38.08914843709527</v>
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
-          <t>Is Elon Musk Coming for Verizon?</t>
+          <t>Neoclouds secure record funds as Nvidia’s Huang says more investment required</t>
         </is>
       </c>
       <c r="AY43" s="90" t="inlineStr">
         <is>
-          <t>2 Growth Stocks to Hold for the Next Decade (Hint: These Aren’t AI Stocks)</t>
+          <t>Prediction: Nvidia Will Outperform Broadcom Over the Next 5 Years</t>
         </is>
       </c>
       <c r="AZ43" s="90" t="inlineStr">
         <is>
-          <t>Not Starlink. Not Starship. Not Grok. $561 Million of SpaceX's $4.4 Billion Profit Came From an Unexpected ...</t>
+          <t>Flagstar Financial, Inc. Q3 2026 Earnings Call Summary</t>
         </is>
       </c>
     </row>
@@ -10262,10 +10262,10 @@
         <v>190.5702056884766</v>
       </c>
       <c r="W44" s="73" t="n">
-        <v>15988368</v>
+        <v>16072134</v>
       </c>
       <c r="X44" s="74" t="n">
-        <v>0.723214928115276</v>
+        <v>0.7268662772618881</v>
       </c>
       <c r="Y44" s="28" t="n">
         <v>54.41618743019004</v>
@@ -10344,17 +10344,17 @@
       </c>
       <c r="AX44" s="79" t="inlineStr">
         <is>
+          <t>Palantir Ruled Out a NATO “Kill Switch.” Here’s Why Its Q3 Expense Line Is the Real Test</t>
+        </is>
+      </c>
+      <c r="AY44" s="79" t="inlineStr">
+        <is>
           <t>Palantir Investors Have One Big Number to Watch in 2027</t>
         </is>
       </c>
-      <c r="AY44" s="79" t="inlineStr">
+      <c r="AZ44" s="79" t="inlineStr">
         <is>
           <t>Palantir Guided for $2.16 Billion in Revenue for Q3. Its Last 2 Quarters Suggest We Should Expect More.</t>
-        </is>
-      </c>
-      <c r="AZ44" s="79" t="inlineStr">
-        <is>
-          <t>Palantir Stock Price Prediction: Is $212 in Reach by Year-End?</t>
         </is>
       </c>
     </row>
@@ -10450,10 +10450,10 @@
         <v>171.4750061035156</v>
       </c>
       <c r="W45" s="84" t="n">
-        <v>7081402</v>
+        <v>7220548</v>
       </c>
       <c r="X45" s="85" t="n">
-        <v>0.7001500802823174</v>
+        <v>0.7134169332604847</v>
       </c>
       <c r="Y45" s="35" t="n">
         <v>47.94911125931755</v>
@@ -10638,10 +10638,10 @@
         <v>49.52199935913086</v>
       </c>
       <c r="W46" s="73" t="n">
-        <v>13324490</v>
+        <v>13364187</v>
       </c>
       <c r="X46" s="74" t="n">
-        <v>0.6317908109633485</v>
+        <v>0.6336134429916498</v>
       </c>
       <c r="Y46" s="28" t="n">
         <v>33.38121001460085</v>
@@ -10826,10 +10826,10 @@
         <v>1228.890014648438</v>
       </c>
       <c r="W47" s="84" t="n">
-        <v>7817941</v>
+        <v>7855877</v>
       </c>
       <c r="X47" s="85" t="n">
-        <v>0.9744426796750221</v>
+        <v>0.9789396515689134</v>
       </c>
       <c r="Y47" s="35" t="n">
         <v>30.35424393432389</v>
@@ -11014,10 +11014,10 @@
         <v>365.2699890136719</v>
       </c>
       <c r="W48" s="73" t="n">
-        <v>34409377</v>
+        <v>34615357</v>
       </c>
       <c r="X48" s="74" t="n">
-        <v>0.949520735632447</v>
+        <v>0.954933326485508</v>
       </c>
       <c r="Y48" s="28" t="n">
         <v>51.52129291158901</v>
@@ -11101,12 +11101,12 @@
       </c>
       <c r="AY48" s="79" t="inlineStr">
         <is>
-          <t>SpaceX earnings, tech sell-off lead to rocky week for investors</t>
+          <t>Tesla Stock Lags Apple Because Of ‘Communications Problem,’ Says Investor Gary Black</t>
         </is>
       </c>
       <c r="AZ48" s="79" t="inlineStr">
         <is>
-          <t>SpaceX CEO Elon Musk is 'one of one': Will the market give Anthropic's Dario Amodei the same leeway?</t>
+          <t>Musk: Optimus and Cybercab “Will Be the Vast Majority of Tesla’s Value” as Earnings Loom</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 23 Oct 2026, 08:33 PM · Yahoo Finance data</t>
+          <t>Built 23 Oct 2026, 11:11 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 23 Oct 2026, 08:33 PM · Yahoo Finance data</t>
+          <t>Built 23 Oct 2026, 11:11 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 23 Oct 2026, 08:33 PM · Yahoo Finance data</t>
+          <t>Built 23 Oct 2026, 11:11 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 23 Oct 2026, 08:33 PM · Yahoo Finance data</t>
+          <t>Built 23 Oct 2026, 11:11 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -43864,7 +43864,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:G22"/>
+  <dimension ref="B2:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -44154,21 +44154,21 @@
     <row r="14">
       <c r="B14" s="24" t="inlineStr">
         <is>
-          <t>ASTS</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="C14" s="101" t="inlineStr">
         <is>
-          <t>AST SpaceMobile, Inc.</t>
+          <t>Amazon.com, Inc.</t>
         </is>
       </c>
       <c r="D14" s="104" t="inlineStr">
         <is>
-          <t>Gapped down 1.5% at the open</t>
+          <t>MACD crossed down</t>
         </is>
       </c>
       <c r="E14" s="26" t="n">
-        <v>0.02630901330204694</v>
+        <v>-0.00950557087785997</v>
       </c>
       <c r="F14" s="27" t="n">
         <v>1</v>
@@ -44192,7 +44192,7 @@
       </c>
       <c r="D15" s="105" t="inlineStr">
         <is>
-          <t>MACD crossed down</t>
+          <t>8 EMA crossed below 21</t>
         </is>
       </c>
       <c r="E15" s="33" t="n">
@@ -44210,24 +44210,24 @@
     <row r="16">
       <c r="B16" s="24" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="C16" s="101" t="inlineStr">
         <is>
-          <t>Amazon.com, Inc.</t>
+          <t>Alphabet Inc.</t>
         </is>
       </c>
       <c r="D16" s="104" t="inlineStr">
         <is>
-          <t>8 EMA crossed below 21</t>
+          <t>Closed below lower band</t>
         </is>
       </c>
       <c r="E16" s="26" t="n">
-        <v>-0.00950557087785997</v>
+        <v>-0.01084926699207589</v>
       </c>
       <c r="F16" s="27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G16" s="23" t="inlineStr">
         <is>
@@ -44238,21 +44238,21 @@
     <row r="17">
       <c r="B17" s="31" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>XLI</t>
         </is>
       </c>
       <c r="C17" s="102" t="inlineStr">
         <is>
-          <t>Alphabet Inc.</t>
+          <t>State Street Industrial Select Sector SPDR ETF</t>
         </is>
       </c>
       <c r="D17" s="105" t="inlineStr">
         <is>
-          <t>Closed below lower band</t>
+          <t>MACD crossed down</t>
         </is>
       </c>
       <c r="E17" s="33" t="n">
-        <v>-0.01084926699207589</v>
+        <v>-0.01265519501241763</v>
       </c>
       <c r="F17" s="34" t="n">
         <v>0</v>
@@ -44276,7 +44276,7 @@
       </c>
       <c r="D18" s="104" t="inlineStr">
         <is>
-          <t>MACD crossed down</t>
+          <t>Closed below lower band</t>
         </is>
       </c>
       <c r="E18" s="26" t="n">
@@ -44294,12 +44294,12 @@
     <row r="19">
       <c r="B19" s="31" t="inlineStr">
         <is>
-          <t>XLI</t>
+          <t>XLC</t>
         </is>
       </c>
       <c r="C19" s="102" t="inlineStr">
         <is>
-          <t>State Street Industrial Select Sector SPDR ETF</t>
+          <t>State Street Communication Services Select Sector SPDR ETF</t>
         </is>
       </c>
       <c r="D19" s="105" t="inlineStr">
@@ -44308,7 +44308,7 @@
         </is>
       </c>
       <c r="E19" s="33" t="n">
-        <v>-0.01265519501241763</v>
+        <v>-0.01778063736056756</v>
       </c>
       <c r="F19" s="34" t="n">
         <v>0</v>
@@ -44322,21 +44322,21 @@
     <row r="20">
       <c r="B20" s="24" t="inlineStr">
         <is>
-          <t>XLC</t>
+          <t>IREN</t>
         </is>
       </c>
       <c r="C20" s="101" t="inlineStr">
         <is>
-          <t>State Street Communication Services Select Sector SPDR ETF</t>
-        </is>
-      </c>
-      <c r="D20" s="104" t="inlineStr">
-        <is>
-          <t>Closed below lower band</t>
+          <t>IREN Limited</t>
+        </is>
+      </c>
+      <c r="D20" s="106" t="inlineStr">
+        <is>
+          <t>RSI oversold (24)</t>
         </is>
       </c>
       <c r="E20" s="26" t="n">
-        <v>-0.01778063736056756</v>
+        <v>-0.02371617157225114</v>
       </c>
       <c r="F20" s="27" t="n">
         <v>0</v>
@@ -44350,21 +44350,21 @@
     <row r="21">
       <c r="B21" s="31" t="inlineStr">
         <is>
-          <t>IREN</t>
+          <t>CRWV</t>
         </is>
       </c>
       <c r="C21" s="102" t="inlineStr">
         <is>
-          <t>IREN Limited</t>
-        </is>
-      </c>
-      <c r="D21" s="106" t="inlineStr">
-        <is>
-          <t>RSI oversold (24)</t>
+          <t>CoreWeave, Inc.</t>
+        </is>
+      </c>
+      <c r="D21" s="107" t="inlineStr">
+        <is>
+          <t>RSI oversold (26)</t>
         </is>
       </c>
       <c r="E21" s="33" t="n">
-        <v>-0.02371617157225114</v>
+        <v>-0.02455032196457463</v>
       </c>
       <c r="F21" s="34" t="n">
         <v>0</v>
@@ -44375,40 +44375,12 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="B22" s="24" t="inlineStr">
-        <is>
-          <t>CRWV</t>
-        </is>
-      </c>
-      <c r="C22" s="101" t="inlineStr">
-        <is>
-          <t>CoreWeave, Inc.</t>
-        </is>
-      </c>
-      <c r="D22" s="107" t="inlineStr">
-        <is>
-          <t>RSI oversold (26)</t>
-        </is>
-      </c>
-      <c r="E22" s="26" t="n">
-        <v>-0.02455032196457463</v>
-      </c>
-      <c r="F22" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G22" s="23" t="inlineStr">
-        <is>
-          <t>Very Weak</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="B5:G22"/>
+  <autoFilter ref="B5:G21"/>
   <mergeCells count="1">
     <mergeCell ref="B2:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="E6:E22">
+  <conditionalFormatting sqref="E6:E21">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="-0.05"/>

</xml_diff>

<commit_message>
Daily workbook: 2026-10-23 23:51 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 23 Oct 2026, 11:11 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 23 Oct 2026, 11:51 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 23 Oct 2026, 11:11 PM · Yahoo Finance data</t>
+          <t>Built 23 Oct 2026, 11:51 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -7524,17 +7524,17 @@
       </c>
       <c r="AX29" s="90" t="inlineStr">
         <is>
+          <t>SpaceX’s 80,000 Cell Site Push A Win For ASTS, Ericsson, Nokia, NextNav, Among Others, Says Roth Capital</t>
+        </is>
+      </c>
+      <c r="AY29" s="90" t="inlineStr">
+        <is>
           <t>Why the Market Dipped But AST SpaceMobile, Inc. (ASTS) Gained Today</t>
         </is>
       </c>
-      <c r="AY29" s="90" t="inlineStr">
+      <c r="AZ29" s="90" t="inlineStr">
         <is>
           <t>T-REX ETFs to Delist and Liquidate</t>
-        </is>
-      </c>
-      <c r="AZ29" s="90" t="inlineStr">
-        <is>
-          <t>Stocktwits Space Race Weekly: RKLB, VSAT Beat SPCX With Modest Gains — ASTS And PL Sink Deeper</t>
         </is>
       </c>
     </row>
@@ -8093,12 +8093,12 @@
       </c>
       <c r="AY32" s="79" t="inlineStr">
         <is>
+          <t>A Surprising New Rival Is Threatening CoreWeave (and It's Not Best Known as an AI Cloud Company)</t>
+        </is>
+      </c>
+      <c r="AZ32" s="79" t="inlineStr">
+        <is>
           <t>CoreWeave appears to have a lender problem, not a customer one</t>
-        </is>
-      </c>
-      <c r="AZ32" s="79" t="inlineStr">
-        <is>
-          <t>CoreWeave Heads for Third Weekly Loss, Weighing on Stocks and Bitcoin Over AI Financing Fears</t>
         </is>
       </c>
     </row>
@@ -8464,12 +8464,12 @@
       </c>
       <c r="AX34" s="79" t="inlineStr">
         <is>
+          <t>Dow Jones Futures: Microsoft, Google, Amazon Lead Earnings Wave; What To Do Amid Mixed Signals</t>
+        </is>
+      </c>
+      <c r="AY34" s="79" t="inlineStr">
+        <is>
           <t>Eric Schmidt Rejects AI Bubble Fears, Says Anthropic Is Growing Twice as Fast as Google Did</t>
-        </is>
-      </c>
-      <c r="AY34" s="79" t="inlineStr">
-        <is>
-          <t>Dow Jones Futures: Microsoft, Google, Amazon Lead Earnings Wave; What To Do Amid Mixed Signals</t>
         </is>
       </c>
       <c r="AZ34" s="79" t="inlineStr">
@@ -9968,17 +9968,17 @@
       </c>
       <c r="AX42" s="79" t="inlineStr">
         <is>
+          <t>SpaceX’s 80,000 Cell Site Push A Win For ASTS, Ericsson, Nokia, NextNav, Among Others, Says Roth Capital</t>
+        </is>
+      </c>
+      <c r="AY42" s="79" t="inlineStr">
+        <is>
           <t>Nokia says robots will drive the next wave of connectivity</t>
         </is>
       </c>
-      <c r="AY42" s="79" t="inlineStr">
+      <c r="AZ42" s="79" t="inlineStr">
         <is>
           <t>Hop-on's Digitalage Targets Enterprise Licensing for AI-Assisted Moderation Technology</t>
-        </is>
-      </c>
-      <c r="AZ42" s="79" t="inlineStr">
-        <is>
-          <t>Nokia: 3 Key Takeaways for Long-Term Investors</t>
         </is>
       </c>
     </row>
@@ -10537,12 +10537,12 @@
       </c>
       <c r="AY45" s="90" t="inlineStr">
         <is>
+          <t>Qualcomm May Be Preparing Another Round of Job Cuts Next Month. Here’s What to Know.</t>
+        </is>
+      </c>
+      <c r="AZ45" s="90" t="inlineStr">
+        <is>
           <t>1 large-cap stock to keep an eye on and 2 we brush off</t>
-        </is>
-      </c>
-      <c r="AZ45" s="90" t="inlineStr">
-        <is>
-          <t>Prediction: This Chip Stock Could Be a Sleeper AI Winner</t>
         </is>
       </c>
     </row>
@@ -10720,17 +10720,17 @@
       </c>
       <c r="AX46" s="79" t="inlineStr">
         <is>
+          <t>Rocket Lab And 2 Top Space Stocks To Watch</t>
+        </is>
+      </c>
+      <c r="AY46" s="79" t="inlineStr">
+        <is>
           <t>Rocket Lab (RKLB) Launched 3 Satellites On An Electron Mission Today</t>
         </is>
       </c>
-      <c r="AY46" s="79" t="inlineStr">
+      <c r="AZ46" s="79" t="inlineStr">
         <is>
           <t>MISSION SUCCESS: Rocket Lab Launches 98th Electron Mission</t>
-        </is>
-      </c>
-      <c r="AZ46" s="79" t="inlineStr">
-        <is>
-          <t>Stocktwits Space Race Weekly: RKLB, VSAT Beat SPCX With Modest Gains — ASTS And PL Sink Deeper</t>
         </is>
       </c>
     </row>
@@ -11008,7 +11008,7 @@
         <v>373.135009765625</v>
       </c>
       <c r="U48" s="72" t="n">
-        <v>377.2999877929688</v>
+        <v>377.2799987792969</v>
       </c>
       <c r="V48" s="72" t="n">
         <v>365.2699890136719</v>
@@ -11068,7 +11068,7 @@
         <v>11.0235077986613</v>
       </c>
       <c r="AO48" s="77" t="n">
-        <v>3.378529308916724</v>
+        <v>3.378145722143803</v>
       </c>
       <c r="AP48" s="72" t="n">
         <v>498.8299865722656</v>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 23 Oct 2026, 11:11 PM · Yahoo Finance data</t>
+          <t>Built 23 Oct 2026, 11:51 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 23 Oct 2026, 11:11 PM · Yahoo Finance data</t>
+          <t>Built 23 Oct 2026, 11:51 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 23 Oct 2026, 11:11 PM · Yahoo Finance data</t>
+          <t>Built 23 Oct 2026, 11:51 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 23 Oct 2026, 11:11 PM · Yahoo Finance data</t>
+          <t>Built 23 Oct 2026, 11:51 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-10-26 23:55 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 26 Oct 2026, 09:45 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 26 Oct 2026, 11:55 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 26 Oct 2026, 09:45 PM · Yahoo Finance data</t>
+          <t>Built 26 Oct 2026, 11:55 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -4564,7 +4564,7 @@
         <v>113.9599990844727</v>
       </c>
       <c r="U12" s="83" t="n">
-        <v>115.3899993896484</v>
+        <v>115.4000015258789</v>
       </c>
       <c r="V12" s="83" t="n">
         <v>113.8399963378906</v>
@@ -4582,7 +4582,7 @@
         <v>65.24823942233033</v>
       </c>
       <c r="AA12" s="35" t="n">
-        <v>16.56838841623103</v>
+        <v>16.57378685930248</v>
       </c>
       <c r="AB12" s="86" t="n">
         <v>0.5753904693836489</v>
@@ -4624,7 +4624,7 @@
         <v>7.285289523187875</v>
       </c>
       <c r="AO12" s="88" t="n">
-        <v>1.440599351390147</v>
+        <v>1.441224625579556</v>
       </c>
       <c r="AP12" s="83" t="n">
         <v>125.0100021362305</v>
@@ -5811,17 +5811,17 @@
       </c>
       <c r="AX19" s="79" t="inlineStr">
         <is>
+          <t>S&amp;P 500, Nasdaq, Dow Begin Week Higher As Anthropic IPO Filing Rekindles AI Enthusiasm — MSFT, AAPL, CART, ...</t>
+        </is>
+      </c>
+      <c r="AY19" s="79" t="inlineStr">
+        <is>
           <t>Exchange-Traded Funds, Equity Futures Higher Pre-Bell Monday Ahead of Big Tech Earnings, Fed Decision</t>
         </is>
       </c>
-      <c r="AY19" s="79" t="inlineStr">
+      <c r="AZ19" s="79" t="inlineStr">
         <is>
           <t>What If You Had Put $1,000 Into Bitcoin, Ethereum, XRP and Solana 5 Years Ago?</t>
-        </is>
-      </c>
-      <c r="AZ19" s="79" t="inlineStr">
-        <is>
-          <t>BUFR Holders Left $62,250 on the Table on a $300,000 Position While Chasing Calm</t>
         </is>
       </c>
     </row>
@@ -6584,17 +6584,17 @@
       </c>
       <c r="AX24" s="79" t="inlineStr">
         <is>
-          <t>The 10 biggest stocks are faltering, and it's dragging the S&amp;P 500 down</t>
+          <t>Mark Cuban puts Bitcoin and Apple in the same bucket</t>
         </is>
       </c>
       <c r="AY24" s="79" t="inlineStr">
         <is>
+          <t>Apple (AAPL) Stock Falls Amid Market Uptick: What Investors Need to Know</t>
+        </is>
+      </c>
+      <c r="AZ24" s="79" t="inlineStr">
+        <is>
           <t>Billionaire predicts 'unhinged' future for iPhone Duo</t>
-        </is>
-      </c>
-      <c r="AZ24" s="79" t="inlineStr">
-        <is>
-          <t>Apple’s iPhone Duo delivery times stretch to January</t>
         </is>
       </c>
     </row>
@@ -6777,12 +6777,12 @@
       </c>
       <c r="AY25" s="90" t="inlineStr">
         <is>
+          <t>Advanced Micro Devices (AMD) Rises Higher Than Market: Key Facts</t>
+        </is>
+      </c>
+      <c r="AZ25" s="90" t="inlineStr">
+        <is>
           <t>Intel Rises 5% as New Street Upgrade Cites Server CPU Shortage; AMD and NVIDIA Gain 3%</t>
-        </is>
-      </c>
-      <c r="AZ25" s="90" t="inlineStr">
-        <is>
-          <t>Meta Seeks About $95 Billion for AI Buildout as Nvidia, AMD and Broadcom Consider Investing in Their Own Cu...</t>
         </is>
       </c>
     </row>
@@ -6960,17 +6960,17 @@
       </c>
       <c r="AX26" s="79" t="inlineStr">
         <is>
+          <t>Target has a problem that sends shoppers to Amazon</t>
+        </is>
+      </c>
+      <c r="AY26" s="79" t="inlineStr">
+        <is>
+          <t>Dow Jones Futures: Elon Musk-Led Tesla Leads Market Higher; Amazon, Alphabet, Microsoft Earnings On Deck</t>
+        </is>
+      </c>
+      <c r="AZ26" s="79" t="inlineStr">
+        <is>
           <t>Tech Earnings Are the Market’s Biggest Story This Week: Here’s Why Microsoft, Amazon, Intel, SanDisk, and A...</t>
-        </is>
-      </c>
-      <c r="AY26" s="79" t="inlineStr">
-        <is>
-          <t>Dow Jones Futures: Elon Musk-Led Tesla Leads Market Higher; Amazon, Alphabet, Microsoft Earnings On Deck</t>
-        </is>
-      </c>
-      <c r="AZ26" s="79" t="inlineStr">
-        <is>
-          <t>Should You Buy Amazon Stock Now or Wait for a Dip?</t>
         </is>
       </c>
     </row>
@@ -7248,7 +7248,7 @@
         <v>211.5800018310547</v>
       </c>
       <c r="U28" s="72" t="n">
-        <v>225.6300048828125</v>
+        <v>225.6699066162109</v>
       </c>
       <c r="V28" s="72" t="n">
         <v>210.8500061035156</v>
@@ -7266,7 +7266,7 @@
         <v>16.30552822768427</v>
       </c>
       <c r="AA28" s="28" t="n">
-        <v>25.89287364402379</v>
+        <v>25.8896061715167</v>
       </c>
       <c r="AB28" s="75" t="n">
         <v>-16.89733810563374</v>
@@ -7308,7 +7308,7 @@
         <v>51.49619933636009</v>
       </c>
       <c r="AO28" s="77" t="n">
-        <v>6.912864351430252</v>
+        <v>6.914140431007726</v>
       </c>
       <c r="AP28" s="72" t="n">
         <v>452.7000122070312</v>
@@ -7336,17 +7336,17 @@
       </c>
       <c r="AX28" s="79" t="inlineStr">
         <is>
+          <t>Arm Holdings (ARM) Faces Jury Breach Ruling As It Unveils Server Security Tie Up</t>
+        </is>
+      </c>
+      <c r="AY28" s="79" t="inlineStr">
+        <is>
           <t>Bulls Insist Arm’s Trio of Multipliers Justify Its Sky High Valuation</t>
         </is>
       </c>
-      <c r="AY28" s="79" t="inlineStr">
+      <c r="AZ28" s="79" t="inlineStr">
         <is>
           <t>Wells Fargo, Arm Holdings And Intuit Object To Stock Tokenization Trading Platform</t>
-        </is>
-      </c>
-      <c r="AZ28" s="79" t="inlineStr">
-        <is>
-          <t>Wells Fargo, Cisco, Intuit Among 6 More Companies Objecting to Tokenized Stocks</t>
         </is>
       </c>
     </row>
@@ -7524,17 +7524,17 @@
       </c>
       <c r="AX29" s="90" t="inlineStr">
         <is>
+          <t>AST SpaceMobile to Host Third Quarter 2026 Business Update Call on November 9, 2026</t>
+        </is>
+      </c>
+      <c r="AY29" s="90" t="inlineStr">
+        <is>
           <t>AST SpaceMobile Advances Brazil Expansion with Anatel’s Approval for S-band Spectrum and Secondary Use of t...</t>
         </is>
       </c>
-      <c r="AY29" s="90" t="inlineStr">
+      <c r="AZ29" s="90" t="inlineStr">
         <is>
           <t>ASTS Stock Slips Overnight: AST Seeks More Spectrum For Broadband Expansion — Market Veteran Flags ‘Sky-Hig...</t>
-        </is>
-      </c>
-      <c r="AZ29" s="90" t="inlineStr">
-        <is>
-          <t>SpaceX’s 80,000 Cell Site Push A Win For AST SpaceMobile, Ericsson, Nokia, NextNav, Among Others, Says Roth...</t>
         </is>
       </c>
     </row>
@@ -7712,17 +7712,17 @@
       </c>
       <c r="AX30" s="79" t="inlineStr">
         <is>
+          <t>Broadcom Partners With Wall Street Bigwigs To Forge $63B Deal To Power Anthropic’s AI Hardware</t>
+        </is>
+      </c>
+      <c r="AY30" s="79" t="inlineStr">
+        <is>
           <t>Broadcom secures $63 billion from banks to finance AI compute sales to Anthropic</t>
         </is>
       </c>
-      <c r="AY30" s="79" t="inlineStr">
-        <is>
-          <t>Bank of America, Blackstone, Citi and Morgan Stanley Announce Landmark $63 Billion Financing Structure to E...</t>
-        </is>
-      </c>
       <c r="AZ30" s="79" t="inlineStr">
         <is>
-          <t>Meta Seeks About $95 Billion for AI Buildout as Nvidia, AMD and Broadcom Consider Investing in Their Own Cu...</t>
+          <t>Broadcom Arranges $63 Billion Deal to Finance Anthropic’s Chips</t>
         </is>
       </c>
     </row>
@@ -8474,7 +8474,7 @@
       </c>
       <c r="AZ34" s="79" t="inlineStr">
         <is>
-          <t>Tech Earnings Are the Market’s Biggest Story This Week: Here’s Why Microsoft, Amazon, Intel, SanDisk, and A...</t>
+          <t>CORRECTING and REPLACING Waymo, Google and Microsoft Alums Raise $30M to Build the Data Layer for Physical AI</t>
         </is>
       </c>
     </row>
@@ -8840,17 +8840,17 @@
       </c>
       <c r="AX36" s="79" t="inlineStr">
         <is>
+          <t>Q2 earnings recap: Intel (NASDAQ:INTC) tops processors and graphics chips stocks</t>
+        </is>
+      </c>
+      <c r="AY36" s="79" t="inlineStr">
+        <is>
+          <t>Intel vs. Nvidia: Flat Trends vs. Rapid Expansion in Revenue</t>
+        </is>
+      </c>
+      <c r="AZ36" s="79" t="inlineStr">
+        <is>
           <t>Tech Earnings Are the Market’s Biggest Story This Week: Here’s Why Microsoft, Amazon, Intel, SanDisk, and A...</t>
-        </is>
-      </c>
-      <c r="AY36" s="79" t="inlineStr">
-        <is>
-          <t>Chip Stocks Find Support Before Key Reports From Intel, Sandisk</t>
-        </is>
-      </c>
-      <c r="AZ36" s="79" t="inlineStr">
-        <is>
-          <t>Intel to Acquire Classiq to Create a Full-stack Quantum Computing Platform</t>
         </is>
       </c>
     </row>
@@ -9028,17 +9028,17 @@
       </c>
       <c r="AX37" s="90" t="inlineStr">
         <is>
+          <t>CORRECTING and REPLACING Waymo, Google and Microsoft Alums Raise $30M to Build the Data Layer for Physical AI</t>
+        </is>
+      </c>
+      <c r="AY37" s="90" t="inlineStr">
+        <is>
+          <t>Dow Jones Futures: Elon Musk-Led Tesla Leads Market Higher; Amazon, Alphabet, Microsoft Earnings On Deck</t>
+        </is>
+      </c>
+      <c r="AZ37" s="90" t="inlineStr">
+        <is>
           <t>Tech Earnings Are the Market’s Biggest Story This Week: Here’s Why Microsoft, Amazon, Intel, SanDisk, and A...</t>
-        </is>
-      </c>
-      <c r="AY37" s="90" t="inlineStr">
-        <is>
-          <t>Dow Jones Futures: Elon Musk-Led Tesla Leads Market Higher; Amazon, Alphabet, Microsoft Earnings On Deck</t>
-        </is>
-      </c>
-      <c r="AZ37" s="90" t="inlineStr">
-        <is>
-          <t>Microsoft offers around 60,000 employees voluntary buyouts</t>
         </is>
       </c>
     </row>
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
-          <t>Business First Bancshares, Inc. Q3 2026 Earnings Call Summary</t>
+          <t>Why Range Resources Stock Surged Today</t>
         </is>
       </c>
       <c r="AY43" s="90" t="inlineStr">
         <is>
-          <t>Verizon Communications Inc. Q3 2026 Earnings Call Summary</t>
+          <t>Intel vs. Nvidia: Flat Trends vs. Rapid Expansion in Revenue</t>
         </is>
       </c>
       <c r="AZ43" s="90" t="inlineStr">
         <is>
-          <t>Bank of Marin Bancorp Q3 2026 Earnings Call Summary</t>
+          <t>Anthropic Just Filed to Go Public. Should You Buy the Stock?</t>
         </is>
       </c>
     </row>
@@ -10537,12 +10537,12 @@
       </c>
       <c r="AY45" s="90" t="inlineStr">
         <is>
-          <t>Is QUALCOMM (QCOM) Undervalued After Reaffirming Its Dividend?</t>
+          <t>Arm Holdings (ARM) Faces Jury Breach Ruling As It Unveils Server Security Tie Up</t>
         </is>
       </c>
       <c r="AZ45" s="90" t="inlineStr">
         <is>
-          <t>Custom System-on-Chip Application-Specific Integrated Circuit (ASIC) Market Global Report 2026 | Capitalize...</t>
+          <t>Qualcomm (QCOM) Laps the Stock Market: Here's Why</t>
         </is>
       </c>
     </row>
@@ -10720,17 +10720,17 @@
       </c>
       <c r="AX46" s="79" t="inlineStr">
         <is>
+          <t>Rocket Lab Corporation (RKLB) Outpaces Stock Market Gains: What You Should Know</t>
+        </is>
+      </c>
+      <c r="AY46" s="79" t="inlineStr">
+        <is>
           <t>Rocket Lab Delayed Neutron Over Voids in a Carbon-Composite Tank Dome. Here's Why That's Better News Than I...</t>
         </is>
       </c>
-      <c r="AY46" s="79" t="inlineStr">
+      <c r="AZ46" s="79" t="inlineStr">
         <is>
           <t>Rocket Lab Shed 25% Over 3 Months: 150% Returns Sure to Come According to This Wall Street Pro</t>
-        </is>
-      </c>
-      <c r="AZ46" s="79" t="inlineStr">
-        <is>
-          <t>What Put Rocket Lab Ahead Of Its Industry?</t>
         </is>
       </c>
     </row>
@@ -11096,17 +11096,17 @@
       </c>
       <c r="AX48" s="79" t="inlineStr">
         <is>
+          <t>TSLA Analyst Ratings Hit Highest Since 2023; ARK Reiterates $4,400 Long-Term Price Target And 80% Robotaxi ...</t>
+        </is>
+      </c>
+      <c r="AY48" s="79" t="inlineStr">
+        <is>
           <t>Dow Jones Futures: Elon Musk-Led Tesla Leads Market Higher; Amazon, Alphabet, Microsoft Earnings On Deck</t>
         </is>
       </c>
-      <c r="AY48" s="79" t="inlineStr">
+      <c r="AZ48" s="79" t="inlineStr">
         <is>
           <t>Tesla Isn’t a Hyperscaler. Why the AI Bears Are Misreading Its $5 Billion Capex Cut.</t>
-        </is>
-      </c>
-      <c r="AZ48" s="79" t="inlineStr">
-        <is>
-          <t>Tesla Stock, Upgraded On SpaceX Prospects, Moves Into A Buy Zone</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 26 Oct 2026, 09:45 PM · Yahoo Finance data</t>
+          <t>Built 26 Oct 2026, 11:55 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 26 Oct 2026, 09:45 PM · Yahoo Finance data</t>
+          <t>Built 26 Oct 2026, 11:55 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 26 Oct 2026, 09:45 PM · Yahoo Finance data</t>
+          <t>Built 26 Oct 2026, 11:55 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 26 Oct 2026, 09:45 PM · Yahoo Finance data</t>
+          <t>Built 26 Oct 2026, 11:55 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-10-27 23:47 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 27 Oct 2026, 09:25 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 27 Oct 2026, 11:47 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 27 Oct 2026, 09:25 PM · Yahoo Finance data</t>
+          <t>Built 27 Oct 2026, 11:47 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -4564,7 +4564,7 @@
         <v>114.8499984741211</v>
       </c>
       <c r="U12" s="83" t="n">
-        <v>115.6399993896484</v>
+        <v>115.6699981689453</v>
       </c>
       <c r="V12" s="83" t="n">
         <v>114.3099975585938</v>
@@ -4582,7 +4582,7 @@
         <v>86.12605677366142</v>
       </c>
       <c r="AA12" s="35" t="n">
-        <v>16.50681538296629</v>
+        <v>16.5234287721434</v>
       </c>
       <c r="AB12" s="86" t="n">
         <v>0.6844597566426955</v>
@@ -4624,7 +4624,7 @@
         <v>7.21241194916674</v>
       </c>
       <c r="AO12" s="88" t="n">
-        <v>1.409865779833797</v>
+        <v>1.411721795430521</v>
       </c>
       <c r="AP12" s="83" t="n">
         <v>125.0100021362305</v>
@@ -5134,7 +5134,7 @@
         <v>187.5700073242188</v>
       </c>
       <c r="U15" s="72" t="n">
-        <v>190.0700073242188</v>
+        <v>190.0899963378906</v>
       </c>
       <c r="V15" s="72" t="n">
         <v>187.1000061035156</v>
@@ -5152,7 +5152,7 @@
         <v>40.43526171224356</v>
       </c>
       <c r="AA15" s="28" t="n">
-        <v>26.22990450288872</v>
+        <v>26.22428771858466</v>
       </c>
       <c r="AB15" s="75" t="n">
         <v>-1.686893111957545</v>
@@ -5194,7 +5194,7 @@
         <v>13.70376528165415</v>
       </c>
       <c r="AO15" s="77" t="n">
-        <v>2.040253616015512</v>
+        <v>2.041007105196714</v>
       </c>
       <c r="AP15" s="72" t="n">
         <v>203.25</v>
@@ -6777,12 +6777,12 @@
       </c>
       <c r="AY25" s="90" t="inlineStr">
         <is>
+          <t>Penguin Solutions, Broadcom, FormFactor, Lattice Semiconductor, and AMD stocks trade up, what you need to know</t>
+        </is>
+      </c>
+      <c r="AZ25" s="90" t="inlineStr">
+        <is>
           <t>I'd Own a Small Position in AMD Stock Through 2030, but I Wouldn't Expect It to Triple Again</t>
-        </is>
-      </c>
-      <c r="AZ25" s="90" t="inlineStr">
-        <is>
-          <t>Cathie Wood Cashes Out AI Chip Stocks, Adds These Aviation Plays</t>
         </is>
       </c>
     </row>
@@ -6965,12 +6965,12 @@
       </c>
       <c r="AY26" s="79" t="inlineStr">
         <is>
-          <t>Is Amazon.com (AMZN) Undervalued As Investors Eye Q3 2026 Earnings?</t>
+          <t>Amazon Backup Power Deal Could Be A Turning Point For Generac Stock</t>
         </is>
       </c>
       <c r="AZ26" s="79" t="inlineStr">
         <is>
-          <t>Oracle Rises 5% as Google TPUs Come to Oracle Cloud and NVIDIA Deal Expands; Amazon Nudges Higher, Microsof...</t>
+          <t>RIVN Stock Rebounds As Unconfirmed Walmart Delivery Van Sparks Fleet Hopes</t>
         </is>
       </c>
     </row>
@@ -7717,12 +7717,12 @@
       </c>
       <c r="AY30" s="79" t="inlineStr">
         <is>
-          <t>The AI economy, Apple's iPhone Duo issues, and Meta partners with Nvidia</t>
+          <t>Intel, Microchip Technology, Marvell Technology, onsemi, and Seagate stocks trade up, what you need to know</t>
         </is>
       </c>
       <c r="AZ30" s="79" t="inlineStr">
         <is>
-          <t>Two Chip Stocks Upgraded To Buy On AI Data-Center Business</t>
+          <t>Penguin Solutions, Broadcom, FormFactor, Lattice Semiconductor, and AMD stocks trade up, what you need to know</t>
         </is>
       </c>
     </row>
@@ -7900,17 +7900,17 @@
       </c>
       <c r="AX31" s="90" t="inlineStr">
         <is>
+          <t>3 Canadian Growth Stocks To Own In October 2026</t>
+        </is>
+      </c>
+      <c r="AY31" s="90" t="inlineStr">
+        <is>
           <t>Cameco vs. Centrus vs. BWX Technologies: Ranking the 3 Nuclear Stocks That Get Paid Before a Reactor Is Built.</t>
         </is>
       </c>
-      <c r="AY31" s="90" t="inlineStr">
+      <c r="AZ31" s="90" t="inlineStr">
         <is>
           <t>Can Cameco’s 89x Premium Valuation Survive Another Big Miss on Oct. 30?</t>
-        </is>
-      </c>
-      <c r="AZ31" s="90" t="inlineStr">
-        <is>
-          <t>3 Canadian Growth Stocks With Earnings Growth Up To 65%</t>
         </is>
       </c>
     </row>
@@ -8088,17 +8088,17 @@
       </c>
       <c r="AX32" s="79" t="inlineStr">
         <is>
+          <t>CoreWeave Stock Surges 6%, But Investors Are Still Worried</t>
+        </is>
+      </c>
+      <c r="AY32" s="79" t="inlineStr">
+        <is>
+          <t>Stock Market Today, Oct. 27: CoreWeave Surges on Denmark Data Center Launch</t>
+        </is>
+      </c>
+      <c r="AZ32" s="79" t="inlineStr">
+        <is>
           <t>Nebius vs. CoreWeave: Which neocloud stock has more debt?</t>
-        </is>
-      </c>
-      <c r="AY32" s="79" t="inlineStr">
-        <is>
-          <t>CoreWeave Announces Date of Third Quarter 2026 Financial Results and Conference Call</t>
-        </is>
-      </c>
-      <c r="AZ32" s="79" t="inlineStr">
-        <is>
-          <t>Crusoe CEO defends CoreWeave amid selloff</t>
         </is>
       </c>
     </row>
@@ -8276,17 +8276,17 @@
       </c>
       <c r="AX33" s="90" t="inlineStr">
         <is>
+          <t>What Dell Technologies Doubters Got Wrong Before A 297% Rally</t>
+        </is>
+      </c>
+      <c r="AY33" s="90" t="inlineStr">
+        <is>
+          <t>Why is Dell (DELL) stock soaring today</t>
+        </is>
+      </c>
+      <c r="AZ33" s="90" t="inlineStr">
+        <is>
           <t>Global Edge Infrastructure Market Report 2026: Size, Share, Trends and Forecast to 2030 | Capitalize on 5G,...</t>
-        </is>
-      </c>
-      <c r="AY33" s="90" t="inlineStr">
-        <is>
-          <t>Dell Technologies vs. Marvell Technology: Which Tech Stock Is the Better Buy in 2026?</t>
-        </is>
-      </c>
-      <c r="AZ33" s="90" t="inlineStr">
-        <is>
-          <t>Dell and HPE Lost Billions in a Day Over 1 Big Worry. Dell Had Already Answered It.</t>
         </is>
       </c>
     </row>
@@ -8840,17 +8840,17 @@
       </c>
       <c r="AX36" s="79" t="inlineStr">
         <is>
+          <t>Intel, Microchip Technology, Marvell Technology, onsemi, and Seagate stocks trade up, what you need to know</t>
+        </is>
+      </c>
+      <c r="AY36" s="79" t="inlineStr">
+        <is>
           <t>IonQ Jumped 7%, Rigetti Up 8% on Intel’s $2.3 Billion Quantum Buy: “Full-Stack Quantum Computing Business”</t>
         </is>
       </c>
-      <c r="AY36" s="79" t="inlineStr">
+      <c r="AZ36" s="79" t="inlineStr">
         <is>
           <t>Intel, Oracle, IBM Join Objections to OKX-ICE Tokenized Stock Venue, Bringing Total to 26</t>
-        </is>
-      </c>
-      <c r="AZ36" s="79" t="inlineStr">
-        <is>
-          <t>Intel faces test of recovery as Wedbush looks beyond Q3 results</t>
         </is>
       </c>
     </row>
@@ -9038,7 +9038,7 @@
       </c>
       <c r="AZ37" s="90" t="inlineStr">
         <is>
-          <t>Artificial Intelligence (AI) in Pharmacovigilance Global Market Report 2026 | Capitalize on 19.6% CAGR to 2...</t>
+          <t>Ascendion Expands AI Advisory Community with Four Global Business and Technology Leaders</t>
         </is>
       </c>
     </row>
@@ -9131,7 +9131,7 @@
         <v>142</v>
       </c>
       <c r="V38" s="72" t="n">
-        <v>138.6999969482422</v>
+        <v>138.6900024414062</v>
       </c>
       <c r="W38" s="73" t="n">
         <v>10571034</v>
@@ -9188,7 +9188,7 @@
         <v>22.09671775744949</v>
       </c>
       <c r="AO38" s="77" t="n">
-        <v>6.546175568266276</v>
+        <v>6.546680443355554</v>
       </c>
       <c r="AP38" s="72" t="n">
         <v>299.7999877929688</v>
@@ -9216,17 +9216,17 @@
       </c>
       <c r="AX38" s="79" t="inlineStr">
         <is>
+          <t>Strategy (MSTR) Stock May Be Undervalued On Bitcoin Policy Shift</t>
+        </is>
+      </c>
+      <c r="AY38" s="79" t="inlineStr">
+        <is>
+          <t>Strive Buys 6,182 BTC as Strategy Pauses Its Bitcoin Buying. Can Treasury Buyers Hold BTC Above $80,000?</t>
+        </is>
+      </c>
+      <c r="AZ38" s="79" t="inlineStr">
+        <is>
           <t>Strategy vs. CleanSpark: Which Bitcoin Stock Has Greater Upside Now?</t>
-        </is>
-      </c>
-      <c r="AY38" s="79" t="inlineStr">
-        <is>
-          <t>Michael Saylor’s Strategy Just Formed a Golden Cross. Why Bitcoin Bulls Shouldn’t Expect Another 700% Rally...</t>
-        </is>
-      </c>
-      <c r="AZ38" s="79" t="inlineStr">
-        <is>
-          <t>Strategy Buys $0 Bitcoin, Repurchases $205M in STRC as Saylor Reveals $5.1B Cash Holdings</t>
         </is>
       </c>
     </row>
@@ -9404,17 +9404,17 @@
       </c>
       <c r="AX39" s="90" t="inlineStr">
         <is>
-          <t>Prediction: This Artificial Intelligence (AI) Memory Stock Will Go Parabolic on Oct. 30</t>
+          <t>What Could Robot Memory Demand Mean For Micron Technology (MU) Stock?</t>
         </is>
       </c>
       <c r="AY39" s="90" t="inlineStr">
         <is>
-          <t>TSM vs. MU: Which Semiconductor Stock Is the Better Buy Post-Earnings?</t>
+          <t>Micron Will Pay Bonuses Half in Stock. At 63, Shares He Hasn’t Sold Could Still Count Toward His $25,560 So...</t>
         </is>
       </c>
       <c r="AZ39" s="90" t="inlineStr">
         <is>
-          <t>Micron, Musk, and Memory. A Big Prediction Is Lifting the Stock.</t>
+          <t>'We're Trading Them Like Baseball Cards': Mark Cuban Warns ‘Everything’s a Meme Stock’ as AAPL, GOOGL and M...</t>
         </is>
       </c>
     </row>
@@ -9785,12 +9785,12 @@
       </c>
       <c r="AY41" s="90" t="inlineStr">
         <is>
+          <t>What Does Netflix (NFLX) Leadership Shakeup Mean For Its Streaming Future?</t>
+        </is>
+      </c>
+      <c r="AZ41" s="90" t="inlineStr">
+        <is>
           <t>3 Magnificent Stocks Trading Near Their 52-Week Lows</t>
-        </is>
-      </c>
-      <c r="AZ41" s="90" t="inlineStr">
-        <is>
-          <t>The Netflix layoffs reveal what corporate America is getting wrong</t>
         </is>
       </c>
     </row>
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
-          <t>Nvidia, AMD Get Their Jollies Hooking Up With Meta's Muse</t>
+          <t>History Says the Stock Market's Best 6 Months Start Nov. 1. Here's How Often They've Paid Off Since 1950.</t>
         </is>
       </c>
       <c r="AY43" s="90" t="inlineStr">
         <is>
-          <t>S&amp;P Global Inc. Q3 2026 Earnings Call Summary</t>
+          <t>Investing $1,000 in Each of These 3 Stocks 20 Years Ago Would Have Created a Portfolio Worth $674,000 Today</t>
         </is>
       </c>
       <c r="AZ43" s="90" t="inlineStr">
         <is>
-          <t>The Simply Good Foods Company Q4 2026 Earnings Call Summary</t>
+          <t>Nvidia’s New $3 Billion AI Bet Is on One of Its Own Customers</t>
         </is>
       </c>
     </row>
@@ -11101,12 +11101,12 @@
       </c>
       <c r="AY48" s="79" t="inlineStr">
         <is>
-          <t>Tesla Stock Rises In A Buy Range; Musk Touts Cybercab Fleet Expansion</t>
+          <t>TSLA Stock Rises As Cybercabs Overtake Model Ys In Authorized Texas Robotaxi Fleet</t>
         </is>
       </c>
       <c r="AZ48" s="79" t="inlineStr">
         <is>
-          <t>Tesla Stock Has Room to Run, If History Is Any Indicator</t>
+          <t>Scott Galloway Warns Tesla Is the ‘Patient’ and SpaceX Its ‘Organ Donor’ in Elon Musk’s $3.5 Trillion Merge...</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 27 Oct 2026, 09:25 PM · Yahoo Finance data</t>
+          <t>Built 27 Oct 2026, 11:47 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 27 Oct 2026, 09:25 PM · Yahoo Finance data</t>
+          <t>Built 27 Oct 2026, 11:47 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 27 Oct 2026, 09:25 PM · Yahoo Finance data</t>
+          <t>Built 27 Oct 2026, 11:47 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 27 Oct 2026, 09:25 PM · Yahoo Finance data</t>
+          <t>Built 27 Oct 2026, 11:47 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-10-29 00:52 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 29 Oct 2026, 12:02 AM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 29 Oct 2026, 12:52 AM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 29 Oct 2026, 12:02 AM · Yahoo Finance data</t>
+          <t>Built 29 Oct 2026, 12:52 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -6594,7 +6594,7 @@
       </c>
       <c r="AZ24" s="79" t="inlineStr">
         <is>
-          <t>Apple Stock And Other Quality Growth Names For Higher Rates</t>
+          <t>November Is Already Dated: HomeView Ships Nov 13, Wells Fargo’s Agent Contract Goes Live Nov 24, Black Frid...</t>
         </is>
       </c>
     </row>
@@ -7712,17 +7712,17 @@
       </c>
       <c r="AX30" s="79" t="inlineStr">
         <is>
-          <t>AMD, Broadcom, and Micron stocks lead chip sector higher for third day in a row</t>
+          <t>Tech rises for third day in a row ahead of Microsoft, Alphabet earnings, Fed decision in focus: AlphaCheck</t>
         </is>
       </c>
       <c r="AY30" s="79" t="inlineStr">
         <is>
-          <t>Tech rises for third day in a row ahead of Microsoft, Alphabet earnings, Fed decision in focus: AlphaCheck</t>
+          <t>2 Millionaire-Maker Custom Silicon Stocks Powering the AI Infrastructure Supercycle</t>
         </is>
       </c>
       <c r="AZ30" s="79" t="inlineStr">
         <is>
-          <t>2 Millionaire-Maker Custom Silicon Stocks Powering the AI Infrastructure Supercycle</t>
+          <t>Broadcom Inc. (AVGO) Laps the Stock Market: Here's Why</t>
         </is>
       </c>
     </row>
@@ -7900,17 +7900,17 @@
       </c>
       <c r="AX31" s="90" t="inlineStr">
         <is>
+          <t>Cameco And 2 Other Canadian Growth Stocks To Watch</t>
+        </is>
+      </c>
+      <c r="AY31" s="90" t="inlineStr">
+        <is>
           <t>CCJ Falls 27.6% in 6 Months as Execution Risks Test the Nuclear Thesis</t>
         </is>
       </c>
-      <c r="AY31" s="90" t="inlineStr">
+      <c r="AZ31" s="90" t="inlineStr">
         <is>
           <t>Cameco's Raised Revenue Outlook Faces a Crucial Execution Test Ahead</t>
-        </is>
-      </c>
-      <c r="AZ31" s="90" t="inlineStr">
-        <is>
-          <t>Is Cameco Worth Buying as Premium Valuation Meets Execution Risk?</t>
         </is>
       </c>
     </row>
@@ -8464,17 +8464,17 @@
       </c>
       <c r="AX34" s="79" t="inlineStr">
         <is>
-          <t>Alphabet CFO walks through the company's Q3 results</t>
+          <t>Dow Jones Futures: Microsoft Rises, But Google, ServiceNow, Fortinet Dive On Earnings</t>
         </is>
       </c>
       <c r="AY34" s="79" t="inlineStr">
         <is>
-          <t>Dow Jones Futures: Microsoft Rises Late, But Google, ServiceNow, Fortinet Dive On Earnings</t>
+          <t>Google Pitches Banks on Splitting Crypto Keys Across Clouds With New Custody Service</t>
         </is>
       </c>
       <c r="AZ34" s="79" t="inlineStr">
         <is>
-          <t>Google Cloud Revenue Just Grew 103%, so Why Is the Stock Falling?</t>
+          <t>Microsoft and Alphabet Just Reported Earnings, Putting the AI Boom to the Test</t>
         </is>
       </c>
     </row>
@@ -9033,12 +9033,12 @@
       </c>
       <c r="AY37" s="90" t="inlineStr">
         <is>
-          <t>Dow Jones Futures: Microsoft Rises Late, But Google, ServiceNow, Fortinet Dive On Earnings</t>
+          <t>Dow Jones Futures: Microsoft Rises, But Google, ServiceNow, Fortinet Dive On Earnings</t>
         </is>
       </c>
       <c r="AZ37" s="90" t="inlineStr">
         <is>
-          <t>MSFT Stock Gains 3% After-Hours As AI Demand Powers Q1 Cloud Revenue, Q2 Guidance Beat With Positive Cash F...</t>
+          <t>Why Is Microsoft (MSFT) Offering Buyouts To 60,000 Employees?</t>
         </is>
       </c>
     </row>
@@ -9404,17 +9404,17 @@
       </c>
       <c r="AX39" s="90" t="inlineStr">
         <is>
+          <t>Here's Why Micron Is a Top AI Stock to Buy Right Now</t>
+        </is>
+      </c>
+      <c r="AY39" s="90" t="inlineStr">
+        <is>
           <t>Micron, SK Hynix, Google, Microsoft, Vertiv, Wendy’s, Enphase, and More Stocks That Explain Today’s Market</t>
         </is>
       </c>
-      <c r="AY39" s="90" t="inlineStr">
+      <c r="AZ39" s="90" t="inlineStr">
         <is>
           <t>SK Hynix Just Delivered Great News for Micron Investors</t>
-        </is>
-      </c>
-      <c r="AZ39" s="90" t="inlineStr">
-        <is>
-          <t>Micron Stock Advances as Rival SK Hynix Fuels AI Frenzy With Two Bombshells</t>
         </is>
       </c>
     </row>
@@ -10161,12 +10161,12 @@
       </c>
       <c r="AY43" s="90" t="inlineStr">
         <is>
-          <t>AI Spending Is Nearing $1 Trillion Annually. These 2 Stocks Are Most at Risk If It Slows.</t>
+          <t>Microsoft and Alphabet Just Reported Earnings, Putting the AI Boom to the Test</t>
         </is>
       </c>
       <c r="AZ43" s="90" t="inlineStr">
         <is>
-          <t>Frontier Group Holdings, Inc. Q3 2026 Earnings Call Summary</t>
+          <t>CrowdStrike (CRWD) Stock Looks Overvalued On Its 5x Three Year Run</t>
         </is>
       </c>
     </row>
@@ -11106,7 +11106,7 @@
       </c>
       <c r="AZ48" s="79" t="inlineStr">
         <is>
-          <t>Tesla Gains Another 4% as ARK Restates $4,400 Robotaxi Target and Musk Teases “A Storm of Cybercabs”</t>
+          <t>History Shows That Buying the Dip Can Yield Huge Profits. Consider Snapping Up These 3 $100+ Stocks Here.</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 29 Oct 2026, 12:02 AM · Yahoo Finance data</t>
+          <t>Built 29 Oct 2026, 12:52 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 29 Oct 2026, 12:02 AM · Yahoo Finance data</t>
+          <t>Built 29 Oct 2026, 12:52 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 29 Oct 2026, 12:02 AM · Yahoo Finance data</t>
+          <t>Built 29 Oct 2026, 12:52 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 29 Oct 2026, 12:02 AM · Yahoo Finance data</t>
+          <t>Built 29 Oct 2026, 12:52 AM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-10-29 23:57 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 29 Oct 2026, 09:55 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 29 Oct 2026, 11:57 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 29 Oct 2026, 09:55 PM · Yahoo Finance data</t>
+          <t>Built 29 Oct 2026, 11:57 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -6965,12 +6965,12 @@
       </c>
       <c r="AY26" s="79" t="inlineStr">
         <is>
-          <t>Amazon's mixed Q3 earnings raises some questions</t>
+          <t>Dow Jones Futures: Amazon, Intel Lead Earnings Losers After Google, ServiceNow, Fortinet Hit Nasdaq</t>
         </is>
       </c>
       <c r="AZ26" s="79" t="inlineStr">
         <is>
-          <t>Dow Jones Futures: Amazon, Intel Lead Earnings Losers After Google, ServiceNow, Fortinet Hit Nasdaq</t>
+          <t>Amazon cloud business accelerates but shares drop on profit miss</t>
         </is>
       </c>
     </row>
@@ -7529,12 +7529,12 @@
       </c>
       <c r="AY29" s="90" t="inlineStr">
         <is>
+          <t>Why the Market Dipped But AST SpaceMobile, Inc. (ASTS) Gained Today</t>
+        </is>
+      </c>
+      <c r="AZ29" s="90" t="inlineStr">
+        <is>
           <t>ASTS Stock Gains On FCC Plan To Expand Direct-To-Phone Spectrum</t>
-        </is>
-      </c>
-      <c r="AZ29" s="90" t="inlineStr">
-        <is>
-          <t>Prediction: ASTS Could Be Entering Its Biggest Growth Phase Yet</t>
         </is>
       </c>
     </row>
@@ -8469,12 +8469,12 @@
       </c>
       <c r="AY34" s="79" t="inlineStr">
         <is>
-          <t>Google's AI chips could change what ChatGPT costs you</t>
+          <t>Google owner Alphabet reports 25% revenue growth in Q3 2026</t>
         </is>
       </c>
       <c r="AZ34" s="79" t="inlineStr">
         <is>
-          <t>Update: US Equity Indexes Decline as Alphabet's Disappointing Earnings Decimate Communication Services</t>
+          <t>Shares of Google’s parent company just had their worst day ever. Here’s what it means</t>
         </is>
       </c>
     </row>
@@ -8845,12 +8845,12 @@
       </c>
       <c r="AY36" s="79" t="inlineStr">
         <is>
-          <t>Supply Constraints a Swing Factor for Intel, Seaport's Goldberg Says</t>
+          <t>What Intel (INTC) Said on Its Q3 Earnings Call</t>
         </is>
       </c>
       <c r="AZ36" s="79" t="inlineStr">
         <is>
-          <t>Intel Server Sales Jump 78%, Q4 Outlook Dims: Rapid Earnings Reaction</t>
+          <t>Amazon cloud business accelerates but shares drop on profit miss</t>
         </is>
       </c>
     </row>
@@ -9028,17 +9028,17 @@
       </c>
       <c r="AX37" s="90" t="inlineStr">
         <is>
+          <t>Billionaire Bill Gates Just Issued a Blunt Warning About Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="AY37" s="90" t="inlineStr">
+        <is>
           <t>Things to consider if a company that made AI-related job cuts wants to rehire you</t>
         </is>
       </c>
-      <c r="AY37" s="90" t="inlineStr">
-        <is>
-          <t>Microsoft, IBD Stock Of The Day, Showing Quickening Cloud Growth</t>
-        </is>
-      </c>
       <c r="AZ37" s="90" t="inlineStr">
         <is>
-          <t>Microsoft, Google report booming AI revenue as the tech reshapes business</t>
+          <t>Big Tech Earnings Couldn’t Ignite Chip Stocks. What The Semis Need Now.</t>
         </is>
       </c>
     </row>
@@ -9216,17 +9216,17 @@
       </c>
       <c r="AX38" s="79" t="inlineStr">
         <is>
-          <t>Strategy (MSTR) Shareholders Approved Daily Dividends On Four Preferred Stocks</t>
+          <t>LIVE: MicroStrategy Q3 2026 earnings call</t>
         </is>
       </c>
       <c r="AY38" s="79" t="inlineStr">
         <is>
-          <t>Strategy's Bitcoin Per Share Falls 3.7%: Rapid Earnings Reaction</t>
+          <t>Strategy Posts $21 Billion Bitcoin Gain. Investors Have Bigger Concerns.</t>
         </is>
       </c>
       <c r="AZ38" s="79" t="inlineStr">
         <is>
-          <t>Strategy: Q3 Earnings Snapshot</t>
+          <t>Strategy (MSTR) Beats Q3 Earnings Estimates</t>
         </is>
       </c>
     </row>
@@ -9409,12 +9409,12 @@
       </c>
       <c r="AY39" s="90" t="inlineStr">
         <is>
+          <t>Micron Is Trading for Less Than 6 Times Forward Earnings. Here's Why That's a Sign to Buy.</t>
+        </is>
+      </c>
+      <c r="AZ39" s="90" t="inlineStr">
+        <is>
           <t>Here's Why Micron (MU) Fell More Than Broader Market</t>
-        </is>
-      </c>
-      <c r="AZ39" s="90" t="inlineStr">
-        <is>
-          <t>Sandisk and Micron Slide 5% as Samsung Miss Cools Memory Rally Ahead of Sandisk Earnings; SK Hynix Falls 3%...</t>
         </is>
       </c>
     </row>
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
-          <t>Caterpillar Inc. Q3 2026 Earnings Call Summary</t>
+          <t>Nvidia's $12.9 billion deal could shape the AI apps you use</t>
         </is>
       </c>
       <c r="AY43" s="90" t="inlineStr">
         <is>
-          <t>Carrier Global Corporation Q3 2026 Earnings Call Summary</t>
+          <t>Kymera Therapeutics, Inc. Q3 2026 Earnings Call Summary</t>
         </is>
       </c>
       <c r="AZ43" s="90" t="inlineStr">
         <is>
-          <t>ATI Inc. Q3 2026 Earnings Call Summary</t>
+          <t>Kimco Realty Corporation Q3 2026 Earnings Call Summary</t>
         </is>
       </c>
     </row>
@@ -10344,17 +10344,17 @@
       </c>
       <c r="AX44" s="79" t="inlineStr">
         <is>
+          <t>JPMorgan Is Bullish on Palantir, Predicts Over 30% Rally on Strong AI Demand</t>
+        </is>
+      </c>
+      <c r="AY44" s="79" t="inlineStr">
+        <is>
           <t>Could $1,000 Invested in Palantir Turn Into $100,000?</t>
         </is>
       </c>
-      <c r="AY44" s="79" t="inlineStr">
+      <c r="AZ44" s="79" t="inlineStr">
         <is>
           <t>Why J.P. Morgan Believes Palantir Stock Is Just Getting Going After a Lackluster 2026</t>
-        </is>
-      </c>
-      <c r="AZ44" s="79" t="inlineStr">
-        <is>
-          <t>Palantir Seen Beating Revenue Estimates, Raising Guidance, Oppenheimer Says</t>
         </is>
       </c>
     </row>
@@ -10913,12 +10913,12 @@
       </c>
       <c r="AY47" s="90" t="inlineStr">
         <is>
+          <t>Sandisk Reports Another Big Earnings Beat. Investors May Have Wanted More.</t>
+        </is>
+      </c>
+      <c r="AZ47" s="90" t="inlineStr">
+        <is>
           <t>Sandisk Clears Fiscal Q1 Targets, Announces 8-For-1 Stock Split</t>
-        </is>
-      </c>
-      <c r="AZ47" s="90" t="inlineStr">
-        <is>
-          <t>Sandisk Revenue Up 378% on Datacenter, Edge: Rapid Earnings Reaction</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 29 Oct 2026, 09:55 PM · Yahoo Finance data</t>
+          <t>Built 29 Oct 2026, 11:57 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 29 Oct 2026, 09:55 PM · Yahoo Finance data</t>
+          <t>Built 29 Oct 2026, 11:57 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 29 Oct 2026, 09:55 PM · Yahoo Finance data</t>
+          <t>Built 29 Oct 2026, 11:57 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 29 Oct 2026, 09:55 PM · Yahoo Finance data</t>
+          <t>Built 29 Oct 2026, 11:57 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Daily workbook: 2026-10-30 23:51 UTC
</commit_message>
<xml_diff>
--- a/docs/data/latest.xlsx
+++ b/docs/data/latest.xlsx
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Built automatically 30 Oct 2026, 09:39 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
+          <t>Built automatically 30 Oct 2026, 11:51 PM · Yahoo Finance data · EMA 8/21 · DMA 50/100/200 · BB 20,2 · MACD 12/26/9</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -3107,7 +3107,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 30 Oct 2026, 09:39 PM · Yahoo Finance data</t>
+          <t>Built 30 Oct 2026, 11:51 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -6589,12 +6589,12 @@
       </c>
       <c r="AY24" s="79" t="inlineStr">
         <is>
+          <t>Apple overtakes Nvidia to become world’s most valuable company amid tech selloff</t>
+        </is>
+      </c>
+      <c r="AZ24" s="79" t="inlineStr">
+        <is>
           <t>Dow Jones Futures: Stock Market Sells Off As Apple, Palantir, Midterm Elections Loom; What To Do</t>
-        </is>
-      </c>
-      <c r="AZ24" s="79" t="inlineStr">
-        <is>
-          <t>Apple Overtakes Nvidia to Become World’s Most Valuable Company</t>
         </is>
       </c>
     </row>
@@ -6772,17 +6772,17 @@
       </c>
       <c r="AX25" s="90" t="inlineStr">
         <is>
+          <t>Cathie Wood Shifts From AI Chips to Robinhood and Air Taxis in Latest ARK Trades</t>
+        </is>
+      </c>
+      <c r="AY25" s="90" t="inlineStr">
+        <is>
           <t>Apple, Super Micro, AMD, Palantir Step Up To Earnings Plate After Tech Sell-Off</t>
         </is>
       </c>
-      <c r="AY25" s="90" t="inlineStr">
+      <c r="AZ25" s="90" t="inlineStr">
         <is>
           <t>Advanced Micro Devices (AMD) Lands First GSI Deployment Under AI Compute Deal</t>
-        </is>
-      </c>
-      <c r="AZ25" s="90" t="inlineStr">
-        <is>
-          <t>AMD Reports on Nov. 3. Here's What You Should Do Before Then.</t>
         </is>
       </c>
     </row>
@@ -6960,17 +6960,17 @@
       </c>
       <c r="AX26" s="79" t="inlineStr">
         <is>
+          <t>Stock Market Today, Oct. 30: Amazon Misses Revenue and Earnings Expectations</t>
+        </is>
+      </c>
+      <c r="AY26" s="79" t="inlineStr">
+        <is>
+          <t>Gene Munster 'More Concerned' About Amazon and Alphabet — Says AI Bots Mean Shopping Edge 'Will Increasingl...</t>
+        </is>
+      </c>
+      <c r="AZ26" s="79" t="inlineStr">
+        <is>
           <t>US Equity Indexes Drop This Week as Disappointing Hyperscaler Results Offset Gains From Anthropic's IPO Boost</t>
-        </is>
-      </c>
-      <c r="AY26" s="79" t="inlineStr">
-        <is>
-          <t>Markets lashed by tech rout as earnings fan AI fears</t>
-        </is>
-      </c>
-      <c r="AZ26" s="79" t="inlineStr">
-        <is>
-          <t>Stocks Plunge Again as AI Trade Unravels. Nasdaq Sees Worst Day Since June.</t>
         </is>
       </c>
     </row>
@@ -8276,17 +8276,17 @@
       </c>
       <c r="AX33" s="90" t="inlineStr">
         <is>
+          <t>What Are Dell Investors Betting On?</t>
+        </is>
+      </c>
+      <c r="AY33" s="90" t="inlineStr">
+        <is>
           <t>Intel Plunges 25% as Weak Outlook and PC Slump Overshadow Earnings Beat; Dell Tumbles 13%, AMD Sinks 10%, N...</t>
         </is>
       </c>
-      <c r="AY33" s="90" t="inlineStr">
+      <c r="AZ33" s="90" t="inlineStr">
         <is>
           <t>HPQ, DELL Stocks Plunge After Intel Flags Prolonged PC Market Weakness</t>
-        </is>
-      </c>
-      <c r="AZ33" s="90" t="inlineStr">
-        <is>
-          <t>Everpure vs. Dell: Which Data Storage Stock is the Better Buy Now?</t>
         </is>
       </c>
     </row>
@@ -8464,17 +8464,17 @@
       </c>
       <c r="AX34" s="79" t="inlineStr">
         <is>
+          <t>Veteran fund manager revamps Alphabet stock price target after brutal sell-off</t>
+        </is>
+      </c>
+      <c r="AY34" s="79" t="inlineStr">
+        <is>
           <t>Cracks are emerging in the AI spending boom</t>
         </is>
       </c>
-      <c r="AY34" s="79" t="inlineStr">
-        <is>
-          <t>Nasdaq sheds more than 700 points as tech stocks slump</t>
-        </is>
-      </c>
       <c r="AZ34" s="79" t="inlineStr">
         <is>
-          <t>US Equity Indexes Drop This Week as Disappointing Hyperscaler Results Offset Gains From Anthropic's IPO Boost</t>
+          <t>Gene Munster 'More Concerned' About Amazon and Alphabet — Says AI Bots Mean Shopping Edge 'Will Increasingl...</t>
         </is>
       </c>
     </row>
@@ -8840,17 +8840,17 @@
       </c>
       <c r="AX36" s="79" t="inlineStr">
         <is>
-          <t>Jim Cramer is ‘furious’ as Intel crashes nearly 30% — but Uncle Sam is the top shareholder. What it means f...</t>
+          <t>Why Arm Holdings Stock Plummeted by Nearly 10% Today</t>
         </is>
       </c>
       <c r="AY36" s="79" t="inlineStr">
         <is>
-          <t>Stock Market Today, Oct. 30: Intel Plunges Nearly 29% as Weak Outlook Rattles Wall Street</t>
+          <t>Is Intel Stock a Buy After Its Post-Earnings Plunge?</t>
         </is>
       </c>
       <c r="AZ36" s="79" t="inlineStr">
         <is>
-          <t>Jim Cramer Admits He Was Wrong About Intel as Stock Plunges 29%</t>
+          <t>Intel CEO reveals a PC problem as Goldman cuts stock target</t>
         </is>
       </c>
     </row>
@@ -10156,17 +10156,17 @@
       </c>
       <c r="AX43" s="90" t="inlineStr">
         <is>
-          <t>General Dynamics Corporation Q3 2026 Earnings Call Summary</t>
+          <t>Nvidia has a stake in SpaceX that came from an unexpected place</t>
         </is>
       </c>
       <c r="AY43" s="90" t="inlineStr">
         <is>
-          <t>RBC Bearings Incorporated Q2 2027 Earnings Call Summary</t>
+          <t>Why CareDx Stock Soared Today</t>
         </is>
       </c>
       <c r="AZ43" s="90" t="inlineStr">
         <is>
-          <t>WisdomTree, Inc. Q3 2026 Earnings Call Summary</t>
+          <t>Apple overtakes Nvidia to become world’s most valuable company amid tech selloff</t>
         </is>
       </c>
     </row>
@@ -10344,17 +10344,17 @@
       </c>
       <c r="AX44" s="79" t="inlineStr">
         <is>
+          <t>Palantir (PLTR) Stock Gets Fair Value Bump After Analysts Lift AI Driven Targets</t>
+        </is>
+      </c>
+      <c r="AY44" s="79" t="inlineStr">
+        <is>
           <t>Dow Jones Futures: Stock Market Sells Off As Apple, Palantir, Midterm Elections Loom; What To Do</t>
         </is>
       </c>
-      <c r="AY44" s="79" t="inlineStr">
+      <c r="AZ44" s="79" t="inlineStr">
         <is>
           <t>Palantir Stock Tests Key Level As Earnings Loom</t>
-        </is>
-      </c>
-      <c r="AZ44" s="79" t="inlineStr">
-        <is>
-          <t>Will Top-Line Improvement Benefit Palantir in Q3 Earnings?</t>
         </is>
       </c>
     </row>
@@ -10918,7 +10918,7 @@
       </c>
       <c r="AZ47" s="90" t="inlineStr">
         <is>
-          <t>Wall Street's Next Blockbuster Stock Split Has Arrived -- The Stock Has Gained 3,050% Since Its 2025 Debut ...</t>
+          <t>Intel, Amazon, Nvidia, ExxonMobil, Sandisk, FedEx Freight, and More Stocks That Explain Today’s Market</t>
         </is>
       </c>
     </row>
@@ -11096,17 +11096,17 @@
       </c>
       <c r="AX48" s="79" t="inlineStr">
         <is>
+          <t>See how Tesla stocks performed for week ending Oct. 30</t>
+        </is>
+      </c>
+      <c r="AY48" s="79" t="inlineStr">
+        <is>
+          <t>Elon Musk vs. Tesla? His Midterm Money Could Work Against His Own Cars</t>
+        </is>
+      </c>
+      <c r="AZ48" s="79" t="inlineStr">
+        <is>
           <t>In A Bad Week For The AI Trade, This One Mag Seven Stock Holds Strong</t>
-        </is>
-      </c>
-      <c r="AY48" s="79" t="inlineStr">
-        <is>
-          <t>Tesla-SpaceX Merger Could Face The Biggest Regulatory Risk In China, BofA Warns</t>
-        </is>
-      </c>
-      <c r="AZ48" s="79" t="inlineStr">
-        <is>
-          <t>Tesla Could Be About to Unlock a Brand-New Revenue Stream. Time to Buy the Stock?</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 30 Oct 2026, 09:39 PM · Yahoo Finance data</t>
+          <t>Built 30 Oct 2026, 11:51 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -19579,7 +19579,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 30 Oct 2026, 09:39 PM · Yahoo Finance data</t>
+          <t>Built 30 Oct 2026, 11:51 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -27515,7 +27515,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 30 Oct 2026, 09:39 PM · Yahoo Finance data</t>
+          <t>Built 30 Oct 2026, 11:51 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">
@@ -35451,7 +35451,7 @@
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Built 30 Oct 2026, 09:39 PM · Yahoo Finance data</t>
+          <t>Built 30 Oct 2026, 11:51 PM · Yahoo Finance data</t>
         </is>
       </c>
       <c r="H3" s="38" t="inlineStr">

</xml_diff>